<commit_message>
[AUTO] Unificación de datos - 2026-09-12 18:11:32
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3331,10 +3331,10 @@
         <v>31</v>
       </c>
       <c r="J34" t="n">
-        <v>30</v>
+        <v>31.4</v>
       </c>
       <c r="K34" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="n">
-        <v>-1</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T34" t="n">
         <v>30.33333333333333</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="K75" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="K79" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="K86" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="K91" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="K321" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="K329" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -29246,10 +29246,10 @@
         <v>24.5</v>
       </c>
       <c r="J333" t="n">
-        <v>25.3</v>
+        <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -29279,7 +29279,7 @@
         <v>28</v>
       </c>
       <c r="S333" t="n">
-        <v>0.8000000000000007</v>
+        <v>0</v>
       </c>
       <c r="T333" t="n">
         <v>24.6</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="K351" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-12 20:02:21
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K75" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K79" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K86" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K91" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -10860,10 +10860,10 @@
         <v>28</v>
       </c>
       <c r="J121" t="n">
-        <v>33.5</v>
+        <v>31.6</v>
       </c>
       <c r="K121" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -10893,7 +10893,7 @@
         <v>28</v>
       </c>
       <c r="S121" t="n">
-        <v>5.5</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T121" t="n">
         <v>30.83333333333333</v>
@@ -13984,10 +13984,10 @@
         <v>24</v>
       </c>
       <c r="J157" t="n">
-        <v>28</v>
+        <v>23.5</v>
       </c>
       <c r="K157" t="n">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="L157" t="inlineStr">
         <is>
@@ -14017,7 +14017,7 @@
         <v>28</v>
       </c>
       <c r="S157" t="n">
-        <v>4</v>
+        <v>-0.5</v>
       </c>
       <c r="T157" t="n">
         <v>25.5</v>
@@ -14676,10 +14676,10 @@
         <v>21</v>
       </c>
       <c r="J165" t="n">
-        <v>25.1</v>
+        <v>20.4</v>
       </c>
       <c r="K165" t="n">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="L165" t="inlineStr">
         <is>
@@ -14709,7 +14709,7 @@
         <v>21</v>
       </c>
       <c r="S165" t="n">
-        <v>4.100000000000001</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T165" t="n">
         <v>24.33333333333333</v>
@@ -20580,10 +20580,10 @@
         <v>31</v>
       </c>
       <c r="J233" t="n">
-        <v>32.3</v>
+        <v>31.2</v>
       </c>
       <c r="K233" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="L233" t="inlineStr">
         <is>
@@ -20611,7 +20611,7 @@
       </c>
       <c r="R233" t="inlineStr"/>
       <c r="S233" t="n">
-        <v>1.299999999999997</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T233" t="n">
         <v>29.3</v>
@@ -21788,10 +21788,10 @@
         <v>21</v>
       </c>
       <c r="J247" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="K247" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L247" t="inlineStr">
         <is>
@@ -21821,7 +21821,7 @@
         <v>21</v>
       </c>
       <c r="S247" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T247" t="n">
         <v>21.2</v>
@@ -22215,10 +22215,10 @@
         <v>21</v>
       </c>
       <c r="J252" t="n">
-        <v>22.3</v>
+        <v>23.1</v>
       </c>
       <c r="K252" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="L252" t="inlineStr">
         <is>
@@ -22248,7 +22248,7 @@
         <v>21</v>
       </c>
       <c r="S252" t="n">
-        <v>1.300000000000001</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="T252" t="n">
         <v>21.8</v>
@@ -25424,10 +25424,10 @@
         <v>21</v>
       </c>
       <c r="J289" t="n">
-        <v>22.8</v>
+        <v>21.7</v>
       </c>
       <c r="K289" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="L289" t="inlineStr">
         <is>
@@ -25457,7 +25457,7 @@
         <v>21</v>
       </c>
       <c r="S289" t="n">
-        <v>1.800000000000001</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T289" t="n">
         <v>21.53333333333333</v>
@@ -27245,10 +27245,10 @@
         <v>24.5</v>
       </c>
       <c r="J310" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="K310" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -27278,7 +27278,7 @@
         <v>28</v>
       </c>
       <c r="S310" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T310" t="n">
         <v>25.13333333333334</v>
@@ -29246,10 +29246,10 @@
         <v>24.5</v>
       </c>
       <c r="J333" t="n">
-        <v>24.5</v>
+        <v>25.3</v>
       </c>
       <c r="K333" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -29279,7 +29279,7 @@
         <v>28</v>
       </c>
       <c r="S333" t="n">
-        <v>0</v>
+        <v>0.8000000000000007</v>
       </c>
       <c r="T333" t="n">
         <v>24.6</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-13 15:41:35
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3159,10 +3159,10 @@
         <v>31</v>
       </c>
       <c r="J32" t="n">
-        <v>16.6</v>
+        <v>32.1</v>
       </c>
       <c r="K32" t="n">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="n">
-        <v>-14.4</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T32" t="n">
         <v>25.6</v>
@@ -4794,10 +4794,10 @@
         <v>31</v>
       </c>
       <c r="J51" t="n">
-        <v>28.3</v>
+        <v>34.5</v>
       </c>
       <c r="K51" t="n">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="n">
-        <v>-2.699999999999999</v>
+        <v>3.5</v>
       </c>
       <c r="T51" t="n">
         <v>31.46666666666667</v>
@@ -5611,7 +5611,7 @@
         <v>3</v>
       </c>
       <c r="V60" t="n">
-        <v>24.52222222222223</v>
+        <v>24.52222222222222</v>
       </c>
       <c r="W60" t="n">
         <v>20.5</v>
@@ -5656,10 +5656,10 @@
         <v>24</v>
       </c>
       <c r="J61" t="n">
-        <v>26.4</v>
+        <v>16.6</v>
       </c>
       <c r="K61" t="n">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -5689,7 +5689,7 @@
         <v>28</v>
       </c>
       <c r="S61" t="n">
-        <v>2.399999999999999</v>
+        <v>-7.399999999999999</v>
       </c>
       <c r="T61" t="n">
         <v>23.4</v>
@@ -5698,7 +5698,7 @@
         <v>3</v>
       </c>
       <c r="V61" t="n">
-        <v>24.64444444444445</v>
+        <v>24.64444444444444</v>
       </c>
       <c r="W61" t="n">
         <v>20.5</v>
@@ -6613,10 +6613,10 @@
         <v>21</v>
       </c>
       <c r="J72" t="n">
-        <v>23.9</v>
+        <v>24.6</v>
       </c>
       <c r="K72" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -6646,7 +6646,7 @@
         <v>21</v>
       </c>
       <c r="S72" t="n">
-        <v>2.899999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T72" t="n">
         <v>22.76666666666667</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="K75" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -6959,10 +6959,10 @@
         <v>28</v>
       </c>
       <c r="J76" t="n">
-        <v>27.3</v>
+        <v>24.1</v>
       </c>
       <c r="K76" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -6992,7 +6992,7 @@
         <v>28</v>
       </c>
       <c r="S76" t="n">
-        <v>-0.6999999999999993</v>
+        <v>-3.899999999999999</v>
       </c>
       <c r="T76" t="n">
         <v>25.33333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="K79" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7566,10 +7566,10 @@
         <v>21</v>
       </c>
       <c r="J83" t="n">
-        <v>19.3</v>
+        <v>20.2</v>
       </c>
       <c r="K83" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -7599,7 +7599,7 @@
         <v>21</v>
       </c>
       <c r="S83" t="n">
-        <v>-1.699999999999999</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T83" t="n">
         <v>20.46666666666667</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="K86" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="K91" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -8994,7 +8994,7 @@
         <v>3</v>
       </c>
       <c r="V99" t="n">
-        <v>26.17777777777777</v>
+        <v>26.17777777777778</v>
       </c>
       <c r="W99" t="n">
         <v>17.5</v>
@@ -12946,10 +12946,10 @@
         <v>35</v>
       </c>
       <c r="J145" t="n">
-        <v>20.3</v>
+        <v>48.5</v>
       </c>
       <c r="K145" t="n">
-        <v>58</v>
+        <v>138</v>
       </c>
       <c r="L145" t="inlineStr">
         <is>
@@ -12979,7 +12979,7 @@
         <v>41</v>
       </c>
       <c r="S145" t="n">
-        <v>-14.7</v>
+        <v>13.5</v>
       </c>
       <c r="T145" t="n">
         <v>30.76666666666667</v>
@@ -13379,10 +13379,10 @@
         <v>35</v>
       </c>
       <c r="J150" t="n">
-        <v>40.9</v>
+        <v>40.2</v>
       </c>
       <c r="K150" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="L150" t="inlineStr">
         <is>
@@ -13412,7 +13412,7 @@
         <v>41</v>
       </c>
       <c r="S150" t="n">
-        <v>5.899999999999999</v>
+        <v>5.200000000000003</v>
       </c>
       <c r="T150" t="n">
         <v>36</v>
@@ -13464,10 +13464,10 @@
         <v>21</v>
       </c>
       <c r="J151" t="n">
-        <v>25.8</v>
+        <v>24.1</v>
       </c>
       <c r="K151" t="n">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="L151" t="inlineStr">
         <is>
@@ -13497,10 +13497,10 @@
         <v>21</v>
       </c>
       <c r="S151" t="n">
-        <v>4.800000000000001</v>
+        <v>3.100000000000001</v>
       </c>
       <c r="T151" t="n">
-        <v>23.43333333333334</v>
+        <v>23.43333333333333</v>
       </c>
       <c r="U151" t="n">
         <v>3</v>
@@ -14245,10 +14245,10 @@
         <v>28</v>
       </c>
       <c r="J160" t="n">
-        <v>29.4</v>
+        <v>31.6</v>
       </c>
       <c r="K160" t="n">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="L160" t="inlineStr">
         <is>
@@ -14278,7 +14278,7 @@
         <v>28</v>
       </c>
       <c r="S160" t="n">
-        <v>1.399999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T160" t="n">
         <v>28.43333333333334</v>
@@ -14417,10 +14417,10 @@
         <v>21</v>
       </c>
       <c r="J162" t="n">
-        <v>26</v>
+        <v>23.9</v>
       </c>
       <c r="K162" t="n">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="L162" t="inlineStr">
         <is>
@@ -14450,7 +14450,7 @@
         <v>21</v>
       </c>
       <c r="S162" t="n">
-        <v>5</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="T162" t="n">
         <v>23.4</v>
@@ -21875,10 +21875,10 @@
         <v>21</v>
       </c>
       <c r="J248" t="n">
-        <v>22.5</v>
+        <v>21.9</v>
       </c>
       <c r="K248" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L248" t="inlineStr">
         <is>
@@ -21906,7 +21906,7 @@
       </c>
       <c r="R248" t="inlineStr"/>
       <c r="S248" t="n">
-        <v>1.5</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T248" t="n">
         <v>21.73333333333333</v>
@@ -23259,10 +23259,10 @@
         <v>28</v>
       </c>
       <c r="J264" t="n">
-        <v>32.3</v>
+        <v>29.9</v>
       </c>
       <c r="K264" t="n">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="L264" t="inlineStr">
         <is>
@@ -23292,7 +23292,7 @@
         <v>28</v>
       </c>
       <c r="S264" t="n">
-        <v>4.299999999999997</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T264" t="n">
         <v>28.53333333333333</v>
@@ -23431,10 +23431,10 @@
         <v>28</v>
       </c>
       <c r="J266" t="n">
-        <v>28.1</v>
+        <v>27</v>
       </c>
       <c r="K266" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L266" t="inlineStr">
         <is>
@@ -23464,7 +23464,7 @@
         <v>28</v>
       </c>
       <c r="S266" t="n">
-        <v>0.1000000000000014</v>
+        <v>-1</v>
       </c>
       <c r="T266" t="n">
         <v>26.96666666666667</v>
@@ -24297,10 +24297,10 @@
         <v>28</v>
       </c>
       <c r="J276" t="n">
-        <v>26.5</v>
+        <v>28.4</v>
       </c>
       <c r="K276" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="L276" t="inlineStr">
         <is>
@@ -24330,7 +24330,7 @@
         <v>28</v>
       </c>
       <c r="S276" t="n">
-        <v>-1.5</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T276" t="n">
         <v>27.53333333333333</v>
@@ -26899,10 +26899,10 @@
         <v>21</v>
       </c>
       <c r="J306" t="n">
-        <v>22</v>
+        <v>19.4</v>
       </c>
       <c r="K306" t="n">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -26932,7 +26932,7 @@
         <v>21</v>
       </c>
       <c r="S306" t="n">
-        <v>1</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T306" t="n">
         <v>20.8</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="K321" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28724,10 +28724,10 @@
         <v>24.5</v>
       </c>
       <c r="J327" t="n">
-        <v>18.6</v>
+        <v>24.3</v>
       </c>
       <c r="K327" t="n">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -28757,10 +28757,10 @@
         <v>28</v>
       </c>
       <c r="S327" t="n">
-        <v>-5.899999999999999</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T327" t="n">
-        <v>21.93333333333333</v>
+        <v>21.93333333333334</v>
       </c>
       <c r="U327" t="n">
         <v>3</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="K329" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="K351" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-13 17:32:09
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -21011,10 +21011,10 @@
         <v>28</v>
       </c>
       <c r="J238" t="n">
-        <v>25.3</v>
+        <v>29.6</v>
       </c>
       <c r="K238" t="n">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="L238" t="inlineStr">
         <is>
@@ -21044,7 +21044,7 @@
         <v>28</v>
       </c>
       <c r="S238" t="n">
-        <v>-2.699999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T238" t="n">
         <v>27.83333333333333</v>
@@ -21098,10 +21098,10 @@
         <v>31</v>
       </c>
       <c r="J239" t="n">
-        <v>33.2</v>
+        <v>32.6</v>
       </c>
       <c r="K239" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L239" t="inlineStr">
         <is>
@@ -21129,7 +21129,7 @@
       </c>
       <c r="R239" t="inlineStr"/>
       <c r="S239" t="n">
-        <v>2.200000000000003</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T239" t="n">
         <v>32.06666666666667</v>
@@ -21183,10 +21183,10 @@
         <v>42</v>
       </c>
       <c r="J240" t="n">
-        <v>15.9</v>
+        <v>52.5</v>
       </c>
       <c r="K240" t="n">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="L240" t="inlineStr">
         <is>
@@ -21216,7 +21216,7 @@
         <v>48</v>
       </c>
       <c r="S240" t="n">
-        <v>-26.1</v>
+        <v>10.5</v>
       </c>
       <c r="T240" t="n">
         <v>39.6</v>
@@ -21875,10 +21875,10 @@
         <v>21</v>
       </c>
       <c r="J248" t="n">
-        <v>21.9</v>
+        <v>22.5</v>
       </c>
       <c r="K248" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="L248" t="inlineStr">
         <is>
@@ -21906,7 +21906,7 @@
       </c>
       <c r="R248" t="inlineStr"/>
       <c r="S248" t="n">
-        <v>0.8999999999999986</v>
+        <v>1.5</v>
       </c>
       <c r="T248" t="n">
         <v>21.73333333333333</v>
@@ -23259,10 +23259,10 @@
         <v>28</v>
       </c>
       <c r="J264" t="n">
-        <v>29.9</v>
+        <v>32.3</v>
       </c>
       <c r="K264" t="n">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="L264" t="inlineStr">
         <is>
@@ -23292,7 +23292,7 @@
         <v>28</v>
       </c>
       <c r="S264" t="n">
-        <v>1.899999999999999</v>
+        <v>4.299999999999997</v>
       </c>
       <c r="T264" t="n">
         <v>28.53333333333333</v>
@@ -23431,10 +23431,10 @@
         <v>28</v>
       </c>
       <c r="J266" t="n">
-        <v>27</v>
+        <v>28.1</v>
       </c>
       <c r="K266" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L266" t="inlineStr">
         <is>
@@ -23464,7 +23464,7 @@
         <v>28</v>
       </c>
       <c r="S266" t="n">
-        <v>-1</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T266" t="n">
         <v>26.96666666666667</v>
@@ -24297,10 +24297,10 @@
         <v>28</v>
       </c>
       <c r="J276" t="n">
-        <v>28.4</v>
+        <v>26.5</v>
       </c>
       <c r="K276" t="n">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="L276" t="inlineStr">
         <is>
@@ -24330,7 +24330,7 @@
         <v>28</v>
       </c>
       <c r="S276" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1.5</v>
       </c>
       <c r="T276" t="n">
         <v>27.53333333333333</v>
@@ -26899,10 +26899,10 @@
         <v>21</v>
       </c>
       <c r="J306" t="n">
-        <v>19.4</v>
+        <v>22</v>
       </c>
       <c r="K306" t="n">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -26932,7 +26932,7 @@
         <v>21</v>
       </c>
       <c r="S306" t="n">
-        <v>-1.600000000000001</v>
+        <v>1</v>
       </c>
       <c r="T306" t="n">
         <v>20.8</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28724,10 +28724,10 @@
         <v>24.5</v>
       </c>
       <c r="J327" t="n">
-        <v>24.3</v>
+        <v>18.6</v>
       </c>
       <c r="K327" t="n">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -28757,10 +28757,10 @@
         <v>28</v>
       </c>
       <c r="S327" t="n">
-        <v>-0.1999999999999993</v>
+        <v>-5.899999999999999</v>
       </c>
       <c r="T327" t="n">
-        <v>21.93333333333334</v>
+        <v>21.93333333333333</v>
       </c>
       <c r="U327" t="n">
         <v>3</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-13 18:38:10
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4446,10 +4446,10 @@
         <v>24</v>
       </c>
       <c r="J47" t="n">
-        <v>23.8</v>
+        <v>24.9</v>
       </c>
       <c r="K47" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -4479,7 +4479,7 @@
         <v>28</v>
       </c>
       <c r="S47" t="n">
-        <v>-0.1999999999999993</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T47" t="n">
         <v>21.43333333333333</v>
@@ -5397,10 +5397,10 @@
         <v>31</v>
       </c>
       <c r="J58" t="n">
-        <v>31.4</v>
+        <v>35.8</v>
       </c>
       <c r="K58" t="n">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
       </c>
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="n">
-        <v>0.3999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T58" t="n">
-        <v>30.66666666666666</v>
+        <v>30.66666666666667</v>
       </c>
       <c r="U58" t="n">
         <v>3</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K75" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7046,10 +7046,10 @@
         <v>28</v>
       </c>
       <c r="J77" t="n">
-        <v>24.8</v>
+        <v>25.9</v>
       </c>
       <c r="K77" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -7079,10 +7079,10 @@
         <v>28</v>
       </c>
       <c r="S77" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="T77" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="U77" t="n">
         <v>3</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K79" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K86" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -7912,10 +7912,10 @@
         <v>21</v>
       </c>
       <c r="J87" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K87" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="L87" t="inlineStr">
         <is>
@@ -7945,7 +7945,7 @@
         <v>21</v>
       </c>
       <c r="S87" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="T87" t="n">
         <v>19.9</v>
@@ -7999,10 +7999,10 @@
         <v>35</v>
       </c>
       <c r="J88" t="n">
-        <v>36.5</v>
+        <v>25.3</v>
       </c>
       <c r="K88" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
         <v>41</v>
       </c>
       <c r="S88" t="n">
-        <v>1.5</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="T88" t="n">
         <v>33.1</v>
@@ -8086,10 +8086,10 @@
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>36.7</v>
+        <v>39.1</v>
       </c>
       <c r="K89" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8119,7 +8119,7 @@
         <v>41</v>
       </c>
       <c r="S89" t="n">
-        <v>1.700000000000003</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T89" t="n">
         <v>35.73333333333333</v>
@@ -8128,7 +8128,7 @@
         <v>3</v>
       </c>
       <c r="V89" t="n">
-        <v>35.86296296296296</v>
+        <v>35.86296296296297</v>
       </c>
       <c r="W89" t="n">
         <v>31.5</v>
@@ -8173,10 +8173,10 @@
         <v>35</v>
       </c>
       <c r="J90" t="n">
-        <v>39.8</v>
+        <v>40.3</v>
       </c>
       <c r="K90" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -8206,7 +8206,7 @@
         <v>41</v>
       </c>
       <c r="S90" t="n">
-        <v>4.799999999999997</v>
+        <v>5.299999999999997</v>
       </c>
       <c r="T90" t="n">
         <v>36.16666666666666</v>
@@ -8215,7 +8215,7 @@
         <v>3</v>
       </c>
       <c r="V90" t="n">
-        <v>38.87407407407408</v>
+        <v>38.87407407407407</v>
       </c>
       <c r="W90" t="n">
         <v>31.5</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K91" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -8345,10 +8345,10 @@
         <v>35</v>
       </c>
       <c r="J92" t="n">
-        <v>33.9</v>
+        <v>36.7</v>
       </c>
       <c r="K92" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
@@ -8378,7 +8378,7 @@
         <v>41</v>
       </c>
       <c r="S92" t="n">
-        <v>-1.100000000000001</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T92" t="n">
         <v>36.2</v>
@@ -8517,10 +8517,10 @@
         <v>21</v>
       </c>
       <c r="J94" t="n">
-        <v>22.5</v>
+        <v>23.7</v>
       </c>
       <c r="K94" t="n">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -8550,7 +8550,7 @@
         <v>21</v>
       </c>
       <c r="S94" t="n">
-        <v>1.5</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="T94" t="n">
         <v>21.9</v>
@@ -8604,10 +8604,10 @@
         <v>35</v>
       </c>
       <c r="J95" t="n">
-        <v>34.1</v>
+        <v>34.3</v>
       </c>
       <c r="K95" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L95" t="inlineStr">
         <is>
@@ -8637,7 +8637,7 @@
         <v>41</v>
       </c>
       <c r="S95" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="T95" t="n">
         <v>35.13333333333333</v>
@@ -8691,10 +8691,10 @@
         <v>35</v>
       </c>
       <c r="J96" t="n">
-        <v>33.8</v>
+        <v>36.6</v>
       </c>
       <c r="K96" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="L96" t="inlineStr">
         <is>
@@ -8724,7 +8724,7 @@
         <v>41</v>
       </c>
       <c r="S96" t="n">
-        <v>-1.200000000000003</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T96" t="n">
         <v>35.73333333333333</v>
@@ -19103,10 +19103,10 @@
         <v>28</v>
       </c>
       <c r="J216" t="n">
-        <v>28.5</v>
+        <v>27.7</v>
       </c>
       <c r="K216" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L216" t="inlineStr">
         <is>
@@ -19136,7 +19136,7 @@
         <v>28</v>
       </c>
       <c r="S216" t="n">
-        <v>0.5</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T216" t="n">
         <v>28.33333333333333</v>
@@ -20060,10 +20060,10 @@
         <v>28</v>
       </c>
       <c r="J227" t="n">
-        <v>29.3</v>
+        <v>30.1</v>
       </c>
       <c r="K227" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="L227" t="inlineStr">
         <is>
@@ -20093,7 +20093,7 @@
         <v>28</v>
       </c>
       <c r="S227" t="n">
-        <v>1.300000000000001</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="T227" t="n">
         <v>28.96666666666667</v>
@@ -20319,10 +20319,10 @@
         <v>21</v>
       </c>
       <c r="J230" t="n">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="K230" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L230" t="inlineStr">
         <is>
@@ -20352,7 +20352,7 @@
         <v>21</v>
       </c>
       <c r="S230" t="n">
-        <v>1.800000000000001</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="T230" t="n">
         <v>21.56666666666667</v>
@@ -20406,10 +20406,10 @@
         <v>28</v>
       </c>
       <c r="J231" t="n">
-        <v>24.5</v>
+        <v>26</v>
       </c>
       <c r="K231" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="L231" t="inlineStr">
         <is>
@@ -20439,7 +20439,7 @@
         <v>28</v>
       </c>
       <c r="S231" t="n">
-        <v>-3.5</v>
+        <v>-2</v>
       </c>
       <c r="T231" t="n">
         <v>25.53333333333333</v>
@@ -20493,10 +20493,10 @@
         <v>28</v>
       </c>
       <c r="J232" t="n">
-        <v>30.9</v>
+        <v>24.9</v>
       </c>
       <c r="K232" t="n">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="L232" t="inlineStr">
         <is>
@@ -20526,7 +20526,7 @@
         <v>28</v>
       </c>
       <c r="S232" t="n">
-        <v>2.899999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T232" t="n">
         <v>27.93333333333333</v>
@@ -20665,10 +20665,10 @@
         <v>42</v>
       </c>
       <c r="J234" t="n">
-        <v>31.1</v>
+        <v>49</v>
       </c>
       <c r="K234" t="n">
-        <v>74</v>
+        <v>116</v>
       </c>
       <c r="L234" t="inlineStr">
         <is>
@@ -20698,7 +20698,7 @@
         <v>48</v>
       </c>
       <c r="S234" t="n">
-        <v>-10.9</v>
+        <v>7</v>
       </c>
       <c r="T234" t="n">
         <v>43.9</v>
@@ -21011,10 +21011,10 @@
         <v>28</v>
       </c>
       <c r="J238" t="n">
-        <v>29.6</v>
+        <v>25.3</v>
       </c>
       <c r="K238" t="n">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="L238" t="inlineStr">
         <is>
@@ -21044,7 +21044,7 @@
         <v>28</v>
       </c>
       <c r="S238" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="T238" t="n">
         <v>27.83333333333333</v>
@@ -21098,10 +21098,10 @@
         <v>31</v>
       </c>
       <c r="J239" t="n">
-        <v>32.6</v>
+        <v>33.2</v>
       </c>
       <c r="K239" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="L239" t="inlineStr">
         <is>
@@ -21129,7 +21129,7 @@
       </c>
       <c r="R239" t="inlineStr"/>
       <c r="S239" t="n">
-        <v>1.600000000000001</v>
+        <v>2.200000000000003</v>
       </c>
       <c r="T239" t="n">
         <v>32.06666666666667</v>
@@ -21183,10 +21183,10 @@
         <v>42</v>
       </c>
       <c r="J240" t="n">
-        <v>52.5</v>
+        <v>15.9</v>
       </c>
       <c r="K240" t="n">
-        <v>125</v>
+        <v>38</v>
       </c>
       <c r="L240" t="inlineStr">
         <is>
@@ -21216,7 +21216,7 @@
         <v>48</v>
       </c>
       <c r="S240" t="n">
-        <v>10.5</v>
+        <v>-26.1</v>
       </c>
       <c r="T240" t="n">
         <v>39.6</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-14 07:40:13
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3588,10 +3588,10 @@
         <v>28</v>
       </c>
       <c r="J37" t="n">
-        <v>27.7</v>
+        <v>26.8</v>
       </c>
       <c r="K37" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -3621,7 +3621,7 @@
         <v>28</v>
       </c>
       <c r="S37" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T37" t="n">
         <v>27.16666666666667</v>
@@ -5235,10 +5235,10 @@
         <v>28</v>
       </c>
       <c r="J56" t="n">
-        <v>27.5</v>
+        <v>29.6</v>
       </c>
       <c r="K56" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -5268,7 +5268,7 @@
         <v>28</v>
       </c>
       <c r="S56" t="n">
-        <v>-0.5</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T56" t="n">
         <v>28.6</v>
@@ -5277,7 +5277,7 @@
         <v>3</v>
       </c>
       <c r="V56" t="n">
-        <v>32.9888888888889</v>
+        <v>32.98888888888889</v>
       </c>
       <c r="W56" t="n">
         <v>24.5</v>
@@ -5322,10 +5322,10 @@
         <v>28</v>
       </c>
       <c r="J57" t="n">
-        <v>32.5</v>
+        <v>30.4</v>
       </c>
       <c r="K57" t="n">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -5355,7 +5355,7 @@
         <v>28</v>
       </c>
       <c r="S57" t="n">
-        <v>4.5</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T57" t="n">
         <v>30.16666666666667</v>
@@ -6710,10 +6710,10 @@
         <v>21</v>
       </c>
       <c r="J73" t="n">
-        <v>22.2</v>
+        <v>20.9</v>
       </c>
       <c r="K73" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -6743,7 +6743,7 @@
         <v>21</v>
       </c>
       <c r="S73" t="n">
-        <v>1.199999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T73" t="n">
         <v>22.03333333333333</v>
@@ -7489,10 +7489,10 @@
         <v>21</v>
       </c>
       <c r="J82" t="n">
-        <v>20</v>
+        <v>19.4</v>
       </c>
       <c r="K82" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -7522,7 +7522,7 @@
         <v>21</v>
       </c>
       <c r="S82" t="n">
-        <v>-1</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T82" t="n">
         <v>20.5</v>
@@ -8531,10 +8531,10 @@
         <v>24.5</v>
       </c>
       <c r="J94" t="n">
-        <v>22.5</v>
+        <v>20.7</v>
       </c>
       <c r="K94" t="n">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -8564,7 +8564,7 @@
         <v>28</v>
       </c>
       <c r="S94" t="n">
-        <v>-2</v>
+        <v>-3.800000000000001</v>
       </c>
       <c r="T94" t="n">
         <v>21.53333333333333</v>
@@ -9053,10 +9053,10 @@
         <v>24.5</v>
       </c>
       <c r="J100" t="n">
-        <v>24.6</v>
+        <v>20.9</v>
       </c>
       <c r="K100" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="L100" t="inlineStr">
         <is>
@@ -9086,7 +9086,7 @@
         <v>28</v>
       </c>
       <c r="S100" t="n">
-        <v>0.1000000000000014</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="T100" t="n">
         <v>23.96666666666667</v>
@@ -10271,10 +10271,10 @@
         <v>24.5</v>
       </c>
       <c r="J114" t="n">
-        <v>24</v>
+        <v>31.1</v>
       </c>
       <c r="K114" t="n">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -10304,7 +10304,7 @@
         <v>28</v>
       </c>
       <c r="S114" t="n">
-        <v>-0.5</v>
+        <v>6.600000000000001</v>
       </c>
       <c r="T114" t="n">
         <v>29.13333333333334</v>
@@ -11924,10 +11924,10 @@
         <v>24.5</v>
       </c>
       <c r="J133" t="n">
-        <v>27.8</v>
+        <v>24.3</v>
       </c>
       <c r="K133" t="n">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -11957,7 +11957,7 @@
         <v>28</v>
       </c>
       <c r="S133" t="n">
-        <v>3.300000000000001</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T133" t="n">
         <v>25</v>
@@ -12618,10 +12618,10 @@
         <v>24.5</v>
       </c>
       <c r="J141" t="n">
-        <v>22.7</v>
+        <v>29.1</v>
       </c>
       <c r="K141" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="L141" t="inlineStr">
         <is>
@@ -12651,7 +12651,7 @@
         <v>28</v>
       </c>
       <c r="S141" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="T141" t="n">
         <v>25.3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-15 07:16:35
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4964,10 +4964,10 @@
         <v>24</v>
       </c>
       <c r="J53" t="n">
-        <v>22.8</v>
+        <v>25.3</v>
       </c>
       <c r="K53" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
         <v>28</v>
       </c>
       <c r="S53" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="T53" t="n">
         <v>24.6</v>
@@ -6613,10 +6613,10 @@
         <v>21</v>
       </c>
       <c r="J72" t="n">
-        <v>24.6</v>
+        <v>23.9</v>
       </c>
       <c r="K72" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -6646,7 +6646,7 @@
         <v>21</v>
       </c>
       <c r="S72" t="n">
-        <v>3.600000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="T72" t="n">
         <v>22.76666666666667</v>
@@ -7046,7 +7046,7 @@
         <v>28</v>
       </c>
       <c r="J77" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="K77" t="n">
         <v>88</v>
@@ -7079,7 +7079,7 @@
         <v>28</v>
       </c>
       <c r="S77" t="n">
-        <v>-3.300000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T77" t="n">
         <v>25.13333333333334</v>
@@ -7133,10 +7133,10 @@
         <v>28</v>
       </c>
       <c r="J78" t="n">
-        <v>30.7</v>
+        <v>29.2</v>
       </c>
       <c r="K78" t="n">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
         <v>28</v>
       </c>
       <c r="S78" t="n">
-        <v>2.699999999999999</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="T78" t="n">
         <v>29.2</v>
@@ -8952,10 +8952,10 @@
         <v>21</v>
       </c>
       <c r="J99" t="n">
-        <v>20.2</v>
+        <v>24.2</v>
       </c>
       <c r="K99" t="n">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="L99" t="inlineStr">
         <is>
@@ -8985,7 +8985,7 @@
         <v>21</v>
       </c>
       <c r="S99" t="n">
-        <v>-0.8000000000000007</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="T99" t="n">
         <v>23.23333333333333</v>
@@ -9039,10 +9039,10 @@
         <v>28</v>
       </c>
       <c r="J100" t="n">
-        <v>29.8</v>
+        <v>25.8</v>
       </c>
       <c r="K100" t="n">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="L100" t="inlineStr">
         <is>
@@ -9072,7 +9072,7 @@
         <v>28</v>
       </c>
       <c r="S100" t="n">
-        <v>1.800000000000001</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="T100" t="n">
         <v>27.73333333333333</v>
@@ -9126,10 +9126,10 @@
         <v>21</v>
       </c>
       <c r="J101" t="n">
-        <v>29</v>
+        <v>18.4</v>
       </c>
       <c r="K101" t="n">
-        <v>138</v>
+        <v>88</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
@@ -9159,7 +9159,7 @@
         <v>21</v>
       </c>
       <c r="S101" t="n">
-        <v>8</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T101" t="n">
         <v>24.53333333333333</v>
@@ -9903,10 +9903,10 @@
         <v>35</v>
       </c>
       <c r="J110" t="n">
-        <v>49.1</v>
+        <v>31.4</v>
       </c>
       <c r="K110" t="n">
-        <v>140</v>
+        <v>90</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -9936,7 +9936,7 @@
         <v>41</v>
       </c>
       <c r="S110" t="n">
-        <v>14.1</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="T110" t="n">
         <v>43.96666666666667</v>
@@ -10164,10 +10164,10 @@
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>22.5</v>
+        <v>26.3</v>
       </c>
       <c r="K113" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         <v>41</v>
       </c>
       <c r="S113" t="n">
-        <v>-12.5</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="T113" t="n">
         <v>25.5</v>
@@ -22045,10 +22045,10 @@
         <v>21</v>
       </c>
       <c r="J250" t="n">
-        <v>24.6</v>
+        <v>13.3</v>
       </c>
       <c r="K250" t="n">
-        <v>117</v>
+        <v>63</v>
       </c>
       <c r="L250" t="inlineStr">
         <is>
@@ -22076,7 +22076,7 @@
       </c>
       <c r="R250" t="inlineStr"/>
       <c r="S250" t="n">
-        <v>3.600000000000001</v>
+        <v>-7.699999999999999</v>
       </c>
       <c r="T250" t="n">
         <v>20.13333333333334</v>
@@ -24036,10 +24036,10 @@
         <v>28</v>
       </c>
       <c r="J273" t="n">
-        <v>28.7</v>
+        <v>27.5</v>
       </c>
       <c r="K273" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="L273" t="inlineStr">
         <is>
@@ -24069,7 +24069,7 @@
         <v>28</v>
       </c>
       <c r="S273" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.5</v>
       </c>
       <c r="T273" t="n">
         <v>28.6</v>
@@ -24078,7 +24078,7 @@
         <v>3</v>
       </c>
       <c r="V273" t="n">
-        <v>32.98888888888889</v>
+        <v>32.9888888888889</v>
       </c>
       <c r="W273" t="n">
         <v>24.5</v>
@@ -24645,10 +24645,10 @@
         <v>21</v>
       </c>
       <c r="J280" t="n">
-        <v>19.9</v>
+        <v>21.4</v>
       </c>
       <c r="K280" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="L280" t="inlineStr">
         <is>
@@ -24678,7 +24678,7 @@
         <v>21</v>
       </c>
       <c r="S280" t="n">
-        <v>-1.100000000000001</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T280" t="n">
         <v>21</v>
@@ -29027,7 +29027,7 @@
         <v>3</v>
       </c>
       <c r="V330" t="n">
-        <v>25.57777777777778</v>
+        <v>25.57777777777777</v>
       </c>
       <c r="W330" t="n">
         <v>21</v>
@@ -29420,10 +29420,10 @@
         <v>24.5</v>
       </c>
       <c r="J335" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="K335" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="L335" t="inlineStr">
         <is>
@@ -29453,7 +29453,7 @@
         <v>28</v>
       </c>
       <c r="S335" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T335" t="n">
         <v>35.8</v>
@@ -30725,10 +30725,10 @@
         <v>24.5</v>
       </c>
       <c r="J350" t="n">
-        <v>27.8</v>
+        <v>24.3</v>
       </c>
       <c r="K350" t="n">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="L350" t="inlineStr">
         <is>
@@ -30758,7 +30758,7 @@
         <v>28</v>
       </c>
       <c r="S350" t="n">
-        <v>3.300000000000001</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T350" t="n">
         <v>25</v>
@@ -31504,10 +31504,10 @@
         <v>24.5</v>
       </c>
       <c r="J359" t="n">
-        <v>27.4</v>
+        <v>23.2</v>
       </c>
       <c r="K359" t="n">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -31537,7 +31537,7 @@
         <v>28</v>
       </c>
       <c r="S359" t="n">
-        <v>2.899999999999999</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T359" t="n">
         <v>24.7</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-15 16:18:10
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2165,7 +2165,7 @@
         <v>3</v>
       </c>
       <c r="V20" t="n">
-        <v>60.65555555555555</v>
+        <v>53.27037037037038</v>
       </c>
       <c r="W20" t="n">
         <v>44.1</v>
@@ -4446,10 +4446,10 @@
         <v>24</v>
       </c>
       <c r="J47" t="n">
-        <v>23.8</v>
+        <v>24.9</v>
       </c>
       <c r="K47" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -4479,7 +4479,7 @@
         <v>28</v>
       </c>
       <c r="S47" t="n">
-        <v>-0.1999999999999993</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T47" t="n">
         <v>21.43333333333333</v>
@@ -4964,10 +4964,10 @@
         <v>24</v>
       </c>
       <c r="J53" t="n">
-        <v>25.3</v>
+        <v>22.8</v>
       </c>
       <c r="K53" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
         <v>28</v>
       </c>
       <c r="S53" t="n">
-        <v>1.300000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T53" t="n">
         <v>24.6</v>
@@ -6613,10 +6613,10 @@
         <v>21</v>
       </c>
       <c r="J72" t="n">
-        <v>23.9</v>
+        <v>24.6</v>
       </c>
       <c r="K72" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -6646,7 +6646,7 @@
         <v>21</v>
       </c>
       <c r="S72" t="n">
-        <v>2.899999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T72" t="n">
         <v>22.76666666666667</v>
@@ -7133,10 +7133,10 @@
         <v>28</v>
       </c>
       <c r="J78" t="n">
-        <v>29.2</v>
+        <v>30.7</v>
       </c>
       <c r="K78" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
         <v>28</v>
       </c>
       <c r="S78" t="n">
-        <v>1.199999999999999</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="T78" t="n">
         <v>29.2</v>
@@ -9903,10 +9903,10 @@
         <v>35</v>
       </c>
       <c r="J110" t="n">
-        <v>31.4</v>
+        <v>49.1</v>
       </c>
       <c r="K110" t="n">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -9936,7 +9936,7 @@
         <v>41</v>
       </c>
       <c r="S110" t="n">
-        <v>-3.600000000000001</v>
+        <v>14.1</v>
       </c>
       <c r="T110" t="n">
         <v>43.96666666666667</v>
@@ -10164,10 +10164,10 @@
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>26.3</v>
+        <v>22.5</v>
       </c>
       <c r="K113" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         <v>41</v>
       </c>
       <c r="S113" t="n">
-        <v>-8.699999999999999</v>
+        <v>-12.5</v>
       </c>
       <c r="T113" t="n">
         <v>25.5</v>
@@ -18931,10 +18931,10 @@
         <v>31</v>
       </c>
       <c r="J214" t="n">
-        <v>33.7</v>
+        <v>36.5</v>
       </c>
       <c r="K214" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -18962,7 +18962,7 @@
       </c>
       <c r="R214" t="inlineStr"/>
       <c r="S214" t="n">
-        <v>2.700000000000003</v>
+        <v>5.5</v>
       </c>
       <c r="T214" t="n">
         <v>33.66666666666666</v>
@@ -22045,10 +22045,10 @@
         <v>21</v>
       </c>
       <c r="J250" t="n">
-        <v>13.3</v>
+        <v>24.6</v>
       </c>
       <c r="K250" t="n">
-        <v>63</v>
+        <v>117</v>
       </c>
       <c r="L250" t="inlineStr">
         <is>
@@ -22076,7 +22076,7 @@
       </c>
       <c r="R250" t="inlineStr"/>
       <c r="S250" t="n">
-        <v>-7.699999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T250" t="n">
         <v>20.13333333333334</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -29420,10 +29420,10 @@
         <v>24.5</v>
       </c>
       <c r="J335" t="n">
-        <v>25.6</v>
+        <v>24</v>
       </c>
       <c r="K335" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="L335" t="inlineStr">
         <is>
@@ -29453,7 +29453,7 @@
         <v>28</v>
       </c>
       <c r="S335" t="n">
-        <v>1.100000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="T335" t="n">
         <v>35.8</v>
@@ -30725,10 +30725,10 @@
         <v>24.5</v>
       </c>
       <c r="J350" t="n">
-        <v>24.3</v>
+        <v>27.8</v>
       </c>
       <c r="K350" t="n">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="L350" t="inlineStr">
         <is>
@@ -30758,7 +30758,7 @@
         <v>28</v>
       </c>
       <c r="S350" t="n">
-        <v>-0.1999999999999993</v>
+        <v>3.300000000000001</v>
       </c>
       <c r="T350" t="n">
         <v>25</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>
@@ -31504,10 +31504,10 @@
         <v>24.5</v>
       </c>
       <c r="J359" t="n">
-        <v>23.2</v>
+        <v>27.4</v>
       </c>
       <c r="K359" t="n">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -31537,7 +31537,7 @@
         <v>28</v>
       </c>
       <c r="S359" t="n">
-        <v>-1.300000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="T359" t="n">
         <v>24.7</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-15 18:15:29
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4446,10 +4446,10 @@
         <v>24</v>
       </c>
       <c r="J47" t="n">
-        <v>24.9</v>
+        <v>23.8</v>
       </c>
       <c r="K47" t="n">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -4479,7 +4479,7 @@
         <v>28</v>
       </c>
       <c r="S47" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T47" t="n">
         <v>21.43333333333333</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="K75" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="K79" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="K86" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="K91" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -18931,10 +18931,10 @@
         <v>31</v>
       </c>
       <c r="J214" t="n">
-        <v>36.5</v>
+        <v>33.7</v>
       </c>
       <c r="K214" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -18962,7 +18962,7 @@
       </c>
       <c r="R214" t="inlineStr"/>
       <c r="S214" t="n">
-        <v>5.5</v>
+        <v>2.700000000000003</v>
       </c>
       <c r="T214" t="n">
         <v>33.66666666666666</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-15 19:34:42
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4187,10 +4187,10 @@
         <v>24</v>
       </c>
       <c r="J44" t="n">
-        <v>22.3</v>
+        <v>19.1</v>
       </c>
       <c r="K44" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -4220,7 +4220,7 @@
         <v>28</v>
       </c>
       <c r="S44" t="n">
-        <v>-1.699999999999999</v>
+        <v>-4.899999999999999</v>
       </c>
       <c r="T44" t="n">
         <v>21.1</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K75" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K79" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7479,10 +7479,10 @@
         <v>21</v>
       </c>
       <c r="J82" t="n">
-        <v>21.2</v>
+        <v>20.2</v>
       </c>
       <c r="K82" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -7512,7 +7512,7 @@
         <v>21</v>
       </c>
       <c r="S82" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T82" t="n">
         <v>22.16666666666667</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K86" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K91" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -19103,10 +19103,10 @@
         <v>28</v>
       </c>
       <c r="J216" t="n">
-        <v>28.5</v>
+        <v>27.7</v>
       </c>
       <c r="K216" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L216" t="inlineStr">
         <is>
@@ -19136,7 +19136,7 @@
         <v>28</v>
       </c>
       <c r="S216" t="n">
-        <v>0.5</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T216" t="n">
         <v>28.33333333333333</v>
@@ -19277,10 +19277,10 @@
         <v>21</v>
       </c>
       <c r="J218" t="n">
-        <v>15.3</v>
+        <v>20.5</v>
       </c>
       <c r="K218" t="n">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="L218" t="inlineStr">
         <is>
@@ -19310,7 +19310,7 @@
         <v>21</v>
       </c>
       <c r="S218" t="n">
-        <v>-5.699999999999999</v>
+        <v>-0.5</v>
       </c>
       <c r="T218" t="n">
         <v>18.26666666666667</v>
@@ -19625,10 +19625,10 @@
         <v>28</v>
       </c>
       <c r="J222" t="n">
-        <v>25.6</v>
+        <v>29.8</v>
       </c>
       <c r="K222" t="n">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="L222" t="inlineStr">
         <is>
@@ -19658,7 +19658,7 @@
         <v>28</v>
       </c>
       <c r="S222" t="n">
-        <v>-2.399999999999999</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="T222" t="n">
         <v>25.9</v>
@@ -19712,10 +19712,10 @@
         <v>28</v>
       </c>
       <c r="J223" t="n">
-        <v>26.7</v>
+        <v>27.3</v>
       </c>
       <c r="K223" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="L223" t="inlineStr">
         <is>
@@ -19745,7 +19745,7 @@
         <v>28</v>
       </c>
       <c r="S223" t="n">
-        <v>-1.300000000000001</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T223" t="n">
         <v>28.56666666666667</v>
@@ -19799,10 +19799,10 @@
         <v>21</v>
       </c>
       <c r="J224" t="n">
-        <v>20.3</v>
+        <v>19.5</v>
       </c>
       <c r="K224" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="L224" t="inlineStr">
         <is>
@@ -19832,7 +19832,7 @@
         <v>21</v>
       </c>
       <c r="S224" t="n">
-        <v>-0.6999999999999993</v>
+        <v>-1.5</v>
       </c>
       <c r="T224" t="n">
         <v>20.3</v>
@@ -19886,10 +19886,10 @@
         <v>21</v>
       </c>
       <c r="J225" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="K225" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L225" t="inlineStr">
         <is>
@@ -19919,7 +19919,7 @@
         <v>21</v>
       </c>
       <c r="S225" t="n">
-        <v>1.600000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="T225" t="n">
         <v>21.96666666666667</v>
@@ -19973,10 +19973,10 @@
         <v>28</v>
       </c>
       <c r="J226" t="n">
-        <v>25</v>
+        <v>22.8</v>
       </c>
       <c r="K226" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="L226" t="inlineStr">
         <is>
@@ -20006,7 +20006,7 @@
         <v>28</v>
       </c>
       <c r="S226" t="n">
-        <v>-3</v>
+        <v>-5.199999999999999</v>
       </c>
       <c r="T226" t="n">
         <v>24.76666666666667</v>
@@ -20060,10 +20060,10 @@
         <v>28</v>
       </c>
       <c r="J227" t="n">
-        <v>29.3</v>
+        <v>30.1</v>
       </c>
       <c r="K227" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="L227" t="inlineStr">
         <is>
@@ -20093,7 +20093,7 @@
         <v>28</v>
       </c>
       <c r="S227" t="n">
-        <v>1.300000000000001</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="T227" t="n">
         <v>28.96666666666667</v>
@@ -20147,10 +20147,10 @@
         <v>21</v>
       </c>
       <c r="J228" t="n">
-        <v>22.9</v>
+        <v>21.7</v>
       </c>
       <c r="K228" t="n">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="L228" t="inlineStr">
         <is>
@@ -20180,7 +20180,7 @@
         <v>21</v>
       </c>
       <c r="S228" t="n">
-        <v>1.899999999999999</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T228" t="n">
         <v>21.83333333333333</v>
@@ -20319,10 +20319,10 @@
         <v>21</v>
       </c>
       <c r="J230" t="n">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="K230" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L230" t="inlineStr">
         <is>
@@ -20352,7 +20352,7 @@
         <v>21</v>
       </c>
       <c r="S230" t="n">
-        <v>1.800000000000001</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="T230" t="n">
         <v>21.56666666666667</v>
@@ -20406,10 +20406,10 @@
         <v>28</v>
       </c>
       <c r="J231" t="n">
-        <v>24.5</v>
+        <v>26</v>
       </c>
       <c r="K231" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="L231" t="inlineStr">
         <is>
@@ -20439,7 +20439,7 @@
         <v>28</v>
       </c>
       <c r="S231" t="n">
-        <v>-3.5</v>
+        <v>-2</v>
       </c>
       <c r="T231" t="n">
         <v>25.53333333333333</v>
@@ -20493,10 +20493,10 @@
         <v>28</v>
       </c>
       <c r="J232" t="n">
-        <v>30.9</v>
+        <v>24.9</v>
       </c>
       <c r="K232" t="n">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="L232" t="inlineStr">
         <is>
@@ -20526,7 +20526,7 @@
         <v>28</v>
       </c>
       <c r="S232" t="n">
-        <v>2.899999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T232" t="n">
         <v>27.93333333333333</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-16 07:16:16
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3331,10 +3331,10 @@
         <v>31</v>
       </c>
       <c r="J34" t="n">
-        <v>31.4</v>
+        <v>30</v>
       </c>
       <c r="K34" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1</v>
       </c>
       <c r="T34" t="n">
         <v>30.33333333333333</v>
@@ -7740,10 +7740,10 @@
         <v>21</v>
       </c>
       <c r="J85" t="n">
-        <v>19.3</v>
+        <v>26</v>
       </c>
       <c r="K85" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
         <v>21</v>
       </c>
       <c r="S85" t="n">
-        <v>-1.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="T85" t="n">
         <v>22</v>
@@ -9597,7 +9597,7 @@
         <v>3</v>
       </c>
       <c r="V106" t="n">
-        <v>24.52222222222223</v>
+        <v>24.52222222222222</v>
       </c>
       <c r="W106" t="n">
         <v>17.5</v>
@@ -11904,10 +11904,10 @@
         <v>35</v>
       </c>
       <c r="J133" t="n">
-        <v>29.2</v>
+        <v>36.1</v>
       </c>
       <c r="K133" t="n">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -11937,7 +11937,7 @@
         <v>41</v>
       </c>
       <c r="S133" t="n">
-        <v>-5.800000000000001</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T133" t="n">
         <v>33.9</v>
@@ -12078,10 +12078,10 @@
         <v>31</v>
       </c>
       <c r="J135" t="n">
-        <v>30.5</v>
+        <v>31.9</v>
       </c>
       <c r="K135" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="L135" t="inlineStr">
         <is>
@@ -12109,7 +12109,7 @@
       </c>
       <c r="R135" t="inlineStr"/>
       <c r="S135" t="n">
-        <v>-0.5</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T135" t="n">
         <v>31.23333333333333</v>
@@ -13723,10 +13723,10 @@
         <v>35</v>
       </c>
       <c r="J154" t="n">
-        <v>36.7</v>
+        <v>31.5</v>
       </c>
       <c r="K154" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -13756,7 +13756,7 @@
         <v>41</v>
       </c>
       <c r="S154" t="n">
-        <v>1.700000000000003</v>
+        <v>-3.5</v>
       </c>
       <c r="T154" t="n">
         <v>35.23333333333333</v>
@@ -14504,10 +14504,10 @@
         <v>21</v>
       </c>
       <c r="J163" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="K163" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="L163" t="inlineStr">
         <is>
@@ -14537,7 +14537,7 @@
         <v>21</v>
       </c>
       <c r="S163" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T163" t="n">
         <v>22.96666666666667</v>
@@ -15720,10 +15720,10 @@
         <v>31</v>
       </c>
       <c r="J177" t="n">
-        <v>34</v>
+        <v>26.9</v>
       </c>
       <c r="K177" t="n">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="L177" t="inlineStr">
         <is>
@@ -15751,10 +15751,10 @@
       </c>
       <c r="R177" t="inlineStr"/>
       <c r="S177" t="n">
-        <v>3</v>
+        <v>-4.100000000000001</v>
       </c>
       <c r="T177" t="n">
-        <v>31.93333333333334</v>
+        <v>31.93333333333333</v>
       </c>
       <c r="U177" t="n">
         <v>3</v>
@@ -16153,10 +16153,10 @@
         <v>21</v>
       </c>
       <c r="J182" t="n">
-        <v>22.3</v>
+        <v>20.7</v>
       </c>
       <c r="K182" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="L182" t="inlineStr">
         <is>
@@ -16186,7 +16186,7 @@
         <v>21</v>
       </c>
       <c r="S182" t="n">
-        <v>1.300000000000001</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T182" t="n">
         <v>21.3</v>
@@ -16501,10 +16501,10 @@
         <v>35</v>
       </c>
       <c r="J186" t="n">
-        <v>32.4</v>
+        <v>32.7</v>
       </c>
       <c r="K186" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L186" t="inlineStr">
         <is>
@@ -16534,7 +16534,7 @@
         <v>41</v>
       </c>
       <c r="S186" t="n">
-        <v>-2.600000000000001</v>
+        <v>-2.299999999999997</v>
       </c>
       <c r="T186" t="n">
         <v>32.26666666666667</v>
@@ -19973,10 +19973,10 @@
         <v>28</v>
       </c>
       <c r="J226" t="n">
-        <v>22.8</v>
+        <v>25</v>
       </c>
       <c r="K226" t="n">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="L226" t="inlineStr">
         <is>
@@ -20006,7 +20006,7 @@
         <v>28</v>
       </c>
       <c r="S226" t="n">
-        <v>-5.199999999999999</v>
+        <v>-3</v>
       </c>
       <c r="T226" t="n">
         <v>24.76666666666667</v>
@@ -20752,10 +20752,10 @@
         <v>31</v>
       </c>
       <c r="J235" t="n">
-        <v>31.5</v>
+        <v>28.1</v>
       </c>
       <c r="K235" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -20783,7 +20783,7 @@
       </c>
       <c r="R235" t="inlineStr"/>
       <c r="S235" t="n">
-        <v>0.5</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="T235" t="n">
         <v>30.6</v>
@@ -21531,10 +21531,10 @@
         <v>21</v>
       </c>
       <c r="J244" t="n">
-        <v>17.3</v>
+        <v>19</v>
       </c>
       <c r="K244" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="L244" t="inlineStr">
         <is>
@@ -21562,7 +21562,7 @@
       </c>
       <c r="R244" t="inlineStr"/>
       <c r="S244" t="n">
-        <v>-3.699999999999999</v>
+        <v>-2</v>
       </c>
       <c r="T244" t="n">
         <v>19.3</v>
@@ -22130,10 +22130,10 @@
         <v>21</v>
       </c>
       <c r="J251" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="K251" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="L251" t="inlineStr">
         <is>
@@ -22161,7 +22161,7 @@
       </c>
       <c r="R251" t="inlineStr"/>
       <c r="S251" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="T251" t="n">
         <v>21.8</v>
@@ -22302,10 +22302,10 @@
         <v>21</v>
       </c>
       <c r="J253" t="n">
-        <v>16.6</v>
+        <v>42.6</v>
       </c>
       <c r="K253" t="n">
-        <v>79</v>
+        <v>203</v>
       </c>
       <c r="L253" t="inlineStr">
         <is>
@@ -22335,7 +22335,7 @@
         <v>21</v>
       </c>
       <c r="S253" t="n">
-        <v>-4.399999999999999</v>
+        <v>21.6</v>
       </c>
       <c r="T253" t="n">
         <v>36.33333333333334</v>
@@ -22389,10 +22389,10 @@
         <v>28</v>
       </c>
       <c r="J254" t="n">
-        <v>26.8</v>
+        <v>27.7</v>
       </c>
       <c r="K254" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L254" t="inlineStr">
         <is>
@@ -22422,7 +22422,7 @@
         <v>28</v>
       </c>
       <c r="S254" t="n">
-        <v>-1.199999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T254" t="n">
         <v>27.16666666666667</v>
@@ -22476,10 +22476,10 @@
         <v>28</v>
       </c>
       <c r="J255" t="n">
-        <v>25.6</v>
+        <v>22.7</v>
       </c>
       <c r="K255" t="n">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="L255" t="inlineStr">
         <is>
@@ -22509,7 +22509,7 @@
         <v>28</v>
       </c>
       <c r="S255" t="n">
-        <v>-2.399999999999999</v>
+        <v>-5.300000000000001</v>
       </c>
       <c r="T255" t="n">
         <v>24.9</v>
@@ -23259,10 +23259,10 @@
         <v>28</v>
       </c>
       <c r="J264" t="n">
-        <v>29.9</v>
+        <v>32.3</v>
       </c>
       <c r="K264" t="n">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="L264" t="inlineStr">
         <is>
@@ -23292,7 +23292,7 @@
         <v>28</v>
       </c>
       <c r="S264" t="n">
-        <v>1.899999999999999</v>
+        <v>4.299999999999997</v>
       </c>
       <c r="T264" t="n">
         <v>28.53333333333333</v>
@@ -23431,10 +23431,10 @@
         <v>28</v>
       </c>
       <c r="J266" t="n">
-        <v>27</v>
+        <v>28.1</v>
       </c>
       <c r="K266" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L266" t="inlineStr">
         <is>
@@ -23464,7 +23464,7 @@
         <v>28</v>
       </c>
       <c r="S266" t="n">
-        <v>-1</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T266" t="n">
         <v>26.96666666666667</v>
@@ -23732,7 +23732,7 @@
         <v>3</v>
       </c>
       <c r="V269" t="n">
-        <v>28.15555555555555</v>
+        <v>28.15555555555556</v>
       </c>
       <c r="W269" t="n">
         <v>24.5</v>
@@ -23777,10 +23777,10 @@
         <v>28</v>
       </c>
       <c r="J270" t="n">
-        <v>26.1</v>
+        <v>27.3</v>
       </c>
       <c r="K270" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="L270" t="inlineStr">
         <is>
@@ -23810,7 +23810,7 @@
         <v>28</v>
       </c>
       <c r="S270" t="n">
-        <v>-1.899999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T270" t="n">
         <v>27.16666666666667</v>
@@ -24687,7 +24687,7 @@
         <v>3</v>
       </c>
       <c r="V280" t="n">
-        <v>24.36666666666666</v>
+        <v>24.36666666666667</v>
       </c>
       <c r="W280" t="n">
         <v>17.5</v>
@@ -24993,10 +24993,10 @@
         <v>21</v>
       </c>
       <c r="J284" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="K284" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L284" t="inlineStr">
         <is>
@@ -25026,7 +25026,7 @@
         <v>21</v>
       </c>
       <c r="S284" t="n">
-        <v>-0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="T284" t="n">
         <v>21.03333333333333</v>
@@ -25080,10 +25080,10 @@
         <v>21</v>
       </c>
       <c r="J285" t="n">
-        <v>18.6</v>
+        <v>18.2</v>
       </c>
       <c r="K285" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L285" t="inlineStr">
         <is>
@@ -25113,7 +25113,7 @@
         <v>21</v>
       </c>
       <c r="S285" t="n">
-        <v>-2.399999999999999</v>
+        <v>-2.800000000000001</v>
       </c>
       <c r="T285" t="n">
         <v>18.23333333333333</v>
@@ -25167,10 +25167,10 @@
         <v>21</v>
       </c>
       <c r="J286" t="n">
-        <v>18.4</v>
+        <v>20.2</v>
       </c>
       <c r="K286" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="L286" t="inlineStr">
         <is>
@@ -25200,16 +25200,16 @@
         <v>21</v>
       </c>
       <c r="S286" t="n">
-        <v>-2.600000000000001</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T286" t="n">
-        <v>19.86666666666666</v>
+        <v>19.86666666666667</v>
       </c>
       <c r="U286" t="n">
         <v>3</v>
       </c>
       <c r="V286" t="n">
-        <v>21.74444444444444</v>
+        <v>21.74444444444445</v>
       </c>
       <c r="W286" t="n">
         <v>17.5</v>
@@ -25944,10 +25944,10 @@
         <v>21</v>
       </c>
       <c r="J295" t="n">
-        <v>20.3</v>
+        <v>21.9</v>
       </c>
       <c r="K295" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="L295" t="inlineStr">
         <is>
@@ -25977,7 +25977,7 @@
         <v>21</v>
       </c>
       <c r="S295" t="n">
-        <v>-0.6999999999999993</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T295" t="n">
         <v>20.9</v>
@@ -26031,10 +26031,10 @@
         <v>21</v>
       </c>
       <c r="J296" t="n">
-        <v>20.1</v>
+        <v>20.8</v>
       </c>
       <c r="K296" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L296" t="inlineStr">
         <is>
@@ -26064,7 +26064,7 @@
         <v>21</v>
       </c>
       <c r="S296" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T296" t="n">
         <v>20.3</v>
@@ -26118,10 +26118,10 @@
         <v>21</v>
       </c>
       <c r="J297" t="n">
-        <v>18</v>
+        <v>21.1</v>
       </c>
       <c r="K297" t="n">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="L297" t="inlineStr">
         <is>
@@ -26151,7 +26151,7 @@
         <v>21</v>
       </c>
       <c r="S297" t="n">
-        <v>-3</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T297" t="n">
         <v>19.53333333333333</v>
@@ -26812,10 +26812,10 @@
         <v>21</v>
       </c>
       <c r="J305" t="n">
-        <v>20.4</v>
+        <v>21.8</v>
       </c>
       <c r="K305" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="L305" t="inlineStr">
         <is>
@@ -26845,7 +26845,7 @@
         <v>21</v>
       </c>
       <c r="S305" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.8000000000000007</v>
       </c>
       <c r="T305" t="n">
         <v>20.76666666666667</v>
@@ -26899,10 +26899,10 @@
         <v>21</v>
       </c>
       <c r="J306" t="n">
-        <v>19.4</v>
+        <v>22</v>
       </c>
       <c r="K306" t="n">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -26932,7 +26932,7 @@
         <v>21</v>
       </c>
       <c r="S306" t="n">
-        <v>-1.600000000000001</v>
+        <v>1</v>
       </c>
       <c r="T306" t="n">
         <v>20.8</v>
@@ -26986,10 +26986,10 @@
         <v>21</v>
       </c>
       <c r="J307" t="n">
-        <v>19.6</v>
+        <v>20.7</v>
       </c>
       <c r="K307" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="L307" t="inlineStr">
         <is>
@@ -27019,7 +27019,7 @@
         <v>21</v>
       </c>
       <c r="S307" t="n">
-        <v>-1.399999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T307" t="n">
         <v>20.23333333333333</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>
@@ -31591,10 +31591,10 @@
         <v>24.5</v>
       </c>
       <c r="J360" t="n">
-        <v>25.1</v>
+        <v>28.6</v>
       </c>
       <c r="K360" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31624,7 +31624,7 @@
         <v>28</v>
       </c>
       <c r="S360" t="n">
-        <v>0.6000000000000014</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T360" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-16 20:48:43
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4707,10 +4707,10 @@
         <v>24</v>
       </c>
       <c r="J50" t="n">
-        <v>26.2</v>
+        <v>23.6</v>
       </c>
       <c r="K50" t="n">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -4740,7 +4740,7 @@
         <v>28</v>
       </c>
       <c r="S50" t="n">
-        <v>2.199999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T50" t="n">
         <v>26.56666666666666</v>
@@ -5223,10 +5223,10 @@
         <v>24</v>
       </c>
       <c r="J56" t="n">
-        <v>20.8</v>
+        <v>22.4</v>
       </c>
       <c r="K56" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
         <v>28</v>
       </c>
       <c r="S56" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T56" t="n">
         <v>21.53333333333333</v>
@@ -5656,10 +5656,10 @@
         <v>24</v>
       </c>
       <c r="J61" t="n">
-        <v>16.6</v>
+        <v>27.2</v>
       </c>
       <c r="K61" t="n">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -5689,7 +5689,7 @@
         <v>28</v>
       </c>
       <c r="S61" t="n">
-        <v>-7.399999999999999</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="T61" t="n">
         <v>23.4</v>
@@ -6352,10 +6352,10 @@
         <v>21</v>
       </c>
       <c r="J69" t="n">
-        <v>17.9</v>
+        <v>21.1</v>
       </c>
       <c r="K69" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -6385,7 +6385,7 @@
         <v>21</v>
       </c>
       <c r="S69" t="n">
-        <v>-3.100000000000001</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T69" t="n">
         <v>18.86666666666667</v>
@@ -7999,10 +7999,10 @@
         <v>35</v>
       </c>
       <c r="J88" t="n">
-        <v>25.3</v>
+        <v>36.5</v>
       </c>
       <c r="K88" t="n">
-        <v>72</v>
+        <v>104</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
         <v>41</v>
       </c>
       <c r="S88" t="n">
-        <v>-9.699999999999999</v>
+        <v>1.5</v>
       </c>
       <c r="T88" t="n">
         <v>33.1</v>
@@ -9816,10 +9816,10 @@
         <v>35</v>
       </c>
       <c r="J109" t="n">
-        <v>29.6</v>
+        <v>27.1</v>
       </c>
       <c r="K109" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -9849,7 +9849,7 @@
         <v>41</v>
       </c>
       <c r="S109" t="n">
-        <v>-5.399999999999999</v>
+        <v>-7.899999999999999</v>
       </c>
       <c r="T109" t="n">
         <v>27.33333333333333</v>
@@ -10251,10 +10251,10 @@
         <v>28</v>
       </c>
       <c r="J114" t="n">
-        <v>29.7</v>
+        <v>32.7</v>
       </c>
       <c r="K114" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -10284,7 +10284,7 @@
         <v>28</v>
       </c>
       <c r="S114" t="n">
-        <v>1.699999999999999</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="T114" t="n">
         <v>29.6</v>
@@ -11208,10 +11208,10 @@
         <v>35</v>
       </c>
       <c r="J125" t="n">
-        <v>30.5</v>
+        <v>35.4</v>
       </c>
       <c r="K125" t="n">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -11241,7 +11241,7 @@
         <v>41</v>
       </c>
       <c r="S125" t="n">
-        <v>-4.5</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T125" t="n">
         <v>34.13333333333333</v>
@@ -16501,10 +16501,10 @@
         <v>35</v>
       </c>
       <c r="J186" t="n">
-        <v>32.4</v>
+        <v>32.7</v>
       </c>
       <c r="K186" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L186" t="inlineStr">
         <is>
@@ -16534,7 +16534,7 @@
         <v>41</v>
       </c>
       <c r="S186" t="n">
-        <v>-2.600000000000001</v>
+        <v>-2.299999999999997</v>
       </c>
       <c r="T186" t="n">
         <v>32.26666666666667</v>
@@ -16675,10 +16675,10 @@
         <v>35</v>
       </c>
       <c r="J188" t="n">
-        <v>30.3</v>
+        <v>26.1</v>
       </c>
       <c r="K188" t="n">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="L188" t="inlineStr">
         <is>
@@ -16708,7 +16708,7 @@
         <v>41</v>
       </c>
       <c r="S188" t="n">
-        <v>-4.699999999999999</v>
+        <v>-8.899999999999999</v>
       </c>
       <c r="T188" t="n">
         <v>33.26666666666667</v>
@@ -18409,10 +18409,10 @@
         <v>28</v>
       </c>
       <c r="J208" t="n">
-        <v>30.7</v>
+        <v>26.9</v>
       </c>
       <c r="K208" t="n">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="L208" t="inlineStr">
         <is>
@@ -18442,7 +18442,7 @@
         <v>28</v>
       </c>
       <c r="S208" t="n">
-        <v>2.699999999999999</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="T208" t="n">
         <v>28.46666666666667</v>
@@ -18670,10 +18670,10 @@
         <v>21</v>
       </c>
       <c r="J211" t="n">
-        <v>20.5</v>
+        <v>22.8</v>
       </c>
       <c r="K211" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="L211" t="inlineStr">
         <is>
@@ -18703,7 +18703,7 @@
         <v>21</v>
       </c>
       <c r="S211" t="n">
-        <v>-0.5</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="T211" t="n">
         <v>22.36666666666666</v>
@@ -20406,10 +20406,10 @@
         <v>28</v>
       </c>
       <c r="J231" t="n">
-        <v>26</v>
+        <v>24.5</v>
       </c>
       <c r="K231" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="L231" t="inlineStr">
         <is>
@@ -20439,7 +20439,7 @@
         <v>28</v>
       </c>
       <c r="S231" t="n">
-        <v>-2</v>
+        <v>-3.5</v>
       </c>
       <c r="T231" t="n">
         <v>25.53333333333333</v>
@@ -20837,10 +20837,10 @@
         <v>24</v>
       </c>
       <c r="J236" t="n">
-        <v>25.9</v>
+        <v>23.6</v>
       </c>
       <c r="K236" t="n">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="L236" t="inlineStr">
         <is>
@@ -20870,7 +20870,7 @@
         <v>28</v>
       </c>
       <c r="S236" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T236" t="n">
         <v>25.13333333333334</v>
@@ -21183,10 +21183,10 @@
         <v>42</v>
       </c>
       <c r="J240" t="n">
-        <v>50.4</v>
+        <v>15.9</v>
       </c>
       <c r="K240" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
       <c r="L240" t="inlineStr">
         <is>
@@ -21216,7 +21216,7 @@
         <v>48</v>
       </c>
       <c r="S240" t="n">
-        <v>8.399999999999999</v>
+        <v>-26.1</v>
       </c>
       <c r="T240" t="n">
         <v>39.6</v>
@@ -25859,10 +25859,10 @@
         <v>21</v>
       </c>
       <c r="J294" t="n">
-        <v>19.8</v>
+        <v>18.9</v>
       </c>
       <c r="K294" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="L294" t="inlineStr">
         <is>
@@ -25892,7 +25892,7 @@
         <v>21</v>
       </c>
       <c r="S294" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="T294" t="n">
         <v>19</v>
@@ -27245,10 +27245,10 @@
         <v>24.5</v>
       </c>
       <c r="J310" t="n">
-        <v>23.9</v>
+        <v>25.1</v>
       </c>
       <c r="K310" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -27278,7 +27278,7 @@
         <v>28</v>
       </c>
       <c r="S310" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T310" t="n">
         <v>25.13333333333334</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>
@@ -31678,10 +31678,10 @@
         <v>21</v>
       </c>
       <c r="J361" t="n">
-        <v>20.2</v>
+        <v>21.1</v>
       </c>
       <c r="K361" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L361" t="inlineStr">
         <is>
@@ -31711,7 +31711,7 @@
         <v>21</v>
       </c>
       <c r="S361" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T361" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-16 21:07:12
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4707,10 +4707,10 @@
         <v>24</v>
       </c>
       <c r="J50" t="n">
-        <v>23.6</v>
+        <v>26.2</v>
       </c>
       <c r="K50" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -4740,7 +4740,7 @@
         <v>28</v>
       </c>
       <c r="S50" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="T50" t="n">
         <v>26.56666666666666</v>
@@ -5223,10 +5223,10 @@
         <v>24</v>
       </c>
       <c r="J56" t="n">
-        <v>22.4</v>
+        <v>20.8</v>
       </c>
       <c r="K56" t="n">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
         <v>28</v>
       </c>
       <c r="S56" t="n">
-        <v>-1.600000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T56" t="n">
         <v>21.53333333333333</v>
@@ -5656,10 +5656,10 @@
         <v>24</v>
       </c>
       <c r="J61" t="n">
-        <v>27.2</v>
+        <v>16.6</v>
       </c>
       <c r="K61" t="n">
-        <v>113</v>
+        <v>69</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -5689,7 +5689,7 @@
         <v>28</v>
       </c>
       <c r="S61" t="n">
-        <v>3.199999999999999</v>
+        <v>-7.399999999999999</v>
       </c>
       <c r="T61" t="n">
         <v>23.4</v>
@@ -6352,10 +6352,10 @@
         <v>21</v>
       </c>
       <c r="J69" t="n">
-        <v>21.1</v>
+        <v>17.9</v>
       </c>
       <c r="K69" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -6385,7 +6385,7 @@
         <v>21</v>
       </c>
       <c r="S69" t="n">
-        <v>0.1000000000000014</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T69" t="n">
         <v>18.86666666666667</v>
@@ -6526,10 +6526,10 @@
         <v>21</v>
       </c>
       <c r="J71" t="n">
-        <v>19.5</v>
+        <v>23.1</v>
       </c>
       <c r="K71" t="n">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -6559,7 +6559,7 @@
         <v>21</v>
       </c>
       <c r="S71" t="n">
-        <v>-1.5</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="T71" t="n">
         <v>20.9</v>
@@ -9903,10 +9903,10 @@
         <v>35</v>
       </c>
       <c r="J110" t="n">
-        <v>49.1</v>
+        <v>31.4</v>
       </c>
       <c r="K110" t="n">
-        <v>140</v>
+        <v>90</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -9936,7 +9936,7 @@
         <v>41</v>
       </c>
       <c r="S110" t="n">
-        <v>14.1</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="T110" t="n">
         <v>43.96666666666667</v>
@@ -9990,10 +9990,10 @@
         <v>35</v>
       </c>
       <c r="J111" t="n">
-        <v>27.3</v>
+        <v>54.5</v>
       </c>
       <c r="K111" t="n">
-        <v>78</v>
+        <v>156</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
@@ -10023,16 +10023,16 @@
         <v>41</v>
       </c>
       <c r="S111" t="n">
-        <v>-7.699999999999999</v>
+        <v>19.5</v>
       </c>
       <c r="T111" t="n">
-        <v>44.9</v>
+        <v>44.90000000000001</v>
       </c>
       <c r="U111" t="n">
         <v>3</v>
       </c>
       <c r="V111" t="n">
-        <v>41.74444444444444</v>
+        <v>41.74444444444445</v>
       </c>
       <c r="W111" t="n">
         <v>31.5</v>
@@ -10077,10 +10077,10 @@
         <v>21</v>
       </c>
       <c r="J112" t="n">
-        <v>24.3</v>
+        <v>19.9</v>
       </c>
       <c r="K112" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -10110,16 +10110,16 @@
         <v>21</v>
       </c>
       <c r="S112" t="n">
-        <v>3.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="T112" t="n">
-        <v>22.56666666666666</v>
+        <v>22.56666666666667</v>
       </c>
       <c r="U112" t="n">
         <v>3</v>
       </c>
       <c r="V112" t="n">
-        <v>36.05555555555555</v>
+        <v>36.05555555555556</v>
       </c>
       <c r="W112" t="n">
         <v>17.5</v>
@@ -10860,10 +10860,10 @@
         <v>28</v>
       </c>
       <c r="J121" t="n">
-        <v>31.6</v>
+        <v>33.5</v>
       </c>
       <c r="K121" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -10893,7 +10893,7 @@
         <v>28</v>
       </c>
       <c r="S121" t="n">
-        <v>3.600000000000001</v>
+        <v>5.5</v>
       </c>
       <c r="T121" t="n">
         <v>30.83333333333333</v>
@@ -11208,10 +11208,10 @@
         <v>35</v>
       </c>
       <c r="J125" t="n">
-        <v>35.4</v>
+        <v>30.5</v>
       </c>
       <c r="K125" t="n">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -11241,7 +11241,7 @@
         <v>41</v>
       </c>
       <c r="S125" t="n">
-        <v>0.3999999999999986</v>
+        <v>-4.5</v>
       </c>
       <c r="T125" t="n">
         <v>34.13333333333333</v>
@@ -20837,10 +20837,10 @@
         <v>24</v>
       </c>
       <c r="J236" t="n">
-        <v>23.6</v>
+        <v>25.9</v>
       </c>
       <c r="K236" t="n">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="L236" t="inlineStr">
         <is>
@@ -20870,7 +20870,7 @@
         <v>28</v>
       </c>
       <c r="S236" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T236" t="n">
         <v>25.13333333333334</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="K321" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="K329" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="K351" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>
@@ -31419,10 +31419,10 @@
         <v>24.5</v>
       </c>
       <c r="J358" t="n">
-        <v>22.7</v>
+        <v>29.1</v>
       </c>
       <c r="K358" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="L358" t="inlineStr">
         <is>
@@ -31452,7 +31452,7 @@
         <v>28</v>
       </c>
       <c r="S358" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="T358" t="n">
         <v>25.3</v>
@@ -31591,10 +31591,10 @@
         <v>24.5</v>
       </c>
       <c r="J360" t="n">
-        <v>28.6</v>
+        <v>25.1</v>
       </c>
       <c r="K360" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31624,7 +31624,7 @@
         <v>28</v>
       </c>
       <c r="S360" t="n">
-        <v>4.100000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T360" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-16 22:42:01
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3930,10 +3930,10 @@
         <v>31</v>
       </c>
       <c r="J41" t="n">
-        <v>29.7</v>
+        <v>32</v>
       </c>
       <c r="K41" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="n">
-        <v>-1.300000000000001</v>
+        <v>1</v>
       </c>
       <c r="T41" t="n">
         <v>30.33333333333333</v>
@@ -5223,10 +5223,10 @@
         <v>24</v>
       </c>
       <c r="J56" t="n">
-        <v>20.8</v>
+        <v>22.4</v>
       </c>
       <c r="K56" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
         <v>28</v>
       </c>
       <c r="S56" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T56" t="n">
         <v>21.53333333333333</v>
@@ -6526,10 +6526,10 @@
         <v>21</v>
       </c>
       <c r="J71" t="n">
-        <v>23.1</v>
+        <v>19.5</v>
       </c>
       <c r="K71" t="n">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -6559,7 +6559,7 @@
         <v>21</v>
       </c>
       <c r="S71" t="n">
-        <v>2.100000000000001</v>
+        <v>-1.5</v>
       </c>
       <c r="T71" t="n">
         <v>20.9</v>
@@ -6959,10 +6959,10 @@
         <v>28</v>
       </c>
       <c r="J76" t="n">
-        <v>24.1</v>
+        <v>27.3</v>
       </c>
       <c r="K76" t="n">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -6992,7 +6992,7 @@
         <v>28</v>
       </c>
       <c r="S76" t="n">
-        <v>-3.899999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T76" t="n">
         <v>25.33333333333333</v>
@@ -9903,10 +9903,10 @@
         <v>35</v>
       </c>
       <c r="J110" t="n">
-        <v>31.4</v>
+        <v>49.1</v>
       </c>
       <c r="K110" t="n">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -9936,7 +9936,7 @@
         <v>41</v>
       </c>
       <c r="S110" t="n">
-        <v>-3.600000000000001</v>
+        <v>14.1</v>
       </c>
       <c r="T110" t="n">
         <v>43.96666666666667</v>
@@ -9990,10 +9990,10 @@
         <v>35</v>
       </c>
       <c r="J111" t="n">
-        <v>54.5</v>
+        <v>27.3</v>
       </c>
       <c r="K111" t="n">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
@@ -10023,16 +10023,16 @@
         <v>41</v>
       </c>
       <c r="S111" t="n">
-        <v>19.5</v>
+        <v>-7.699999999999999</v>
       </c>
       <c r="T111" t="n">
-        <v>44.90000000000001</v>
+        <v>44.9</v>
       </c>
       <c r="U111" t="n">
         <v>3</v>
       </c>
       <c r="V111" t="n">
-        <v>41.74444444444445</v>
+        <v>41.74444444444444</v>
       </c>
       <c r="W111" t="n">
         <v>31.5</v>
@@ -10077,10 +10077,10 @@
         <v>21</v>
       </c>
       <c r="J112" t="n">
-        <v>19.9</v>
+        <v>24.3</v>
       </c>
       <c r="K112" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -10110,16 +10110,16 @@
         <v>21</v>
       </c>
       <c r="S112" t="n">
-        <v>-1.100000000000001</v>
+        <v>3.300000000000001</v>
       </c>
       <c r="T112" t="n">
-        <v>22.56666666666667</v>
+        <v>22.56666666666666</v>
       </c>
       <c r="U112" t="n">
         <v>3</v>
       </c>
       <c r="V112" t="n">
-        <v>36.05555555555556</v>
+        <v>36.05555555555555</v>
       </c>
       <c r="W112" t="n">
         <v>17.5</v>
@@ -15111,10 +15111,10 @@
         <v>28</v>
       </c>
       <c r="J170" t="n">
-        <v>27</v>
+        <v>24.8</v>
       </c>
       <c r="K170" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
@@ -15144,7 +15144,7 @@
         <v>28</v>
       </c>
       <c r="S170" t="n">
-        <v>-1</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T170" t="n">
         <v>26.4</v>
@@ -18235,10 +18235,10 @@
         <v>28</v>
       </c>
       <c r="J206" t="n">
-        <v>27.7</v>
+        <v>28.9</v>
       </c>
       <c r="K206" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="L206" t="inlineStr">
         <is>
@@ -18268,7 +18268,7 @@
         <v>28</v>
       </c>
       <c r="S206" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T206" t="n">
         <v>28.4</v>
@@ -19538,10 +19538,10 @@
         <v>28</v>
       </c>
       <c r="J221" t="n">
-        <v>14.6</v>
+        <v>27.2</v>
       </c>
       <c r="K221" t="n">
-        <v>52</v>
+        <v>97</v>
       </c>
       <c r="L221" t="inlineStr">
         <is>
@@ -19571,7 +19571,7 @@
         <v>28</v>
       </c>
       <c r="S221" t="n">
-        <v>-13.4</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T221" t="n">
         <v>23.53333333333333</v>
@@ -20060,10 +20060,10 @@
         <v>28</v>
       </c>
       <c r="J227" t="n">
-        <v>29.3</v>
+        <v>27.5</v>
       </c>
       <c r="K227" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="L227" t="inlineStr">
         <is>
@@ -20093,7 +20093,7 @@
         <v>28</v>
       </c>
       <c r="S227" t="n">
-        <v>1.300000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="T227" t="n">
         <v>28.96666666666667</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -29942,10 +29942,10 @@
         <v>24.5</v>
       </c>
       <c r="J341" t="n">
-        <v>26.3</v>
+        <v>28.4</v>
       </c>
       <c r="K341" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="L341" t="inlineStr">
         <is>
@@ -29975,7 +29975,7 @@
         <v>28</v>
       </c>
       <c r="S341" t="n">
-        <v>1.800000000000001</v>
+        <v>3.899999999999999</v>
       </c>
       <c r="T341" t="n">
         <v>26.36666666666666</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>
@@ -31419,10 +31419,10 @@
         <v>24.5</v>
       </c>
       <c r="J358" t="n">
-        <v>29.1</v>
+        <v>22.7</v>
       </c>
       <c r="K358" t="n">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="L358" t="inlineStr">
         <is>
@@ -31452,7 +31452,7 @@
         <v>28</v>
       </c>
       <c r="S358" t="n">
-        <v>4.600000000000001</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="T358" t="n">
         <v>25.3</v>
@@ -31591,10 +31591,10 @@
         <v>24.5</v>
       </c>
       <c r="J360" t="n">
-        <v>25.1</v>
+        <v>28.6</v>
       </c>
       <c r="K360" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31624,7 +31624,7 @@
         <v>28</v>
       </c>
       <c r="S360" t="n">
-        <v>0.6000000000000014</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T360" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-17 07:12:24
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3244,10 +3244,10 @@
         <v>28</v>
       </c>
       <c r="J33" t="n">
-        <v>26.9</v>
+        <v>27.1</v>
       </c>
       <c r="K33" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -3277,7 +3277,7 @@
         <v>28</v>
       </c>
       <c r="S33" t="n">
-        <v>-1.100000000000001</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T33" t="n">
         <v>27.23333333333333</v>
@@ -3331,10 +3331,10 @@
         <v>31</v>
       </c>
       <c r="J34" t="n">
-        <v>30</v>
+        <v>31.4</v>
       </c>
       <c r="K34" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="n">
-        <v>-1</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T34" t="n">
         <v>30.33333333333333</v>
@@ -4879,10 +4879,10 @@
         <v>31</v>
       </c>
       <c r="J52" t="n">
-        <v>30.5</v>
+        <v>38.5</v>
       </c>
       <c r="K52" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="n">
-        <v>-0.5</v>
+        <v>7.5</v>
       </c>
       <c r="T52" t="n">
         <v>35.86666666666667</v>
@@ -4964,10 +4964,10 @@
         <v>24</v>
       </c>
       <c r="J53" t="n">
-        <v>25.3</v>
+        <v>22.8</v>
       </c>
       <c r="K53" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
         <v>28</v>
       </c>
       <c r="S53" t="n">
-        <v>1.300000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T53" t="n">
         <v>24.6</v>
@@ -5051,10 +5051,10 @@
         <v>24</v>
       </c>
       <c r="J54" t="n">
-        <v>25</v>
+        <v>21.2</v>
       </c>
       <c r="K54" t="n">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -5084,7 +5084,7 @@
         <v>28</v>
       </c>
       <c r="S54" t="n">
-        <v>1</v>
+        <v>-2.800000000000001</v>
       </c>
       <c r="T54" t="n">
         <v>22.7</v>
@@ -5138,10 +5138,10 @@
         <v>31</v>
       </c>
       <c r="J55" t="n">
-        <v>37.1</v>
+        <v>18.8</v>
       </c>
       <c r="K55" t="n">
-        <v>120</v>
+        <v>61</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="n">
-        <v>6.100000000000001</v>
+        <v>-12.2</v>
       </c>
       <c r="T55" t="n">
         <v>31.73333333333333</v>
@@ -5223,10 +5223,10 @@
         <v>24</v>
       </c>
       <c r="J56" t="n">
-        <v>22.4</v>
+        <v>20.8</v>
       </c>
       <c r="K56" t="n">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -5256,7 +5256,7 @@
         <v>28</v>
       </c>
       <c r="S56" t="n">
-        <v>-1.600000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T56" t="n">
         <v>21.53333333333333</v>
@@ -5310,10 +5310,10 @@
         <v>24</v>
       </c>
       <c r="J57" t="n">
-        <v>15.3</v>
+        <v>25.5</v>
       </c>
       <c r="K57" t="n">
-        <v>64</v>
+        <v>106</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -5343,7 +5343,7 @@
         <v>28</v>
       </c>
       <c r="S57" t="n">
-        <v>-8.699999999999999</v>
+        <v>1.5</v>
       </c>
       <c r="T57" t="n">
         <v>22.46666666666667</v>
@@ -5397,10 +5397,10 @@
         <v>31</v>
       </c>
       <c r="J58" t="n">
-        <v>24.8</v>
+        <v>31.4</v>
       </c>
       <c r="K58" t="n">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
       </c>
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="n">
-        <v>-6.199999999999999</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T58" t="n">
-        <v>30.66666666666667</v>
+        <v>30.66666666666666</v>
       </c>
       <c r="U58" t="n">
         <v>3</v>
@@ -5482,10 +5482,10 @@
         <v>24</v>
       </c>
       <c r="J59" t="n">
-        <v>24.7</v>
+        <v>22.1</v>
       </c>
       <c r="K59" t="n">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
         <v>28</v>
       </c>
       <c r="S59" t="n">
-        <v>0.6999999999999993</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="T59" t="n">
         <v>23.8</v>
@@ -5569,10 +5569,10 @@
         <v>24</v>
       </c>
       <c r="J60" t="n">
-        <v>25.9</v>
+        <v>23.1</v>
       </c>
       <c r="K60" t="n">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -5602,7 +5602,7 @@
         <v>28</v>
       </c>
       <c r="S60" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T60" t="n">
         <v>24.1</v>
@@ -5656,10 +5656,10 @@
         <v>24</v>
       </c>
       <c r="J61" t="n">
-        <v>26.4</v>
+        <v>16.6</v>
       </c>
       <c r="K61" t="n">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -5689,7 +5689,7 @@
         <v>28</v>
       </c>
       <c r="S61" t="n">
-        <v>2.399999999999999</v>
+        <v>-7.399999999999999</v>
       </c>
       <c r="T61" t="n">
         <v>23.4</v>
@@ -5743,10 +5743,10 @@
         <v>24</v>
       </c>
       <c r="J62" t="n">
-        <v>23.4</v>
+        <v>25.7</v>
       </c>
       <c r="K62" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -5776,7 +5776,7 @@
         <v>28</v>
       </c>
       <c r="S62" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="T62" t="n">
         <v>24.46666666666667</v>
@@ -5830,10 +5830,10 @@
         <v>28</v>
       </c>
       <c r="J63" t="n">
-        <v>31.6</v>
+        <v>30.4</v>
       </c>
       <c r="K63" t="n">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
@@ -5863,7 +5863,7 @@
         <v>28</v>
       </c>
       <c r="S63" t="n">
-        <v>3.600000000000001</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T63" t="n">
         <v>29.86666666666666</v>
@@ -5917,10 +5917,10 @@
         <v>28</v>
       </c>
       <c r="J64" t="n">
-        <v>29</v>
+        <v>30.5</v>
       </c>
       <c r="K64" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -5950,7 +5950,7 @@
         <v>28</v>
       </c>
       <c r="S64" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="T64" t="n">
         <v>29.13333333333334</v>
@@ -6307,7 +6307,7 @@
         <v>3</v>
       </c>
       <c r="V68" t="n">
-        <v>37.02962962962962</v>
+        <v>37.02962962962963</v>
       </c>
       <c r="W68" t="n">
         <v>31.5</v>
@@ -6481,7 +6481,7 @@
         <v>3</v>
       </c>
       <c r="V70" t="n">
-        <v>38.42962962962962</v>
+        <v>38.42962962962963</v>
       </c>
       <c r="W70" t="n">
         <v>31.5</v>
@@ -6700,10 +6700,10 @@
         <v>35</v>
       </c>
       <c r="J73" t="n">
-        <v>40.8</v>
+        <v>33.5</v>
       </c>
       <c r="K73" t="n">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -6733,10 +6733,10 @@
         <v>41</v>
       </c>
       <c r="S73" t="n">
-        <v>5.799999999999997</v>
+        <v>-1.5</v>
       </c>
       <c r="T73" t="n">
-        <v>37.56666666666666</v>
+        <v>37.56666666666667</v>
       </c>
       <c r="U73" t="n">
         <v>3</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="K75" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="K79" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="K86" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8086,10 +8086,10 @@
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>31.4</v>
+        <v>36.7</v>
       </c>
       <c r="K89" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8119,7 +8119,7 @@
         <v>41</v>
       </c>
       <c r="S89" t="n">
-        <v>-3.600000000000001</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T89" t="n">
         <v>35.73333333333333</v>
@@ -8128,7 +8128,7 @@
         <v>3</v>
       </c>
       <c r="V89" t="n">
-        <v>35.86296296296297</v>
+        <v>35.86296296296296</v>
       </c>
       <c r="W89" t="n">
         <v>31.5</v>
@@ -8173,10 +8173,10 @@
         <v>35</v>
       </c>
       <c r="J90" t="n">
-        <v>40.3</v>
+        <v>39.8</v>
       </c>
       <c r="K90" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -8206,7 +8206,7 @@
         <v>41</v>
       </c>
       <c r="S90" t="n">
-        <v>5.299999999999997</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T90" t="n">
         <v>36.16666666666666</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="K91" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -11295,10 +11295,10 @@
         <v>21</v>
       </c>
       <c r="J126" t="n">
-        <v>23.6</v>
+        <v>23.2</v>
       </c>
       <c r="K126" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L126" t="inlineStr">
         <is>
@@ -11328,10 +11328,10 @@
         <v>21</v>
       </c>
       <c r="S126" t="n">
-        <v>2.600000000000001</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="T126" t="n">
-        <v>22.36666666666667</v>
+        <v>22.36666666666666</v>
       </c>
       <c r="U126" t="n">
         <v>3</v>
@@ -12772,10 +12772,10 @@
         <v>35</v>
       </c>
       <c r="J143" t="n">
-        <v>46</v>
+        <v>37.5</v>
       </c>
       <c r="K143" t="n">
-        <v>131</v>
+        <v>107</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
@@ -12805,7 +12805,7 @@
         <v>41</v>
       </c>
       <c r="S143" t="n">
-        <v>11</v>
+        <v>2.5</v>
       </c>
       <c r="T143" t="n">
         <v>38.3</v>
@@ -12946,10 +12946,10 @@
         <v>35</v>
       </c>
       <c r="J145" t="n">
-        <v>20.3</v>
+        <v>48.5</v>
       </c>
       <c r="K145" t="n">
-        <v>58</v>
+        <v>138</v>
       </c>
       <c r="L145" t="inlineStr">
         <is>
@@ -12979,7 +12979,7 @@
         <v>41</v>
       </c>
       <c r="S145" t="n">
-        <v>-14.7</v>
+        <v>13.5</v>
       </c>
       <c r="T145" t="n">
         <v>30.76666666666667</v>
@@ -15198,10 +15198,10 @@
         <v>35</v>
       </c>
       <c r="J171" t="n">
-        <v>24.1</v>
+        <v>40.5</v>
       </c>
       <c r="K171" t="n">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="L171" t="inlineStr">
         <is>
@@ -15231,7 +15231,7 @@
         <v>41</v>
       </c>
       <c r="S171" t="n">
-        <v>-10.9</v>
+        <v>5.5</v>
       </c>
       <c r="T171" t="n">
         <v>34.6</v>
@@ -15633,10 +15633,10 @@
         <v>21</v>
       </c>
       <c r="J176" t="n">
-        <v>19.3</v>
+        <v>13</v>
       </c>
       <c r="K176" t="n">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="L176" t="inlineStr">
         <is>
@@ -15666,7 +15666,7 @@
         <v>21</v>
       </c>
       <c r="S176" t="n">
-        <v>-1.699999999999999</v>
+        <v>-8</v>
       </c>
       <c r="T176" t="n">
         <v>18.23333333333333</v>
@@ -16675,10 +16675,10 @@
         <v>35</v>
       </c>
       <c r="J188" t="n">
-        <v>43.4</v>
+        <v>26.1</v>
       </c>
       <c r="K188" t="n">
-        <v>124</v>
+        <v>74</v>
       </c>
       <c r="L188" t="inlineStr">
         <is>
@@ -16708,7 +16708,7 @@
         <v>41</v>
       </c>
       <c r="S188" t="n">
-        <v>8.399999999999999</v>
+        <v>-8.899999999999999</v>
       </c>
       <c r="T188" t="n">
         <v>33.26666666666667</v>
@@ -18496,10 +18496,10 @@
         <v>28</v>
       </c>
       <c r="J209" t="n">
-        <v>32.6</v>
+        <v>26.2</v>
       </c>
       <c r="K209" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="L209" t="inlineStr">
         <is>
@@ -18529,7 +18529,7 @@
         <v>28</v>
       </c>
       <c r="S209" t="n">
-        <v>4.600000000000001</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="T209" t="n">
         <v>30.03333333333333</v>
@@ -18931,10 +18931,10 @@
         <v>31</v>
       </c>
       <c r="J214" t="n">
-        <v>36.5</v>
+        <v>33.7</v>
       </c>
       <c r="K214" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -18962,7 +18962,7 @@
       </c>
       <c r="R214" t="inlineStr"/>
       <c r="S214" t="n">
-        <v>5.5</v>
+        <v>2.700000000000003</v>
       </c>
       <c r="T214" t="n">
         <v>33.66666666666666</v>
@@ -19406,7 +19406,7 @@
         <v>3</v>
       </c>
       <c r="V219" t="n">
-        <v>19.75555555555555</v>
+        <v>19.75555555555556</v>
       </c>
       <c r="W219" t="n">
         <v>17.5</v>
@@ -20752,10 +20752,10 @@
         <v>31</v>
       </c>
       <c r="J235" t="n">
-        <v>31.5</v>
+        <v>28.1</v>
       </c>
       <c r="K235" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="L235" t="inlineStr">
         <is>
@@ -20783,7 +20783,7 @@
       </c>
       <c r="R235" t="inlineStr"/>
       <c r="S235" t="n">
-        <v>0.5</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="T235" t="n">
         <v>30.6</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-17 18:17:12
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3671,10 +3671,10 @@
         <v>24</v>
       </c>
       <c r="J38" t="n">
-        <v>25.6</v>
+        <v>21.4</v>
       </c>
       <c r="K38" t="n">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
         <v>28</v>
       </c>
       <c r="S38" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T38" t="n">
         <v>23.8</v>
@@ -5482,10 +5482,10 @@
         <v>24</v>
       </c>
       <c r="J59" t="n">
-        <v>22.1</v>
+        <v>24.7</v>
       </c>
       <c r="K59" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
         <v>28</v>
       </c>
       <c r="S59" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T59" t="n">
         <v>23.8</v>
@@ -5611,7 +5611,7 @@
         <v>3</v>
       </c>
       <c r="V60" t="n">
-        <v>24.52222222222222</v>
+        <v>24.52222222222223</v>
       </c>
       <c r="W60" t="n">
         <v>20.5</v>
@@ -5656,10 +5656,10 @@
         <v>24</v>
       </c>
       <c r="J61" t="n">
-        <v>16.6</v>
+        <v>26.4</v>
       </c>
       <c r="K61" t="n">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -5689,7 +5689,7 @@
         <v>28</v>
       </c>
       <c r="S61" t="n">
-        <v>-7.399999999999999</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T61" t="n">
         <v>23.4</v>
@@ -5698,7 +5698,7 @@
         <v>3</v>
       </c>
       <c r="V61" t="n">
-        <v>24.64444444444444</v>
+        <v>24.64444444444445</v>
       </c>
       <c r="W61" t="n">
         <v>20.5</v>
@@ -6439,10 +6439,10 @@
         <v>35</v>
       </c>
       <c r="J70" t="n">
-        <v>35</v>
+        <v>32.4</v>
       </c>
       <c r="K70" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -6472,7 +6472,7 @@
         <v>41</v>
       </c>
       <c r="S70" t="n">
-        <v>0</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T70" t="n">
         <v>34.83333333333334</v>
@@ -6959,10 +6959,10 @@
         <v>28</v>
       </c>
       <c r="J76" t="n">
-        <v>24.1</v>
+        <v>27.3</v>
       </c>
       <c r="K76" t="n">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -6992,7 +6992,7 @@
         <v>28</v>
       </c>
       <c r="S76" t="n">
-        <v>-3.899999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T76" t="n">
         <v>25.33333333333333</v>
@@ -7046,7 +7046,7 @@
         <v>28</v>
       </c>
       <c r="J77" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="K77" t="n">
         <v>88</v>
@@ -7079,10 +7079,10 @@
         <v>28</v>
       </c>
       <c r="S77" t="n">
-        <v>-3.199999999999999</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="T77" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="U77" t="n">
         <v>3</v>
@@ -7133,10 +7133,10 @@
         <v>28</v>
       </c>
       <c r="J78" t="n">
-        <v>30.7</v>
+        <v>27.7</v>
       </c>
       <c r="K78" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
         <v>28</v>
       </c>
       <c r="S78" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T78" t="n">
         <v>29.2</v>
@@ -7392,10 +7392,10 @@
         <v>35</v>
       </c>
       <c r="J81" t="n">
-        <v>32.4</v>
+        <v>39.8</v>
       </c>
       <c r="K81" t="n">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -7425,7 +7425,7 @@
         <v>41</v>
       </c>
       <c r="S81" t="n">
-        <v>-2.600000000000001</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T81" t="n">
         <v>36.03333333333333</v>
@@ -10860,10 +10860,10 @@
         <v>28</v>
       </c>
       <c r="J121" t="n">
-        <v>31.6</v>
+        <v>33.5</v>
       </c>
       <c r="K121" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -10893,7 +10893,7 @@
         <v>28</v>
       </c>
       <c r="S121" t="n">
-        <v>3.600000000000001</v>
+        <v>5.5</v>
       </c>
       <c r="T121" t="n">
         <v>30.83333333333333</v>
@@ -14332,10 +14332,10 @@
         <v>31</v>
       </c>
       <c r="J161" t="n">
-        <v>26.6</v>
+        <v>28.7</v>
       </c>
       <c r="K161" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="L161" t="inlineStr">
         <is>
@@ -14363,7 +14363,7 @@
       </c>
       <c r="R161" t="inlineStr"/>
       <c r="S161" t="n">
-        <v>-4.399999999999999</v>
+        <v>-2.300000000000001</v>
       </c>
       <c r="T161" t="n">
         <v>28.66666666666667</v>
@@ -16934,10 +16934,10 @@
         <v>31</v>
       </c>
       <c r="J191" t="n">
-        <v>38.5</v>
+        <v>36.1</v>
       </c>
       <c r="K191" t="n">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="L191" t="inlineStr">
         <is>
@@ -16965,7 +16965,7 @@
       </c>
       <c r="R191" t="inlineStr"/>
       <c r="S191" t="n">
-        <v>7.5</v>
+        <v>5.100000000000001</v>
       </c>
       <c r="T191" t="n">
         <v>33.5</v>
@@ -22045,10 +22045,10 @@
         <v>21</v>
       </c>
       <c r="J250" t="n">
-        <v>13.3</v>
+        <v>24.6</v>
       </c>
       <c r="K250" t="n">
-        <v>63</v>
+        <v>117</v>
       </c>
       <c r="L250" t="inlineStr">
         <is>
@@ -22076,10 +22076,10 @@
       </c>
       <c r="R250" t="inlineStr"/>
       <c r="S250" t="n">
-        <v>-7.699999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T250" t="n">
-        <v>20.13333333333333</v>
+        <v>20.13333333333334</v>
       </c>
       <c r="U250" t="n">
         <v>3</v>
@@ -29681,10 +29681,10 @@
         <v>24.5</v>
       </c>
       <c r="J338" t="n">
-        <v>23.5</v>
+        <v>24.5</v>
       </c>
       <c r="K338" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L338" t="inlineStr">
         <is>
@@ -29714,7 +29714,7 @@
         <v>28</v>
       </c>
       <c r="S338" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T338" t="n">
         <v>24.13333333333334</v>
@@ -29768,10 +29768,10 @@
         <v>24.5</v>
       </c>
       <c r="J339" t="n">
-        <v>24.8</v>
+        <v>14</v>
       </c>
       <c r="K339" t="n">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="L339" t="inlineStr">
         <is>
@@ -29801,7 +29801,7 @@
         <v>28</v>
       </c>
       <c r="S339" t="n">
-        <v>0.3000000000000007</v>
+        <v>-10.5</v>
       </c>
       <c r="T339" t="n">
         <v>21.96666666666667</v>
@@ -31419,10 +31419,10 @@
         <v>24.5</v>
       </c>
       <c r="J358" t="n">
-        <v>22.7</v>
+        <v>29.1</v>
       </c>
       <c r="K358" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="L358" t="inlineStr">
         <is>
@@ -31452,7 +31452,7 @@
         <v>28</v>
       </c>
       <c r="S358" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="T358" t="n">
         <v>25.3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-17 22:44:33
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4964,10 +4964,10 @@
         <v>24</v>
       </c>
       <c r="J53" t="n">
-        <v>22.8</v>
+        <v>25.3</v>
       </c>
       <c r="K53" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -4997,7 +4997,7 @@
         <v>28</v>
       </c>
       <c r="S53" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="T53" t="n">
         <v>24.6</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K75" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K79" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K86" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K91" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -10425,10 +10425,10 @@
         <v>28</v>
       </c>
       <c r="J116" t="n">
-        <v>27.6</v>
+        <v>30.7</v>
       </c>
       <c r="K116" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="L116" t="inlineStr">
         <is>
@@ -10458,7 +10458,7 @@
         <v>28</v>
       </c>
       <c r="S116" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="T116" t="n">
         <v>28.03333333333333</v>
@@ -15285,10 +15285,10 @@
         <v>24</v>
       </c>
       <c r="J172" t="n">
-        <v>26.2</v>
+        <v>29.3</v>
       </c>
       <c r="K172" t="n">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="L172" t="inlineStr">
         <is>
@@ -15318,7 +15318,7 @@
         <v>28</v>
       </c>
       <c r="S172" t="n">
-        <v>2.199999999999999</v>
+        <v>5.300000000000001</v>
       </c>
       <c r="T172" t="n">
         <v>24.66666666666667</v>
@@ -21788,10 +21788,10 @@
         <v>21</v>
       </c>
       <c r="J247" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="K247" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L247" t="inlineStr">
         <is>
@@ -21821,7 +21821,7 @@
         <v>21</v>
       </c>
       <c r="S247" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T247" t="n">
         <v>21.2</v>
@@ -23949,10 +23949,10 @@
         <v>21</v>
       </c>
       <c r="J272" t="n">
-        <v>17.8</v>
+        <v>18.3</v>
       </c>
       <c r="K272" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="L272" t="inlineStr">
         <is>
@@ -23982,7 +23982,7 @@
         <v>21</v>
       </c>
       <c r="S272" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="T272" t="n">
         <v>18.73333333333333</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="K321" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="K329" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -29594,10 +29594,10 @@
         <v>24.5</v>
       </c>
       <c r="J337" t="n">
-        <v>24</v>
+        <v>24.7</v>
       </c>
       <c r="K337" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="L337" t="inlineStr">
         <is>
@@ -29627,7 +29627,7 @@
         <v>28</v>
       </c>
       <c r="S337" t="n">
-        <v>-0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T337" t="n">
         <v>24.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="K351" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-18 07:08:57
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -7133,10 +7133,10 @@
         <v>28</v>
       </c>
       <c r="J78" t="n">
-        <v>27.7</v>
+        <v>30.7</v>
       </c>
       <c r="K78" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
         <v>28</v>
       </c>
       <c r="S78" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="T78" t="n">
         <v>29.2</v>
@@ -7305,10 +7305,10 @@
         <v>21</v>
       </c>
       <c r="J80" t="n">
-        <v>17.9</v>
+        <v>26.4</v>
       </c>
       <c r="K80" t="n">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -7338,7 +7338,7 @@
         <v>21</v>
       </c>
       <c r="S80" t="n">
-        <v>-3.100000000000001</v>
+        <v>5.399999999999999</v>
       </c>
       <c r="T80" t="n">
         <v>21.3</v>
@@ -9126,10 +9126,10 @@
         <v>21</v>
       </c>
       <c r="J101" t="n">
-        <v>29</v>
+        <v>18.4</v>
       </c>
       <c r="K101" t="n">
-        <v>138</v>
+        <v>88</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
@@ -9159,7 +9159,7 @@
         <v>21</v>
       </c>
       <c r="S101" t="n">
-        <v>8</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T101" t="n">
         <v>24.53333333333333</v>
@@ -10251,10 +10251,10 @@
         <v>28</v>
       </c>
       <c r="J114" t="n">
-        <v>29.7</v>
+        <v>32.7</v>
       </c>
       <c r="K114" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -10284,7 +10284,7 @@
         <v>28</v>
       </c>
       <c r="S114" t="n">
-        <v>1.699999999999999</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="T114" t="n">
         <v>29.6</v>
@@ -10860,10 +10860,10 @@
         <v>28</v>
       </c>
       <c r="J121" t="n">
-        <v>33.5</v>
+        <v>31.6</v>
       </c>
       <c r="K121" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -10893,7 +10893,7 @@
         <v>28</v>
       </c>
       <c r="S121" t="n">
-        <v>5.5</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T121" t="n">
         <v>30.83333333333333</v>
@@ -14158,10 +14158,10 @@
         <v>21</v>
       </c>
       <c r="J159" t="n">
-        <v>26.3</v>
+        <v>20.8</v>
       </c>
       <c r="K159" t="n">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="L159" t="inlineStr">
         <is>
@@ -14191,7 +14191,7 @@
         <v>21</v>
       </c>
       <c r="S159" t="n">
-        <v>5.300000000000001</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T159" t="n">
         <v>24.5</v>
@@ -15111,10 +15111,10 @@
         <v>28</v>
       </c>
       <c r="J170" t="n">
-        <v>24.8</v>
+        <v>27</v>
       </c>
       <c r="K170" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
@@ -15144,7 +15144,7 @@
         <v>28</v>
       </c>
       <c r="S170" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1</v>
       </c>
       <c r="T170" t="n">
         <v>26.4</v>
@@ -19277,10 +19277,10 @@
         <v>21</v>
       </c>
       <c r="J218" t="n">
-        <v>15.3</v>
+        <v>20.5</v>
       </c>
       <c r="K218" t="n">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="L218" t="inlineStr">
         <is>
@@ -19310,7 +19310,7 @@
         <v>21</v>
       </c>
       <c r="S218" t="n">
-        <v>-5.699999999999999</v>
+        <v>-0.5</v>
       </c>
       <c r="T218" t="n">
         <v>18.26666666666667</v>
@@ -19886,10 +19886,10 @@
         <v>21</v>
       </c>
       <c r="J225" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="K225" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L225" t="inlineStr">
         <is>
@@ -19919,7 +19919,7 @@
         <v>21</v>
       </c>
       <c r="S225" t="n">
-        <v>1.600000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="T225" t="n">
         <v>21.96666666666667</v>
@@ -20319,10 +20319,10 @@
         <v>21</v>
       </c>
       <c r="J230" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="K230" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L230" t="inlineStr">
         <is>
@@ -20352,7 +20352,7 @@
         <v>21</v>
       </c>
       <c r="S230" t="n">
-        <v>1.699999999999999</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="T230" t="n">
         <v>21.56666666666667</v>
@@ -22389,10 +22389,10 @@
         <v>28</v>
       </c>
       <c r="J254" t="n">
-        <v>26.8</v>
+        <v>27.7</v>
       </c>
       <c r="K254" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L254" t="inlineStr">
         <is>
@@ -22422,7 +22422,7 @@
         <v>28</v>
       </c>
       <c r="S254" t="n">
-        <v>-1.199999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T254" t="n">
         <v>27.16666666666667</v>
@@ -24471,10 +24471,10 @@
         <v>28</v>
       </c>
       <c r="J278" t="n">
-        <v>29</v>
+        <v>28.2</v>
       </c>
       <c r="K278" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="L278" t="inlineStr">
         <is>
@@ -24504,7 +24504,7 @@
         <v>28</v>
       </c>
       <c r="S278" t="n">
-        <v>1</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T278" t="n">
         <v>28.2</v>
@@ -24819,10 +24819,10 @@
         <v>21</v>
       </c>
       <c r="J282" t="n">
-        <v>24</v>
+        <v>19.8</v>
       </c>
       <c r="K282" t="n">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="L282" t="inlineStr">
         <is>
@@ -24852,7 +24852,7 @@
         <v>21</v>
       </c>
       <c r="S282" t="n">
-        <v>3</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T282" t="n">
         <v>22.96666666666667</v>
@@ -25511,10 +25511,10 @@
         <v>21</v>
       </c>
       <c r="J290" t="n">
-        <v>20.9</v>
+        <v>22.2</v>
       </c>
       <c r="K290" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="L290" t="inlineStr">
         <is>
@@ -25544,7 +25544,7 @@
         <v>21</v>
       </c>
       <c r="S290" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="T290" t="n">
         <v>22.03333333333333</v>
@@ -25598,10 +25598,10 @@
         <v>21</v>
       </c>
       <c r="J291" t="n">
-        <v>22</v>
+        <v>20.9</v>
       </c>
       <c r="K291" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L291" t="inlineStr">
         <is>
@@ -25631,7 +25631,7 @@
         <v>21</v>
       </c>
       <c r="S291" t="n">
-        <v>1</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T291" t="n">
         <v>21.23333333333333</v>
@@ -26551,10 +26551,10 @@
         <v>21</v>
       </c>
       <c r="J302" t="n">
-        <v>21.2</v>
+        <v>20.4</v>
       </c>
       <c r="K302" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="L302" t="inlineStr">
         <is>
@@ -26584,16 +26584,16 @@
         <v>21</v>
       </c>
       <c r="S302" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T302" t="n">
-        <v>21.16666666666666</v>
+        <v>21.16666666666667</v>
       </c>
       <c r="U302" t="n">
         <v>3</v>
       </c>
       <c r="V302" t="n">
-        <v>22.05555555555555</v>
+        <v>22.05555555555556</v>
       </c>
       <c r="W302" t="n">
         <v>17.5</v>
@@ -29027,7 +29027,7 @@
         <v>3</v>
       </c>
       <c r="V330" t="n">
-        <v>25.57777777777777</v>
+        <v>25.57777777777778</v>
       </c>
       <c r="W330" t="n">
         <v>21</v>
@@ -30984,10 +30984,10 @@
         <v>24.5</v>
       </c>
       <c r="J353" t="n">
-        <v>31.7</v>
+        <v>28.5</v>
       </c>
       <c r="K353" t="n">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="L353" t="inlineStr">
         <is>
@@ -31017,7 +31017,7 @@
         <v>28</v>
       </c>
       <c r="S353" t="n">
-        <v>7.199999999999999</v>
+        <v>4</v>
       </c>
       <c r="T353" t="n">
         <v>28.1</v>
@@ -31678,10 +31678,10 @@
         <v>21</v>
       </c>
       <c r="J361" t="n">
-        <v>20.2</v>
+        <v>21.1</v>
       </c>
       <c r="K361" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L361" t="inlineStr">
         <is>
@@ -31711,7 +31711,7 @@
         <v>21</v>
       </c>
       <c r="S361" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T361" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-18 15:55:55
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -8086,10 +8086,10 @@
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>36.7</v>
+        <v>39.1</v>
       </c>
       <c r="K89" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8119,16 +8119,16 @@
         <v>41</v>
       </c>
       <c r="S89" t="n">
-        <v>1.700000000000003</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T89" t="n">
-        <v>35.73333333333333</v>
+        <v>35.73333333333334</v>
       </c>
       <c r="U89" t="n">
         <v>3</v>
       </c>
       <c r="V89" t="n">
-        <v>35.86296296296296</v>
+        <v>35.86296296296297</v>
       </c>
       <c r="W89" t="n">
         <v>31.5</v>
@@ -10077,10 +10077,10 @@
         <v>21</v>
       </c>
       <c r="J112" t="n">
-        <v>24.3</v>
+        <v>19.9</v>
       </c>
       <c r="K112" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -10110,10 +10110,10 @@
         <v>21</v>
       </c>
       <c r="S112" t="n">
-        <v>3.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="T112" t="n">
-        <v>22.56666666666666</v>
+        <v>22.56666666666667</v>
       </c>
       <c r="U112" t="n">
         <v>3</v>
@@ -10860,10 +10860,10 @@
         <v>28</v>
       </c>
       <c r="J121" t="n">
-        <v>31.6</v>
+        <v>33.5</v>
       </c>
       <c r="K121" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -10893,7 +10893,7 @@
         <v>28</v>
       </c>
       <c r="S121" t="n">
-        <v>3.600000000000001</v>
+        <v>5.5</v>
       </c>
       <c r="T121" t="n">
         <v>30.83333333333333</v>
@@ -19277,10 +19277,10 @@
         <v>21</v>
       </c>
       <c r="J218" t="n">
-        <v>20.5</v>
+        <v>15.3</v>
       </c>
       <c r="K218" t="n">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="L218" t="inlineStr">
         <is>
@@ -19310,7 +19310,7 @@
         <v>21</v>
       </c>
       <c r="S218" t="n">
-        <v>-0.5</v>
+        <v>-5.699999999999999</v>
       </c>
       <c r="T218" t="n">
         <v>18.26666666666667</v>
@@ -19886,10 +19886,10 @@
         <v>21</v>
       </c>
       <c r="J225" t="n">
-        <v>22.5</v>
+        <v>22.6</v>
       </c>
       <c r="K225" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L225" t="inlineStr">
         <is>
@@ -19919,7 +19919,7 @@
         <v>21</v>
       </c>
       <c r="S225" t="n">
-        <v>1.5</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T225" t="n">
         <v>21.96666666666667</v>
@@ -22650,10 +22650,10 @@
         <v>28</v>
       </c>
       <c r="J257" t="n">
-        <v>27.1</v>
+        <v>26.7</v>
       </c>
       <c r="K257" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L257" t="inlineStr">
         <is>
@@ -22683,7 +22683,7 @@
         <v>28</v>
       </c>
       <c r="S257" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T257" t="n">
         <v>26.3</v>
@@ -25254,10 +25254,10 @@
         <v>21</v>
       </c>
       <c r="J287" t="n">
-        <v>20.5</v>
+        <v>20.9</v>
       </c>
       <c r="K287" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L287" t="inlineStr">
         <is>
@@ -25285,7 +25285,7 @@
       </c>
       <c r="R287" t="inlineStr"/>
       <c r="S287" t="n">
-        <v>-0.5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T287" t="n">
         <v>20.2</v>
@@ -25598,10 +25598,10 @@
         <v>21</v>
       </c>
       <c r="J291" t="n">
-        <v>20.9</v>
+        <v>22</v>
       </c>
       <c r="K291" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L291" t="inlineStr">
         <is>
@@ -25631,7 +25631,7 @@
         <v>21</v>
       </c>
       <c r="S291" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1</v>
       </c>
       <c r="T291" t="n">
         <v>21.23333333333333</v>
@@ -25859,10 +25859,10 @@
         <v>21</v>
       </c>
       <c r="J294" t="n">
-        <v>19.8</v>
+        <v>18.9</v>
       </c>
       <c r="K294" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="L294" t="inlineStr">
         <is>
@@ -25892,7 +25892,7 @@
         <v>21</v>
       </c>
       <c r="S294" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="T294" t="n">
         <v>19</v>
@@ -26551,10 +26551,10 @@
         <v>21</v>
       </c>
       <c r="J302" t="n">
-        <v>20.4</v>
+        <v>21.2</v>
       </c>
       <c r="K302" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L302" t="inlineStr">
         <is>
@@ -26584,16 +26584,16 @@
         <v>21</v>
       </c>
       <c r="S302" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T302" t="n">
-        <v>21.16666666666667</v>
+        <v>21.16666666666666</v>
       </c>
       <c r="U302" t="n">
         <v>3</v>
       </c>
       <c r="V302" t="n">
-        <v>22.05555555555556</v>
+        <v>22.05555555555555</v>
       </c>
       <c r="W302" t="n">
         <v>17.5</v>
@@ -28115,10 +28115,10 @@
         <v>24.5</v>
       </c>
       <c r="J320" t="n">
-        <v>21.5</v>
+        <v>33.3</v>
       </c>
       <c r="K320" t="n">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="L320" t="inlineStr">
         <is>
@@ -28148,7 +28148,7 @@
         <v>28</v>
       </c>
       <c r="S320" t="n">
-        <v>-3</v>
+        <v>8.799999999999997</v>
       </c>
       <c r="T320" t="n">
         <v>29.5</v>
@@ -29027,7 +29027,7 @@
         <v>3</v>
       </c>
       <c r="V330" t="n">
-        <v>25.57777777777778</v>
+        <v>25.57777777777777</v>
       </c>
       <c r="W330" t="n">
         <v>21</v>
@@ -29420,10 +29420,10 @@
         <v>24.5</v>
       </c>
       <c r="J335" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="K335" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="L335" t="inlineStr">
         <is>
@@ -29453,7 +29453,7 @@
         <v>28</v>
       </c>
       <c r="S335" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T335" t="n">
         <v>35.8</v>
@@ -31504,10 +31504,10 @@
         <v>24.5</v>
       </c>
       <c r="J359" t="n">
-        <v>27.4</v>
+        <v>23.5</v>
       </c>
       <c r="K359" t="n">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -31537,7 +31537,7 @@
         <v>28</v>
       </c>
       <c r="S359" t="n">
-        <v>2.899999999999999</v>
+        <v>-1</v>
       </c>
       <c r="T359" t="n">
         <v>24.7</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-18 17:48:38
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -8086,10 +8086,10 @@
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>39.1</v>
+        <v>36.7</v>
       </c>
       <c r="K89" t="n">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8119,16 +8119,16 @@
         <v>41</v>
       </c>
       <c r="S89" t="n">
-        <v>4.100000000000001</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T89" t="n">
-        <v>35.73333333333334</v>
+        <v>35.73333333333333</v>
       </c>
       <c r="U89" t="n">
         <v>3</v>
       </c>
       <c r="V89" t="n">
-        <v>35.86296296296297</v>
+        <v>35.86296296296296</v>
       </c>
       <c r="W89" t="n">
         <v>31.5</v>
@@ -8517,10 +8517,10 @@
         <v>21</v>
       </c>
       <c r="J94" t="n">
-        <v>22.5</v>
+        <v>19.5</v>
       </c>
       <c r="K94" t="n">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -8550,7 +8550,7 @@
         <v>21</v>
       </c>
       <c r="S94" t="n">
-        <v>1.5</v>
+        <v>-1.5</v>
       </c>
       <c r="T94" t="n">
         <v>21.9</v>
@@ -9816,10 +9816,10 @@
         <v>35</v>
       </c>
       <c r="J109" t="n">
-        <v>27.1</v>
+        <v>29.6</v>
       </c>
       <c r="K109" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -9849,7 +9849,7 @@
         <v>41</v>
       </c>
       <c r="S109" t="n">
-        <v>-7.899999999999999</v>
+        <v>-5.399999999999999</v>
       </c>
       <c r="T109" t="n">
         <v>27.33333333333333</v>
@@ -10077,10 +10077,10 @@
         <v>21</v>
       </c>
       <c r="J112" t="n">
-        <v>19.9</v>
+        <v>24.3</v>
       </c>
       <c r="K112" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -10110,10 +10110,10 @@
         <v>21</v>
       </c>
       <c r="S112" t="n">
-        <v>-1.100000000000001</v>
+        <v>3.300000000000001</v>
       </c>
       <c r="T112" t="n">
-        <v>22.56666666666667</v>
+        <v>22.56666666666666</v>
       </c>
       <c r="U112" t="n">
         <v>3</v>
@@ -10164,10 +10164,10 @@
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="K113" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         <v>41</v>
       </c>
       <c r="S113" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="T113" t="n">
         <v>25.5</v>
@@ -11382,10 +11382,10 @@
         <v>28</v>
       </c>
       <c r="J127" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="K127" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
@@ -11415,7 +11415,7 @@
         <v>28</v>
       </c>
       <c r="S127" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="T127" t="n">
         <v>25.36666666666666</v>
@@ -20580,10 +20580,10 @@
         <v>31</v>
       </c>
       <c r="J233" t="n">
-        <v>32.3</v>
+        <v>31.2</v>
       </c>
       <c r="K233" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="L233" t="inlineStr">
         <is>
@@ -20611,7 +20611,7 @@
       </c>
       <c r="R233" t="inlineStr"/>
       <c r="S233" t="n">
-        <v>1.299999999999997</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T233" t="n">
         <v>29.3</v>
@@ -22650,10 +22650,10 @@
         <v>28</v>
       </c>
       <c r="J257" t="n">
-        <v>26.7</v>
+        <v>27.1</v>
       </c>
       <c r="K257" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L257" t="inlineStr">
         <is>
@@ -22683,7 +22683,7 @@
         <v>28</v>
       </c>
       <c r="S257" t="n">
-        <v>-1.300000000000001</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T257" t="n">
         <v>26.3</v>
@@ -25254,10 +25254,10 @@
         <v>21</v>
       </c>
       <c r="J287" t="n">
-        <v>20.9</v>
+        <v>20.5</v>
       </c>
       <c r="K287" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="L287" t="inlineStr">
         <is>
@@ -25285,7 +25285,7 @@
       </c>
       <c r="R287" t="inlineStr"/>
       <c r="S287" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.5</v>
       </c>
       <c r="T287" t="n">
         <v>20.2</v>
@@ -26551,10 +26551,10 @@
         <v>21</v>
       </c>
       <c r="J302" t="n">
-        <v>21.2</v>
+        <v>20.4</v>
       </c>
       <c r="K302" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="L302" t="inlineStr">
         <is>
@@ -26584,16 +26584,16 @@
         <v>21</v>
       </c>
       <c r="S302" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T302" t="n">
-        <v>21.16666666666666</v>
+        <v>21.16666666666667</v>
       </c>
       <c r="U302" t="n">
         <v>3</v>
       </c>
       <c r="V302" t="n">
-        <v>22.05555555555555</v>
+        <v>22.05555555555556</v>
       </c>
       <c r="W302" t="n">
         <v>17.5</v>
@@ -26986,10 +26986,10 @@
         <v>21</v>
       </c>
       <c r="J307" t="n">
-        <v>20.7</v>
+        <v>19.6</v>
       </c>
       <c r="K307" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="L307" t="inlineStr">
         <is>
@@ -27019,7 +27019,7 @@
         <v>21</v>
       </c>
       <c r="S307" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.399999999999999</v>
       </c>
       <c r="T307" t="n">
         <v>20.23333333333333</v>
@@ -27419,10 +27419,10 @@
         <v>24.5</v>
       </c>
       <c r="J312" t="n">
-        <v>23.3</v>
+        <v>25.8</v>
       </c>
       <c r="K312" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="L312" t="inlineStr">
         <is>
@@ -27452,7 +27452,7 @@
         <v>28</v>
       </c>
       <c r="S312" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="T312" t="n">
         <v>24.26666666666667</v>
@@ -28115,10 +28115,10 @@
         <v>24.5</v>
       </c>
       <c r="J320" t="n">
-        <v>33.3</v>
+        <v>21.5</v>
       </c>
       <c r="K320" t="n">
-        <v>136</v>
+        <v>88</v>
       </c>
       <c r="L320" t="inlineStr">
         <is>
@@ -28148,7 +28148,7 @@
         <v>28</v>
       </c>
       <c r="S320" t="n">
-        <v>8.799999999999997</v>
+        <v>-3</v>
       </c>
       <c r="T320" t="n">
         <v>29.5</v>
@@ -28550,10 +28550,10 @@
         <v>24.5</v>
       </c>
       <c r="J325" t="n">
-        <v>23.6</v>
+        <v>27</v>
       </c>
       <c r="K325" t="n">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="L325" t="inlineStr">
         <is>
@@ -28583,7 +28583,7 @@
         <v>28</v>
       </c>
       <c r="S325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>2.5</v>
       </c>
       <c r="T325" t="n">
         <v>24.93333333333333</v>
@@ -29420,10 +29420,10 @@
         <v>24.5</v>
       </c>
       <c r="J335" t="n">
-        <v>25.6</v>
+        <v>24</v>
       </c>
       <c r="K335" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="L335" t="inlineStr">
         <is>
@@ -29453,7 +29453,7 @@
         <v>28</v>
       </c>
       <c r="S335" t="n">
-        <v>1.100000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="T335" t="n">
         <v>35.8</v>
@@ -30984,10 +30984,10 @@
         <v>24.5</v>
       </c>
       <c r="J353" t="n">
-        <v>28.5</v>
+        <v>31.7</v>
       </c>
       <c r="K353" t="n">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="L353" t="inlineStr">
         <is>
@@ -31017,7 +31017,7 @@
         <v>28</v>
       </c>
       <c r="S353" t="n">
-        <v>4</v>
+        <v>7.199999999999999</v>
       </c>
       <c r="T353" t="n">
         <v>28.1</v>
@@ -31504,10 +31504,10 @@
         <v>24.5</v>
       </c>
       <c r="J359" t="n">
-        <v>23.5</v>
+        <v>27.4</v>
       </c>
       <c r="K359" t="n">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -31537,7 +31537,7 @@
         <v>28</v>
       </c>
       <c r="S359" t="n">
-        <v>-1</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="T359" t="n">
         <v>24.7</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-18 18:58:00
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5743,10 +5743,10 @@
         <v>24</v>
       </c>
       <c r="J62" t="n">
-        <v>25.7</v>
+        <v>23.4</v>
       </c>
       <c r="K62" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -5776,7 +5776,7 @@
         <v>28</v>
       </c>
       <c r="S62" t="n">
-        <v>1.699999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T62" t="n">
         <v>24.46666666666667</v>
@@ -6178,10 +6178,10 @@
         <v>35</v>
       </c>
       <c r="J67" t="n">
-        <v>34.3</v>
+        <v>32.3</v>
       </c>
       <c r="K67" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -6211,7 +6211,7 @@
         <v>41</v>
       </c>
       <c r="S67" t="n">
-        <v>-0.7000000000000028</v>
+        <v>-2.700000000000003</v>
       </c>
       <c r="T67" t="n">
         <v>32.96666666666666</v>
@@ -7305,10 +7305,10 @@
         <v>21</v>
       </c>
       <c r="J80" t="n">
-        <v>26.4</v>
+        <v>17.9</v>
       </c>
       <c r="K80" t="n">
-        <v>126</v>
+        <v>85</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -7338,7 +7338,7 @@
         <v>21</v>
       </c>
       <c r="S80" t="n">
-        <v>5.399999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T80" t="n">
         <v>21.3</v>
@@ -8517,10 +8517,10 @@
         <v>21</v>
       </c>
       <c r="J94" t="n">
-        <v>19.5</v>
+        <v>22.5</v>
       </c>
       <c r="K94" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -8550,7 +8550,7 @@
         <v>21</v>
       </c>
       <c r="S94" t="n">
-        <v>-1.5</v>
+        <v>1.5</v>
       </c>
       <c r="T94" t="n">
         <v>21.9</v>
@@ -9816,10 +9816,10 @@
         <v>35</v>
       </c>
       <c r="J109" t="n">
-        <v>29.6</v>
+        <v>27.1</v>
       </c>
       <c r="K109" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -9849,7 +9849,7 @@
         <v>41</v>
       </c>
       <c r="S109" t="n">
-        <v>-5.399999999999999</v>
+        <v>-7.899999999999999</v>
       </c>
       <c r="T109" t="n">
         <v>27.33333333333333</v>
@@ -10164,10 +10164,10 @@
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>27.7</v>
+        <v>22.5</v>
       </c>
       <c r="K113" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         <v>41</v>
       </c>
       <c r="S113" t="n">
-        <v>-7.300000000000001</v>
+        <v>-12.5</v>
       </c>
       <c r="T113" t="n">
         <v>25.5</v>
@@ -11382,10 +11382,10 @@
         <v>28</v>
       </c>
       <c r="J127" t="n">
-        <v>24.6</v>
+        <v>27.7</v>
       </c>
       <c r="K127" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
@@ -11415,7 +11415,7 @@
         <v>28</v>
       </c>
       <c r="S127" t="n">
-        <v>-3.399999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T127" t="n">
         <v>25.36666666666666</v>
@@ -13031,10 +13031,10 @@
         <v>35</v>
       </c>
       <c r="J146" t="n">
-        <v>38.6</v>
+        <v>38.2</v>
       </c>
       <c r="K146" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L146" t="inlineStr">
         <is>
@@ -13064,10 +13064,10 @@
         <v>41</v>
       </c>
       <c r="S146" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T146" t="n">
-        <v>36.56666666666667</v>
+        <v>36.56666666666666</v>
       </c>
       <c r="U146" t="n">
         <v>3</v>
@@ -13118,10 +13118,10 @@
         <v>35</v>
       </c>
       <c r="J147" t="n">
-        <v>36.9</v>
+        <v>34.4</v>
       </c>
       <c r="K147" t="n">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="L147" t="inlineStr">
         <is>
@@ -13151,7 +13151,7 @@
         <v>41</v>
       </c>
       <c r="S147" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T147" t="n">
         <v>35.53333333333333</v>
@@ -13292,10 +13292,10 @@
         <v>28</v>
       </c>
       <c r="J149" t="n">
-        <v>30.2</v>
+        <v>30.7</v>
       </c>
       <c r="K149" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
@@ -13325,7 +13325,7 @@
         <v>28</v>
       </c>
       <c r="S149" t="n">
-        <v>2.199999999999999</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="T149" t="n">
         <v>29.23333333333333</v>
@@ -13334,7 +13334,7 @@
         <v>3</v>
       </c>
       <c r="V149" t="n">
-        <v>33.02222222222222</v>
+        <v>33.02222222222223</v>
       </c>
       <c r="W149" t="n">
         <v>24.5</v>
@@ -13636,10 +13636,10 @@
         <v>35</v>
       </c>
       <c r="J153" t="n">
-        <v>38.2</v>
+        <v>34.6</v>
       </c>
       <c r="K153" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="L153" t="inlineStr">
         <is>
@@ -13669,10 +13669,10 @@
         <v>41</v>
       </c>
       <c r="S153" t="n">
-        <v>3.200000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T153" t="n">
-        <v>36.93333333333334</v>
+        <v>36.93333333333333</v>
       </c>
       <c r="U153" t="n">
         <v>3</v>
@@ -13723,10 +13723,10 @@
         <v>35</v>
       </c>
       <c r="J154" t="n">
-        <v>36.7</v>
+        <v>31.5</v>
       </c>
       <c r="K154" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -13756,7 +13756,7 @@
         <v>41</v>
       </c>
       <c r="S154" t="n">
-        <v>1.700000000000003</v>
+        <v>-3.5</v>
       </c>
       <c r="T154" t="n">
         <v>35.23333333333333</v>
@@ -13765,7 +13765,7 @@
         <v>3</v>
       </c>
       <c r="V154" t="n">
-        <v>37.52962962962963</v>
+        <v>37.52962962962962</v>
       </c>
       <c r="W154" t="n">
         <v>31.5</v>
@@ -13810,10 +13810,10 @@
         <v>28</v>
       </c>
       <c r="J155" t="n">
-        <v>36</v>
+        <v>27.9</v>
       </c>
       <c r="K155" t="n">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>
@@ -13843,7 +13843,7 @@
         <v>28</v>
       </c>
       <c r="S155" t="n">
-        <v>8</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T155" t="n">
         <v>34</v>
@@ -20580,10 +20580,10 @@
         <v>31</v>
       </c>
       <c r="J233" t="n">
-        <v>31.2</v>
+        <v>32.3</v>
       </c>
       <c r="K233" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L233" t="inlineStr">
         <is>
@@ -20611,7 +20611,7 @@
       </c>
       <c r="R233" t="inlineStr"/>
       <c r="S233" t="n">
-        <v>0.1999999999999993</v>
+        <v>1.299999999999997</v>
       </c>
       <c r="T233" t="n">
         <v>29.3</v>
@@ -26986,10 +26986,10 @@
         <v>21</v>
       </c>
       <c r="J307" t="n">
-        <v>19.6</v>
+        <v>20.7</v>
       </c>
       <c r="K307" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="L307" t="inlineStr">
         <is>
@@ -27019,7 +27019,7 @@
         <v>21</v>
       </c>
       <c r="S307" t="n">
-        <v>-1.399999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T307" t="n">
         <v>20.23333333333333</v>
@@ -27419,10 +27419,10 @@
         <v>24.5</v>
       </c>
       <c r="J312" t="n">
-        <v>25.8</v>
+        <v>23.3</v>
       </c>
       <c r="K312" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="L312" t="inlineStr">
         <is>
@@ -27452,7 +27452,7 @@
         <v>28</v>
       </c>
       <c r="S312" t="n">
-        <v>1.300000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T312" t="n">
         <v>24.26666666666667</v>
@@ -28550,10 +28550,10 @@
         <v>24.5</v>
       </c>
       <c r="J325" t="n">
-        <v>27</v>
+        <v>23.6</v>
       </c>
       <c r="K325" t="n">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="L325" t="inlineStr">
         <is>
@@ -28583,7 +28583,7 @@
         <v>28</v>
       </c>
       <c r="S325" t="n">
-        <v>2.5</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T325" t="n">
         <v>24.93333333333333</v>
@@ -30984,10 +30984,10 @@
         <v>24.5</v>
       </c>
       <c r="J353" t="n">
-        <v>31.7</v>
+        <v>28.5</v>
       </c>
       <c r="K353" t="n">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="L353" t="inlineStr">
         <is>
@@ -31017,7 +31017,7 @@
         <v>28</v>
       </c>
       <c r="S353" t="n">
-        <v>7.199999999999999</v>
+        <v>4</v>
       </c>
       <c r="T353" t="n">
         <v>28.1</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-18 20:20:22
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5743,10 +5743,10 @@
         <v>24</v>
       </c>
       <c r="J62" t="n">
-        <v>23.4</v>
+        <v>25.7</v>
       </c>
       <c r="K62" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -5776,7 +5776,7 @@
         <v>28</v>
       </c>
       <c r="S62" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="T62" t="n">
         <v>24.46666666666667</v>
@@ -6178,10 +6178,10 @@
         <v>35</v>
       </c>
       <c r="J67" t="n">
-        <v>32.3</v>
+        <v>34.3</v>
       </c>
       <c r="K67" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -6211,7 +6211,7 @@
         <v>41</v>
       </c>
       <c r="S67" t="n">
-        <v>-2.700000000000003</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="T67" t="n">
         <v>32.96666666666666</v>
@@ -6439,10 +6439,10 @@
         <v>35</v>
       </c>
       <c r="J70" t="n">
-        <v>32.4</v>
+        <v>35</v>
       </c>
       <c r="K70" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -6472,7 +6472,7 @@
         <v>41</v>
       </c>
       <c r="S70" t="n">
-        <v>-2.600000000000001</v>
+        <v>0</v>
       </c>
       <c r="T70" t="n">
         <v>34.83333333333334</v>
@@ -7305,10 +7305,10 @@
         <v>21</v>
       </c>
       <c r="J80" t="n">
-        <v>17.9</v>
+        <v>26.4</v>
       </c>
       <c r="K80" t="n">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -7338,7 +7338,7 @@
         <v>21</v>
       </c>
       <c r="S80" t="n">
-        <v>-3.100000000000001</v>
+        <v>5.399999999999999</v>
       </c>
       <c r="T80" t="n">
         <v>21.3</v>
@@ -11121,10 +11121,10 @@
         <v>21</v>
       </c>
       <c r="J124" t="n">
-        <v>21.6</v>
+        <v>19.4</v>
       </c>
       <c r="K124" t="n">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -11154,7 +11154,7 @@
         <v>21</v>
       </c>
       <c r="S124" t="n">
-        <v>0.6000000000000014</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T124" t="n">
         <v>19.93333333333333</v>
@@ -13031,10 +13031,10 @@
         <v>35</v>
       </c>
       <c r="J146" t="n">
-        <v>38.2</v>
+        <v>38.6</v>
       </c>
       <c r="K146" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="L146" t="inlineStr">
         <is>
@@ -13064,10 +13064,10 @@
         <v>41</v>
       </c>
       <c r="S146" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T146" t="n">
-        <v>36.56666666666666</v>
+        <v>36.56666666666667</v>
       </c>
       <c r="U146" t="n">
         <v>3</v>
@@ -13118,10 +13118,10 @@
         <v>35</v>
       </c>
       <c r="J147" t="n">
-        <v>34.4</v>
+        <v>36.9</v>
       </c>
       <c r="K147" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="L147" t="inlineStr">
         <is>
@@ -13151,7 +13151,7 @@
         <v>41</v>
       </c>
       <c r="S147" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T147" t="n">
         <v>35.53333333333333</v>
@@ -13292,10 +13292,10 @@
         <v>28</v>
       </c>
       <c r="J149" t="n">
-        <v>30.7</v>
+        <v>30.2</v>
       </c>
       <c r="K149" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="L149" t="inlineStr">
         <is>
@@ -13325,7 +13325,7 @@
         <v>28</v>
       </c>
       <c r="S149" t="n">
-        <v>2.699999999999999</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="T149" t="n">
         <v>29.23333333333333</v>
@@ -13334,7 +13334,7 @@
         <v>3</v>
       </c>
       <c r="V149" t="n">
-        <v>33.02222222222223</v>
+        <v>33.02222222222222</v>
       </c>
       <c r="W149" t="n">
         <v>24.5</v>
@@ -13636,10 +13636,10 @@
         <v>35</v>
       </c>
       <c r="J153" t="n">
-        <v>34.6</v>
+        <v>38.2</v>
       </c>
       <c r="K153" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="L153" t="inlineStr">
         <is>
@@ -13669,10 +13669,10 @@
         <v>41</v>
       </c>
       <c r="S153" t="n">
-        <v>-0.3999999999999986</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T153" t="n">
-        <v>36.93333333333333</v>
+        <v>36.93333333333334</v>
       </c>
       <c r="U153" t="n">
         <v>3</v>
@@ -13723,10 +13723,10 @@
         <v>35</v>
       </c>
       <c r="J154" t="n">
-        <v>31.5</v>
+        <v>36.7</v>
       </c>
       <c r="K154" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -13756,7 +13756,7 @@
         <v>41</v>
       </c>
       <c r="S154" t="n">
-        <v>-3.5</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T154" t="n">
         <v>35.23333333333333</v>
@@ -13765,7 +13765,7 @@
         <v>3</v>
       </c>
       <c r="V154" t="n">
-        <v>37.52962962962962</v>
+        <v>37.52962962962963</v>
       </c>
       <c r="W154" t="n">
         <v>31.5</v>
@@ -13810,10 +13810,10 @@
         <v>28</v>
       </c>
       <c r="J155" t="n">
-        <v>27.9</v>
+        <v>36</v>
       </c>
       <c r="K155" t="n">
-        <v>100</v>
+        <v>128</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>
@@ -13843,7 +13843,7 @@
         <v>28</v>
       </c>
       <c r="S155" t="n">
-        <v>-0.1000000000000014</v>
+        <v>8</v>
       </c>
       <c r="T155" t="n">
         <v>34</v>
@@ -14591,10 +14591,10 @@
         <v>31</v>
       </c>
       <c r="J164" t="n">
-        <v>32.1</v>
+        <v>28.6</v>
       </c>
       <c r="K164" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="L164" t="inlineStr">
         <is>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="R164" t="inlineStr"/>
       <c r="S164" t="n">
-        <v>1.100000000000001</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="T164" t="n">
         <v>30.7</v>
@@ -17193,10 +17193,10 @@
         <v>31</v>
       </c>
       <c r="J194" t="n">
-        <v>36.6</v>
+        <v>36</v>
       </c>
       <c r="K194" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="L194" t="inlineStr">
         <is>
@@ -17224,7 +17224,7 @@
       </c>
       <c r="R194" t="inlineStr"/>
       <c r="S194" t="n">
-        <v>5.600000000000001</v>
+        <v>5</v>
       </c>
       <c r="T194" t="n">
         <v>33.6</v>
@@ -18931,10 +18931,10 @@
         <v>31</v>
       </c>
       <c r="J214" t="n">
-        <v>33.7</v>
+        <v>36.5</v>
       </c>
       <c r="K214" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -18962,7 +18962,7 @@
       </c>
       <c r="R214" t="inlineStr"/>
       <c r="S214" t="n">
-        <v>2.700000000000003</v>
+        <v>5.5</v>
       </c>
       <c r="T214" t="n">
         <v>33.66666666666666</v>
@@ -22130,10 +22130,10 @@
         <v>21</v>
       </c>
       <c r="J251" t="n">
-        <v>21.3</v>
+        <v>23.8</v>
       </c>
       <c r="K251" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="L251" t="inlineStr">
         <is>
@@ -22161,7 +22161,7 @@
       </c>
       <c r="R251" t="inlineStr"/>
       <c r="S251" t="n">
-        <v>0.3000000000000007</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T251" t="n">
         <v>21.8</v>
@@ -22302,10 +22302,10 @@
         <v>21</v>
       </c>
       <c r="J253" t="n">
-        <v>42.6</v>
+        <v>16.6</v>
       </c>
       <c r="K253" t="n">
-        <v>203</v>
+        <v>79</v>
       </c>
       <c r="L253" t="inlineStr">
         <is>
@@ -22335,7 +22335,7 @@
         <v>21</v>
       </c>
       <c r="S253" t="n">
-        <v>21.6</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="T253" t="n">
         <v>36.33333333333334</v>
@@ -23949,10 +23949,10 @@
         <v>21</v>
       </c>
       <c r="J272" t="n">
-        <v>17.8</v>
+        <v>18.3</v>
       </c>
       <c r="K272" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="L272" t="inlineStr">
         <is>
@@ -23982,7 +23982,7 @@
         <v>21</v>
       </c>
       <c r="S272" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="T272" t="n">
         <v>18.73333333333333</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>
@@ -31678,10 +31678,10 @@
         <v>21</v>
       </c>
       <c r="J361" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="K361" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L361" t="inlineStr">
         <is>
@@ -31711,7 +31711,7 @@
         <v>21</v>
       </c>
       <c r="S361" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T361" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-18 22:18:35
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4533,10 +4533,10 @@
         <v>24</v>
       </c>
       <c r="J48" t="n">
-        <v>22.1</v>
+        <v>25.9</v>
       </c>
       <c r="K48" t="n">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v>28</v>
       </c>
       <c r="S48" t="n">
-        <v>-1.899999999999999</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T48" t="n">
         <v>24.23333333333333</v>
@@ -5397,10 +5397,10 @@
         <v>31</v>
       </c>
       <c r="J58" t="n">
-        <v>31.4</v>
+        <v>35.8</v>
       </c>
       <c r="K58" t="n">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
       </c>
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="n">
-        <v>0.3999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T58" t="n">
-        <v>30.66666666666666</v>
+        <v>30.66666666666667</v>
       </c>
       <c r="U58" t="n">
         <v>3</v>
@@ -5482,10 +5482,10 @@
         <v>24</v>
       </c>
       <c r="J59" t="n">
-        <v>22.1</v>
+        <v>24.7</v>
       </c>
       <c r="K59" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -5515,7 +5515,7 @@
         <v>28</v>
       </c>
       <c r="S59" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T59" t="n">
         <v>23.8</v>
@@ -6439,10 +6439,10 @@
         <v>35</v>
       </c>
       <c r="J70" t="n">
-        <v>35</v>
+        <v>32.4</v>
       </c>
       <c r="K70" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -6472,7 +6472,7 @@
         <v>41</v>
       </c>
       <c r="S70" t="n">
-        <v>0</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T70" t="n">
         <v>34.83333333333334</v>
@@ -7046,7 +7046,7 @@
         <v>28</v>
       </c>
       <c r="J77" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="K77" t="n">
         <v>88</v>
@@ -7079,7 +7079,7 @@
         <v>28</v>
       </c>
       <c r="S77" t="n">
-        <v>-3.199999999999999</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="T77" t="n">
         <v>25.13333333333334</v>
@@ -10164,10 +10164,10 @@
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="K113" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         <v>41</v>
       </c>
       <c r="S113" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="T113" t="n">
         <v>25.5</v>
@@ -11121,10 +11121,10 @@
         <v>21</v>
       </c>
       <c r="J124" t="n">
-        <v>19.4</v>
+        <v>21.6</v>
       </c>
       <c r="K124" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -11154,7 +11154,7 @@
         <v>21</v>
       </c>
       <c r="S124" t="n">
-        <v>-1.600000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T124" t="n">
         <v>19.93333333333333</v>
@@ -11208,10 +11208,10 @@
         <v>35</v>
       </c>
       <c r="J125" t="n">
-        <v>30.5</v>
+        <v>35.4</v>
       </c>
       <c r="K125" t="n">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -11241,7 +11241,7 @@
         <v>41</v>
       </c>
       <c r="S125" t="n">
-        <v>-4.5</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T125" t="n">
         <v>34.13333333333333</v>
@@ -11250,7 +11250,7 @@
         <v>3</v>
       </c>
       <c r="V125" t="n">
-        <v>36.32592592592593</v>
+        <v>36.32592592592592</v>
       </c>
       <c r="W125" t="n">
         <v>31.5</v>
@@ -11295,10 +11295,10 @@
         <v>21</v>
       </c>
       <c r="J126" t="n">
-        <v>23.2</v>
+        <v>20.3</v>
       </c>
       <c r="K126" t="n">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="L126" t="inlineStr">
         <is>
@@ -11328,10 +11328,10 @@
         <v>21</v>
       </c>
       <c r="S126" t="n">
-        <v>2.199999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T126" t="n">
-        <v>22.36666666666666</v>
+        <v>22.36666666666667</v>
       </c>
       <c r="U126" t="n">
         <v>3</v>
@@ -11382,10 +11382,10 @@
         <v>28</v>
       </c>
       <c r="J127" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="K127" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
@@ -11415,10 +11415,10 @@
         <v>28</v>
       </c>
       <c r="S127" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="T127" t="n">
-        <v>25.36666666666666</v>
+        <v>25.36666666666667</v>
       </c>
       <c r="U127" t="n">
         <v>3</v>
@@ -11469,10 +11469,10 @@
         <v>35</v>
       </c>
       <c r="J128" t="n">
-        <v>33.9</v>
+        <v>30.7</v>
       </c>
       <c r="K128" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="L128" t="inlineStr">
         <is>
@@ -11502,7 +11502,7 @@
         <v>41</v>
       </c>
       <c r="S128" t="n">
-        <v>-1.100000000000001</v>
+        <v>-4.300000000000001</v>
       </c>
       <c r="T128" t="n">
         <v>31.83333333333333</v>
@@ -11511,7 +11511,7 @@
         <v>3</v>
       </c>
       <c r="V128" t="n">
-        <v>34.15555555555556</v>
+        <v>34.15555555555555</v>
       </c>
       <c r="W128" t="n">
         <v>31.5</v>
@@ -11730,10 +11730,10 @@
         <v>35</v>
       </c>
       <c r="J131" t="n">
-        <v>36.6</v>
+        <v>36.5</v>
       </c>
       <c r="K131" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -11763,7 +11763,7 @@
         <v>41</v>
       </c>
       <c r="S131" t="n">
-        <v>1.600000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="T131" t="n">
         <v>35.63333333333333</v>
@@ -11772,7 +11772,7 @@
         <v>3</v>
       </c>
       <c r="V131" t="n">
-        <v>41.38148148148148</v>
+        <v>41.38148148148147</v>
       </c>
       <c r="W131" t="n">
         <v>31.5</v>
@@ -11817,10 +11817,10 @@
         <v>28</v>
       </c>
       <c r="J132" t="n">
-        <v>33.1</v>
+        <v>29.9</v>
       </c>
       <c r="K132" t="n">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="L132" t="inlineStr">
         <is>
@@ -11850,7 +11850,7 @@
         <v>28</v>
       </c>
       <c r="S132" t="n">
-        <v>5.100000000000001</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T132" t="n">
         <v>28.06666666666666</v>
@@ -11904,10 +11904,10 @@
         <v>35</v>
       </c>
       <c r="J133" t="n">
-        <v>36.1</v>
+        <v>36.4</v>
       </c>
       <c r="K133" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -11937,7 +11937,7 @@
         <v>41</v>
       </c>
       <c r="S133" t="n">
-        <v>1.100000000000001</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="T133" t="n">
         <v>33.9</v>
@@ -14591,10 +14591,10 @@
         <v>31</v>
       </c>
       <c r="J164" t="n">
-        <v>28.6</v>
+        <v>32.1</v>
       </c>
       <c r="K164" t="n">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="L164" t="inlineStr">
         <is>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="R164" t="inlineStr"/>
       <c r="S164" t="n">
-        <v>-2.399999999999999</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T164" t="n">
         <v>30.7</v>
@@ -17193,10 +17193,10 @@
         <v>31</v>
       </c>
       <c r="J194" t="n">
-        <v>36</v>
+        <v>36.6</v>
       </c>
       <c r="K194" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L194" t="inlineStr">
         <is>
@@ -17224,7 +17224,7 @@
       </c>
       <c r="R194" t="inlineStr"/>
       <c r="S194" t="n">
-        <v>5</v>
+        <v>5.600000000000001</v>
       </c>
       <c r="T194" t="n">
         <v>33.6</v>
@@ -18931,10 +18931,10 @@
         <v>31</v>
       </c>
       <c r="J214" t="n">
-        <v>36.5</v>
+        <v>33.7</v>
       </c>
       <c r="K214" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -18962,7 +18962,7 @@
       </c>
       <c r="R214" t="inlineStr"/>
       <c r="S214" t="n">
-        <v>5.5</v>
+        <v>2.700000000000003</v>
       </c>
       <c r="T214" t="n">
         <v>33.66666666666666</v>
@@ -20234,10 +20234,10 @@
         <v>31</v>
       </c>
       <c r="J229" t="n">
-        <v>29.5</v>
+        <v>27.2</v>
       </c>
       <c r="K229" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="L229" t="inlineStr">
         <is>
@@ -20265,7 +20265,7 @@
       </c>
       <c r="R229" t="inlineStr"/>
       <c r="S229" t="n">
-        <v>-1.5</v>
+        <v>-3.800000000000001</v>
       </c>
       <c r="T229" t="n">
         <v>30.6</v>
@@ -22130,10 +22130,10 @@
         <v>21</v>
       </c>
       <c r="J251" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="K251" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="L251" t="inlineStr">
         <is>
@@ -22161,7 +22161,7 @@
       </c>
       <c r="R251" t="inlineStr"/>
       <c r="S251" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="T251" t="n">
         <v>21.8</v>
@@ -22302,10 +22302,10 @@
         <v>21</v>
       </c>
       <c r="J253" t="n">
-        <v>16.6</v>
+        <v>42.6</v>
       </c>
       <c r="K253" t="n">
-        <v>79</v>
+        <v>203</v>
       </c>
       <c r="L253" t="inlineStr">
         <is>
@@ -22335,7 +22335,7 @@
         <v>21</v>
       </c>
       <c r="S253" t="n">
-        <v>-4.399999999999999</v>
+        <v>21.6</v>
       </c>
       <c r="T253" t="n">
         <v>36.33333333333334</v>
@@ -23949,10 +23949,10 @@
         <v>21</v>
       </c>
       <c r="J272" t="n">
-        <v>18.3</v>
+        <v>17.8</v>
       </c>
       <c r="K272" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L272" t="inlineStr">
         <is>
@@ -23982,7 +23982,7 @@
         <v>21</v>
       </c>
       <c r="S272" t="n">
-        <v>-2.699999999999999</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T272" t="n">
         <v>18.73333333333333</v>
@@ -31678,10 +31678,10 @@
         <v>21</v>
       </c>
       <c r="J361" t="n">
-        <v>20.2</v>
+        <v>21.1</v>
       </c>
       <c r="K361" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L361" t="inlineStr">
         <is>
@@ -31711,7 +31711,7 @@
         <v>21</v>
       </c>
       <c r="S361" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T361" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-19 02:43:16
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -602,11 +602,11 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="n">
@@ -687,11 +687,11 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R3" t="n">
         <v>28</v>
@@ -774,11 +774,11 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="n">
@@ -859,11 +859,11 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R5" t="n">
         <v>48</v>
@@ -946,11 +946,11 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R6" t="n">
         <v>41</v>
@@ -1033,11 +1033,11 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R7" t="n">
         <v>48</v>
@@ -1120,11 +1120,11 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R8" t="n">
         <v>41</v>
@@ -1207,11 +1207,11 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q9" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
@@ -1292,11 +1292,11 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
@@ -1377,11 +1377,11 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="n">
@@ -1462,11 +1462,11 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="n">
@@ -1547,11 +1547,11 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="n">
@@ -1632,11 +1632,11 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R14" t="n">
         <v>21</v>
@@ -1719,11 +1719,11 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="n">
@@ -1804,11 +1804,11 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="n">
@@ -1889,11 +1889,11 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="n">
@@ -1974,11 +1974,11 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R18" t="n">
         <v>34</v>
@@ -2061,11 +2061,11 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="n">
@@ -2146,11 +2146,11 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R20" t="n">
         <v>48</v>
@@ -2233,11 +2233,11 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R21" t="n">
         <v>34</v>
@@ -2320,11 +2320,11 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R22" t="n">
         <v>28</v>
@@ -2407,11 +2407,11 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R23" t="n">
         <v>28</v>
@@ -2494,11 +2494,11 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R24" t="n">
         <v>28</v>
@@ -2581,11 +2581,11 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R25" t="n">
         <v>28</v>
@@ -2666,11 +2666,11 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="n">
@@ -2751,11 +2751,11 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R27" t="n">
         <v>28</v>
@@ -2838,11 +2838,11 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R28" t="n">
         <v>28</v>
@@ -2925,11 +2925,11 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R29" t="n">
         <v>28</v>
@@ -3012,11 +3012,11 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
@@ -3097,11 +3097,11 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="n">
@@ -3182,11 +3182,11 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="n">
@@ -3267,11 +3267,11 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R33" t="n">
         <v>28</v>
@@ -3354,11 +3354,11 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="n">
@@ -3439,11 +3439,11 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="n">
@@ -3524,11 +3524,11 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q36" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="n">
@@ -3609,11 +3609,11 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q37" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="n">
@@ -3694,11 +3694,11 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R38" t="n">
         <v>28</v>
@@ -3781,11 +3781,11 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="n">
@@ -3866,11 +3866,11 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R40" t="n">
         <v>28</v>
@@ -3953,11 +3953,11 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="n">
@@ -4038,11 +4038,11 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q42" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="n">
@@ -4123,11 +4123,11 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q43" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R43" t="n">
         <v>28</v>
@@ -4210,11 +4210,11 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q44" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R44" t="n">
         <v>28</v>
@@ -4297,11 +4297,11 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q45" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="n">
@@ -4382,11 +4382,11 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q46" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R46" t="n">
         <v>28</v>
@@ -4469,11 +4469,11 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q47" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R47" t="n">
         <v>28</v>
@@ -4556,11 +4556,11 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R48" t="n">
         <v>28</v>
@@ -4643,11 +4643,11 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q49" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R49" t="n">
         <v>28</v>
@@ -4730,11 +4730,11 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q50" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R50" t="n">
         <v>28</v>
@@ -4817,11 +4817,11 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q51" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="n">
@@ -4902,11 +4902,11 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q52" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="n">
@@ -4987,11 +4987,11 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q53" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R53" t="n">
         <v>28</v>
@@ -5074,11 +5074,11 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q54" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R54" t="n">
         <v>28</v>
@@ -5161,11 +5161,11 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q55" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="n">
@@ -5246,11 +5246,11 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q56" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R56" t="n">
         <v>28</v>
@@ -5333,11 +5333,11 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q57" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R57" t="n">
         <v>28</v>
@@ -5420,11 +5420,11 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q58" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="n">
@@ -5505,11 +5505,11 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q59" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R59" t="n">
         <v>28</v>
@@ -5592,11 +5592,11 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q60" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R60" t="n">
         <v>28</v>
@@ -5656,10 +5656,10 @@
         <v>24</v>
       </c>
       <c r="J61" t="n">
-        <v>16.6</v>
+        <v>27.2</v>
       </c>
       <c r="K61" t="n">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -5679,17 +5679,17 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q61" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R61" t="n">
         <v>28</v>
       </c>
       <c r="S61" t="n">
-        <v>-7.399999999999999</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="T61" t="n">
         <v>23.4</v>
@@ -5766,11 +5766,11 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q62" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R62" t="n">
         <v>28</v>
@@ -5853,11 +5853,11 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q63" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R63" t="n">
         <v>28</v>
@@ -5940,11 +5940,11 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q64" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R64" t="n">
         <v>28</v>
@@ -6027,11 +6027,11 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q65" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R65" t="n">
         <v>28</v>
@@ -6091,10 +6091,10 @@
         <v>21</v>
       </c>
       <c r="J66" t="n">
-        <v>19.7</v>
+        <v>20.3</v>
       </c>
       <c r="K66" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -6114,17 +6114,17 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q66" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R66" t="n">
         <v>21</v>
       </c>
       <c r="S66" t="n">
-        <v>-1.300000000000001</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T66" t="n">
         <v>20.03333333333333</v>
@@ -6201,11 +6201,11 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q67" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R67" t="n">
         <v>41</v>
@@ -6288,11 +6288,11 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q68" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R68" t="n">
         <v>41</v>
@@ -6375,11 +6375,11 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q69" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R69" t="n">
         <v>21</v>
@@ -6462,11 +6462,11 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q70" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R70" t="n">
         <v>41</v>
@@ -6549,11 +6549,11 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q71" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R71" t="n">
         <v>21</v>
@@ -6636,11 +6636,11 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q72" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R72" t="n">
         <v>21</v>
@@ -6723,11 +6723,11 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q73" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R73" t="n">
         <v>41</v>
@@ -6810,11 +6810,11 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q74" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R74" t="n">
         <v>21</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K75" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6897,15 +6897,15 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q75" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -6982,11 +6982,11 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q76" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R76" t="n">
         <v>28</v>
@@ -7069,11 +7069,11 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q77" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R77" t="n">
         <v>28</v>
@@ -7156,11 +7156,11 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q78" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R78" t="n">
         <v>28</v>
@@ -7243,11 +7243,11 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q79" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
@@ -7328,11 +7328,11 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q80" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R80" t="n">
         <v>21</v>
@@ -7415,11 +7415,11 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q81" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R81" t="n">
         <v>41</v>
@@ -7502,11 +7502,11 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q82" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R82" t="n">
         <v>21</v>
@@ -7589,11 +7589,11 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q83" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R83" t="n">
         <v>21</v>
@@ -7676,11 +7676,11 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q84" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R84" t="n">
         <v>21</v>
@@ -7763,11 +7763,11 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q85" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R85" t="n">
         <v>21</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K86" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7850,15 +7850,15 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q86" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -7935,11 +7935,11 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q87" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R87" t="n">
         <v>21</v>
@@ -8022,11 +8022,11 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q88" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R88" t="n">
         <v>41</v>
@@ -8109,11 +8109,11 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q89" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R89" t="n">
         <v>41</v>
@@ -8196,11 +8196,11 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q90" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R90" t="n">
         <v>41</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K91" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8283,15 +8283,15 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q91" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -8368,11 +8368,11 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q92" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R92" t="n">
         <v>41</v>
@@ -8455,11 +8455,11 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q93" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R93" t="inlineStr"/>
       <c r="S93" t="n">
@@ -8540,11 +8540,11 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q94" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R94" t="n">
         <v>21</v>
@@ -8627,11 +8627,11 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q95" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R95" t="n">
         <v>41</v>
@@ -8714,11 +8714,11 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q96" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R96" t="n">
         <v>41</v>
@@ -8801,11 +8801,11 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q97" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R97" t="n">
         <v>28</v>
@@ -8888,11 +8888,11 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q98" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R98" t="n">
         <v>41</v>
@@ -8975,11 +8975,11 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q99" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R99" t="n">
         <v>21</v>
@@ -9062,11 +9062,11 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q100" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R100" t="n">
         <v>28</v>
@@ -9149,11 +9149,11 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q101" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R101" t="n">
         <v>21</v>
@@ -9236,11 +9236,11 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q102" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R102" t="inlineStr"/>
       <c r="S102" t="n">
@@ -9321,11 +9321,11 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q103" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R103" t="inlineStr"/>
       <c r="S103" t="n">
@@ -9406,11 +9406,11 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q104" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R104" t="inlineStr"/>
       <c r="S104" t="n">
@@ -9468,10 +9468,10 @@
         <v>35</v>
       </c>
       <c r="J105" t="n">
-        <v>38</v>
+        <v>39.5</v>
       </c>
       <c r="K105" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
@@ -9491,17 +9491,17 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q105" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R105" t="n">
         <v>41</v>
       </c>
       <c r="S105" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="T105" t="n">
         <v>37.06666666666667</v>
@@ -9578,11 +9578,11 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q106" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R106" t="n">
         <v>21</v>
@@ -9665,11 +9665,11 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q107" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R107" t="n">
         <v>41</v>
@@ -9752,11 +9752,11 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q108" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R108" t="n">
         <v>41</v>
@@ -9839,11 +9839,11 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q109" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R109" t="n">
         <v>41</v>
@@ -9926,11 +9926,11 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q110" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R110" t="n">
         <v>41</v>
@@ -10013,11 +10013,11 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q111" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R111" t="n">
         <v>41</v>
@@ -10100,11 +10100,11 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q112" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R112" t="n">
         <v>21</v>
@@ -10187,11 +10187,11 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q113" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R113" t="n">
         <v>41</v>
@@ -10274,11 +10274,11 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q114" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R114" t="n">
         <v>28</v>
@@ -10361,11 +10361,11 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q115" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R115" t="n">
         <v>41</v>
@@ -10448,11 +10448,11 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q116" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R116" t="n">
         <v>28</v>
@@ -10535,11 +10535,11 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q117" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R117" t="n">
         <v>41</v>
@@ -10622,11 +10622,11 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q118" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R118" t="n">
         <v>41</v>
@@ -10709,11 +10709,11 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q119" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R119" t="n">
         <v>41</v>
@@ -10796,11 +10796,11 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q120" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R120" t="n">
         <v>21</v>
@@ -10860,10 +10860,10 @@
         <v>28</v>
       </c>
       <c r="J121" t="n">
-        <v>33.5</v>
+        <v>31.6</v>
       </c>
       <c r="K121" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -10883,17 +10883,17 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q121" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R121" t="n">
         <v>28</v>
       </c>
       <c r="S121" t="n">
-        <v>5.5</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T121" t="n">
         <v>30.83333333333333</v>
@@ -10970,11 +10970,11 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q122" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R122" t="n">
         <v>21</v>
@@ -11057,11 +11057,11 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q123" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R123" t="n">
         <v>21</v>
@@ -11121,10 +11121,10 @@
         <v>21</v>
       </c>
       <c r="J124" t="n">
-        <v>21.6</v>
+        <v>19.4</v>
       </c>
       <c r="K124" t="n">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="L124" t="inlineStr">
         <is>
@@ -11144,17 +11144,17 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q124" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R124" t="n">
         <v>21</v>
       </c>
       <c r="S124" t="n">
-        <v>0.6000000000000014</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T124" t="n">
         <v>19.93333333333333</v>
@@ -11231,11 +11231,11 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q125" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R125" t="n">
         <v>41</v>
@@ -11318,11 +11318,11 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q126" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R126" t="n">
         <v>21</v>
@@ -11405,11 +11405,11 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q127" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R127" t="n">
         <v>28</v>
@@ -11492,11 +11492,11 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q128" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R128" t="n">
         <v>41</v>
@@ -11579,11 +11579,11 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q129" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R129" t="n">
         <v>28</v>
@@ -11666,11 +11666,11 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q130" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R130" t="n">
         <v>21</v>
@@ -11753,11 +11753,11 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q131" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R131" t="n">
         <v>41</v>
@@ -11840,11 +11840,11 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q132" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R132" t="n">
         <v>28</v>
@@ -11927,11 +11927,11 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q133" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R133" t="n">
         <v>41</v>
@@ -12014,11 +12014,11 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q134" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R134" t="n">
         <v>41</v>
@@ -12078,10 +12078,10 @@
         <v>31</v>
       </c>
       <c r="J135" t="n">
-        <v>31.9</v>
+        <v>30.5</v>
       </c>
       <c r="K135" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="L135" t="inlineStr">
         <is>
@@ -12101,15 +12101,15 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q135" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R135" t="inlineStr"/>
       <c r="S135" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.5</v>
       </c>
       <c r="T135" t="n">
         <v>31.23333333333333</v>
@@ -12186,11 +12186,11 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q136" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R136" t="n">
         <v>28</v>
@@ -12273,11 +12273,11 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q137" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R137" t="n">
         <v>41</v>
@@ -12337,10 +12337,10 @@
         <v>28</v>
       </c>
       <c r="J138" t="n">
-        <v>27.4</v>
+        <v>27.9</v>
       </c>
       <c r="K138" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L138" t="inlineStr">
         <is>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q138" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R138" t="n">
         <v>28</v>
       </c>
       <c r="S138" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T138" t="n">
         <v>28.4</v>
@@ -12447,11 +12447,11 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q139" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R139" t="n">
         <v>41</v>
@@ -12534,11 +12534,11 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q140" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R140" t="n">
         <v>41</v>
@@ -12621,11 +12621,11 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q141" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R141" t="n">
         <v>41</v>
@@ -12708,11 +12708,11 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q142" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R142" t="n">
         <v>41</v>
@@ -12795,11 +12795,11 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q143" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R143" t="n">
         <v>41</v>
@@ -12882,11 +12882,11 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q144" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R144" t="n">
         <v>41</v>
@@ -12969,11 +12969,11 @@
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q145" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R145" t="n">
         <v>41</v>
@@ -13054,11 +13054,11 @@
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q146" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R146" t="n">
         <v>41</v>
@@ -13141,11 +13141,11 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q147" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R147" t="n">
         <v>41</v>
@@ -13228,11 +13228,11 @@
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q148" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R148" t="n">
         <v>28</v>
@@ -13315,11 +13315,11 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q149" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R149" t="n">
         <v>28</v>
@@ -13402,11 +13402,11 @@
       </c>
       <c r="P150" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q150" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R150" t="n">
         <v>41</v>
@@ -13487,11 +13487,11 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q151" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R151" t="n">
         <v>21</v>
@@ -13572,11 +13572,11 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q152" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R152" t="n">
         <v>41</v>
@@ -13659,11 +13659,11 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q153" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R153" t="n">
         <v>41</v>
@@ -13746,11 +13746,11 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q154" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R154" t="n">
         <v>41</v>
@@ -13833,11 +13833,11 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q155" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R155" t="n">
         <v>28</v>
@@ -13920,11 +13920,11 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q156" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R156" t="n">
         <v>21</v>
@@ -14007,11 +14007,11 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q157" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R157" t="n">
         <v>28</v>
@@ -14094,11 +14094,11 @@
       </c>
       <c r="P158" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q158" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R158" t="n">
         <v>21</v>
@@ -14181,11 +14181,11 @@
       </c>
       <c r="P159" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q159" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R159" t="n">
         <v>21</v>
@@ -14268,11 +14268,11 @@
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q160" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R160" t="n">
         <v>28</v>
@@ -14355,11 +14355,11 @@
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q161" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R161" t="inlineStr"/>
       <c r="S161" t="n">
@@ -14440,11 +14440,11 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q162" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R162" t="n">
         <v>21</v>
@@ -14527,11 +14527,11 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q163" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R163" t="n">
         <v>21</v>
@@ -14614,11 +14614,11 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q164" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R164" t="inlineStr"/>
       <c r="S164" t="n">
@@ -14699,11 +14699,11 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q165" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R165" t="n">
         <v>21</v>
@@ -14786,11 +14786,11 @@
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q166" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R166" t="n">
         <v>41</v>
@@ -14873,11 +14873,11 @@
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q167" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R167" t="n">
         <v>21</v>
@@ -14960,11 +14960,11 @@
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q168" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R168" t="n">
         <v>28</v>
@@ -15047,11 +15047,11 @@
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q169" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R169" t="n">
         <v>41</v>
@@ -15111,10 +15111,10 @@
         <v>28</v>
       </c>
       <c r="J170" t="n">
-        <v>27</v>
+        <v>24.8</v>
       </c>
       <c r="K170" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
@@ -15134,17 +15134,17 @@
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q170" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R170" t="n">
         <v>28</v>
       </c>
       <c r="S170" t="n">
-        <v>-1</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T170" t="n">
         <v>26.4</v>
@@ -15221,11 +15221,11 @@
       </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q171" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R171" t="n">
         <v>41</v>
@@ -15308,11 +15308,11 @@
       </c>
       <c r="P172" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q172" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R172" t="n">
         <v>28</v>
@@ -15395,11 +15395,11 @@
       </c>
       <c r="P173" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q173" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R173" t="n">
         <v>21</v>
@@ -15482,11 +15482,11 @@
       </c>
       <c r="P174" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q174" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R174" t="n">
         <v>28</v>
@@ -15569,11 +15569,11 @@
       </c>
       <c r="P175" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q175" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R175" t="n">
         <v>28</v>
@@ -15656,11 +15656,11 @@
       </c>
       <c r="P176" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q176" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R176" t="n">
         <v>21</v>
@@ -15743,11 +15743,11 @@
       </c>
       <c r="P177" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q177" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R177" t="inlineStr"/>
       <c r="S177" t="n">
@@ -15828,11 +15828,11 @@
       </c>
       <c r="P178" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q178" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R178" t="n">
         <v>28</v>
@@ -15915,11 +15915,11 @@
       </c>
       <c r="P179" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q179" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R179" t="n">
         <v>41</v>
@@ -16002,11 +16002,11 @@
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q180" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R180" t="n">
         <v>21</v>
@@ -16089,11 +16089,11 @@
       </c>
       <c r="P181" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q181" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R181" t="n">
         <v>28</v>
@@ -16176,11 +16176,11 @@
       </c>
       <c r="P182" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q182" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R182" t="n">
         <v>21</v>
@@ -16263,11 +16263,11 @@
       </c>
       <c r="P183" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q183" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R183" t="n">
         <v>28</v>
@@ -16350,11 +16350,11 @@
       </c>
       <c r="P184" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q184" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R184" t="n">
         <v>28</v>
@@ -16437,11 +16437,11 @@
       </c>
       <c r="P185" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q185" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R185" t="n">
         <v>28</v>
@@ -16524,11 +16524,11 @@
       </c>
       <c r="P186" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q186" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R186" t="n">
         <v>41</v>
@@ -16611,11 +16611,11 @@
       </c>
       <c r="P187" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q187" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R187" t="n">
         <v>28</v>
@@ -16698,11 +16698,11 @@
       </c>
       <c r="P188" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q188" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R188" t="n">
         <v>41</v>
@@ -16783,11 +16783,11 @@
       </c>
       <c r="P189" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q189" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R189" t="n">
         <v>41</v>
@@ -16870,11 +16870,11 @@
       </c>
       <c r="P190" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q190" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R190" t="n">
         <v>21</v>
@@ -16957,11 +16957,11 @@
       </c>
       <c r="P191" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q191" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R191" t="inlineStr"/>
       <c r="S191" t="n">
@@ -17042,11 +17042,11 @@
       </c>
       <c r="P192" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q192" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R192" t="n">
         <v>21</v>
@@ -17106,10 +17106,10 @@
         <v>21</v>
       </c>
       <c r="J193" t="n">
-        <v>22.6</v>
+        <v>20.6</v>
       </c>
       <c r="K193" t="n">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="L193" t="inlineStr">
         <is>
@@ -17129,17 +17129,17 @@
       </c>
       <c r="P193" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q193" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R193" t="n">
         <v>21</v>
       </c>
       <c r="S193" t="n">
-        <v>1.600000000000001</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T193" t="n">
         <v>21.5</v>
@@ -17216,11 +17216,11 @@
       </c>
       <c r="P194" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q194" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R194" t="inlineStr"/>
       <c r="S194" t="n">
@@ -17301,11 +17301,11 @@
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q195" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R195" t="n">
         <v>21</v>
@@ -17388,11 +17388,11 @@
       </c>
       <c r="P196" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q196" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R196" t="n">
         <v>28</v>
@@ -17475,11 +17475,11 @@
       </c>
       <c r="P197" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q197" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R197" t="n">
         <v>21</v>
@@ -17562,11 +17562,11 @@
       </c>
       <c r="P198" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q198" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R198" t="n">
         <v>28</v>
@@ -17649,11 +17649,11 @@
       </c>
       <c r="P199" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q199" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R199" t="n">
         <v>21</v>
@@ -17736,11 +17736,11 @@
       </c>
       <c r="P200" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q200" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R200" t="n">
         <v>28</v>
@@ -17823,11 +17823,11 @@
       </c>
       <c r="P201" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q201" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R201" t="n">
         <v>21</v>
@@ -17910,11 +17910,11 @@
       </c>
       <c r="P202" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q202" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R202" t="n">
         <v>21</v>
@@ -17997,11 +17997,11 @@
       </c>
       <c r="P203" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q203" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R203" t="n">
         <v>28</v>
@@ -18061,10 +18061,10 @@
         <v>28</v>
       </c>
       <c r="J204" t="n">
-        <v>26.8</v>
+        <v>27.9</v>
       </c>
       <c r="K204" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L204" t="inlineStr">
         <is>
@@ -18084,17 +18084,17 @@
       </c>
       <c r="P204" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q204" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R204" t="n">
         <v>28</v>
       </c>
       <c r="S204" t="n">
-        <v>-1.199999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T204" t="n">
         <v>27.86666666666666</v>
@@ -18171,11 +18171,11 @@
       </c>
       <c r="P205" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q205" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R205" t="n">
         <v>28</v>
@@ -18258,11 +18258,11 @@
       </c>
       <c r="P206" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q206" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R206" t="n">
         <v>28</v>
@@ -18345,11 +18345,11 @@
       </c>
       <c r="P207" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q207" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R207" t="n">
         <v>28</v>
@@ -18432,11 +18432,11 @@
       </c>
       <c r="P208" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q208" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R208" t="n">
         <v>28</v>
@@ -18519,11 +18519,11 @@
       </c>
       <c r="P209" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q209" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R209" t="n">
         <v>28</v>
@@ -18583,10 +18583,10 @@
         <v>28</v>
       </c>
       <c r="J210" t="n">
-        <v>24.7</v>
+        <v>29.2</v>
       </c>
       <c r="K210" t="n">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="L210" t="inlineStr">
         <is>
@@ -18606,17 +18606,17 @@
       </c>
       <c r="P210" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q210" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R210" t="n">
         <v>28</v>
       </c>
       <c r="S210" t="n">
-        <v>-3.300000000000001</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="T210" t="n">
         <v>28.1</v>
@@ -18693,11 +18693,11 @@
       </c>
       <c r="P211" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q211" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R211" t="n">
         <v>21</v>
@@ -18780,11 +18780,11 @@
       </c>
       <c r="P212" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q212" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R212" t="n">
         <v>28</v>
@@ -18867,11 +18867,11 @@
       </c>
       <c r="P213" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q213" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R213" t="n">
         <v>28</v>
@@ -18954,11 +18954,11 @@
       </c>
       <c r="P214" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q214" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R214" t="inlineStr"/>
       <c r="S214" t="n">
@@ -19039,11 +19039,11 @@
       </c>
       <c r="P215" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q215" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R215" t="n">
         <v>28</v>
@@ -19126,11 +19126,11 @@
       </c>
       <c r="P216" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q216" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R216" t="n">
         <v>28</v>
@@ -19213,11 +19213,11 @@
       </c>
       <c r="P217" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q217" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R217" t="n">
         <v>28</v>
@@ -19300,11 +19300,11 @@
       </c>
       <c r="P218" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q218" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R218" t="n">
         <v>21</v>
@@ -19387,11 +19387,11 @@
       </c>
       <c r="P219" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q219" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R219" t="n">
         <v>21</v>
@@ -19474,11 +19474,11 @@
       </c>
       <c r="P220" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q220" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R220" t="n">
         <v>28</v>
@@ -19561,11 +19561,11 @@
       </c>
       <c r="P221" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q221" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R221" t="n">
         <v>28</v>
@@ -19648,11 +19648,11 @@
       </c>
       <c r="P222" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q222" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R222" t="n">
         <v>28</v>
@@ -19735,11 +19735,11 @@
       </c>
       <c r="P223" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q223" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R223" t="n">
         <v>28</v>
@@ -19822,11 +19822,11 @@
       </c>
       <c r="P224" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q224" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R224" t="n">
         <v>21</v>
@@ -19909,11 +19909,11 @@
       </c>
       <c r="P225" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q225" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R225" t="n">
         <v>21</v>
@@ -19996,11 +19996,11 @@
       </c>
       <c r="P226" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q226" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R226" t="n">
         <v>28</v>
@@ -20083,11 +20083,11 @@
       </c>
       <c r="P227" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q227" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R227" t="n">
         <v>28</v>
@@ -20170,11 +20170,11 @@
       </c>
       <c r="P228" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q228" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R228" t="n">
         <v>21</v>
@@ -20257,11 +20257,11 @@
       </c>
       <c r="P229" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q229" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R229" t="inlineStr"/>
       <c r="S229" t="n">
@@ -20342,11 +20342,11 @@
       </c>
       <c r="P230" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q230" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R230" t="n">
         <v>21</v>
@@ -20429,11 +20429,11 @@
       </c>
       <c r="P231" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q231" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R231" t="n">
         <v>28</v>
@@ -20493,10 +20493,10 @@
         <v>28</v>
       </c>
       <c r="J232" t="n">
-        <v>30.9</v>
+        <v>24.9</v>
       </c>
       <c r="K232" t="n">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="L232" t="inlineStr">
         <is>
@@ -20516,17 +20516,17 @@
       </c>
       <c r="P232" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q232" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R232" t="n">
         <v>28</v>
       </c>
       <c r="S232" t="n">
-        <v>2.899999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T232" t="n">
         <v>27.93333333333333</v>
@@ -20603,11 +20603,11 @@
       </c>
       <c r="P233" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q233" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R233" t="inlineStr"/>
       <c r="S233" t="n">
@@ -20688,11 +20688,11 @@
       </c>
       <c r="P234" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q234" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R234" t="n">
         <v>48</v>
@@ -20775,11 +20775,11 @@
       </c>
       <c r="P235" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q235" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R235" t="inlineStr"/>
       <c r="S235" t="n">
@@ -20860,11 +20860,11 @@
       </c>
       <c r="P236" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q236" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R236" t="n">
         <v>28</v>
@@ -20947,11 +20947,11 @@
       </c>
       <c r="P237" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q237" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R237" t="n">
         <v>28</v>
@@ -21034,11 +21034,11 @@
       </c>
       <c r="P238" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q238" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R238" t="n">
         <v>28</v>
@@ -21121,11 +21121,11 @@
       </c>
       <c r="P239" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q239" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R239" t="inlineStr"/>
       <c r="S239" t="n">
@@ -21206,11 +21206,11 @@
       </c>
       <c r="P240" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q240" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R240" t="n">
         <v>48</v>
@@ -21293,11 +21293,11 @@
       </c>
       <c r="P241" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q241" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R241" t="n">
         <v>28</v>
@@ -21380,11 +21380,11 @@
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q242" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R242" t="n">
         <v>21</v>
@@ -21467,11 +21467,11 @@
       </c>
       <c r="P243" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q243" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R243" t="n">
         <v>28</v>
@@ -21554,11 +21554,11 @@
       </c>
       <c r="P244" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="Q244" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="R244" t="inlineStr"/>
       <c r="S244" t="n">

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-19 15:26:44
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3843,10 +3843,10 @@
         <v>24</v>
       </c>
       <c r="J40" t="n">
-        <v>16.2</v>
+        <v>15.7</v>
       </c>
       <c r="K40" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -3876,7 +3876,7 @@
         <v>28</v>
       </c>
       <c r="S40" t="n">
-        <v>-7.800000000000001</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="T40" t="n">
         <v>16.5</v>
@@ -4533,10 +4533,10 @@
         <v>24</v>
       </c>
       <c r="J48" t="n">
-        <v>25.9</v>
+        <v>22.1</v>
       </c>
       <c r="K48" t="n">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v>28</v>
       </c>
       <c r="S48" t="n">
-        <v>1.899999999999999</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="T48" t="n">
         <v>24.23333333333333</v>
@@ -5397,10 +5397,10 @@
         <v>31</v>
       </c>
       <c r="J58" t="n">
-        <v>35.8</v>
+        <v>31.4</v>
       </c>
       <c r="K58" t="n">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
       </c>
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="n">
-        <v>4.799999999999997</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T58" t="n">
-        <v>30.66666666666667</v>
+        <v>30.66666666666666</v>
       </c>
       <c r="U58" t="n">
         <v>3</v>
@@ -5917,10 +5917,10 @@
         <v>28</v>
       </c>
       <c r="J64" t="n">
-        <v>30.5</v>
+        <v>27.9</v>
       </c>
       <c r="K64" t="n">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -5950,7 +5950,7 @@
         <v>28</v>
       </c>
       <c r="S64" t="n">
-        <v>2.5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T64" t="n">
         <v>29.13333333333334</v>
@@ -6091,10 +6091,10 @@
         <v>21</v>
       </c>
       <c r="J66" t="n">
-        <v>20.1</v>
+        <v>19.7</v>
       </c>
       <c r="K66" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -6124,7 +6124,7 @@
         <v>21</v>
       </c>
       <c r="S66" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T66" t="n">
         <v>20.03333333333333</v>
@@ -6613,10 +6613,10 @@
         <v>21</v>
       </c>
       <c r="J72" t="n">
-        <v>19.8</v>
+        <v>24.6</v>
       </c>
       <c r="K72" t="n">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -6646,7 +6646,7 @@
         <v>21</v>
       </c>
       <c r="S72" t="n">
-        <v>-1.199999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T72" t="n">
         <v>22.76666666666667</v>
@@ -7133,10 +7133,10 @@
         <v>28</v>
       </c>
       <c r="J78" t="n">
-        <v>30.7</v>
+        <v>29.2</v>
       </c>
       <c r="K78" t="n">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
         <v>28</v>
       </c>
       <c r="S78" t="n">
-        <v>2.699999999999999</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="T78" t="n">
         <v>29.2</v>
@@ -7479,10 +7479,10 @@
         <v>21</v>
       </c>
       <c r="J82" t="n">
-        <v>21.2</v>
+        <v>20.2</v>
       </c>
       <c r="K82" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -7512,7 +7512,7 @@
         <v>21</v>
       </c>
       <c r="S82" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T82" t="n">
         <v>22.16666666666667</v>
@@ -8086,10 +8086,10 @@
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>39.1</v>
+        <v>36.7</v>
       </c>
       <c r="K89" t="n">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8119,16 +8119,16 @@
         <v>41</v>
       </c>
       <c r="S89" t="n">
-        <v>4.100000000000001</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T89" t="n">
-        <v>35.73333333333334</v>
+        <v>35.73333333333333</v>
       </c>
       <c r="U89" t="n">
         <v>3</v>
       </c>
       <c r="V89" t="n">
-        <v>35.86296296296297</v>
+        <v>35.86296296296296</v>
       </c>
       <c r="W89" t="n">
         <v>31.5</v>
@@ -9816,10 +9816,10 @@
         <v>35</v>
       </c>
       <c r="J109" t="n">
-        <v>27.1</v>
+        <v>29.6</v>
       </c>
       <c r="K109" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -9849,7 +9849,7 @@
         <v>41</v>
       </c>
       <c r="S109" t="n">
-        <v>-7.899999999999999</v>
+        <v>-5.399999999999999</v>
       </c>
       <c r="T109" t="n">
         <v>27.33333333333333</v>
@@ -10164,10 +10164,10 @@
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="K113" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         <v>41</v>
       </c>
       <c r="S113" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="T113" t="n">
         <v>25.5</v>
@@ -10599,10 +10599,10 @@
         <v>35</v>
       </c>
       <c r="J118" t="n">
-        <v>34.9</v>
+        <v>37.4</v>
       </c>
       <c r="K118" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -10632,7 +10632,7 @@
         <v>41</v>
       </c>
       <c r="S118" t="n">
-        <v>-0.1000000000000014</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T118" t="n">
         <v>35.63333333333333</v>
@@ -11208,10 +11208,10 @@
         <v>35</v>
       </c>
       <c r="J125" t="n">
-        <v>30.5</v>
+        <v>35.4</v>
       </c>
       <c r="K125" t="n">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -11241,7 +11241,7 @@
         <v>41</v>
       </c>
       <c r="S125" t="n">
-        <v>-4.5</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T125" t="n">
         <v>34.13333333333333</v>
@@ -11382,10 +11382,10 @@
         <v>28</v>
       </c>
       <c r="J127" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="K127" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
@@ -11415,7 +11415,7 @@
         <v>28</v>
       </c>
       <c r="S127" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="T127" t="n">
         <v>25.36666666666666</v>
@@ -16675,10 +16675,10 @@
         <v>35</v>
       </c>
       <c r="J188" t="n">
-        <v>43.4</v>
+        <v>26.1</v>
       </c>
       <c r="K188" t="n">
-        <v>124</v>
+        <v>74</v>
       </c>
       <c r="L188" t="inlineStr">
         <is>
@@ -16708,7 +16708,7 @@
         <v>41</v>
       </c>
       <c r="S188" t="n">
-        <v>8.399999999999999</v>
+        <v>-8.899999999999999</v>
       </c>
       <c r="T188" t="n">
         <v>33.26666666666667</v>
@@ -16847,10 +16847,10 @@
         <v>21</v>
       </c>
       <c r="J190" t="n">
-        <v>21.2</v>
+        <v>22</v>
       </c>
       <c r="K190" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="L190" t="inlineStr">
         <is>
@@ -16880,7 +16880,7 @@
         <v>21</v>
       </c>
       <c r="S190" t="n">
-        <v>0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="T190" t="n">
         <v>21.2</v>
@@ -17019,10 +17019,10 @@
         <v>21</v>
       </c>
       <c r="J192" t="n">
-        <v>23</v>
+        <v>20.7</v>
       </c>
       <c r="K192" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="L192" t="inlineStr">
         <is>
@@ -17052,7 +17052,7 @@
         <v>21</v>
       </c>
       <c r="S192" t="n">
-        <v>2</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T192" t="n">
         <v>21.5</v>
@@ -17800,10 +17800,10 @@
         <v>21</v>
       </c>
       <c r="J201" t="n">
-        <v>21.4</v>
+        <v>20.8</v>
       </c>
       <c r="K201" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L201" t="inlineStr">
         <is>
@@ -17833,7 +17833,7 @@
         <v>21</v>
       </c>
       <c r="S201" t="n">
-        <v>0.3999999999999986</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T201" t="n">
         <v>21.16666666666667</v>
@@ -17887,10 +17887,10 @@
         <v>21</v>
       </c>
       <c r="J202" t="n">
-        <v>20.7</v>
+        <v>23.1</v>
       </c>
       <c r="K202" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="L202" t="inlineStr">
         <is>
@@ -17920,7 +17920,7 @@
         <v>21</v>
       </c>
       <c r="S202" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="T202" t="n">
         <v>22.13333333333334</v>
@@ -17929,7 +17929,7 @@
         <v>3</v>
       </c>
       <c r="V202" t="n">
-        <v>24.33333333333334</v>
+        <v>24.33333333333333</v>
       </c>
       <c r="W202" t="n">
         <v>17.5</v>
@@ -17974,10 +17974,10 @@
         <v>24</v>
       </c>
       <c r="J203" t="n">
-        <v>20.4</v>
+        <v>21.6</v>
       </c>
       <c r="K203" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="L203" t="inlineStr">
         <is>
@@ -18007,7 +18007,7 @@
         <v>28</v>
       </c>
       <c r="S203" t="n">
-        <v>-3.600000000000001</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="T203" t="n">
         <v>22.5</v>
@@ -18061,10 +18061,10 @@
         <v>28</v>
       </c>
       <c r="J204" t="n">
-        <v>27.9</v>
+        <v>26.8</v>
       </c>
       <c r="K204" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L204" t="inlineStr">
         <is>
@@ -18094,7 +18094,7 @@
         <v>28</v>
       </c>
       <c r="S204" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T204" t="n">
         <v>27.86666666666666</v>
@@ -18148,10 +18148,10 @@
         <v>28</v>
       </c>
       <c r="J205" t="n">
-        <v>27.7</v>
+        <v>26.1</v>
       </c>
       <c r="K205" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="L205" t="inlineStr">
         <is>
@@ -18181,7 +18181,7 @@
         <v>28</v>
       </c>
       <c r="S205" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="T205" t="n">
         <v>27.5</v>
@@ -18235,10 +18235,10 @@
         <v>28</v>
       </c>
       <c r="J206" t="n">
-        <v>28.9</v>
+        <v>27.7</v>
       </c>
       <c r="K206" t="n">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="L206" t="inlineStr">
         <is>
@@ -18268,7 +18268,7 @@
         <v>28</v>
       </c>
       <c r="S206" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T206" t="n">
         <v>28.4</v>
@@ -18322,10 +18322,10 @@
         <v>28</v>
       </c>
       <c r="J207" t="n">
-        <v>25.7</v>
+        <v>29.1</v>
       </c>
       <c r="K207" t="n">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="L207" t="inlineStr">
         <is>
@@ -18355,7 +18355,7 @@
         <v>28</v>
       </c>
       <c r="S207" t="n">
-        <v>-2.300000000000001</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T207" t="n">
         <v>27.53333333333333</v>
@@ -18409,10 +18409,10 @@
         <v>28</v>
       </c>
       <c r="J208" t="n">
-        <v>30.7</v>
+        <v>26.9</v>
       </c>
       <c r="K208" t="n">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="L208" t="inlineStr">
         <is>
@@ -18442,7 +18442,7 @@
         <v>28</v>
       </c>
       <c r="S208" t="n">
-        <v>2.699999999999999</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="T208" t="n">
         <v>28.46666666666667</v>
@@ -18496,10 +18496,10 @@
         <v>28</v>
       </c>
       <c r="J209" t="n">
-        <v>32.6</v>
+        <v>26.2</v>
       </c>
       <c r="K209" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="L209" t="inlineStr">
         <is>
@@ -18529,7 +18529,7 @@
         <v>28</v>
       </c>
       <c r="S209" t="n">
-        <v>4.600000000000001</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="T209" t="n">
         <v>30.03333333333333</v>
@@ -18583,10 +18583,10 @@
         <v>28</v>
       </c>
       <c r="J210" t="n">
-        <v>29.2</v>
+        <v>24.7</v>
       </c>
       <c r="K210" t="n">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="L210" t="inlineStr">
         <is>
@@ -18616,7 +18616,7 @@
         <v>28</v>
       </c>
       <c r="S210" t="n">
-        <v>1.199999999999999</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="T210" t="n">
         <v>28.1</v>
@@ -18670,10 +18670,10 @@
         <v>21</v>
       </c>
       <c r="J211" t="n">
-        <v>20.5</v>
+        <v>22.8</v>
       </c>
       <c r="K211" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="L211" t="inlineStr">
         <is>
@@ -18703,7 +18703,7 @@
         <v>21</v>
       </c>
       <c r="S211" t="n">
-        <v>-0.5</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="T211" t="n">
         <v>22.36666666666666</v>
@@ -18757,10 +18757,10 @@
         <v>28</v>
       </c>
       <c r="J212" t="n">
-        <v>26.6</v>
+        <v>28.6</v>
       </c>
       <c r="K212" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="L212" t="inlineStr">
         <is>
@@ -18790,7 +18790,7 @@
         <v>28</v>
       </c>
       <c r="S212" t="n">
-        <v>-1.399999999999999</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T212" t="n">
         <v>26.83333333333333</v>
@@ -18844,10 +18844,10 @@
         <v>28</v>
       </c>
       <c r="J213" t="n">
-        <v>27.4</v>
+        <v>24.5</v>
       </c>
       <c r="K213" t="n">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="L213" t="inlineStr">
         <is>
@@ -18877,7 +18877,7 @@
         <v>28</v>
       </c>
       <c r="S213" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-3.5</v>
       </c>
       <c r="T213" t="n">
         <v>26.16666666666667</v>
@@ -19016,10 +19016,10 @@
         <v>28</v>
       </c>
       <c r="J215" t="n">
-        <v>25.4</v>
+        <v>30.3</v>
       </c>
       <c r="K215" t="n">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="L215" t="inlineStr">
         <is>
@@ -19049,7 +19049,7 @@
         <v>28</v>
       </c>
       <c r="S215" t="n">
-        <v>-2.600000000000001</v>
+        <v>2.300000000000001</v>
       </c>
       <c r="T215" t="n">
         <v>28.86666666666666</v>
@@ -19190,10 +19190,10 @@
         <v>28</v>
       </c>
       <c r="J217" t="n">
-        <v>27.7</v>
+        <v>28.7</v>
       </c>
       <c r="K217" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="L217" t="inlineStr">
         <is>
@@ -19223,7 +19223,7 @@
         <v>28</v>
       </c>
       <c r="S217" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T217" t="n">
         <v>28.13333333333334</v>
@@ -19277,10 +19277,10 @@
         <v>21</v>
       </c>
       <c r="J218" t="n">
-        <v>20.5</v>
+        <v>15.3</v>
       </c>
       <c r="K218" t="n">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="L218" t="inlineStr">
         <is>
@@ -19310,7 +19310,7 @@
         <v>21</v>
       </c>
       <c r="S218" t="n">
-        <v>-0.5</v>
+        <v>-5.699999999999999</v>
       </c>
       <c r="T218" t="n">
         <v>18.26666666666667</v>
@@ -19364,10 +19364,10 @@
         <v>21</v>
       </c>
       <c r="J219" t="n">
-        <v>11.6</v>
+        <v>19.6</v>
       </c>
       <c r="K219" t="n">
-        <v>55</v>
+        <v>93</v>
       </c>
       <c r="L219" t="inlineStr">
         <is>
@@ -19397,7 +19397,7 @@
         <v>21</v>
       </c>
       <c r="S219" t="n">
-        <v>-9.4</v>
+        <v>-1.399999999999999</v>
       </c>
       <c r="T219" t="n">
         <v>16.96666666666667</v>
@@ -19406,7 +19406,7 @@
         <v>3</v>
       </c>
       <c r="V219" t="n">
-        <v>19.75555555555555</v>
+        <v>19.75555555555556</v>
       </c>
       <c r="W219" t="n">
         <v>17.5</v>
@@ -19451,10 +19451,10 @@
         <v>28</v>
       </c>
       <c r="J220" t="n">
-        <v>27.8</v>
+        <v>25.7</v>
       </c>
       <c r="K220" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="L220" t="inlineStr">
         <is>
@@ -19484,7 +19484,7 @@
         <v>28</v>
       </c>
       <c r="S220" t="n">
-        <v>-0.1999999999999993</v>
+        <v>-2.300000000000001</v>
       </c>
       <c r="T220" t="n">
         <v>27.66666666666667</v>
@@ -19538,10 +19538,10 @@
         <v>28</v>
       </c>
       <c r="J221" t="n">
-        <v>27.2</v>
+        <v>14.6</v>
       </c>
       <c r="K221" t="n">
-        <v>97</v>
+        <v>52</v>
       </c>
       <c r="L221" t="inlineStr">
         <is>
@@ -19571,7 +19571,7 @@
         <v>28</v>
       </c>
       <c r="S221" t="n">
-        <v>-0.8000000000000007</v>
+        <v>-13.4</v>
       </c>
       <c r="T221" t="n">
         <v>23.53333333333333</v>
@@ -19625,10 +19625,10 @@
         <v>28</v>
       </c>
       <c r="J222" t="n">
-        <v>29.8</v>
+        <v>25.6</v>
       </c>
       <c r="K222" t="n">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="L222" t="inlineStr">
         <is>
@@ -19658,7 +19658,7 @@
         <v>28</v>
       </c>
       <c r="S222" t="n">
-        <v>1.800000000000001</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="T222" t="n">
         <v>25.9</v>
@@ -19712,10 +19712,10 @@
         <v>28</v>
       </c>
       <c r="J223" t="n">
-        <v>27.3</v>
+        <v>26.7</v>
       </c>
       <c r="K223" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L223" t="inlineStr">
         <is>
@@ -19745,7 +19745,7 @@
         <v>28</v>
       </c>
       <c r="S223" t="n">
-        <v>-0.6999999999999993</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T223" t="n">
         <v>28.56666666666667</v>
@@ -19799,10 +19799,10 @@
         <v>21</v>
       </c>
       <c r="J224" t="n">
-        <v>19.5</v>
+        <v>20.3</v>
       </c>
       <c r="K224" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="L224" t="inlineStr">
         <is>
@@ -19832,7 +19832,7 @@
         <v>21</v>
       </c>
       <c r="S224" t="n">
-        <v>-1.5</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T224" t="n">
         <v>20.3</v>
@@ -19886,10 +19886,10 @@
         <v>21</v>
       </c>
       <c r="J225" t="n">
-        <v>22.5</v>
+        <v>22.6</v>
       </c>
       <c r="K225" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L225" t="inlineStr">
         <is>
@@ -19919,7 +19919,7 @@
         <v>21</v>
       </c>
       <c r="S225" t="n">
-        <v>1.5</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T225" t="n">
         <v>21.96666666666667</v>
@@ -27767,10 +27767,10 @@
         <v>24.5</v>
       </c>
       <c r="J316" t="n">
-        <v>30.6</v>
+        <v>23.5</v>
       </c>
       <c r="K316" t="n">
-        <v>125</v>
+        <v>96</v>
       </c>
       <c r="L316" t="inlineStr">
         <is>
@@ -27800,7 +27800,7 @@
         <v>28</v>
       </c>
       <c r="S316" t="n">
-        <v>6.100000000000001</v>
+        <v>-1</v>
       </c>
       <c r="T316" t="n">
         <v>27.7</v>
@@ -27854,10 +27854,10 @@
         <v>24.5</v>
       </c>
       <c r="J317" t="n">
-        <v>20.9</v>
+        <v>24.6</v>
       </c>
       <c r="K317" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="L317" t="inlineStr">
         <is>
@@ -27887,7 +27887,7 @@
         <v>28</v>
       </c>
       <c r="S317" t="n">
-        <v>-3.600000000000001</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T317" t="n">
         <v>23.96666666666667</v>
@@ -29768,10 +29768,10 @@
         <v>24.5</v>
       </c>
       <c r="J339" t="n">
-        <v>14</v>
+        <v>24.8</v>
       </c>
       <c r="K339" t="n">
-        <v>57</v>
+        <v>101</v>
       </c>
       <c r="L339" t="inlineStr">
         <is>
@@ -29801,7 +29801,7 @@
         <v>28</v>
       </c>
       <c r="S339" t="n">
-        <v>-10.5</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="T339" t="n">
         <v>21.96666666666667</v>
@@ -31504,10 +31504,10 @@
         <v>24.5</v>
       </c>
       <c r="J359" t="n">
-        <v>27.4</v>
+        <v>23.2</v>
       </c>
       <c r="K359" t="n">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -31537,7 +31537,7 @@
         <v>28</v>
       </c>
       <c r="S359" t="n">
-        <v>2.899999999999999</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T359" t="n">
         <v>24.7</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-19 17:19:40
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3843,10 +3843,10 @@
         <v>24</v>
       </c>
       <c r="J40" t="n">
-        <v>15.7</v>
+        <v>16.2</v>
       </c>
       <c r="K40" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -3876,7 +3876,7 @@
         <v>28</v>
       </c>
       <c r="S40" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.800000000000001</v>
       </c>
       <c r="T40" t="n">
         <v>16.5</v>
@@ -4794,10 +4794,10 @@
         <v>31</v>
       </c>
       <c r="J51" t="n">
-        <v>34.5</v>
+        <v>28.3</v>
       </c>
       <c r="K51" t="n">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="n">
-        <v>3.5</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="T51" t="n">
         <v>31.46666666666667</v>
@@ -5917,10 +5917,10 @@
         <v>28</v>
       </c>
       <c r="J64" t="n">
-        <v>27.9</v>
+        <v>30.5</v>
       </c>
       <c r="K64" t="n">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -5950,7 +5950,7 @@
         <v>28</v>
       </c>
       <c r="S64" t="n">
-        <v>-0.1000000000000014</v>
+        <v>2.5</v>
       </c>
       <c r="T64" t="n">
         <v>29.13333333333334</v>
@@ -7133,10 +7133,10 @@
         <v>28</v>
       </c>
       <c r="J78" t="n">
-        <v>29.2</v>
+        <v>30.7</v>
       </c>
       <c r="K78" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
         <v>28</v>
       </c>
       <c r="S78" t="n">
-        <v>1.199999999999999</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="T78" t="n">
         <v>29.2</v>
@@ -7479,10 +7479,10 @@
         <v>21</v>
       </c>
       <c r="J82" t="n">
-        <v>20.2</v>
+        <v>21.2</v>
       </c>
       <c r="K82" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -7512,7 +7512,7 @@
         <v>21</v>
       </c>
       <c r="S82" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T82" t="n">
         <v>22.16666666666667</v>
@@ -9816,10 +9816,10 @@
         <v>35</v>
       </c>
       <c r="J109" t="n">
-        <v>29.6</v>
+        <v>27.1</v>
       </c>
       <c r="K109" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -9849,7 +9849,7 @@
         <v>41</v>
       </c>
       <c r="S109" t="n">
-        <v>-5.399999999999999</v>
+        <v>-7.899999999999999</v>
       </c>
       <c r="T109" t="n">
         <v>27.33333333333333</v>
@@ -10164,10 +10164,10 @@
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>27.7</v>
+        <v>22.5</v>
       </c>
       <c r="K113" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         <v>41</v>
       </c>
       <c r="S113" t="n">
-        <v>-7.300000000000001</v>
+        <v>-12.5</v>
       </c>
       <c r="T113" t="n">
         <v>25.5</v>
@@ -10251,10 +10251,10 @@
         <v>28</v>
       </c>
       <c r="J114" t="n">
-        <v>32.7</v>
+        <v>29.7</v>
       </c>
       <c r="K114" t="n">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -10284,7 +10284,7 @@
         <v>28</v>
       </c>
       <c r="S114" t="n">
-        <v>4.700000000000003</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="T114" t="n">
         <v>29.6</v>
@@ -10338,10 +10338,10 @@
         <v>35</v>
       </c>
       <c r="J115" t="n">
-        <v>22.7</v>
+        <v>24.2</v>
       </c>
       <c r="K115" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="L115" t="inlineStr">
         <is>
@@ -10371,7 +10371,7 @@
         <v>41</v>
       </c>
       <c r="S115" t="n">
-        <v>-12.3</v>
+        <v>-10.8</v>
       </c>
       <c r="T115" t="n">
         <v>23.13333333333334</v>
@@ -11208,10 +11208,10 @@
         <v>35</v>
       </c>
       <c r="J125" t="n">
-        <v>35.4</v>
+        <v>30.5</v>
       </c>
       <c r="K125" t="n">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -11241,7 +11241,7 @@
         <v>41</v>
       </c>
       <c r="S125" t="n">
-        <v>0.3999999999999986</v>
+        <v>-4.5</v>
       </c>
       <c r="T125" t="n">
         <v>34.13333333333333</v>
@@ -11382,10 +11382,10 @@
         <v>28</v>
       </c>
       <c r="J127" t="n">
-        <v>24.6</v>
+        <v>27.7</v>
       </c>
       <c r="K127" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="L127" t="inlineStr">
         <is>
@@ -11415,7 +11415,7 @@
         <v>28</v>
       </c>
       <c r="S127" t="n">
-        <v>-3.399999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T127" t="n">
         <v>25.36666666666666</v>
@@ -17974,10 +17974,10 @@
         <v>24</v>
       </c>
       <c r="J203" t="n">
-        <v>21.6</v>
+        <v>20.4</v>
       </c>
       <c r="K203" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="L203" t="inlineStr">
         <is>
@@ -18007,7 +18007,7 @@
         <v>28</v>
       </c>
       <c r="S203" t="n">
-        <v>-2.399999999999999</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="T203" t="n">
         <v>22.5</v>
@@ -29333,10 +29333,10 @@
         <v>24.5</v>
       </c>
       <c r="J334" t="n">
-        <v>24.3</v>
+        <v>24.4</v>
       </c>
       <c r="K334" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L334" t="inlineStr">
         <is>
@@ -29366,7 +29366,7 @@
         <v>28</v>
       </c>
       <c r="S334" t="n">
-        <v>-0.1999999999999993</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T334" t="n">
         <v>24.26666666666667</v>
@@ -29768,10 +29768,10 @@
         <v>24.5</v>
       </c>
       <c r="J339" t="n">
-        <v>24.8</v>
+        <v>14</v>
       </c>
       <c r="K339" t="n">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="L339" t="inlineStr">
         <is>
@@ -29801,7 +29801,7 @@
         <v>28</v>
       </c>
       <c r="S339" t="n">
-        <v>0.3000000000000007</v>
+        <v>-10.5</v>
       </c>
       <c r="T339" t="n">
         <v>21.96666666666667</v>
@@ -31504,10 +31504,10 @@
         <v>24.5</v>
       </c>
       <c r="J359" t="n">
-        <v>23.2</v>
+        <v>27.4</v>
       </c>
       <c r="K359" t="n">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -31537,7 +31537,7 @@
         <v>28</v>
       </c>
       <c r="S359" t="n">
-        <v>-1.300000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="T359" t="n">
         <v>24.7</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-19 18:31:18
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4794,10 +4794,10 @@
         <v>31</v>
       </c>
       <c r="J51" t="n">
-        <v>28.3</v>
+        <v>34.5</v>
       </c>
       <c r="K51" t="n">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="n">
-        <v>-2.699999999999999</v>
+        <v>3.5</v>
       </c>
       <c r="T51" t="n">
         <v>31.46666666666667</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="K75" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -6959,10 +6959,10 @@
         <v>28</v>
       </c>
       <c r="J76" t="n">
-        <v>24.1</v>
+        <v>27.3</v>
       </c>
       <c r="K76" t="n">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -6992,7 +6992,7 @@
         <v>28</v>
       </c>
       <c r="S76" t="n">
-        <v>-3.899999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T76" t="n">
         <v>25.33333333333333</v>
@@ -7046,7 +7046,7 @@
         <v>28</v>
       </c>
       <c r="J77" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="K77" t="n">
         <v>88</v>
@@ -7079,10 +7079,10 @@
         <v>28</v>
       </c>
       <c r="S77" t="n">
-        <v>-3.199999999999999</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="T77" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="U77" t="n">
         <v>3</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="K79" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="K86" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="K91" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -10251,10 +10251,10 @@
         <v>28</v>
       </c>
       <c r="J114" t="n">
-        <v>29.7</v>
+        <v>32.7</v>
       </c>
       <c r="K114" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="L114" t="inlineStr">
         <is>
@@ -10284,7 +10284,7 @@
         <v>28</v>
       </c>
       <c r="S114" t="n">
-        <v>1.699999999999999</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="T114" t="n">
         <v>29.6</v>
@@ -10338,10 +10338,10 @@
         <v>35</v>
       </c>
       <c r="J115" t="n">
-        <v>24.2</v>
+        <v>22.7</v>
       </c>
       <c r="K115" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="L115" t="inlineStr">
         <is>
@@ -10371,7 +10371,7 @@
         <v>41</v>
       </c>
       <c r="S115" t="n">
-        <v>-10.8</v>
+        <v>-12.3</v>
       </c>
       <c r="T115" t="n">
         <v>23.13333333333334</v>
@@ -21788,10 +21788,10 @@
         <v>21</v>
       </c>
       <c r="J247" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="K247" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L247" t="inlineStr">
         <is>
@@ -21821,7 +21821,7 @@
         <v>21</v>
       </c>
       <c r="S247" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T247" t="n">
         <v>21.2</v>
@@ -27245,10 +27245,10 @@
         <v>24.5</v>
       </c>
       <c r="J310" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="K310" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -27278,7 +27278,7 @@
         <v>28</v>
       </c>
       <c r="S310" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T310" t="n">
         <v>25.13333333333334</v>
@@ -27332,10 +27332,10 @@
         <v>24.5</v>
       </c>
       <c r="J311" t="n">
-        <v>22.5</v>
+        <v>20.7</v>
       </c>
       <c r="K311" t="n">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="L311" t="inlineStr">
         <is>
@@ -27365,7 +27365,7 @@
         <v>28</v>
       </c>
       <c r="S311" t="n">
-        <v>-2</v>
+        <v>-3.800000000000001</v>
       </c>
       <c r="T311" t="n">
         <v>21.53333333333333</v>
@@ -29333,10 +29333,10 @@
         <v>24.5</v>
       </c>
       <c r="J334" t="n">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
       <c r="K334" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L334" t="inlineStr">
         <is>
@@ -29366,7 +29366,7 @@
         <v>28</v>
       </c>
       <c r="S334" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T334" t="n">
         <v>24.26666666666667</v>
@@ -29420,10 +29420,10 @@
         <v>24.5</v>
       </c>
       <c r="J335" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="K335" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="L335" t="inlineStr">
         <is>
@@ -29453,7 +29453,7 @@
         <v>28</v>
       </c>
       <c r="S335" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T335" t="n">
         <v>35.8</v>
@@ -31591,10 +31591,10 @@
         <v>24.5</v>
       </c>
       <c r="J360" t="n">
-        <v>28.6</v>
+        <v>25.1</v>
       </c>
       <c r="K360" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31624,7 +31624,7 @@
         <v>28</v>
       </c>
       <c r="S360" t="n">
-        <v>4.100000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T360" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-19 19:56:20
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3074,7 +3074,7 @@
         <v>31</v>
       </c>
       <c r="J31" t="n">
-        <v>28.7</v>
+        <v>28.8</v>
       </c>
       <c r="K31" t="n">
         <v>93</v>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="n">
-        <v>-2.300000000000001</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="T31" t="n">
         <v>28.36666666666666</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K75" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -6959,10 +6959,10 @@
         <v>28</v>
       </c>
       <c r="J76" t="n">
-        <v>27.3</v>
+        <v>24.1</v>
       </c>
       <c r="K76" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -6992,7 +6992,7 @@
         <v>28</v>
       </c>
       <c r="S76" t="n">
-        <v>-0.6999999999999993</v>
+        <v>-3.899999999999999</v>
       </c>
       <c r="T76" t="n">
         <v>25.33333333333333</v>
@@ -7046,7 +7046,7 @@
         <v>28</v>
       </c>
       <c r="J77" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="K77" t="n">
         <v>88</v>
@@ -7079,10 +7079,10 @@
         <v>28</v>
       </c>
       <c r="S77" t="n">
-        <v>-3.300000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T77" t="n">
-        <v>25.13333333333333</v>
+        <v>25.13333333333334</v>
       </c>
       <c r="U77" t="n">
         <v>3</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K79" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K86" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K91" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -14158,10 +14158,10 @@
         <v>21</v>
       </c>
       <c r="J159" t="n">
-        <v>20.8</v>
+        <v>26.4</v>
       </c>
       <c r="K159" t="n">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="L159" t="inlineStr">
         <is>
@@ -14191,7 +14191,7 @@
         <v>21</v>
       </c>
       <c r="S159" t="n">
-        <v>-0.1999999999999993</v>
+        <v>5.399999999999999</v>
       </c>
       <c r="T159" t="n">
         <v>24.5</v>
@@ -18061,10 +18061,10 @@
         <v>28</v>
       </c>
       <c r="J204" t="n">
-        <v>26.8</v>
+        <v>27.9</v>
       </c>
       <c r="K204" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L204" t="inlineStr">
         <is>
@@ -18094,7 +18094,7 @@
         <v>28</v>
       </c>
       <c r="S204" t="n">
-        <v>-1.199999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T204" t="n">
         <v>27.86666666666666</v>
@@ -19973,10 +19973,10 @@
         <v>28</v>
       </c>
       <c r="J226" t="n">
-        <v>25</v>
+        <v>22.8</v>
       </c>
       <c r="K226" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="L226" t="inlineStr">
         <is>
@@ -20006,7 +20006,7 @@
         <v>28</v>
       </c>
       <c r="S226" t="n">
-        <v>-3</v>
+        <v>-5.199999999999999</v>
       </c>
       <c r="T226" t="n">
         <v>24.76666666666667</v>
@@ -20319,10 +20319,10 @@
         <v>21</v>
       </c>
       <c r="J230" t="n">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="K230" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L230" t="inlineStr">
         <is>
@@ -20352,7 +20352,7 @@
         <v>21</v>
       </c>
       <c r="S230" t="n">
-        <v>1.800000000000001</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="T230" t="n">
         <v>21.56666666666667</v>
@@ -21788,10 +21788,10 @@
         <v>21</v>
       </c>
       <c r="J247" t="n">
-        <v>21.2</v>
+        <v>21.5</v>
       </c>
       <c r="K247" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L247" t="inlineStr">
         <is>
@@ -21821,7 +21821,7 @@
         <v>21</v>
       </c>
       <c r="S247" t="n">
-        <v>0.1999999999999993</v>
+        <v>0.5</v>
       </c>
       <c r="T247" t="n">
         <v>21.2</v>
@@ -22215,10 +22215,10 @@
         <v>21</v>
       </c>
       <c r="J252" t="n">
-        <v>22.3</v>
+        <v>23.1</v>
       </c>
       <c r="K252" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="L252" t="inlineStr">
         <is>
@@ -22248,7 +22248,7 @@
         <v>21</v>
       </c>
       <c r="S252" t="n">
-        <v>1.300000000000001</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="T252" t="n">
         <v>21.8</v>
@@ -22389,10 +22389,10 @@
         <v>28</v>
       </c>
       <c r="J254" t="n">
-        <v>27.7</v>
+        <v>26.8</v>
       </c>
       <c r="K254" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L254" t="inlineStr">
         <is>
@@ -22422,7 +22422,7 @@
         <v>28</v>
       </c>
       <c r="S254" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T254" t="n">
         <v>27.16666666666667</v>
@@ -23172,10 +23172,10 @@
         <v>28</v>
       </c>
       <c r="J263" t="n">
-        <v>28.7</v>
+        <v>23.6</v>
       </c>
       <c r="K263" t="n">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="L263" t="inlineStr">
         <is>
@@ -23205,7 +23205,7 @@
         <v>28</v>
       </c>
       <c r="S263" t="n">
-        <v>0.6999999999999993</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="T263" t="n">
         <v>27</v>
@@ -27073,10 +27073,10 @@
         <v>21</v>
       </c>
       <c r="J308" t="n">
-        <v>20.6</v>
+        <v>26.5</v>
       </c>
       <c r="K308" t="n">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="L308" t="inlineStr">
         <is>
@@ -27106,7 +27106,7 @@
         <v>21</v>
       </c>
       <c r="S308" t="n">
-        <v>-0.3999999999999986</v>
+        <v>5.5</v>
       </c>
       <c r="T308" t="n">
         <v>23.9</v>
@@ -27245,10 +27245,10 @@
         <v>24.5</v>
       </c>
       <c r="J310" t="n">
-        <v>23.9</v>
+        <v>25.1</v>
       </c>
       <c r="K310" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -27278,7 +27278,7 @@
         <v>28</v>
       </c>
       <c r="S310" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T310" t="n">
         <v>25.13333333333334</v>
@@ -27332,10 +27332,10 @@
         <v>24.5</v>
       </c>
       <c r="J311" t="n">
-        <v>20.7</v>
+        <v>22.5</v>
       </c>
       <c r="K311" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="L311" t="inlineStr">
         <is>
@@ -27365,7 +27365,7 @@
         <v>28</v>
       </c>
       <c r="S311" t="n">
-        <v>-3.800000000000001</v>
+        <v>-2</v>
       </c>
       <c r="T311" t="n">
         <v>21.53333333333333</v>
@@ -29072,10 +29072,10 @@
         <v>24.5</v>
       </c>
       <c r="J331" t="n">
-        <v>31.1</v>
+        <v>24</v>
       </c>
       <c r="K331" t="n">
-        <v>127</v>
+        <v>98</v>
       </c>
       <c r="L331" t="inlineStr">
         <is>
@@ -29105,7 +29105,7 @@
         <v>28</v>
       </c>
       <c r="S331" t="n">
-        <v>6.600000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="T331" t="n">
         <v>29.13333333333334</v>
@@ -29420,10 +29420,10 @@
         <v>24.5</v>
       </c>
       <c r="J335" t="n">
-        <v>25.6</v>
+        <v>24</v>
       </c>
       <c r="K335" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="L335" t="inlineStr">
         <is>
@@ -29453,7 +29453,7 @@
         <v>28</v>
       </c>
       <c r="S335" t="n">
-        <v>1.100000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="T335" t="n">
         <v>35.8</v>
@@ -31591,10 +31591,10 @@
         <v>24.5</v>
       </c>
       <c r="J360" t="n">
-        <v>25.1</v>
+        <v>28.6</v>
       </c>
       <c r="K360" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31624,7 +31624,7 @@
         <v>28</v>
       </c>
       <c r="S360" t="n">
-        <v>0.6000000000000014</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T360" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-20 07:32:15
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5743,10 +5743,10 @@
         <v>24</v>
       </c>
       <c r="J62" t="n">
-        <v>23.4</v>
+        <v>25.7</v>
       </c>
       <c r="K62" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -5776,7 +5776,7 @@
         <v>28</v>
       </c>
       <c r="S62" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="T62" t="n">
         <v>24.46666666666667</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="K75" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="K79" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="K86" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="K91" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -10077,10 +10077,10 @@
         <v>21</v>
       </c>
       <c r="J112" t="n">
-        <v>19.9</v>
+        <v>24.3</v>
       </c>
       <c r="K112" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -10110,10 +10110,10 @@
         <v>21</v>
       </c>
       <c r="S112" t="n">
-        <v>-1.100000000000001</v>
+        <v>3.300000000000001</v>
       </c>
       <c r="T112" t="n">
-        <v>22.56666666666667</v>
+        <v>22.56666666666666</v>
       </c>
       <c r="U112" t="n">
         <v>3</v>
@@ -10512,10 +10512,10 @@
         <v>35</v>
       </c>
       <c r="J117" t="n">
-        <v>44.6</v>
+        <v>40.9</v>
       </c>
       <c r="K117" t="n">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="L117" t="inlineStr">
         <is>
@@ -10545,7 +10545,7 @@
         <v>41</v>
       </c>
       <c r="S117" t="n">
-        <v>9.600000000000001</v>
+        <v>5.899999999999999</v>
       </c>
       <c r="T117" t="n">
         <v>38.96666666666667</v>
@@ -11469,10 +11469,10 @@
         <v>35</v>
       </c>
       <c r="J128" t="n">
-        <v>30.7</v>
+        <v>33.9</v>
       </c>
       <c r="K128" t="n">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="L128" t="inlineStr">
         <is>
@@ -11502,7 +11502,7 @@
         <v>41</v>
       </c>
       <c r="S128" t="n">
-        <v>-4.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="T128" t="n">
         <v>31.83333333333333</v>
@@ -20837,10 +20837,10 @@
         <v>24</v>
       </c>
       <c r="J236" t="n">
-        <v>23.6</v>
+        <v>25.9</v>
       </c>
       <c r="K236" t="n">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="L236" t="inlineStr">
         <is>
@@ -20870,7 +20870,7 @@
         <v>28</v>
       </c>
       <c r="S236" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T236" t="n">
         <v>25.13333333333334</v>
@@ -24123,10 +24123,10 @@
         <v>28</v>
       </c>
       <c r="J274" t="n">
-        <v>32.5</v>
+        <v>27.6</v>
       </c>
       <c r="K274" t="n">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="L274" t="inlineStr">
         <is>
@@ -24156,7 +24156,7 @@
         <v>28</v>
       </c>
       <c r="S274" t="n">
-        <v>4.5</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T274" t="n">
         <v>30.16666666666667</v>
@@ -25859,10 +25859,10 @@
         <v>21</v>
       </c>
       <c r="J294" t="n">
-        <v>18.9</v>
+        <v>19.8</v>
       </c>
       <c r="K294" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="L294" t="inlineStr">
         <is>
@@ -25892,7 +25892,7 @@
         <v>21</v>
       </c>
       <c r="S294" t="n">
-        <v>-2.100000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T294" t="n">
         <v>19</v>
@@ -25944,10 +25944,10 @@
         <v>21</v>
       </c>
       <c r="J295" t="n">
-        <v>21.9</v>
+        <v>20.3</v>
       </c>
       <c r="K295" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="L295" t="inlineStr">
         <is>
@@ -25977,7 +25977,7 @@
         <v>21</v>
       </c>
       <c r="S295" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T295" t="n">
         <v>20.9</v>
@@ -27073,10 +27073,10 @@
         <v>21</v>
       </c>
       <c r="J308" t="n">
-        <v>20.6</v>
+        <v>26.5</v>
       </c>
       <c r="K308" t="n">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="L308" t="inlineStr">
         <is>
@@ -27106,7 +27106,7 @@
         <v>21</v>
       </c>
       <c r="S308" t="n">
-        <v>-0.3999999999999986</v>
+        <v>5.5</v>
       </c>
       <c r="T308" t="n">
         <v>23.9</v>
@@ -27593,10 +27593,10 @@
         <v>24.5</v>
       </c>
       <c r="J314" t="n">
-        <v>30.7</v>
+        <v>22.3</v>
       </c>
       <c r="K314" t="n">
-        <v>125</v>
+        <v>91</v>
       </c>
       <c r="L314" t="inlineStr">
         <is>
@@ -27626,7 +27626,7 @@
         <v>28</v>
       </c>
       <c r="S314" t="n">
-        <v>6.199999999999999</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="T314" t="n">
         <v>24.76666666666667</v>
@@ -27854,10 +27854,10 @@
         <v>24.5</v>
       </c>
       <c r="J317" t="n">
-        <v>20.9</v>
+        <v>24.6</v>
       </c>
       <c r="K317" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="L317" t="inlineStr">
         <is>
@@ -27887,7 +27887,7 @@
         <v>28</v>
       </c>
       <c r="S317" t="n">
-        <v>-3.600000000000001</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T317" t="n">
         <v>23.96666666666667</v>
@@ -31504,10 +31504,10 @@
         <v>24.5</v>
       </c>
       <c r="J359" t="n">
-        <v>27.4</v>
+        <v>23.2</v>
       </c>
       <c r="K359" t="n">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -31537,7 +31537,7 @@
         <v>28</v>
       </c>
       <c r="S359" t="n">
-        <v>2.899999999999999</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T359" t="n">
         <v>24.7</v>
@@ -31591,10 +31591,10 @@
         <v>24.5</v>
       </c>
       <c r="J360" t="n">
-        <v>28.6</v>
+        <v>25.1</v>
       </c>
       <c r="K360" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31624,7 +31624,7 @@
         <v>28</v>
       </c>
       <c r="S360" t="n">
-        <v>4.100000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T360" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-20 18:35:36
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2902,10 +2902,10 @@
         <v>24</v>
       </c>
       <c r="J29" t="n">
-        <v>21.6</v>
+        <v>15.8</v>
       </c>
       <c r="K29" t="n">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
         <v>28</v>
       </c>
       <c r="S29" t="n">
-        <v>-2.399999999999999</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="T29" t="n">
         <v>19.2</v>
@@ -5611,7 +5611,7 @@
         <v>3</v>
       </c>
       <c r="V60" t="n">
-        <v>24.52222222222222</v>
+        <v>24.52222222222223</v>
       </c>
       <c r="W60" t="n">
         <v>20.5</v>
@@ -5656,10 +5656,10 @@
         <v>24</v>
       </c>
       <c r="J61" t="n">
-        <v>16.6</v>
+        <v>26.4</v>
       </c>
       <c r="K61" t="n">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -5689,7 +5689,7 @@
         <v>28</v>
       </c>
       <c r="S61" t="n">
-        <v>-7.399999999999999</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T61" t="n">
         <v>23.4</v>
@@ -5698,7 +5698,7 @@
         <v>3</v>
       </c>
       <c r="V61" t="n">
-        <v>24.64444444444444</v>
+        <v>24.64444444444445</v>
       </c>
       <c r="W61" t="n">
         <v>20.5</v>
@@ -5743,10 +5743,10 @@
         <v>24</v>
       </c>
       <c r="J62" t="n">
-        <v>25.7</v>
+        <v>23.4</v>
       </c>
       <c r="K62" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -5776,7 +5776,7 @@
         <v>28</v>
       </c>
       <c r="S62" t="n">
-        <v>1.699999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T62" t="n">
         <v>24.46666666666667</v>
@@ -6307,7 +6307,7 @@
         <v>3</v>
       </c>
       <c r="V68" t="n">
-        <v>37.02962962962963</v>
+        <v>37.02962962962962</v>
       </c>
       <c r="W68" t="n">
         <v>31.5</v>
@@ -6481,7 +6481,7 @@
         <v>3</v>
       </c>
       <c r="V70" t="n">
-        <v>38.42962962962963</v>
+        <v>38.42962962962962</v>
       </c>
       <c r="W70" t="n">
         <v>31.5</v>
@@ -6613,10 +6613,10 @@
         <v>21</v>
       </c>
       <c r="J72" t="n">
-        <v>24.6</v>
+        <v>23.9</v>
       </c>
       <c r="K72" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -6646,7 +6646,7 @@
         <v>21</v>
       </c>
       <c r="S72" t="n">
-        <v>3.600000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="T72" t="n">
         <v>22.76666666666667</v>
@@ -6700,10 +6700,10 @@
         <v>35</v>
       </c>
       <c r="J73" t="n">
-        <v>33.5</v>
+        <v>40.8</v>
       </c>
       <c r="K73" t="n">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -6733,10 +6733,10 @@
         <v>41</v>
       </c>
       <c r="S73" t="n">
-        <v>-1.5</v>
+        <v>5.799999999999997</v>
       </c>
       <c r="T73" t="n">
-        <v>37.56666666666667</v>
+        <v>37.56666666666666</v>
       </c>
       <c r="U73" t="n">
         <v>3</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K75" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7133,10 +7133,10 @@
         <v>28</v>
       </c>
       <c r="J78" t="n">
-        <v>30.7</v>
+        <v>27.7</v>
       </c>
       <c r="K78" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
         <v>28</v>
       </c>
       <c r="S78" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T78" t="n">
         <v>29.2</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K79" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7305,10 +7305,10 @@
         <v>21</v>
       </c>
       <c r="J80" t="n">
-        <v>26.4</v>
+        <v>17.9</v>
       </c>
       <c r="K80" t="n">
-        <v>126</v>
+        <v>85</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -7338,7 +7338,7 @@
         <v>21</v>
       </c>
       <c r="S80" t="n">
-        <v>5.399999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T80" t="n">
         <v>21.3</v>
@@ -7392,10 +7392,10 @@
         <v>35</v>
       </c>
       <c r="J81" t="n">
-        <v>32.4</v>
+        <v>39.8</v>
       </c>
       <c r="K81" t="n">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -7425,7 +7425,7 @@
         <v>41</v>
       </c>
       <c r="S81" t="n">
-        <v>-2.600000000000001</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T81" t="n">
         <v>36.03333333333333</v>
@@ -7479,10 +7479,10 @@
         <v>21</v>
       </c>
       <c r="J82" t="n">
-        <v>21.2</v>
+        <v>25.1</v>
       </c>
       <c r="K82" t="n">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -7512,7 +7512,7 @@
         <v>21</v>
       </c>
       <c r="S82" t="n">
-        <v>0.1999999999999993</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T82" t="n">
         <v>22.16666666666667</v>
@@ -7566,10 +7566,10 @@
         <v>21</v>
       </c>
       <c r="J83" t="n">
-        <v>20.2</v>
+        <v>19.3</v>
       </c>
       <c r="K83" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -7599,7 +7599,7 @@
         <v>21</v>
       </c>
       <c r="S83" t="n">
-        <v>-0.8000000000000007</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T83" t="n">
         <v>20.46666666666667</v>
@@ -7653,10 +7653,10 @@
         <v>21</v>
       </c>
       <c r="J84" t="n">
-        <v>23.8</v>
+        <v>24.7</v>
       </c>
       <c r="K84" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7686,7 +7686,7 @@
         <v>21</v>
       </c>
       <c r="S84" t="n">
-        <v>2.800000000000001</v>
+        <v>3.699999999999999</v>
       </c>
       <c r="T84" t="n">
         <v>22.53333333333333</v>
@@ -7740,10 +7740,10 @@
         <v>21</v>
       </c>
       <c r="J85" t="n">
-        <v>19.3</v>
+        <v>26</v>
       </c>
       <c r="K85" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
         <v>21</v>
       </c>
       <c r="S85" t="n">
-        <v>-1.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="T85" t="n">
         <v>22</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K86" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K91" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -8952,10 +8952,10 @@
         <v>21</v>
       </c>
       <c r="J99" t="n">
-        <v>24.2</v>
+        <v>20.2</v>
       </c>
       <c r="K99" t="n">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="L99" t="inlineStr">
         <is>
@@ -8985,7 +8985,7 @@
         <v>21</v>
       </c>
       <c r="S99" t="n">
-        <v>3.199999999999999</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T99" t="n">
         <v>23.23333333333333</v>
@@ -10425,10 +10425,10 @@
         <v>28</v>
       </c>
       <c r="J116" t="n">
-        <v>27.6</v>
+        <v>30.7</v>
       </c>
       <c r="K116" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="L116" t="inlineStr">
         <is>
@@ -10458,7 +10458,7 @@
         <v>28</v>
       </c>
       <c r="S116" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="T116" t="n">
         <v>28.03333333333333</v>
@@ -10599,10 +10599,10 @@
         <v>35</v>
       </c>
       <c r="J118" t="n">
-        <v>37.4</v>
+        <v>34.6</v>
       </c>
       <c r="K118" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -10632,7 +10632,7 @@
         <v>41</v>
       </c>
       <c r="S118" t="n">
-        <v>2.399999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T118" t="n">
         <v>35.63333333333333</v>
@@ -13984,10 +13984,10 @@
         <v>24</v>
       </c>
       <c r="J157" t="n">
-        <v>28</v>
+        <v>23.5</v>
       </c>
       <c r="K157" t="n">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="L157" t="inlineStr">
         <is>
@@ -14017,7 +14017,7 @@
         <v>28</v>
       </c>
       <c r="S157" t="n">
-        <v>4</v>
+        <v>-0.5</v>
       </c>
       <c r="T157" t="n">
         <v>25.5</v>
@@ -20966,7 +20966,7 @@
         <v>3</v>
       </c>
       <c r="V237" t="n">
-        <v>22.92222222222222</v>
+        <v>22.92222222222223</v>
       </c>
       <c r="W237" t="n">
         <v>20.5</v>
@@ -21960,10 +21960,10 @@
         <v>21</v>
       </c>
       <c r="J249" t="n">
-        <v>21.5</v>
+        <v>20.7</v>
       </c>
       <c r="K249" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="L249" t="inlineStr">
         <is>
@@ -21991,7 +21991,7 @@
       </c>
       <c r="R249" t="inlineStr"/>
       <c r="S249" t="n">
-        <v>0.5</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T249" t="n">
         <v>20.63333333333334</v>
@@ -22389,10 +22389,10 @@
         <v>28</v>
       </c>
       <c r="J254" t="n">
-        <v>27.7</v>
+        <v>26.8</v>
       </c>
       <c r="K254" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="L254" t="inlineStr">
         <is>
@@ -22422,7 +22422,7 @@
         <v>28</v>
       </c>
       <c r="S254" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T254" t="n">
         <v>27.16666666666667</v>
@@ -24471,10 +24471,10 @@
         <v>28</v>
       </c>
       <c r="J278" t="n">
-        <v>28.2</v>
+        <v>29</v>
       </c>
       <c r="K278" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L278" t="inlineStr">
         <is>
@@ -24504,7 +24504,7 @@
         <v>28</v>
       </c>
       <c r="S278" t="n">
-        <v>0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="T278" t="n">
         <v>28.2</v>
@@ -24993,10 +24993,10 @@
         <v>21</v>
       </c>
       <c r="J284" t="n">
-        <v>22</v>
+        <v>20.8</v>
       </c>
       <c r="K284" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L284" t="inlineStr">
         <is>
@@ -25026,7 +25026,7 @@
         <v>21</v>
       </c>
       <c r="S284" t="n">
-        <v>1</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T284" t="n">
         <v>21.03333333333333</v>
@@ -25685,10 +25685,10 @@
         <v>21</v>
       </c>
       <c r="J292" t="n">
-        <v>20.4</v>
+        <v>21.1</v>
       </c>
       <c r="K292" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="L292" t="inlineStr">
         <is>
@@ -25718,7 +25718,7 @@
         <v>21</v>
       </c>
       <c r="S292" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T292" t="n">
         <v>20.76666666666667</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="K321" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28637,10 +28637,10 @@
         <v>24.5</v>
       </c>
       <c r="J326" t="n">
-        <v>21.4</v>
+        <v>25.4</v>
       </c>
       <c r="K326" t="n">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="L326" t="inlineStr">
         <is>
@@ -28670,7 +28670,7 @@
         <v>28</v>
       </c>
       <c r="S326" t="n">
-        <v>-3.100000000000001</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T326" t="n">
         <v>23.96666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="K329" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="K351" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>
@@ -31678,10 +31678,10 @@
         <v>21</v>
       </c>
       <c r="J361" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="K361" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L361" t="inlineStr">
         <is>
@@ -31711,7 +31711,7 @@
         <v>21</v>
       </c>
       <c r="S361" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T361" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-20 20:09:06
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2902,10 +2902,10 @@
         <v>24</v>
       </c>
       <c r="J29" t="n">
-        <v>15.8</v>
+        <v>21.6</v>
       </c>
       <c r="K29" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
         <v>28</v>
       </c>
       <c r="S29" t="n">
-        <v>-8.199999999999999</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="T29" t="n">
         <v>19.2</v>
@@ -5611,7 +5611,7 @@
         <v>3</v>
       </c>
       <c r="V60" t="n">
-        <v>24.52222222222223</v>
+        <v>24.52222222222222</v>
       </c>
       <c r="W60" t="n">
         <v>20.5</v>
@@ -5656,10 +5656,10 @@
         <v>24</v>
       </c>
       <c r="J61" t="n">
-        <v>26.4</v>
+        <v>16.6</v>
       </c>
       <c r="K61" t="n">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -5689,7 +5689,7 @@
         <v>28</v>
       </c>
       <c r="S61" t="n">
-        <v>2.399999999999999</v>
+        <v>-7.399999999999999</v>
       </c>
       <c r="T61" t="n">
         <v>23.4</v>
@@ -5698,7 +5698,7 @@
         <v>3</v>
       </c>
       <c r="V61" t="n">
-        <v>24.64444444444445</v>
+        <v>24.64444444444444</v>
       </c>
       <c r="W61" t="n">
         <v>20.5</v>
@@ -5743,10 +5743,10 @@
         <v>24</v>
       </c>
       <c r="J62" t="n">
-        <v>23.4</v>
+        <v>25.7</v>
       </c>
       <c r="K62" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -5776,7 +5776,7 @@
         <v>28</v>
       </c>
       <c r="S62" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="T62" t="n">
         <v>24.46666666666667</v>
@@ -6307,7 +6307,7 @@
         <v>3</v>
       </c>
       <c r="V68" t="n">
-        <v>37.02962962962962</v>
+        <v>37.02962962962963</v>
       </c>
       <c r="W68" t="n">
         <v>31.5</v>
@@ -6481,7 +6481,7 @@
         <v>3</v>
       </c>
       <c r="V70" t="n">
-        <v>38.42962962962962</v>
+        <v>38.42962962962963</v>
       </c>
       <c r="W70" t="n">
         <v>31.5</v>
@@ -6613,10 +6613,10 @@
         <v>21</v>
       </c>
       <c r="J72" t="n">
-        <v>23.9</v>
+        <v>24.6</v>
       </c>
       <c r="K72" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -6646,7 +6646,7 @@
         <v>21</v>
       </c>
       <c r="S72" t="n">
-        <v>2.899999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T72" t="n">
         <v>22.76666666666667</v>
@@ -6700,10 +6700,10 @@
         <v>35</v>
       </c>
       <c r="J73" t="n">
-        <v>40.8</v>
+        <v>33.5</v>
       </c>
       <c r="K73" t="n">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -6733,10 +6733,10 @@
         <v>41</v>
       </c>
       <c r="S73" t="n">
-        <v>5.799999999999997</v>
+        <v>-1.5</v>
       </c>
       <c r="T73" t="n">
-        <v>37.56666666666666</v>
+        <v>37.56666666666667</v>
       </c>
       <c r="U73" t="n">
         <v>3</v>
@@ -7133,10 +7133,10 @@
         <v>28</v>
       </c>
       <c r="J78" t="n">
-        <v>27.7</v>
+        <v>30.7</v>
       </c>
       <c r="K78" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
         <v>28</v>
       </c>
       <c r="S78" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="T78" t="n">
         <v>29.2</v>
@@ -7305,10 +7305,10 @@
         <v>21</v>
       </c>
       <c r="J80" t="n">
-        <v>17.9</v>
+        <v>26.4</v>
       </c>
       <c r="K80" t="n">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -7338,7 +7338,7 @@
         <v>21</v>
       </c>
       <c r="S80" t="n">
-        <v>-3.100000000000001</v>
+        <v>5.399999999999999</v>
       </c>
       <c r="T80" t="n">
         <v>21.3</v>
@@ -7392,10 +7392,10 @@
         <v>35</v>
       </c>
       <c r="J81" t="n">
-        <v>39.8</v>
+        <v>32.4</v>
       </c>
       <c r="K81" t="n">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -7425,7 +7425,7 @@
         <v>41</v>
       </c>
       <c r="S81" t="n">
-        <v>4.799999999999997</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T81" t="n">
         <v>36.03333333333333</v>
@@ -7479,10 +7479,10 @@
         <v>21</v>
       </c>
       <c r="J82" t="n">
-        <v>25.1</v>
+        <v>21.2</v>
       </c>
       <c r="K82" t="n">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -7512,7 +7512,7 @@
         <v>21</v>
       </c>
       <c r="S82" t="n">
-        <v>4.100000000000001</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T82" t="n">
         <v>22.16666666666667</v>
@@ -7566,10 +7566,10 @@
         <v>21</v>
       </c>
       <c r="J83" t="n">
-        <v>19.3</v>
+        <v>20.2</v>
       </c>
       <c r="K83" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -7599,7 +7599,7 @@
         <v>21</v>
       </c>
       <c r="S83" t="n">
-        <v>-1.699999999999999</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T83" t="n">
         <v>20.46666666666667</v>
@@ -7653,10 +7653,10 @@
         <v>21</v>
       </c>
       <c r="J84" t="n">
-        <v>24.7</v>
+        <v>23.8</v>
       </c>
       <c r="K84" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7686,7 +7686,7 @@
         <v>21</v>
       </c>
       <c r="S84" t="n">
-        <v>3.699999999999999</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T84" t="n">
         <v>22.53333333333333</v>
@@ -7740,10 +7740,10 @@
         <v>21</v>
       </c>
       <c r="J85" t="n">
-        <v>26</v>
+        <v>19.3</v>
       </c>
       <c r="K85" t="n">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
         <v>21</v>
       </c>
       <c r="S85" t="n">
-        <v>5</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T85" t="n">
         <v>22</v>
@@ -8952,10 +8952,10 @@
         <v>21</v>
       </c>
       <c r="J99" t="n">
-        <v>20.2</v>
+        <v>24.2</v>
       </c>
       <c r="K99" t="n">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="L99" t="inlineStr">
         <is>
@@ -8985,7 +8985,7 @@
         <v>21</v>
       </c>
       <c r="S99" t="n">
-        <v>-0.8000000000000007</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="T99" t="n">
         <v>23.23333333333333</v>
@@ -9642,10 +9642,10 @@
         <v>35</v>
       </c>
       <c r="J107" t="n">
-        <v>39.8</v>
+        <v>34.1</v>
       </c>
       <c r="K107" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="L107" t="inlineStr">
         <is>
@@ -9675,7 +9675,7 @@
         <v>41</v>
       </c>
       <c r="S107" t="n">
-        <v>4.799999999999997</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T107" t="n">
         <v>36.83333333333334</v>
@@ -10425,10 +10425,10 @@
         <v>28</v>
       </c>
       <c r="J116" t="n">
-        <v>30.7</v>
+        <v>27.6</v>
       </c>
       <c r="K116" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="L116" t="inlineStr">
         <is>
@@ -10458,7 +10458,7 @@
         <v>28</v>
       </c>
       <c r="S116" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T116" t="n">
         <v>28.03333333333333</v>
@@ -10599,10 +10599,10 @@
         <v>35</v>
       </c>
       <c r="J118" t="n">
-        <v>34.6</v>
+        <v>37.4</v>
       </c>
       <c r="K118" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -10632,7 +10632,7 @@
         <v>41</v>
       </c>
       <c r="S118" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T118" t="n">
         <v>35.63333333333333</v>
@@ -11904,10 +11904,10 @@
         <v>35</v>
       </c>
       <c r="J133" t="n">
-        <v>36.1</v>
+        <v>29.2</v>
       </c>
       <c r="K133" t="n">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -11937,7 +11937,7 @@
         <v>41</v>
       </c>
       <c r="S133" t="n">
-        <v>1.100000000000001</v>
+        <v>-5.800000000000001</v>
       </c>
       <c r="T133" t="n">
         <v>33.9</v>
@@ -13810,10 +13810,10 @@
         <v>28</v>
       </c>
       <c r="J155" t="n">
-        <v>36</v>
+        <v>27.9</v>
       </c>
       <c r="K155" t="n">
-        <v>128</v>
+        <v>100</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>
@@ -13843,7 +13843,7 @@
         <v>28</v>
       </c>
       <c r="S155" t="n">
-        <v>8</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T155" t="n">
         <v>34</v>
@@ -13984,10 +13984,10 @@
         <v>24</v>
       </c>
       <c r="J157" t="n">
-        <v>23.5</v>
+        <v>28</v>
       </c>
       <c r="K157" t="n">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="L157" t="inlineStr">
         <is>
@@ -14017,7 +14017,7 @@
         <v>28</v>
       </c>
       <c r="S157" t="n">
-        <v>-0.5</v>
+        <v>4</v>
       </c>
       <c r="T157" t="n">
         <v>25.5</v>
@@ -20234,10 +20234,10 @@
         <v>31</v>
       </c>
       <c r="J229" t="n">
-        <v>29.5</v>
+        <v>27.2</v>
       </c>
       <c r="K229" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="L229" t="inlineStr">
         <is>
@@ -20265,7 +20265,7 @@
       </c>
       <c r="R229" t="inlineStr"/>
       <c r="S229" t="n">
-        <v>-1.5</v>
+        <v>-3.800000000000001</v>
       </c>
       <c r="T229" t="n">
         <v>30.6</v>
@@ -20966,7 +20966,7 @@
         <v>3</v>
       </c>
       <c r="V237" t="n">
-        <v>22.92222222222223</v>
+        <v>22.92222222222222</v>
       </c>
       <c r="W237" t="n">
         <v>20.5</v>
@@ -21011,10 +21011,10 @@
         <v>28</v>
       </c>
       <c r="J238" t="n">
-        <v>25.3</v>
+        <v>29.6</v>
       </c>
       <c r="K238" t="n">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="L238" t="inlineStr">
         <is>
@@ -21044,7 +21044,7 @@
         <v>28</v>
       </c>
       <c r="S238" t="n">
-        <v>-2.699999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T238" t="n">
         <v>27.83333333333333</v>
@@ -21960,10 +21960,10 @@
         <v>21</v>
       </c>
       <c r="J249" t="n">
-        <v>20.7</v>
+        <v>21.5</v>
       </c>
       <c r="K249" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="L249" t="inlineStr">
         <is>
@@ -21991,7 +21991,7 @@
       </c>
       <c r="R249" t="inlineStr"/>
       <c r="S249" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.5</v>
       </c>
       <c r="T249" t="n">
         <v>20.63333333333334</v>
@@ -22389,7 +22389,7 @@
         <v>28</v>
       </c>
       <c r="J254" t="n">
-        <v>26.8</v>
+        <v>27</v>
       </c>
       <c r="K254" t="n">
         <v>96</v>
@@ -22422,7 +22422,7 @@
         <v>28</v>
       </c>
       <c r="S254" t="n">
-        <v>-1.199999999999999</v>
+        <v>-1</v>
       </c>
       <c r="T254" t="n">
         <v>27.16666666666667</v>
@@ -22824,10 +22824,10 @@
         <v>28</v>
       </c>
       <c r="J259" t="n">
-        <v>28.9</v>
+        <v>28.1</v>
       </c>
       <c r="K259" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="L259" t="inlineStr">
         <is>
@@ -22857,7 +22857,7 @@
         <v>28</v>
       </c>
       <c r="S259" t="n">
-        <v>0.8999999999999986</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T259" t="n">
         <v>28.03333333333333</v>
@@ -24471,10 +24471,10 @@
         <v>28</v>
       </c>
       <c r="J278" t="n">
-        <v>29</v>
+        <v>28.2</v>
       </c>
       <c r="K278" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="L278" t="inlineStr">
         <is>
@@ -24504,7 +24504,7 @@
         <v>28</v>
       </c>
       <c r="S278" t="n">
-        <v>1</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T278" t="n">
         <v>28.2</v>
@@ -24993,10 +24993,10 @@
         <v>21</v>
       </c>
       <c r="J284" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="K284" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L284" t="inlineStr">
         <is>
@@ -25026,7 +25026,7 @@
         <v>21</v>
       </c>
       <c r="S284" t="n">
-        <v>-0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="T284" t="n">
         <v>21.03333333333333</v>
@@ -25685,10 +25685,10 @@
         <v>21</v>
       </c>
       <c r="J292" t="n">
-        <v>21.1</v>
+        <v>20.4</v>
       </c>
       <c r="K292" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="L292" t="inlineStr">
         <is>
@@ -25718,7 +25718,7 @@
         <v>21</v>
       </c>
       <c r="S292" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T292" t="n">
         <v>20.76666666666667</v>
@@ -28637,10 +28637,10 @@
         <v>24.5</v>
       </c>
       <c r="J326" t="n">
-        <v>25.4</v>
+        <v>21.4</v>
       </c>
       <c r="K326" t="n">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="L326" t="inlineStr">
         <is>
@@ -28670,7 +28670,7 @@
         <v>28</v>
       </c>
       <c r="S326" t="n">
-        <v>0.8999999999999986</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T326" t="n">
         <v>23.96666666666667</v>
@@ -30984,10 +30984,10 @@
         <v>24.5</v>
       </c>
       <c r="J353" t="n">
-        <v>28.5</v>
+        <v>31.7</v>
       </c>
       <c r="K353" t="n">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="L353" t="inlineStr">
         <is>
@@ -31017,7 +31017,7 @@
         <v>28</v>
       </c>
       <c r="S353" t="n">
-        <v>4</v>
+        <v>7.199999999999999</v>
       </c>
       <c r="T353" t="n">
         <v>28.1</v>
@@ -31419,10 +31419,10 @@
         <v>24.5</v>
       </c>
       <c r="J358" t="n">
-        <v>22.7</v>
+        <v>29.1</v>
       </c>
       <c r="K358" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="L358" t="inlineStr">
         <is>
@@ -31452,7 +31452,7 @@
         <v>28</v>
       </c>
       <c r="S358" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="T358" t="n">
         <v>25.3</v>
@@ -31678,10 +31678,10 @@
         <v>21</v>
       </c>
       <c r="J361" t="n">
-        <v>20.2</v>
+        <v>21.1</v>
       </c>
       <c r="K361" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L361" t="inlineStr">
         <is>
@@ -31711,7 +31711,7 @@
         <v>21</v>
       </c>
       <c r="S361" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T361" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-20 22:14:51
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4446,10 +4446,10 @@
         <v>24</v>
       </c>
       <c r="J47" t="n">
-        <v>23.8</v>
+        <v>24.9</v>
       </c>
       <c r="K47" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -4479,7 +4479,7 @@
         <v>28</v>
       </c>
       <c r="S47" t="n">
-        <v>-0.1999999999999993</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T47" t="n">
         <v>21.43333333333333</v>
@@ -5138,10 +5138,10 @@
         <v>31</v>
       </c>
       <c r="J55" t="n">
-        <v>18.8</v>
+        <v>37.1</v>
       </c>
       <c r="K55" t="n">
-        <v>61</v>
+        <v>120</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="n">
-        <v>-12.2</v>
+        <v>6.100000000000001</v>
       </c>
       <c r="T55" t="n">
         <v>31.73333333333333</v>
@@ -7653,10 +7653,10 @@
         <v>21</v>
       </c>
       <c r="J84" t="n">
-        <v>23.8</v>
+        <v>24.7</v>
       </c>
       <c r="K84" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7686,7 +7686,7 @@
         <v>21</v>
       </c>
       <c r="S84" t="n">
-        <v>2.800000000000001</v>
+        <v>3.699999999999999</v>
       </c>
       <c r="T84" t="n">
         <v>22.53333333333333</v>
@@ -9642,10 +9642,10 @@
         <v>35</v>
       </c>
       <c r="J107" t="n">
-        <v>34.1</v>
+        <v>39.8</v>
       </c>
       <c r="K107" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="L107" t="inlineStr">
         <is>
@@ -9675,7 +9675,7 @@
         <v>41</v>
       </c>
       <c r="S107" t="n">
-        <v>-0.8999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T107" t="n">
         <v>36.83333333333334</v>
@@ -11643,10 +11643,10 @@
         <v>21</v>
       </c>
       <c r="J130" t="n">
-        <v>24</v>
+        <v>20.4</v>
       </c>
       <c r="K130" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="L130" t="inlineStr">
         <is>
@@ -11676,7 +11676,7 @@
         <v>21</v>
       </c>
       <c r="S130" t="n">
-        <v>3</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T130" t="n">
         <v>22.16666666666667</v>
@@ -11904,10 +11904,10 @@
         <v>35</v>
       </c>
       <c r="J133" t="n">
-        <v>29.2</v>
+        <v>36.1</v>
       </c>
       <c r="K133" t="n">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -11937,7 +11937,7 @@
         <v>41</v>
       </c>
       <c r="S133" t="n">
-        <v>-5.800000000000001</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T133" t="n">
         <v>33.9</v>
@@ -13810,10 +13810,10 @@
         <v>28</v>
       </c>
       <c r="J155" t="n">
-        <v>27.9</v>
+        <v>36</v>
       </c>
       <c r="K155" t="n">
-        <v>100</v>
+        <v>128</v>
       </c>
       <c r="L155" t="inlineStr">
         <is>
@@ -13843,7 +13843,7 @@
         <v>28</v>
       </c>
       <c r="S155" t="n">
-        <v>-0.1000000000000014</v>
+        <v>8</v>
       </c>
       <c r="T155" t="n">
         <v>34</v>
@@ -18931,10 +18931,10 @@
         <v>31</v>
       </c>
       <c r="J214" t="n">
-        <v>33.7</v>
+        <v>36.5</v>
       </c>
       <c r="K214" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -18962,7 +18962,7 @@
       </c>
       <c r="R214" t="inlineStr"/>
       <c r="S214" t="n">
-        <v>2.700000000000003</v>
+        <v>5.5</v>
       </c>
       <c r="T214" t="n">
         <v>33.66666666666666</v>
@@ -20234,10 +20234,10 @@
         <v>31</v>
       </c>
       <c r="J229" t="n">
-        <v>27.2</v>
+        <v>29.5</v>
       </c>
       <c r="K229" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="L229" t="inlineStr">
         <is>
@@ -20265,7 +20265,7 @@
       </c>
       <c r="R229" t="inlineStr"/>
       <c r="S229" t="n">
-        <v>-3.800000000000001</v>
+        <v>-1.5</v>
       </c>
       <c r="T229" t="n">
         <v>30.6</v>
@@ -21011,10 +21011,10 @@
         <v>28</v>
       </c>
       <c r="J238" t="n">
-        <v>29.6</v>
+        <v>25.3</v>
       </c>
       <c r="K238" t="n">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="L238" t="inlineStr">
         <is>
@@ -21044,7 +21044,7 @@
         <v>28</v>
       </c>
       <c r="S238" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="T238" t="n">
         <v>27.83333333333333</v>
@@ -22389,10 +22389,10 @@
         <v>28</v>
       </c>
       <c r="J254" t="n">
-        <v>27</v>
+        <v>27.7</v>
       </c>
       <c r="K254" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L254" t="inlineStr">
         <is>
@@ -22422,7 +22422,7 @@
         <v>28</v>
       </c>
       <c r="S254" t="n">
-        <v>-1</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T254" t="n">
         <v>27.16666666666667</v>
@@ -22824,10 +22824,10 @@
         <v>28</v>
       </c>
       <c r="J259" t="n">
-        <v>28.1</v>
+        <v>28.9</v>
       </c>
       <c r="K259" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="L259" t="inlineStr">
         <is>
@@ -22857,7 +22857,7 @@
         <v>28</v>
       </c>
       <c r="S259" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T259" t="n">
         <v>28.03333333333333</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>
@@ -30984,10 +30984,10 @@
         <v>24.5</v>
       </c>
       <c r="J353" t="n">
-        <v>31.7</v>
+        <v>28.5</v>
       </c>
       <c r="K353" t="n">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="L353" t="inlineStr">
         <is>
@@ -31017,7 +31017,7 @@
         <v>28</v>
       </c>
       <c r="S353" t="n">
-        <v>7.199999999999999</v>
+        <v>4</v>
       </c>
       <c r="T353" t="n">
         <v>28.1</v>
@@ -31419,10 +31419,10 @@
         <v>24.5</v>
       </c>
       <c r="J358" t="n">
-        <v>29.1</v>
+        <v>22.7</v>
       </c>
       <c r="K358" t="n">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="L358" t="inlineStr">
         <is>
@@ -31452,7 +31452,7 @@
         <v>28</v>
       </c>
       <c r="S358" t="n">
-        <v>4.600000000000001</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="T358" t="n">
         <v>25.3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-21 07:42:04
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -23690,10 +23690,10 @@
         <v>28</v>
       </c>
       <c r="J269" t="n">
-        <v>29.8</v>
+        <v>27.2</v>
       </c>
       <c r="K269" t="n">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="L269" t="inlineStr">
         <is>
@@ -23723,7 +23723,7 @@
         <v>28</v>
       </c>
       <c r="S269" t="n">
-        <v>1.800000000000001</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T269" t="n">
         <v>28.43333333333333</v>
@@ -25209,7 +25209,7 @@
         <v>3</v>
       </c>
       <c r="V286" t="n">
-        <v>21.74444444444444</v>
+        <v>21.74444444444445</v>
       </c>
       <c r="W286" t="n">
         <v>17.5</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-21 19:25:54
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5051,10 +5051,10 @@
         <v>24</v>
       </c>
       <c r="J54" t="n">
-        <v>21.2</v>
+        <v>25</v>
       </c>
       <c r="K54" t="n">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -5084,7 +5084,7 @@
         <v>28</v>
       </c>
       <c r="S54" t="n">
-        <v>-2.800000000000001</v>
+        <v>1</v>
       </c>
       <c r="T54" t="n">
         <v>22.7</v>
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K75" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K79" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K86" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8086,10 +8086,10 @@
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>36.7</v>
+        <v>39.1</v>
       </c>
       <c r="K89" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8119,16 +8119,16 @@
         <v>41</v>
       </c>
       <c r="S89" t="n">
-        <v>1.700000000000003</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T89" t="n">
-        <v>35.73333333333333</v>
+        <v>35.73333333333334</v>
       </c>
       <c r="U89" t="n">
         <v>3</v>
       </c>
       <c r="V89" t="n">
-        <v>35.86296296296296</v>
+        <v>35.86296296296297</v>
       </c>
       <c r="W89" t="n">
         <v>31.5</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K91" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -9816,10 +9816,10 @@
         <v>35</v>
       </c>
       <c r="J109" t="n">
-        <v>27.1</v>
+        <v>29.6</v>
       </c>
       <c r="K109" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
@@ -9849,7 +9849,7 @@
         <v>41</v>
       </c>
       <c r="S109" t="n">
-        <v>-7.899999999999999</v>
+        <v>-5.399999999999999</v>
       </c>
       <c r="T109" t="n">
         <v>27.33333333333333</v>
@@ -10164,10 +10164,10 @@
         <v>35</v>
       </c>
       <c r="J113" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="K113" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
@@ -10197,7 +10197,7 @@
         <v>41</v>
       </c>
       <c r="S113" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="T113" t="n">
         <v>25.5</v>
@@ -14504,10 +14504,10 @@
         <v>21</v>
       </c>
       <c r="J163" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="K163" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="L163" t="inlineStr">
         <is>
@@ -14537,7 +14537,7 @@
         <v>21</v>
       </c>
       <c r="S163" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T163" t="n">
         <v>22.96666666666667</v>
@@ -19538,10 +19538,10 @@
         <v>28</v>
       </c>
       <c r="J221" t="n">
-        <v>14.6</v>
+        <v>27.2</v>
       </c>
       <c r="K221" t="n">
-        <v>52</v>
+        <v>97</v>
       </c>
       <c r="L221" t="inlineStr">
         <is>
@@ -19571,7 +19571,7 @@
         <v>28</v>
       </c>
       <c r="S221" t="n">
-        <v>-13.4</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T221" t="n">
         <v>23.53333333333333</v>
@@ -25337,10 +25337,10 @@
         <v>21</v>
       </c>
       <c r="J288" t="n">
-        <v>25.9</v>
+        <v>22.6</v>
       </c>
       <c r="K288" t="n">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="L288" t="inlineStr">
         <is>
@@ -25370,7 +25370,7 @@
         <v>21</v>
       </c>
       <c r="S288" t="n">
-        <v>4.899999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T288" t="n">
         <v>22.7</v>
@@ -31678,10 +31678,10 @@
         <v>21</v>
       </c>
       <c r="J361" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="K361" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L361" t="inlineStr">
         <is>
@@ -31711,7 +31711,7 @@
         <v>21</v>
       </c>
       <c r="S361" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T361" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-23 07:22:16
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5265,7 +5265,7 @@
         <v>3</v>
       </c>
       <c r="V56" t="n">
-        <v>23.14444444444445</v>
+        <v>23.14444444444444</v>
       </c>
       <c r="W56" t="n">
         <v>20.5</v>
@@ -5569,10 +5569,10 @@
         <v>24</v>
       </c>
       <c r="J60" t="n">
-        <v>23.1</v>
+        <v>25.9</v>
       </c>
       <c r="K60" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -5602,7 +5602,7 @@
         <v>28</v>
       </c>
       <c r="S60" t="n">
-        <v>-0.8999999999999986</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T60" t="n">
         <v>24.1</v>
@@ -7653,10 +7653,10 @@
         <v>21</v>
       </c>
       <c r="J84" t="n">
-        <v>23.8</v>
+        <v>24.7</v>
       </c>
       <c r="K84" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7686,7 +7686,7 @@
         <v>21</v>
       </c>
       <c r="S84" t="n">
-        <v>2.800000000000001</v>
+        <v>3.699999999999999</v>
       </c>
       <c r="T84" t="n">
         <v>22.53333333333333</v>
@@ -7740,10 +7740,10 @@
         <v>21</v>
       </c>
       <c r="J85" t="n">
-        <v>26</v>
+        <v>19.3</v>
       </c>
       <c r="K85" t="n">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
         <v>21</v>
       </c>
       <c r="S85" t="n">
-        <v>5</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T85" t="n">
         <v>22</v>
@@ -15024,10 +15024,10 @@
         <v>35</v>
       </c>
       <c r="J169" t="n">
-        <v>34</v>
+        <v>39.3</v>
       </c>
       <c r="K169" t="n">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="L169" t="inlineStr">
         <is>
@@ -15057,7 +15057,7 @@
         <v>41</v>
       </c>
       <c r="S169" t="n">
-        <v>-1</v>
+        <v>4.299999999999997</v>
       </c>
       <c r="T169" t="n">
         <v>36.3</v>
@@ -15111,10 +15111,10 @@
         <v>28</v>
       </c>
       <c r="J170" t="n">
-        <v>27</v>
+        <v>24.8</v>
       </c>
       <c r="K170" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
@@ -15144,7 +15144,7 @@
         <v>28</v>
       </c>
       <c r="S170" t="n">
-        <v>-1</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T170" t="n">
         <v>26.4</v>
@@ -15372,10 +15372,10 @@
         <v>21</v>
       </c>
       <c r="J173" t="n">
-        <v>20.5</v>
+        <v>23.8</v>
       </c>
       <c r="K173" t="n">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="L173" t="inlineStr">
         <is>
@@ -15405,7 +15405,7 @@
         <v>21</v>
       </c>
       <c r="S173" t="n">
-        <v>-0.5</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T173" t="n">
         <v>21.66666666666667</v>
@@ -15459,10 +15459,10 @@
         <v>28</v>
       </c>
       <c r="J174" t="n">
-        <v>27.7</v>
+        <v>31.6</v>
       </c>
       <c r="K174" t="n">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="L174" t="inlineStr">
         <is>
@@ -15492,7 +15492,7 @@
         <v>28</v>
       </c>
       <c r="S174" t="n">
-        <v>-0.3000000000000007</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T174" t="n">
         <v>30.13333333333334</v>
@@ -15546,7 +15546,7 @@
         <v>28</v>
       </c>
       <c r="J175" t="n">
-        <v>26.4</v>
+        <v>26.3</v>
       </c>
       <c r="K175" t="n">
         <v>94</v>
@@ -15579,7 +15579,7 @@
         <v>28</v>
       </c>
       <c r="S175" t="n">
-        <v>-1.600000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T175" t="n">
         <v>26.6</v>
@@ -15633,10 +15633,10 @@
         <v>21</v>
       </c>
       <c r="J176" t="n">
-        <v>13</v>
+        <v>19.3</v>
       </c>
       <c r="K176" t="n">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="L176" t="inlineStr">
         <is>
@@ -15666,7 +15666,7 @@
         <v>21</v>
       </c>
       <c r="S176" t="n">
-        <v>-8</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T176" t="n">
         <v>18.23333333333333</v>
@@ -15805,10 +15805,10 @@
         <v>28</v>
       </c>
       <c r="J178" t="n">
-        <v>23.6</v>
+        <v>29</v>
       </c>
       <c r="K178" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="L178" t="inlineStr">
         <is>
@@ -15838,7 +15838,7 @@
         <v>28</v>
       </c>
       <c r="S178" t="n">
-        <v>-4.399999999999999</v>
+        <v>1</v>
       </c>
       <c r="T178" t="n">
         <v>25.33333333333333</v>
@@ -15892,10 +15892,10 @@
         <v>35</v>
       </c>
       <c r="J179" t="n">
-        <v>38.3</v>
+        <v>34.3</v>
       </c>
       <c r="K179" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="L179" t="inlineStr">
         <is>
@@ -15925,7 +15925,7 @@
         <v>41</v>
       </c>
       <c r="S179" t="n">
-        <v>3.299999999999997</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="T179" t="n">
         <v>35.66666666666666</v>
@@ -15979,7 +15979,7 @@
         <v>21</v>
       </c>
       <c r="J180" t="n">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="K180" t="n">
         <v>108</v>
@@ -16012,10 +16012,10 @@
         <v>21</v>
       </c>
       <c r="S180" t="n">
-        <v>1.699999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T180" t="n">
-        <v>21.86666666666666</v>
+        <v>21.86666666666667</v>
       </c>
       <c r="U180" t="n">
         <v>3</v>
@@ -16066,10 +16066,10 @@
         <v>28</v>
       </c>
       <c r="J181" t="n">
-        <v>36.4</v>
+        <v>40.2</v>
       </c>
       <c r="K181" t="n">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="L181" t="inlineStr">
         <is>
@@ -16099,7 +16099,7 @@
         <v>28</v>
       </c>
       <c r="S181" t="n">
-        <v>8.399999999999999</v>
+        <v>12.2</v>
       </c>
       <c r="T181" t="n">
         <v>33.36666666666667</v>
@@ -16153,10 +16153,10 @@
         <v>21</v>
       </c>
       <c r="J182" t="n">
-        <v>20.7</v>
+        <v>20.9</v>
       </c>
       <c r="K182" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L182" t="inlineStr">
         <is>
@@ -16186,7 +16186,7 @@
         <v>21</v>
       </c>
       <c r="S182" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T182" t="n">
         <v>21.3</v>
@@ -23085,10 +23085,10 @@
         <v>28</v>
       </c>
       <c r="J262" t="n">
-        <v>32.5</v>
+        <v>24.7</v>
       </c>
       <c r="K262" t="n">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="L262" t="inlineStr">
         <is>
@@ -23118,7 +23118,7 @@
         <v>28</v>
       </c>
       <c r="S262" t="n">
-        <v>4.5</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="T262" t="n">
         <v>29.5</v>
@@ -24687,7 +24687,7 @@
         <v>3</v>
       </c>
       <c r="V280" t="n">
-        <v>24.36666666666666</v>
+        <v>24.36666666666667</v>
       </c>
       <c r="W280" t="n">
         <v>17.5</v>
@@ -27245,10 +27245,10 @@
         <v>24.5</v>
       </c>
       <c r="J310" t="n">
-        <v>23.9</v>
+        <v>25.1</v>
       </c>
       <c r="K310" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -27278,7 +27278,7 @@
         <v>28</v>
       </c>
       <c r="S310" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T310" t="n">
         <v>25.13333333333334</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28550,10 +28550,10 @@
         <v>24.5</v>
       </c>
       <c r="J325" t="n">
-        <v>27</v>
+        <v>23.6</v>
       </c>
       <c r="K325" t="n">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="L325" t="inlineStr">
         <is>
@@ -28583,7 +28583,7 @@
         <v>28</v>
       </c>
       <c r="S325" t="n">
-        <v>2.5</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T325" t="n">
         <v>24.93333333333333</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -29159,10 +29159,10 @@
         <v>24.5</v>
       </c>
       <c r="J332" t="n">
-        <v>24.9</v>
+        <v>26.9</v>
       </c>
       <c r="K332" t="n">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="L332" t="inlineStr">
         <is>
@@ -29192,7 +29192,7 @@
         <v>28</v>
       </c>
       <c r="S332" t="n">
-        <v>0.3999999999999986</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T332" t="n">
         <v>24.26666666666667</v>
@@ -31504,10 +31504,10 @@
         <v>24.5</v>
       </c>
       <c r="J359" t="n">
-        <v>27.4</v>
+        <v>23.2</v>
       </c>
       <c r="K359" t="n">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -31537,7 +31537,7 @@
         <v>28</v>
       </c>
       <c r="S359" t="n">
-        <v>2.899999999999999</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T359" t="n">
         <v>24.7</v>
@@ -31591,10 +31591,10 @@
         <v>24.5</v>
       </c>
       <c r="J360" t="n">
-        <v>28.6</v>
+        <v>25.1</v>
       </c>
       <c r="K360" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31624,7 +31624,7 @@
         <v>28</v>
       </c>
       <c r="S360" t="n">
-        <v>4.100000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T360" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-23 16:11:23
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3331,10 +3331,10 @@
         <v>31</v>
       </c>
       <c r="J34" t="n">
-        <v>31.4</v>
+        <v>30</v>
       </c>
       <c r="K34" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1</v>
       </c>
       <c r="T34" t="n">
         <v>30.33333333333333</v>
@@ -3541,7 +3541,7 @@
         <v>3</v>
       </c>
       <c r="V36" t="n">
-        <v>33.03333333333333</v>
+        <v>35.05555555555556</v>
       </c>
       <c r="W36" t="n">
         <v>27.5</v>
@@ -5265,7 +5265,7 @@
         <v>3</v>
       </c>
       <c r="V56" t="n">
-        <v>23.14444444444444</v>
+        <v>23.14444444444445</v>
       </c>
       <c r="W56" t="n">
         <v>20.5</v>
@@ -5569,10 +5569,10 @@
         <v>24</v>
       </c>
       <c r="J60" t="n">
-        <v>25.9</v>
+        <v>23.1</v>
       </c>
       <c r="K60" t="n">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -5602,7 +5602,7 @@
         <v>28</v>
       </c>
       <c r="S60" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T60" t="n">
         <v>24.1</v>
@@ -7653,10 +7653,10 @@
         <v>21</v>
       </c>
       <c r="J84" t="n">
-        <v>24.7</v>
+        <v>23.8</v>
       </c>
       <c r="K84" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7686,7 +7686,7 @@
         <v>21</v>
       </c>
       <c r="S84" t="n">
-        <v>3.699999999999999</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T84" t="n">
         <v>22.53333333333333</v>
@@ -11730,10 +11730,10 @@
         <v>35</v>
       </c>
       <c r="J131" t="n">
-        <v>36.6</v>
+        <v>36.5</v>
       </c>
       <c r="K131" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -11763,7 +11763,7 @@
         <v>41</v>
       </c>
       <c r="S131" t="n">
-        <v>1.600000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="T131" t="n">
         <v>35.63333333333333</v>
@@ -12250,10 +12250,10 @@
         <v>35</v>
       </c>
       <c r="J137" t="n">
-        <v>45.3</v>
+        <v>45.2</v>
       </c>
       <c r="K137" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L137" t="inlineStr">
         <is>
@@ -12283,7 +12283,7 @@
         <v>41</v>
       </c>
       <c r="S137" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="T137" t="n">
         <v>41</v>
@@ -15024,10 +15024,10 @@
         <v>35</v>
       </c>
       <c r="J169" t="n">
-        <v>39.3</v>
+        <v>34</v>
       </c>
       <c r="K169" t="n">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="L169" t="inlineStr">
         <is>
@@ -15057,7 +15057,7 @@
         <v>41</v>
       </c>
       <c r="S169" t="n">
-        <v>4.299999999999997</v>
+        <v>-1</v>
       </c>
       <c r="T169" t="n">
         <v>36.3</v>
@@ -15111,10 +15111,10 @@
         <v>28</v>
       </c>
       <c r="J170" t="n">
-        <v>24.8</v>
+        <v>27</v>
       </c>
       <c r="K170" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="L170" t="inlineStr">
         <is>
@@ -15144,7 +15144,7 @@
         <v>28</v>
       </c>
       <c r="S170" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1</v>
       </c>
       <c r="T170" t="n">
         <v>26.4</v>
@@ -15372,10 +15372,10 @@
         <v>21</v>
       </c>
       <c r="J173" t="n">
-        <v>23.8</v>
+        <v>20.5</v>
       </c>
       <c r="K173" t="n">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="L173" t="inlineStr">
         <is>
@@ -15405,7 +15405,7 @@
         <v>21</v>
       </c>
       <c r="S173" t="n">
-        <v>2.800000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="T173" t="n">
         <v>21.66666666666667</v>
@@ -15459,10 +15459,10 @@
         <v>28</v>
       </c>
       <c r="J174" t="n">
-        <v>31.6</v>
+        <v>27.7</v>
       </c>
       <c r="K174" t="n">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="L174" t="inlineStr">
         <is>
@@ -15492,7 +15492,7 @@
         <v>28</v>
       </c>
       <c r="S174" t="n">
-        <v>3.600000000000001</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T174" t="n">
         <v>30.13333333333334</v>
@@ -15546,7 +15546,7 @@
         <v>28</v>
       </c>
       <c r="J175" t="n">
-        <v>26.3</v>
+        <v>26.4</v>
       </c>
       <c r="K175" t="n">
         <v>94</v>
@@ -15579,7 +15579,7 @@
         <v>28</v>
       </c>
       <c r="S175" t="n">
-        <v>-1.699999999999999</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T175" t="n">
         <v>26.6</v>
@@ -15633,10 +15633,10 @@
         <v>21</v>
       </c>
       <c r="J176" t="n">
-        <v>19.3</v>
+        <v>13</v>
       </c>
       <c r="K176" t="n">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="L176" t="inlineStr">
         <is>
@@ -15666,7 +15666,7 @@
         <v>21</v>
       </c>
       <c r="S176" t="n">
-        <v>-1.699999999999999</v>
+        <v>-8</v>
       </c>
       <c r="T176" t="n">
         <v>18.23333333333333</v>
@@ -15805,10 +15805,10 @@
         <v>28</v>
       </c>
       <c r="J178" t="n">
-        <v>29</v>
+        <v>23.6</v>
       </c>
       <c r="K178" t="n">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="L178" t="inlineStr">
         <is>
@@ -15838,7 +15838,7 @@
         <v>28</v>
       </c>
       <c r="S178" t="n">
-        <v>1</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="T178" t="n">
         <v>25.33333333333333</v>
@@ -15892,10 +15892,10 @@
         <v>35</v>
       </c>
       <c r="J179" t="n">
-        <v>34.3</v>
+        <v>38.3</v>
       </c>
       <c r="K179" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="L179" t="inlineStr">
         <is>
@@ -15925,7 +15925,7 @@
         <v>41</v>
       </c>
       <c r="S179" t="n">
-        <v>-0.7000000000000028</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T179" t="n">
         <v>35.66666666666666</v>
@@ -15979,7 +15979,7 @@
         <v>21</v>
       </c>
       <c r="J180" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="K180" t="n">
         <v>108</v>
@@ -16012,10 +16012,10 @@
         <v>21</v>
       </c>
       <c r="S180" t="n">
-        <v>1.600000000000001</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="T180" t="n">
-        <v>21.86666666666667</v>
+        <v>21.86666666666666</v>
       </c>
       <c r="U180" t="n">
         <v>3</v>
@@ -16066,10 +16066,10 @@
         <v>28</v>
       </c>
       <c r="J181" t="n">
-        <v>40.2</v>
+        <v>36.4</v>
       </c>
       <c r="K181" t="n">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="L181" t="inlineStr">
         <is>
@@ -16099,7 +16099,7 @@
         <v>28</v>
       </c>
       <c r="S181" t="n">
-        <v>12.2</v>
+        <v>8.399999999999999</v>
       </c>
       <c r="T181" t="n">
         <v>33.36666666666667</v>
@@ -16153,10 +16153,10 @@
         <v>21</v>
       </c>
       <c r="J182" t="n">
-        <v>20.9</v>
+        <v>20.7</v>
       </c>
       <c r="K182" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L182" t="inlineStr">
         <is>
@@ -16186,7 +16186,7 @@
         <v>21</v>
       </c>
       <c r="S182" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T182" t="n">
         <v>21.3</v>
@@ -17539,10 +17539,10 @@
         <v>28</v>
       </c>
       <c r="J198" t="n">
-        <v>29.3</v>
+        <v>26.7</v>
       </c>
       <c r="K198" t="n">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="L198" t="inlineStr">
         <is>
@@ -17572,7 +17572,7 @@
         <v>28</v>
       </c>
       <c r="S198" t="n">
-        <v>1.300000000000001</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T198" t="n">
         <v>29.3</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>
@@ -31504,10 +31504,10 @@
         <v>24.5</v>
       </c>
       <c r="J359" t="n">
-        <v>23.2</v>
+        <v>27.4</v>
       </c>
       <c r="K359" t="n">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="L359" t="inlineStr">
         <is>
@@ -31537,7 +31537,7 @@
         <v>28</v>
       </c>
       <c r="S359" t="n">
-        <v>-1.300000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="T359" t="n">
         <v>24.7</v>
@@ -31591,10 +31591,10 @@
         <v>24.5</v>
       </c>
       <c r="J360" t="n">
-        <v>25.1</v>
+        <v>28.6</v>
       </c>
       <c r="K360" t="n">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31624,7 +31624,7 @@
         <v>28</v>
       </c>
       <c r="S360" t="n">
-        <v>0.6000000000000014</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T360" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-23 22:46:28
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -6874,10 +6874,10 @@
         <v>31</v>
       </c>
       <c r="J75" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K75" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T75" t="n">
         <v>32.03333333333333</v>
@@ -7220,10 +7220,10 @@
         <v>31</v>
       </c>
       <c r="J79" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K79" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T79" t="n">
         <v>36</v>
@@ -7392,10 +7392,10 @@
         <v>35</v>
       </c>
       <c r="J81" t="n">
-        <v>32.4</v>
+        <v>39.8</v>
       </c>
       <c r="K81" t="n">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -7425,7 +7425,7 @@
         <v>41</v>
       </c>
       <c r="S81" t="n">
-        <v>-2.600000000000001</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T81" t="n">
         <v>36.03333333333333</v>
@@ -7827,10 +7827,10 @@
         <v>31</v>
       </c>
       <c r="J86" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K86" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L86" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T86" t="n">
         <v>33.63333333333333</v>
@@ -8173,10 +8173,10 @@
         <v>35</v>
       </c>
       <c r="J90" t="n">
-        <v>39.8</v>
+        <v>40.3</v>
       </c>
       <c r="K90" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -8206,7 +8206,7 @@
         <v>41</v>
       </c>
       <c r="S90" t="n">
-        <v>4.799999999999997</v>
+        <v>5.299999999999997</v>
       </c>
       <c r="T90" t="n">
         <v>36.16666666666666</v>
@@ -8260,10 +8260,10 @@
         <v>31</v>
       </c>
       <c r="J91" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K91" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L91" t="inlineStr">
         <is>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T91" t="n">
         <v>32.76666666666667</v>
@@ -8733,7 +8733,7 @@
         <v>3</v>
       </c>
       <c r="V96" t="n">
-        <v>37.43333333333333</v>
+        <v>37.43333333333334</v>
       </c>
       <c r="W96" t="n">
         <v>31.5</v>
@@ -8865,10 +8865,10 @@
         <v>35</v>
       </c>
       <c r="J98" t="n">
-        <v>38.4</v>
+        <v>34</v>
       </c>
       <c r="K98" t="n">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="L98" t="inlineStr">
         <is>
@@ -8898,7 +8898,7 @@
         <v>41</v>
       </c>
       <c r="S98" t="n">
-        <v>3.399999999999999</v>
+        <v>-1</v>
       </c>
       <c r="T98" t="n">
         <v>36.5</v>
@@ -9903,10 +9903,10 @@
         <v>35</v>
       </c>
       <c r="J110" t="n">
-        <v>49.1</v>
+        <v>31.4</v>
       </c>
       <c r="K110" t="n">
-        <v>140</v>
+        <v>90</v>
       </c>
       <c r="L110" t="inlineStr">
         <is>
@@ -9936,7 +9936,7 @@
         <v>41</v>
       </c>
       <c r="S110" t="n">
-        <v>14.1</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="T110" t="n">
         <v>43.96666666666667</v>
@@ -14504,10 +14504,10 @@
         <v>21</v>
       </c>
       <c r="J163" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="K163" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="L163" t="inlineStr">
         <is>
@@ -14537,7 +14537,7 @@
         <v>21</v>
       </c>
       <c r="S163" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T163" t="n">
         <v>22.96666666666667</v>
@@ -20234,10 +20234,10 @@
         <v>31</v>
       </c>
       <c r="J229" t="n">
-        <v>29.5</v>
+        <v>27.2</v>
       </c>
       <c r="K229" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="L229" t="inlineStr">
         <is>
@@ -20265,7 +20265,7 @@
       </c>
       <c r="R229" t="inlineStr"/>
       <c r="S229" t="n">
-        <v>-1.5</v>
+        <v>-3.800000000000001</v>
       </c>
       <c r="T229" t="n">
         <v>30.6</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-25 07:11:06
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -21960,10 +21960,10 @@
         <v>21</v>
       </c>
       <c r="J249" t="n">
-        <v>24.6</v>
+        <v>13.3</v>
       </c>
       <c r="K249" t="n">
-        <v>117</v>
+        <v>63</v>
       </c>
       <c r="L249" t="inlineStr">
         <is>
@@ -21991,10 +21991,10 @@
       </c>
       <c r="R249" t="inlineStr"/>
       <c r="S249" t="n">
-        <v>3.600000000000001</v>
+        <v>-7.699999999999999</v>
       </c>
       <c r="T249" t="n">
-        <v>20.13333333333334</v>
+        <v>20.13333333333333</v>
       </c>
       <c r="U249" t="n">
         <v>3</v>
@@ -22130,10 +22130,10 @@
         <v>21</v>
       </c>
       <c r="J251" t="n">
-        <v>23.1</v>
+        <v>22.3</v>
       </c>
       <c r="K251" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="L251" t="inlineStr">
         <is>
@@ -22163,7 +22163,7 @@
         <v>21</v>
       </c>
       <c r="S251" t="n">
-        <v>2.100000000000001</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="T251" t="n">
         <v>21.8</v>
@@ -27073,10 +27073,10 @@
         <v>24.5</v>
       </c>
       <c r="J308" t="n">
-        <v>22.6</v>
+        <v>25</v>
       </c>
       <c r="K308" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="L308" t="inlineStr">
         <is>
@@ -27106,7 +27106,7 @@
         <v>28</v>
       </c>
       <c r="S308" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="T308" t="n">
         <v>24.8</v>
@@ -27421,10 +27421,10 @@
         <v>24.5</v>
       </c>
       <c r="J312" t="n">
-        <v>24.8</v>
+        <v>22.8</v>
       </c>
       <c r="K312" t="n">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="L312" t="inlineStr">
         <is>
@@ -27454,7 +27454,7 @@
         <v>28</v>
       </c>
       <c r="S312" t="n">
-        <v>0.3000000000000007</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T312" t="n">
         <v>24.1</v>
@@ -28117,10 +28117,10 @@
         <v>24.5</v>
       </c>
       <c r="J320" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K320" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L320" t="inlineStr">
         <is>
@@ -28150,7 +28150,7 @@
         <v>28</v>
       </c>
       <c r="S320" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T320" t="n">
         <v>24.66666666666667</v>
@@ -28813,10 +28813,10 @@
         <v>24.5</v>
       </c>
       <c r="J328" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K328" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L328" t="inlineStr">
         <is>
@@ -28846,7 +28846,7 @@
         <v>28</v>
       </c>
       <c r="S328" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T328" t="n">
         <v>27.1</v>
@@ -30727,10 +30727,10 @@
         <v>24.5</v>
       </c>
       <c r="J350" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K350" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L350" t="inlineStr">
         <is>
@@ -30760,10 +30760,10 @@
         <v>28</v>
       </c>
       <c r="S350" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T350" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U350" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-25 18:40:23
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4794,10 +4794,10 @@
         <v>31</v>
       </c>
       <c r="J51" t="n">
-        <v>30.5</v>
+        <v>38.5</v>
       </c>
       <c r="K51" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="n">
-        <v>-0.5</v>
+        <v>7.5</v>
       </c>
       <c r="T51" t="n">
         <v>35.86666666666667</v>
@@ -5180,7 +5180,7 @@
         <v>3</v>
       </c>
       <c r="V55" t="n">
-        <v>23.14444444444445</v>
+        <v>23.14444444444444</v>
       </c>
       <c r="W55" t="n">
         <v>20.5</v>
@@ -5484,10 +5484,10 @@
         <v>24</v>
       </c>
       <c r="J59" t="n">
-        <v>23.1</v>
+        <v>25.9</v>
       </c>
       <c r="K59" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -5517,7 +5517,7 @@
         <v>28</v>
       </c>
       <c r="S59" t="n">
-        <v>-0.8999999999999986</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T59" t="n">
         <v>24.1</v>
@@ -6093,10 +6093,10 @@
         <v>35</v>
       </c>
       <c r="J66" t="n">
-        <v>34.3</v>
+        <v>32.3</v>
       </c>
       <c r="K66" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -6126,7 +6126,7 @@
         <v>41</v>
       </c>
       <c r="S66" t="n">
-        <v>-0.7000000000000028</v>
+        <v>-2.700000000000003</v>
       </c>
       <c r="T66" t="n">
         <v>32.96666666666666</v>
@@ -8001,10 +8001,10 @@
         <v>35</v>
       </c>
       <c r="J88" t="n">
-        <v>39.1</v>
+        <v>36.7</v>
       </c>
       <c r="K88" t="n">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
@@ -8034,16 +8034,16 @@
         <v>41</v>
       </c>
       <c r="S88" t="n">
-        <v>4.100000000000001</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T88" t="n">
-        <v>35.73333333333334</v>
+        <v>35.73333333333333</v>
       </c>
       <c r="U88" t="n">
         <v>3</v>
       </c>
       <c r="V88" t="n">
-        <v>35.86296296296297</v>
+        <v>35.86296296296296</v>
       </c>
       <c r="W88" t="n">
         <v>31.5</v>
@@ -9992,10 +9992,10 @@
         <v>21</v>
       </c>
       <c r="J111" t="n">
-        <v>19.9</v>
+        <v>24.3</v>
       </c>
       <c r="K111" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
@@ -10025,10 +10025,10 @@
         <v>21</v>
       </c>
       <c r="S111" t="n">
-        <v>-1.100000000000001</v>
+        <v>3.300000000000001</v>
       </c>
       <c r="T111" t="n">
-        <v>22.56666666666667</v>
+        <v>22.56666666666666</v>
       </c>
       <c r="U111" t="n">
         <v>3</v>
@@ -16934,10 +16934,10 @@
         <v>21</v>
       </c>
       <c r="J191" t="n">
-        <v>20.7</v>
+        <v>23</v>
       </c>
       <c r="K191" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="L191" t="inlineStr">
         <is>
@@ -16967,7 +16967,7 @@
         <v>21</v>
       </c>
       <c r="S191" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2</v>
       </c>
       <c r="T191" t="n">
         <v>21.5</v>
@@ -18411,10 +18411,10 @@
         <v>28</v>
       </c>
       <c r="J208" t="n">
-        <v>26.2</v>
+        <v>32.6</v>
       </c>
       <c r="K208" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="L208" t="inlineStr">
         <is>
@@ -18444,7 +18444,7 @@
         <v>28</v>
       </c>
       <c r="S208" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="T208" t="n">
         <v>30.03333333333333</v>
@@ -20321,10 +20321,10 @@
         <v>28</v>
       </c>
       <c r="J230" t="n">
-        <v>24.5</v>
+        <v>26.1</v>
       </c>
       <c r="K230" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="L230" t="inlineStr">
         <is>
@@ -20354,7 +20354,7 @@
         <v>28</v>
       </c>
       <c r="S230" t="n">
-        <v>-3.5</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="T230" t="n">
         <v>25.53333333333333</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-25 23:10:42
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3758,10 +3758,10 @@
         <v>24</v>
       </c>
       <c r="J39" t="n">
-        <v>16.2</v>
+        <v>15.7</v>
       </c>
       <c r="K39" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -3791,7 +3791,7 @@
         <v>28</v>
       </c>
       <c r="S39" t="n">
-        <v>-7.800000000000001</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="T39" t="n">
         <v>16.5</v>
@@ -6789,10 +6789,10 @@
         <v>31</v>
       </c>
       <c r="J74" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K74" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
@@ -6820,7 +6820,7 @@
       </c>
       <c r="R74" t="inlineStr"/>
       <c r="S74" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T74" t="n">
         <v>32.03333333333333</v>
@@ -7135,10 +7135,10 @@
         <v>31</v>
       </c>
       <c r="J78" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K78" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -7166,7 +7166,7 @@
       </c>
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T78" t="n">
         <v>36</v>
@@ -7394,10 +7394,10 @@
         <v>21</v>
       </c>
       <c r="J81" t="n">
-        <v>21.2</v>
+        <v>20.2</v>
       </c>
       <c r="K81" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -7427,7 +7427,7 @@
         <v>21</v>
       </c>
       <c r="S81" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T81" t="n">
         <v>22.16666666666667</v>
@@ -7742,10 +7742,10 @@
         <v>31</v>
       </c>
       <c r="J85" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K85" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T85" t="n">
         <v>33.63333333333333</v>
@@ -8175,10 +8175,10 @@
         <v>31</v>
       </c>
       <c r="J90" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K90" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -8206,7 +8206,7 @@
       </c>
       <c r="R90" t="inlineStr"/>
       <c r="S90" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T90" t="n">
         <v>32.76666666666667</v>
@@ -10079,10 +10079,10 @@
         <v>35</v>
       </c>
       <c r="J112" t="n">
-        <v>22.5</v>
+        <v>26.3</v>
       </c>
       <c r="K112" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="L112" t="inlineStr">
         <is>
@@ -10112,7 +10112,7 @@
         <v>41</v>
       </c>
       <c r="S112" t="n">
-        <v>-12.5</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="T112" t="n">
         <v>25.5</v>
@@ -12165,10 +12165,10 @@
         <v>35</v>
       </c>
       <c r="J136" t="n">
-        <v>45.3</v>
+        <v>45.2</v>
       </c>
       <c r="K136" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L136" t="inlineStr">
         <is>
@@ -12198,7 +12198,7 @@
         <v>41</v>
       </c>
       <c r="S136" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="T136" t="n">
         <v>41</v>
@@ -18846,10 +18846,10 @@
         <v>31</v>
       </c>
       <c r="J213" t="n">
-        <v>33.7</v>
+        <v>36.5</v>
       </c>
       <c r="K213" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="L213" t="inlineStr">
         <is>
@@ -18877,7 +18877,7 @@
       </c>
       <c r="R213" t="inlineStr"/>
       <c r="S213" t="n">
-        <v>2.700000000000003</v>
+        <v>5.5</v>
       </c>
       <c r="T213" t="n">
         <v>33.66666666666666</v>
@@ -21446,10 +21446,10 @@
         <v>21</v>
       </c>
       <c r="J243" t="n">
-        <v>17.3</v>
+        <v>19</v>
       </c>
       <c r="K243" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="L243" t="inlineStr">
         <is>
@@ -21477,7 +21477,7 @@
       </c>
       <c r="R243" t="inlineStr"/>
       <c r="S243" t="n">
-        <v>-3.699999999999999</v>
+        <v>-2</v>
       </c>
       <c r="T243" t="n">
         <v>19.3</v>
@@ -23346,10 +23346,10 @@
         <v>28</v>
       </c>
       <c r="J265" t="n">
-        <v>28.1</v>
+        <v>27</v>
       </c>
       <c r="K265" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L265" t="inlineStr">
         <is>
@@ -23379,7 +23379,7 @@
         <v>28</v>
       </c>
       <c r="S265" t="n">
-        <v>0.1000000000000014</v>
+        <v>-1</v>
       </c>
       <c r="T265" t="n">
         <v>26.96666666666667</v>
@@ -24386,10 +24386,10 @@
         <v>28</v>
       </c>
       <c r="J277" t="n">
-        <v>28.2</v>
+        <v>29</v>
       </c>
       <c r="K277" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="L277" t="inlineStr">
         <is>
@@ -24419,7 +24419,7 @@
         <v>28</v>
       </c>
       <c r="S277" t="n">
-        <v>0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="T277" t="n">
         <v>28.2</v>
@@ -24602,7 +24602,7 @@
         <v>3</v>
       </c>
       <c r="V279" t="n">
-        <v>24.36666666666666</v>
+        <v>24.36666666666667</v>
       </c>
       <c r="W279" t="n">
         <v>17.5</v>
@@ -25426,10 +25426,10 @@
         <v>21</v>
       </c>
       <c r="J289" t="n">
-        <v>22.2</v>
+        <v>23</v>
       </c>
       <c r="K289" t="n">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="L289" t="inlineStr">
         <is>
@@ -25459,7 +25459,7 @@
         <v>21</v>
       </c>
       <c r="S289" t="n">
-        <v>1.199999999999999</v>
+        <v>2</v>
       </c>
       <c r="T289" t="n">
         <v>22.03333333333333</v>
@@ -26640,10 +26640,10 @@
         <v>21</v>
       </c>
       <c r="J303" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="K303" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L303" t="inlineStr">
         <is>
@@ -26673,10 +26673,10 @@
         <v>21</v>
       </c>
       <c r="S303" t="n">
-        <v>-1.100000000000001</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T303" t="n">
-        <v>19.63333333333334</v>
+        <v>19.63333333333333</v>
       </c>
       <c r="U303" t="n">
         <v>3</v>
@@ -27856,10 +27856,10 @@
         <v>24.5</v>
       </c>
       <c r="J317" t="n">
-        <v>26.8</v>
+        <v>22.5</v>
       </c>
       <c r="K317" t="n">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="L317" t="inlineStr">
         <is>
@@ -27889,7 +27889,7 @@
         <v>28</v>
       </c>
       <c r="S317" t="n">
-        <v>2.300000000000001</v>
+        <v>-2</v>
       </c>
       <c r="T317" t="n">
         <v>26.3</v>
@@ -27943,10 +27943,10 @@
         <v>24.5</v>
       </c>
       <c r="J318" t="n">
-        <v>23.7</v>
+        <v>28.3</v>
       </c>
       <c r="K318" t="n">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="L318" t="inlineStr">
         <is>
@@ -27976,7 +27976,7 @@
         <v>28</v>
       </c>
       <c r="S318" t="n">
-        <v>-0.8000000000000007</v>
+        <v>3.800000000000001</v>
       </c>
       <c r="T318" t="n">
         <v>25.7</v>
@@ -28465,10 +28465,10 @@
         <v>24.5</v>
       </c>
       <c r="J324" t="n">
-        <v>23.6</v>
+        <v>27</v>
       </c>
       <c r="K324" t="n">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="L324" t="inlineStr">
         <is>
@@ -28498,7 +28498,7 @@
         <v>28</v>
       </c>
       <c r="S324" t="n">
-        <v>-0.8999999999999986</v>
+        <v>2.5</v>
       </c>
       <c r="T324" t="n">
         <v>24.93333333333333</v>
@@ -28726,10 +28726,10 @@
         <v>24.5</v>
       </c>
       <c r="J327" t="n">
-        <v>27.3</v>
+        <v>20.8</v>
       </c>
       <c r="K327" t="n">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -28759,7 +28759,7 @@
         <v>28</v>
       </c>
       <c r="S327" t="n">
-        <v>2.800000000000001</v>
+        <v>-3.699999999999999</v>
       </c>
       <c r="T327" t="n">
         <v>22.6</v>
@@ -30553,10 +30553,10 @@
         <v>24.5</v>
       </c>
       <c r="J348" t="n">
-        <v>24.1</v>
+        <v>26.7</v>
       </c>
       <c r="K348" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="L348" t="inlineStr">
         <is>
@@ -30586,7 +30586,7 @@
         <v>28</v>
       </c>
       <c r="S348" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="T348" t="n">
         <v>24.9</v>
@@ -30640,10 +30640,10 @@
         <v>24.5</v>
       </c>
       <c r="J349" t="n">
-        <v>22.9</v>
+        <v>27.8</v>
       </c>
       <c r="K349" t="n">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="L349" t="inlineStr">
         <is>
@@ -30673,7 +30673,7 @@
         <v>28</v>
       </c>
       <c r="S349" t="n">
-        <v>-1.600000000000001</v>
+        <v>3.300000000000001</v>
       </c>
       <c r="T349" t="n">
         <v>25</v>
@@ -30727,10 +30727,10 @@
         <v>24.5</v>
       </c>
       <c r="J350" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="K350" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="L350" t="inlineStr">
         <is>
@@ -30760,10 +30760,10 @@
         <v>28</v>
       </c>
       <c r="S350" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="T350" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="U350" t="n">
         <v>3</v>
@@ -31334,10 +31334,10 @@
         <v>24.5</v>
       </c>
       <c r="J357" t="n">
-        <v>22.7</v>
+        <v>29.1</v>
       </c>
       <c r="K357" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="L357" t="inlineStr">
         <is>
@@ -31367,7 +31367,7 @@
         <v>28</v>
       </c>
       <c r="S357" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="T357" t="n">
         <v>25.3</v>
@@ -31593,10 +31593,10 @@
         <v>21</v>
       </c>
       <c r="J360" t="n">
-        <v>17.6</v>
+        <v>18.2</v>
       </c>
       <c r="K360" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31624,16 +31624,16 @@
       </c>
       <c r="R360" t="inlineStr"/>
       <c r="S360" t="n">
-        <v>-3.399999999999999</v>
+        <v>-2.800000000000001</v>
       </c>
       <c r="T360" t="n">
-        <v>18.13333333333334</v>
+        <v>18.13333333333333</v>
       </c>
       <c r="U360" t="n">
         <v>3</v>
       </c>
       <c r="V360" t="n">
-        <v>27.25555555555556</v>
+        <v>27.25555555555555</v>
       </c>
       <c r="W360" t="n">
         <v>17.5</v>
@@ -31678,10 +31678,10 @@
         <v>21</v>
       </c>
       <c r="J361" t="n">
-        <v>20.2</v>
+        <v>21.1</v>
       </c>
       <c r="K361" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L361" t="inlineStr">
         <is>
@@ -31711,7 +31711,7 @@
         <v>21</v>
       </c>
       <c r="S361" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T361" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-26 07:10:06
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5834,10 +5834,10 @@
         <v>28</v>
       </c>
       <c r="J63" t="n">
-        <v>26.2</v>
+        <v>25.6</v>
       </c>
       <c r="K63" t="n">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
@@ -5867,7 +5867,7 @@
         <v>28</v>
       </c>
       <c r="S63" t="n">
-        <v>-1.800000000000001</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="T63" t="n">
         <v>26.1</v>
@@ -9472,10 +9472,10 @@
         <v>35</v>
       </c>
       <c r="J105" t="n">
-        <v>34.1</v>
+        <v>39.8</v>
       </c>
       <c r="K105" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
@@ -9505,7 +9505,7 @@
         <v>41</v>
       </c>
       <c r="S105" t="n">
-        <v>-0.8999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T105" t="n">
         <v>36.83333333333334</v>
@@ -9994,10 +9994,10 @@
         <v>35</v>
       </c>
       <c r="J111" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="K111" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
@@ -10027,7 +10027,7 @@
         <v>41</v>
       </c>
       <c r="S111" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="T111" t="n">
         <v>25.5</v>
@@ -10951,10 +10951,10 @@
         <v>21</v>
       </c>
       <c r="J122" t="n">
-        <v>21.6</v>
+        <v>19.4</v>
       </c>
       <c r="K122" t="n">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="L122" t="inlineStr">
         <is>
@@ -10984,7 +10984,7 @@
         <v>21</v>
       </c>
       <c r="S122" t="n">
-        <v>0.6000000000000014</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T122" t="n">
         <v>19.93333333333333</v>
@@ -11212,10 +11212,10 @@
         <v>28</v>
       </c>
       <c r="J125" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="K125" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -11245,7 +11245,7 @@
         <v>28</v>
       </c>
       <c r="S125" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="T125" t="n">
         <v>25.36666666666666</v>
@@ -12080,10 +12080,10 @@
         <v>35</v>
       </c>
       <c r="J135" t="n">
-        <v>45.3</v>
+        <v>45.2</v>
       </c>
       <c r="K135" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="L135" t="inlineStr">
         <is>
@@ -12113,7 +12113,7 @@
         <v>41</v>
       </c>
       <c r="S135" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="T135" t="n">
         <v>41</v>
@@ -12861,10 +12861,10 @@
         <v>35</v>
       </c>
       <c r="J144" t="n">
-        <v>38.6</v>
+        <v>32.9</v>
       </c>
       <c r="K144" t="n">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="L144" t="inlineStr">
         <is>
@@ -12894,10 +12894,10 @@
         <v>41</v>
       </c>
       <c r="S144" t="n">
-        <v>3.600000000000001</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="T144" t="n">
-        <v>36.56666666666667</v>
+        <v>36.56666666666666</v>
       </c>
       <c r="U144" t="n">
         <v>3</v>
@@ -18761,10 +18761,10 @@
         <v>31</v>
       </c>
       <c r="J212" t="n">
-        <v>33.7</v>
+        <v>36.5</v>
       </c>
       <c r="K212" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="L212" t="inlineStr">
         <is>
@@ -18792,7 +18792,7 @@
       </c>
       <c r="R212" t="inlineStr"/>
       <c r="S212" t="n">
-        <v>2.700000000000003</v>
+        <v>5.5</v>
       </c>
       <c r="T212" t="n">
         <v>33.66666666666666</v>
@@ -21618,10 +21618,10 @@
         <v>21</v>
       </c>
       <c r="J245" t="n">
-        <v>21.2</v>
+        <v>21.5</v>
       </c>
       <c r="K245" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L245" t="inlineStr">
         <is>
@@ -21651,7 +21651,7 @@
         <v>21</v>
       </c>
       <c r="S245" t="n">
-        <v>0.1999999999999993</v>
+        <v>0.5</v>
       </c>
       <c r="T245" t="n">
         <v>21.2</v>
@@ -22567,10 +22567,10 @@
         <v>28</v>
       </c>
       <c r="J256" t="n">
-        <v>27.1</v>
+        <v>27.6</v>
       </c>
       <c r="K256" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="L256" t="inlineStr">
         <is>
@@ -22600,7 +22600,7 @@
         <v>28</v>
       </c>
       <c r="S256" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T256" t="n">
         <v>27.4</v>
@@ -22654,10 +22654,10 @@
         <v>28</v>
       </c>
       <c r="J257" t="n">
-        <v>28.1</v>
+        <v>28.9</v>
       </c>
       <c r="K257" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="L257" t="inlineStr">
         <is>
@@ -22687,7 +22687,7 @@
         <v>28</v>
       </c>
       <c r="S257" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T257" t="n">
         <v>28.03333333333333</v>
@@ -22741,10 +22741,10 @@
         <v>28</v>
       </c>
       <c r="J258" t="n">
-        <v>28.4</v>
+        <v>27.2</v>
       </c>
       <c r="K258" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="L258" t="inlineStr">
         <is>
@@ -22774,10 +22774,10 @@
         <v>28</v>
       </c>
       <c r="S258" t="n">
-        <v>0.3999999999999986</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T258" t="n">
-        <v>28.06666666666667</v>
+        <v>28.06666666666666</v>
       </c>
       <c r="U258" t="n">
         <v>3</v>
@@ -26903,10 +26903,10 @@
         <v>21</v>
       </c>
       <c r="J306" t="n">
-        <v>26.5</v>
+        <v>20.6</v>
       </c>
       <c r="K306" t="n">
-        <v>126</v>
+        <v>98</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -26936,7 +26936,7 @@
         <v>21</v>
       </c>
       <c r="S306" t="n">
-        <v>5.5</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T306" t="n">
         <v>23.9</v>
@@ -28032,10 +28032,10 @@
         <v>24.5</v>
       </c>
       <c r="J319" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K319" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L319" t="inlineStr">
         <is>
@@ -28065,7 +28065,7 @@
         <v>28</v>
       </c>
       <c r="S319" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T319" t="n">
         <v>24.66666666666667</v>
@@ -28728,10 +28728,10 @@
         <v>24.5</v>
       </c>
       <c r="J327" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K327" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -28761,7 +28761,7 @@
         <v>28</v>
       </c>
       <c r="S327" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T327" t="n">
         <v>27.1</v>
@@ -30642,10 +30642,10 @@
         <v>24.5</v>
       </c>
       <c r="J349" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K349" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L349" t="inlineStr">
         <is>
@@ -30675,10 +30675,10 @@
         <v>28</v>
       </c>
       <c r="S349" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T349" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U349" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-26 15:50:01
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3161,10 +3161,10 @@
         <v>31</v>
       </c>
       <c r="J32" t="n">
-        <v>31.4</v>
+        <v>30</v>
       </c>
       <c r="K32" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1</v>
       </c>
       <c r="T32" t="n">
         <v>30.33333333333333</v>
@@ -6137,7 +6137,7 @@
         <v>3</v>
       </c>
       <c r="V66" t="n">
-        <v>37.02962962962963</v>
+        <v>37.02962962962962</v>
       </c>
       <c r="W66" t="n">
         <v>31.5</v>
@@ -6311,7 +6311,7 @@
         <v>3</v>
       </c>
       <c r="V68" t="n">
-        <v>38.42962962962963</v>
+        <v>38.42962962962962</v>
       </c>
       <c r="W68" t="n">
         <v>31.5</v>
@@ -6530,10 +6530,10 @@
         <v>35</v>
       </c>
       <c r="J71" t="n">
-        <v>33.5</v>
+        <v>38.4</v>
       </c>
       <c r="K71" t="n">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -6563,10 +6563,10 @@
         <v>41</v>
       </c>
       <c r="S71" t="n">
-        <v>-1.5</v>
+        <v>3.399999999999999</v>
       </c>
       <c r="T71" t="n">
-        <v>37.56666666666667</v>
+        <v>37.56666666666666</v>
       </c>
       <c r="U71" t="n">
         <v>3</v>
@@ -6876,10 +6876,10 @@
         <v>28</v>
       </c>
       <c r="J75" t="n">
-        <v>24.8</v>
+        <v>25.9</v>
       </c>
       <c r="K75" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6909,10 +6909,10 @@
         <v>28</v>
       </c>
       <c r="S75" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="T75" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="U75" t="n">
         <v>3</v>
@@ -9472,10 +9472,10 @@
         <v>35</v>
       </c>
       <c r="J105" t="n">
-        <v>39.8</v>
+        <v>34.1</v>
       </c>
       <c r="K105" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
@@ -9505,7 +9505,7 @@
         <v>41</v>
       </c>
       <c r="S105" t="n">
-        <v>4.799999999999997</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T105" t="n">
         <v>36.83333333333334</v>
@@ -9994,10 +9994,10 @@
         <v>35</v>
       </c>
       <c r="J111" t="n">
-        <v>27.7</v>
+        <v>22.5</v>
       </c>
       <c r="K111" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
@@ -10027,7 +10027,7 @@
         <v>41</v>
       </c>
       <c r="S111" t="n">
-        <v>-7.300000000000001</v>
+        <v>-12.5</v>
       </c>
       <c r="T111" t="n">
         <v>25.5</v>
@@ -10951,10 +10951,10 @@
         <v>21</v>
       </c>
       <c r="J122" t="n">
-        <v>19.4</v>
+        <v>21.6</v>
       </c>
       <c r="K122" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="L122" t="inlineStr">
         <is>
@@ -10984,7 +10984,7 @@
         <v>21</v>
       </c>
       <c r="S122" t="n">
-        <v>-1.600000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T122" t="n">
         <v>19.93333333333333</v>
@@ -12080,10 +12080,10 @@
         <v>35</v>
       </c>
       <c r="J135" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="K135" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="L135" t="inlineStr">
         <is>
@@ -12113,7 +12113,7 @@
         <v>41</v>
       </c>
       <c r="S135" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="T135" t="n">
         <v>41</v>
@@ -12776,10 +12776,10 @@
         <v>35</v>
       </c>
       <c r="J143" t="n">
-        <v>48.5</v>
+        <v>20.3</v>
       </c>
       <c r="K143" t="n">
-        <v>138</v>
+        <v>58</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
@@ -12809,7 +12809,7 @@
         <v>41</v>
       </c>
       <c r="S143" t="n">
-        <v>13.5</v>
+        <v>-14.7</v>
       </c>
       <c r="T143" t="n">
         <v>30.76666666666667</v>
@@ -12861,10 +12861,10 @@
         <v>35</v>
       </c>
       <c r="J144" t="n">
-        <v>32.9</v>
+        <v>38.6</v>
       </c>
       <c r="K144" t="n">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="L144" t="inlineStr">
         <is>
@@ -12894,10 +12894,10 @@
         <v>41</v>
       </c>
       <c r="S144" t="n">
-        <v>-2.100000000000001</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T144" t="n">
-        <v>36.56666666666666</v>
+        <v>36.56666666666667</v>
       </c>
       <c r="U144" t="n">
         <v>3</v>
@@ -13379,10 +13379,10 @@
         <v>35</v>
       </c>
       <c r="J150" t="n">
-        <v>32.4</v>
+        <v>37.3</v>
       </c>
       <c r="K150" t="n">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="L150" t="inlineStr">
         <is>
@@ -13412,10 +13412,10 @@
         <v>41</v>
       </c>
       <c r="S150" t="n">
-        <v>-2.600000000000001</v>
+        <v>2.299999999999997</v>
       </c>
       <c r="T150" t="n">
-        <v>36.6</v>
+        <v>36.59999999999999</v>
       </c>
       <c r="U150" t="n">
         <v>3</v>
@@ -14247,10 +14247,10 @@
         <v>21</v>
       </c>
       <c r="J160" t="n">
-        <v>23.9</v>
+        <v>26</v>
       </c>
       <c r="K160" t="n">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="L160" t="inlineStr">
         <is>
@@ -14280,7 +14280,7 @@
         <v>21</v>
       </c>
       <c r="S160" t="n">
-        <v>2.899999999999999</v>
+        <v>5</v>
       </c>
       <c r="T160" t="n">
         <v>23.4</v>
@@ -14334,10 +14334,10 @@
         <v>21</v>
       </c>
       <c r="J161" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="K161" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="L161" t="inlineStr">
         <is>
@@ -14367,7 +14367,7 @@
         <v>21</v>
       </c>
       <c r="S161" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="T161" t="n">
         <v>22.96666666666667</v>
@@ -14506,10 +14506,10 @@
         <v>21</v>
       </c>
       <c r="J163" t="n">
-        <v>25.1</v>
+        <v>20.4</v>
       </c>
       <c r="K163" t="n">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="L163" t="inlineStr">
         <is>
@@ -14539,7 +14539,7 @@
         <v>21</v>
       </c>
       <c r="S163" t="n">
-        <v>4.100000000000001</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T163" t="n">
         <v>24.33333333333333</v>
@@ -14593,10 +14593,10 @@
         <v>35</v>
       </c>
       <c r="J164" t="n">
-        <v>34.7</v>
+        <v>37.2</v>
       </c>
       <c r="K164" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="L164" t="inlineStr">
         <is>
@@ -14626,7 +14626,7 @@
         <v>41</v>
       </c>
       <c r="S164" t="n">
-        <v>-0.2999999999999972</v>
+        <v>2.200000000000003</v>
       </c>
       <c r="T164" t="n">
         <v>37.26666666666667</v>
@@ -14680,10 +14680,10 @@
         <v>21</v>
       </c>
       <c r="J165" t="n">
-        <v>20.8</v>
+        <v>23.4</v>
       </c>
       <c r="K165" t="n">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="L165" t="inlineStr">
         <is>
@@ -14713,7 +14713,7 @@
         <v>21</v>
       </c>
       <c r="S165" t="n">
-        <v>-0.1999999999999993</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T165" t="n">
         <v>23.4</v>
@@ -18761,10 +18761,10 @@
         <v>31</v>
       </c>
       <c r="J212" t="n">
-        <v>36.5</v>
+        <v>33.7</v>
       </c>
       <c r="K212" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="L212" t="inlineStr">
         <is>
@@ -18792,7 +18792,7 @@
       </c>
       <c r="R212" t="inlineStr"/>
       <c r="S212" t="n">
-        <v>5.5</v>
+        <v>2.700000000000003</v>
       </c>
       <c r="T212" t="n">
         <v>33.66666666666666</v>
@@ -21618,10 +21618,10 @@
         <v>21</v>
       </c>
       <c r="J245" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="K245" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L245" t="inlineStr">
         <is>
@@ -21651,7 +21651,7 @@
         <v>21</v>
       </c>
       <c r="S245" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T245" t="n">
         <v>21.2</v>
@@ -21960,10 +21960,10 @@
         <v>21</v>
       </c>
       <c r="J249" t="n">
-        <v>21.3</v>
+        <v>23.8</v>
       </c>
       <c r="K249" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="L249" t="inlineStr">
         <is>
@@ -21991,7 +21991,7 @@
       </c>
       <c r="R249" t="inlineStr"/>
       <c r="S249" t="n">
-        <v>0.3000000000000007</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T249" t="n">
         <v>21.8</v>
@@ -24823,10 +24823,10 @@
         <v>21</v>
       </c>
       <c r="J282" t="n">
-        <v>22</v>
+        <v>20.8</v>
       </c>
       <c r="K282" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L282" t="inlineStr">
         <is>
@@ -24856,7 +24856,7 @@
         <v>21</v>
       </c>
       <c r="S282" t="n">
-        <v>1</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T282" t="n">
         <v>21.03333333333333</v>
@@ -25254,10 +25254,10 @@
         <v>21</v>
       </c>
       <c r="J287" t="n">
-        <v>22.8</v>
+        <v>21.7</v>
       </c>
       <c r="K287" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="L287" t="inlineStr">
         <is>
@@ -25287,7 +25287,7 @@
         <v>21</v>
       </c>
       <c r="S287" t="n">
-        <v>1.800000000000001</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T287" t="n">
         <v>21.53333333333333</v>
@@ -26555,10 +26555,10 @@
         <v>21</v>
       </c>
       <c r="J302" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="K302" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L302" t="inlineStr">
         <is>
@@ -26588,10 +26588,10 @@
         <v>21</v>
       </c>
       <c r="S302" t="n">
-        <v>-1.100000000000001</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T302" t="n">
-        <v>19.63333333333334</v>
+        <v>19.63333333333333</v>
       </c>
       <c r="U302" t="n">
         <v>3</v>
@@ -27075,10 +27075,10 @@
         <v>24.5</v>
       </c>
       <c r="J308" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="K308" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="L308" t="inlineStr">
         <is>
@@ -27108,7 +27108,7 @@
         <v>28</v>
       </c>
       <c r="S308" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T308" t="n">
         <v>25.13333333333334</v>
@@ -28032,10 +28032,10 @@
         <v>24.5</v>
       </c>
       <c r="J319" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="K319" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L319" t="inlineStr">
         <is>
@@ -28065,7 +28065,7 @@
         <v>28</v>
       </c>
       <c r="S319" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T319" t="n">
         <v>24.66666666666667</v>
@@ -28728,10 +28728,10 @@
         <v>24.5</v>
       </c>
       <c r="J327" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="K327" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -28761,7 +28761,7 @@
         <v>28</v>
       </c>
       <c r="S327" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T327" t="n">
         <v>27.1</v>
@@ -29250,10 +29250,10 @@
         <v>24.5</v>
       </c>
       <c r="J333" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="K333" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -29283,7 +29283,7 @@
         <v>28</v>
       </c>
       <c r="S333" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T333" t="n">
         <v>35.8</v>
@@ -30642,10 +30642,10 @@
         <v>24.5</v>
       </c>
       <c r="J349" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="K349" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="L349" t="inlineStr">
         <is>
@@ -30675,10 +30675,10 @@
         <v>28</v>
       </c>
       <c r="S349" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="T349" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="U349" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-26 17:52:43
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3161,10 +3161,10 @@
         <v>31</v>
       </c>
       <c r="J32" t="n">
-        <v>30</v>
+        <v>31.4</v>
       </c>
       <c r="K32" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="n">
-        <v>-1</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T32" t="n">
         <v>30.33333333333333</v>
@@ -6137,7 +6137,7 @@
         <v>3</v>
       </c>
       <c r="V66" t="n">
-        <v>37.02962962962962</v>
+        <v>37.02962962962963</v>
       </c>
       <c r="W66" t="n">
         <v>31.5</v>
@@ -6311,7 +6311,7 @@
         <v>3</v>
       </c>
       <c r="V68" t="n">
-        <v>38.42962962962962</v>
+        <v>38.42962962962963</v>
       </c>
       <c r="W68" t="n">
         <v>31.5</v>
@@ -6530,10 +6530,10 @@
         <v>35</v>
       </c>
       <c r="J71" t="n">
-        <v>38.4</v>
+        <v>33.5</v>
       </c>
       <c r="K71" t="n">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -6563,10 +6563,10 @@
         <v>41</v>
       </c>
       <c r="S71" t="n">
-        <v>3.399999999999999</v>
+        <v>-1.5</v>
       </c>
       <c r="T71" t="n">
-        <v>37.56666666666666</v>
+        <v>37.56666666666667</v>
       </c>
       <c r="U71" t="n">
         <v>3</v>
@@ -6704,10 +6704,10 @@
         <v>31</v>
       </c>
       <c r="J73" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="K73" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -6735,7 +6735,7 @@
       </c>
       <c r="R73" t="inlineStr"/>
       <c r="S73" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T73" t="n">
         <v>32.03333333333333</v>
@@ -6876,10 +6876,10 @@
         <v>28</v>
       </c>
       <c r="J75" t="n">
-        <v>25.9</v>
+        <v>24.8</v>
       </c>
       <c r="K75" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6909,10 +6909,10 @@
         <v>28</v>
       </c>
       <c r="S75" t="n">
-        <v>-2.100000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T75" t="n">
-        <v>25.13333333333333</v>
+        <v>25.13333333333334</v>
       </c>
       <c r="U75" t="n">
         <v>3</v>
@@ -7050,10 +7050,10 @@
         <v>31</v>
       </c>
       <c r="J77" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="K77" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="T77" t="n">
         <v>36</v>
@@ -7657,10 +7657,10 @@
         <v>31</v>
       </c>
       <c r="J84" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="K84" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T84" t="n">
         <v>33.63333333333333</v>
@@ -8090,10 +8090,10 @@
         <v>31</v>
       </c>
       <c r="J89" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="K89" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="R89" t="inlineStr"/>
       <c r="S89" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T89" t="n">
         <v>32.76666666666667</v>
@@ -9472,10 +9472,10 @@
         <v>35</v>
       </c>
       <c r="J105" t="n">
-        <v>34.1</v>
+        <v>39.8</v>
       </c>
       <c r="K105" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
@@ -9505,7 +9505,7 @@
         <v>41</v>
       </c>
       <c r="S105" t="n">
-        <v>-0.8999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T105" t="n">
         <v>36.83333333333334</v>
@@ -11212,10 +11212,10 @@
         <v>28</v>
       </c>
       <c r="J125" t="n">
-        <v>24.6</v>
+        <v>27.7</v>
       </c>
       <c r="K125" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
@@ -11245,7 +11245,7 @@
         <v>28</v>
       </c>
       <c r="S125" t="n">
-        <v>-3.399999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T125" t="n">
         <v>25.36666666666666</v>
@@ -12776,10 +12776,10 @@
         <v>35</v>
       </c>
       <c r="J143" t="n">
-        <v>20.3</v>
+        <v>48.5</v>
       </c>
       <c r="K143" t="n">
-        <v>58</v>
+        <v>138</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
@@ -12809,7 +12809,7 @@
         <v>41</v>
       </c>
       <c r="S143" t="n">
-        <v>-14.7</v>
+        <v>13.5</v>
       </c>
       <c r="T143" t="n">
         <v>30.76666666666667</v>
@@ -13379,10 +13379,10 @@
         <v>35</v>
       </c>
       <c r="J150" t="n">
-        <v>37.3</v>
+        <v>32.4</v>
       </c>
       <c r="K150" t="n">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="L150" t="inlineStr">
         <is>
@@ -13412,10 +13412,10 @@
         <v>41</v>
       </c>
       <c r="S150" t="n">
-        <v>2.299999999999997</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T150" t="n">
-        <v>36.59999999999999</v>
+        <v>36.6</v>
       </c>
       <c r="U150" t="n">
         <v>3</v>
@@ -14247,10 +14247,10 @@
         <v>21</v>
       </c>
       <c r="J160" t="n">
-        <v>26</v>
+        <v>23.9</v>
       </c>
       <c r="K160" t="n">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="L160" t="inlineStr">
         <is>
@@ -14280,7 +14280,7 @@
         <v>21</v>
       </c>
       <c r="S160" t="n">
-        <v>5</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="T160" t="n">
         <v>23.4</v>
@@ -14334,10 +14334,10 @@
         <v>21</v>
       </c>
       <c r="J161" t="n">
-        <v>20.9</v>
+        <v>22.9</v>
       </c>
       <c r="K161" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="L161" t="inlineStr">
         <is>
@@ -14367,7 +14367,7 @@
         <v>21</v>
       </c>
       <c r="S161" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T161" t="n">
         <v>22.96666666666667</v>
@@ -14506,10 +14506,10 @@
         <v>21</v>
       </c>
       <c r="J163" t="n">
-        <v>20.4</v>
+        <v>25.1</v>
       </c>
       <c r="K163" t="n">
-        <v>97</v>
+        <v>119</v>
       </c>
       <c r="L163" t="inlineStr">
         <is>
@@ -14539,7 +14539,7 @@
         <v>21</v>
       </c>
       <c r="S163" t="n">
-        <v>-0.6000000000000014</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T163" t="n">
         <v>24.33333333333333</v>
@@ -14593,10 +14593,10 @@
         <v>35</v>
       </c>
       <c r="J164" t="n">
-        <v>37.2</v>
+        <v>34.7</v>
       </c>
       <c r="K164" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="L164" t="inlineStr">
         <is>
@@ -14626,7 +14626,7 @@
         <v>41</v>
       </c>
       <c r="S164" t="n">
-        <v>2.200000000000003</v>
+        <v>-0.2999999999999972</v>
       </c>
       <c r="T164" t="n">
         <v>37.26666666666667</v>
@@ -14680,10 +14680,10 @@
         <v>21</v>
       </c>
       <c r="J165" t="n">
-        <v>23.4</v>
+        <v>20.8</v>
       </c>
       <c r="K165" t="n">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="L165" t="inlineStr">
         <is>
@@ -14713,7 +14713,7 @@
         <v>21</v>
       </c>
       <c r="S165" t="n">
-        <v>2.399999999999999</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T165" t="n">
         <v>23.4</v>
@@ -21618,10 +21618,10 @@
         <v>21</v>
       </c>
       <c r="J245" t="n">
-        <v>21.2</v>
+        <v>21.5</v>
       </c>
       <c r="K245" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L245" t="inlineStr">
         <is>
@@ -21651,7 +21651,7 @@
         <v>21</v>
       </c>
       <c r="S245" t="n">
-        <v>0.1999999999999993</v>
+        <v>0.5</v>
       </c>
       <c r="T245" t="n">
         <v>21.2</v>
@@ -21960,10 +21960,10 @@
         <v>21</v>
       </c>
       <c r="J249" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="K249" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="L249" t="inlineStr">
         <is>
@@ -21991,7 +21991,7 @@
       </c>
       <c r="R249" t="inlineStr"/>
       <c r="S249" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="T249" t="n">
         <v>21.8</v>
@@ -24823,10 +24823,10 @@
         <v>21</v>
       </c>
       <c r="J282" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="K282" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L282" t="inlineStr">
         <is>
@@ -24856,7 +24856,7 @@
         <v>21</v>
       </c>
       <c r="S282" t="n">
-        <v>-0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="T282" t="n">
         <v>21.03333333333333</v>
@@ -25254,10 +25254,10 @@
         <v>21</v>
       </c>
       <c r="J287" t="n">
-        <v>21.7</v>
+        <v>22.8</v>
       </c>
       <c r="K287" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="L287" t="inlineStr">
         <is>
@@ -25287,7 +25287,7 @@
         <v>21</v>
       </c>
       <c r="S287" t="n">
-        <v>0.6999999999999993</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="T287" t="n">
         <v>21.53333333333333</v>
@@ -26555,10 +26555,10 @@
         <v>21</v>
       </c>
       <c r="J302" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="K302" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L302" t="inlineStr">
         <is>
@@ -26588,10 +26588,10 @@
         <v>21</v>
       </c>
       <c r="S302" t="n">
-        <v>-1.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="T302" t="n">
-        <v>19.63333333333333</v>
+        <v>19.63333333333334</v>
       </c>
       <c r="U302" t="n">
         <v>3</v>
@@ -27075,10 +27075,10 @@
         <v>24.5</v>
       </c>
       <c r="J308" t="n">
-        <v>23.9</v>
+        <v>25.1</v>
       </c>
       <c r="K308" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="L308" t="inlineStr">
         <is>
@@ -27108,7 +27108,7 @@
         <v>28</v>
       </c>
       <c r="S308" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="T308" t="n">
         <v>25.13333333333334</v>
@@ -28032,10 +28032,10 @@
         <v>24.5</v>
       </c>
       <c r="J319" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K319" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L319" t="inlineStr">
         <is>
@@ -28065,7 +28065,7 @@
         <v>28</v>
       </c>
       <c r="S319" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T319" t="n">
         <v>24.66666666666667</v>
@@ -28728,10 +28728,10 @@
         <v>24.5</v>
       </c>
       <c r="J327" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K327" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -28761,7 +28761,7 @@
         <v>28</v>
       </c>
       <c r="S327" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T327" t="n">
         <v>27.1</v>
@@ -29250,10 +29250,10 @@
         <v>24.5</v>
       </c>
       <c r="J333" t="n">
-        <v>25.6</v>
+        <v>24</v>
       </c>
       <c r="K333" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -29283,7 +29283,7 @@
         <v>28</v>
       </c>
       <c r="S333" t="n">
-        <v>1.100000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="T333" t="n">
         <v>35.8</v>
@@ -30642,10 +30642,10 @@
         <v>24.5</v>
       </c>
       <c r="J349" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K349" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L349" t="inlineStr">
         <is>
@@ -30675,10 +30675,10 @@
         <v>28</v>
       </c>
       <c r="S349" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T349" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U349" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-26 19:04:53
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3501,10 +3501,10 @@
         <v>24</v>
       </c>
       <c r="J36" t="n">
-        <v>25.6</v>
+        <v>21.4</v>
       </c>
       <c r="K36" t="n">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -3534,7 +3534,7 @@
         <v>28</v>
       </c>
       <c r="S36" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T36" t="n">
         <v>23.8</v>
@@ -6704,10 +6704,10 @@
         <v>31</v>
       </c>
       <c r="J73" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K73" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -6735,7 +6735,7 @@
       </c>
       <c r="R73" t="inlineStr"/>
       <c r="S73" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T73" t="n">
         <v>32.03333333333333</v>
@@ -6876,7 +6876,7 @@
         <v>28</v>
       </c>
       <c r="J75" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="K75" t="n">
         <v>88</v>
@@ -6909,7 +6909,7 @@
         <v>28</v>
       </c>
       <c r="S75" t="n">
-        <v>-3.199999999999999</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="T75" t="n">
         <v>25.13333333333334</v>
@@ -7050,10 +7050,10 @@
         <v>31</v>
       </c>
       <c r="J77" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K77" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T77" t="n">
         <v>36</v>
@@ -7570,10 +7570,10 @@
         <v>21</v>
       </c>
       <c r="J83" t="n">
-        <v>19.3</v>
+        <v>26</v>
       </c>
       <c r="K83" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -7603,7 +7603,7 @@
         <v>21</v>
       </c>
       <c r="S83" t="n">
-        <v>-1.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="T83" t="n">
         <v>22</v>
@@ -7657,10 +7657,10 @@
         <v>31</v>
       </c>
       <c r="J84" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K84" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T84" t="n">
         <v>33.63333333333333</v>
@@ -8090,10 +8090,10 @@
         <v>31</v>
       </c>
       <c r="J89" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K89" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="R89" t="inlineStr"/>
       <c r="S89" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T89" t="n">
         <v>32.76666666666667</v>
@@ -9994,10 +9994,10 @@
         <v>35</v>
       </c>
       <c r="J111" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="K111" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
@@ -10027,7 +10027,7 @@
         <v>41</v>
       </c>
       <c r="S111" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="T111" t="n">
         <v>25.5</v>
@@ -10603,10 +10603,10 @@
         <v>21</v>
       </c>
       <c r="J118" t="n">
-        <v>19.3</v>
+        <v>26</v>
       </c>
       <c r="K118" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -10636,7 +10636,7 @@
         <v>21</v>
       </c>
       <c r="S118" t="n">
-        <v>-1.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="T118" t="n">
         <v>23.7</v>
@@ -16849,10 +16849,10 @@
         <v>21</v>
       </c>
       <c r="J190" t="n">
-        <v>20.7</v>
+        <v>23</v>
       </c>
       <c r="K190" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="L190" t="inlineStr">
         <is>
@@ -16882,7 +16882,7 @@
         <v>21</v>
       </c>
       <c r="S190" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2</v>
       </c>
       <c r="T190" t="n">
         <v>21.5</v>
@@ -18933,10 +18933,10 @@
         <v>28</v>
       </c>
       <c r="J214" t="n">
-        <v>28.5</v>
+        <v>27.7</v>
       </c>
       <c r="K214" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -18966,7 +18966,7 @@
         <v>28</v>
       </c>
       <c r="S214" t="n">
-        <v>0.5</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T214" t="n">
         <v>28.33333333333333</v>
@@ -19890,10 +19890,10 @@
         <v>28</v>
       </c>
       <c r="J225" t="n">
-        <v>29.3</v>
+        <v>30.1</v>
       </c>
       <c r="K225" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="L225" t="inlineStr">
         <is>
@@ -19923,7 +19923,7 @@
         <v>28</v>
       </c>
       <c r="S225" t="n">
-        <v>1.300000000000001</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="T225" t="n">
         <v>28.96666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-26 20:32:47
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3501,10 +3501,10 @@
         <v>24</v>
       </c>
       <c r="J36" t="n">
-        <v>21.4</v>
+        <v>25.6</v>
       </c>
       <c r="K36" t="n">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -3534,7 +3534,7 @@
         <v>28</v>
       </c>
       <c r="S36" t="n">
-        <v>-2.600000000000001</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T36" t="n">
         <v>23.8</v>
@@ -6704,10 +6704,10 @@
         <v>31</v>
       </c>
       <c r="J73" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="K73" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -6735,7 +6735,7 @@
       </c>
       <c r="R73" t="inlineStr"/>
       <c r="S73" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T73" t="n">
         <v>32.03333333333333</v>
@@ -6876,7 +6876,7 @@
         <v>28</v>
       </c>
       <c r="J75" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="K75" t="n">
         <v>88</v>
@@ -6909,7 +6909,7 @@
         <v>28</v>
       </c>
       <c r="S75" t="n">
-        <v>-3.300000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T75" t="n">
         <v>25.13333333333334</v>
@@ -7050,10 +7050,10 @@
         <v>31</v>
       </c>
       <c r="J77" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="K77" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="T77" t="n">
         <v>36</v>
@@ -7570,10 +7570,10 @@
         <v>21</v>
       </c>
       <c r="J83" t="n">
-        <v>26</v>
+        <v>19.3</v>
       </c>
       <c r="K83" t="n">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
@@ -7603,7 +7603,7 @@
         <v>21</v>
       </c>
       <c r="S83" t="n">
-        <v>5</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T83" t="n">
         <v>22</v>
@@ -7657,10 +7657,10 @@
         <v>31</v>
       </c>
       <c r="J84" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="K84" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T84" t="n">
         <v>33.63333333333333</v>
@@ -8090,10 +8090,10 @@
         <v>31</v>
       </c>
       <c r="J89" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="K89" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="R89" t="inlineStr"/>
       <c r="S89" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T89" t="n">
         <v>32.76666666666667</v>
@@ -9994,10 +9994,10 @@
         <v>35</v>
       </c>
       <c r="J111" t="n">
-        <v>27.7</v>
+        <v>22.5</v>
       </c>
       <c r="K111" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="L111" t="inlineStr">
         <is>
@@ -10027,7 +10027,7 @@
         <v>41</v>
       </c>
       <c r="S111" t="n">
-        <v>-7.300000000000001</v>
+        <v>-12.5</v>
       </c>
       <c r="T111" t="n">
         <v>25.5</v>
@@ -10603,10 +10603,10 @@
         <v>21</v>
       </c>
       <c r="J118" t="n">
-        <v>26</v>
+        <v>19.3</v>
       </c>
       <c r="K118" t="n">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="L118" t="inlineStr">
         <is>
@@ -10636,7 +10636,7 @@
         <v>21</v>
       </c>
       <c r="S118" t="n">
-        <v>5</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T118" t="n">
         <v>23.7</v>
@@ -16849,10 +16849,10 @@
         <v>21</v>
       </c>
       <c r="J190" t="n">
-        <v>23</v>
+        <v>20.7</v>
       </c>
       <c r="K190" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="L190" t="inlineStr">
         <is>
@@ -16882,7 +16882,7 @@
         <v>21</v>
       </c>
       <c r="S190" t="n">
-        <v>2</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T190" t="n">
         <v>21.5</v>
@@ -18933,10 +18933,10 @@
         <v>28</v>
       </c>
       <c r="J214" t="n">
-        <v>27.7</v>
+        <v>28.5</v>
       </c>
       <c r="K214" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="L214" t="inlineStr">
         <is>
@@ -18966,7 +18966,7 @@
         <v>28</v>
       </c>
       <c r="S214" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.5</v>
       </c>
       <c r="T214" t="n">
         <v>28.33333333333333</v>
@@ -19890,10 +19890,10 @@
         <v>28</v>
       </c>
       <c r="J225" t="n">
-        <v>30.1</v>
+        <v>29.3</v>
       </c>
       <c r="K225" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L225" t="inlineStr">
         <is>
@@ -19923,7 +19923,7 @@
         <v>28</v>
       </c>
       <c r="S225" t="n">
-        <v>2.100000000000001</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="T225" t="n">
         <v>28.96666666666667</v>
@@ -27510,10 +27510,10 @@
         <v>24.5</v>
       </c>
       <c r="J313" t="n">
-        <v>23.4</v>
+        <v>23.9</v>
       </c>
       <c r="K313" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="L313" t="inlineStr">
         <is>
@@ -27543,7 +27543,7 @@
         <v>28</v>
       </c>
       <c r="S313" t="n">
-        <v>-1.100000000000001</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T313" t="n">
         <v>23.56666666666666</v>
@@ -28032,10 +28032,10 @@
         <v>24.5</v>
       </c>
       <c r="J319" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="K319" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L319" t="inlineStr">
         <is>
@@ -28065,7 +28065,7 @@
         <v>28</v>
       </c>
       <c r="S319" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T319" t="n">
         <v>24.66666666666667</v>
@@ -28728,10 +28728,10 @@
         <v>24.5</v>
       </c>
       <c r="J327" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="K327" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -28761,7 +28761,7 @@
         <v>28</v>
       </c>
       <c r="S327" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T327" t="n">
         <v>27.1</v>
@@ -28989,10 +28989,10 @@
         <v>24.5</v>
       </c>
       <c r="J330" t="n">
-        <v>26.9</v>
+        <v>21</v>
       </c>
       <c r="K330" t="n">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="L330" t="inlineStr">
         <is>
@@ -29022,7 +29022,7 @@
         <v>28</v>
       </c>
       <c r="S330" t="n">
-        <v>2.399999999999999</v>
+        <v>-3.5</v>
       </c>
       <c r="T330" t="n">
         <v>24.26666666666667</v>
@@ -29511,10 +29511,10 @@
         <v>24.5</v>
       </c>
       <c r="J336" t="n">
-        <v>24.5</v>
+        <v>23.5</v>
       </c>
       <c r="K336" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L336" t="inlineStr">
         <is>
@@ -29544,7 +29544,7 @@
         <v>28</v>
       </c>
       <c r="S336" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T336" t="n">
         <v>24.13333333333334</v>
@@ -30642,10 +30642,10 @@
         <v>24.5</v>
       </c>
       <c r="J349" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="K349" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="L349" t="inlineStr">
         <is>
@@ -30675,10 +30675,10 @@
         <v>28</v>
       </c>
       <c r="S349" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="T349" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="U349" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-27 16:28:35
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5441,7 +5441,7 @@
         <v>3</v>
       </c>
       <c r="V58" t="n">
-        <v>24.52222222222222</v>
+        <v>24.52222222222223</v>
       </c>
       <c r="W58" t="n">
         <v>20.5</v>
@@ -5486,10 +5486,10 @@
         <v>24</v>
       </c>
       <c r="J59" t="n">
-        <v>16.6</v>
+        <v>26.4</v>
       </c>
       <c r="K59" t="n">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -5519,7 +5519,7 @@
         <v>28</v>
       </c>
       <c r="S59" t="n">
-        <v>-7.399999999999999</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T59" t="n">
         <v>23.4</v>
@@ -5528,7 +5528,7 @@
         <v>3</v>
       </c>
       <c r="V59" t="n">
-        <v>24.64444444444444</v>
+        <v>24.64444444444445</v>
       </c>
       <c r="W59" t="n">
         <v>20.5</v>
@@ -5921,10 +5921,10 @@
         <v>21</v>
       </c>
       <c r="J64" t="n">
-        <v>19.7</v>
+        <v>20.3</v>
       </c>
       <c r="K64" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -5954,7 +5954,7 @@
         <v>21</v>
       </c>
       <c r="S64" t="n">
-        <v>-1.300000000000001</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T64" t="n">
         <v>20.03333333333333</v>
@@ -6008,10 +6008,10 @@
         <v>35</v>
       </c>
       <c r="J65" t="n">
-        <v>34.3</v>
+        <v>32.3</v>
       </c>
       <c r="K65" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -6041,7 +6041,7 @@
         <v>41</v>
       </c>
       <c r="S65" t="n">
-        <v>-0.7000000000000028</v>
+        <v>-2.700000000000003</v>
       </c>
       <c r="T65" t="n">
         <v>32.96666666666666</v>
@@ -6095,10 +6095,10 @@
         <v>35</v>
       </c>
       <c r="J66" t="n">
-        <v>38.1</v>
+        <v>31.8</v>
       </c>
       <c r="K66" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -6128,7 +6128,7 @@
         <v>41</v>
       </c>
       <c r="S66" t="n">
-        <v>3.100000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T66" t="n">
         <v>35.3</v>
@@ -6137,7 +6137,7 @@
         <v>3</v>
       </c>
       <c r="V66" t="n">
-        <v>37.02962962962963</v>
+        <v>37.02962962962962</v>
       </c>
       <c r="W66" t="n">
         <v>31.5</v>
@@ -6182,10 +6182,10 @@
         <v>21</v>
       </c>
       <c r="J67" t="n">
-        <v>17.9</v>
+        <v>17.6</v>
       </c>
       <c r="K67" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -6215,7 +6215,7 @@
         <v>21</v>
       </c>
       <c r="S67" t="n">
-        <v>-3.100000000000001</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="T67" t="n">
         <v>18.86666666666667</v>
@@ -6269,10 +6269,10 @@
         <v>35</v>
       </c>
       <c r="J68" t="n">
-        <v>32.4</v>
+        <v>35</v>
       </c>
       <c r="K68" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -6302,7 +6302,7 @@
         <v>41</v>
       </c>
       <c r="S68" t="n">
-        <v>-2.600000000000001</v>
+        <v>0</v>
       </c>
       <c r="T68" t="n">
         <v>34.83333333333334</v>
@@ -6311,7 +6311,7 @@
         <v>3</v>
       </c>
       <c r="V68" t="n">
-        <v>38.42962962962963</v>
+        <v>38.42962962962962</v>
       </c>
       <c r="W68" t="n">
         <v>31.5</v>
@@ -6356,10 +6356,10 @@
         <v>21</v>
       </c>
       <c r="J69" t="n">
-        <v>19.5</v>
+        <v>23.1</v>
       </c>
       <c r="K69" t="n">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -6389,7 +6389,7 @@
         <v>21</v>
       </c>
       <c r="S69" t="n">
-        <v>-1.5</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="T69" t="n">
         <v>20.9</v>
@@ -6443,10 +6443,10 @@
         <v>21</v>
       </c>
       <c r="J70" t="n">
-        <v>24.6</v>
+        <v>23.9</v>
       </c>
       <c r="K70" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -6476,7 +6476,7 @@
         <v>21</v>
       </c>
       <c r="S70" t="n">
-        <v>3.600000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="T70" t="n">
         <v>22.76666666666667</v>
@@ -6530,10 +6530,10 @@
         <v>35</v>
       </c>
       <c r="J71" t="n">
-        <v>33.5</v>
+        <v>40.8</v>
       </c>
       <c r="K71" t="n">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -6563,10 +6563,10 @@
         <v>41</v>
       </c>
       <c r="S71" t="n">
-        <v>-1.5</v>
+        <v>5.799999999999997</v>
       </c>
       <c r="T71" t="n">
-        <v>37.56666666666667</v>
+        <v>37.56666666666666</v>
       </c>
       <c r="U71" t="n">
         <v>3</v>
@@ -6704,10 +6704,10 @@
         <v>31</v>
       </c>
       <c r="J73" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="K73" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -6735,7 +6735,7 @@
       </c>
       <c r="R73" t="inlineStr"/>
       <c r="S73" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T73" t="n">
         <v>32.03333333333333</v>
@@ -6789,10 +6789,10 @@
         <v>28</v>
       </c>
       <c r="J74" t="n">
-        <v>24.1</v>
+        <v>27.3</v>
       </c>
       <c r="K74" t="n">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
@@ -6822,7 +6822,7 @@
         <v>28</v>
       </c>
       <c r="S74" t="n">
-        <v>-3.899999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="T74" t="n">
         <v>25.33333333333333</v>
@@ -6876,7 +6876,7 @@
         <v>28</v>
       </c>
       <c r="J75" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="K75" t="n">
         <v>88</v>
@@ -6909,10 +6909,10 @@
         <v>28</v>
       </c>
       <c r="S75" t="n">
-        <v>-3.199999999999999</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="T75" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="U75" t="n">
         <v>3</v>
@@ -7050,10 +7050,10 @@
         <v>31</v>
       </c>
       <c r="J77" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="K77" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="T77" t="n">
         <v>36</v>
@@ -7483,10 +7483,10 @@
         <v>21</v>
       </c>
       <c r="J82" t="n">
-        <v>23.8</v>
+        <v>24.7</v>
       </c>
       <c r="K82" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -7516,7 +7516,7 @@
         <v>21</v>
       </c>
       <c r="S82" t="n">
-        <v>2.800000000000001</v>
+        <v>3.699999999999999</v>
       </c>
       <c r="T82" t="n">
         <v>22.53333333333333</v>
@@ -7657,10 +7657,10 @@
         <v>31</v>
       </c>
       <c r="J84" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="K84" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="T84" t="n">
         <v>33.63333333333333</v>
@@ -8090,10 +8090,10 @@
         <v>31</v>
       </c>
       <c r="J89" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="K89" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="R89" t="inlineStr"/>
       <c r="S89" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T89" t="n">
         <v>32.76666666666667</v>
@@ -9472,10 +9472,10 @@
         <v>35</v>
       </c>
       <c r="J105" t="n">
-        <v>39.8</v>
+        <v>34.1</v>
       </c>
       <c r="K105" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
@@ -9505,7 +9505,7 @@
         <v>41</v>
       </c>
       <c r="S105" t="n">
-        <v>4.799999999999997</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T105" t="n">
         <v>36.83333333333334</v>
@@ -10864,10 +10864,10 @@
         <v>21</v>
       </c>
       <c r="J121" t="n">
-        <v>22.6</v>
+        <v>18.4</v>
       </c>
       <c r="K121" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -10897,10 +10897,10 @@
         <v>21</v>
       </c>
       <c r="S121" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T121" t="n">
-        <v>22.93333333333334</v>
+        <v>22.93333333333333</v>
       </c>
       <c r="U121" t="n">
         <v>3</v>
@@ -11734,10 +11734,10 @@
         <v>35</v>
       </c>
       <c r="J131" t="n">
-        <v>36.1</v>
+        <v>36.4</v>
       </c>
       <c r="K131" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -11767,7 +11767,7 @@
         <v>41</v>
       </c>
       <c r="S131" t="n">
-        <v>1.100000000000001</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="T131" t="n">
         <v>33.9</v>
@@ -29814,7 +29814,7 @@
         <v>3</v>
       </c>
       <c r="V339" t="n">
-        <v>23.35555555555555</v>
+        <v>23.35555555555556</v>
       </c>
       <c r="W339" t="n">
         <v>21</v>
@@ -29859,10 +29859,10 @@
         <v>24.5</v>
       </c>
       <c r="J340" t="n">
-        <v>23.3</v>
+        <v>25.4</v>
       </c>
       <c r="K340" t="n">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="L340" t="inlineStr">
         <is>
@@ -29892,10 +29892,10 @@
         <v>28</v>
       </c>
       <c r="S340" t="n">
-        <v>-1.199999999999999</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T340" t="n">
-        <v>24.56666666666666</v>
+        <v>24.56666666666667</v>
       </c>
       <c r="U340" t="n">
         <v>3</v>
@@ -30033,10 +30033,10 @@
         <v>24.5</v>
       </c>
       <c r="J342" t="n">
-        <v>22.3</v>
+        <v>23.3</v>
       </c>
       <c r="K342" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -30066,7 +30066,7 @@
         <v>28</v>
       </c>
       <c r="S342" t="n">
-        <v>-2.199999999999999</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T342" t="n">
         <v>23.03333333333333</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-27 18:24:44
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5441,7 +5441,7 @@
         <v>3</v>
       </c>
       <c r="V58" t="n">
-        <v>24.52222222222223</v>
+        <v>24.52222222222222</v>
       </c>
       <c r="W58" t="n">
         <v>20.5</v>
@@ -5486,10 +5486,10 @@
         <v>24</v>
       </c>
       <c r="J59" t="n">
-        <v>26.4</v>
+        <v>16.6</v>
       </c>
       <c r="K59" t="n">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -5519,7 +5519,7 @@
         <v>28</v>
       </c>
       <c r="S59" t="n">
-        <v>2.399999999999999</v>
+        <v>-7.399999999999999</v>
       </c>
       <c r="T59" t="n">
         <v>23.4</v>
@@ -5528,7 +5528,7 @@
         <v>3</v>
       </c>
       <c r="V59" t="n">
-        <v>24.64444444444445</v>
+        <v>24.64444444444444</v>
       </c>
       <c r="W59" t="n">
         <v>20.5</v>
@@ -5921,10 +5921,10 @@
         <v>21</v>
       </c>
       <c r="J64" t="n">
-        <v>20.3</v>
+        <v>19.7</v>
       </c>
       <c r="K64" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -5954,7 +5954,7 @@
         <v>21</v>
       </c>
       <c r="S64" t="n">
-        <v>-0.6999999999999993</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="T64" t="n">
         <v>20.03333333333333</v>
@@ -6008,10 +6008,10 @@
         <v>35</v>
       </c>
       <c r="J65" t="n">
-        <v>32.3</v>
+        <v>34.3</v>
       </c>
       <c r="K65" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -6041,7 +6041,7 @@
         <v>41</v>
       </c>
       <c r="S65" t="n">
-        <v>-2.700000000000003</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="T65" t="n">
         <v>32.96666666666666</v>
@@ -6095,10 +6095,10 @@
         <v>35</v>
       </c>
       <c r="J66" t="n">
-        <v>31.8</v>
+        <v>38.1</v>
       </c>
       <c r="K66" t="n">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -6128,7 +6128,7 @@
         <v>41</v>
       </c>
       <c r="S66" t="n">
-        <v>-3.199999999999999</v>
+        <v>3.100000000000001</v>
       </c>
       <c r="T66" t="n">
         <v>35.3</v>
@@ -6137,7 +6137,7 @@
         <v>3</v>
       </c>
       <c r="V66" t="n">
-        <v>37.02962962962962</v>
+        <v>37.02962962962963</v>
       </c>
       <c r="W66" t="n">
         <v>31.5</v>
@@ -6182,10 +6182,10 @@
         <v>21</v>
       </c>
       <c r="J67" t="n">
-        <v>17.6</v>
+        <v>17.9</v>
       </c>
       <c r="K67" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -6215,7 +6215,7 @@
         <v>21</v>
       </c>
       <c r="S67" t="n">
-        <v>-3.399999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T67" t="n">
         <v>18.86666666666667</v>
@@ -6269,10 +6269,10 @@
         <v>35</v>
       </c>
       <c r="J68" t="n">
-        <v>35</v>
+        <v>32.4</v>
       </c>
       <c r="K68" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -6302,7 +6302,7 @@
         <v>41</v>
       </c>
       <c r="S68" t="n">
-        <v>0</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="T68" t="n">
         <v>34.83333333333334</v>
@@ -6311,7 +6311,7 @@
         <v>3</v>
       </c>
       <c r="V68" t="n">
-        <v>38.42962962962962</v>
+        <v>38.42962962962963</v>
       </c>
       <c r="W68" t="n">
         <v>31.5</v>
@@ -6356,10 +6356,10 @@
         <v>21</v>
       </c>
       <c r="J69" t="n">
-        <v>23.1</v>
+        <v>19.5</v>
       </c>
       <c r="K69" t="n">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -6389,7 +6389,7 @@
         <v>21</v>
       </c>
       <c r="S69" t="n">
-        <v>2.100000000000001</v>
+        <v>-1.5</v>
       </c>
       <c r="T69" t="n">
         <v>20.9</v>
@@ -6443,10 +6443,10 @@
         <v>21</v>
       </c>
       <c r="J70" t="n">
-        <v>23.9</v>
+        <v>24.6</v>
       </c>
       <c r="K70" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -6476,7 +6476,7 @@
         <v>21</v>
       </c>
       <c r="S70" t="n">
-        <v>2.899999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="T70" t="n">
         <v>22.76666666666667</v>
@@ -6530,10 +6530,10 @@
         <v>35</v>
       </c>
       <c r="J71" t="n">
-        <v>40.8</v>
+        <v>33.5</v>
       </c>
       <c r="K71" t="n">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -6563,10 +6563,10 @@
         <v>41</v>
       </c>
       <c r="S71" t="n">
-        <v>5.799999999999997</v>
+        <v>-1.5</v>
       </c>
       <c r="T71" t="n">
-        <v>37.56666666666666</v>
+        <v>37.56666666666667</v>
       </c>
       <c r="U71" t="n">
         <v>3</v>
@@ -6789,10 +6789,10 @@
         <v>28</v>
       </c>
       <c r="J74" t="n">
-        <v>27.3</v>
+        <v>24.1</v>
       </c>
       <c r="K74" t="n">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
@@ -6822,7 +6822,7 @@
         <v>28</v>
       </c>
       <c r="S74" t="n">
-        <v>-0.6999999999999993</v>
+        <v>-3.899999999999999</v>
       </c>
       <c r="T74" t="n">
         <v>25.33333333333333</v>
@@ -6876,7 +6876,7 @@
         <v>28</v>
       </c>
       <c r="J75" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="K75" t="n">
         <v>88</v>
@@ -6909,10 +6909,10 @@
         <v>28</v>
       </c>
       <c r="S75" t="n">
-        <v>-3.300000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="T75" t="n">
-        <v>25.13333333333333</v>
+        <v>25.13333333333334</v>
       </c>
       <c r="U75" t="n">
         <v>3</v>
@@ -7483,10 +7483,10 @@
         <v>21</v>
       </c>
       <c r="J82" t="n">
-        <v>24.7</v>
+        <v>23.8</v>
       </c>
       <c r="K82" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -7516,7 +7516,7 @@
         <v>21</v>
       </c>
       <c r="S82" t="n">
-        <v>3.699999999999999</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T82" t="n">
         <v>22.53333333333333</v>
@@ -9472,10 +9472,10 @@
         <v>35</v>
       </c>
       <c r="J105" t="n">
-        <v>34.1</v>
+        <v>39.8</v>
       </c>
       <c r="K105" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
@@ -9505,7 +9505,7 @@
         <v>41</v>
       </c>
       <c r="S105" t="n">
-        <v>-0.8999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T105" t="n">
         <v>36.83333333333334</v>
@@ -10864,10 +10864,10 @@
         <v>21</v>
       </c>
       <c r="J121" t="n">
-        <v>18.4</v>
+        <v>22.6</v>
       </c>
       <c r="K121" t="n">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
@@ -10897,10 +10897,10 @@
         <v>21</v>
       </c>
       <c r="S121" t="n">
-        <v>-2.600000000000001</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T121" t="n">
-        <v>22.93333333333333</v>
+        <v>22.93333333333334</v>
       </c>
       <c r="U121" t="n">
         <v>3</v>
@@ -10951,10 +10951,10 @@
         <v>21</v>
       </c>
       <c r="J122" t="n">
-        <v>21.6</v>
+        <v>19.4</v>
       </c>
       <c r="K122" t="n">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="L122" t="inlineStr">
         <is>
@@ -10984,7 +10984,7 @@
         <v>21</v>
       </c>
       <c r="S122" t="n">
-        <v>0.6000000000000014</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T122" t="n">
         <v>19.93333333333333</v>
@@ -11734,10 +11734,10 @@
         <v>35</v>
       </c>
       <c r="J131" t="n">
-        <v>36.4</v>
+        <v>36.1</v>
       </c>
       <c r="K131" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L131" t="inlineStr">
         <is>
@@ -11767,7 +11767,7 @@
         <v>41</v>
       </c>
       <c r="S131" t="n">
-        <v>1.399999999999999</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="T131" t="n">
         <v>33.9</v>
@@ -29814,7 +29814,7 @@
         <v>3</v>
       </c>
       <c r="V339" t="n">
-        <v>23.35555555555556</v>
+        <v>23.35555555555555</v>
       </c>
       <c r="W339" t="n">
         <v>21</v>
@@ -29859,10 +29859,10 @@
         <v>24.5</v>
       </c>
       <c r="J340" t="n">
-        <v>25.4</v>
+        <v>23.3</v>
       </c>
       <c r="K340" t="n">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="L340" t="inlineStr">
         <is>
@@ -29892,10 +29892,10 @@
         <v>28</v>
       </c>
       <c r="S340" t="n">
-        <v>0.8999999999999986</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T340" t="n">
-        <v>24.56666666666667</v>
+        <v>24.56666666666666</v>
       </c>
       <c r="U340" t="n">
         <v>3</v>
@@ -30033,10 +30033,10 @@
         <v>24.5</v>
       </c>
       <c r="J342" t="n">
-        <v>23.3</v>
+        <v>22.3</v>
       </c>
       <c r="K342" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="L342" t="inlineStr">
         <is>
@@ -30066,7 +30066,7 @@
         <v>28</v>
       </c>
       <c r="S342" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="T342" t="n">
         <v>23.03333333333333</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-27 22:54:19
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3161,10 +3161,10 @@
         <v>31</v>
       </c>
       <c r="J32" t="n">
-        <v>30</v>
+        <v>31.4</v>
       </c>
       <c r="K32" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="n">
-        <v>-1</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T32" t="n">
         <v>30.33333333333333</v>
@@ -6704,10 +6704,10 @@
         <v>31</v>
       </c>
       <c r="J73" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="K73" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -6735,7 +6735,7 @@
       </c>
       <c r="R73" t="inlineStr"/>
       <c r="S73" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T73" t="n">
         <v>32.03333333333333</v>
@@ -7050,10 +7050,10 @@
         <v>31</v>
       </c>
       <c r="J77" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="K77" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="T77" t="n">
         <v>36</v>
@@ -7657,10 +7657,10 @@
         <v>31</v>
       </c>
       <c r="J84" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="K84" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="T84" t="n">
         <v>33.63333333333333</v>
@@ -8090,10 +8090,10 @@
         <v>31</v>
       </c>
       <c r="J89" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="K89" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8121,7 +8121,7 @@
       </c>
       <c r="R89" t="inlineStr"/>
       <c r="S89" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="T89" t="n">
         <v>32.76666666666667</v>
@@ -10690,10 +10690,10 @@
         <v>28</v>
       </c>
       <c r="J119" t="n">
-        <v>27.4</v>
+        <v>33.5</v>
       </c>
       <c r="K119" t="n">
-        <v>98</v>
+        <v>120</v>
       </c>
       <c r="L119" t="inlineStr">
         <is>
@@ -10723,7 +10723,7 @@
         <v>28</v>
       </c>
       <c r="S119" t="n">
-        <v>-0.6000000000000014</v>
+        <v>5.5</v>
       </c>
       <c r="T119" t="n">
         <v>30.83333333333333</v>
@@ -11038,10 +11038,10 @@
         <v>35</v>
       </c>
       <c r="J123" t="n">
-        <v>35.4</v>
+        <v>30.5</v>
       </c>
       <c r="K123" t="n">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="L123" t="inlineStr">
         <is>
@@ -11071,7 +11071,7 @@
         <v>41</v>
       </c>
       <c r="S123" t="n">
-        <v>0.3999999999999986</v>
+        <v>-4.5</v>
       </c>
       <c r="T123" t="n">
         <v>34.13333333333333</v>
@@ -11908,10 +11908,10 @@
         <v>31</v>
       </c>
       <c r="J133" t="n">
-        <v>30.5</v>
+        <v>31.9</v>
       </c>
       <c r="K133" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
@@ -11939,7 +11939,7 @@
       </c>
       <c r="R133" t="inlineStr"/>
       <c r="S133" t="n">
-        <v>-0.5</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="T133" t="n">
         <v>31.23333333333333</v>
@@ -13727,10 +13727,10 @@
         <v>21</v>
       </c>
       <c r="J154" t="n">
-        <v>19.1</v>
+        <v>22.2</v>
       </c>
       <c r="K154" t="n">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -13760,7 +13760,7 @@
         <v>21</v>
       </c>
       <c r="S154" t="n">
-        <v>-1.899999999999999</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="T154" t="n">
         <v>21.83333333333333</v>
@@ -21361,10 +21361,10 @@
         <v>21</v>
       </c>
       <c r="J242" t="n">
-        <v>19</v>
+        <v>17.3</v>
       </c>
       <c r="K242" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="L242" t="inlineStr">
         <is>
@@ -21392,7 +21392,7 @@
       </c>
       <c r="R242" t="inlineStr"/>
       <c r="S242" t="n">
-        <v>-2</v>
+        <v>-3.699999999999999</v>
       </c>
       <c r="T242" t="n">
         <v>19.3</v>
@@ -28032,10 +28032,10 @@
         <v>24.5</v>
       </c>
       <c r="J319" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="K319" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L319" t="inlineStr">
         <is>
@@ -28065,7 +28065,7 @@
         <v>28</v>
       </c>
       <c r="S319" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T319" t="n">
         <v>24.66666666666667</v>
@@ -28728,10 +28728,10 @@
         <v>24.5</v>
       </c>
       <c r="J327" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="K327" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -28761,7 +28761,7 @@
         <v>28</v>
       </c>
       <c r="S327" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T327" t="n">
         <v>27.1</v>
@@ -30642,10 +30642,10 @@
         <v>24.5</v>
       </c>
       <c r="J349" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="K349" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="L349" t="inlineStr">
         <is>
@@ -30675,10 +30675,10 @@
         <v>28</v>
       </c>
       <c r="S349" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="T349" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="U349" t="n">
         <v>3</v>
@@ -31593,10 +31593,10 @@
         <v>21</v>
       </c>
       <c r="J360" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="K360" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L360" t="inlineStr">
         <is>
@@ -31626,7 +31626,7 @@
         <v>21</v>
       </c>
       <c r="S360" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="T360" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-28 08:16:38
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3161,10 +3161,10 @@
         <v>31</v>
       </c>
       <c r="J32" t="n">
-        <v>30</v>
+        <v>31.4</v>
       </c>
       <c r="K32" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="n">
-        <v>-1</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T32" t="n">
         <v>30.33333333333333</v>
@@ -5053,10 +5053,10 @@
         <v>24</v>
       </c>
       <c r="J54" t="n">
-        <v>20.8</v>
+        <v>22.4</v>
       </c>
       <c r="K54" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -5086,7 +5086,7 @@
         <v>28</v>
       </c>
       <c r="S54" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T54" t="n">
         <v>21.53333333333333</v>
@@ -5140,10 +5140,10 @@
         <v>24</v>
       </c>
       <c r="J55" t="n">
-        <v>25.5</v>
+        <v>26.6</v>
       </c>
       <c r="K55" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
         <v>28</v>
       </c>
       <c r="S55" t="n">
-        <v>1.5</v>
+        <v>2.600000000000001</v>
       </c>
       <c r="T55" t="n">
         <v>22.46666666666667</v>
@@ -5486,10 +5486,10 @@
         <v>24</v>
       </c>
       <c r="J59" t="n">
-        <v>16.6</v>
+        <v>27.2</v>
       </c>
       <c r="K59" t="n">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -5519,7 +5519,7 @@
         <v>28</v>
       </c>
       <c r="S59" t="n">
-        <v>-7.399999999999999</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="T59" t="n">
         <v>23.4</v>
@@ -6876,10 +6876,10 @@
         <v>28</v>
       </c>
       <c r="J75" t="n">
-        <v>24.8</v>
+        <v>25.9</v>
       </c>
       <c r="K75" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -6909,10 +6909,10 @@
         <v>28</v>
       </c>
       <c r="S75" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="T75" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="U75" t="n">
         <v>3</v>
@@ -12167,10 +12167,10 @@
         <v>28</v>
       </c>
       <c r="J136" t="n">
-        <v>27.9</v>
+        <v>27.4</v>
       </c>
       <c r="K136" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="L136" t="inlineStr">
         <is>
@@ -12200,7 +12200,7 @@
         <v>28</v>
       </c>
       <c r="S136" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="T136" t="n">
         <v>28.4</v>
@@ -12341,10 +12341,10 @@
         <v>35</v>
       </c>
       <c r="J138" t="n">
-        <v>34.7</v>
+        <v>39.7</v>
       </c>
       <c r="K138" t="n">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="L138" t="inlineStr">
         <is>
@@ -12374,7 +12374,7 @@
         <v>41</v>
       </c>
       <c r="S138" t="n">
-        <v>-0.2999999999999972</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="T138" t="n">
         <v>37.66666666666667</v>
@@ -21531,10 +21531,10 @@
         <v>21</v>
       </c>
       <c r="J244" t="n">
-        <v>20</v>
+        <v>22.4</v>
       </c>
       <c r="K244" t="n">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="L244" t="inlineStr">
         <is>
@@ -21564,7 +21564,7 @@
         <v>21</v>
       </c>
       <c r="S244" t="n">
-        <v>-1</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="T244" t="n">
         <v>20.96666666666667</v>
@@ -21618,10 +21618,10 @@
         <v>21</v>
       </c>
       <c r="J245" t="n">
-        <v>21.2</v>
+        <v>21.5</v>
       </c>
       <c r="K245" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L245" t="inlineStr">
         <is>
@@ -21651,7 +21651,7 @@
         <v>21</v>
       </c>
       <c r="S245" t="n">
-        <v>0.1999999999999993</v>
+        <v>0.5</v>
       </c>
       <c r="T245" t="n">
         <v>21.2</v>
@@ -21705,10 +21705,10 @@
         <v>21</v>
       </c>
       <c r="J246" t="n">
-        <v>21.9</v>
+        <v>22.5</v>
       </c>
       <c r="K246" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="L246" t="inlineStr">
         <is>
@@ -21736,7 +21736,7 @@
       </c>
       <c r="R246" t="inlineStr"/>
       <c r="S246" t="n">
-        <v>0.8999999999999986</v>
+        <v>1.5</v>
       </c>
       <c r="T246" t="n">
         <v>21.73333333333333</v>
@@ -27249,10 +27249,10 @@
         <v>24.5</v>
       </c>
       <c r="J310" t="n">
-        <v>25.8</v>
+        <v>23.3</v>
       </c>
       <c r="K310" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="L310" t="inlineStr">
         <is>
@@ -27282,7 +27282,7 @@
         <v>28</v>
       </c>
       <c r="S310" t="n">
-        <v>1.300000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T310" t="n">
         <v>24.26666666666667</v>
@@ -27945,10 +27945,10 @@
         <v>24.5</v>
       </c>
       <c r="J318" t="n">
-        <v>33.3</v>
+        <v>21.5</v>
       </c>
       <c r="K318" t="n">
-        <v>136</v>
+        <v>88</v>
       </c>
       <c r="L318" t="inlineStr">
         <is>
@@ -27978,7 +27978,7 @@
         <v>28</v>
       </c>
       <c r="S318" t="n">
-        <v>8.799999999999997</v>
+        <v>-3</v>
       </c>
       <c r="T318" t="n">
         <v>29.5</v>
@@ -28032,10 +28032,10 @@
         <v>24.5</v>
       </c>
       <c r="J319" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K319" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L319" t="inlineStr">
         <is>
@@ -28065,7 +28065,7 @@
         <v>28</v>
       </c>
       <c r="S319" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T319" t="n">
         <v>24.66666666666667</v>
@@ -28728,10 +28728,10 @@
         <v>24.5</v>
       </c>
       <c r="J327" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K327" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L327" t="inlineStr">
         <is>
@@ -28761,7 +28761,7 @@
         <v>28</v>
       </c>
       <c r="S327" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T327" t="n">
         <v>27.1</v>
@@ -30642,10 +30642,10 @@
         <v>24.5</v>
       </c>
       <c r="J349" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K349" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L349" t="inlineStr">
         <is>
@@ -30675,10 +30675,10 @@
         <v>28</v>
       </c>
       <c r="S349" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T349" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U349" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-29 20:33:21
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3501,10 +3501,10 @@
         <v>31</v>
       </c>
       <c r="J36" t="n">
-        <v>27.8</v>
+        <v>36.5</v>
       </c>
       <c r="K36" t="n">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="n">
-        <v>-3.199999999999999</v>
+        <v>5.5</v>
       </c>
       <c r="T36" t="n">
         <v>33.03333333333333</v>
@@ -4794,10 +4794,10 @@
         <v>31</v>
       </c>
       <c r="J51" t="n">
-        <v>30.5</v>
+        <v>38.5</v>
       </c>
       <c r="K51" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="n">
-        <v>-0.5</v>
+        <v>7.5</v>
       </c>
       <c r="T51" t="n">
         <v>35.86666666666667</v>
@@ -6354,10 +6354,10 @@
         <v>35</v>
       </c>
       <c r="J69" t="n">
-        <v>32.4</v>
+        <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -6387,7 +6387,7 @@
         <v>41</v>
       </c>
       <c r="S69" t="n">
-        <v>-2.600000000000001</v>
+        <v>0</v>
       </c>
       <c r="T69" t="n">
         <v>34.83333333333334</v>
@@ -7697,7 +7697,7 @@
         <v>3</v>
       </c>
       <c r="V84" t="n">
-        <v>24.43333333333334</v>
+        <v>24.43333333333333</v>
       </c>
       <c r="W84" t="n">
         <v>17.5</v>
@@ -8909,7 +8909,7 @@
         <v>3</v>
       </c>
       <c r="V98" t="n">
-        <v>26.17777777777778</v>
+        <v>26.17777777777777</v>
       </c>
       <c r="W98" t="n">
         <v>17.5</v>
@@ -10514,10 +10514,10 @@
         <v>35</v>
       </c>
       <c r="J117" t="n">
-        <v>37.4</v>
+        <v>34.6</v>
       </c>
       <c r="K117" t="n">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="L117" t="inlineStr">
         <is>
@@ -10547,7 +10547,7 @@
         <v>41</v>
       </c>
       <c r="S117" t="n">
-        <v>2.399999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="T117" t="n">
         <v>35.63333333333333</v>
@@ -10775,10 +10775,10 @@
         <v>28</v>
       </c>
       <c r="J120" t="n">
-        <v>31.6</v>
+        <v>33.5</v>
       </c>
       <c r="K120" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="L120" t="inlineStr">
         <is>
@@ -10808,7 +10808,7 @@
         <v>28</v>
       </c>
       <c r="S120" t="n">
-        <v>3.600000000000001</v>
+        <v>5.5</v>
       </c>
       <c r="T120" t="n">
         <v>30.83333333333333</v>
@@ -14160,10 +14160,10 @@
         <v>28</v>
       </c>
       <c r="J159" t="n">
-        <v>31.6</v>
+        <v>29.4</v>
       </c>
       <c r="K159" t="n">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="L159" t="inlineStr">
         <is>
@@ -14193,16 +14193,16 @@
         <v>28</v>
       </c>
       <c r="S159" t="n">
-        <v>3.600000000000001</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="T159" t="n">
-        <v>28.43333333333334</v>
+        <v>28.43333333333333</v>
       </c>
       <c r="U159" t="n">
         <v>3</v>
       </c>
       <c r="V159" t="n">
-        <v>30.78888888888889</v>
+        <v>30.78888888888888</v>
       </c>
       <c r="W159" t="n">
         <v>24.5</v>
@@ -15720,10 +15720,10 @@
         <v>28</v>
       </c>
       <c r="J177" t="n">
-        <v>23.6</v>
+        <v>29</v>
       </c>
       <c r="K177" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="L177" t="inlineStr">
         <is>
@@ -15753,7 +15753,7 @@
         <v>28</v>
       </c>
       <c r="S177" t="n">
-        <v>-4.399999999999999</v>
+        <v>1</v>
       </c>
       <c r="T177" t="n">
         <v>25.33333333333333</v>
@@ -16503,10 +16503,10 @@
         <v>28</v>
       </c>
       <c r="J186" t="n">
-        <v>27.9</v>
+        <v>25.7</v>
       </c>
       <c r="K186" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="L186" t="inlineStr">
         <is>
@@ -16536,7 +16536,7 @@
         <v>28</v>
       </c>
       <c r="S186" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-2.300000000000001</v>
       </c>
       <c r="T186" t="n">
         <v>26.76666666666667</v>
@@ -17021,10 +17021,10 @@
         <v>21</v>
       </c>
       <c r="J192" t="n">
-        <v>20.6</v>
+        <v>22.6</v>
       </c>
       <c r="K192" t="n">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="L192" t="inlineStr">
         <is>
@@ -17054,7 +17054,7 @@
         <v>21</v>
       </c>
       <c r="S192" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T192" t="n">
         <v>21.5</v>
@@ -18324,10 +18324,10 @@
         <v>28</v>
       </c>
       <c r="J207" t="n">
-        <v>26.9</v>
+        <v>27.8</v>
       </c>
       <c r="K207" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="L207" t="inlineStr">
         <is>
@@ -18357,7 +18357,7 @@
         <v>28</v>
       </c>
       <c r="S207" t="n">
-        <v>-1.100000000000001</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T207" t="n">
         <v>28.46666666666667</v>
@@ -20839,10 +20839,10 @@
         <v>24</v>
       </c>
       <c r="J236" t="n">
-        <v>26.8</v>
+        <v>25.3</v>
       </c>
       <c r="K236" t="n">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="L236" t="inlineStr">
         <is>
@@ -20872,7 +20872,7 @@
         <v>28</v>
       </c>
       <c r="S236" t="n">
-        <v>2.800000000000001</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="T236" t="n">
         <v>24.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-30 08:00:26
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -21703,10 +21703,10 @@
         <v>21</v>
       </c>
       <c r="J246" t="n">
-        <v>21.2</v>
+        <v>21.5</v>
       </c>
       <c r="K246" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L246" t="inlineStr">
         <is>
@@ -21736,7 +21736,7 @@
         <v>21</v>
       </c>
       <c r="S246" t="n">
-        <v>0.1999999999999993</v>
+        <v>0.5</v>
       </c>
       <c r="T246" t="n">
         <v>21.2</v>
@@ -24125,10 +24125,10 @@
         <v>28</v>
       </c>
       <c r="J274" t="n">
-        <v>26.3</v>
+        <v>27.8</v>
       </c>
       <c r="K274" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="L274" t="inlineStr">
         <is>
@@ -24158,7 +24158,7 @@
         <v>28</v>
       </c>
       <c r="S274" t="n">
-        <v>-1.699999999999999</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="T274" t="n">
         <v>27.36666666666666</v>
@@ -24386,10 +24386,10 @@
         <v>28</v>
       </c>
       <c r="J277" t="n">
-        <v>27.4</v>
+        <v>28.2</v>
       </c>
       <c r="K277" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="L277" t="inlineStr">
         <is>
@@ -24419,7 +24419,7 @@
         <v>28</v>
       </c>
       <c r="S277" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T277" t="n">
         <v>28.2</v>
@@ -28117,10 +28117,10 @@
         <v>24.5</v>
       </c>
       <c r="J320" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K320" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L320" t="inlineStr">
         <is>
@@ -28150,7 +28150,7 @@
         <v>28</v>
       </c>
       <c r="S320" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T320" t="n">
         <v>24.66666666666667</v>
@@ -28813,10 +28813,10 @@
         <v>24.5</v>
       </c>
       <c r="J328" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K328" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L328" t="inlineStr">
         <is>
@@ -28846,7 +28846,7 @@
         <v>28</v>
       </c>
       <c r="S328" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T328" t="n">
         <v>27.1</v>
@@ -28900,10 +28900,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>19.3</v>
+        <v>21.4</v>
       </c>
       <c r="K329" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28933,7 +28933,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-5.199999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>21.1</v>
@@ -28942,7 +28942,7 @@
         <v>3</v>
       </c>
       <c r="V329" t="n">
-        <v>25.57777777777778</v>
+        <v>25.57777777777777</v>
       </c>
       <c r="W329" t="n">
         <v>21</v>
@@ -29335,10 +29335,10 @@
         <v>24.5</v>
       </c>
       <c r="J334" t="n">
-        <v>25.6</v>
+        <v>24</v>
       </c>
       <c r="K334" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="L334" t="inlineStr">
         <is>
@@ -29368,7 +29368,7 @@
         <v>28</v>
       </c>
       <c r="S334" t="n">
-        <v>1.100000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="T334" t="n">
         <v>35.8</v>
@@ -30727,10 +30727,10 @@
         <v>24.5</v>
       </c>
       <c r="J350" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K350" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L350" t="inlineStr">
         <is>
@@ -30760,10 +30760,10 @@
         <v>28</v>
       </c>
       <c r="S350" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T350" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U350" t="n">
         <v>3</v>
@@ -31765,10 +31765,10 @@
         <v>21</v>
       </c>
       <c r="J362" t="n">
-        <v>22</v>
+        <v>18.9</v>
       </c>
       <c r="K362" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="L362" t="inlineStr">
         <is>
@@ -31796,7 +31796,7 @@
       </c>
       <c r="R362" t="inlineStr"/>
       <c r="S362" t="n">
-        <v>1</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="T362" t="n">
         <v>19.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-30 20:38:12
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4879,10 +4879,10 @@
         <v>31</v>
       </c>
       <c r="J52" t="n">
-        <v>38.5</v>
+        <v>30.5</v>
       </c>
       <c r="K52" t="n">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="n">
-        <v>7.5</v>
+        <v>-0.5</v>
       </c>
       <c r="T52" t="n">
         <v>35.86666666666667</v>
@@ -5265,7 +5265,7 @@
         <v>3</v>
       </c>
       <c r="V56" t="n">
-        <v>23.14444444444445</v>
+        <v>23.14444444444444</v>
       </c>
       <c r="W56" t="n">
         <v>20.5</v>
@@ -5569,10 +5569,10 @@
         <v>24</v>
       </c>
       <c r="J60" t="n">
-        <v>23.1</v>
+        <v>25.9</v>
       </c>
       <c r="K60" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -5602,7 +5602,7 @@
         <v>28</v>
       </c>
       <c r="S60" t="n">
-        <v>-0.8999999999999986</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="T60" t="n">
         <v>24.1</v>
@@ -6526,10 +6526,10 @@
         <v>21</v>
       </c>
       <c r="J71" t="n">
-        <v>23.1</v>
+        <v>19.5</v>
       </c>
       <c r="K71" t="n">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -6559,7 +6559,7 @@
         <v>21</v>
       </c>
       <c r="S71" t="n">
-        <v>2.100000000000001</v>
+        <v>-1.5</v>
       </c>
       <c r="T71" t="n">
         <v>20.9</v>
@@ -7740,10 +7740,10 @@
         <v>21</v>
       </c>
       <c r="J85" t="n">
-        <v>19.3</v>
+        <v>26</v>
       </c>
       <c r="K85" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
         <v>21</v>
       </c>
       <c r="S85" t="n">
-        <v>-1.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="T85" t="n">
         <v>22</v>
@@ -7782,7 +7782,7 @@
         <v>3</v>
       </c>
       <c r="V85" t="n">
-        <v>24.43333333333333</v>
+        <v>24.43333333333334</v>
       </c>
       <c r="W85" t="n">
         <v>17.5</v>
@@ -7912,10 +7912,10 @@
         <v>21</v>
       </c>
       <c r="J87" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K87" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="L87" t="inlineStr">
         <is>
@@ -7945,7 +7945,7 @@
         <v>21</v>
       </c>
       <c r="S87" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="T87" t="n">
         <v>19.9</v>
@@ -7999,10 +7999,10 @@
         <v>35</v>
       </c>
       <c r="J88" t="n">
-        <v>36.5</v>
+        <v>25.3</v>
       </c>
       <c r="K88" t="n">
-        <v>104</v>
+        <v>72</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
         <v>41</v>
       </c>
       <c r="S88" t="n">
-        <v>1.5</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="T88" t="n">
         <v>33.1</v>
@@ -8086,10 +8086,10 @@
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>36.7</v>
+        <v>39.1</v>
       </c>
       <c r="K89" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8119,7 +8119,7 @@
         <v>41</v>
       </c>
       <c r="S89" t="n">
-        <v>1.700000000000003</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="T89" t="n">
         <v>35.73333333333333</v>
@@ -8128,7 +8128,7 @@
         <v>3</v>
       </c>
       <c r="V89" t="n">
-        <v>35.86296296296296</v>
+        <v>35.86296296296297</v>
       </c>
       <c r="W89" t="n">
         <v>31.5</v>
@@ -8173,10 +8173,10 @@
         <v>35</v>
       </c>
       <c r="J90" t="n">
-        <v>39.8</v>
+        <v>40.3</v>
       </c>
       <c r="K90" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -8206,7 +8206,7 @@
         <v>41</v>
       </c>
       <c r="S90" t="n">
-        <v>4.799999999999997</v>
+        <v>5.299999999999997</v>
       </c>
       <c r="T90" t="n">
         <v>36.16666666666666</v>
@@ -8215,7 +8215,7 @@
         <v>3</v>
       </c>
       <c r="V90" t="n">
-        <v>38.87407407407408</v>
+        <v>38.87407407407407</v>
       </c>
       <c r="W90" t="n">
         <v>31.5</v>
@@ -8345,10 +8345,10 @@
         <v>35</v>
       </c>
       <c r="J92" t="n">
-        <v>33.9</v>
+        <v>36.7</v>
       </c>
       <c r="K92" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
@@ -8378,7 +8378,7 @@
         <v>41</v>
       </c>
       <c r="S92" t="n">
-        <v>-1.100000000000001</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T92" t="n">
         <v>36.2</v>
@@ -9642,10 +9642,10 @@
         <v>35</v>
       </c>
       <c r="J107" t="n">
-        <v>34.1</v>
+        <v>39.8</v>
       </c>
       <c r="K107" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="L107" t="inlineStr">
         <is>
@@ -9675,7 +9675,7 @@
         <v>41</v>
       </c>
       <c r="S107" t="n">
-        <v>-0.8999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T107" t="n">
         <v>36.83333333333334</v>
@@ -11034,10 +11034,10 @@
         <v>21</v>
       </c>
       <c r="J123" t="n">
-        <v>18.4</v>
+        <v>22.6</v>
       </c>
       <c r="K123" t="n">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="L123" t="inlineStr">
         <is>
@@ -11067,10 +11067,10 @@
         <v>21</v>
       </c>
       <c r="S123" t="n">
-        <v>-2.600000000000001</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T123" t="n">
-        <v>22.93333333333333</v>
+        <v>22.93333333333334</v>
       </c>
       <c r="U123" t="n">
         <v>3</v>
@@ -12772,10 +12772,10 @@
         <v>35</v>
       </c>
       <c r="J143" t="n">
-        <v>37.5</v>
+        <v>31.4</v>
       </c>
       <c r="K143" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
@@ -12805,7 +12805,7 @@
         <v>41</v>
       </c>
       <c r="S143" t="n">
-        <v>2.5</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="T143" t="n">
         <v>38.3</v>
@@ -13723,10 +13723,10 @@
         <v>35</v>
       </c>
       <c r="J154" t="n">
-        <v>36.7</v>
+        <v>37.5</v>
       </c>
       <c r="K154" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -13756,7 +13756,7 @@
         <v>41</v>
       </c>
       <c r="S154" t="n">
-        <v>1.700000000000003</v>
+        <v>2.5</v>
       </c>
       <c r="T154" t="n">
         <v>35.23333333333333</v>
@@ -17887,10 +17887,10 @@
         <v>21</v>
       </c>
       <c r="J202" t="n">
-        <v>23.1</v>
+        <v>22.6</v>
       </c>
       <c r="K202" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="L202" t="inlineStr">
         <is>
@@ -17920,7 +17920,7 @@
         <v>21</v>
       </c>
       <c r="S202" t="n">
-        <v>2.100000000000001</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="T202" t="n">
         <v>22.13333333333334</v>
@@ -18148,10 +18148,10 @@
         <v>28</v>
       </c>
       <c r="J205" t="n">
-        <v>26.1</v>
+        <v>27.7</v>
       </c>
       <c r="K205" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="L205" t="inlineStr">
         <is>
@@ -18181,7 +18181,7 @@
         <v>28</v>
       </c>
       <c r="S205" t="n">
-        <v>-1.899999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="T205" t="n">
         <v>27.5</v>
@@ -20060,10 +20060,10 @@
         <v>28</v>
       </c>
       <c r="J227" t="n">
-        <v>30.1</v>
+        <v>29.3</v>
       </c>
       <c r="K227" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="L227" t="inlineStr">
         <is>
@@ -20093,7 +20093,7 @@
         <v>28</v>
       </c>
       <c r="S227" t="n">
-        <v>2.100000000000001</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="T227" t="n">
         <v>28.96666666666667</v>
@@ -21788,10 +21788,10 @@
         <v>21</v>
       </c>
       <c r="J247" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="K247" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L247" t="inlineStr">
         <is>
@@ -21821,7 +21821,7 @@
         <v>21</v>
       </c>
       <c r="S247" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="T247" t="n">
         <v>21.2</v>
@@ -24732,10 +24732,10 @@
         <v>21</v>
       </c>
       <c r="J281" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
       <c r="K281" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L281" t="inlineStr">
         <is>
@@ -24765,7 +24765,7 @@
         <v>21</v>
       </c>
       <c r="S281" t="n">
-        <v>-3.399999999999999</v>
+        <v>-3.699999999999999</v>
       </c>
       <c r="T281" t="n">
         <v>17.43333333333333</v>
@@ -25337,10 +25337,10 @@
         <v>21</v>
       </c>
       <c r="J288" t="n">
-        <v>22.6</v>
+        <v>25.9</v>
       </c>
       <c r="K288" t="n">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="L288" t="inlineStr">
         <is>
@@ -25370,7 +25370,7 @@
         <v>21</v>
       </c>
       <c r="S288" t="n">
-        <v>1.600000000000001</v>
+        <v>4.899999999999999</v>
       </c>
       <c r="T288" t="n">
         <v>22.7</v>
@@ -26899,10 +26899,10 @@
         <v>21</v>
       </c>
       <c r="J306" t="n">
-        <v>22</v>
+        <v>19.4</v>
       </c>
       <c r="K306" t="n">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -26932,7 +26932,7 @@
         <v>21</v>
       </c>
       <c r="S306" t="n">
-        <v>1</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="T306" t="n">
         <v>20.8</v>
@@ -27419,10 +27419,10 @@
         <v>24.5</v>
       </c>
       <c r="J312" t="n">
-        <v>23.3</v>
+        <v>25.8</v>
       </c>
       <c r="K312" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="L312" t="inlineStr">
         <is>
@@ -27452,7 +27452,7 @@
         <v>28</v>
       </c>
       <c r="S312" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="T312" t="n">
         <v>24.26666666666667</v>
@@ -29246,10 +29246,10 @@
         <v>24.5</v>
       </c>
       <c r="J333" t="n">
-        <v>24.5</v>
+        <v>25.3</v>
       </c>
       <c r="K333" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="L333" t="inlineStr">
         <is>
@@ -29279,7 +29279,7 @@
         <v>28</v>
       </c>
       <c r="S333" t="n">
-        <v>0</v>
+        <v>0.8000000000000007</v>
       </c>
       <c r="T333" t="n">
         <v>24.6</v>
@@ -31763,10 +31763,10 @@
         <v>21</v>
       </c>
       <c r="J362" t="n">
-        <v>20.2</v>
+        <v>21.1</v>
       </c>
       <c r="K362" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L362" t="inlineStr">
         <is>
@@ -31796,7 +31796,7 @@
         <v>21</v>
       </c>
       <c r="S362" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="T362" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-09-30 21:51:08
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3541,7 +3541,7 @@
         <v>3</v>
       </c>
       <c r="V36" t="n">
-        <v>43.06666666666667</v>
+        <v>42.37777777777777</v>
       </c>
       <c r="W36" t="n">
         <v>27.5</v>
@@ -4015,10 +4015,10 @@
         <v>31</v>
       </c>
       <c r="J42" t="n">
-        <v>30.7</v>
+        <v>31.4</v>
       </c>
       <c r="K42" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="T42" t="n">
         <v>32.63333333333333</v>
@@ -4879,10 +4879,10 @@
         <v>31</v>
       </c>
       <c r="J52" t="n">
-        <v>30.5</v>
+        <v>38.5</v>
       </c>
       <c r="K52" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="n">
-        <v>-0.5</v>
+        <v>7.5</v>
       </c>
       <c r="T52" t="n">
         <v>35.86666666666667</v>
@@ -5138,10 +5138,10 @@
         <v>31</v>
       </c>
       <c r="J55" t="n">
-        <v>18.8</v>
+        <v>37.1</v>
       </c>
       <c r="K55" t="n">
-        <v>61</v>
+        <v>120</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="n">
-        <v>-12.2</v>
+        <v>6.100000000000001</v>
       </c>
       <c r="T55" t="n">
         <v>31.73333333333333</v>
@@ -5265,7 +5265,7 @@
         <v>3</v>
       </c>
       <c r="V56" t="n">
-        <v>23.14444444444444</v>
+        <v>23.14444444444445</v>
       </c>
       <c r="W56" t="n">
         <v>20.5</v>
@@ -5569,10 +5569,10 @@
         <v>24</v>
       </c>
       <c r="J60" t="n">
-        <v>25.9</v>
+        <v>23.1</v>
       </c>
       <c r="K60" t="n">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -5602,7 +5602,7 @@
         <v>28</v>
       </c>
       <c r="S60" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="T60" t="n">
         <v>24.1</v>
@@ -7305,10 +7305,10 @@
         <v>21</v>
       </c>
       <c r="J80" t="n">
-        <v>26.4</v>
+        <v>17.9</v>
       </c>
       <c r="K80" t="n">
-        <v>126</v>
+        <v>85</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -7338,7 +7338,7 @@
         <v>21</v>
       </c>
       <c r="S80" t="n">
-        <v>5.399999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="T80" t="n">
         <v>21.3</v>
@@ -7740,10 +7740,10 @@
         <v>21</v>
       </c>
       <c r="J85" t="n">
-        <v>26</v>
+        <v>19.3</v>
       </c>
       <c r="K85" t="n">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -7773,7 +7773,7 @@
         <v>21</v>
       </c>
       <c r="S85" t="n">
-        <v>5</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="T85" t="n">
         <v>22</v>
@@ -7782,7 +7782,7 @@
         <v>3</v>
       </c>
       <c r="V85" t="n">
-        <v>24.43333333333334</v>
+        <v>24.43333333333333</v>
       </c>
       <c r="W85" t="n">
         <v>17.5</v>
@@ -7912,10 +7912,10 @@
         <v>21</v>
       </c>
       <c r="J87" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K87" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="L87" t="inlineStr">
         <is>
@@ -7945,7 +7945,7 @@
         <v>21</v>
       </c>
       <c r="S87" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="T87" t="n">
         <v>19.9</v>
@@ -7999,10 +7999,10 @@
         <v>35</v>
       </c>
       <c r="J88" t="n">
-        <v>25.3</v>
+        <v>36.5</v>
       </c>
       <c r="K88" t="n">
-        <v>72</v>
+        <v>104</v>
       </c>
       <c r="L88" t="inlineStr">
         <is>
@@ -8032,7 +8032,7 @@
         <v>41</v>
       </c>
       <c r="S88" t="n">
-        <v>-9.699999999999999</v>
+        <v>1.5</v>
       </c>
       <c r="T88" t="n">
         <v>33.1</v>
@@ -8086,10 +8086,10 @@
         <v>35</v>
       </c>
       <c r="J89" t="n">
-        <v>39.1</v>
+        <v>36.7</v>
       </c>
       <c r="K89" t="n">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
@@ -8119,7 +8119,7 @@
         <v>41</v>
       </c>
       <c r="S89" t="n">
-        <v>4.100000000000001</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T89" t="n">
         <v>35.73333333333333</v>
@@ -8128,7 +8128,7 @@
         <v>3</v>
       </c>
       <c r="V89" t="n">
-        <v>35.86296296296297</v>
+        <v>35.86296296296296</v>
       </c>
       <c r="W89" t="n">
         <v>31.5</v>
@@ -8173,10 +8173,10 @@
         <v>35</v>
       </c>
       <c r="J90" t="n">
-        <v>40.3</v>
+        <v>39.8</v>
       </c>
       <c r="K90" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="L90" t="inlineStr">
         <is>
@@ -8206,7 +8206,7 @@
         <v>41</v>
       </c>
       <c r="S90" t="n">
-        <v>5.299999999999997</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="T90" t="n">
         <v>36.16666666666666</v>
@@ -8215,7 +8215,7 @@
         <v>3</v>
       </c>
       <c r="V90" t="n">
-        <v>38.87407407407407</v>
+        <v>38.87407407407408</v>
       </c>
       <c r="W90" t="n">
         <v>31.5</v>
@@ -8345,10 +8345,10 @@
         <v>35</v>
       </c>
       <c r="J92" t="n">
-        <v>36.7</v>
+        <v>33.9</v>
       </c>
       <c r="K92" t="n">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="L92" t="inlineStr">
         <is>
@@ -8378,7 +8378,7 @@
         <v>41</v>
       </c>
       <c r="S92" t="n">
-        <v>1.700000000000003</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="T92" t="n">
         <v>36.2</v>
@@ -12772,10 +12772,10 @@
         <v>35</v>
       </c>
       <c r="J143" t="n">
-        <v>31.4</v>
+        <v>37.5</v>
       </c>
       <c r="K143" t="n">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="L143" t="inlineStr">
         <is>
@@ -12805,7 +12805,7 @@
         <v>41</v>
       </c>
       <c r="S143" t="n">
-        <v>-3.600000000000001</v>
+        <v>2.5</v>
       </c>
       <c r="T143" t="n">
         <v>38.3</v>
@@ -13723,10 +13723,10 @@
         <v>35</v>
       </c>
       <c r="J154" t="n">
-        <v>37.5</v>
+        <v>36.7</v>
       </c>
       <c r="K154" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L154" t="inlineStr">
         <is>
@@ -13756,7 +13756,7 @@
         <v>41</v>
       </c>
       <c r="S154" t="n">
-        <v>2.5</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="T154" t="n">
         <v>35.23333333333333</v>
@@ -17887,10 +17887,10 @@
         <v>21</v>
       </c>
       <c r="J202" t="n">
-        <v>22.6</v>
+        <v>23.1</v>
       </c>
       <c r="K202" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="L202" t="inlineStr">
         <is>
@@ -17920,7 +17920,7 @@
         <v>21</v>
       </c>
       <c r="S202" t="n">
-        <v>1.600000000000001</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="T202" t="n">
         <v>22.13333333333334</v>
@@ -18148,10 +18148,10 @@
         <v>28</v>
       </c>
       <c r="J205" t="n">
-        <v>27.7</v>
+        <v>26.1</v>
       </c>
       <c r="K205" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="L205" t="inlineStr">
         <is>
@@ -18181,7 +18181,7 @@
         <v>28</v>
       </c>
       <c r="S205" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="T205" t="n">
         <v>27.5</v>
@@ -21788,10 +21788,10 @@
         <v>21</v>
       </c>
       <c r="J247" t="n">
-        <v>21.2</v>
+        <v>21.5</v>
       </c>
       <c r="K247" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L247" t="inlineStr">
         <is>
@@ -21821,7 +21821,7 @@
         <v>21</v>
       </c>
       <c r="S247" t="n">
-        <v>0.1999999999999993</v>
+        <v>0.5</v>
       </c>
       <c r="T247" t="n">
         <v>21.2</v>
@@ -24732,10 +24732,10 @@
         <v>21</v>
       </c>
       <c r="J281" t="n">
-        <v>17.3</v>
+        <v>17.6</v>
       </c>
       <c r="K281" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="L281" t="inlineStr">
         <is>
@@ -24765,7 +24765,7 @@
         <v>21</v>
       </c>
       <c r="S281" t="n">
-        <v>-3.699999999999999</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="T281" t="n">
         <v>17.43333333333333</v>
@@ -26899,10 +26899,10 @@
         <v>21</v>
       </c>
       <c r="J306" t="n">
-        <v>19.4</v>
+        <v>22</v>
       </c>
       <c r="K306" t="n">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="L306" t="inlineStr">
         <is>
@@ -26932,7 +26932,7 @@
         <v>21</v>
       </c>
       <c r="S306" t="n">
-        <v>-1.600000000000001</v>
+        <v>1</v>
       </c>
       <c r="T306" t="n">
         <v>20.8</v>
@@ -27419,10 +27419,10 @@
         <v>24.5</v>
       </c>
       <c r="J312" t="n">
-        <v>25.8</v>
+        <v>23.3</v>
       </c>
       <c r="K312" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="L312" t="inlineStr">
         <is>
@@ -27452,7 +27452,7 @@
         <v>28</v>
       </c>
       <c r="S312" t="n">
-        <v>1.300000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="T312" t="n">
         <v>24.26666666666667</v>
@@ -28202,10 +28202,10 @@
         <v>24.5</v>
       </c>
       <c r="J321" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K321" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L321" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         <v>28</v>
       </c>
       <c r="S321" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T321" t="n">
         <v>24.66666666666667</v>
@@ -28898,10 +28898,10 @@
         <v>24.5</v>
       </c>
       <c r="J329" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K329" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L329" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         <v>28</v>
       </c>
       <c r="S329" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T329" t="n">
         <v>27.1</v>
@@ -30812,10 +30812,10 @@
         <v>24.5</v>
       </c>
       <c r="J351" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K351" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L351" t="inlineStr">
         <is>
@@ -30845,10 +30845,10 @@
         <v>28</v>
       </c>
       <c r="S351" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T351" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U351" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-01 19:35:47
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -22387,10 +22387,10 @@
         <v>21</v>
       </c>
       <c r="J254" t="n">
-        <v>23.1</v>
+        <v>22.3</v>
       </c>
       <c r="K254" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="L254" t="inlineStr">
         <is>
@@ -22420,7 +22420,7 @@
         <v>21</v>
       </c>
       <c r="S254" t="n">
-        <v>2.100000000000001</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="T254" t="n">
         <v>21.8</v>
@@ -27330,10 +27330,10 @@
         <v>24.5</v>
       </c>
       <c r="J311" t="n">
-        <v>22.6</v>
+        <v>25</v>
       </c>
       <c r="K311" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="L311" t="inlineStr">
         <is>
@@ -27363,7 +27363,7 @@
         <v>28</v>
       </c>
       <c r="S311" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="T311" t="n">
         <v>24.8</v>
@@ -27939,10 +27939,10 @@
         <v>24.5</v>
       </c>
       <c r="J318" t="n">
-        <v>30.6</v>
+        <v>23.5</v>
       </c>
       <c r="K318" t="n">
-        <v>125</v>
+        <v>96</v>
       </c>
       <c r="L318" t="inlineStr">
         <is>
@@ -27972,7 +27972,7 @@
         <v>28</v>
       </c>
       <c r="S318" t="n">
-        <v>6.100000000000001</v>
+        <v>-1</v>
       </c>
       <c r="T318" t="n">
         <v>27.7</v>
@@ -28374,10 +28374,10 @@
         <v>24.5</v>
       </c>
       <c r="J323" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="K323" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="L323" t="inlineStr">
         <is>
@@ -28407,7 +28407,7 @@
         <v>28</v>
       </c>
       <c r="S323" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="T323" t="n">
         <v>24.66666666666667</v>
@@ -29070,10 +29070,10 @@
         <v>24.5</v>
       </c>
       <c r="J331" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="K331" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="L331" t="inlineStr">
         <is>
@@ -29103,7 +29103,7 @@
         <v>28</v>
       </c>
       <c r="S331" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="T331" t="n">
         <v>27.1</v>
@@ -29331,10 +29331,10 @@
         <v>24.5</v>
       </c>
       <c r="J334" t="n">
-        <v>21</v>
+        <v>26.9</v>
       </c>
       <c r="K334" t="n">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="L334" t="inlineStr">
         <is>
@@ -29364,7 +29364,7 @@
         <v>28</v>
       </c>
       <c r="S334" t="n">
-        <v>-3.5</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="T334" t="n">
         <v>24.26666666666667</v>
@@ -30984,10 +30984,10 @@
         <v>24.5</v>
       </c>
       <c r="J353" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="K353" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="L353" t="inlineStr">
         <is>
@@ -31017,10 +31017,10 @@
         <v>28</v>
       </c>
       <c r="S353" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="T353" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="U353" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-03 15:50:04
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4723,10 +4723,10 @@
         <v>24</v>
       </c>
       <c r="K49" t="n">
-        <v>23.8</v>
+        <v>24.9</v>
       </c>
       <c r="L49" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="M49" t="inlineStr">
         <is>
@@ -4756,7 +4756,7 @@
         <v>28</v>
       </c>
       <c r="T49" t="n">
-        <v>-0.1999999999999993</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U49" t="n">
         <v>21.43333333333333</v>
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L77" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7441,10 +7441,10 @@
         <v>28</v>
       </c>
       <c r="K80" t="n">
-        <v>30.7</v>
+        <v>29.2</v>
       </c>
       <c r="L80" t="n">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         <v>28</v>
       </c>
       <c r="T80" t="n">
-        <v>2.699999999999999</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="U80" t="n">
         <v>29.2</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L81" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -7791,10 +7791,10 @@
         <v>21</v>
       </c>
       <c r="K84" t="n">
-        <v>21.2</v>
+        <v>20.2</v>
       </c>
       <c r="L84" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="M84" t="inlineStr">
         <is>
@@ -7824,7 +7824,7 @@
         <v>21</v>
       </c>
       <c r="T84" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U84" t="n">
         <v>22.16666666666667</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L88" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L93" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -9979,10 +9979,10 @@
         <v>35</v>
       </c>
       <c r="K109" t="n">
-        <v>39.8</v>
+        <v>34.1</v>
       </c>
       <c r="L109" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="M109" t="inlineStr">
         <is>
@@ -10012,7 +10012,7 @@
         <v>41</v>
       </c>
       <c r="T109" t="n">
-        <v>4.799999999999997</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U109" t="n">
         <v>36.83333333333334</v>
@@ -12443,10 +12443,10 @@
         <v>31</v>
       </c>
       <c r="K137" t="n">
-        <v>31.9</v>
+        <v>31.3</v>
       </c>
       <c r="L137" t="n">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="M137" t="inlineStr">
         <is>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="S137" t="inlineStr"/>
       <c r="T137" t="n">
-        <v>0.8999999999999986</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U137" t="n">
         <v>31.23333333333333</v>
@@ -23225,10 +23225,10 @@
         <v>28</v>
       </c>
       <c r="K260" t="n">
-        <v>27.1</v>
+        <v>27.6</v>
       </c>
       <c r="L260" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M260" t="inlineStr">
         <is>
@@ -23258,7 +23258,7 @@
         <v>28</v>
       </c>
       <c r="T260" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U260" t="n">
         <v>27.4</v>
@@ -23489,10 +23489,10 @@
         <v>28</v>
       </c>
       <c r="K263" t="n">
-        <v>26.6</v>
+        <v>26.5</v>
       </c>
       <c r="L263" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M263" t="inlineStr">
         <is>
@@ -23522,7 +23522,7 @@
         <v>28</v>
       </c>
       <c r="T263" t="n">
-        <v>-1.399999999999999</v>
+        <v>-1.5</v>
       </c>
       <c r="U263" t="n">
         <v>26.36666666666666</v>
@@ -23577,10 +23577,10 @@
         <v>28</v>
       </c>
       <c r="K264" t="n">
-        <v>24.7</v>
+        <v>32.5</v>
       </c>
       <c r="L264" t="n">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="M264" t="inlineStr">
         <is>
@@ -23610,7 +23610,7 @@
         <v>28</v>
       </c>
       <c r="T264" t="n">
-        <v>-3.300000000000001</v>
+        <v>4.5</v>
       </c>
       <c r="U264" t="n">
         <v>29.5</v>
@@ -25507,10 +25507,10 @@
         <v>21</v>
       </c>
       <c r="K286" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="L286" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M286" t="inlineStr">
         <is>
@@ -25540,7 +25540,7 @@
         <v>21</v>
       </c>
       <c r="T286" t="n">
-        <v>-0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="U286" t="n">
         <v>21.03333333333333</v>
@@ -25943,10 +25943,10 @@
         <v>21</v>
       </c>
       <c r="K291" t="n">
-        <v>21.7</v>
+        <v>22.8</v>
       </c>
       <c r="L291" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="M291" t="inlineStr">
         <is>
@@ -25976,7 +25976,7 @@
         <v>21</v>
       </c>
       <c r="T291" t="n">
-        <v>0.6999999999999993</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="U291" t="n">
         <v>21.53333333333333</v>
@@ -26645,10 +26645,10 @@
         <v>21</v>
       </c>
       <c r="K299" t="n">
-        <v>18</v>
+        <v>21.1</v>
       </c>
       <c r="L299" t="n">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="M299" t="inlineStr">
         <is>
@@ -26678,7 +26678,7 @@
         <v>21</v>
       </c>
       <c r="T299" t="n">
-        <v>-3</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U299" t="n">
         <v>19.53333333333333</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L323" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L331" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -30777,10 +30777,10 @@
         <v>24.5</v>
       </c>
       <c r="K346" t="n">
-        <v>23.3</v>
+        <v>22.3</v>
       </c>
       <c r="L346" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="M346" t="inlineStr">
         <is>
@@ -30810,7 +30810,7 @@
         <v>28</v>
       </c>
       <c r="T346" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="U346" t="n">
         <v>23.03333333333333</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L353" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>
@@ -31831,10 +31831,10 @@
         <v>24.5</v>
       </c>
       <c r="K358" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="L358" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="M358" t="inlineStr">
         <is>
@@ -31864,7 +31864,7 @@
         <v>28</v>
       </c>
       <c r="T358" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U358" t="n">
         <v>26.4</v>
@@ -31919,10 +31919,10 @@
         <v>24.5</v>
       </c>
       <c r="K359" t="n">
-        <v>21.9</v>
+        <v>21.2</v>
       </c>
       <c r="L359" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="M359" t="inlineStr">
         <is>
@@ -31952,7 +31952,7 @@
         <v>28</v>
       </c>
       <c r="T359" t="n">
-        <v>-2.600000000000001</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="U359" t="n">
         <v>20.8</v>
@@ -32093,10 +32093,10 @@
         <v>24.5</v>
       </c>
       <c r="K361" t="n">
-        <v>27.4</v>
+        <v>23.5</v>
       </c>
       <c r="L361" t="n">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="M361" t="inlineStr">
         <is>
@@ -32126,7 +32126,7 @@
         <v>28</v>
       </c>
       <c r="T361" t="n">
-        <v>2.899999999999999</v>
+        <v>-1</v>
       </c>
       <c r="U361" t="n">
         <v>24.7</v>
@@ -32181,10 +32181,10 @@
         <v>24.5</v>
       </c>
       <c r="K362" t="n">
-        <v>28.6</v>
+        <v>25.1</v>
       </c>
       <c r="L362" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="M362" t="inlineStr">
         <is>
@@ -32214,7 +32214,7 @@
         <v>28</v>
       </c>
       <c r="T362" t="n">
-        <v>4.100000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U362" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-03 20:31:03
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3335,10 +3335,10 @@
         <v>31</v>
       </c>
       <c r="K33" t="n">
-        <v>31.4</v>
+        <v>29.6</v>
       </c>
       <c r="L33" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1.399999999999999</v>
       </c>
       <c r="U33" t="n">
         <v>30.33333333333333</v>
@@ -5161,10 +5161,10 @@
         <v>31</v>
       </c>
       <c r="K54" t="n">
-        <v>38.5</v>
+        <v>30.5</v>
       </c>
       <c r="L54" t="n">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="M54" t="inlineStr">
         <is>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="n">
-        <v>7.5</v>
+        <v>-0.5</v>
       </c>
       <c r="U54" t="n">
         <v>35.86666666666667</v>
@@ -6475,10 +6475,10 @@
         <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>34.3</v>
+        <v>32.3</v>
       </c>
       <c r="L69" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>41</v>
       </c>
       <c r="T69" t="n">
-        <v>-0.7000000000000028</v>
+        <v>-2.700000000000003</v>
       </c>
       <c r="U69" t="n">
         <v>32.96666666666666</v>
@@ -6605,7 +6605,7 @@
         <v>3</v>
       </c>
       <c r="W70" t="n">
-        <v>37.02962962962963</v>
+        <v>37.02962962962962</v>
       </c>
       <c r="X70" t="n">
         <v>31.5</v>
@@ -6739,10 +6739,10 @@
         <v>35</v>
       </c>
       <c r="K72" t="n">
-        <v>32.4</v>
+        <v>35</v>
       </c>
       <c r="L72" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="M72" t="inlineStr">
         <is>
@@ -6772,7 +6772,7 @@
         <v>41</v>
       </c>
       <c r="T72" t="n">
-        <v>-2.600000000000001</v>
+        <v>0</v>
       </c>
       <c r="U72" t="n">
         <v>34.83333333333334</v>
@@ -6781,7 +6781,7 @@
         <v>3</v>
       </c>
       <c r="W72" t="n">
-        <v>38.42962962962963</v>
+        <v>38.42962962962962</v>
       </c>
       <c r="X72" t="n">
         <v>31.5</v>
@@ -7003,10 +7003,10 @@
         <v>35</v>
       </c>
       <c r="K75" t="n">
-        <v>33.5</v>
+        <v>40.8</v>
       </c>
       <c r="L75" t="n">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -7036,10 +7036,10 @@
         <v>41</v>
       </c>
       <c r="T75" t="n">
-        <v>-1.5</v>
+        <v>5.799999999999997</v>
       </c>
       <c r="U75" t="n">
-        <v>37.56666666666667</v>
+        <v>37.56666666666666</v>
       </c>
       <c r="V75" t="n">
         <v>3</v>
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L77" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7353,10 +7353,10 @@
         <v>28</v>
       </c>
       <c r="K79" t="n">
-        <v>24.8</v>
+        <v>25.9</v>
       </c>
       <c r="L79" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7386,10 +7386,10 @@
         <v>28</v>
       </c>
       <c r="T79" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U79" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="V79" t="n">
         <v>3</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L81" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L88" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L93" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -12221,7 +12221,7 @@
         <v>3</v>
       </c>
       <c r="W134" t="n">
-        <v>29.6111111111111</v>
+        <v>29.61111111111111</v>
       </c>
       <c r="X134" t="n">
         <v>24.5</v>
@@ -12267,10 +12267,10 @@
         <v>35</v>
       </c>
       <c r="K135" t="n">
-        <v>36.1</v>
+        <v>29.2</v>
       </c>
       <c r="L135" t="n">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="M135" t="inlineStr">
         <is>
@@ -12300,7 +12300,7 @@
         <v>41</v>
       </c>
       <c r="T135" t="n">
-        <v>1.100000000000001</v>
+        <v>-5.800000000000001</v>
       </c>
       <c r="U135" t="n">
         <v>33.9</v>
@@ -14107,10 +14107,10 @@
         <v>35</v>
       </c>
       <c r="K156" t="n">
-        <v>36.7</v>
+        <v>31.5</v>
       </c>
       <c r="L156" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="M156" t="inlineStr">
         <is>
@@ -14140,7 +14140,7 @@
         <v>41</v>
       </c>
       <c r="T156" t="n">
-        <v>1.700000000000003</v>
+        <v>-3.5</v>
       </c>
       <c r="U156" t="n">
         <v>35.23333333333333</v>
@@ -15423,10 +15423,10 @@
         <v>35</v>
       </c>
       <c r="K171" t="n">
-        <v>34</v>
+        <v>39.3</v>
       </c>
       <c r="L171" t="n">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="M171" t="inlineStr">
         <is>
@@ -15456,7 +15456,7 @@
         <v>41</v>
       </c>
       <c r="T171" t="n">
-        <v>-1</v>
+        <v>4.299999999999997</v>
       </c>
       <c r="U171" t="n">
         <v>36.3</v>
@@ -16301,10 +16301,10 @@
         <v>35</v>
       </c>
       <c r="K181" t="n">
-        <v>38.3</v>
+        <v>34.3</v>
       </c>
       <c r="L181" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="M181" t="inlineStr">
         <is>
@@ -16334,7 +16334,7 @@
         <v>41</v>
       </c>
       <c r="T181" t="n">
-        <v>3.299999999999997</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="U181" t="n">
         <v>35.66666666666666</v>
@@ -22265,10 +22265,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>21.2</v>
+        <v>21.5</v>
       </c>
       <c r="L249" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22298,7 +22298,7 @@
         <v>21</v>
       </c>
       <c r="T249" t="n">
-        <v>0.1999999999999993</v>
+        <v>0.5</v>
       </c>
       <c r="U249" t="n">
         <v>21.2</v>
@@ -24539,10 +24539,10 @@
         <v>28</v>
       </c>
       <c r="K275" t="n">
-        <v>28.7</v>
+        <v>27.5</v>
       </c>
       <c r="L275" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="M275" t="inlineStr">
         <is>
@@ -24572,7 +24572,7 @@
         <v>28</v>
       </c>
       <c r="T275" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.5</v>
       </c>
       <c r="U275" t="n">
         <v>28.6</v>
@@ -24581,7 +24581,7 @@
         <v>3</v>
       </c>
       <c r="W275" t="n">
-        <v>32.98888888888889</v>
+        <v>32.9888888888889</v>
       </c>
       <c r="X275" t="n">
         <v>24.5</v>
@@ -25855,10 +25855,10 @@
         <v>21</v>
       </c>
       <c r="K290" t="n">
-        <v>22.6</v>
+        <v>25.9</v>
       </c>
       <c r="L290" t="n">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="M290" t="inlineStr">
         <is>
@@ -25888,7 +25888,7 @@
         <v>21</v>
       </c>
       <c r="T290" t="n">
-        <v>1.600000000000001</v>
+        <v>4.899999999999999</v>
       </c>
       <c r="U290" t="n">
         <v>22.7</v>
@@ -27697,10 +27697,10 @@
         <v>24.5</v>
       </c>
       <c r="K311" t="n">
-        <v>22.6</v>
+        <v>25</v>
       </c>
       <c r="L311" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="M311" t="inlineStr">
         <is>
@@ -27730,7 +27730,7 @@
         <v>28</v>
       </c>
       <c r="T311" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="U311" t="n">
         <v>24.8</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L323" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L331" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L353" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>
@@ -32355,10 +32355,10 @@
         <v>21</v>
       </c>
       <c r="K364" t="n">
-        <v>20.2</v>
+        <v>21.1</v>
       </c>
       <c r="L364" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="M364" t="inlineStr">
         <is>
@@ -32388,7 +32388,7 @@
         <v>21</v>
       </c>
       <c r="T364" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U364" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-03 22:46:13
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3335,10 +3335,10 @@
         <v>31</v>
       </c>
       <c r="K33" t="n">
-        <v>29.6</v>
+        <v>31.4</v>
       </c>
       <c r="L33" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
-        <v>-1.399999999999999</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U33" t="n">
         <v>30.33333333333333</v>
@@ -5161,10 +5161,10 @@
         <v>31</v>
       </c>
       <c r="K54" t="n">
-        <v>30.5</v>
+        <v>38.5</v>
       </c>
       <c r="L54" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="M54" t="inlineStr">
         <is>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="n">
-        <v>-0.5</v>
+        <v>7.5</v>
       </c>
       <c r="U54" t="n">
         <v>35.86666666666667</v>
@@ -6475,10 +6475,10 @@
         <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>32.3</v>
+        <v>34.3</v>
       </c>
       <c r="L69" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>41</v>
       </c>
       <c r="T69" t="n">
-        <v>-2.700000000000003</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="U69" t="n">
         <v>32.96666666666666</v>
@@ -6605,7 +6605,7 @@
         <v>3</v>
       </c>
       <c r="W70" t="n">
-        <v>37.02962962962962</v>
+        <v>37.02962962962963</v>
       </c>
       <c r="X70" t="n">
         <v>31.5</v>
@@ -6739,10 +6739,10 @@
         <v>35</v>
       </c>
       <c r="K72" t="n">
-        <v>35</v>
+        <v>32.4</v>
       </c>
       <c r="L72" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="M72" t="inlineStr">
         <is>
@@ -6772,7 +6772,7 @@
         <v>41</v>
       </c>
       <c r="T72" t="n">
-        <v>0</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U72" t="n">
         <v>34.83333333333334</v>
@@ -6781,7 +6781,7 @@
         <v>3</v>
       </c>
       <c r="W72" t="n">
-        <v>38.42962962962962</v>
+        <v>38.42962962962963</v>
       </c>
       <c r="X72" t="n">
         <v>31.5</v>
@@ -7003,10 +7003,10 @@
         <v>35</v>
       </c>
       <c r="K75" t="n">
-        <v>40.8</v>
+        <v>33.5</v>
       </c>
       <c r="L75" t="n">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -7036,10 +7036,10 @@
         <v>41</v>
       </c>
       <c r="T75" t="n">
-        <v>5.799999999999997</v>
+        <v>-1.5</v>
       </c>
       <c r="U75" t="n">
-        <v>37.56666666666666</v>
+        <v>37.56666666666667</v>
       </c>
       <c r="V75" t="n">
         <v>3</v>
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L77" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7353,10 +7353,10 @@
         <v>28</v>
       </c>
       <c r="K79" t="n">
-        <v>25.9</v>
+        <v>24.8</v>
       </c>
       <c r="L79" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7386,10 +7386,10 @@
         <v>28</v>
       </c>
       <c r="T79" t="n">
-        <v>-2.100000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U79" t="n">
-        <v>25.13333333333333</v>
+        <v>25.13333333333334</v>
       </c>
       <c r="V79" t="n">
         <v>3</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L81" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L88" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L93" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -12221,7 +12221,7 @@
         <v>3</v>
       </c>
       <c r="W134" t="n">
-        <v>29.61111111111111</v>
+        <v>29.6111111111111</v>
       </c>
       <c r="X134" t="n">
         <v>24.5</v>
@@ -12267,10 +12267,10 @@
         <v>35</v>
       </c>
       <c r="K135" t="n">
-        <v>29.2</v>
+        <v>36.1</v>
       </c>
       <c r="L135" t="n">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="M135" t="inlineStr">
         <is>
@@ -12300,7 +12300,7 @@
         <v>41</v>
       </c>
       <c r="T135" t="n">
-        <v>-5.800000000000001</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U135" t="n">
         <v>33.9</v>
@@ -14107,10 +14107,10 @@
         <v>35</v>
       </c>
       <c r="K156" t="n">
-        <v>31.5</v>
+        <v>36.7</v>
       </c>
       <c r="L156" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="M156" t="inlineStr">
         <is>
@@ -14140,7 +14140,7 @@
         <v>41</v>
       </c>
       <c r="T156" t="n">
-        <v>-3.5</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U156" t="n">
         <v>35.23333333333333</v>
@@ -15423,10 +15423,10 @@
         <v>35</v>
       </c>
       <c r="K171" t="n">
-        <v>39.3</v>
+        <v>34</v>
       </c>
       <c r="L171" t="n">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="M171" t="inlineStr">
         <is>
@@ -15456,7 +15456,7 @@
         <v>41</v>
       </c>
       <c r="T171" t="n">
-        <v>4.299999999999997</v>
+        <v>-1</v>
       </c>
       <c r="U171" t="n">
         <v>36.3</v>
@@ -16301,10 +16301,10 @@
         <v>35</v>
       </c>
       <c r="K181" t="n">
-        <v>34.3</v>
+        <v>38.3</v>
       </c>
       <c r="L181" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="M181" t="inlineStr">
         <is>
@@ -16334,7 +16334,7 @@
         <v>41</v>
       </c>
       <c r="T181" t="n">
-        <v>-0.7000000000000028</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U181" t="n">
         <v>35.66666666666666</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L323" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L331" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L353" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-04 07:51:51
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -6475,10 +6475,10 @@
         <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>32.3</v>
+        <v>34.3</v>
       </c>
       <c r="L69" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>41</v>
       </c>
       <c r="T69" t="n">
-        <v>-2.700000000000003</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="U69" t="n">
         <v>32.96666666666666</v>
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L77" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L81" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L88" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L93" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -10771,10 +10771,10 @@
         <v>28</v>
       </c>
       <c r="K118" t="n">
-        <v>30.7</v>
+        <v>27.6</v>
       </c>
       <c r="L118" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -10804,7 +10804,7 @@
         <v>28</v>
       </c>
       <c r="T118" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U118" t="n">
         <v>28.03333333333333</v>
@@ -10859,10 +10859,10 @@
         <v>35</v>
       </c>
       <c r="K119" t="n">
-        <v>44.6</v>
+        <v>40.9</v>
       </c>
       <c r="L119" t="n">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="M119" t="inlineStr">
         <is>
@@ -10892,7 +10892,7 @@
         <v>41</v>
       </c>
       <c r="T119" t="n">
-        <v>9.600000000000001</v>
+        <v>5.899999999999999</v>
       </c>
       <c r="U119" t="n">
         <v>38.96666666666667</v>
@@ -10947,10 +10947,10 @@
         <v>35</v>
       </c>
       <c r="K120" t="n">
-        <v>34.6</v>
+        <v>37.4</v>
       </c>
       <c r="L120" t="n">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="M120" t="inlineStr">
         <is>
@@ -10980,7 +10980,7 @@
         <v>41</v>
       </c>
       <c r="T120" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U120" t="n">
         <v>35.63333333333333</v>
@@ -11035,10 +11035,10 @@
         <v>35</v>
       </c>
       <c r="K121" t="n">
-        <v>38.6</v>
+        <v>39.7</v>
       </c>
       <c r="L121" t="n">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="M121" t="inlineStr">
         <is>
@@ -11068,7 +11068,7 @@
         <v>41</v>
       </c>
       <c r="T121" t="n">
-        <v>3.600000000000001</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="U121" t="n">
         <v>37.46666666666667</v>
@@ -11123,10 +11123,10 @@
         <v>21</v>
       </c>
       <c r="K122" t="n">
-        <v>26</v>
+        <v>19.3</v>
       </c>
       <c r="L122" t="n">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="M122" t="inlineStr">
         <is>
@@ -11156,7 +11156,7 @@
         <v>21</v>
       </c>
       <c r="T122" t="n">
-        <v>5</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U122" t="n">
         <v>23.7</v>
@@ -23665,10 +23665,10 @@
         <v>28</v>
       </c>
       <c r="K265" t="n">
-        <v>23.6</v>
+        <v>28.7</v>
       </c>
       <c r="L265" t="n">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="M265" t="inlineStr">
         <is>
@@ -23698,7 +23698,7 @@
         <v>28</v>
       </c>
       <c r="T265" t="n">
-        <v>-4.399999999999999</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U265" t="n">
         <v>27</v>
@@ -24979,10 +24979,10 @@
         <v>28</v>
       </c>
       <c r="K280" t="n">
-        <v>29</v>
+        <v>28.2</v>
       </c>
       <c r="L280" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="M280" t="inlineStr">
         <is>
@@ -25012,7 +25012,7 @@
         <v>28</v>
       </c>
       <c r="T280" t="n">
-        <v>1</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U280" t="n">
         <v>28.2</v>
@@ -25197,7 +25197,7 @@
         <v>3</v>
       </c>
       <c r="W282" t="n">
-        <v>24.36666666666666</v>
+        <v>24.36666666666667</v>
       </c>
       <c r="X282" t="n">
         <v>17.5</v>
@@ -27347,10 +27347,10 @@
         <v>21</v>
       </c>
       <c r="K307" t="n">
-        <v>20.4</v>
+        <v>21.8</v>
       </c>
       <c r="L307" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="M307" t="inlineStr">
         <is>
@@ -27380,7 +27380,7 @@
         <v>21</v>
       </c>
       <c r="T307" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.8000000000000007</v>
       </c>
       <c r="U307" t="n">
         <v>20.76666666666667</v>
@@ -29587,7 +29587,7 @@
         <v>3</v>
       </c>
       <c r="W332" t="n">
-        <v>25.57777777777778</v>
+        <v>25.57777777777777</v>
       </c>
       <c r="X332" t="n">
         <v>21</v>
@@ -30953,10 +30953,10 @@
         <v>24.5</v>
       </c>
       <c r="K348" t="n">
-        <v>23.4</v>
+        <v>28.9</v>
       </c>
       <c r="L348" t="n">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="M348" t="inlineStr">
         <is>
@@ -30986,7 +30986,7 @@
         <v>28</v>
       </c>
       <c r="T348" t="n">
-        <v>-1.100000000000001</v>
+        <v>4.399999999999999</v>
       </c>
       <c r="U348" t="n">
         <v>29.46666666666667</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>28.5</v>
+        <v>31.7</v>
       </c>
       <c r="L355" t="n">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,7 +31600,7 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>4</v>
+        <v>7.199999999999999</v>
       </c>
       <c r="U355" t="n">
         <v>28.1</v>
@@ -32181,10 +32181,10 @@
         <v>24.5</v>
       </c>
       <c r="K362" t="n">
-        <v>28.6</v>
+        <v>23.3</v>
       </c>
       <c r="L362" t="n">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="M362" t="inlineStr">
         <is>
@@ -32214,7 +32214,7 @@
         <v>28</v>
       </c>
       <c r="T362" t="n">
-        <v>4.100000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U362" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-04 19:05:55
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L77" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L81" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L88" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8493,10 +8493,10 @@
         <v>35</v>
       </c>
       <c r="K92" t="n">
-        <v>40.3</v>
+        <v>39.8</v>
       </c>
       <c r="L92" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -8526,7 +8526,7 @@
         <v>41</v>
       </c>
       <c r="T92" t="n">
-        <v>5.299999999999997</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="U92" t="n">
         <v>36.16666666666666</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L93" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -11299,10 +11299,10 @@
         <v>21</v>
       </c>
       <c r="K124" t="n">
-        <v>20.4</v>
+        <v>23.7</v>
       </c>
       <c r="L124" t="n">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11332,7 +11332,7 @@
         <v>21</v>
       </c>
       <c r="T124" t="n">
-        <v>-0.6000000000000014</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U124" t="n">
         <v>21.43333333333333</v>
@@ -12617,10 +12617,10 @@
         <v>35</v>
       </c>
       <c r="K139" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="L139" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="M139" t="inlineStr">
         <is>
@@ -12650,7 +12650,7 @@
         <v>41</v>
       </c>
       <c r="T139" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="U139" t="n">
         <v>41</v>
@@ -14283,10 +14283,10 @@
         <v>21</v>
       </c>
       <c r="K158" t="n">
-        <v>19.1</v>
+        <v>22.2</v>
       </c>
       <c r="L158" t="n">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="M158" t="inlineStr">
         <is>
@@ -14316,7 +14316,7 @@
         <v>21</v>
       </c>
       <c r="T158" t="n">
-        <v>-1.899999999999999</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="U158" t="n">
         <v>21.83333333333333</v>
@@ -15511,10 +15511,10 @@
         <v>28</v>
       </c>
       <c r="K172" t="n">
-        <v>24.8</v>
+        <v>27</v>
       </c>
       <c r="L172" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="M172" t="inlineStr">
         <is>
@@ -15544,7 +15544,7 @@
         <v>28</v>
       </c>
       <c r="T172" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1</v>
       </c>
       <c r="U172" t="n">
         <v>26.4</v>
@@ -22611,10 +22611,10 @@
         <v>21</v>
       </c>
       <c r="K253" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="L253" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="M253" t="inlineStr">
         <is>
@@ -22642,7 +22642,7 @@
       </c>
       <c r="S253" t="inlineStr"/>
       <c r="T253" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U253" t="n">
         <v>21.8</v>
@@ -24891,10 +24891,10 @@
         <v>28</v>
       </c>
       <c r="K279" t="n">
-        <v>27.5</v>
+        <v>25.7</v>
       </c>
       <c r="L279" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="M279" t="inlineStr">
         <is>
@@ -24924,7 +24924,7 @@
         <v>28</v>
       </c>
       <c r="T279" t="n">
-        <v>-0.5</v>
+        <v>-2.300000000000001</v>
       </c>
       <c r="U279" t="n">
         <v>27</v>
@@ -25725,7 +25725,7 @@
         <v>3</v>
       </c>
       <c r="W288" t="n">
-        <v>21.74444444444445</v>
+        <v>21.74444444444444</v>
       </c>
       <c r="X288" t="n">
         <v>17.5</v>
@@ -26207,10 +26207,10 @@
         <v>21</v>
       </c>
       <c r="K294" t="n">
-        <v>20.4</v>
+        <v>20.8</v>
       </c>
       <c r="L294" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M294" t="inlineStr">
         <is>
@@ -26240,7 +26240,7 @@
         <v>21</v>
       </c>
       <c r="T294" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U294" t="n">
         <v>20.76666666666667</v>
@@ -27523,10 +27523,10 @@
         <v>21</v>
       </c>
       <c r="K309" t="n">
-        <v>20.7</v>
+        <v>19.6</v>
       </c>
       <c r="L309" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="M309" t="inlineStr">
         <is>
@@ -27556,7 +27556,7 @@
         <v>21</v>
       </c>
       <c r="T309" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.399999999999999</v>
       </c>
       <c r="U309" t="n">
         <v>20.23333333333333</v>
@@ -27785,10 +27785,10 @@
         <v>24.5</v>
       </c>
       <c r="K312" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="L312" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="M312" t="inlineStr">
         <is>
@@ -27818,7 +27818,7 @@
         <v>28</v>
       </c>
       <c r="T312" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U312" t="n">
         <v>25.13333333333334</v>
@@ -29985,10 +29985,10 @@
         <v>24.5</v>
       </c>
       <c r="K337" t="n">
-        <v>25.6</v>
+        <v>24</v>
       </c>
       <c r="L337" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="M337" t="inlineStr">
         <is>
@@ -30018,7 +30018,7 @@
         <v>28</v>
       </c>
       <c r="T337" t="n">
-        <v>1.100000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="U337" t="n">
         <v>35.8</v>
@@ -30337,10 +30337,10 @@
         <v>24.5</v>
       </c>
       <c r="K341" t="n">
-        <v>14</v>
+        <v>27.1</v>
       </c>
       <c r="L341" t="n">
-        <v>57</v>
+        <v>111</v>
       </c>
       <c r="M341" t="inlineStr">
         <is>
@@ -30370,7 +30370,7 @@
         <v>28</v>
       </c>
       <c r="T341" t="n">
-        <v>-10.5</v>
+        <v>2.600000000000001</v>
       </c>
       <c r="U341" t="n">
         <v>21.96666666666667</v>
@@ -32355,10 +32355,10 @@
         <v>21</v>
       </c>
       <c r="K364" t="n">
-        <v>21.1</v>
+        <v>21.4</v>
       </c>
       <c r="L364" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M364" t="inlineStr">
         <is>
@@ -32388,7 +32388,7 @@
         <v>21</v>
       </c>
       <c r="T364" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U364" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-05 22:28:08
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -24101,10 +24101,10 @@
         <v>28</v>
       </c>
       <c r="K270" t="n">
-        <v>26.4</v>
+        <v>25.1</v>
       </c>
       <c r="L270" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="M270" t="inlineStr">
         <is>
@@ -24134,7 +24134,7 @@
         <v>28</v>
       </c>
       <c r="T270" t="n">
-        <v>-1.600000000000001</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="U270" t="n">
         <v>25.53333333333333</v>
@@ -25855,10 +25855,10 @@
         <v>21</v>
       </c>
       <c r="K290" t="n">
-        <v>25.9</v>
+        <v>22.6</v>
       </c>
       <c r="L290" t="n">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="M290" t="inlineStr">
         <is>
@@ -25888,7 +25888,7 @@
         <v>21</v>
       </c>
       <c r="T290" t="n">
-        <v>4.899999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U290" t="n">
         <v>22.7</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L323" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L331" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L353" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>
@@ -31919,10 +31919,10 @@
         <v>24.5</v>
       </c>
       <c r="K359" t="n">
-        <v>21.9</v>
+        <v>21.2</v>
       </c>
       <c r="L359" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="M359" t="inlineStr">
         <is>
@@ -31952,7 +31952,7 @@
         <v>28</v>
       </c>
       <c r="T359" t="n">
-        <v>-2.600000000000001</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="U359" t="n">
         <v>20.8</v>
@@ -32007,10 +32007,10 @@
         <v>24.5</v>
       </c>
       <c r="K360" t="n">
-        <v>22.7</v>
+        <v>29.1</v>
       </c>
       <c r="L360" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="M360" t="inlineStr">
         <is>
@@ -32040,7 +32040,7 @@
         <v>28</v>
       </c>
       <c r="T360" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="U360" t="n">
         <v>25.3</v>
@@ -32355,10 +32355,10 @@
         <v>21</v>
       </c>
       <c r="K364" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="L364" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M364" t="inlineStr">
         <is>
@@ -32388,7 +32388,7 @@
         <v>21</v>
       </c>
       <c r="T364" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U364" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-06 04:15:53
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2987,10 +2987,10 @@
         <v>24</v>
       </c>
       <c r="K29" t="n">
-        <v>21.6</v>
+        <v>15.8</v>
       </c>
       <c r="L29" t="n">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3020,7 +3020,7 @@
         <v>28</v>
       </c>
       <c r="T29" t="n">
-        <v>-2.399999999999999</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="U29" t="n">
         <v>19.2</v>
@@ -3335,10 +3335,10 @@
         <v>31</v>
       </c>
       <c r="K33" t="n">
-        <v>31.4</v>
+        <v>30</v>
       </c>
       <c r="L33" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1</v>
       </c>
       <c r="U33" t="n">
         <v>30.33333333333333</v>
@@ -4113,10 +4113,10 @@
         <v>24</v>
       </c>
       <c r="K42" t="n">
-        <v>17.6</v>
+        <v>16.2</v>
       </c>
       <c r="L42" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="M42" t="inlineStr">
         <is>
@@ -4146,7 +4146,7 @@
         <v>28</v>
       </c>
       <c r="T42" t="n">
-        <v>-6.399999999999999</v>
+        <v>-7.800000000000001</v>
       </c>
       <c r="U42" t="n">
         <v>16.5</v>
@@ -6299,10 +6299,10 @@
         <v>28</v>
       </c>
       <c r="K67" t="n">
-        <v>25.6</v>
+        <v>26.2</v>
       </c>
       <c r="L67" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -6332,7 +6332,7 @@
         <v>28</v>
       </c>
       <c r="T67" t="n">
-        <v>-2.399999999999999</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="U67" t="n">
         <v>26.1</v>
@@ -6915,10 +6915,10 @@
         <v>21</v>
       </c>
       <c r="K74" t="n">
-        <v>24.6</v>
+        <v>23.9</v>
       </c>
       <c r="L74" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="M74" t="inlineStr">
         <is>
@@ -6948,7 +6948,7 @@
         <v>21</v>
       </c>
       <c r="T74" t="n">
-        <v>3.600000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="U74" t="n">
         <v>22.76666666666667</v>
@@ -9457,10 +9457,10 @@
         <v>21</v>
       </c>
       <c r="K103" t="n">
-        <v>29</v>
+        <v>18.4</v>
       </c>
       <c r="L103" t="n">
-        <v>138</v>
+        <v>88</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9490,7 +9490,7 @@
         <v>21</v>
       </c>
       <c r="T103" t="n">
-        <v>8</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U103" t="n">
         <v>24.53333333333333</v>
@@ -9803,10 +9803,10 @@
         <v>35</v>
       </c>
       <c r="K107" t="n">
-        <v>39.5</v>
+        <v>38</v>
       </c>
       <c r="L107" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="M107" t="inlineStr">
         <is>
@@ -9836,7 +9836,7 @@
         <v>41</v>
       </c>
       <c r="T107" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="U107" t="n">
         <v>37.06666666666667</v>
@@ -11211,10 +11211,10 @@
         <v>28</v>
       </c>
       <c r="K123" t="n">
-        <v>33.5</v>
+        <v>31.6</v>
       </c>
       <c r="L123" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="M123" t="inlineStr">
         <is>
@@ -11244,7 +11244,7 @@
         <v>28</v>
       </c>
       <c r="T123" t="n">
-        <v>5.5</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U123" t="n">
         <v>30.83333333333333</v>
@@ -11299,10 +11299,10 @@
         <v>21</v>
       </c>
       <c r="K124" t="n">
-        <v>23.7</v>
+        <v>20.4</v>
       </c>
       <c r="L124" t="n">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11332,7 +11332,7 @@
         <v>21</v>
       </c>
       <c r="T124" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U124" t="n">
         <v>21.43333333333333</v>
@@ -11387,10 +11387,10 @@
         <v>21</v>
       </c>
       <c r="K125" t="n">
-        <v>22.6</v>
+        <v>18.4</v>
       </c>
       <c r="L125" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="M125" t="inlineStr">
         <is>
@@ -11420,7 +11420,7 @@
         <v>21</v>
       </c>
       <c r="T125" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U125" t="n">
         <v>22.93333333333334</v>
@@ -11563,10 +11563,10 @@
         <v>35</v>
       </c>
       <c r="K127" t="n">
-        <v>30.5</v>
+        <v>35.4</v>
       </c>
       <c r="L127" t="n">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="M127" t="inlineStr">
         <is>
@@ -11596,7 +11596,7 @@
         <v>41</v>
       </c>
       <c r="T127" t="n">
-        <v>-4.5</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U127" t="n">
         <v>34.13333333333333</v>
@@ -11605,7 +11605,7 @@
         <v>3</v>
       </c>
       <c r="W127" t="n">
-        <v>36.32592592592593</v>
+        <v>36.32592592592592</v>
       </c>
       <c r="X127" t="n">
         <v>31.5</v>
@@ -11651,10 +11651,10 @@
         <v>21</v>
       </c>
       <c r="K128" t="n">
-        <v>23.2</v>
+        <v>20.3</v>
       </c>
       <c r="L128" t="n">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="M128" t="inlineStr">
         <is>
@@ -11684,10 +11684,10 @@
         <v>21</v>
       </c>
       <c r="T128" t="n">
-        <v>2.199999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="U128" t="n">
-        <v>22.36666666666666</v>
+        <v>22.36666666666667</v>
       </c>
       <c r="V128" t="n">
         <v>3</v>
@@ -11739,10 +11739,10 @@
         <v>28</v>
       </c>
       <c r="K129" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="L129" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="M129" t="inlineStr">
         <is>
@@ -11772,10 +11772,10 @@
         <v>28</v>
       </c>
       <c r="T129" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U129" t="n">
-        <v>25.36666666666666</v>
+        <v>25.36666666666667</v>
       </c>
       <c r="V129" t="n">
         <v>3</v>
@@ -11827,10 +11827,10 @@
         <v>35</v>
       </c>
       <c r="K130" t="n">
-        <v>33.9</v>
+        <v>30.7</v>
       </c>
       <c r="L130" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -11860,7 +11860,7 @@
         <v>41</v>
       </c>
       <c r="T130" t="n">
-        <v>-1.100000000000001</v>
+        <v>-4.300000000000001</v>
       </c>
       <c r="U130" t="n">
         <v>31.83333333333333</v>
@@ -11869,7 +11869,7 @@
         <v>3</v>
       </c>
       <c r="W130" t="n">
-        <v>34.15555555555556</v>
+        <v>34.15555555555555</v>
       </c>
       <c r="X130" t="n">
         <v>31.5</v>
@@ -12003,10 +12003,10 @@
         <v>21</v>
       </c>
       <c r="K132" t="n">
-        <v>24</v>
+        <v>20.4</v>
       </c>
       <c r="L132" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="M132" t="inlineStr">
         <is>
@@ -12036,7 +12036,7 @@
         <v>21</v>
       </c>
       <c r="T132" t="n">
-        <v>3</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U132" t="n">
         <v>22.16666666666667</v>
@@ -12091,10 +12091,10 @@
         <v>35</v>
       </c>
       <c r="K133" t="n">
-        <v>36.6</v>
+        <v>36.5</v>
       </c>
       <c r="L133" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M133" t="inlineStr">
         <is>
@@ -12124,7 +12124,7 @@
         <v>41</v>
       </c>
       <c r="T133" t="n">
-        <v>1.600000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="U133" t="n">
         <v>35.63333333333333</v>
@@ -12133,7 +12133,7 @@
         <v>3</v>
       </c>
       <c r="W133" t="n">
-        <v>41.38148148148148</v>
+        <v>41.38148148148147</v>
       </c>
       <c r="X133" t="n">
         <v>31.5</v>
@@ -12179,10 +12179,10 @@
         <v>28</v>
       </c>
       <c r="K134" t="n">
-        <v>33.1</v>
+        <v>29.9</v>
       </c>
       <c r="L134" t="n">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="M134" t="inlineStr">
         <is>
@@ -12212,7 +12212,7 @@
         <v>28</v>
       </c>
       <c r="T134" t="n">
-        <v>5.100000000000001</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U134" t="n">
         <v>28.06666666666666</v>
@@ -14371,10 +14371,10 @@
         <v>24</v>
       </c>
       <c r="K159" t="n">
-        <v>23.5</v>
+        <v>28</v>
       </c>
       <c r="L159" t="n">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="M159" t="inlineStr">
         <is>
@@ -14404,7 +14404,7 @@
         <v>28</v>
       </c>
       <c r="T159" t="n">
-        <v>-0.5</v>
+        <v>4</v>
       </c>
       <c r="U159" t="n">
         <v>25.5</v>
@@ -17179,10 +17179,10 @@
         <v>35</v>
       </c>
       <c r="K191" t="n">
-        <v>33.2</v>
+        <v>35.9</v>
       </c>
       <c r="L191" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="M191" t="inlineStr">
         <is>
@@ -17212,7 +17212,7 @@
         <v>41</v>
       </c>
       <c r="T191" t="n">
-        <v>-1.799999999999997</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U191" t="n">
         <v>35.16666666666666</v>
@@ -17441,10 +17441,10 @@
         <v>21</v>
       </c>
       <c r="K194" t="n">
-        <v>20.7</v>
+        <v>23</v>
       </c>
       <c r="L194" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="M194" t="inlineStr">
         <is>
@@ -17474,7 +17474,7 @@
         <v>21</v>
       </c>
       <c r="T194" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2</v>
       </c>
       <c r="U194" t="n">
         <v>21.5</v>
@@ -21217,10 +21217,10 @@
         <v>31</v>
       </c>
       <c r="K237" t="n">
-        <v>28.1</v>
+        <v>31.5</v>
       </c>
       <c r="L237" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="M237" t="inlineStr">
         <is>
@@ -21248,7 +21248,7 @@
       </c>
       <c r="S237" t="inlineStr"/>
       <c r="T237" t="n">
-        <v>-2.899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="U237" t="n">
         <v>30.6</v>
@@ -21433,7 +21433,7 @@
         <v>3</v>
       </c>
       <c r="W239" t="n">
-        <v>22.92222222222222</v>
+        <v>22.92222222222223</v>
       </c>
       <c r="X239" t="n">
         <v>20.5</v>
@@ -22265,10 +22265,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="L249" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22298,7 +22298,7 @@
         <v>21</v>
       </c>
       <c r="T249" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U249" t="n">
         <v>21.2</v>
@@ -24539,10 +24539,10 @@
         <v>28</v>
       </c>
       <c r="K275" t="n">
-        <v>27.5</v>
+        <v>28.7</v>
       </c>
       <c r="L275" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="M275" t="inlineStr">
         <is>
@@ -24572,7 +24572,7 @@
         <v>28</v>
       </c>
       <c r="T275" t="n">
-        <v>-0.5</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U275" t="n">
         <v>28.6</v>
@@ -24581,7 +24581,7 @@
         <v>3</v>
       </c>
       <c r="W275" t="n">
-        <v>32.9888888888889</v>
+        <v>32.98888888888889</v>
       </c>
       <c r="X275" t="n">
         <v>24.5</v>
@@ -25067,10 +25067,10 @@
         <v>28</v>
       </c>
       <c r="K281" t="n">
-        <v>28.3</v>
+        <v>27.2</v>
       </c>
       <c r="L281" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M281" t="inlineStr">
         <is>
@@ -25100,7 +25100,7 @@
         <v>28</v>
       </c>
       <c r="T281" t="n">
-        <v>0.3000000000000007</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U281" t="n">
         <v>27.4</v>
@@ -26733,10 +26733,10 @@
         <v>21</v>
       </c>
       <c r="K300" t="n">
-        <v>22.6</v>
+        <v>20.4</v>
       </c>
       <c r="L300" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="M300" t="inlineStr">
         <is>
@@ -26764,7 +26764,7 @@
       </c>
       <c r="S300" t="inlineStr"/>
       <c r="T300" t="n">
-        <v>1.600000000000001</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U300" t="n">
         <v>21.8</v>
@@ -28313,10 +28313,10 @@
         <v>24.5</v>
       </c>
       <c r="K318" t="n">
-        <v>23.5</v>
+        <v>30.6</v>
       </c>
       <c r="L318" t="n">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="M318" t="inlineStr">
         <is>
@@ -28346,7 +28346,7 @@
         <v>28</v>
       </c>
       <c r="T318" t="n">
-        <v>-1</v>
+        <v>6.100000000000001</v>
       </c>
       <c r="U318" t="n">
         <v>27.7</v>
@@ -28665,10 +28665,10 @@
         <v>24.5</v>
       </c>
       <c r="K322" t="n">
-        <v>33.3</v>
+        <v>21.5</v>
       </c>
       <c r="L322" t="n">
-        <v>136</v>
+        <v>88</v>
       </c>
       <c r="M322" t="inlineStr">
         <is>
@@ -28698,7 +28698,7 @@
         <v>28</v>
       </c>
       <c r="T322" t="n">
-        <v>8.799999999999997</v>
+        <v>-3</v>
       </c>
       <c r="U322" t="n">
         <v>29.5</v>
@@ -29545,10 +29545,10 @@
         <v>24.5</v>
       </c>
       <c r="K332" t="n">
-        <v>19.3</v>
+        <v>21.4</v>
       </c>
       <c r="L332" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="M332" t="inlineStr">
         <is>
@@ -29578,7 +29578,7 @@
         <v>28</v>
       </c>
       <c r="T332" t="n">
-        <v>-5.199999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="U332" t="n">
         <v>21.1</v>
@@ -31479,10 +31479,10 @@
         <v>24.5</v>
       </c>
       <c r="K354" t="n">
-        <v>28.8</v>
+        <v>24.3</v>
       </c>
       <c r="L354" t="n">
-        <v>118</v>
+        <v>99</v>
       </c>
       <c r="M354" t="inlineStr">
         <is>
@@ -31512,7 +31512,7 @@
         <v>28</v>
       </c>
       <c r="T354" t="n">
-        <v>4.300000000000001</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U354" t="n">
         <v>25.6</v>
@@ -32007,10 +32007,10 @@
         <v>24.5</v>
       </c>
       <c r="K360" t="n">
-        <v>22.7</v>
+        <v>29.1</v>
       </c>
       <c r="L360" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="M360" t="inlineStr">
         <is>
@@ -32040,7 +32040,7 @@
         <v>28</v>
       </c>
       <c r="T360" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="U360" t="n">
         <v>25.3</v>
@@ -32181,10 +32181,10 @@
         <v>24.5</v>
       </c>
       <c r="K362" t="n">
-        <v>28.6</v>
+        <v>25.1</v>
       </c>
       <c r="L362" t="n">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="M362" t="inlineStr">
         <is>
@@ -32214,7 +32214,7 @@
         <v>28</v>
       </c>
       <c r="T362" t="n">
-        <v>4.100000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U362" t="n">
         <v>25.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-06 18:03:06
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3333,10 +3333,10 @@
         <v>21</v>
       </c>
       <c r="K33" t="n">
-        <v>13.3</v>
+        <v>24.6</v>
       </c>
       <c r="L33" t="n">
-        <v>63</v>
+        <v>117</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
-        <v>-7.699999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U33" t="n">
         <v>20.13333333333334</v>
@@ -3593,10 +3593,10 @@
         <v>21</v>
       </c>
       <c r="K36" t="n">
-        <v>49.8</v>
+        <v>42.6</v>
       </c>
       <c r="L36" t="n">
-        <v>237</v>
+        <v>203</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3626,7 +3626,7 @@
         <v>21</v>
       </c>
       <c r="T36" t="n">
-        <v>28.8</v>
+        <v>21.6</v>
       </c>
       <c r="U36" t="n">
         <v>36.33333333333334</v>
@@ -3681,10 +3681,10 @@
         <v>28</v>
       </c>
       <c r="K37" t="n">
-        <v>26.8</v>
+        <v>27.7</v>
       </c>
       <c r="L37" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3714,7 +3714,7 @@
         <v>28</v>
       </c>
       <c r="T37" t="n">
-        <v>-1.199999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U37" t="n">
         <v>27.16666666666667</v>
@@ -4121,10 +4121,10 @@
         <v>28</v>
       </c>
       <c r="K42" t="n">
-        <v>28.1</v>
+        <v>28.9</v>
       </c>
       <c r="L42" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="M42" t="inlineStr">
         <is>
@@ -4154,7 +4154,7 @@
         <v>28</v>
       </c>
       <c r="T42" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U42" t="n">
         <v>28.03333333333333</v>
@@ -5039,7 +5039,7 @@
         <v>3</v>
       </c>
       <c r="W52" t="n">
-        <v>28.15555555555555</v>
+        <v>28.15555555555556</v>
       </c>
       <c r="X52" t="n">
         <v>24.5</v>
@@ -5523,10 +5523,10 @@
         <v>28</v>
       </c>
       <c r="K58" t="n">
-        <v>26.3</v>
+        <v>27.8</v>
       </c>
       <c r="L58" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -5556,7 +5556,7 @@
         <v>28</v>
       </c>
       <c r="T58" t="n">
-        <v>-1.699999999999999</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U58" t="n">
         <v>27.36666666666666</v>
@@ -9561,10 +9561,10 @@
         <v>24.5</v>
       </c>
       <c r="K104" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L104" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M104" t="inlineStr">
         <is>
@@ -9594,7 +9594,7 @@
         <v>28</v>
       </c>
       <c r="T104" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U104" t="n">
         <v>24.66666666666667</v>
@@ -10265,10 +10265,10 @@
         <v>24.5</v>
       </c>
       <c r="K112" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L112" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M112" t="inlineStr">
         <is>
@@ -10298,7 +10298,7 @@
         <v>28</v>
       </c>
       <c r="T112" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U112" t="n">
         <v>27.1</v>
@@ -12201,10 +12201,10 @@
         <v>24.5</v>
       </c>
       <c r="K134" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L134" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M134" t="inlineStr">
         <is>
@@ -12234,10 +12234,10 @@
         <v>28</v>
       </c>
       <c r="T134" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U134" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V134" t="n">
         <v>3</v>
@@ -13337,10 +13337,10 @@
         <v>21</v>
       </c>
       <c r="K147" t="n">
-        <v>18.2</v>
+        <v>19.8</v>
       </c>
       <c r="L147" t="n">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="M147" t="inlineStr">
         <is>
@@ -13370,7 +13370,7 @@
         <v>21</v>
       </c>
       <c r="T147" t="n">
-        <v>-2.800000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U147" t="n">
         <v>18.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-06 22:14:31
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2987,10 +2987,10 @@
         <v>24</v>
       </c>
       <c r="K29" t="n">
-        <v>15.8</v>
+        <v>21.6</v>
       </c>
       <c r="L29" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3020,7 +3020,7 @@
         <v>28</v>
       </c>
       <c r="T29" t="n">
-        <v>-8.199999999999999</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="U29" t="n">
         <v>19.2</v>
@@ -3247,10 +3247,10 @@
         <v>28</v>
       </c>
       <c r="K32" t="n">
-        <v>26.9</v>
+        <v>27.1</v>
       </c>
       <c r="L32" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3280,7 +3280,7 @@
         <v>28</v>
       </c>
       <c r="T32" t="n">
-        <v>-1.100000000000001</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U32" t="n">
         <v>27.23333333333333</v>
@@ -3853,10 +3853,10 @@
         <v>31</v>
       </c>
       <c r="K39" t="n">
-        <v>27.8</v>
+        <v>36.5</v>
       </c>
       <c r="L39" t="n">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="M39" t="inlineStr">
         <is>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="n">
-        <v>-3.199999999999999</v>
+        <v>5.5</v>
       </c>
       <c r="U39" t="n">
         <v>33.03333333333333</v>
@@ -5161,10 +5161,10 @@
         <v>31</v>
       </c>
       <c r="K54" t="n">
-        <v>30.5</v>
+        <v>38.5</v>
       </c>
       <c r="L54" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="M54" t="inlineStr">
         <is>
@@ -5192,7 +5192,7 @@
       </c>
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="n">
-        <v>-0.5</v>
+        <v>7.5</v>
       </c>
       <c r="U54" t="n">
         <v>35.86666666666667</v>
@@ -6605,7 +6605,7 @@
         <v>3</v>
       </c>
       <c r="W70" t="n">
-        <v>37.02962962962962</v>
+        <v>37.02962962962963</v>
       </c>
       <c r="X70" t="n">
         <v>31.5</v>
@@ -6781,7 +6781,7 @@
         <v>3</v>
       </c>
       <c r="W72" t="n">
-        <v>38.42962962962962</v>
+        <v>38.42962962962963</v>
       </c>
       <c r="X72" t="n">
         <v>31.5</v>
@@ -7003,10 +7003,10 @@
         <v>35</v>
       </c>
       <c r="K75" t="n">
-        <v>40.8</v>
+        <v>33.5</v>
       </c>
       <c r="L75" t="n">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="M75" t="inlineStr">
         <is>
@@ -7036,10 +7036,10 @@
         <v>41</v>
       </c>
       <c r="T75" t="n">
-        <v>5.799999999999997</v>
+        <v>-1.5</v>
       </c>
       <c r="U75" t="n">
-        <v>37.56666666666666</v>
+        <v>37.56666666666667</v>
       </c>
       <c r="V75" t="n">
         <v>3</v>
@@ -9457,10 +9457,10 @@
         <v>21</v>
       </c>
       <c r="K103" t="n">
-        <v>29</v>
+        <v>18.4</v>
       </c>
       <c r="L103" t="n">
-        <v>138</v>
+        <v>88</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9490,7 +9490,7 @@
         <v>21</v>
       </c>
       <c r="T103" t="n">
-        <v>8</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U103" t="n">
         <v>24.53333333333333</v>
@@ -9979,10 +9979,10 @@
         <v>35</v>
       </c>
       <c r="K109" t="n">
-        <v>34.1</v>
+        <v>39.8</v>
       </c>
       <c r="L109" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="M109" t="inlineStr">
         <is>
@@ -10012,7 +10012,7 @@
         <v>41</v>
       </c>
       <c r="T109" t="n">
-        <v>-0.8999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="U109" t="n">
         <v>36.83333333333334</v>
@@ -10507,10 +10507,10 @@
         <v>35</v>
       </c>
       <c r="K115" t="n">
-        <v>26.3</v>
+        <v>22.5</v>
       </c>
       <c r="L115" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         <v>41</v>
       </c>
       <c r="T115" t="n">
-        <v>-8.699999999999999</v>
+        <v>-12.5</v>
       </c>
       <c r="U115" t="n">
         <v>25.5</v>
@@ -13057,10 +13057,10 @@
         <v>35</v>
       </c>
       <c r="K144" t="n">
-        <v>37.4</v>
+        <v>41.3</v>
       </c>
       <c r="L144" t="n">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="M144" t="inlineStr">
         <is>
@@ -13090,10 +13090,10 @@
         <v>41</v>
       </c>
       <c r="T144" t="n">
-        <v>2.399999999999999</v>
+        <v>6.299999999999997</v>
       </c>
       <c r="U144" t="n">
-        <v>37.06666666666667</v>
+        <v>37.06666666666666</v>
       </c>
       <c r="V144" t="n">
         <v>3</v>
@@ -13495,10 +13495,10 @@
         <v>35</v>
       </c>
       <c r="K149" t="n">
-        <v>34.4</v>
+        <v>36.9</v>
       </c>
       <c r="L149" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="M149" t="inlineStr">
         <is>
@@ -13528,7 +13528,7 @@
         <v>41</v>
       </c>
       <c r="T149" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U149" t="n">
         <v>35.53333333333333</v>
@@ -14635,10 +14635,10 @@
         <v>28</v>
       </c>
       <c r="K162" t="n">
-        <v>31.6</v>
+        <v>29.4</v>
       </c>
       <c r="L162" t="n">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="M162" t="inlineStr">
         <is>
@@ -14668,16 +14668,16 @@
         <v>28</v>
       </c>
       <c r="T162" t="n">
-        <v>3.600000000000001</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="U162" t="n">
-        <v>28.43333333333334</v>
+        <v>28.43333333333333</v>
       </c>
       <c r="V162" t="n">
         <v>3</v>
       </c>
       <c r="W162" t="n">
-        <v>30.78888888888889</v>
+        <v>30.78888888888888</v>
       </c>
       <c r="X162" t="n">
         <v>24.5</v>
@@ -16213,10 +16213,10 @@
         <v>28</v>
       </c>
       <c r="K180" t="n">
-        <v>23.6</v>
+        <v>29</v>
       </c>
       <c r="L180" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="M180" t="inlineStr">
         <is>
@@ -16246,7 +16246,7 @@
         <v>28</v>
       </c>
       <c r="T180" t="n">
-        <v>-4.399999999999999</v>
+        <v>1</v>
       </c>
       <c r="U180" t="n">
         <v>25.33333333333333</v>
@@ -17005,10 +17005,10 @@
         <v>28</v>
       </c>
       <c r="K189" t="n">
-        <v>25.7</v>
+        <v>27.9</v>
       </c>
       <c r="L189" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="M189" t="inlineStr">
         <is>
@@ -17038,7 +17038,7 @@
         <v>28</v>
       </c>
       <c r="T189" t="n">
-        <v>-2.300000000000001</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U189" t="n">
         <v>26.76666666666667</v>
@@ -17093,10 +17093,10 @@
         <v>35</v>
       </c>
       <c r="K190" t="n">
-        <v>43.4</v>
+        <v>26.1</v>
       </c>
       <c r="L190" t="n">
-        <v>124</v>
+        <v>74</v>
       </c>
       <c r="M190" t="inlineStr">
         <is>
@@ -17126,7 +17126,7 @@
         <v>41</v>
       </c>
       <c r="T190" t="n">
-        <v>8.399999999999999</v>
+        <v>-8.899999999999999</v>
       </c>
       <c r="U190" t="n">
         <v>33.26666666666667</v>
@@ -19549,10 +19549,10 @@
         <v>28</v>
       </c>
       <c r="K218" t="n">
-        <v>28.8</v>
+        <v>28.5</v>
       </c>
       <c r="L218" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M218" t="inlineStr">
         <is>
@@ -19582,7 +19582,7 @@
         <v>28</v>
       </c>
       <c r="T218" t="n">
-        <v>0.8000000000000007</v>
+        <v>0.5</v>
       </c>
       <c r="U218" t="n">
         <v>28.33333333333333</v>
@@ -19637,10 +19637,10 @@
         <v>28</v>
       </c>
       <c r="K219" t="n">
-        <v>28.7</v>
+        <v>27.7</v>
       </c>
       <c r="L219" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M219" t="inlineStr">
         <is>
@@ -19670,7 +19670,7 @@
         <v>28</v>
       </c>
       <c r="T219" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U219" t="n">
         <v>28.13333333333334</v>
@@ -19855,7 +19855,7 @@
         <v>3</v>
       </c>
       <c r="W221" t="n">
-        <v>19.75555555555555</v>
+        <v>19.75555555555556</v>
       </c>
       <c r="X221" t="n">
         <v>17.5</v>
@@ -20605,10 +20605,10 @@
         <v>21</v>
       </c>
       <c r="K230" t="n">
-        <v>21.7</v>
+        <v>22.9</v>
       </c>
       <c r="L230" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="M230" t="inlineStr">
         <is>
@@ -20638,7 +20638,7 @@
         <v>21</v>
       </c>
       <c r="T230" t="n">
-        <v>0.6999999999999993</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U230" t="n">
         <v>21.83333333333333</v>
@@ -20867,10 +20867,10 @@
         <v>28</v>
       </c>
       <c r="K233" t="n">
-        <v>26.1</v>
+        <v>24.5</v>
       </c>
       <c r="L233" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="M233" t="inlineStr">
         <is>
@@ -20900,7 +20900,7 @@
         <v>28</v>
       </c>
       <c r="T233" t="n">
-        <v>-1.899999999999999</v>
+        <v>-3.5</v>
       </c>
       <c r="U233" t="n">
         <v>25.53333333333333</v>
@@ -21129,10 +21129,10 @@
         <v>42</v>
       </c>
       <c r="K236" t="n">
-        <v>31.1</v>
+        <v>51.6</v>
       </c>
       <c r="L236" t="n">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="M236" t="inlineStr">
         <is>
@@ -21162,7 +21162,7 @@
         <v>48</v>
       </c>
       <c r="T236" t="n">
-        <v>-10.9</v>
+        <v>9.600000000000001</v>
       </c>
       <c r="U236" t="n">
         <v>43.9</v>
@@ -21433,7 +21433,7 @@
         <v>3</v>
       </c>
       <c r="W239" t="n">
-        <v>22.92222222222223</v>
+        <v>22.92222222222222</v>
       </c>
       <c r="X239" t="n">
         <v>20.5</v>
@@ -21653,10 +21653,10 @@
         <v>42</v>
       </c>
       <c r="K242" t="n">
-        <v>15.9</v>
+        <v>50.4</v>
       </c>
       <c r="L242" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="M242" t="inlineStr">
         <is>
@@ -21686,7 +21686,7 @@
         <v>48</v>
       </c>
       <c r="T242" t="n">
-        <v>-26.1</v>
+        <v>8.399999999999999</v>
       </c>
       <c r="U242" t="n">
         <v>39.6</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-07 01:26:24
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -606,11 +606,11 @@
         </is>
       </c>
       <c r="P2" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
@@ -694,11 +694,11 @@
         </is>
       </c>
       <c r="P3" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R3" s="2" t="n">
@@ -784,11 +784,11 @@
         </is>
       </c>
       <c r="P4" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
@@ -872,11 +872,11 @@
         </is>
       </c>
       <c r="P5" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R5" s="2" t="n">
@@ -962,11 +962,11 @@
         </is>
       </c>
       <c r="P6" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
@@ -1052,11 +1052,11 @@
         </is>
       </c>
       <c r="P7" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R7" s="2" t="n">
@@ -1142,11 +1142,11 @@
         </is>
       </c>
       <c r="P8" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
@@ -1232,11 +1232,11 @@
         </is>
       </c>
       <c r="P9" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R9" s="2" t="n">
@@ -1320,11 +1320,11 @@
         </is>
       </c>
       <c r="P10" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
@@ -1408,11 +1408,11 @@
         </is>
       </c>
       <c r="P11" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R11" s="2" t="n">
@@ -1496,11 +1496,11 @@
         </is>
       </c>
       <c r="P12" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
@@ -1584,11 +1584,11 @@
         </is>
       </c>
       <c r="P13" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R13" s="2" t="n">
@@ -1674,11 +1674,11 @@
         </is>
       </c>
       <c r="P14" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
@@ -1762,11 +1762,11 @@
         </is>
       </c>
       <c r="P15" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R15" s="2" t="n">
@@ -1850,11 +1850,11 @@
         </is>
       </c>
       <c r="P16" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
@@ -1938,11 +1938,11 @@
         </is>
       </c>
       <c r="P17" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R17" s="2" t="n">
@@ -2028,11 +2028,11 @@
         </is>
       </c>
       <c r="P18" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
@@ -2116,11 +2116,11 @@
         </is>
       </c>
       <c r="P19" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R19" s="2" t="n">
@@ -2204,11 +2204,11 @@
         </is>
       </c>
       <c r="P20" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
@@ -2294,11 +2294,11 @@
         </is>
       </c>
       <c r="P21" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R21" s="2" t="n">
@@ -2384,11 +2384,11 @@
         </is>
       </c>
       <c r="P22" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
@@ -2474,11 +2474,11 @@
         </is>
       </c>
       <c r="P23" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R23" s="2" t="n">
@@ -2564,11 +2564,11 @@
         </is>
       </c>
       <c r="P24" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
@@ -2654,11 +2654,11 @@
         </is>
       </c>
       <c r="P25" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R25" s="2" t="n">
@@ -2742,11 +2742,11 @@
         </is>
       </c>
       <c r="P26" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
@@ -2830,11 +2830,11 @@
         </is>
       </c>
       <c r="P27" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R27" s="2" t="n">
@@ -2918,11 +2918,11 @@
         </is>
       </c>
       <c r="P28" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
@@ -3004,11 +3004,11 @@
         </is>
       </c>
       <c r="P29" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R29" s="2" t="n">
@@ -3092,11 +3092,11 @@
         </is>
       </c>
       <c r="P30" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
@@ -3180,11 +3180,11 @@
         </is>
       </c>
       <c r="P31" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R31" s="2" t="n">
@@ -3266,11 +3266,11 @@
         </is>
       </c>
       <c r="P32" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
@@ -3352,11 +3352,11 @@
         </is>
       </c>
       <c r="P33" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R33" s="2" t="n">
@@ -3438,11 +3438,11 @@
         </is>
       </c>
       <c r="P34" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
@@ -3524,11 +3524,11 @@
         </is>
       </c>
       <c r="P35" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R35" s="2" t="n">
@@ -3612,11 +3612,11 @@
         </is>
       </c>
       <c r="P36" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -3700,11 +3700,11 @@
         </is>
       </c>
       <c r="P37" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R37" s="2" t="n">
@@ -3788,11 +3788,11 @@
         </is>
       </c>
       <c r="P38" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R38" s="2" t="n">
@@ -3876,11 +3876,11 @@
         </is>
       </c>
       <c r="P39" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R39" s="2" t="n">
@@ -3964,11 +3964,11 @@
         </is>
       </c>
       <c r="P40" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R40" s="2" t="n">
@@ -4052,11 +4052,11 @@
         </is>
       </c>
       <c r="P41" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R41" s="2" t="n">
@@ -4140,11 +4140,11 @@
         </is>
       </c>
       <c r="P42" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R42" s="2" t="n">
@@ -4228,11 +4228,11 @@
         </is>
       </c>
       <c r="P43" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R43" s="2" t="n">
@@ -4316,11 +4316,11 @@
         </is>
       </c>
       <c r="P44" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R44" s="2" t="n">
@@ -4404,11 +4404,11 @@
         </is>
       </c>
       <c r="P45" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R45" s="2" t="n">
@@ -4492,11 +4492,11 @@
         </is>
       </c>
       <c r="P46" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R46" s="2" t="n">
@@ -4580,11 +4580,11 @@
         </is>
       </c>
       <c r="P47" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R47" s="2" t="n">
@@ -4666,11 +4666,11 @@
         </is>
       </c>
       <c r="P48" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R48" s="2" t="n">
@@ -4754,11 +4754,11 @@
         </is>
       </c>
       <c r="P49" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R49" s="2" t="n">
@@ -4821,10 +4821,10 @@
         <v>28</v>
       </c>
       <c r="K50" t="n">
-        <v>31.4</v>
+        <v>21.8</v>
       </c>
       <c r="L50" t="n">
-        <v>112</v>
+        <v>78</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
@@ -4840,11 +4840,11 @@
         </is>
       </c>
       <c r="P50" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R50" s="2" t="n">
@@ -4854,7 +4854,7 @@
         <v>28</v>
       </c>
       <c r="T50" t="n">
-        <v>3.399999999999999</v>
+        <v>-6.199999999999999</v>
       </c>
       <c r="U50" t="n">
         <v>28.2</v>
@@ -4928,11 +4928,11 @@
         </is>
       </c>
       <c r="P51" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R51" s="2" t="n">
@@ -5016,11 +5016,11 @@
         </is>
       </c>
       <c r="P52" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R52" s="2" t="n">
@@ -5104,11 +5104,11 @@
         </is>
       </c>
       <c r="P53" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R53" s="2" t="n">
@@ -5192,11 +5192,11 @@
         </is>
       </c>
       <c r="P54" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R54" s="2" t="n">
@@ -5278,11 +5278,11 @@
         </is>
       </c>
       <c r="P55" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R55" s="2" t="n">
@@ -5366,11 +5366,11 @@
         </is>
       </c>
       <c r="P56" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R56" s="2" t="n">
@@ -5454,11 +5454,11 @@
         </is>
       </c>
       <c r="P57" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R57" s="2" t="n">
@@ -5542,11 +5542,11 @@
         </is>
       </c>
       <c r="P58" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R58" s="2" t="n">
@@ -5630,11 +5630,11 @@
         </is>
       </c>
       <c r="P59" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R59" s="2" t="n">
@@ -5718,11 +5718,11 @@
         </is>
       </c>
       <c r="P60" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R60" s="2" t="n">
@@ -5806,11 +5806,11 @@
         </is>
       </c>
       <c r="P61" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R61" s="2" t="n">
@@ -5894,11 +5894,11 @@
         </is>
       </c>
       <c r="P62" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R62" s="2" t="n">
@@ -5982,11 +5982,11 @@
         </is>
       </c>
       <c r="P63" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R63" s="2" t="n">
@@ -6070,11 +6070,11 @@
         </is>
       </c>
       <c r="P64" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R64" s="2" t="n">
@@ -6158,11 +6158,11 @@
         </is>
       </c>
       <c r="P65" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R65" s="2" t="n">
@@ -6246,11 +6246,11 @@
         </is>
       </c>
       <c r="P66" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R66" s="2" t="n">
@@ -6334,11 +6334,11 @@
         </is>
       </c>
       <c r="P67" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R67" s="2" t="n">
@@ -6422,11 +6422,11 @@
         </is>
       </c>
       <c r="P68" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R68" s="2" t="n">
@@ -6510,11 +6510,11 @@
         </is>
       </c>
       <c r="P69" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R69" s="2" t="n">
@@ -6598,11 +6598,11 @@
         </is>
       </c>
       <c r="P70" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R70" s="2" t="n">
@@ -6682,11 +6682,11 @@
         </is>
       </c>
       <c r="P71" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R71" s="2" t="n">
@@ -6770,11 +6770,11 @@
         </is>
       </c>
       <c r="P72" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R72" s="2" t="n">
@@ -6858,11 +6858,11 @@
         </is>
       </c>
       <c r="P73" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R73" s="2" t="n">
@@ -6946,11 +6946,11 @@
         </is>
       </c>
       <c r="P74" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R74" s="2" t="n">
@@ -7034,11 +7034,11 @@
         </is>
       </c>
       <c r="P75" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R75" s="2" t="n">
@@ -7122,11 +7122,11 @@
         </is>
       </c>
       <c r="P76" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R76" s="2" t="n">
@@ -7210,11 +7210,11 @@
         </is>
       </c>
       <c r="P77" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R77" s="2" t="n">
@@ -7296,11 +7296,11 @@
         </is>
       </c>
       <c r="P78" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R78" s="2" t="n">
@@ -7384,11 +7384,11 @@
         </is>
       </c>
       <c r="P79" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R79" s="2" t="n">
@@ -7472,11 +7472,11 @@
         </is>
       </c>
       <c r="P80" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R80" s="2" t="n">
@@ -7560,11 +7560,11 @@
         </is>
       </c>
       <c r="P81" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R81" s="2" t="n">
@@ -7646,11 +7646,11 @@
         </is>
       </c>
       <c r="P82" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R82" s="2" t="n">
@@ -7734,11 +7734,11 @@
         </is>
       </c>
       <c r="P83" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R83" s="2" t="n">
@@ -7822,11 +7822,11 @@
         </is>
       </c>
       <c r="P84" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R84" s="2" t="n">
@@ -7910,11 +7910,11 @@
         </is>
       </c>
       <c r="P85" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R85" s="2" t="n">
@@ -7998,11 +7998,11 @@
         </is>
       </c>
       <c r="P86" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R86" s="2" t="n">
@@ -8086,11 +8086,11 @@
         </is>
       </c>
       <c r="P87" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R87" s="2" t="n">
@@ -8174,11 +8174,11 @@
         </is>
       </c>
       <c r="P88" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R88" s="2" t="n">
@@ -8262,11 +8262,11 @@
         </is>
       </c>
       <c r="P89" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R89" s="2" t="n">
@@ -8350,11 +8350,11 @@
         </is>
       </c>
       <c r="P90" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R90" s="2" t="n">
@@ -8438,11 +8438,11 @@
         </is>
       </c>
       <c r="P91" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R91" s="2" t="n">
@@ -8524,11 +8524,11 @@
         </is>
       </c>
       <c r="P92" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R92" s="2" t="n">
@@ -8612,11 +8612,11 @@
         </is>
       </c>
       <c r="P93" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R93" s="2" t="n">
@@ -8700,11 +8700,11 @@
         </is>
       </c>
       <c r="P94" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R94" s="2" t="n">
@@ -8788,11 +8788,11 @@
         </is>
       </c>
       <c r="P95" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R95" s="2" t="n">
@@ -8876,11 +8876,11 @@
         </is>
       </c>
       <c r="P96" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R96" s="2" t="n">
@@ -8964,11 +8964,11 @@
         </is>
       </c>
       <c r="P97" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R97" s="2" t="n">
@@ -9052,11 +9052,11 @@
         </is>
       </c>
       <c r="P98" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R98" s="2" t="n">
@@ -9140,11 +9140,11 @@
         </is>
       </c>
       <c r="P99" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R99" s="2" t="n">
@@ -9228,11 +9228,11 @@
         </is>
       </c>
       <c r="P100" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R100" s="2" t="n">
@@ -9316,11 +9316,11 @@
         </is>
       </c>
       <c r="P101" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R101" s="2" t="n">
@@ -9404,11 +9404,11 @@
         </is>
       </c>
       <c r="P102" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R102" s="2" t="n">
@@ -9492,11 +9492,11 @@
         </is>
       </c>
       <c r="P103" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R103" s="2" t="n">
@@ -9580,11 +9580,11 @@
         </is>
       </c>
       <c r="P104" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R104" s="2" t="n">
@@ -9668,11 +9668,11 @@
         </is>
       </c>
       <c r="P105" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R105" s="2" t="n">
@@ -9756,11 +9756,11 @@
         </is>
       </c>
       <c r="P106" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R106" s="2" t="n">
@@ -9844,11 +9844,11 @@
         </is>
       </c>
       <c r="P107" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R107" s="2" t="n">
@@ -9932,11 +9932,11 @@
         </is>
       </c>
       <c r="P108" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R108" s="2" t="n">
@@ -10020,11 +10020,11 @@
         </is>
       </c>
       <c r="P109" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R109" s="2" t="n">
@@ -10108,11 +10108,11 @@
         </is>
       </c>
       <c r="P110" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R110" s="2" t="n">
@@ -10196,11 +10196,11 @@
         </is>
       </c>
       <c r="P111" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R111" s="2" t="n">
@@ -10284,11 +10284,11 @@
         </is>
       </c>
       <c r="P112" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R112" s="2" t="n">
@@ -10372,11 +10372,11 @@
         </is>
       </c>
       <c r="P113" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R113" s="2" t="n">
@@ -10460,11 +10460,11 @@
         </is>
       </c>
       <c r="P114" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R114" s="2" t="n">
@@ -10548,11 +10548,11 @@
         </is>
       </c>
       <c r="P115" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R115" s="2" t="n">
@@ -10636,11 +10636,11 @@
         </is>
       </c>
       <c r="P116" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R116" s="2" t="n">
@@ -10724,11 +10724,11 @@
         </is>
       </c>
       <c r="P117" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R117" s="2" t="n">
@@ -10793,10 +10793,10 @@
         <v>24.5</v>
       </c>
       <c r="K118" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="L118" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -10812,11 +10812,11 @@
         </is>
       </c>
       <c r="P118" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R118" s="2" t="n">
@@ -10826,7 +10826,7 @@
         <v>28</v>
       </c>
       <c r="T118" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U118" t="n">
         <v>35.8</v>
@@ -10900,11 +10900,11 @@
         </is>
       </c>
       <c r="P119" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R119" s="2" t="n">
@@ -10988,11 +10988,11 @@
         </is>
       </c>
       <c r="P120" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R120" s="2" t="n">
@@ -11076,11 +11076,11 @@
         </is>
       </c>
       <c r="P121" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R121" s="2" t="n">
@@ -11164,11 +11164,11 @@
         </is>
       </c>
       <c r="P122" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R122" s="2" t="n">
@@ -11252,11 +11252,11 @@
         </is>
       </c>
       <c r="P123" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R123" s="2" t="n">
@@ -11340,11 +11340,11 @@
         </is>
       </c>
       <c r="P124" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R124" s="2" t="n">
@@ -11428,11 +11428,11 @@
         </is>
       </c>
       <c r="P125" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R125" s="2" t="n">
@@ -11516,11 +11516,11 @@
         </is>
       </c>
       <c r="P126" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R126" s="2" t="n">
@@ -11604,11 +11604,11 @@
         </is>
       </c>
       <c r="P127" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R127" s="2" t="n">
@@ -11692,11 +11692,11 @@
         </is>
       </c>
       <c r="P128" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R128" s="2" t="n">
@@ -11780,11 +11780,11 @@
         </is>
       </c>
       <c r="P129" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R129" s="2" t="n">
@@ -11868,11 +11868,11 @@
         </is>
       </c>
       <c r="P130" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R130" s="2" t="n">
@@ -11956,11 +11956,11 @@
         </is>
       </c>
       <c r="P131" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R131" s="2" t="n">
@@ -12044,11 +12044,11 @@
         </is>
       </c>
       <c r="P132" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R132" s="2" t="n">
@@ -12132,11 +12132,11 @@
         </is>
       </c>
       <c r="P133" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R133" s="2" t="n">
@@ -12220,11 +12220,11 @@
         </is>
       </c>
       <c r="P134" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R134" s="2" t="n">
@@ -12306,11 +12306,11 @@
         </is>
       </c>
       <c r="P135" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R135" s="2" t="n">
@@ -12394,11 +12394,11 @@
         </is>
       </c>
       <c r="P136" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R136" s="2" t="n">
@@ -12482,11 +12482,11 @@
         </is>
       </c>
       <c r="P137" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R137" s="2" t="n">
@@ -12570,11 +12570,11 @@
         </is>
       </c>
       <c r="P138" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R138" s="2" t="n">
@@ -12658,11 +12658,11 @@
         </is>
       </c>
       <c r="P139" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R139" s="2" t="n">
@@ -12746,11 +12746,11 @@
         </is>
       </c>
       <c r="P140" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R140" s="2" t="n">
@@ -12834,11 +12834,11 @@
         </is>
       </c>
       <c r="P141" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R141" s="2" t="n">
@@ -12920,11 +12920,11 @@
         </is>
       </c>
       <c r="P142" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R142" s="2" t="n">
@@ -13008,11 +13008,11 @@
         </is>
       </c>
       <c r="P143" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R143" s="2" t="n">
@@ -13096,11 +13096,11 @@
         </is>
       </c>
       <c r="P144" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R144" s="2" t="n">
@@ -13182,11 +13182,11 @@
         </is>
       </c>
       <c r="P145" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R145" s="2" t="n">
@@ -13270,11 +13270,11 @@
         </is>
       </c>
       <c r="P146" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R146" s="2" t="n">
@@ -13356,11 +13356,11 @@
         </is>
       </c>
       <c r="P147" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R147" s="2" t="n">

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-07 08:14:00
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -23313,10 +23313,10 @@
         <v>28</v>
       </c>
       <c r="K261" t="n">
-        <v>28.9</v>
+        <v>28.1</v>
       </c>
       <c r="L261" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="M261" t="inlineStr">
         <is>
@@ -23346,7 +23346,7 @@
         <v>28</v>
       </c>
       <c r="T261" t="n">
-        <v>0.8999999999999986</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U261" t="n">
         <v>28.03333333333333</v>
@@ -24365,10 +24365,10 @@
         <v>21</v>
       </c>
       <c r="K273" t="n">
-        <v>16.3</v>
+        <v>26.4</v>
       </c>
       <c r="L273" t="n">
-        <v>78</v>
+        <v>126</v>
       </c>
       <c r="M273" t="inlineStr">
         <is>
@@ -24398,7 +24398,7 @@
         <v>21</v>
       </c>
       <c r="T273" t="n">
-        <v>-4.699999999999999</v>
+        <v>5.399999999999999</v>
       </c>
       <c r="U273" t="n">
         <v>22.9</v>
@@ -27611,10 +27611,10 @@
         <v>21</v>
       </c>
       <c r="K310" t="n">
-        <v>20.6</v>
+        <v>26.5</v>
       </c>
       <c r="L310" t="n">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="M310" t="inlineStr">
         <is>
@@ -27644,7 +27644,7 @@
         <v>21</v>
       </c>
       <c r="T310" t="n">
-        <v>-0.3999999999999986</v>
+        <v>5.5</v>
       </c>
       <c r="U310" t="n">
         <v>23.9</v>
@@ -27697,10 +27697,10 @@
         <v>24.5</v>
       </c>
       <c r="K311" t="n">
-        <v>25</v>
+        <v>22.6</v>
       </c>
       <c r="L311" t="n">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="M311" t="inlineStr">
         <is>
@@ -27730,7 +27730,7 @@
         <v>28</v>
       </c>
       <c r="T311" t="n">
-        <v>0.5</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="U311" t="n">
         <v>24.8</v>
@@ -28577,10 +28577,10 @@
         <v>24.5</v>
       </c>
       <c r="K321" t="n">
-        <v>23.7</v>
+        <v>28.3</v>
       </c>
       <c r="L321" t="n">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="M321" t="inlineStr">
         <is>
@@ -28610,7 +28610,7 @@
         <v>28</v>
       </c>
       <c r="T321" t="n">
-        <v>-0.8000000000000007</v>
+        <v>3.800000000000001</v>
       </c>
       <c r="U321" t="n">
         <v>25.7</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L323" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L331" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -29897,10 +29897,10 @@
         <v>24.5</v>
       </c>
       <c r="K336" t="n">
-        <v>24.3</v>
+        <v>24.4</v>
       </c>
       <c r="L336" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M336" t="inlineStr">
         <is>
@@ -29930,7 +29930,7 @@
         <v>28</v>
       </c>
       <c r="T336" t="n">
-        <v>-0.1999999999999993</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U336" t="n">
         <v>24.26666666666667</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L353" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-07 18:33:12
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -1253,7 +1253,7 @@
         <v>3</v>
       </c>
       <c r="W9" t="n">
-        <v>36.26666666666667</v>
+        <v>33.6</v>
       </c>
       <c r="X9" t="n">
         <v>28</v>
@@ -2227,7 +2227,7 @@
         <v>3</v>
       </c>
       <c r="W20" t="n">
-        <v>57.06666666666667</v>
+        <v>55.38518518518518</v>
       </c>
       <c r="X20" t="n">
         <v>44.1</v>
@@ -3247,10 +3247,10 @@
         <v>28</v>
       </c>
       <c r="K32" t="n">
-        <v>27.1</v>
+        <v>26.9</v>
       </c>
       <c r="L32" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3280,7 +3280,7 @@
         <v>28</v>
       </c>
       <c r="T32" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U32" t="n">
         <v>27.23333333333333</v>
@@ -3421,10 +3421,10 @@
         <v>31</v>
       </c>
       <c r="K34" t="n">
-        <v>36</v>
+        <v>30.9</v>
       </c>
       <c r="L34" t="n">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="n">
-        <v>5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U34" t="n">
         <v>33.03333333333333</v>
@@ -3507,10 +3507,10 @@
         <v>31</v>
       </c>
       <c r="K35" t="n">
-        <v>31.6</v>
+        <v>29.8</v>
       </c>
       <c r="L35" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3538,7 +3538,7 @@
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="n">
-        <v>0.6000000000000014</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U35" t="n">
         <v>30.4</v>
@@ -4113,10 +4113,10 @@
         <v>24</v>
       </c>
       <c r="K42" t="n">
-        <v>16.2</v>
+        <v>15.7</v>
       </c>
       <c r="L42" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="M42" t="inlineStr">
         <is>
@@ -4146,7 +4146,7 @@
         <v>28</v>
       </c>
       <c r="T42" t="n">
-        <v>-7.800000000000001</v>
+        <v>-8.300000000000001</v>
       </c>
       <c r="U42" t="n">
         <v>16.5</v>
@@ -5423,10 +5423,10 @@
         <v>31</v>
       </c>
       <c r="K57" t="n">
-        <v>18.8</v>
+        <v>39.3</v>
       </c>
       <c r="L57" t="n">
-        <v>61</v>
+        <v>127</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="n">
-        <v>-12.2</v>
+        <v>8.299999999999997</v>
       </c>
       <c r="U57" t="n">
         <v>31.73333333333333</v>
@@ -5509,10 +5509,10 @@
         <v>24</v>
       </c>
       <c r="K58" t="n">
-        <v>20.8</v>
+        <v>21.4</v>
       </c>
       <c r="L58" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -5542,7 +5542,7 @@
         <v>28</v>
       </c>
       <c r="T58" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U58" t="n">
         <v>21.53333333333333</v>
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L77" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7353,7 +7353,7 @@
         <v>28</v>
       </c>
       <c r="K79" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="L79" t="n">
         <v>88</v>
@@ -7386,7 +7386,7 @@
         <v>28</v>
       </c>
       <c r="T79" t="n">
-        <v>-3.199999999999999</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="U79" t="n">
         <v>25.13333333333334</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L81" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -7615,10 +7615,10 @@
         <v>21</v>
       </c>
       <c r="K82" t="n">
-        <v>26.4</v>
+        <v>17.9</v>
       </c>
       <c r="L82" t="n">
-        <v>126</v>
+        <v>85</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
         <v>21</v>
       </c>
       <c r="T82" t="n">
-        <v>5.399999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="U82" t="n">
         <v>21.3</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L88" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L93" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -12969,10 +12969,10 @@
         <v>35</v>
       </c>
       <c r="K143" t="n">
-        <v>39.9</v>
+        <v>29.7</v>
       </c>
       <c r="L143" t="n">
-        <v>114</v>
+        <v>85</v>
       </c>
       <c r="M143" t="inlineStr">
         <is>
@@ -13002,7 +13002,7 @@
         <v>41</v>
       </c>
       <c r="T143" t="n">
-        <v>4.899999999999999</v>
+        <v>-5.300000000000001</v>
       </c>
       <c r="U143" t="n">
         <v>37</v>
@@ -14897,10 +14897,10 @@
         <v>21</v>
       </c>
       <c r="K165" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="L165" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="M165" t="inlineStr">
         <is>
@@ -14930,7 +14930,7 @@
         <v>21</v>
       </c>
       <c r="T165" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U165" t="n">
         <v>22.96666666666667</v>
@@ -16477,10 +16477,10 @@
         <v>28</v>
       </c>
       <c r="K183" t="n">
-        <v>36.4</v>
+        <v>40.2</v>
       </c>
       <c r="L183" t="n">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="M183" t="inlineStr">
         <is>
@@ -16510,7 +16510,7 @@
         <v>28</v>
       </c>
       <c r="T183" t="n">
-        <v>8.399999999999999</v>
+        <v>12.2</v>
       </c>
       <c r="U183" t="n">
         <v>33.36666666666667</v>
@@ -17093,10 +17093,10 @@
         <v>35</v>
       </c>
       <c r="K190" t="n">
-        <v>26.1</v>
+        <v>43.4</v>
       </c>
       <c r="L190" t="n">
-        <v>74</v>
+        <v>124</v>
       </c>
       <c r="M190" t="inlineStr">
         <is>
@@ -17126,7 +17126,7 @@
         <v>41</v>
       </c>
       <c r="T190" t="n">
-        <v>-8.899999999999999</v>
+        <v>8.399999999999999</v>
       </c>
       <c r="U190" t="n">
         <v>33.26666666666667</v>
@@ -18319,10 +18319,10 @@
         <v>21</v>
       </c>
       <c r="K204" t="n">
-        <v>23.1</v>
+        <v>20.7</v>
       </c>
       <c r="L204" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="M204" t="inlineStr">
         <is>
@@ -18352,7 +18352,7 @@
         <v>21</v>
       </c>
       <c r="T204" t="n">
-        <v>2.100000000000001</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U204" t="n">
         <v>22.13333333333334</v>
@@ -18361,7 +18361,7 @@
         <v>3</v>
       </c>
       <c r="W204" t="n">
-        <v>24.33333333333333</v>
+        <v>24.33333333333334</v>
       </c>
       <c r="X204" t="n">
         <v>17.5</v>
@@ -18495,10 +18495,10 @@
         <v>28</v>
       </c>
       <c r="K206" t="n">
-        <v>26.8</v>
+        <v>27.9</v>
       </c>
       <c r="L206" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="M206" t="inlineStr">
         <is>
@@ -18528,7 +18528,7 @@
         <v>28</v>
       </c>
       <c r="T206" t="n">
-        <v>-1.199999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U206" t="n">
         <v>27.86666666666666</v>
@@ -18583,10 +18583,10 @@
         <v>28</v>
       </c>
       <c r="K207" t="n">
-        <v>26.1</v>
+        <v>27.7</v>
       </c>
       <c r="L207" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="M207" t="inlineStr">
         <is>
@@ -18616,7 +18616,7 @@
         <v>28</v>
       </c>
       <c r="T207" t="n">
-        <v>-1.899999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U207" t="n">
         <v>27.5</v>
@@ -18671,10 +18671,10 @@
         <v>28</v>
       </c>
       <c r="K208" t="n">
-        <v>27.7</v>
+        <v>28.9</v>
       </c>
       <c r="L208" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="M208" t="inlineStr">
         <is>
@@ -18704,7 +18704,7 @@
         <v>28</v>
       </c>
       <c r="T208" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U208" t="n">
         <v>28.4</v>
@@ -18847,10 +18847,10 @@
         <v>28</v>
       </c>
       <c r="K210" t="n">
-        <v>26.9</v>
+        <v>30.7</v>
       </c>
       <c r="L210" t="n">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="M210" t="inlineStr">
         <is>
@@ -18880,7 +18880,7 @@
         <v>28</v>
       </c>
       <c r="T210" t="n">
-        <v>-1.100000000000001</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U210" t="n">
         <v>28.46666666666667</v>
@@ -18935,10 +18935,10 @@
         <v>28</v>
       </c>
       <c r="K211" t="n">
-        <v>26.2</v>
+        <v>32.6</v>
       </c>
       <c r="L211" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="M211" t="inlineStr">
         <is>
@@ -18968,7 +18968,7 @@
         <v>28</v>
       </c>
       <c r="T211" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="U211" t="n">
         <v>30.03333333333333</v>
@@ -19023,10 +19023,10 @@
         <v>28</v>
       </c>
       <c r="K212" t="n">
-        <v>24.7</v>
+        <v>29.2</v>
       </c>
       <c r="L212" t="n">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="M212" t="inlineStr">
         <is>
@@ -19056,7 +19056,7 @@
         <v>28</v>
       </c>
       <c r="T212" t="n">
-        <v>-3.300000000000001</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="U212" t="n">
         <v>28.1</v>
@@ -20867,10 +20867,10 @@
         <v>28</v>
       </c>
       <c r="K233" t="n">
-        <v>24.5</v>
+        <v>26</v>
       </c>
       <c r="L233" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="M233" t="inlineStr">
         <is>
@@ -20900,7 +20900,7 @@
         <v>28</v>
       </c>
       <c r="T233" t="n">
-        <v>-3.5</v>
+        <v>-2</v>
       </c>
       <c r="U233" t="n">
         <v>25.53333333333333</v>
@@ -20955,10 +20955,10 @@
         <v>28</v>
       </c>
       <c r="K234" t="n">
-        <v>30.9</v>
+        <v>24.9</v>
       </c>
       <c r="L234" t="n">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="M234" t="inlineStr">
         <is>
@@ -20988,7 +20988,7 @@
         <v>28</v>
       </c>
       <c r="T234" t="n">
-        <v>2.899999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="U234" t="n">
         <v>27.93333333333333</v>
@@ -23313,10 +23313,10 @@
         <v>28</v>
       </c>
       <c r="K261" t="n">
-        <v>28.1</v>
+        <v>28.9</v>
       </c>
       <c r="L261" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="M261" t="inlineStr">
         <is>
@@ -23346,7 +23346,7 @@
         <v>28</v>
       </c>
       <c r="T261" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U261" t="n">
         <v>28.03333333333333</v>
@@ -24365,10 +24365,10 @@
         <v>21</v>
       </c>
       <c r="K273" t="n">
-        <v>26.4</v>
+        <v>16.3</v>
       </c>
       <c r="L273" t="n">
-        <v>126</v>
+        <v>78</v>
       </c>
       <c r="M273" t="inlineStr">
         <is>
@@ -24398,7 +24398,7 @@
         <v>21</v>
       </c>
       <c r="T273" t="n">
-        <v>5.399999999999999</v>
+        <v>-4.699999999999999</v>
       </c>
       <c r="U273" t="n">
         <v>22.9</v>
@@ -27611,10 +27611,10 @@
         <v>21</v>
       </c>
       <c r="K310" t="n">
-        <v>26.5</v>
+        <v>20.6</v>
       </c>
       <c r="L310" t="n">
-        <v>126</v>
+        <v>98</v>
       </c>
       <c r="M310" t="inlineStr">
         <is>
@@ -27644,7 +27644,7 @@
         <v>21</v>
       </c>
       <c r="T310" t="n">
-        <v>5.5</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U310" t="n">
         <v>23.9</v>
@@ -27697,10 +27697,10 @@
         <v>24.5</v>
       </c>
       <c r="K311" t="n">
-        <v>22.6</v>
+        <v>25</v>
       </c>
       <c r="L311" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="M311" t="inlineStr">
         <is>
@@ -27730,7 +27730,7 @@
         <v>28</v>
       </c>
       <c r="T311" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="U311" t="n">
         <v>24.8</v>
@@ -28577,10 +28577,10 @@
         <v>24.5</v>
       </c>
       <c r="K321" t="n">
-        <v>28.3</v>
+        <v>23.7</v>
       </c>
       <c r="L321" t="n">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="M321" t="inlineStr">
         <is>
@@ -28610,7 +28610,7 @@
         <v>28</v>
       </c>
       <c r="T321" t="n">
-        <v>3.800000000000001</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U321" t="n">
         <v>25.7</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L323" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L331" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -29897,10 +29897,10 @@
         <v>24.5</v>
       </c>
       <c r="K336" t="n">
-        <v>24.4</v>
+        <v>24.3</v>
       </c>
       <c r="L336" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M336" t="inlineStr">
         <is>
@@ -29930,7 +29930,7 @@
         <v>28</v>
       </c>
       <c r="T336" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U336" t="n">
         <v>24.26666666666667</v>
@@ -30379,7 +30379,7 @@
         <v>3</v>
       </c>
       <c r="W341" t="n">
-        <v>31.23333333333333</v>
+        <v>30.57777777777778</v>
       </c>
       <c r="X341" t="n">
         <v>21</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L353" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-07 20:01:57
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3247,10 +3247,10 @@
         <v>28</v>
       </c>
       <c r="K32" t="n">
-        <v>26.9</v>
+        <v>27.1</v>
       </c>
       <c r="L32" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3280,7 +3280,7 @@
         <v>28</v>
       </c>
       <c r="T32" t="n">
-        <v>-1.100000000000001</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U32" t="n">
         <v>27.23333333333333</v>
@@ -3421,10 +3421,10 @@
         <v>31</v>
       </c>
       <c r="K34" t="n">
-        <v>30.9</v>
+        <v>36</v>
       </c>
       <c r="L34" t="n">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="n">
-        <v>-0.1000000000000014</v>
+        <v>5</v>
       </c>
       <c r="U34" t="n">
         <v>33.03333333333333</v>
@@ -3507,10 +3507,10 @@
         <v>31</v>
       </c>
       <c r="K35" t="n">
-        <v>29.8</v>
+        <v>31.6</v>
       </c>
       <c r="L35" t="n">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3538,7 +3538,7 @@
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="n">
-        <v>-1.199999999999999</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U35" t="n">
         <v>30.4</v>
@@ -4113,10 +4113,10 @@
         <v>24</v>
       </c>
       <c r="K42" t="n">
-        <v>15.7</v>
+        <v>16.2</v>
       </c>
       <c r="L42" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="M42" t="inlineStr">
         <is>
@@ -4146,7 +4146,7 @@
         <v>28</v>
       </c>
       <c r="T42" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.800000000000001</v>
       </c>
       <c r="U42" t="n">
         <v>16.5</v>
@@ -5423,10 +5423,10 @@
         <v>31</v>
       </c>
       <c r="K57" t="n">
-        <v>39.3</v>
+        <v>18.8</v>
       </c>
       <c r="L57" t="n">
-        <v>127</v>
+        <v>61</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="n">
-        <v>8.299999999999997</v>
+        <v>-12.2</v>
       </c>
       <c r="U57" t="n">
         <v>31.73333333333333</v>
@@ -5509,10 +5509,10 @@
         <v>24</v>
       </c>
       <c r="K58" t="n">
-        <v>21.4</v>
+        <v>20.8</v>
       </c>
       <c r="L58" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -5542,7 +5542,7 @@
         <v>28</v>
       </c>
       <c r="T58" t="n">
-        <v>-2.600000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U58" t="n">
         <v>21.53333333333333</v>
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L77" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7353,7 +7353,7 @@
         <v>28</v>
       </c>
       <c r="K79" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="L79" t="n">
         <v>88</v>
@@ -7386,7 +7386,7 @@
         <v>28</v>
       </c>
       <c r="T79" t="n">
-        <v>-3.300000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U79" t="n">
         <v>25.13333333333334</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L81" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -7615,10 +7615,10 @@
         <v>21</v>
       </c>
       <c r="K82" t="n">
-        <v>17.9</v>
+        <v>26.4</v>
       </c>
       <c r="L82" t="n">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
         <v>21</v>
       </c>
       <c r="T82" t="n">
-        <v>-3.100000000000001</v>
+        <v>5.399999999999999</v>
       </c>
       <c r="U82" t="n">
         <v>21.3</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L88" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L93" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -12969,10 +12969,10 @@
         <v>35</v>
       </c>
       <c r="K143" t="n">
-        <v>29.7</v>
+        <v>39.9</v>
       </c>
       <c r="L143" t="n">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="M143" t="inlineStr">
         <is>
@@ -13002,7 +13002,7 @@
         <v>41</v>
       </c>
       <c r="T143" t="n">
-        <v>-5.300000000000001</v>
+        <v>4.899999999999999</v>
       </c>
       <c r="U143" t="n">
         <v>37</v>
@@ -14897,10 +14897,10 @@
         <v>21</v>
       </c>
       <c r="K165" t="n">
-        <v>20.9</v>
+        <v>22.9</v>
       </c>
       <c r="L165" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="M165" t="inlineStr">
         <is>
@@ -14930,7 +14930,7 @@
         <v>21</v>
       </c>
       <c r="T165" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U165" t="n">
         <v>22.96666666666667</v>
@@ -16477,10 +16477,10 @@
         <v>28</v>
       </c>
       <c r="K183" t="n">
-        <v>40.2</v>
+        <v>36.4</v>
       </c>
       <c r="L183" t="n">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="M183" t="inlineStr">
         <is>
@@ -16510,7 +16510,7 @@
         <v>28</v>
       </c>
       <c r="T183" t="n">
-        <v>12.2</v>
+        <v>8.399999999999999</v>
       </c>
       <c r="U183" t="n">
         <v>33.36666666666667</v>
@@ -17093,10 +17093,10 @@
         <v>35</v>
       </c>
       <c r="K190" t="n">
-        <v>43.4</v>
+        <v>26.1</v>
       </c>
       <c r="L190" t="n">
-        <v>124</v>
+        <v>74</v>
       </c>
       <c r="M190" t="inlineStr">
         <is>
@@ -17126,7 +17126,7 @@
         <v>41</v>
       </c>
       <c r="T190" t="n">
-        <v>8.399999999999999</v>
+        <v>-8.899999999999999</v>
       </c>
       <c r="U190" t="n">
         <v>33.26666666666667</v>
@@ -18319,10 +18319,10 @@
         <v>21</v>
       </c>
       <c r="K204" t="n">
-        <v>20.7</v>
+        <v>23.1</v>
       </c>
       <c r="L204" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="M204" t="inlineStr">
         <is>
@@ -18352,7 +18352,7 @@
         <v>21</v>
       </c>
       <c r="T204" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="U204" t="n">
         <v>22.13333333333334</v>
@@ -18361,7 +18361,7 @@
         <v>3</v>
       </c>
       <c r="W204" t="n">
-        <v>24.33333333333334</v>
+        <v>24.33333333333333</v>
       </c>
       <c r="X204" t="n">
         <v>17.5</v>
@@ -18495,10 +18495,10 @@
         <v>28</v>
       </c>
       <c r="K206" t="n">
-        <v>27.9</v>
+        <v>26.8</v>
       </c>
       <c r="L206" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M206" t="inlineStr">
         <is>
@@ -18528,7 +18528,7 @@
         <v>28</v>
       </c>
       <c r="T206" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U206" t="n">
         <v>27.86666666666666</v>
@@ -18583,10 +18583,10 @@
         <v>28</v>
       </c>
       <c r="K207" t="n">
-        <v>27.7</v>
+        <v>26.1</v>
       </c>
       <c r="L207" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="M207" t="inlineStr">
         <is>
@@ -18616,7 +18616,7 @@
         <v>28</v>
       </c>
       <c r="T207" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="U207" t="n">
         <v>27.5</v>
@@ -18671,10 +18671,10 @@
         <v>28</v>
       </c>
       <c r="K208" t="n">
-        <v>28.9</v>
+        <v>27.7</v>
       </c>
       <c r="L208" t="n">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="M208" t="inlineStr">
         <is>
@@ -18704,7 +18704,7 @@
         <v>28</v>
       </c>
       <c r="T208" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U208" t="n">
         <v>28.4</v>
@@ -18847,10 +18847,10 @@
         <v>28</v>
       </c>
       <c r="K210" t="n">
-        <v>30.7</v>
+        <v>26.9</v>
       </c>
       <c r="L210" t="n">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="M210" t="inlineStr">
         <is>
@@ -18880,7 +18880,7 @@
         <v>28</v>
       </c>
       <c r="T210" t="n">
-        <v>2.699999999999999</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U210" t="n">
         <v>28.46666666666667</v>
@@ -18935,10 +18935,10 @@
         <v>28</v>
       </c>
       <c r="K211" t="n">
-        <v>32.6</v>
+        <v>26.2</v>
       </c>
       <c r="L211" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="M211" t="inlineStr">
         <is>
@@ -18968,7 +18968,7 @@
         <v>28</v>
       </c>
       <c r="T211" t="n">
-        <v>4.600000000000001</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="U211" t="n">
         <v>30.03333333333333</v>
@@ -19023,10 +19023,10 @@
         <v>28</v>
       </c>
       <c r="K212" t="n">
-        <v>29.2</v>
+        <v>24.7</v>
       </c>
       <c r="L212" t="n">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="M212" t="inlineStr">
         <is>
@@ -19056,7 +19056,7 @@
         <v>28</v>
       </c>
       <c r="T212" t="n">
-        <v>1.199999999999999</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="U212" t="n">
         <v>28.1</v>
@@ -20867,10 +20867,10 @@
         <v>28</v>
       </c>
       <c r="K233" t="n">
-        <v>26</v>
+        <v>24.5</v>
       </c>
       <c r="L233" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="M233" t="inlineStr">
         <is>
@@ -20900,7 +20900,7 @@
         <v>28</v>
       </c>
       <c r="T233" t="n">
-        <v>-2</v>
+        <v>-3.5</v>
       </c>
       <c r="U233" t="n">
         <v>25.53333333333333</v>
@@ -20955,10 +20955,10 @@
         <v>28</v>
       </c>
       <c r="K234" t="n">
-        <v>24.9</v>
+        <v>30.9</v>
       </c>
       <c r="L234" t="n">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="M234" t="inlineStr">
         <is>
@@ -20988,7 +20988,7 @@
         <v>28</v>
       </c>
       <c r="T234" t="n">
-        <v>-3.100000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="U234" t="n">
         <v>27.93333333333333</v>
@@ -22265,10 +22265,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="L249" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22298,7 +22298,7 @@
         <v>21</v>
       </c>
       <c r="T249" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U249" t="n">
         <v>21.2</v>
@@ -23577,10 +23577,10 @@
         <v>28</v>
       </c>
       <c r="K264" t="n">
-        <v>24.7</v>
+        <v>32.5</v>
       </c>
       <c r="L264" t="n">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="M264" t="inlineStr">
         <is>
@@ -23610,7 +23610,7 @@
         <v>28</v>
       </c>
       <c r="T264" t="n">
-        <v>-3.300000000000001</v>
+        <v>4.5</v>
       </c>
       <c r="U264" t="n">
         <v>29.5</v>
@@ -24627,10 +24627,10 @@
         <v>28</v>
       </c>
       <c r="K276" t="n">
-        <v>27.6</v>
+        <v>32.5</v>
       </c>
       <c r="L276" t="n">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="M276" t="inlineStr">
         <is>
@@ -24660,7 +24660,7 @@
         <v>28</v>
       </c>
       <c r="T276" t="n">
-        <v>-0.3999999999999986</v>
+        <v>4.5</v>
       </c>
       <c r="U276" t="n">
         <v>30.16666666666667</v>
@@ -27785,10 +27785,10 @@
         <v>24.5</v>
       </c>
       <c r="K312" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="L312" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="M312" t="inlineStr">
         <is>
@@ -27818,7 +27818,7 @@
         <v>28</v>
       </c>
       <c r="T312" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U312" t="n">
         <v>25.13333333333334</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L323" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L331" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L353" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-08 00:04:32
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -606,11 +606,11 @@
         </is>
       </c>
       <c r="P2" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
@@ -694,11 +694,11 @@
         </is>
       </c>
       <c r="P3" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R3" s="2" t="n">
@@ -784,11 +784,11 @@
         </is>
       </c>
       <c r="P4" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
@@ -872,11 +872,11 @@
         </is>
       </c>
       <c r="P5" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R5" s="2" t="n">
@@ -962,11 +962,11 @@
         </is>
       </c>
       <c r="P6" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
@@ -1052,11 +1052,11 @@
         </is>
       </c>
       <c r="P7" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R7" s="2" t="n">
@@ -1142,11 +1142,11 @@
         </is>
       </c>
       <c r="P8" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
@@ -1232,11 +1232,11 @@
         </is>
       </c>
       <c r="P9" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R9" s="2" t="n">
@@ -1320,11 +1320,11 @@
         </is>
       </c>
       <c r="P10" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
@@ -1408,11 +1408,11 @@
         </is>
       </c>
       <c r="P11" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R11" s="2" t="n">
@@ -1496,11 +1496,11 @@
         </is>
       </c>
       <c r="P12" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
@@ -1584,11 +1584,11 @@
         </is>
       </c>
       <c r="P13" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R13" s="2" t="n">
@@ -1674,11 +1674,11 @@
         </is>
       </c>
       <c r="P14" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
@@ -1762,11 +1762,11 @@
         </is>
       </c>
       <c r="P15" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R15" s="2" t="n">
@@ -1850,11 +1850,11 @@
         </is>
       </c>
       <c r="P16" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
@@ -1938,11 +1938,11 @@
         </is>
       </c>
       <c r="P17" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R17" s="2" t="n">
@@ -2028,11 +2028,11 @@
         </is>
       </c>
       <c r="P18" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
@@ -2116,11 +2116,11 @@
         </is>
       </c>
       <c r="P19" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R19" s="2" t="n">
@@ -2204,11 +2204,11 @@
         </is>
       </c>
       <c r="P20" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
@@ -2294,11 +2294,11 @@
         </is>
       </c>
       <c r="P21" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R21" s="2" t="n">
@@ -2384,11 +2384,11 @@
         </is>
       </c>
       <c r="P22" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
@@ -2474,11 +2474,11 @@
         </is>
       </c>
       <c r="P23" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R23" s="2" t="n">
@@ -2564,11 +2564,11 @@
         </is>
       </c>
       <c r="P24" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
@@ -2654,11 +2654,11 @@
         </is>
       </c>
       <c r="P25" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R25" s="2" t="n">
@@ -2742,11 +2742,11 @@
         </is>
       </c>
       <c r="P26" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
@@ -2830,11 +2830,11 @@
         </is>
       </c>
       <c r="P27" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R27" s="2" t="n">

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-08 01:41:36
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -610,11 +610,11 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
@@ -698,11 +698,11 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R3" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S3" t="n">
         <v>28</v>
@@ -788,11 +788,11 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
@@ -876,11 +876,11 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R5" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S5" t="n">
         <v>48</v>
@@ -966,11 +966,11 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S6" t="n">
         <v>41</v>
@@ -1056,11 +1056,11 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R7" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S7" t="n">
         <v>48</v>
@@ -1146,11 +1146,11 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S8" t="n">
         <v>41</v>
@@ -1236,11 +1236,11 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R9" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
@@ -1324,11 +1324,11 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
@@ -1412,11 +1412,11 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R11" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="n">
@@ -1500,11 +1500,11 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
@@ -1588,11 +1588,11 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R13" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S13" t="n">
         <v>21</v>
@@ -1678,11 +1678,11 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="n">
@@ -1766,11 +1766,11 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R15" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="n">
@@ -1854,11 +1854,11 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="n">
@@ -1942,11 +1942,11 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R17" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S17" t="n">
         <v>34</v>
@@ -2032,11 +2032,11 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="n">
@@ -2120,11 +2120,11 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R19" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S19" t="n">
         <v>48</v>
@@ -2208,11 +2208,11 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S20" t="n">
         <v>48</v>
@@ -2298,11 +2298,11 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R21" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S21" t="n">
         <v>34</v>
@@ -2388,11 +2388,11 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S22" t="n">
         <v>28</v>
@@ -2478,11 +2478,11 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R23" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S23" t="n">
         <v>28</v>
@@ -2568,11 +2568,11 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S24" t="n">
         <v>28</v>
@@ -2658,11 +2658,11 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R25" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S25" t="n">
         <v>28</v>
@@ -2746,11 +2746,11 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="n">
@@ -2834,11 +2834,11 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R27" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="S27" t="n">
         <v>28</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-08 19:58:56
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4723,10 +4723,10 @@
         <v>24</v>
       </c>
       <c r="K49" t="n">
-        <v>25.9</v>
+        <v>22.1</v>
       </c>
       <c r="L49" t="n">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="M49" t="inlineStr">
         <is>
@@ -4756,7 +4756,7 @@
         <v>28</v>
       </c>
       <c r="T49" t="n">
-        <v>1.899999999999999</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="U49" t="n">
         <v>24.23333333333333</v>
@@ -5947,10 +5947,10 @@
         <v>24</v>
       </c>
       <c r="K63" t="n">
-        <v>23.4</v>
+        <v>25.7</v>
       </c>
       <c r="L63" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="M63" t="inlineStr">
         <is>
@@ -5980,7 +5980,7 @@
         <v>28</v>
       </c>
       <c r="T63" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="U63" t="n">
         <v>24.46666666666667</v>
@@ -7091,10 +7091,10 @@
         <v>31</v>
       </c>
       <c r="K76" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L76" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U76" t="n">
         <v>32.03333333333333</v>
@@ -7441,10 +7441,10 @@
         <v>31</v>
       </c>
       <c r="K80" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L80" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7472,7 +7472,7 @@
       </c>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U80" t="n">
         <v>36</v>
@@ -8055,10 +8055,10 @@
         <v>31</v>
       </c>
       <c r="K87" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L87" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M87" t="inlineStr">
         <is>
@@ -8086,7 +8086,7 @@
       </c>
       <c r="S87" t="inlineStr"/>
       <c r="T87" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U87" t="n">
         <v>33.63333333333333</v>
@@ -8493,10 +8493,10 @@
         <v>31</v>
       </c>
       <c r="K92" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L92" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="S92" t="inlineStr"/>
       <c r="T92" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U92" t="n">
         <v>32.76666666666667</v>
@@ -12617,10 +12617,10 @@
         <v>28</v>
       </c>
       <c r="K139" t="n">
-        <v>27.9</v>
+        <v>27.4</v>
       </c>
       <c r="L139" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="M139" t="inlineStr">
         <is>
@@ -12650,7 +12650,7 @@
         <v>28</v>
       </c>
       <c r="T139" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U139" t="n">
         <v>28.4</v>
@@ -12793,10 +12793,10 @@
         <v>35</v>
       </c>
       <c r="K141" t="n">
-        <v>34.7</v>
+        <v>39.7</v>
       </c>
       <c r="L141" t="n">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="M141" t="inlineStr">
         <is>
@@ -12826,7 +12826,7 @@
         <v>41</v>
       </c>
       <c r="T141" t="n">
-        <v>-0.2999999999999972</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="U141" t="n">
         <v>37.66666666666667</v>
@@ -22177,10 +22177,10 @@
         <v>21</v>
       </c>
       <c r="K248" t="n">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="L248" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M248" t="inlineStr">
         <is>
@@ -22210,7 +22210,7 @@
         <v>21</v>
       </c>
       <c r="T248" t="n">
-        <v>0.5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U248" t="n">
         <v>21.2</v>
@@ -24539,10 +24539,10 @@
         <v>28</v>
       </c>
       <c r="K275" t="n">
-        <v>27.6</v>
+        <v>32.5</v>
       </c>
       <c r="L275" t="n">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="M275" t="inlineStr">
         <is>
@@ -24572,7 +24572,7 @@
         <v>28</v>
       </c>
       <c r="T275" t="n">
-        <v>-0.3999999999999986</v>
+        <v>4.5</v>
       </c>
       <c r="U275" t="n">
         <v>30.16666666666667</v>
@@ -24979,10 +24979,10 @@
         <v>28</v>
       </c>
       <c r="K280" t="n">
-        <v>28.3</v>
+        <v>26.7</v>
       </c>
       <c r="L280" t="n">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="M280" t="inlineStr">
         <is>
@@ -25012,7 +25012,7 @@
         <v>28</v>
       </c>
       <c r="T280" t="n">
-        <v>0.3000000000000007</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U280" t="n">
         <v>27.4</v>
@@ -25067,10 +25067,10 @@
         <v>21</v>
       </c>
       <c r="K281" t="n">
-        <v>21.4</v>
+        <v>19.9</v>
       </c>
       <c r="L281" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="M281" t="inlineStr">
         <is>
@@ -25100,7 +25100,7 @@
         <v>21</v>
       </c>
       <c r="T281" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U281" t="n">
         <v>21</v>
@@ -28355,7 +28355,7 @@
         <v>3</v>
       </c>
       <c r="W318" t="n">
-        <v>27.24444444444444</v>
+        <v>27.24444444444445</v>
       </c>
       <c r="X318" t="n">
         <v>21</v>
@@ -29897,10 +29897,10 @@
         <v>24.5</v>
       </c>
       <c r="K336" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="L336" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="M336" t="inlineStr">
         <is>
@@ -29930,7 +29930,7 @@
         <v>28</v>
       </c>
       <c r="T336" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U336" t="n">
         <v>35.8</v>
@@ -30073,10 +30073,10 @@
         <v>24.5</v>
       </c>
       <c r="K338" t="n">
-        <v>24.7</v>
+        <v>24</v>
       </c>
       <c r="L338" t="n">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="M338" t="inlineStr">
         <is>
@@ -30106,7 +30106,7 @@
         <v>28</v>
       </c>
       <c r="T338" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.5</v>
       </c>
       <c r="U338" t="n">
         <v>24.1</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-09 08:32:04
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3159,10 +3159,10 @@
         <v>28</v>
       </c>
       <c r="K31" t="n">
-        <v>26.9</v>
+        <v>27.1</v>
       </c>
       <c r="L31" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -3192,7 +3192,7 @@
         <v>28</v>
       </c>
       <c r="T31" t="n">
-        <v>-1.100000000000001</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U31" t="n">
         <v>27.23333333333333</v>
@@ -4025,10 +4025,10 @@
         <v>24</v>
       </c>
       <c r="K41" t="n">
-        <v>15.7</v>
+        <v>16.2</v>
       </c>
       <c r="L41" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
@@ -4058,7 +4058,7 @@
         <v>28</v>
       </c>
       <c r="T41" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.800000000000001</v>
       </c>
       <c r="U41" t="n">
         <v>16.5</v>
@@ -4723,10 +4723,10 @@
         <v>24</v>
       </c>
       <c r="K49" t="n">
-        <v>25.9</v>
+        <v>22.1</v>
       </c>
       <c r="L49" t="n">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="M49" t="inlineStr">
         <is>
@@ -4756,7 +4756,7 @@
         <v>28</v>
       </c>
       <c r="T49" t="n">
-        <v>1.899999999999999</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="U49" t="n">
         <v>24.23333333333333</v>
@@ -10419,10 +10419,10 @@
         <v>35</v>
       </c>
       <c r="K114" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="L114" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="M114" t="inlineStr">
         <is>
@@ -10452,7 +10452,7 @@
         <v>41</v>
       </c>
       <c r="T114" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="U114" t="n">
         <v>25.5</v>
@@ -10683,10 +10683,10 @@
         <v>28</v>
       </c>
       <c r="K117" t="n">
-        <v>30.7</v>
+        <v>27.6</v>
       </c>
       <c r="L117" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="M117" t="inlineStr">
         <is>
@@ -10716,7 +10716,7 @@
         <v>28</v>
       </c>
       <c r="T117" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U117" t="n">
         <v>28.03333333333333</v>
@@ -21041,10 +21041,10 @@
         <v>42</v>
       </c>
       <c r="K235" t="n">
-        <v>49</v>
+        <v>31.1</v>
       </c>
       <c r="L235" t="n">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="M235" t="inlineStr">
         <is>
@@ -21074,7 +21074,7 @@
         <v>48</v>
       </c>
       <c r="T235" t="n">
-        <v>7</v>
+        <v>-10.9</v>
       </c>
       <c r="U235" t="n">
         <v>43.9</v>
@@ -21479,10 +21479,10 @@
         <v>31</v>
       </c>
       <c r="K240" t="n">
-        <v>33.2</v>
+        <v>32.6</v>
       </c>
       <c r="L240" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="M240" t="inlineStr">
         <is>
@@ -21510,7 +21510,7 @@
       </c>
       <c r="S240" t="inlineStr"/>
       <c r="T240" t="n">
-        <v>2.200000000000003</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U240" t="n">
         <v>32.06666666666667</v>
@@ -21565,10 +21565,10 @@
         <v>42</v>
       </c>
       <c r="K241" t="n">
-        <v>15.9</v>
+        <v>52.5</v>
       </c>
       <c r="L241" t="n">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="M241" t="inlineStr">
         <is>
@@ -21598,7 +21598,7 @@
         <v>48</v>
       </c>
       <c r="T241" t="n">
-        <v>-26.1</v>
+        <v>10.5</v>
       </c>
       <c r="U241" t="n">
         <v>39.6</v>
@@ -21653,10 +21653,10 @@
         <v>28</v>
       </c>
       <c r="K242" t="n">
-        <v>29.8</v>
+        <v>28.6</v>
       </c>
       <c r="L242" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="M242" t="inlineStr">
         <is>
@@ -21686,7 +21686,7 @@
         <v>28</v>
       </c>
       <c r="T242" t="n">
-        <v>1.800000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U242" t="n">
         <v>28.63333333333334</v>
@@ -21741,10 +21741,10 @@
         <v>21</v>
       </c>
       <c r="K243" t="n">
-        <v>21.7</v>
+        <v>19.7</v>
       </c>
       <c r="L243" t="n">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="M243" t="inlineStr">
         <is>
@@ -21774,7 +21774,7 @@
         <v>21</v>
       </c>
       <c r="T243" t="n">
-        <v>0.6999999999999993</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U243" t="n">
         <v>21</v>
@@ -21829,10 +21829,10 @@
         <v>28</v>
       </c>
       <c r="K244" t="n">
-        <v>26.1</v>
+        <v>38.4</v>
       </c>
       <c r="L244" t="n">
-        <v>93</v>
+        <v>137</v>
       </c>
       <c r="M244" t="inlineStr">
         <is>
@@ -21862,7 +21862,7 @@
         <v>28</v>
       </c>
       <c r="T244" t="n">
-        <v>-1.899999999999999</v>
+        <v>10.4</v>
       </c>
       <c r="U244" t="n">
         <v>35.16666666666666</v>
@@ -21917,10 +21917,10 @@
         <v>21</v>
       </c>
       <c r="K245" t="n">
-        <v>17.3</v>
+        <v>19</v>
       </c>
       <c r="L245" t="n">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="M245" t="inlineStr">
         <is>
@@ -21948,7 +21948,7 @@
       </c>
       <c r="S245" t="inlineStr"/>
       <c r="T245" t="n">
-        <v>-3.699999999999999</v>
+        <v>-2</v>
       </c>
       <c r="U245" t="n">
         <v>19.3</v>
@@ -23489,10 +23489,10 @@
         <v>28</v>
       </c>
       <c r="K263" t="n">
-        <v>24.7</v>
+        <v>32.5</v>
       </c>
       <c r="L263" t="n">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="M263" t="inlineStr">
         <is>
@@ -23522,7 +23522,7 @@
         <v>28</v>
       </c>
       <c r="T263" t="n">
-        <v>-3.300000000000001</v>
+        <v>4.5</v>
       </c>
       <c r="U263" t="n">
         <v>29.5</v>
@@ -23665,10 +23665,10 @@
         <v>28</v>
       </c>
       <c r="K265" t="n">
-        <v>29.9</v>
+        <v>32.3</v>
       </c>
       <c r="L265" t="n">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="M265" t="inlineStr">
         <is>
@@ -23698,7 +23698,7 @@
         <v>28</v>
       </c>
       <c r="T265" t="n">
-        <v>1.899999999999999</v>
+        <v>4.299999999999997</v>
       </c>
       <c r="U265" t="n">
         <v>28.53333333333333</v>
@@ -23839,10 +23839,10 @@
         <v>28</v>
       </c>
       <c r="K267" t="n">
-        <v>27</v>
+        <v>28.1</v>
       </c>
       <c r="L267" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="M267" t="inlineStr">
         <is>
@@ -23872,7 +23872,7 @@
         <v>28</v>
       </c>
       <c r="T267" t="n">
-        <v>-1</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U267" t="n">
         <v>26.96666666666667</v>
@@ -24143,7 +24143,7 @@
         <v>3</v>
       </c>
       <c r="W270" t="n">
-        <v>28.15555555555555</v>
+        <v>28.15555555555556</v>
       </c>
       <c r="X270" t="n">
         <v>24.5</v>
@@ -24189,10 +24189,10 @@
         <v>28</v>
       </c>
       <c r="K271" t="n">
-        <v>26.1</v>
+        <v>27.3</v>
       </c>
       <c r="L271" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="M271" t="inlineStr">
         <is>
@@ -24222,7 +24222,7 @@
         <v>28</v>
       </c>
       <c r="T271" t="n">
-        <v>-1.899999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="U271" t="n">
         <v>27.16666666666667</v>
@@ -24277,10 +24277,10 @@
         <v>21</v>
       </c>
       <c r="K272" t="n">
-        <v>26.4</v>
+        <v>16.3</v>
       </c>
       <c r="L272" t="n">
-        <v>126</v>
+        <v>78</v>
       </c>
       <c r="M272" t="inlineStr">
         <is>
@@ -24310,7 +24310,7 @@
         <v>21</v>
       </c>
       <c r="T272" t="n">
-        <v>5.399999999999999</v>
+        <v>-4.699999999999999</v>
       </c>
       <c r="U272" t="n">
         <v>22.9</v>
@@ -25419,10 +25419,10 @@
         <v>21</v>
       </c>
       <c r="K285" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="L285" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M285" t="inlineStr">
         <is>
@@ -25452,7 +25452,7 @@
         <v>21</v>
       </c>
       <c r="T285" t="n">
-        <v>-0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="U285" t="n">
         <v>21.03333333333333</v>
@@ -25507,10 +25507,10 @@
         <v>21</v>
       </c>
       <c r="K286" t="n">
-        <v>18.6</v>
+        <v>18.2</v>
       </c>
       <c r="L286" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="M286" t="inlineStr">
         <is>
@@ -25540,7 +25540,7 @@
         <v>21</v>
       </c>
       <c r="T286" t="n">
-        <v>-2.399999999999999</v>
+        <v>-2.800000000000001</v>
       </c>
       <c r="U286" t="n">
         <v>18.23333333333333</v>
@@ -25595,10 +25595,10 @@
         <v>21</v>
       </c>
       <c r="K287" t="n">
-        <v>18.4</v>
+        <v>20.2</v>
       </c>
       <c r="L287" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="M287" t="inlineStr">
         <is>
@@ -25628,16 +25628,16 @@
         <v>21</v>
       </c>
       <c r="T287" t="n">
-        <v>-2.600000000000001</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U287" t="n">
-        <v>19.86666666666666</v>
+        <v>19.86666666666667</v>
       </c>
       <c r="V287" t="n">
         <v>3</v>
       </c>
       <c r="W287" t="n">
-        <v>21.74444444444444</v>
+        <v>21.74444444444445</v>
       </c>
       <c r="X287" t="n">
         <v>17.5</v>
@@ -25767,10 +25767,10 @@
         <v>21</v>
       </c>
       <c r="K289" t="n">
-        <v>25.9</v>
+        <v>22.6</v>
       </c>
       <c r="L289" t="n">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="M289" t="inlineStr">
         <is>
@@ -25800,7 +25800,7 @@
         <v>21</v>
       </c>
       <c r="T289" t="n">
-        <v>4.899999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U289" t="n">
         <v>22.7</v>
@@ -26381,10 +26381,10 @@
         <v>21</v>
       </c>
       <c r="K296" t="n">
-        <v>20.3</v>
+        <v>21.9</v>
       </c>
       <c r="L296" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="M296" t="inlineStr">
         <is>
@@ -26414,7 +26414,7 @@
         <v>21</v>
       </c>
       <c r="T296" t="n">
-        <v>-0.6999999999999993</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U296" t="n">
         <v>20.9</v>
@@ -26469,10 +26469,10 @@
         <v>21</v>
       </c>
       <c r="K297" t="n">
-        <v>20.1</v>
+        <v>20.8</v>
       </c>
       <c r="L297" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="M297" t="inlineStr">
         <is>
@@ -26502,7 +26502,7 @@
         <v>21</v>
       </c>
       <c r="T297" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U297" t="n">
         <v>20.3</v>
@@ -27259,10 +27259,10 @@
         <v>21</v>
       </c>
       <c r="K306" t="n">
-        <v>20.4</v>
+        <v>21.8</v>
       </c>
       <c r="L306" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="M306" t="inlineStr">
         <is>
@@ -27292,7 +27292,7 @@
         <v>21</v>
       </c>
       <c r="T306" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.8000000000000007</v>
       </c>
       <c r="U306" t="n">
         <v>20.76666666666667</v>
@@ -27347,10 +27347,10 @@
         <v>21</v>
       </c>
       <c r="K307" t="n">
-        <v>19.4</v>
+        <v>22</v>
       </c>
       <c r="L307" t="n">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="M307" t="inlineStr">
         <is>
@@ -27380,7 +27380,7 @@
         <v>21</v>
       </c>
       <c r="T307" t="n">
-        <v>-1.600000000000001</v>
+        <v>1</v>
       </c>
       <c r="U307" t="n">
         <v>20.8</v>
@@ -27435,10 +27435,10 @@
         <v>21</v>
       </c>
       <c r="K308" t="n">
-        <v>19.6</v>
+        <v>20.7</v>
       </c>
       <c r="L308" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="M308" t="inlineStr">
         <is>
@@ -27468,7 +27468,7 @@
         <v>21</v>
       </c>
       <c r="T308" t="n">
-        <v>-1.399999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U308" t="n">
         <v>20.23333333333333</v>
@@ -27961,10 +27961,10 @@
         <v>24.5</v>
       </c>
       <c r="K314" t="n">
-        <v>22.8</v>
+        <v>24.8</v>
       </c>
       <c r="L314" t="n">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="M314" t="inlineStr">
         <is>
@@ -27994,7 +27994,7 @@
         <v>28</v>
       </c>
       <c r="T314" t="n">
-        <v>-1.699999999999999</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U314" t="n">
         <v>24.1</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-10 01:44:43
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -606,11 +606,11 @@
         </is>
       </c>
       <c r="P2" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
@@ -694,11 +694,11 @@
         </is>
       </c>
       <c r="P3" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R3" s="2" t="n">
@@ -784,11 +784,11 @@
         </is>
       </c>
       <c r="P4" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
@@ -872,11 +872,11 @@
         </is>
       </c>
       <c r="P5" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R5" s="2" t="n">
@@ -962,11 +962,11 @@
         </is>
       </c>
       <c r="P6" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
@@ -1052,11 +1052,11 @@
         </is>
       </c>
       <c r="P7" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R7" s="2" t="n">
@@ -1142,11 +1142,11 @@
         </is>
       </c>
       <c r="P8" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
@@ -1232,11 +1232,11 @@
         </is>
       </c>
       <c r="P9" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R9" s="2" t="n">
@@ -1320,11 +1320,11 @@
         </is>
       </c>
       <c r="P10" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
@@ -1408,11 +1408,11 @@
         </is>
       </c>
       <c r="P11" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R11" s="2" t="n">
@@ -1496,11 +1496,11 @@
         </is>
       </c>
       <c r="P12" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
@@ -1586,11 +1586,11 @@
         </is>
       </c>
       <c r="P13" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R13" s="2" t="n">
@@ -1674,11 +1674,11 @@
         </is>
       </c>
       <c r="P14" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
@@ -1762,11 +1762,11 @@
         </is>
       </c>
       <c r="P15" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R15" s="2" t="n">
@@ -1850,11 +1850,11 @@
         </is>
       </c>
       <c r="P16" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
@@ -1940,11 +1940,11 @@
         </is>
       </c>
       <c r="P17" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R17" s="2" t="n">
@@ -2028,11 +2028,11 @@
         </is>
       </c>
       <c r="P18" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
@@ -2116,11 +2116,11 @@
         </is>
       </c>
       <c r="P19" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R19" s="2" t="n">
@@ -2206,11 +2206,11 @@
         </is>
       </c>
       <c r="P20" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
@@ -2296,11 +2296,11 @@
         </is>
       </c>
       <c r="P21" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R21" s="2" t="n">
@@ -2386,11 +2386,11 @@
         </is>
       </c>
       <c r="P22" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
@@ -2476,11 +2476,11 @@
         </is>
       </c>
       <c r="P23" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R23" s="2" t="n">
@@ -2566,11 +2566,11 @@
         </is>
       </c>
       <c r="P24" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
@@ -2654,11 +2654,11 @@
         </is>
       </c>
       <c r="P25" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R25" s="2" t="n">
@@ -2742,11 +2742,11 @@
         </is>
       </c>
       <c r="P26" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
@@ -2830,11 +2830,11 @@
         </is>
       </c>
       <c r="P27" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R27" s="2" t="n">
@@ -2918,11 +2918,11 @@
         </is>
       </c>
       <c r="P28" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
@@ -3006,11 +3006,11 @@
         </is>
       </c>
       <c r="P29" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R29" s="2" t="n">
@@ -3092,11 +3092,11 @@
         </is>
       </c>
       <c r="P30" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
@@ -3178,11 +3178,11 @@
         </is>
       </c>
       <c r="P31" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R31" s="2" t="n">
@@ -3266,11 +3266,11 @@
         </is>
       </c>
       <c r="P32" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
@@ -3352,11 +3352,11 @@
         </is>
       </c>
       <c r="P33" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R33" s="2" t="n">
@@ -3438,11 +3438,11 @@
         </is>
       </c>
       <c r="P34" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
@@ -3524,11 +3524,11 @@
         </is>
       </c>
       <c r="P35" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R35" s="2" t="n">
@@ -3610,11 +3610,11 @@
         </is>
       </c>
       <c r="P36" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -3698,11 +3698,11 @@
         </is>
       </c>
       <c r="P37" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R37" s="2" t="n">
@@ -3784,11 +3784,11 @@
         </is>
       </c>
       <c r="P38" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R38" s="2" t="n">
@@ -3870,11 +3870,11 @@
         </is>
       </c>
       <c r="P39" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R39" s="2" t="n">
@@ -3939,10 +3939,10 @@
         <v>31</v>
       </c>
       <c r="K40" t="n">
-        <v>30.1</v>
+        <v>32.8</v>
       </c>
       <c r="L40" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
@@ -3958,11 +3958,11 @@
         </is>
       </c>
       <c r="P40" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R40" s="2" t="n">
@@ -3970,7 +3970,7 @@
       </c>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="n">
-        <v>-0.8999999999999986</v>
+        <v>1.799999999999997</v>
       </c>
       <c r="U40" t="n">
         <v>32.13333333333333</v>
@@ -4025,10 +4025,10 @@
         <v>24</v>
       </c>
       <c r="K41" t="n">
-        <v>16.2</v>
+        <v>17.6</v>
       </c>
       <c r="L41" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
@@ -4044,11 +4044,11 @@
         </is>
       </c>
       <c r="P41" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R41" s="2" t="n">
@@ -4058,7 +4058,7 @@
         <v>28</v>
       </c>
       <c r="T41" t="n">
-        <v>-7.800000000000001</v>
+        <v>-6.399999999999999</v>
       </c>
       <c r="U41" t="n">
         <v>16.5</v>
@@ -4132,11 +4132,11 @@
         </is>
       </c>
       <c r="P42" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R42" s="2" t="n">
@@ -4218,11 +4218,11 @@
         </is>
       </c>
       <c r="P43" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R43" s="2" t="n">
@@ -4304,11 +4304,11 @@
         </is>
       </c>
       <c r="P44" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R44" s="2" t="n">
@@ -4392,11 +4392,11 @@
         </is>
       </c>
       <c r="P45" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R45" s="2" t="n">
@@ -4480,11 +4480,11 @@
         </is>
       </c>
       <c r="P46" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R46" s="2" t="n">
@@ -4566,11 +4566,11 @@
         </is>
       </c>
       <c r="P47" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R47" s="2" t="n">
@@ -4654,11 +4654,11 @@
         </is>
       </c>
       <c r="P48" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R48" s="2" t="n">
@@ -4742,11 +4742,11 @@
         </is>
       </c>
       <c r="P49" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R49" s="2" t="n">
@@ -4830,11 +4830,11 @@
         </is>
       </c>
       <c r="P50" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R50" s="2" t="n">
@@ -4918,11 +4918,11 @@
         </is>
       </c>
       <c r="P51" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R51" s="2" t="n">
@@ -5006,11 +5006,11 @@
         </is>
       </c>
       <c r="P52" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R52" s="2" t="n">
@@ -5092,11 +5092,11 @@
         </is>
       </c>
       <c r="P53" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R53" s="2" t="n">
@@ -5178,11 +5178,11 @@
         </is>
       </c>
       <c r="P54" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R54" s="2" t="n">
@@ -5266,11 +5266,11 @@
         </is>
       </c>
       <c r="P55" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R55" s="2" t="n">
@@ -5354,11 +5354,11 @@
         </is>
       </c>
       <c r="P56" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R56" s="2" t="n">
@@ -5440,11 +5440,11 @@
         </is>
       </c>
       <c r="P57" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R57" s="2" t="n">
@@ -5528,11 +5528,11 @@
         </is>
       </c>
       <c r="P58" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R58" s="2" t="n">
@@ -5616,11 +5616,11 @@
         </is>
       </c>
       <c r="P59" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R59" s="2" t="n">
@@ -5702,11 +5702,11 @@
         </is>
       </c>
       <c r="P60" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R60" s="2" t="n">
@@ -5790,11 +5790,11 @@
         </is>
       </c>
       <c r="P61" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R61" s="2" t="n">
@@ -5878,11 +5878,11 @@
         </is>
       </c>
       <c r="P62" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R62" s="2" t="n">
@@ -5966,11 +5966,11 @@
         </is>
       </c>
       <c r="P63" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R63" s="2" t="n">
@@ -6054,11 +6054,11 @@
         </is>
       </c>
       <c r="P64" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R64" s="2" t="n">
@@ -6142,11 +6142,11 @@
         </is>
       </c>
       <c r="P65" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R65" s="2" t="n">
@@ -6230,11 +6230,11 @@
         </is>
       </c>
       <c r="P66" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R66" s="2" t="n">
@@ -6318,11 +6318,11 @@
         </is>
       </c>
       <c r="P67" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R67" s="2" t="n">
@@ -6406,11 +6406,11 @@
         </is>
       </c>
       <c r="P68" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R68" s="2" t="n">
@@ -6494,11 +6494,11 @@
         </is>
       </c>
       <c r="P69" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R69" s="2" t="n">
@@ -6582,11 +6582,11 @@
         </is>
       </c>
       <c r="P70" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R70" s="2" t="n">
@@ -6670,11 +6670,11 @@
         </is>
       </c>
       <c r="P71" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R71" s="2" t="n">
@@ -6758,11 +6758,11 @@
         </is>
       </c>
       <c r="P72" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R72" s="2" t="n">
@@ -6846,11 +6846,11 @@
         </is>
       </c>
       <c r="P73" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R73" s="2" t="n">
@@ -6934,11 +6934,11 @@
         </is>
       </c>
       <c r="P74" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R74" s="2" t="n">
@@ -7022,11 +7022,11 @@
         </is>
       </c>
       <c r="P75" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R75" s="2" t="n">
@@ -7091,10 +7091,10 @@
         <v>31</v>
       </c>
       <c r="K76" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L76" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -7110,11 +7110,11 @@
         </is>
       </c>
       <c r="P76" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R76" s="2" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U76" t="n">
         <v>32.03333333333333</v>
@@ -7196,11 +7196,11 @@
         </is>
       </c>
       <c r="P77" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R77" s="2" t="n">
@@ -7284,11 +7284,11 @@
         </is>
       </c>
       <c r="P78" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R78" s="2" t="n">
@@ -7372,11 +7372,11 @@
         </is>
       </c>
       <c r="P79" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R79" s="2" t="n">
@@ -7441,10 +7441,10 @@
         <v>31</v>
       </c>
       <c r="K80" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L80" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7460,11 +7460,11 @@
         </is>
       </c>
       <c r="P80" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R80" s="2" t="n">
@@ -7472,7 +7472,7 @@
       </c>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U80" t="n">
         <v>36</v>
@@ -7546,11 +7546,11 @@
         </is>
       </c>
       <c r="P81" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R81" s="2" t="n">
@@ -7615,10 +7615,10 @@
         <v>35</v>
       </c>
       <c r="K82" t="n">
-        <v>32.4</v>
+        <v>39.8</v>
       </c>
       <c r="L82" t="n">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7634,11 +7634,11 @@
         </is>
       </c>
       <c r="P82" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R82" s="2" t="n">
@@ -7648,7 +7648,7 @@
         <v>41</v>
       </c>
       <c r="T82" t="n">
-        <v>-2.600000000000001</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="U82" t="n">
         <v>36.03333333333333</v>
@@ -7722,11 +7722,11 @@
         </is>
       </c>
       <c r="P83" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R83" s="2" t="n">
@@ -7810,11 +7810,11 @@
         </is>
       </c>
       <c r="P84" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R84" s="2" t="n">
@@ -7898,11 +7898,11 @@
         </is>
       </c>
       <c r="P85" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R85" s="2" t="n">
@@ -7986,11 +7986,11 @@
         </is>
       </c>
       <c r="P86" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R86" s="2" t="n">
@@ -8055,10 +8055,10 @@
         <v>31</v>
       </c>
       <c r="K87" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L87" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M87" t="inlineStr">
         <is>
@@ -8074,11 +8074,11 @@
         </is>
       </c>
       <c r="P87" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R87" s="2" t="n">
@@ -8086,7 +8086,7 @@
       </c>
       <c r="S87" t="inlineStr"/>
       <c r="T87" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U87" t="n">
         <v>33.63333333333333</v>
@@ -8160,11 +8160,11 @@
         </is>
       </c>
       <c r="P88" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R88" s="2" t="n">
@@ -8248,11 +8248,11 @@
         </is>
       </c>
       <c r="P89" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R89" s="2" t="n">
@@ -8336,11 +8336,11 @@
         </is>
       </c>
       <c r="P90" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R90" s="2" t="n">
@@ -8424,11 +8424,11 @@
         </is>
       </c>
       <c r="P91" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R91" s="2" t="n">
@@ -8493,10 +8493,10 @@
         <v>31</v>
       </c>
       <c r="K92" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L92" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -8512,11 +8512,11 @@
         </is>
       </c>
       <c r="P92" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R92" s="2" t="n">
@@ -8524,7 +8524,7 @@
       </c>
       <c r="S92" t="inlineStr"/>
       <c r="T92" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U92" t="n">
         <v>32.76666666666667</v>
@@ -8598,11 +8598,11 @@
         </is>
       </c>
       <c r="P93" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R93" s="2" t="n">
@@ -8686,11 +8686,11 @@
         </is>
       </c>
       <c r="P94" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R94" s="2" t="n">
@@ -8772,11 +8772,11 @@
         </is>
       </c>
       <c r="P95" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R95" s="2" t="n">
@@ -8860,11 +8860,11 @@
         </is>
       </c>
       <c r="P96" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R96" s="2" t="n">
@@ -8948,11 +8948,11 @@
         </is>
       </c>
       <c r="P97" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R97" s="2" t="n">
@@ -9036,11 +9036,11 @@
         </is>
       </c>
       <c r="P98" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R98" s="2" t="n">
@@ -9124,11 +9124,11 @@
         </is>
       </c>
       <c r="P99" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R99" s="2" t="n">
@@ -9212,11 +9212,11 @@
         </is>
       </c>
       <c r="P100" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R100" s="2" t="n">
@@ -9300,11 +9300,11 @@
         </is>
       </c>
       <c r="P101" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R101" s="2" t="n">
@@ -9388,11 +9388,11 @@
         </is>
       </c>
       <c r="P102" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R102" s="2" t="n">
@@ -9476,11 +9476,11 @@
         </is>
       </c>
       <c r="P103" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R103" s="2" t="n">
@@ -9562,11 +9562,11 @@
         </is>
       </c>
       <c r="P104" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R104" s="2" t="n">
@@ -9648,11 +9648,11 @@
         </is>
       </c>
       <c r="P105" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R105" s="2" t="n">
@@ -9734,11 +9734,11 @@
         </is>
       </c>
       <c r="P106" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R106" s="2" t="n">
@@ -9822,11 +9822,11 @@
         </is>
       </c>
       <c r="P107" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R107" s="2" t="n">
@@ -9910,11 +9910,11 @@
         </is>
       </c>
       <c r="P108" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R108" s="2" t="n">
@@ -9998,11 +9998,11 @@
         </is>
       </c>
       <c r="P109" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R109" s="2" t="n">
@@ -10086,11 +10086,11 @@
         </is>
       </c>
       <c r="P110" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R110" s="2" t="n">
@@ -10174,11 +10174,11 @@
         </is>
       </c>
       <c r="P111" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R111" s="2" t="n">
@@ -10262,11 +10262,11 @@
         </is>
       </c>
       <c r="P112" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R112" s="2" t="n">
@@ -10350,11 +10350,11 @@
         </is>
       </c>
       <c r="P113" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R113" s="2" t="n">
@@ -10438,11 +10438,11 @@
         </is>
       </c>
       <c r="P114" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R114" s="2" t="n">
@@ -10526,11 +10526,11 @@
         </is>
       </c>
       <c r="P115" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R115" s="2" t="n">
@@ -10614,11 +10614,11 @@
         </is>
       </c>
       <c r="P116" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R116" s="2" t="n">
@@ -10683,10 +10683,10 @@
         <v>28</v>
       </c>
       <c r="K117" t="n">
-        <v>27.6</v>
+        <v>30.7</v>
       </c>
       <c r="L117" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="M117" t="inlineStr">
         <is>
@@ -10702,11 +10702,11 @@
         </is>
       </c>
       <c r="P117" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R117" s="2" t="n">
@@ -10716,7 +10716,7 @@
         <v>28</v>
       </c>
       <c r="T117" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U117" t="n">
         <v>28.03333333333333</v>
@@ -10790,11 +10790,11 @@
         </is>
       </c>
       <c r="P118" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R118" s="2" t="n">
@@ -10878,11 +10878,11 @@
         </is>
       </c>
       <c r="P119" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R119" s="2" t="n">
@@ -10966,11 +10966,11 @@
         </is>
       </c>
       <c r="P120" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R120" s="2" t="n">
@@ -11054,11 +11054,11 @@
         </is>
       </c>
       <c r="P121" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R121" s="2" t="n">
@@ -11142,11 +11142,11 @@
         </is>
       </c>
       <c r="P122" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R122" s="2" t="n">
@@ -11230,11 +11230,11 @@
         </is>
       </c>
       <c r="P123" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R123" s="2" t="n">
@@ -11299,10 +11299,10 @@
         <v>21</v>
       </c>
       <c r="K124" t="n">
-        <v>22.6</v>
+        <v>18.4</v>
       </c>
       <c r="L124" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11318,11 +11318,11 @@
         </is>
       </c>
       <c r="P124" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R124" s="2" t="n">
@@ -11332,10 +11332,10 @@
         <v>21</v>
       </c>
       <c r="T124" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U124" t="n">
-        <v>22.93333333333334</v>
+        <v>22.93333333333333</v>
       </c>
       <c r="V124" t="n">
         <v>3</v>
@@ -11406,11 +11406,11 @@
         </is>
       </c>
       <c r="P125" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R125" s="2" t="n">
@@ -11494,11 +11494,11 @@
         </is>
       </c>
       <c r="P126" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R126" s="2" t="n">
@@ -11582,11 +11582,11 @@
         </is>
       </c>
       <c r="P127" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R127" s="2" t="n">
@@ -11670,11 +11670,11 @@
         </is>
       </c>
       <c r="P128" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R128" s="2" t="n">
@@ -11758,11 +11758,11 @@
         </is>
       </c>
       <c r="P129" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R129" s="2" t="n">
@@ -11846,11 +11846,11 @@
         </is>
       </c>
       <c r="P130" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R130" s="2" t="n">
@@ -11934,11 +11934,11 @@
         </is>
       </c>
       <c r="P131" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R131" s="2" t="n">
@@ -12022,11 +12022,11 @@
         </is>
       </c>
       <c r="P132" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R132" s="2" t="n">
@@ -12110,11 +12110,11 @@
         </is>
       </c>
       <c r="P133" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R133" s="2" t="n">
@@ -12198,11 +12198,11 @@
         </is>
       </c>
       <c r="P134" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R134" s="2" t="n">
@@ -12286,11 +12286,11 @@
         </is>
       </c>
       <c r="P135" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R135" s="2" t="n">
@@ -12374,11 +12374,11 @@
         </is>
       </c>
       <c r="P136" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R136" s="2" t="n">
@@ -12460,11 +12460,11 @@
         </is>
       </c>
       <c r="P137" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R137" s="2" t="n">
@@ -12548,11 +12548,11 @@
         </is>
       </c>
       <c r="P138" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R138" s="2" t="n">
@@ -12636,11 +12636,11 @@
         </is>
       </c>
       <c r="P139" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R139" s="2" t="n">
@@ -12724,11 +12724,11 @@
         </is>
       </c>
       <c r="P140" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R140" s="2" t="n">
@@ -12812,11 +12812,11 @@
         </is>
       </c>
       <c r="P141" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R141" s="2" t="n">
@@ -12900,11 +12900,11 @@
         </is>
       </c>
       <c r="P142" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R142" s="2" t="n">
@@ -12988,11 +12988,11 @@
         </is>
       </c>
       <c r="P143" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R143" s="2" t="n">
@@ -13076,11 +13076,11 @@
         </is>
       </c>
       <c r="P144" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R144" s="2" t="n">
@@ -13164,11 +13164,11 @@
         </is>
       </c>
       <c r="P145" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R145" s="2" t="n">
@@ -13252,11 +13252,11 @@
         </is>
       </c>
       <c r="P146" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R146" s="2" t="n">
@@ -13338,11 +13338,11 @@
         </is>
       </c>
       <c r="P147" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R147" s="2" t="n">
@@ -13426,11 +13426,11 @@
         </is>
       </c>
       <c r="P148" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R148" s="2" t="n">
@@ -13514,11 +13514,11 @@
         </is>
       </c>
       <c r="P149" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R149" s="2" t="n">
@@ -13602,11 +13602,11 @@
         </is>
       </c>
       <c r="P150" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R150" s="2" t="n">
@@ -13690,11 +13690,11 @@
         </is>
       </c>
       <c r="P151" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R151" s="2" t="n">
@@ -13776,11 +13776,11 @@
         </is>
       </c>
       <c r="P152" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R152" s="2" t="n">
@@ -13862,11 +13862,11 @@
         </is>
       </c>
       <c r="P153" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R153" s="2" t="n">
@@ -13950,11 +13950,11 @@
         </is>
       </c>
       <c r="P154" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R154" s="2" t="n">
@@ -14038,11 +14038,11 @@
         </is>
       </c>
       <c r="P155" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R155" s="2" t="n">
@@ -14126,11 +14126,11 @@
         </is>
       </c>
       <c r="P156" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R156" s="2" t="n">
@@ -14214,11 +14214,11 @@
         </is>
       </c>
       <c r="P157" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R157" s="2" t="n">
@@ -14302,11 +14302,11 @@
         </is>
       </c>
       <c r="P158" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R158" s="2" t="n">
@@ -14390,11 +14390,11 @@
         </is>
       </c>
       <c r="P159" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R159" s="2" t="n">
@@ -14478,11 +14478,11 @@
         </is>
       </c>
       <c r="P160" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R160" s="2" t="n">
@@ -14566,11 +14566,11 @@
         </is>
       </c>
       <c r="P161" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R161" s="2" t="n">
@@ -14654,11 +14654,11 @@
         </is>
       </c>
       <c r="P162" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R162" s="2" t="n">
@@ -14721,10 +14721,10 @@
         <v>21</v>
       </c>
       <c r="K163" t="n">
-        <v>23.9</v>
+        <v>26</v>
       </c>
       <c r="L163" t="n">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="M163" t="inlineStr">
         <is>
@@ -14740,11 +14740,11 @@
         </is>
       </c>
       <c r="P163" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R163" s="2" t="n">
@@ -14754,7 +14754,7 @@
         <v>21</v>
       </c>
       <c r="T163" t="n">
-        <v>2.899999999999999</v>
+        <v>5</v>
       </c>
       <c r="U163" t="n">
         <v>23.4</v>
@@ -14828,11 +14828,11 @@
         </is>
       </c>
       <c r="P164" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R164" s="2" t="n">
@@ -14916,11 +14916,11 @@
         </is>
       </c>
       <c r="P165" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q165" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R165" s="2" t="n">
@@ -15002,11 +15002,11 @@
         </is>
       </c>
       <c r="P166" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R166" s="2" t="n">
@@ -15090,11 +15090,11 @@
         </is>
       </c>
       <c r="P167" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R167" s="2" t="n">
@@ -15178,11 +15178,11 @@
         </is>
       </c>
       <c r="P168" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R168" s="2" t="n">
@@ -15266,11 +15266,11 @@
         </is>
       </c>
       <c r="P169" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R169" s="2" t="n">
@@ -15354,11 +15354,11 @@
         </is>
       </c>
       <c r="P170" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R170" s="2" t="n">
@@ -15442,11 +15442,11 @@
         </is>
       </c>
       <c r="P171" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R171" s="2" t="n">
@@ -15530,11 +15530,11 @@
         </is>
       </c>
       <c r="P172" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R172" s="2" t="n">
@@ -15599,10 +15599,10 @@
         <v>24</v>
       </c>
       <c r="K173" t="n">
-        <v>26.2</v>
+        <v>18.5</v>
       </c>
       <c r="L173" t="n">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="M173" t="inlineStr">
         <is>
@@ -15618,11 +15618,11 @@
         </is>
       </c>
       <c r="P173" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q173" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R173" s="2" t="n">
@@ -15632,7 +15632,7 @@
         <v>28</v>
       </c>
       <c r="T173" t="n">
-        <v>2.199999999999999</v>
+        <v>-5.5</v>
       </c>
       <c r="U173" t="n">
         <v>24.66666666666667</v>
@@ -15706,11 +15706,11 @@
         </is>
       </c>
       <c r="P174" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q174" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R174" s="2" t="n">
@@ -15794,11 +15794,11 @@
         </is>
       </c>
       <c r="P175" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q175" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R175" s="2" t="n">
@@ -15882,11 +15882,11 @@
         </is>
       </c>
       <c r="P176" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R176" s="2" t="n">
@@ -15970,11 +15970,11 @@
         </is>
       </c>
       <c r="P177" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q177" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R177" s="2" t="n">
@@ -16058,11 +16058,11 @@
         </is>
       </c>
       <c r="P178" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q178" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R178" s="2" t="n">
@@ -16144,11 +16144,11 @@
         </is>
       </c>
       <c r="P179" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q179" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R179" s="2" t="n">
@@ -16232,11 +16232,11 @@
         </is>
       </c>
       <c r="P180" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q180" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R180" s="2" t="n">
@@ -16320,11 +16320,11 @@
         </is>
       </c>
       <c r="P181" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q181" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R181" s="2" t="n">
@@ -16408,11 +16408,11 @@
         </is>
       </c>
       <c r="P182" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R182" s="2" t="n">
@@ -16496,11 +16496,11 @@
         </is>
       </c>
       <c r="P183" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q183" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R183" s="2" t="n">
@@ -16584,11 +16584,11 @@
         </is>
       </c>
       <c r="P184" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q184" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R184" s="2" t="n">
@@ -16672,11 +16672,11 @@
         </is>
       </c>
       <c r="P185" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q185" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R185" s="2" t="n">
@@ -16760,11 +16760,11 @@
         </is>
       </c>
       <c r="P186" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q186" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R186" s="2" t="n">
@@ -16848,11 +16848,11 @@
         </is>
       </c>
       <c r="P187" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q187" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R187" s="2" t="n">
@@ -16936,11 +16936,11 @@
         </is>
       </c>
       <c r="P188" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R188" s="2" t="n">
@@ -17024,11 +17024,11 @@
         </is>
       </c>
       <c r="P189" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R189" s="2" t="n">
@@ -17110,11 +17110,11 @@
         </is>
       </c>
       <c r="P190" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q190" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R190" s="2" t="n">
@@ -17179,10 +17179,10 @@
         <v>21</v>
       </c>
       <c r="K191" t="n">
-        <v>22</v>
+        <v>21.2</v>
       </c>
       <c r="L191" t="n">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="M191" t="inlineStr">
         <is>
@@ -17198,11 +17198,11 @@
         </is>
       </c>
       <c r="P191" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q191" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R191" s="2" t="n">
@@ -17212,7 +17212,7 @@
         <v>21</v>
       </c>
       <c r="T191" t="n">
-        <v>1</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U191" t="n">
         <v>21.2</v>
@@ -17286,11 +17286,11 @@
         </is>
       </c>
       <c r="P192" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q192" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R192" s="2" t="n">
@@ -17372,11 +17372,11 @@
         </is>
       </c>
       <c r="P193" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R193" s="2" t="n">
@@ -17460,11 +17460,11 @@
         </is>
       </c>
       <c r="P194" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q194" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R194" s="2" t="n">
@@ -17548,11 +17548,11 @@
         </is>
       </c>
       <c r="P195" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q195" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R195" s="2" t="n">
@@ -17634,11 +17634,11 @@
         </is>
       </c>
       <c r="P196" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q196" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R196" s="2" t="n">
@@ -17722,11 +17722,11 @@
         </is>
       </c>
       <c r="P197" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q197" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R197" s="2" t="n">
@@ -17810,11 +17810,11 @@
         </is>
       </c>
       <c r="P198" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q198" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R198" s="2" t="n">
@@ -17898,11 +17898,11 @@
         </is>
       </c>
       <c r="P199" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q199" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R199" s="2" t="n">
@@ -17986,11 +17986,11 @@
         </is>
       </c>
       <c r="P200" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R200" s="2" t="n">
@@ -18055,10 +18055,10 @@
         <v>28</v>
       </c>
       <c r="K201" t="n">
-        <v>28.7</v>
+        <v>27.6</v>
       </c>
       <c r="L201" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M201" t="inlineStr">
         <is>
@@ -18074,11 +18074,11 @@
         </is>
       </c>
       <c r="P201" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q201" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R201" s="2" t="n">
@@ -18088,7 +18088,7 @@
         <v>28</v>
       </c>
       <c r="T201" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U201" t="n">
         <v>28</v>
@@ -18143,10 +18143,10 @@
         <v>21</v>
       </c>
       <c r="K202" t="n">
-        <v>20.8</v>
+        <v>21.4</v>
       </c>
       <c r="L202" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M202" t="inlineStr">
         <is>
@@ -18162,11 +18162,11 @@
         </is>
       </c>
       <c r="P202" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q202" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R202" s="2" t="n">
@@ -18176,7 +18176,7 @@
         <v>21</v>
       </c>
       <c r="T202" t="n">
-        <v>-0.1999999999999993</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U202" t="n">
         <v>21.16666666666667</v>
@@ -18250,11 +18250,11 @@
         </is>
       </c>
       <c r="P203" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q203" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R203" s="2" t="n">
@@ -18338,11 +18338,11 @@
         </is>
       </c>
       <c r="P204" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q204" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R204" s="2" t="n">
@@ -18426,11 +18426,11 @@
         </is>
       </c>
       <c r="P205" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q205" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R205" s="2" t="n">
@@ -18514,11 +18514,11 @@
         </is>
       </c>
       <c r="P206" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q206" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R206" s="2" t="n">
@@ -18583,10 +18583,10 @@
         <v>28</v>
       </c>
       <c r="K207" t="n">
-        <v>27.7</v>
+        <v>28.9</v>
       </c>
       <c r="L207" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="M207" t="inlineStr">
         <is>
@@ -18602,11 +18602,11 @@
         </is>
       </c>
       <c r="P207" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q207" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R207" s="2" t="n">
@@ -18616,7 +18616,7 @@
         <v>28</v>
       </c>
       <c r="T207" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U207" t="n">
         <v>28.4</v>
@@ -18690,11 +18690,11 @@
         </is>
       </c>
       <c r="P208" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q208" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R208" s="2" t="n">
@@ -18778,11 +18778,11 @@
         </is>
       </c>
       <c r="P209" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q209" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R209" s="2" t="n">
@@ -18866,11 +18866,11 @@
         </is>
       </c>
       <c r="P210" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q210" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R210" s="2" t="n">
@@ -18954,11 +18954,11 @@
         </is>
       </c>
       <c r="P211" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q211" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R211" s="2" t="n">
@@ -19042,11 +19042,11 @@
         </is>
       </c>
       <c r="P212" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q212" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R212" s="2" t="n">
@@ -19130,11 +19130,11 @@
         </is>
       </c>
       <c r="P213" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q213" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R213" s="2" t="n">
@@ -19218,11 +19218,11 @@
         </is>
       </c>
       <c r="P214" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q214" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R214" s="2" t="n">
@@ -19306,11 +19306,11 @@
         </is>
       </c>
       <c r="P215" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q215" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R215" s="2" t="n">
@@ -19392,11 +19392,11 @@
         </is>
       </c>
       <c r="P216" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q216" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R216" s="2" t="n">
@@ -19480,11 +19480,11 @@
         </is>
       </c>
       <c r="P217" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q217" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R217" s="2" t="n">
@@ -19568,11 +19568,11 @@
         </is>
       </c>
       <c r="P218" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q218" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R218" s="2" t="n">
@@ -19656,11 +19656,11 @@
         </is>
       </c>
       <c r="P219" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q219" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R219" s="2" t="n">
@@ -19744,11 +19744,11 @@
         </is>
       </c>
       <c r="P220" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q220" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R220" s="2" t="n">
@@ -19832,11 +19832,11 @@
         </is>
       </c>
       <c r="P221" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q221" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R221" s="2" t="n">
@@ -19920,11 +19920,11 @@
         </is>
       </c>
       <c r="P222" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q222" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R222" s="2" t="n">
@@ -20008,11 +20008,11 @@
         </is>
       </c>
       <c r="P223" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q223" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R223" s="2" t="n">
@@ -20096,11 +20096,11 @@
         </is>
       </c>
       <c r="P224" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q224" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R224" s="2" t="n">
@@ -20184,11 +20184,11 @@
         </is>
       </c>
       <c r="P225" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q225" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R225" s="2" t="n">
@@ -20272,11 +20272,11 @@
         </is>
       </c>
       <c r="P226" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q226" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R226" s="2" t="n">
@@ -20360,11 +20360,11 @@
         </is>
       </c>
       <c r="P227" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q227" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R227" s="2" t="n">
@@ -20448,11 +20448,11 @@
         </is>
       </c>
       <c r="P228" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q228" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R228" s="2" t="n">
@@ -20536,11 +20536,11 @@
         </is>
       </c>
       <c r="P229" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q229" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R229" s="2" t="n">
@@ -20624,11 +20624,11 @@
         </is>
       </c>
       <c r="P230" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q230" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R230" s="2" t="n">
@@ -20710,11 +20710,11 @@
         </is>
       </c>
       <c r="P231" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q231" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R231" s="2" t="n">
@@ -20798,11 +20798,11 @@
         </is>
       </c>
       <c r="P232" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q232" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R232" s="2" t="n">
@@ -20886,11 +20886,11 @@
         </is>
       </c>
       <c r="P233" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q233" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R233" s="2" t="n">
@@ -20974,11 +20974,11 @@
         </is>
       </c>
       <c r="P234" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q234" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R234" s="2" t="n">
@@ -21060,11 +21060,11 @@
         </is>
       </c>
       <c r="P235" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q235" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R235" s="2" t="n">
@@ -21148,11 +21148,11 @@
         </is>
       </c>
       <c r="P236" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q236" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R236" s="2" t="n">
@@ -21234,11 +21234,11 @@
         </is>
       </c>
       <c r="P237" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q237" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R237" s="2" t="n">
@@ -21322,11 +21322,11 @@
         </is>
       </c>
       <c r="P238" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q238" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R238" s="2" t="n">
@@ -21410,11 +21410,11 @@
         </is>
       </c>
       <c r="P239" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q239" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R239" s="2" t="n">
@@ -21498,11 +21498,11 @@
         </is>
       </c>
       <c r="P240" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q240" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R240" s="2" t="n">
@@ -21584,11 +21584,11 @@
         </is>
       </c>
       <c r="P241" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q241" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R241" s="2" t="n">
@@ -21672,11 +21672,11 @@
         </is>
       </c>
       <c r="P242" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q242" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R242" s="2" t="n">
@@ -21760,11 +21760,11 @@
         </is>
       </c>
       <c r="P243" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q243" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R243" s="2" t="n">
@@ -21848,11 +21848,11 @@
         </is>
       </c>
       <c r="P244" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q244" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R244" s="2" t="n">
@@ -21936,11 +21936,11 @@
         </is>
       </c>
       <c r="P245" s="2" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="Q245" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R245" s="2" t="n">

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-10 18:35:26
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5073,10 +5073,10 @@
         <v>31</v>
       </c>
       <c r="K53" t="n">
-        <v>38.5</v>
+        <v>30.5</v>
       </c>
       <c r="L53" t="n">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="M53" t="inlineStr">
         <is>
@@ -5104,7 +5104,7 @@
       </c>
       <c r="S53" t="inlineStr"/>
       <c r="T53" t="n">
-        <v>7.5</v>
+        <v>-0.5</v>
       </c>
       <c r="U53" t="n">
         <v>35.86666666666667</v>
@@ -5159,10 +5159,10 @@
         <v>24</v>
       </c>
       <c r="K54" t="n">
-        <v>22.8</v>
+        <v>25.3</v>
       </c>
       <c r="L54" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="M54" t="inlineStr">
         <is>
@@ -5192,7 +5192,7 @@
         <v>28</v>
       </c>
       <c r="T54" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="U54" t="n">
         <v>24.6</v>
@@ -5247,10 +5247,10 @@
         <v>24</v>
       </c>
       <c r="K55" t="n">
-        <v>21.2</v>
+        <v>25</v>
       </c>
       <c r="L55" t="n">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
         <v>28</v>
       </c>
       <c r="T55" t="n">
-        <v>-2.800000000000001</v>
+        <v>1</v>
       </c>
       <c r="U55" t="n">
         <v>22.7</v>
@@ -5335,10 +5335,10 @@
         <v>31</v>
       </c>
       <c r="K56" t="n">
-        <v>18.8</v>
+        <v>37.1</v>
       </c>
       <c r="L56" t="n">
-        <v>61</v>
+        <v>120</v>
       </c>
       <c r="M56" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="n">
-        <v>-12.2</v>
+        <v>6.100000000000001</v>
       </c>
       <c r="U56" t="n">
         <v>31.73333333333333</v>
@@ -5421,10 +5421,10 @@
         <v>24</v>
       </c>
       <c r="K57" t="n">
-        <v>20.8</v>
+        <v>22.4</v>
       </c>
       <c r="L57" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
@@ -5454,7 +5454,7 @@
         <v>28</v>
       </c>
       <c r="T57" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U57" t="n">
         <v>21.53333333333333</v>
@@ -5509,10 +5509,10 @@
         <v>24</v>
       </c>
       <c r="K58" t="n">
-        <v>25.5</v>
+        <v>15.3</v>
       </c>
       <c r="L58" t="n">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -5542,7 +5542,7 @@
         <v>28</v>
       </c>
       <c r="T58" t="n">
-        <v>1.5</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="U58" t="n">
         <v>22.46666666666667</v>
@@ -5597,10 +5597,10 @@
         <v>31</v>
       </c>
       <c r="K59" t="n">
-        <v>31.4</v>
+        <v>24.8</v>
       </c>
       <c r="L59" t="n">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
@@ -5628,10 +5628,10 @@
       </c>
       <c r="S59" t="inlineStr"/>
       <c r="T59" t="n">
-        <v>0.3999999999999986</v>
+        <v>-6.199999999999999</v>
       </c>
       <c r="U59" t="n">
-        <v>30.66666666666666</v>
+        <v>30.66666666666667</v>
       </c>
       <c r="V59" t="n">
         <v>3</v>
@@ -5683,10 +5683,10 @@
         <v>24</v>
       </c>
       <c r="K60" t="n">
-        <v>22.1</v>
+        <v>24.7</v>
       </c>
       <c r="L60" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
@@ -5716,7 +5716,7 @@
         <v>28</v>
       </c>
       <c r="T60" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U60" t="n">
         <v>23.8</v>
@@ -5771,10 +5771,10 @@
         <v>24</v>
       </c>
       <c r="K61" t="n">
-        <v>23.1</v>
+        <v>25.9</v>
       </c>
       <c r="L61" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
@@ -5804,7 +5804,7 @@
         <v>28</v>
       </c>
       <c r="T61" t="n">
-        <v>-0.8999999999999986</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U61" t="n">
         <v>24.1</v>
@@ -5859,10 +5859,10 @@
         <v>24</v>
       </c>
       <c r="K62" t="n">
-        <v>16.6</v>
+        <v>26.4</v>
       </c>
       <c r="L62" t="n">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
@@ -5892,7 +5892,7 @@
         <v>28</v>
       </c>
       <c r="T62" t="n">
-        <v>-7.399999999999999</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U62" t="n">
         <v>23.4</v>
@@ -5947,10 +5947,10 @@
         <v>24</v>
       </c>
       <c r="K63" t="n">
-        <v>25.7</v>
+        <v>23.4</v>
       </c>
       <c r="L63" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="M63" t="inlineStr">
         <is>
@@ -5980,7 +5980,7 @@
         <v>28</v>
       </c>
       <c r="T63" t="n">
-        <v>1.699999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U63" t="n">
         <v>24.46666666666667</v>
@@ -6035,10 +6035,10 @@
         <v>28</v>
       </c>
       <c r="K64" t="n">
-        <v>30.4</v>
+        <v>31.6</v>
       </c>
       <c r="L64" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
@@ -6068,7 +6068,7 @@
         <v>28</v>
       </c>
       <c r="T64" t="n">
-        <v>2.399999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U64" t="n">
         <v>29.86666666666666</v>
@@ -10067,10 +10067,10 @@
         <v>35</v>
       </c>
       <c r="K110" t="n">
-        <v>27.1</v>
+        <v>29.6</v>
       </c>
       <c r="L110" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="M110" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
         <v>41</v>
       </c>
       <c r="T110" t="n">
-        <v>-7.899999999999999</v>
+        <v>-5.399999999999999</v>
       </c>
       <c r="U110" t="n">
         <v>27.33333333333333</v>
@@ -10155,10 +10155,10 @@
         <v>35</v>
       </c>
       <c r="K111" t="n">
-        <v>49.1</v>
+        <v>31.4</v>
       </c>
       <c r="L111" t="n">
-        <v>140</v>
+        <v>90</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -10188,7 +10188,7 @@
         <v>41</v>
       </c>
       <c r="T111" t="n">
-        <v>14.1</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="U111" t="n">
         <v>43.96666666666667</v>
@@ -10243,10 +10243,10 @@
         <v>35</v>
       </c>
       <c r="K112" t="n">
-        <v>27.3</v>
+        <v>54.5</v>
       </c>
       <c r="L112" t="n">
-        <v>78</v>
+        <v>156</v>
       </c>
       <c r="M112" t="inlineStr">
         <is>
@@ -10276,16 +10276,16 @@
         <v>41</v>
       </c>
       <c r="T112" t="n">
-        <v>-7.699999999999999</v>
+        <v>19.5</v>
       </c>
       <c r="U112" t="n">
-        <v>44.9</v>
+        <v>44.90000000000001</v>
       </c>
       <c r="V112" t="n">
         <v>3</v>
       </c>
       <c r="W112" t="n">
-        <v>41.74444444444444</v>
+        <v>41.74444444444445</v>
       </c>
       <c r="X112" t="n">
         <v>31.5</v>
@@ -10331,10 +10331,10 @@
         <v>21</v>
       </c>
       <c r="K113" t="n">
-        <v>24.3</v>
+        <v>19.9</v>
       </c>
       <c r="L113" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="M113" t="inlineStr">
         <is>
@@ -10364,16 +10364,16 @@
         <v>21</v>
       </c>
       <c r="T113" t="n">
-        <v>3.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U113" t="n">
-        <v>22.56666666666666</v>
+        <v>22.56666666666667</v>
       </c>
       <c r="V113" t="n">
         <v>3</v>
       </c>
       <c r="W113" t="n">
-        <v>36.05555555555555</v>
+        <v>36.05555555555556</v>
       </c>
       <c r="X113" t="n">
         <v>17.5</v>
@@ -10507,10 +10507,10 @@
         <v>28</v>
       </c>
       <c r="K115" t="n">
-        <v>32.7</v>
+        <v>26.4</v>
       </c>
       <c r="L115" t="n">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         <v>28</v>
       </c>
       <c r="T115" t="n">
-        <v>4.700000000000003</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U115" t="n">
         <v>29.6</v>
@@ -22697,10 +22697,10 @@
         <v>21</v>
       </c>
       <c r="K254" t="n">
-        <v>42.6</v>
+        <v>16.6</v>
       </c>
       <c r="L254" t="n">
-        <v>203</v>
+        <v>79</v>
       </c>
       <c r="M254" t="inlineStr">
         <is>
@@ -22730,7 +22730,7 @@
         <v>21</v>
       </c>
       <c r="T254" t="n">
-        <v>21.6</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="U254" t="n">
         <v>36.33333333333334</v>
@@ -23137,10 +23137,10 @@
         <v>28</v>
       </c>
       <c r="K259" t="n">
-        <v>27.1</v>
+        <v>27.6</v>
       </c>
       <c r="L259" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M259" t="inlineStr">
         <is>
@@ -23170,7 +23170,7 @@
         <v>28</v>
       </c>
       <c r="T259" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U259" t="n">
         <v>27.4</v>
@@ -23225,10 +23225,10 @@
         <v>28</v>
       </c>
       <c r="K260" t="n">
-        <v>28.1</v>
+        <v>28.9</v>
       </c>
       <c r="L260" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="M260" t="inlineStr">
         <is>
@@ -23258,7 +23258,7 @@
         <v>28</v>
       </c>
       <c r="T260" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U260" t="n">
         <v>28.03333333333333</v>
@@ -23313,10 +23313,10 @@
         <v>28</v>
       </c>
       <c r="K261" t="n">
-        <v>28.4</v>
+        <v>27.2</v>
       </c>
       <c r="L261" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M261" t="inlineStr">
         <is>
@@ -23346,10 +23346,10 @@
         <v>28</v>
       </c>
       <c r="T261" t="n">
-        <v>0.3999999999999986</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U261" t="n">
-        <v>28.06666666666667</v>
+        <v>28.06666666666666</v>
       </c>
       <c r="V261" t="n">
         <v>3</v>
@@ -24143,7 +24143,7 @@
         <v>3</v>
       </c>
       <c r="W270" t="n">
-        <v>28.15555555555556</v>
+        <v>28.15555555555555</v>
       </c>
       <c r="X270" t="n">
         <v>24.5</v>
@@ -24493,7 +24493,7 @@
         <v>3</v>
       </c>
       <c r="W274" t="n">
-        <v>32.9888888888889</v>
+        <v>32.98888888888889</v>
       </c>
       <c r="X274" t="n">
         <v>24.5</v>
@@ -26469,10 +26469,10 @@
         <v>21</v>
       </c>
       <c r="K297" t="n">
-        <v>20.8</v>
+        <v>20.1</v>
       </c>
       <c r="L297" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="M297" t="inlineStr">
         <is>
@@ -26502,7 +26502,7 @@
         <v>21</v>
       </c>
       <c r="T297" t="n">
-        <v>-0.1999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U297" t="n">
         <v>20.3</v>
@@ -27873,10 +27873,10 @@
         <v>24.5</v>
       </c>
       <c r="K313" t="n">
-        <v>23.3</v>
+        <v>25.8</v>
       </c>
       <c r="L313" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="M313" t="inlineStr">
         <is>
@@ -27906,7 +27906,7 @@
         <v>28</v>
       </c>
       <c r="T313" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="U313" t="n">
         <v>24.26666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-10 23:17:13
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2987,10 +2987,10 @@
         <v>31</v>
       </c>
       <c r="K29" t="n">
-        <v>29.3</v>
+        <v>31.1</v>
       </c>
       <c r="L29" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="n">
-        <v>-1.699999999999999</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U29" t="n">
         <v>31.2</v>
@@ -6123,10 +6123,10 @@
         <v>28</v>
       </c>
       <c r="K65" t="n">
-        <v>27.9</v>
+        <v>30.5</v>
       </c>
       <c r="L65" t="n">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v>28</v>
       </c>
       <c r="T65" t="n">
-        <v>-0.1000000000000014</v>
+        <v>2.5</v>
       </c>
       <c r="U65" t="n">
         <v>29.13333333333334</v>
@@ -7091,10 +7091,10 @@
         <v>31</v>
       </c>
       <c r="K76" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L76" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U76" t="n">
         <v>32.03333333333333</v>
@@ -7441,10 +7441,10 @@
         <v>31</v>
       </c>
       <c r="K80" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L80" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7472,7 +7472,7 @@
       </c>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U80" t="n">
         <v>36</v>
@@ -8055,10 +8055,10 @@
         <v>31</v>
       </c>
       <c r="K87" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L87" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M87" t="inlineStr">
         <is>
@@ -8086,7 +8086,7 @@
       </c>
       <c r="S87" t="inlineStr"/>
       <c r="T87" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U87" t="n">
         <v>33.63333333333333</v>
@@ -8493,10 +8493,10 @@
         <v>31</v>
       </c>
       <c r="K92" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L92" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="S92" t="inlineStr"/>
       <c r="T92" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U92" t="n">
         <v>32.76666666666667</v>
@@ -9715,10 +9715,10 @@
         <v>35</v>
       </c>
       <c r="K106" t="n">
-        <v>39.5</v>
+        <v>38</v>
       </c>
       <c r="L106" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="M106" t="inlineStr">
         <is>
@@ -9748,7 +9748,7 @@
         <v>41</v>
       </c>
       <c r="T106" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="U106" t="n">
         <v>37.06666666666667</v>
@@ -15071,10 +15071,10 @@
         <v>35</v>
       </c>
       <c r="K167" t="n">
-        <v>37.2</v>
+        <v>34.7</v>
       </c>
       <c r="L167" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="M167" t="inlineStr">
         <is>
@@ -15104,7 +15104,7 @@
         <v>41</v>
       </c>
       <c r="T167" t="n">
-        <v>2.200000000000003</v>
+        <v>-0.2999999999999972</v>
       </c>
       <c r="U167" t="n">
         <v>37.26666666666667</v>
@@ -15159,10 +15159,10 @@
         <v>21</v>
       </c>
       <c r="K168" t="n">
-        <v>23.4</v>
+        <v>20.8</v>
       </c>
       <c r="L168" t="n">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="M168" t="inlineStr">
         <is>
@@ -15192,7 +15192,7 @@
         <v>21</v>
       </c>
       <c r="T168" t="n">
-        <v>2.399999999999999</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U168" t="n">
         <v>23.4</v>
@@ -15335,10 +15335,10 @@
         <v>35</v>
       </c>
       <c r="K170" t="n">
-        <v>39.3</v>
+        <v>34</v>
       </c>
       <c r="L170" t="n">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="M170" t="inlineStr">
         <is>
@@ -15368,7 +15368,7 @@
         <v>41</v>
       </c>
       <c r="T170" t="n">
-        <v>4.299999999999997</v>
+        <v>-1</v>
       </c>
       <c r="U170" t="n">
         <v>36.3</v>
@@ -15423,10 +15423,10 @@
         <v>28</v>
       </c>
       <c r="K171" t="n">
-        <v>24.8</v>
+        <v>27</v>
       </c>
       <c r="L171" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="M171" t="inlineStr">
         <is>
@@ -15456,7 +15456,7 @@
         <v>28</v>
       </c>
       <c r="T171" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1</v>
       </c>
       <c r="U171" t="n">
         <v>26.4</v>
@@ -21741,10 +21741,10 @@
         <v>21</v>
       </c>
       <c r="K243" t="n">
-        <v>19.7</v>
+        <v>21.7</v>
       </c>
       <c r="L243" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="M243" t="inlineStr">
         <is>
@@ -21774,7 +21774,7 @@
         <v>21</v>
       </c>
       <c r="T243" t="n">
-        <v>-1.300000000000001</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U243" t="n">
         <v>21</v>
@@ -23665,10 +23665,10 @@
         <v>28</v>
       </c>
       <c r="K265" t="n">
-        <v>32.3</v>
+        <v>29.9</v>
       </c>
       <c r="L265" t="n">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="M265" t="inlineStr">
         <is>
@@ -23698,7 +23698,7 @@
         <v>28</v>
       </c>
       <c r="T265" t="n">
-        <v>4.299999999999997</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U265" t="n">
         <v>28.53333333333333</v>
@@ -25243,10 +25243,10 @@
         <v>21</v>
       </c>
       <c r="K283" t="n">
-        <v>19.8</v>
+        <v>24</v>
       </c>
       <c r="L283" t="n">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="M283" t="inlineStr">
         <is>
@@ -25276,7 +25276,7 @@
         <v>21</v>
       </c>
       <c r="T283" t="n">
-        <v>-1.199999999999999</v>
+        <v>3</v>
       </c>
       <c r="U283" t="n">
         <v>22.96666666666667</v>
@@ -25767,10 +25767,10 @@
         <v>21</v>
       </c>
       <c r="K289" t="n">
-        <v>25.9</v>
+        <v>22.6</v>
       </c>
       <c r="L289" t="n">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="M289" t="inlineStr">
         <is>
@@ -25800,7 +25800,7 @@
         <v>21</v>
       </c>
       <c r="T289" t="n">
-        <v>4.899999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U289" t="n">
         <v>22.7</v>
@@ -25943,10 +25943,10 @@
         <v>21</v>
       </c>
       <c r="K291" t="n">
-        <v>22.2</v>
+        <v>20.9</v>
       </c>
       <c r="L291" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="M291" t="inlineStr">
         <is>
@@ -25976,7 +25976,7 @@
         <v>21</v>
       </c>
       <c r="T291" t="n">
-        <v>1.199999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U291" t="n">
         <v>22.03333333333333</v>
@@ -26995,10 +26995,10 @@
         <v>21</v>
       </c>
       <c r="K303" t="n">
-        <v>20.4</v>
+        <v>21.2</v>
       </c>
       <c r="L303" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="M303" t="inlineStr">
         <is>
@@ -27028,16 +27028,16 @@
         <v>21</v>
       </c>
       <c r="T303" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U303" t="n">
-        <v>21.16666666666667</v>
+        <v>21.16666666666666</v>
       </c>
       <c r="V303" t="n">
         <v>3</v>
       </c>
       <c r="W303" t="n">
-        <v>22.05555555555556</v>
+        <v>22.05555555555555</v>
       </c>
       <c r="X303" t="n">
         <v>17.5</v>
@@ -28313,10 +28313,10 @@
         <v>24.5</v>
       </c>
       <c r="K318" t="n">
-        <v>24.6</v>
+        <v>20.9</v>
       </c>
       <c r="L318" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="M318" t="inlineStr">
         <is>
@@ -28346,7 +28346,7 @@
         <v>28</v>
       </c>
       <c r="T318" t="n">
-        <v>0.1000000000000014</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="U318" t="n">
         <v>23.96666666666667</v>
@@ -28665,10 +28665,10 @@
         <v>24.5</v>
       </c>
       <c r="K322" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L322" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M322" t="inlineStr">
         <is>
@@ -28698,7 +28698,7 @@
         <v>28</v>
       </c>
       <c r="T322" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U322" t="n">
         <v>24.66666666666667</v>
@@ -29369,10 +29369,10 @@
         <v>24.5</v>
       </c>
       <c r="K330" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L330" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M330" t="inlineStr">
         <is>
@@ -29402,7 +29402,7 @@
         <v>28</v>
       </c>
       <c r="T330" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U330" t="n">
         <v>27.1</v>
@@ -31305,10 +31305,10 @@
         <v>24.5</v>
       </c>
       <c r="K352" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L352" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M352" t="inlineStr">
         <is>
@@ -31338,10 +31338,10 @@
         <v>28</v>
       </c>
       <c r="T352" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U352" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V352" t="n">
         <v>3</v>
@@ -32267,10 +32267,10 @@
         <v>21</v>
       </c>
       <c r="K363" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="L363" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M363" t="inlineStr">
         <is>
@@ -32300,7 +32300,7 @@
         <v>21</v>
       </c>
       <c r="T363" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U363" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-11 23:34:03
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3505,10 +3505,10 @@
         <v>31</v>
       </c>
       <c r="K35" t="n">
-        <v>38.5</v>
+        <v>27.8</v>
       </c>
       <c r="L35" t="n">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="n">
-        <v>7.5</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U35" t="n">
         <v>35.83333333333334</v>
@@ -3591,10 +3591,10 @@
         <v>28</v>
       </c>
       <c r="K36" t="n">
-        <v>22.1</v>
+        <v>33.2</v>
       </c>
       <c r="L36" t="n">
-        <v>79</v>
+        <v>118</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3624,7 +3624,7 @@
         <v>28</v>
       </c>
       <c r="T36" t="n">
-        <v>-5.899999999999999</v>
+        <v>5.200000000000003</v>
       </c>
       <c r="U36" t="n">
         <v>30.1</v>
@@ -3679,10 +3679,10 @@
         <v>31</v>
       </c>
       <c r="K37" t="n">
-        <v>32.6</v>
+        <v>30.9</v>
       </c>
       <c r="L37" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="n">
-        <v>1.600000000000001</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U37" t="n">
         <v>30.8</v>
@@ -3719,7 +3719,7 @@
         <v>3</v>
       </c>
       <c r="W37" t="n">
-        <v>41.12222222222223</v>
+        <v>41.12222222222222</v>
       </c>
       <c r="X37" t="n">
         <v>27.5</v>
@@ -4113,10 +4113,10 @@
         <v>31</v>
       </c>
       <c r="K42" t="n">
-        <v>32</v>
+        <v>29.7</v>
       </c>
       <c r="L42" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M42" t="inlineStr">
         <is>
@@ -4144,7 +4144,7 @@
       </c>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="n">
-        <v>1</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U42" t="n">
         <v>30.33333333333333</v>
@@ -6475,10 +6475,10 @@
         <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>31.8</v>
+        <v>38.1</v>
       </c>
       <c r="L69" t="n">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>41</v>
       </c>
       <c r="T69" t="n">
-        <v>-3.199999999999999</v>
+        <v>3.100000000000001</v>
       </c>
       <c r="U69" t="n">
         <v>35.3</v>
@@ -9105,10 +9105,10 @@
         <v>35</v>
       </c>
       <c r="K99" t="n">
-        <v>38.4</v>
+        <v>37.1</v>
       </c>
       <c r="L99" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M99" t="inlineStr">
         <is>
@@ -9138,7 +9138,7 @@
         <v>41</v>
       </c>
       <c r="T99" t="n">
-        <v>3.399999999999999</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="U99" t="n">
         <v>36.5</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-12 03:45:11
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -610,11 +610,11 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
@@ -698,11 +698,11 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R3" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S3" t="n">
         <v>28</v>
@@ -788,11 +788,11 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
@@ -876,11 +876,11 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R5" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S5" t="n">
         <v>48</v>
@@ -966,11 +966,11 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S6" t="n">
         <v>41</v>
@@ -1056,11 +1056,11 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R7" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S7" t="n">
         <v>48</v>
@@ -1146,11 +1146,11 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S8" t="n">
         <v>41</v>
@@ -1236,11 +1236,11 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R9" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
@@ -1324,11 +1324,11 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
@@ -1412,11 +1412,11 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R11" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="n">
@@ -1500,11 +1500,11 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S12" t="n">
         <v>21</v>
@@ -1590,11 +1590,11 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R13" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="n">
@@ -1678,11 +1678,11 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="n">
@@ -1766,11 +1766,11 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R15" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="n">
@@ -1854,11 +1854,11 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S16" t="n">
         <v>34</v>
@@ -1944,11 +1944,11 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R17" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="n">
@@ -2032,11 +2032,11 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S18" t="n">
         <v>48</v>
@@ -2120,11 +2120,11 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R19" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S19" t="n">
         <v>48</v>
@@ -2210,11 +2210,11 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S20" t="n">
         <v>34</v>
@@ -2300,11 +2300,11 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R21" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S21" t="n">
         <v>28</v>
@@ -2390,11 +2390,11 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S22" t="n">
         <v>28</v>
@@ -2480,11 +2480,11 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R23" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S23" t="n">
         <v>28</v>
@@ -2570,11 +2570,11 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S24" t="n">
         <v>28</v>
@@ -2658,11 +2658,11 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R25" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="n">
@@ -2746,11 +2746,11 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S26" t="n">
         <v>28</v>
@@ -2834,11 +2834,11 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R27" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="n">
@@ -2920,11 +2920,11 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S28" t="n">
         <v>21</v>
@@ -3008,11 +3008,11 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R29" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S29" t="n">
         <v>21</v>
@@ -3096,11 +3096,11 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="n">
@@ -3182,11 +3182,11 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R31" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="n">
@@ -3268,11 +3268,11 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="n">
@@ -3354,11 +3354,11 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R33" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S34" t="n">
         <v>21</v>
@@ -3528,11 +3528,11 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R35" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S35" t="n">
         <v>21</v>
@@ -3616,11 +3616,11 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S36" t="n">
         <v>28</v>
@@ -3704,11 +3704,11 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R37" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S37" t="n">
         <v>28</v>
@@ -3792,11 +3792,11 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R38" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S38" t="n">
         <v>28</v>
@@ -3880,11 +3880,11 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R39" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S39" t="n">
         <v>28</v>
@@ -3968,11 +3968,11 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R40" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S40" t="n">
         <v>28</v>
@@ -4056,11 +4056,11 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R41" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S41" t="n">
         <v>28</v>
@@ -4144,11 +4144,11 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R42" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S42" t="n">
         <v>28</v>
@@ -4232,11 +4232,11 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R43" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S43" t="n">
         <v>28</v>
@@ -4320,11 +4320,11 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R44" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S44" t="n">
         <v>28</v>
@@ -4408,11 +4408,11 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R45" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S45" t="n">
         <v>28</v>
@@ -4496,11 +4496,11 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R46" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S46" t="n">
         <v>28</v>
@@ -4582,11 +4582,11 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R47" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S47" t="n">
         <v>28</v>
@@ -4670,11 +4670,11 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R48" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S48" t="n">
         <v>28</v>
@@ -4756,11 +4756,11 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R49" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S49" t="n">
         <v>28</v>
@@ -4844,11 +4844,11 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R50" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S50" t="n">
         <v>28</v>
@@ -4932,11 +4932,11 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R51" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S51" t="n">
         <v>28</v>
@@ -5020,11 +5020,11 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R52" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S52" t="n">
         <v>28</v>
@@ -5194,11 +5194,11 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R54" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S54" t="n">
         <v>21</v>
@@ -5282,11 +5282,11 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R55" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S55" t="n">
         <v>28</v>
@@ -5347,10 +5347,10 @@
         <v>28</v>
       </c>
       <c r="K56" t="n">
-        <v>27.6</v>
+        <v>32.5</v>
       </c>
       <c r="L56" t="n">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="M56" t="inlineStr">
         <is>
@@ -5370,17 +5370,17 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R56" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S56" t="n">
         <v>28</v>
       </c>
       <c r="T56" t="n">
-        <v>-0.3999999999999986</v>
+        <v>4.5</v>
       </c>
       <c r="U56" t="n">
         <v>30.16666666666667</v>
@@ -5458,11 +5458,11 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R57" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S57" t="n">
         <v>28</v>
@@ -5546,11 +5546,11 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R58" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S58" t="n">
         <v>28</v>
@@ -5634,11 +5634,11 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R59" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S59" t="n">
         <v>28</v>
@@ -5722,11 +5722,11 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R60" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S60" t="n">
         <v>28</v>
@@ -5810,11 +5810,11 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R61" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S61" t="n">
         <v>28</v>
@@ -5898,11 +5898,11 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R62" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S62" t="n">
         <v>21</v>
@@ -5986,11 +5986,11 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R63" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S63" t="n">
         <v>21</v>
@@ -6074,11 +6074,11 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R64" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S64" t="n">
         <v>21</v>
@@ -6162,11 +6162,11 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R65" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S65" t="n">
         <v>21</v>
@@ -6250,11 +6250,11 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R66" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S66" t="n">
         <v>21</v>
@@ -6338,11 +6338,11 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R67" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S67" t="n">
         <v>21</v>
@@ -6426,11 +6426,11 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R68" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S68" t="n">
         <v>21</v>
@@ -6598,11 +6598,11 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R70" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S70" t="n">
         <v>21</v>
@@ -6686,11 +6686,11 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R71" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S71" t="n">
         <v>21</v>
@@ -6774,11 +6774,11 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R72" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S72" t="n">
         <v>21</v>
@@ -6862,11 +6862,11 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R73" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S73" t="n">
         <v>21</v>
@@ -6950,11 +6950,11 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R74" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S74" t="n">
         <v>21</v>
@@ -7038,11 +7038,11 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R75" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S75" t="n">
         <v>21</v>
@@ -7212,11 +7212,11 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R77" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S77" t="n">
         <v>21</v>
@@ -7300,11 +7300,11 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R78" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S78" t="n">
         <v>21</v>
@@ -7388,11 +7388,11 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R79" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S79" t="n">
         <v>21</v>
@@ -7476,11 +7476,11 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R80" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="n">
@@ -7562,11 +7562,11 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R81" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S81" t="n">
         <v>21</v>
@@ -7650,11 +7650,11 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R82" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S82" t="n">
         <v>21</v>
@@ -7738,11 +7738,11 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R83" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S83" t="n">
         <v>21</v>
@@ -7826,11 +7826,11 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R84" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S84" t="n">
         <v>21</v>
@@ -7914,11 +7914,11 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R85" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S85" t="n">
         <v>21</v>
@@ -8002,11 +8002,11 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R86" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S86" t="n">
         <v>21</v>
@@ -8090,11 +8090,11 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R87" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S87" t="n">
         <v>21</v>
@@ -8178,11 +8178,11 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R88" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S88" t="n">
         <v>21</v>
@@ -8266,11 +8266,11 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R89" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S89" t="n">
         <v>21</v>
@@ -8440,11 +8440,11 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R91" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S91" t="n">
         <v>28</v>
@@ -8528,11 +8528,11 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R92" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S92" t="n">
         <v>28</v>
@@ -8616,11 +8616,11 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R93" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S93" t="n">
         <v>28</v>
@@ -8704,11 +8704,11 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R94" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S94" t="n">
         <v>28</v>
@@ -8792,11 +8792,11 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R95" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S95" t="n">
         <v>28</v>
@@ -8880,11 +8880,11 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R96" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S96" t="n">
         <v>28</v>
@@ -8968,11 +8968,11 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R97" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S97" t="n">
         <v>28</v>
@@ -9056,11 +9056,11 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R98" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S98" t="n">
         <v>28</v>
@@ -9144,11 +9144,11 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R99" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S99" t="n">
         <v>28</v>
@@ -9232,11 +9232,11 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R100" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S100" t="n">
         <v>28</v>
@@ -9320,11 +9320,11 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R101" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S101" t="n">
         <v>28</v>
@@ -9408,11 +9408,11 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R102" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S102" t="n">
         <v>28</v>
@@ -9496,11 +9496,11 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R103" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S103" t="n">
         <v>28</v>
@@ -9584,11 +9584,11 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R104" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S104" t="n">
         <v>28</v>
@@ -9672,11 +9672,11 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R105" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S105" t="n">
         <v>28</v>
@@ -9760,11 +9760,11 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R106" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S106" t="n">
         <v>28</v>
@@ -9848,11 +9848,11 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R107" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S107" t="n">
         <v>28</v>
@@ -9936,11 +9936,11 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R108" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S108" t="n">
         <v>28</v>
@@ -10024,11 +10024,11 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R109" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S109" t="n">
         <v>28</v>
@@ -10112,11 +10112,11 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R110" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S110" t="n">
         <v>28</v>
@@ -10200,11 +10200,11 @@
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R111" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S111" t="n">
         <v>28</v>
@@ -10288,11 +10288,11 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R112" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S112" t="n">
         <v>28</v>
@@ -10376,11 +10376,11 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R113" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S113" t="n">
         <v>28</v>
@@ -10464,11 +10464,11 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R114" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S114" t="n">
         <v>28</v>
@@ -10552,11 +10552,11 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R115" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S115" t="n">
         <v>28</v>
@@ -10640,11 +10640,11 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R116" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S116" t="n">
         <v>28</v>
@@ -10728,11 +10728,11 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R117" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S117" t="n">
         <v>28</v>
@@ -10816,11 +10816,11 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R118" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S118" t="n">
         <v>28</v>
@@ -10904,11 +10904,11 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R119" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S119" t="n">
         <v>28</v>
@@ -10992,11 +10992,11 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R120" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S120" t="n">
         <v>28</v>
@@ -11080,11 +11080,11 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R121" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S121" t="n">
         <v>28</v>
@@ -11168,11 +11168,11 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R122" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S122" t="n">
         <v>28</v>
@@ -11256,11 +11256,11 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R123" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S123" t="n">
         <v>28</v>
@@ -11344,11 +11344,11 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R124" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S124" t="n">
         <v>28</v>
@@ -11432,11 +11432,11 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R125" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S125" t="n">
         <v>28</v>
@@ -11520,11 +11520,11 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R126" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S126" t="n">
         <v>28</v>
@@ -11608,11 +11608,11 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R127" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S127" t="n">
         <v>28</v>
@@ -11696,11 +11696,11 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R128" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S128" t="n">
         <v>28</v>
@@ -11784,11 +11784,11 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R129" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S129" t="n">
         <v>28</v>
@@ -11872,11 +11872,11 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R130" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S130" t="n">
         <v>28</v>
@@ -11960,11 +11960,11 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R131" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S131" t="n">
         <v>28</v>
@@ -12048,11 +12048,11 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R132" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S132" t="n">
         <v>28</v>
@@ -12222,11 +12222,11 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R134" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S134" t="n">
         <v>28</v>
@@ -12310,11 +12310,11 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R135" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S135" t="n">
         <v>28</v>
@@ -12398,11 +12398,11 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R136" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S136" t="n">
         <v>28</v>
@@ -12486,11 +12486,11 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R137" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S137" t="n">
         <v>28</v>
@@ -12574,11 +12574,11 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R138" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S138" t="n">
         <v>28</v>
@@ -12662,11 +12662,11 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R139" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S139" t="n">
         <v>28</v>
@@ -12750,11 +12750,11 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R140" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S140" t="n">
         <v>28</v>
@@ -12836,11 +12836,11 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R141" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S141" t="n">
         <v>28</v>
@@ -12924,11 +12924,11 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R142" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S142" t="n">
         <v>28</v>
@@ -13012,11 +13012,11 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R143" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S143" t="inlineStr"/>
       <c r="T143" t="n">
@@ -13098,11 +13098,11 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R144" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S144" t="n">
         <v>21</v>
@@ -13186,11 +13186,11 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R145" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S145" t="inlineStr"/>
       <c r="T145" t="n">
@@ -13272,11 +13272,11 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>EXISTENTE</t>
+          <t>NUEVO</t>
         </is>
       </c>
       <c r="R146" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="S146" t="n">
         <v>21</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-13 03:01:40
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -7091,10 +7091,10 @@
         <v>31</v>
       </c>
       <c r="K76" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L76" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U76" t="n">
         <v>32.03333333333333</v>
@@ -7441,10 +7441,10 @@
         <v>31</v>
       </c>
       <c r="K80" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L80" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7472,7 +7472,7 @@
       </c>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U80" t="n">
         <v>36</v>
@@ -8055,10 +8055,10 @@
         <v>31</v>
       </c>
       <c r="K87" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L87" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M87" t="inlineStr">
         <is>
@@ -8086,7 +8086,7 @@
       </c>
       <c r="S87" t="inlineStr"/>
       <c r="T87" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U87" t="n">
         <v>33.63333333333333</v>
@@ -8493,10 +8493,10 @@
         <v>31</v>
       </c>
       <c r="K92" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L92" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="S92" t="inlineStr"/>
       <c r="T92" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U92" t="n">
         <v>32.76666666666667</v>
@@ -9845,7 +9845,7 @@
         <v>3</v>
       </c>
       <c r="W107" t="n">
-        <v>24.52222222222223</v>
+        <v>24.52222222222222</v>
       </c>
       <c r="X107" t="n">
         <v>17.5</v>
@@ -11299,10 +11299,10 @@
         <v>21</v>
       </c>
       <c r="K124" t="n">
-        <v>22.6</v>
+        <v>18.4</v>
       </c>
       <c r="L124" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11332,10 +11332,10 @@
         <v>21</v>
       </c>
       <c r="T124" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U124" t="n">
-        <v>22.93333333333334</v>
+        <v>22.93333333333333</v>
       </c>
       <c r="V124" t="n">
         <v>3</v>
@@ -11387,10 +11387,10 @@
         <v>21</v>
       </c>
       <c r="K125" t="n">
-        <v>21.6</v>
+        <v>19.4</v>
       </c>
       <c r="L125" t="n">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="M125" t="inlineStr">
         <is>
@@ -11420,7 +11420,7 @@
         <v>21</v>
       </c>
       <c r="T125" t="n">
-        <v>0.6000000000000014</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U125" t="n">
         <v>19.93333333333333</v>
@@ -12529,10 +12529,10 @@
         <v>35</v>
       </c>
       <c r="K138" t="n">
-        <v>45.3</v>
+        <v>45.2</v>
       </c>
       <c r="L138" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M138" t="inlineStr">
         <is>
@@ -12562,7 +12562,7 @@
         <v>41</v>
       </c>
       <c r="T138" t="n">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="U138" t="n">
         <v>41</v>
@@ -12793,10 +12793,10 @@
         <v>35</v>
       </c>
       <c r="K141" t="n">
-        <v>39.7</v>
+        <v>34.7</v>
       </c>
       <c r="L141" t="n">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="M141" t="inlineStr">
         <is>
@@ -12826,10 +12826,10 @@
         <v>41</v>
       </c>
       <c r="T141" t="n">
-        <v>4.700000000000003</v>
+        <v>-0.2999999999999972</v>
       </c>
       <c r="U141" t="n">
-        <v>37.66666666666667</v>
+        <v>37.66666666666666</v>
       </c>
       <c r="V141" t="n">
         <v>3</v>
@@ -16213,10 +16213,10 @@
         <v>35</v>
       </c>
       <c r="K180" t="n">
-        <v>38.3</v>
+        <v>34.3</v>
       </c>
       <c r="L180" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="M180" t="inlineStr">
         <is>
@@ -16246,7 +16246,7 @@
         <v>41</v>
       </c>
       <c r="T180" t="n">
-        <v>3.299999999999997</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="U180" t="n">
         <v>35.66666666666666</v>
@@ -22089,10 +22089,10 @@
         <v>21</v>
       </c>
       <c r="K247" t="n">
-        <v>22.4</v>
+        <v>20</v>
       </c>
       <c r="L247" t="n">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="M247" t="inlineStr">
         <is>
@@ -22122,7 +22122,7 @@
         <v>21</v>
       </c>
       <c r="T247" t="n">
-        <v>1.399999999999999</v>
+        <v>-1</v>
       </c>
       <c r="U247" t="n">
         <v>20.96666666666667</v>
@@ -22177,10 +22177,10 @@
         <v>21</v>
       </c>
       <c r="K248" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="L248" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M248" t="inlineStr">
         <is>
@@ -22210,7 +22210,7 @@
         <v>21</v>
       </c>
       <c r="T248" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U248" t="n">
         <v>21.2</v>
@@ -24451,10 +24451,10 @@
         <v>28</v>
       </c>
       <c r="K274" t="n">
-        <v>27.5</v>
+        <v>28.7</v>
       </c>
       <c r="L274" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="M274" t="inlineStr">
         <is>
@@ -24484,7 +24484,7 @@
         <v>28</v>
       </c>
       <c r="T274" t="n">
-        <v>-0.5</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U274" t="n">
         <v>28.6</v>
@@ -24493,7 +24493,7 @@
         <v>3</v>
       </c>
       <c r="W274" t="n">
-        <v>32.9888888888889</v>
+        <v>32.98888888888889</v>
       </c>
       <c r="X274" t="n">
         <v>24.5</v>
@@ -26995,10 +26995,10 @@
         <v>21</v>
       </c>
       <c r="K303" t="n">
-        <v>20.4</v>
+        <v>21.9</v>
       </c>
       <c r="L303" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="M303" t="inlineStr">
         <is>
@@ -27028,16 +27028,16 @@
         <v>21</v>
       </c>
       <c r="T303" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U303" t="n">
-        <v>21.16666666666667</v>
+        <v>21.16666666666666</v>
       </c>
       <c r="V303" t="n">
         <v>3</v>
       </c>
       <c r="W303" t="n">
-        <v>22.05555555555556</v>
+        <v>22.05555555555555</v>
       </c>
       <c r="X303" t="n">
         <v>17.5</v>
@@ -27697,10 +27697,10 @@
         <v>24.5</v>
       </c>
       <c r="K311" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="L311" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="M311" t="inlineStr">
         <is>
@@ -27730,7 +27730,7 @@
         <v>28</v>
       </c>
       <c r="T311" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U311" t="n">
         <v>25.13333333333334</v>
@@ -28665,10 +28665,10 @@
         <v>24.5</v>
       </c>
       <c r="K322" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L322" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M322" t="inlineStr">
         <is>
@@ -28698,7 +28698,7 @@
         <v>28</v>
       </c>
       <c r="T322" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U322" t="n">
         <v>24.66666666666667</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>25.1</v>
+        <v>26.1</v>
       </c>
       <c r="L323" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>0.6000000000000014</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -28841,10 +28841,10 @@
         <v>24.5</v>
       </c>
       <c r="K324" t="n">
-        <v>29.7</v>
+        <v>31.9</v>
       </c>
       <c r="L324" t="n">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="M324" t="inlineStr">
         <is>
@@ -28874,7 +28874,7 @@
         <v>28</v>
       </c>
       <c r="T324" t="n">
-        <v>5.199999999999999</v>
+        <v>7.399999999999999</v>
       </c>
       <c r="U324" t="n">
         <v>27.5</v>
@@ -29369,10 +29369,10 @@
         <v>24.5</v>
       </c>
       <c r="K330" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L330" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M330" t="inlineStr">
         <is>
@@ -29402,7 +29402,7 @@
         <v>28</v>
       </c>
       <c r="T330" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U330" t="n">
         <v>27.1</v>
@@ -31305,10 +31305,10 @@
         <v>24.5</v>
       </c>
       <c r="K352" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L352" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M352" t="inlineStr">
         <is>
@@ -31338,10 +31338,10 @@
         <v>28</v>
       </c>
       <c r="T352" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U352" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V352" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-13 04:57:18
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -7091,10 +7091,10 @@
         <v>31</v>
       </c>
       <c r="K76" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L76" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U76" t="n">
         <v>32.03333333333333</v>
@@ -7441,10 +7441,10 @@
         <v>31</v>
       </c>
       <c r="K80" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L80" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7472,7 +7472,7 @@
       </c>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U80" t="n">
         <v>36</v>
@@ -8055,10 +8055,10 @@
         <v>31</v>
       </c>
       <c r="K87" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L87" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M87" t="inlineStr">
         <is>
@@ -8086,7 +8086,7 @@
       </c>
       <c r="S87" t="inlineStr"/>
       <c r="T87" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U87" t="n">
         <v>33.63333333333333</v>
@@ -8493,10 +8493,10 @@
         <v>31</v>
       </c>
       <c r="K92" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L92" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="S92" t="inlineStr"/>
       <c r="T92" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U92" t="n">
         <v>32.76666666666667</v>
@@ -9845,7 +9845,7 @@
         <v>3</v>
       </c>
       <c r="W107" t="n">
-        <v>24.52222222222222</v>
+        <v>24.52222222222223</v>
       </c>
       <c r="X107" t="n">
         <v>17.5</v>
@@ -11299,10 +11299,10 @@
         <v>21</v>
       </c>
       <c r="K124" t="n">
-        <v>18.4</v>
+        <v>22.6</v>
       </c>
       <c r="L124" t="n">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11332,10 +11332,10 @@
         <v>21</v>
       </c>
       <c r="T124" t="n">
-        <v>-2.600000000000001</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U124" t="n">
-        <v>22.93333333333333</v>
+        <v>22.93333333333334</v>
       </c>
       <c r="V124" t="n">
         <v>3</v>
@@ -11387,10 +11387,10 @@
         <v>21</v>
       </c>
       <c r="K125" t="n">
-        <v>19.4</v>
+        <v>21.6</v>
       </c>
       <c r="L125" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="M125" t="inlineStr">
         <is>
@@ -11420,7 +11420,7 @@
         <v>21</v>
       </c>
       <c r="T125" t="n">
-        <v>-1.600000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U125" t="n">
         <v>19.93333333333333</v>
@@ -12529,10 +12529,10 @@
         <v>35</v>
       </c>
       <c r="K138" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="L138" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="M138" t="inlineStr">
         <is>
@@ -12562,7 +12562,7 @@
         <v>41</v>
       </c>
       <c r="T138" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="U138" t="n">
         <v>41</v>
@@ -12793,10 +12793,10 @@
         <v>35</v>
       </c>
       <c r="K141" t="n">
-        <v>34.7</v>
+        <v>39.7</v>
       </c>
       <c r="L141" t="n">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="M141" t="inlineStr">
         <is>
@@ -12826,10 +12826,10 @@
         <v>41</v>
       </c>
       <c r="T141" t="n">
-        <v>-0.2999999999999972</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="U141" t="n">
-        <v>37.66666666666666</v>
+        <v>37.66666666666667</v>
       </c>
       <c r="V141" t="n">
         <v>3</v>
@@ -16213,10 +16213,10 @@
         <v>35</v>
       </c>
       <c r="K180" t="n">
-        <v>34.3</v>
+        <v>38.3</v>
       </c>
       <c r="L180" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="M180" t="inlineStr">
         <is>
@@ -16246,7 +16246,7 @@
         <v>41</v>
       </c>
       <c r="T180" t="n">
-        <v>-0.7000000000000028</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U180" t="n">
         <v>35.66666666666666</v>
@@ -22089,10 +22089,10 @@
         <v>21</v>
       </c>
       <c r="K247" t="n">
-        <v>20</v>
+        <v>22.4</v>
       </c>
       <c r="L247" t="n">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="M247" t="inlineStr">
         <is>
@@ -22122,7 +22122,7 @@
         <v>21</v>
       </c>
       <c r="T247" t="n">
-        <v>-1</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="U247" t="n">
         <v>20.96666666666667</v>
@@ -22177,10 +22177,10 @@
         <v>21</v>
       </c>
       <c r="K248" t="n">
-        <v>21.2</v>
+        <v>21.5</v>
       </c>
       <c r="L248" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="M248" t="inlineStr">
         <is>
@@ -22210,7 +22210,7 @@
         <v>21</v>
       </c>
       <c r="T248" t="n">
-        <v>0.1999999999999993</v>
+        <v>0.5</v>
       </c>
       <c r="U248" t="n">
         <v>21.2</v>
@@ -22523,10 +22523,10 @@
         <v>21</v>
       </c>
       <c r="K252" t="n">
-        <v>21.3</v>
+        <v>23.8</v>
       </c>
       <c r="L252" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="M252" t="inlineStr">
         <is>
@@ -22554,7 +22554,7 @@
       </c>
       <c r="S252" t="inlineStr"/>
       <c r="T252" t="n">
-        <v>0.3000000000000007</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U252" t="n">
         <v>21.8</v>
@@ -22697,10 +22697,10 @@
         <v>21</v>
       </c>
       <c r="K254" t="n">
-        <v>42.6</v>
+        <v>16.6</v>
       </c>
       <c r="L254" t="n">
-        <v>203</v>
+        <v>79</v>
       </c>
       <c r="M254" t="inlineStr">
         <is>
@@ -22730,7 +22730,7 @@
         <v>21</v>
       </c>
       <c r="T254" t="n">
-        <v>21.6</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="U254" t="n">
         <v>36.33333333333334</v>
@@ -24363,10 +24363,10 @@
         <v>21</v>
       </c>
       <c r="K273" t="n">
-        <v>17.8</v>
+        <v>18.3</v>
       </c>
       <c r="L273" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="M273" t="inlineStr">
         <is>
@@ -24396,7 +24396,7 @@
         <v>21</v>
       </c>
       <c r="T273" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="U273" t="n">
         <v>18.73333333333333</v>
@@ -24451,10 +24451,10 @@
         <v>28</v>
       </c>
       <c r="K274" t="n">
-        <v>28.7</v>
+        <v>27.5</v>
       </c>
       <c r="L274" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="M274" t="inlineStr">
         <is>
@@ -24484,7 +24484,7 @@
         <v>28</v>
       </c>
       <c r="T274" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.5</v>
       </c>
       <c r="U274" t="n">
         <v>28.6</v>
@@ -24493,7 +24493,7 @@
         <v>3</v>
       </c>
       <c r="W274" t="n">
-        <v>32.98888888888889</v>
+        <v>32.9888888888889</v>
       </c>
       <c r="X274" t="n">
         <v>24.5</v>
@@ -26995,10 +26995,10 @@
         <v>21</v>
       </c>
       <c r="K303" t="n">
-        <v>21.9</v>
+        <v>20.4</v>
       </c>
       <c r="L303" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="M303" t="inlineStr">
         <is>
@@ -27028,16 +27028,16 @@
         <v>21</v>
       </c>
       <c r="T303" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U303" t="n">
-        <v>21.16666666666666</v>
+        <v>21.16666666666667</v>
       </c>
       <c r="V303" t="n">
         <v>3</v>
       </c>
       <c r="W303" t="n">
-        <v>22.05555555555555</v>
+        <v>22.05555555555556</v>
       </c>
       <c r="X303" t="n">
         <v>17.5</v>
@@ -27697,10 +27697,10 @@
         <v>24.5</v>
       </c>
       <c r="K311" t="n">
-        <v>23.9</v>
+        <v>25.1</v>
       </c>
       <c r="L311" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="M311" t="inlineStr">
         <is>
@@ -27730,7 +27730,7 @@
         <v>28</v>
       </c>
       <c r="T311" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U311" t="n">
         <v>25.13333333333334</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>26.1</v>
+        <v>25.1</v>
       </c>
       <c r="L323" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>1.600000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -28841,10 +28841,10 @@
         <v>24.5</v>
       </c>
       <c r="K324" t="n">
-        <v>31.9</v>
+        <v>29.7</v>
       </c>
       <c r="L324" t="n">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="M324" t="inlineStr">
         <is>
@@ -28874,7 +28874,7 @@
         <v>28</v>
       </c>
       <c r="T324" t="n">
-        <v>7.399999999999999</v>
+        <v>5.199999999999999</v>
       </c>
       <c r="U324" t="n">
         <v>27.5</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-14 21:17:51
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -6491,10 +6491,10 @@
         <v>21</v>
       </c>
       <c r="K69" t="n">
-        <v>20.5</v>
+        <v>20.9</v>
       </c>
       <c r="L69" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="S69" t="inlineStr"/>
       <c r="T69" t="n">
-        <v>-0.5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U69" t="n">
         <v>20.2</v>
@@ -6575,10 +6575,10 @@
         <v>21</v>
       </c>
       <c r="K70" t="n">
-        <v>25.9</v>
+        <v>22.6</v>
       </c>
       <c r="L70" t="n">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -6608,7 +6608,7 @@
         <v>21</v>
       </c>
       <c r="T70" t="n">
-        <v>4.899999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U70" t="n">
         <v>22.7</v>
@@ -7103,10 +7103,10 @@
         <v>21</v>
       </c>
       <c r="K76" t="n">
-        <v>18.9</v>
+        <v>19.8</v>
       </c>
       <c r="L76" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -7136,7 +7136,7 @@
         <v>21</v>
       </c>
       <c r="T76" t="n">
-        <v>-2.100000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U76" t="n">
         <v>19</v>
@@ -7453,10 +7453,10 @@
         <v>21</v>
       </c>
       <c r="K80" t="n">
-        <v>20.4</v>
+        <v>22.6</v>
       </c>
       <c r="L80" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U80" t="n">
         <v>21.8</v>
@@ -8505,10 +8505,10 @@
         <v>24.5</v>
       </c>
       <c r="K92" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="L92" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -8538,7 +8538,7 @@
         <v>28</v>
       </c>
       <c r="T92" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U92" t="n">
         <v>25.13333333333334</v>
@@ -8857,10 +8857,10 @@
         <v>24.5</v>
       </c>
       <c r="K96" t="n">
-        <v>30.7</v>
+        <v>21.3</v>
       </c>
       <c r="L96" t="n">
-        <v>125</v>
+        <v>87</v>
       </c>
       <c r="M96" t="inlineStr">
         <is>
@@ -8890,7 +8890,7 @@
         <v>28</v>
       </c>
       <c r="T96" t="n">
-        <v>6.199999999999999</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U96" t="n">
         <v>24.76666666666667</v>
@@ -9473,10 +9473,10 @@
         <v>24.5</v>
       </c>
       <c r="K103" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L103" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9506,7 +9506,7 @@
         <v>28</v>
       </c>
       <c r="T103" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U103" t="n">
         <v>24.66666666666667</v>
@@ -10177,10 +10177,10 @@
         <v>24.5</v>
       </c>
       <c r="K111" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L111" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -10210,7 +10210,7 @@
         <v>28</v>
       </c>
       <c r="T111" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U111" t="n">
         <v>27.1</v>
@@ -11099,7 +11099,7 @@
         <v>3</v>
       </c>
       <c r="W121" t="n">
-        <v>30.57777777777778</v>
+        <v>26.84444444444444</v>
       </c>
       <c r="X121" t="n">
         <v>21</v>
@@ -12025,10 +12025,10 @@
         <v>24.5</v>
       </c>
       <c r="K132" t="n">
-        <v>27.8</v>
+        <v>22.9</v>
       </c>
       <c r="L132" t="n">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="M132" t="inlineStr">
         <is>
@@ -12058,7 +12058,7 @@
         <v>28</v>
       </c>
       <c r="T132" t="n">
-        <v>3.300000000000001</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U132" t="n">
         <v>25</v>
@@ -12113,10 +12113,10 @@
         <v>24.5</v>
       </c>
       <c r="K133" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L133" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M133" t="inlineStr">
         <is>
@@ -12146,10 +12146,10 @@
         <v>28</v>
       </c>
       <c r="T133" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U133" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V133" t="n">
         <v>3</v>
@@ -12287,10 +12287,10 @@
         <v>24.5</v>
       </c>
       <c r="K135" t="n">
-        <v>28.5</v>
+        <v>31.7</v>
       </c>
       <c r="L135" t="n">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="M135" t="inlineStr">
         <is>
@@ -12320,7 +12320,7 @@
         <v>28</v>
       </c>
       <c r="T135" t="n">
-        <v>4</v>
+        <v>7.199999999999999</v>
       </c>
       <c r="U135" t="n">
         <v>28.1</v>
@@ -12551,10 +12551,10 @@
         <v>24.5</v>
       </c>
       <c r="K138" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="L138" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="M138" t="inlineStr">
         <is>
@@ -12584,7 +12584,7 @@
         <v>28</v>
       </c>
       <c r="T138" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U138" t="n">
         <v>26.4</v>
@@ -12727,10 +12727,10 @@
         <v>24.5</v>
       </c>
       <c r="K140" t="n">
-        <v>22.7</v>
+        <v>29.1</v>
       </c>
       <c r="L140" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="M140" t="inlineStr">
         <is>
@@ -12760,7 +12760,7 @@
         <v>28</v>
       </c>
       <c r="T140" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="U140" t="n">
         <v>25.3</v>
@@ -12989,10 +12989,10 @@
         <v>21</v>
       </c>
       <c r="K143" t="n">
-        <v>17.6</v>
+        <v>18.2</v>
       </c>
       <c r="L143" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="M143" t="inlineStr">
         <is>
@@ -13020,16 +13020,16 @@
       </c>
       <c r="S143" t="inlineStr"/>
       <c r="T143" t="n">
-        <v>-3.399999999999999</v>
+        <v>-2.800000000000001</v>
       </c>
       <c r="U143" t="n">
-        <v>18.13333333333334</v>
+        <v>18.13333333333333</v>
       </c>
       <c r="V143" t="n">
         <v>3</v>
       </c>
       <c r="W143" t="n">
-        <v>27.25555555555556</v>
+        <v>27.25555555555555</v>
       </c>
       <c r="X143" t="n">
         <v>17.5</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-15 07:02:39
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X370"/>
+  <dimension ref="A1:X371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4811,10 +4811,10 @@
         <v>24</v>
       </c>
       <c r="K50" t="n">
-        <v>24.9</v>
+        <v>23.8</v>
       </c>
       <c r="L50" t="n">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
@@ -4844,7 +4844,7 @@
         <v>28</v>
       </c>
       <c r="T50" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U50" t="n">
         <v>21.43333333333333</v>
@@ -4899,10 +4899,10 @@
         <v>24</v>
       </c>
       <c r="K51" t="n">
-        <v>25.9</v>
+        <v>22.1</v>
       </c>
       <c r="L51" t="n">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
@@ -4932,7 +4932,7 @@
         <v>28</v>
       </c>
       <c r="T51" t="n">
-        <v>1.899999999999999</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="U51" t="n">
         <v>24.23333333333333</v>
@@ -5773,10 +5773,10 @@
         <v>31</v>
       </c>
       <c r="K61" t="n">
-        <v>35.8</v>
+        <v>31.4</v>
       </c>
       <c r="L61" t="n">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
@@ -5804,10 +5804,10 @@
       </c>
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="n">
-        <v>4.799999999999997</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U61" t="n">
-        <v>30.66666666666667</v>
+        <v>30.66666666666666</v>
       </c>
       <c r="V61" t="n">
         <v>3</v>
@@ -7353,10 +7353,10 @@
         <v>28</v>
       </c>
       <c r="K79" t="n">
-        <v>24.1</v>
+        <v>27.3</v>
       </c>
       <c r="L79" t="n">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7386,7 +7386,7 @@
         <v>28</v>
       </c>
       <c r="T79" t="n">
-        <v>-3.899999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="U79" t="n">
         <v>25.33333333333333</v>
@@ -7441,7 +7441,7 @@
         <v>28</v>
       </c>
       <c r="K80" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="L80" t="n">
         <v>88</v>
@@ -7474,7 +7474,7 @@
         <v>28</v>
       </c>
       <c r="T80" t="n">
-        <v>-3.300000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U80" t="n">
         <v>25.13333333333334</v>
@@ -7967,10 +7967,10 @@
         <v>21</v>
       </c>
       <c r="K86" t="n">
-        <v>19.3</v>
+        <v>20.2</v>
       </c>
       <c r="L86" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="M86" t="inlineStr">
         <is>
@@ -8000,7 +8000,7 @@
         <v>21</v>
       </c>
       <c r="T86" t="n">
-        <v>-1.699999999999999</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U86" t="n">
         <v>20.46666666666667</v>
@@ -11299,10 +11299,10 @@
         <v>28</v>
       </c>
       <c r="K124" t="n">
-        <v>33.5</v>
+        <v>31.6</v>
       </c>
       <c r="L124" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11332,7 +11332,7 @@
         <v>28</v>
       </c>
       <c r="T124" t="n">
-        <v>5.5</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U124" t="n">
         <v>30.83333333333333</v>
@@ -13233,10 +13233,10 @@
         <v>35</v>
       </c>
       <c r="K146" t="n">
-        <v>37.5</v>
+        <v>46</v>
       </c>
       <c r="L146" t="n">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="M146" t="inlineStr">
         <is>
@@ -13266,7 +13266,7 @@
         <v>41</v>
       </c>
       <c r="T146" t="n">
-        <v>2.5</v>
+        <v>11</v>
       </c>
       <c r="U146" t="n">
         <v>38.3</v>
@@ -13321,10 +13321,10 @@
         <v>35</v>
       </c>
       <c r="K147" t="n">
-        <v>27.7</v>
+        <v>26.2</v>
       </c>
       <c r="L147" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="M147" t="inlineStr">
         <is>
@@ -13354,7 +13354,7 @@
         <v>41</v>
       </c>
       <c r="T147" t="n">
-        <v>-7.300000000000001</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="U147" t="n">
         <v>26.5</v>
@@ -13495,10 +13495,10 @@
         <v>35</v>
       </c>
       <c r="K149" t="n">
-        <v>38.6</v>
+        <v>38.2</v>
       </c>
       <c r="L149" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M149" t="inlineStr">
         <is>
@@ -13528,10 +13528,10 @@
         <v>41</v>
       </c>
       <c r="T149" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U149" t="n">
-        <v>36.56666666666667</v>
+        <v>36.56666666666666</v>
       </c>
       <c r="V149" t="n">
         <v>3</v>
@@ -13583,10 +13583,10 @@
         <v>35</v>
       </c>
       <c r="K150" t="n">
-        <v>36.9</v>
+        <v>34.4</v>
       </c>
       <c r="L150" t="n">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="M150" t="inlineStr">
         <is>
@@ -13616,7 +13616,7 @@
         <v>41</v>
       </c>
       <c r="T150" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U150" t="n">
         <v>35.53333333333333</v>
@@ -13625,7 +13625,7 @@
         <v>3</v>
       </c>
       <c r="W150" t="n">
-        <v>36.47037037037038</v>
+        <v>36.47037037037036</v>
       </c>
       <c r="X150" t="n">
         <v>31.5</v>
@@ -13671,10 +13671,10 @@
         <v>28</v>
       </c>
       <c r="K151" t="n">
-        <v>35.4</v>
+        <v>31.9</v>
       </c>
       <c r="L151" t="n">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="M151" t="inlineStr">
         <is>
@@ -13704,7 +13704,7 @@
         <v>28</v>
       </c>
       <c r="T151" t="n">
-        <v>7.399999999999999</v>
+        <v>3.899999999999999</v>
       </c>
       <c r="U151" t="n">
         <v>31.73333333333333</v>
@@ -13759,10 +13759,10 @@
         <v>28</v>
       </c>
       <c r="K152" t="n">
-        <v>30.2</v>
+        <v>30.7</v>
       </c>
       <c r="L152" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="M152" t="inlineStr">
         <is>
@@ -13792,7 +13792,7 @@
         <v>28</v>
       </c>
       <c r="T152" t="n">
-        <v>2.199999999999999</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U152" t="n">
         <v>29.23333333333333</v>
@@ -13801,7 +13801,7 @@
         <v>3</v>
       </c>
       <c r="W152" t="n">
-        <v>33.02222222222222</v>
+        <v>33.02222222222223</v>
       </c>
       <c r="X152" t="n">
         <v>24.5</v>
@@ -14019,10 +14019,10 @@
         <v>35</v>
       </c>
       <c r="K155" t="n">
-        <v>32.4</v>
+        <v>37.3</v>
       </c>
       <c r="L155" t="n">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="M155" t="inlineStr">
         <is>
@@ -14052,7 +14052,7 @@
         <v>41</v>
       </c>
       <c r="T155" t="n">
-        <v>-2.600000000000001</v>
+        <v>2.299999999999997</v>
       </c>
       <c r="U155" t="n">
         <v>36.6</v>
@@ -17267,10 +17267,10 @@
         <v>35</v>
       </c>
       <c r="K192" t="n">
-        <v>35.9</v>
+        <v>36.4</v>
       </c>
       <c r="L192" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="M192" t="inlineStr">
         <is>
@@ -17300,7 +17300,7 @@
         <v>41</v>
       </c>
       <c r="T192" t="n">
-        <v>0.8999999999999986</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="U192" t="n">
         <v>35.16666666666666</v>
@@ -17791,10 +17791,10 @@
         <v>21</v>
       </c>
       <c r="K198" t="n">
-        <v>23.9</v>
+        <v>20.7</v>
       </c>
       <c r="L198" t="n">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="M198" t="inlineStr">
         <is>
@@ -17824,7 +17824,7 @@
         <v>21</v>
       </c>
       <c r="T198" t="n">
-        <v>2.899999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U198" t="n">
         <v>22.5</v>
@@ -19943,7 +19943,7 @@
         <v>3</v>
       </c>
       <c r="W222" t="n">
-        <v>19.75555555555556</v>
+        <v>19.75555555555555</v>
       </c>
       <c r="X222" t="n">
         <v>17.5</v>
@@ -20517,10 +20517,10 @@
         <v>28</v>
       </c>
       <c r="K229" t="n">
-        <v>25</v>
+        <v>22.8</v>
       </c>
       <c r="L229" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="M229" t="inlineStr">
         <is>
@@ -20550,7 +20550,7 @@
         <v>28</v>
       </c>
       <c r="T229" t="n">
-        <v>-3</v>
+        <v>-5.199999999999999</v>
       </c>
       <c r="U229" t="n">
         <v>24.76666666666667</v>
@@ -32573,7 +32573,7 @@
         <v>3</v>
       </c>
       <c r="W366" t="n">
-        <v>16.92222222222222</v>
+        <v>23.52222222222222</v>
       </c>
       <c r="X366" t="n">
         <v>17.5</v>
@@ -32661,7 +32661,7 @@
         <v>3</v>
       </c>
       <c r="W367" t="n">
-        <v>19.13333333333333</v>
+        <v>22.68888888888889</v>
       </c>
       <c r="X367" t="n">
         <v>17.5</v>
@@ -32675,7 +32675,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>PL24</t>
+          <t>PL-43</t>
         </is>
       </c>
       <c r="C368" t="inlineStr"/>
@@ -32686,17 +32686,17 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>CIMEANTACION PLATAFORMA ZARPA Y ZAPATA EJE C-12 ZAPATA EJE E-6</t>
+          <t>Plataforma muros eje E-12, F-10, F-11</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
         <is>
-          <t>9/25/2026 12:00:00 AM</t>
+          <t>10/12/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H368" t="inlineStr"/>
@@ -32707,14 +32707,14 @@
         <v>21</v>
       </c>
       <c r="K368" t="n">
-        <v>18.9</v>
+        <v>23.6</v>
       </c>
       <c r="L368" t="n">
-        <v>90</v>
+        <v>112</v>
       </c>
       <c r="M368" t="inlineStr">
         <is>
-          <t>AUTOCOMPAC</t>
+          <t>MURO</t>
         </is>
       </c>
       <c r="N368" t="n">
@@ -32722,7 +32722,7 @@
       </c>
       <c r="O368" t="inlineStr">
         <is>
-          <t>AUTOCOMPAC-21-28</t>
+          <t>MURO-21-28</t>
         </is>
       </c>
       <c r="P368" s="2" t="n">
@@ -32736,18 +32736,20 @@
       <c r="R368" s="2" t="n">
         <v>46310</v>
       </c>
-      <c r="S368" t="inlineStr"/>
+      <c r="S368" t="n">
+        <v>21</v>
+      </c>
       <c r="T368" t="n">
-        <v>-2.100000000000001</v>
+        <v>2.600000000000001</v>
       </c>
       <c r="U368" t="n">
-        <v>19.9</v>
+        <v>22.76666666666667</v>
       </c>
       <c r="V368" t="n">
         <v>3</v>
       </c>
       <c r="W368" t="n">
-        <v>23.37777777777778</v>
+        <v>17.14444444444445</v>
       </c>
       <c r="X368" t="n">
         <v>17.5</v>
@@ -32761,7 +32763,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>PL30</t>
+          <t>PL24</t>
         </is>
       </c>
       <c r="C369" t="inlineStr"/>
@@ -32772,17 +32774,17 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>VIGAS PLACA PLATAFORMA PISO 1 EJE A-B, 11,10,09</t>
+          <t>CIMEANTACION PLATAFORMA ZARPA Y ZAPATA EJE C-12 ZAPATA EJE E-6</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>10/1/2026 12:00:00 AM</t>
+          <t>9/25/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H369" t="inlineStr"/>
@@ -32793,14 +32795,14 @@
         <v>21</v>
       </c>
       <c r="K369" t="n">
-        <v>23.5</v>
+        <v>18.9</v>
       </c>
       <c r="L369" t="n">
-        <v>112</v>
+        <v>90</v>
       </c>
       <c r="M369" t="inlineStr">
         <is>
-          <t>PLACA</t>
+          <t>AUTOCOMPAC</t>
         </is>
       </c>
       <c r="N369" t="n">
@@ -32808,7 +32810,7 @@
       </c>
       <c r="O369" t="inlineStr">
         <is>
-          <t>PLACA-21-28</t>
+          <t>AUTOCOMPAC-21-28</t>
         </is>
       </c>
       <c r="P369" s="2" t="n">
@@ -32822,20 +32824,18 @@
       <c r="R369" s="2" t="n">
         <v>46310</v>
       </c>
-      <c r="S369" t="n">
-        <v>21</v>
-      </c>
+      <c r="S369" t="inlineStr"/>
       <c r="T369" t="n">
-        <v>2.5</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U369" t="n">
-        <v>22.16666666666667</v>
+        <v>19.9</v>
       </c>
       <c r="V369" t="n">
         <v>3</v>
       </c>
       <c r="W369" t="n">
-        <v>25.15555555555556</v>
+        <v>23.37777777777778</v>
       </c>
       <c r="X369" t="n">
         <v>17.5</v>
@@ -32849,7 +32849,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>SC 05</t>
+          <t>PL30</t>
         </is>
       </c>
       <c r="C370" t="inlineStr"/>
@@ -32860,17 +32860,17 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>VIGAS CIMENTACION PLACA SUPERIOR EJE 1-3 ENTRE A Y F-SC</t>
+          <t>VIGAS PLACA PLATAFORMA PISO 1 EJE A-B, 11,10,09</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
         <is>
-          <t>9/24/2026 12:00:00 AM</t>
+          <t>10/1/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H370" t="inlineStr"/>
@@ -32881,51 +32881,139 @@
         <v>21</v>
       </c>
       <c r="K370" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="L370" t="n">
+        <v>112</v>
+      </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>PLACA</t>
+        </is>
+      </c>
+      <c r="N370" t="n">
+        <v>21</v>
+      </c>
+      <c r="O370" t="inlineStr">
+        <is>
+          <t>PLACA-21-28</t>
+        </is>
+      </c>
+      <c r="P370" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="Q370" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="R370" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="S370" t="n">
+        <v>21</v>
+      </c>
+      <c r="T370" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="U370" t="n">
+        <v>22.16666666666667</v>
+      </c>
+      <c r="V370" t="n">
+        <v>3</v>
+      </c>
+      <c r="W370" t="n">
+        <v>25.15555555555556</v>
+      </c>
+      <c r="X370" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>VIALE 26</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>SC 05</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr"/>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>VIGAS CIMENTACION PLACA SUPERIOR EJE 1-3 ENTRE A Y F-SC</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>9/24/2026 12:00:00 AM</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr"/>
+      <c r="I371" t="n">
+        <v>28</v>
+      </c>
+      <c r="J371" t="n">
+        <v>21</v>
+      </c>
+      <c r="K371" t="n">
         <v>19.8</v>
       </c>
-      <c r="L370" t="n">
+      <c r="L371" t="n">
         <v>94</v>
       </c>
-      <c r="M370" t="inlineStr">
+      <c r="M371" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="N370" t="n">
-        <v>21</v>
-      </c>
-      <c r="O370" t="inlineStr">
+      <c r="N371" t="n">
+        <v>21</v>
+      </c>
+      <c r="O371" t="inlineStr">
         <is>
           <t>PLACA-21-28</t>
         </is>
       </c>
-      <c r="P370" s="2" t="n">
-        <v>46310</v>
-      </c>
-      <c r="Q370" t="inlineStr">
-        <is>
-          <t>NUEVO</t>
-        </is>
-      </c>
-      <c r="R370" s="2" t="n">
-        <v>46310</v>
-      </c>
-      <c r="S370" t="n">
-        <v>21</v>
-      </c>
-      <c r="T370" t="n">
+      <c r="P371" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="Q371" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="R371" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="S371" t="n">
+        <v>21</v>
+      </c>
+      <c r="T371" t="n">
         <v>-1.199999999999999</v>
       </c>
-      <c r="U370" t="n">
+      <c r="U371" t="n">
         <v>18.9</v>
       </c>
-      <c r="V370" t="n">
-        <v>3</v>
-      </c>
-      <c r="W370" t="n">
+      <c r="V371" t="n">
+        <v>3</v>
+      </c>
+      <c r="W371" t="n">
         <v>22.93333333333334</v>
       </c>
-      <c r="X370" t="n">
+      <c r="X371" t="n">
         <v>17.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-15 22:59:33
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3417,10 +3417,10 @@
         <v>31</v>
       </c>
       <c r="K34" t="n">
-        <v>27.8</v>
+        <v>38.5</v>
       </c>
       <c r="L34" t="n">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="n">
-        <v>-3.199999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="U34" t="n">
         <v>35.83333333333334</v>
@@ -3503,10 +3503,10 @@
         <v>28</v>
       </c>
       <c r="K35" t="n">
-        <v>33.2</v>
+        <v>22.1</v>
       </c>
       <c r="L35" t="n">
-        <v>118</v>
+        <v>79</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
         <v>28</v>
       </c>
       <c r="T35" t="n">
-        <v>5.200000000000003</v>
+        <v>-5.899999999999999</v>
       </c>
       <c r="U35" t="n">
         <v>30.1</v>
@@ -3591,10 +3591,10 @@
         <v>31</v>
       </c>
       <c r="K36" t="n">
-        <v>30.9</v>
+        <v>32.6</v>
       </c>
       <c r="L36" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U36" t="n">
         <v>30.8</v>
@@ -3631,7 +3631,7 @@
         <v>3</v>
       </c>
       <c r="W36" t="n">
-        <v>41.12222222222222</v>
+        <v>41.12222222222223</v>
       </c>
       <c r="X36" t="n">
         <v>27.5</v>
@@ -3677,10 +3677,10 @@
         <v>28</v>
       </c>
       <c r="K37" t="n">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="L37" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3710,7 +3710,7 @@
         <v>28</v>
       </c>
       <c r="T37" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="U37" t="n">
         <v>30.53333333333333</v>
@@ -3765,10 +3765,10 @@
         <v>28</v>
       </c>
       <c r="K38" t="n">
-        <v>24.9</v>
+        <v>32.4</v>
       </c>
       <c r="L38" t="n">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
         <v>28</v>
       </c>
       <c r="T38" t="n">
-        <v>-3.100000000000001</v>
+        <v>4.399999999999999</v>
       </c>
       <c r="U38" t="n">
         <v>31.5</v>
@@ -6475,10 +6475,10 @@
         <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>34.3</v>
+        <v>32.3</v>
       </c>
       <c r="L69" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>41</v>
       </c>
       <c r="T69" t="n">
-        <v>-0.7000000000000028</v>
+        <v>-2.700000000000003</v>
       </c>
       <c r="U69" t="n">
         <v>32.96666666666666</v>
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L77" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7441,10 +7441,10 @@
         <v>28</v>
       </c>
       <c r="K80" t="n">
-        <v>30.7</v>
+        <v>27.7</v>
       </c>
       <c r="L80" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         <v>28</v>
       </c>
       <c r="T80" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U80" t="n">
         <v>29.2</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L81" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -7615,10 +7615,10 @@
         <v>21</v>
       </c>
       <c r="K82" t="n">
-        <v>26.4</v>
+        <v>17.9</v>
       </c>
       <c r="L82" t="n">
-        <v>126</v>
+        <v>85</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
         <v>21</v>
       </c>
       <c r="T82" t="n">
-        <v>5.399999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="U82" t="n">
         <v>21.3</v>
@@ -7703,10 +7703,10 @@
         <v>35</v>
       </c>
       <c r="K83" t="n">
-        <v>32.4</v>
+        <v>39.8</v>
       </c>
       <c r="L83" t="n">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7736,7 +7736,7 @@
         <v>41</v>
       </c>
       <c r="T83" t="n">
-        <v>-2.600000000000001</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="U83" t="n">
         <v>36.03333333333333</v>
@@ -7879,10 +7879,10 @@
         <v>21</v>
       </c>
       <c r="K85" t="n">
-        <v>20.2</v>
+        <v>19.3</v>
       </c>
       <c r="L85" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="M85" t="inlineStr">
         <is>
@@ -7912,7 +7912,7 @@
         <v>21</v>
       </c>
       <c r="T85" t="n">
-        <v>-0.8000000000000007</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U85" t="n">
         <v>20.46666666666667</v>
@@ -7967,10 +7967,10 @@
         <v>21</v>
       </c>
       <c r="K86" t="n">
-        <v>23.8</v>
+        <v>24.7</v>
       </c>
       <c r="L86" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="M86" t="inlineStr">
         <is>
@@ -8000,7 +8000,7 @@
         <v>21</v>
       </c>
       <c r="T86" t="n">
-        <v>2.800000000000001</v>
+        <v>3.699999999999999</v>
       </c>
       <c r="U86" t="n">
         <v>22.53333333333333</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L88" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L93" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -13407,10 +13407,10 @@
         <v>35</v>
       </c>
       <c r="K148" t="n">
-        <v>38.6</v>
+        <v>38.2</v>
       </c>
       <c r="L148" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M148" t="inlineStr">
         <is>
@@ -13440,10 +13440,10 @@
         <v>41</v>
       </c>
       <c r="T148" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U148" t="n">
-        <v>36.56666666666667</v>
+        <v>36.56666666666666</v>
       </c>
       <c r="V148" t="n">
         <v>3</v>
@@ -13495,10 +13495,10 @@
         <v>35</v>
       </c>
       <c r="K149" t="n">
-        <v>36.9</v>
+        <v>34.4</v>
       </c>
       <c r="L149" t="n">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="M149" t="inlineStr">
         <is>
@@ -13528,7 +13528,7 @@
         <v>41</v>
       </c>
       <c r="T149" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U149" t="n">
         <v>35.53333333333333</v>
@@ -21303,10 +21303,10 @@
         <v>24</v>
       </c>
       <c r="K238" t="n">
-        <v>25.9</v>
+        <v>23.6</v>
       </c>
       <c r="L238" t="n">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="M238" t="inlineStr">
         <is>
@@ -21336,7 +21336,7 @@
         <v>28</v>
       </c>
       <c r="T238" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U238" t="n">
         <v>25.13333333333334</v>
@@ -22265,10 +22265,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="L249" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22298,7 +22298,7 @@
         <v>21</v>
       </c>
       <c r="T249" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U249" t="n">
         <v>21.2</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L323" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L331" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -29633,10 +29633,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>31.1</v>
+        <v>24</v>
       </c>
       <c r="L333" t="n">
-        <v>127</v>
+        <v>98</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29666,7 +29666,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>6.600000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="U333" t="n">
         <v>29.13333333333334</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L353" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>
@@ -32269,10 +32269,10 @@
         <v>21</v>
       </c>
       <c r="K363" t="n">
-        <v>17.6</v>
+        <v>18.2</v>
       </c>
       <c r="L363" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="M363" t="inlineStr">
         <is>
@@ -32300,16 +32300,16 @@
       </c>
       <c r="S363" t="inlineStr"/>
       <c r="T363" t="n">
-        <v>-3.399999999999999</v>
+        <v>-2.800000000000001</v>
       </c>
       <c r="U363" t="n">
-        <v>18.13333333333334</v>
+        <v>18.13333333333333</v>
       </c>
       <c r="V363" t="n">
         <v>3</v>
       </c>
       <c r="W363" t="n">
-        <v>27.25555555555556</v>
+        <v>27.25555555555555</v>
       </c>
       <c r="X363" t="n">
         <v>17.5</v>
@@ -32707,10 +32707,10 @@
         <v>21</v>
       </c>
       <c r="K368" t="n">
-        <v>18.9</v>
+        <v>22</v>
       </c>
       <c r="L368" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="M368" t="inlineStr">
         <is>
@@ -32738,7 +32738,7 @@
       </c>
       <c r="S368" t="inlineStr"/>
       <c r="T368" t="n">
-        <v>-2.100000000000001</v>
+        <v>1</v>
       </c>
       <c r="U368" t="n">
         <v>19.9</v>
@@ -32881,10 +32881,10 @@
         <v>21</v>
       </c>
       <c r="K370" t="n">
-        <v>19.8</v>
+        <v>18.7</v>
       </c>
       <c r="L370" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M370" t="inlineStr">
         <is>
@@ -32914,7 +32914,7 @@
         <v>21</v>
       </c>
       <c r="T370" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.300000000000001</v>
       </c>
       <c r="U370" t="n">
         <v>18.9</v>
@@ -32923,7 +32923,7 @@
         <v>3</v>
       </c>
       <c r="W370" t="n">
-        <v>22.93333333333334</v>
+        <v>22.93333333333333</v>
       </c>
       <c r="X370" t="n">
         <v>17.5</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-16 16:10:38
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L77" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L81" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L88" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L93" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -14723,10 +14723,10 @@
         <v>31</v>
       </c>
       <c r="K163" t="n">
-        <v>26.6</v>
+        <v>28.7</v>
       </c>
       <c r="L163" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="M163" t="inlineStr">
         <is>
@@ -14754,7 +14754,7 @@
       </c>
       <c r="S163" t="inlineStr"/>
       <c r="T163" t="n">
-        <v>-4.399999999999999</v>
+        <v>-2.300000000000001</v>
       </c>
       <c r="U163" t="n">
         <v>28.66666666666667</v>
@@ -18407,10 +18407,10 @@
         <v>24</v>
       </c>
       <c r="K205" t="n">
-        <v>20.4</v>
+        <v>21.6</v>
       </c>
       <c r="L205" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="M205" t="inlineStr">
         <is>
@@ -18440,7 +18440,7 @@
         <v>28</v>
       </c>
       <c r="T205" t="n">
-        <v>-3.600000000000001</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="U205" t="n">
         <v>22.5</v>
@@ -22265,10 +22265,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="L249" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22298,7 +22298,7 @@
         <v>21</v>
       </c>
       <c r="T249" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U249" t="n">
         <v>21.2</v>
@@ -22611,10 +22611,10 @@
         <v>21</v>
       </c>
       <c r="K253" t="n">
-        <v>21.3</v>
+        <v>23.8</v>
       </c>
       <c r="L253" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="M253" t="inlineStr">
         <is>
@@ -22642,7 +22642,7 @@
       </c>
       <c r="S253" t="inlineStr"/>
       <c r="T253" t="n">
-        <v>0.3000000000000007</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U253" t="n">
         <v>21.8</v>
@@ -22785,10 +22785,10 @@
         <v>21</v>
       </c>
       <c r="K255" t="n">
-        <v>42.6</v>
+        <v>16.6</v>
       </c>
       <c r="L255" t="n">
-        <v>203</v>
+        <v>79</v>
       </c>
       <c r="M255" t="inlineStr">
         <is>
@@ -22818,7 +22818,7 @@
         <v>21</v>
       </c>
       <c r="T255" t="n">
-        <v>21.6</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="U255" t="n">
         <v>36.33333333333334</v>
@@ -23753,10 +23753,10 @@
         <v>28</v>
       </c>
       <c r="K266" t="n">
-        <v>32.3</v>
+        <v>29.9</v>
       </c>
       <c r="L266" t="n">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="M266" t="inlineStr">
         <is>
@@ -23786,7 +23786,7 @@
         <v>28</v>
       </c>
       <c r="T266" t="n">
-        <v>4.299999999999997</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U266" t="n">
         <v>28.53333333333333</v>
@@ -23927,10 +23927,10 @@
         <v>28</v>
       </c>
       <c r="K268" t="n">
-        <v>28.1</v>
+        <v>27</v>
       </c>
       <c r="L268" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M268" t="inlineStr">
         <is>
@@ -23960,7 +23960,7 @@
         <v>28</v>
       </c>
       <c r="T268" t="n">
-        <v>0.1000000000000014</v>
+        <v>-1</v>
       </c>
       <c r="U268" t="n">
         <v>26.96666666666667</v>
@@ -24231,7 +24231,7 @@
         <v>3</v>
       </c>
       <c r="W271" t="n">
-        <v>28.15555555555556</v>
+        <v>28.15555555555555</v>
       </c>
       <c r="X271" t="n">
         <v>24.5</v>
@@ -24277,10 +24277,10 @@
         <v>28</v>
       </c>
       <c r="K272" t="n">
-        <v>27.3</v>
+        <v>26.1</v>
       </c>
       <c r="L272" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="M272" t="inlineStr">
         <is>
@@ -24310,7 +24310,7 @@
         <v>28</v>
       </c>
       <c r="T272" t="n">
-        <v>-0.6999999999999993</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="U272" t="n">
         <v>27.16666666666667</v>
@@ -25507,10 +25507,10 @@
         <v>21</v>
       </c>
       <c r="K286" t="n">
-        <v>22</v>
+        <v>20.8</v>
       </c>
       <c r="L286" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M286" t="inlineStr">
         <is>
@@ -25540,7 +25540,7 @@
         <v>21</v>
       </c>
       <c r="T286" t="n">
-        <v>1</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U286" t="n">
         <v>21.03333333333333</v>
@@ -25595,10 +25595,10 @@
         <v>21</v>
       </c>
       <c r="K287" t="n">
-        <v>18.2</v>
+        <v>18.6</v>
       </c>
       <c r="L287" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="M287" t="inlineStr">
         <is>
@@ -25628,7 +25628,7 @@
         <v>21</v>
       </c>
       <c r="T287" t="n">
-        <v>-2.800000000000001</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="U287" t="n">
         <v>18.23333333333333</v>
@@ -25683,10 +25683,10 @@
         <v>21</v>
       </c>
       <c r="K288" t="n">
-        <v>20.2</v>
+        <v>18.4</v>
       </c>
       <c r="L288" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="M288" t="inlineStr">
         <is>
@@ -25716,16 +25716,16 @@
         <v>21</v>
       </c>
       <c r="T288" t="n">
-        <v>-0.8000000000000007</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U288" t="n">
-        <v>19.86666666666667</v>
+        <v>19.86666666666666</v>
       </c>
       <c r="V288" t="n">
         <v>3</v>
       </c>
       <c r="W288" t="n">
-        <v>21.74444444444445</v>
+        <v>21.74444444444444</v>
       </c>
       <c r="X288" t="n">
         <v>17.5</v>
@@ -26469,10 +26469,10 @@
         <v>21</v>
       </c>
       <c r="K297" t="n">
-        <v>21.9</v>
+        <v>20.3</v>
       </c>
       <c r="L297" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="M297" t="inlineStr">
         <is>
@@ -26502,7 +26502,7 @@
         <v>21</v>
       </c>
       <c r="T297" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="U297" t="n">
         <v>20.9</v>
@@ -26557,10 +26557,10 @@
         <v>21</v>
       </c>
       <c r="K298" t="n">
-        <v>20.8</v>
+        <v>20.1</v>
       </c>
       <c r="L298" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="M298" t="inlineStr">
         <is>
@@ -26590,7 +26590,7 @@
         <v>21</v>
       </c>
       <c r="T298" t="n">
-        <v>-0.1999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U298" t="n">
         <v>20.3</v>
@@ -27347,10 +27347,10 @@
         <v>21</v>
       </c>
       <c r="K307" t="n">
-        <v>21.8</v>
+        <v>20.4</v>
       </c>
       <c r="L307" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="M307" t="inlineStr">
         <is>
@@ -27380,7 +27380,7 @@
         <v>21</v>
       </c>
       <c r="T307" t="n">
-        <v>0.8000000000000007</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U307" t="n">
         <v>20.76666666666667</v>
@@ -27435,10 +27435,10 @@
         <v>21</v>
       </c>
       <c r="K308" t="n">
-        <v>22</v>
+        <v>19.4</v>
       </c>
       <c r="L308" t="n">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="M308" t="inlineStr">
         <is>
@@ -27468,7 +27468,7 @@
         <v>21</v>
       </c>
       <c r="T308" t="n">
-        <v>1</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U308" t="n">
         <v>20.8</v>
@@ -27523,10 +27523,10 @@
         <v>21</v>
       </c>
       <c r="K309" t="n">
-        <v>20.7</v>
+        <v>19.6</v>
       </c>
       <c r="L309" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="M309" t="inlineStr">
         <is>
@@ -27556,7 +27556,7 @@
         <v>21</v>
       </c>
       <c r="T309" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.399999999999999</v>
       </c>
       <c r="U309" t="n">
         <v>20.23333333333333</v>
@@ -28401,10 +28401,10 @@
         <v>24.5</v>
       </c>
       <c r="K319" t="n">
-        <v>24.6</v>
+        <v>20.9</v>
       </c>
       <c r="L319" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="M319" t="inlineStr">
         <is>
@@ -28434,7 +28434,7 @@
         <v>28</v>
       </c>
       <c r="T319" t="n">
-        <v>0.1000000000000014</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="U319" t="n">
         <v>23.96666666666667</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L323" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L331" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L353" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-16 19:24:05
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3329,10 +3329,10 @@
         <v>21</v>
       </c>
       <c r="K33" t="n">
-        <v>23.1</v>
+        <v>22.3</v>
       </c>
       <c r="L33" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3362,7 +3362,7 @@
         <v>21</v>
       </c>
       <c r="T33" t="n">
-        <v>2.100000000000001</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="U33" t="n">
         <v>21.8</v>
@@ -5875,10 +5875,10 @@
         <v>21</v>
       </c>
       <c r="K62" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
       <c r="L62" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
@@ -5908,7 +5908,7 @@
         <v>21</v>
       </c>
       <c r="T62" t="n">
-        <v>-3.399999999999999</v>
+        <v>-3.699999999999999</v>
       </c>
       <c r="U62" t="n">
         <v>17.43333333333333</v>
@@ -8067,10 +8067,10 @@
         <v>21</v>
       </c>
       <c r="K87" t="n">
-        <v>22</v>
+        <v>19.4</v>
       </c>
       <c r="L87" t="n">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="M87" t="inlineStr">
         <is>
@@ -8100,7 +8100,7 @@
         <v>21</v>
       </c>
       <c r="T87" t="n">
-        <v>1</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U87" t="n">
         <v>20.8</v>
@@ -8505,10 +8505,10 @@
         <v>24.5</v>
       </c>
       <c r="K92" t="n">
-        <v>20.7</v>
+        <v>22.5</v>
       </c>
       <c r="L92" t="n">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -8538,7 +8538,7 @@
         <v>28</v>
       </c>
       <c r="T92" t="n">
-        <v>-3.800000000000001</v>
+        <v>-2</v>
       </c>
       <c r="U92" t="n">
         <v>21.53333333333333</v>
@@ -10617,10 +10617,10 @@
         <v>24.5</v>
       </c>
       <c r="K116" t="n">
-        <v>24</v>
+        <v>57.8</v>
       </c>
       <c r="L116" t="n">
-        <v>98</v>
+        <v>236</v>
       </c>
       <c r="M116" t="inlineStr">
         <is>
@@ -10650,7 +10650,7 @@
         <v>28</v>
       </c>
       <c r="T116" t="n">
-        <v>-0.5</v>
+        <v>33.3</v>
       </c>
       <c r="U116" t="n">
         <v>35.8</v>
@@ -11011,7 +11011,7 @@
         <v>3</v>
       </c>
       <c r="W120" t="n">
-        <v>29.35555555555556</v>
+        <v>29.17777777777778</v>
       </c>
       <c r="X120" t="n">
         <v>21</v>
@@ -12199,10 +12199,10 @@
         <v>24.5</v>
       </c>
       <c r="K134" t="n">
-        <v>31.7</v>
+        <v>28.5</v>
       </c>
       <c r="L134" t="n">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="M134" t="inlineStr">
         <is>
@@ -12232,7 +12232,7 @@
         <v>28</v>
       </c>
       <c r="T134" t="n">
-        <v>7.199999999999999</v>
+        <v>4</v>
       </c>
       <c r="U134" t="n">
         <v>28.1</v>
@@ -12901,10 +12901,10 @@
         <v>21</v>
       </c>
       <c r="K142" t="n">
-        <v>18.2</v>
+        <v>17.6</v>
       </c>
       <c r="L142" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M142" t="inlineStr">
         <is>
@@ -12932,16 +12932,16 @@
       </c>
       <c r="S142" t="inlineStr"/>
       <c r="T142" t="n">
-        <v>-2.800000000000001</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U142" t="n">
-        <v>18.13333333333333</v>
+        <v>18.13333333333334</v>
       </c>
       <c r="V142" t="n">
         <v>3</v>
       </c>
       <c r="W142" t="n">
-        <v>27.25555555555555</v>
+        <v>27.25555555555556</v>
       </c>
       <c r="X142" t="n">
         <v>17.5</v>
@@ -13513,10 +13513,10 @@
         <v>21</v>
       </c>
       <c r="K149" t="n">
-        <v>19.8</v>
+        <v>18.7</v>
       </c>
       <c r="L149" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M149" t="inlineStr">
         <is>
@@ -13546,7 +13546,7 @@
         <v>21</v>
       </c>
       <c r="T149" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.300000000000001</v>
       </c>
       <c r="U149" t="n">
         <v>18.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-17 00:22:57
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -606,11 +606,11 @@
         </is>
       </c>
       <c r="P2" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
@@ -694,11 +694,11 @@
         </is>
       </c>
       <c r="P3" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R3" s="2" t="n">
@@ -784,11 +784,11 @@
         </is>
       </c>
       <c r="P4" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
@@ -872,11 +872,11 @@
         </is>
       </c>
       <c r="P5" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R5" s="2" t="n">
@@ -962,11 +962,11 @@
         </is>
       </c>
       <c r="P6" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
@@ -1052,11 +1052,11 @@
         </is>
       </c>
       <c r="P7" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R7" s="2" t="n">
@@ -1142,11 +1142,11 @@
         </is>
       </c>
       <c r="P8" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
@@ -1232,11 +1232,11 @@
         </is>
       </c>
       <c r="P9" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R9" s="2" t="n">
@@ -1320,11 +1320,11 @@
         </is>
       </c>
       <c r="P10" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
@@ -1408,11 +1408,11 @@
         </is>
       </c>
       <c r="P11" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R11" s="2" t="n">
@@ -1498,11 +1498,11 @@
         </is>
       </c>
       <c r="P12" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
@@ -1586,11 +1586,11 @@
         </is>
       </c>
       <c r="P13" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R13" s="2" t="n">
@@ -1674,11 +1674,11 @@
         </is>
       </c>
       <c r="P14" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
@@ -1762,11 +1762,11 @@
         </is>
       </c>
       <c r="P15" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R15" s="2" t="n">
@@ -1852,11 +1852,11 @@
         </is>
       </c>
       <c r="P16" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
@@ -1940,11 +1940,11 @@
         </is>
       </c>
       <c r="P17" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R17" s="2" t="n">
@@ -2028,11 +2028,11 @@
         </is>
       </c>
       <c r="P18" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
@@ -2118,11 +2118,11 @@
         </is>
       </c>
       <c r="P19" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R19" s="2" t="n">
@@ -2208,11 +2208,11 @@
         </is>
       </c>
       <c r="P20" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
@@ -2298,11 +2298,11 @@
         </is>
       </c>
       <c r="P21" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R21" s="2" t="n">
@@ -2388,11 +2388,11 @@
         </is>
       </c>
       <c r="P22" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
@@ -2478,11 +2478,11 @@
         </is>
       </c>
       <c r="P23" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R23" s="2" t="n">
@@ -2566,11 +2566,11 @@
         </is>
       </c>
       <c r="P24" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
@@ -2654,11 +2654,11 @@
         </is>
       </c>
       <c r="P25" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R25" s="2" t="n">
@@ -2742,11 +2742,11 @@
         </is>
       </c>
       <c r="P26" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
@@ -2828,11 +2828,11 @@
         </is>
       </c>
       <c r="P27" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R27" s="2" t="n">
@@ -2916,11 +2916,11 @@
         </is>
       </c>
       <c r="P28" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
@@ -2985,10 +2985,10 @@
         <v>21</v>
       </c>
       <c r="K29" t="n">
-        <v>21.9</v>
+        <v>22.5</v>
       </c>
       <c r="L29" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3004,11 +3004,11 @@
         </is>
       </c>
       <c r="P29" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R29" s="2" t="n">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="n">
-        <v>0.8999999999999986</v>
+        <v>1.5</v>
       </c>
       <c r="U29" t="n">
         <v>21.73333333333333</v>
@@ -3090,11 +3090,11 @@
         </is>
       </c>
       <c r="P30" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
@@ -3176,11 +3176,11 @@
         </is>
       </c>
       <c r="P31" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R31" s="2" t="n">
@@ -3262,11 +3262,11 @@
         </is>
       </c>
       <c r="P32" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
@@ -3348,11 +3348,11 @@
         </is>
       </c>
       <c r="P33" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R33" s="2" t="n">
@@ -3436,11 +3436,11 @@
         </is>
       </c>
       <c r="P34" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
@@ -3524,11 +3524,11 @@
         </is>
       </c>
       <c r="P35" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R35" s="2" t="n">
@@ -3593,10 +3593,10 @@
         <v>28</v>
       </c>
       <c r="K36" t="n">
-        <v>22.7</v>
+        <v>26.4</v>
       </c>
       <c r="L36" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3612,11 +3612,11 @@
         </is>
       </c>
       <c r="P36" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -3626,7 +3626,7 @@
         <v>28</v>
       </c>
       <c r="T36" t="n">
-        <v>-5.300000000000001</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U36" t="n">
         <v>24.9</v>
@@ -3681,10 +3681,10 @@
         <v>28</v>
       </c>
       <c r="K37" t="n">
-        <v>29.1</v>
+        <v>26</v>
       </c>
       <c r="L37" t="n">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3700,11 +3700,11 @@
         </is>
       </c>
       <c r="P37" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R37" s="2" t="n">
@@ -3714,7 +3714,7 @@
         <v>28</v>
       </c>
       <c r="T37" t="n">
-        <v>1.100000000000001</v>
+        <v>-2</v>
       </c>
       <c r="U37" t="n">
         <v>27.33333333333333</v>
@@ -3788,11 +3788,11 @@
         </is>
       </c>
       <c r="P38" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R38" s="2" t="n">
@@ -3876,11 +3876,11 @@
         </is>
       </c>
       <c r="P39" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R39" s="2" t="n">
@@ -3964,11 +3964,11 @@
         </is>
       </c>
       <c r="P40" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R40" s="2" t="n">
@@ -4033,10 +4033,10 @@
         <v>28</v>
       </c>
       <c r="K41" t="n">
-        <v>28.4</v>
+        <v>27.2</v>
       </c>
       <c r="L41" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
@@ -4052,11 +4052,11 @@
         </is>
       </c>
       <c r="P41" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R41" s="2" t="n">
@@ -4066,7 +4066,7 @@
         <v>28</v>
       </c>
       <c r="T41" t="n">
-        <v>0.3999999999999986</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U41" t="n">
         <v>28.06666666666666</v>
@@ -4140,11 +4140,11 @@
         </is>
       </c>
       <c r="P42" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R42" s="2" t="n">
@@ -4228,11 +4228,11 @@
         </is>
       </c>
       <c r="P43" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R43" s="2" t="n">
@@ -4316,11 +4316,11 @@
         </is>
       </c>
       <c r="P44" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R44" s="2" t="n">
@@ -4404,11 +4404,11 @@
         </is>
       </c>
       <c r="P45" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R45" s="2" t="n">
@@ -4490,11 +4490,11 @@
         </is>
       </c>
       <c r="P46" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R46" s="2" t="n">
@@ -4578,11 +4578,11 @@
         </is>
       </c>
       <c r="P47" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R47" s="2" t="n">
@@ -4664,11 +4664,11 @@
         </is>
       </c>
       <c r="P48" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R48" s="2" t="n">
@@ -4752,11 +4752,11 @@
         </is>
       </c>
       <c r="P49" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R49" s="2" t="n">
@@ -4840,11 +4840,11 @@
         </is>
       </c>
       <c r="P50" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R50" s="2" t="n">
@@ -4928,11 +4928,11 @@
         </is>
       </c>
       <c r="P51" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R51" s="2" t="n">
@@ -5016,11 +5016,11 @@
         </is>
       </c>
       <c r="P52" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R52" s="2" t="n">
@@ -5102,11 +5102,11 @@
         </is>
       </c>
       <c r="P53" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R53" s="2" t="n">
@@ -5190,11 +5190,11 @@
         </is>
       </c>
       <c r="P54" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R54" s="2" t="n">
@@ -5278,11 +5278,11 @@
         </is>
       </c>
       <c r="P55" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R55" s="2" t="n">
@@ -5366,11 +5366,11 @@
         </is>
       </c>
       <c r="P56" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R56" s="2" t="n">
@@ -5435,10 +5435,10 @@
         <v>28</v>
       </c>
       <c r="K57" t="n">
-        <v>26.5</v>
+        <v>28.4</v>
       </c>
       <c r="L57" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="M57" t="inlineStr">
         <is>
@@ -5454,11 +5454,11 @@
         </is>
       </c>
       <c r="P57" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R57" s="2" t="n">
@@ -5468,7 +5468,7 @@
         <v>28</v>
       </c>
       <c r="T57" t="n">
-        <v>-1.5</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U57" t="n">
         <v>27.53333333333333</v>
@@ -5523,10 +5523,10 @@
         <v>28</v>
       </c>
       <c r="K58" t="n">
-        <v>27.5</v>
+        <v>27.8</v>
       </c>
       <c r="L58" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -5542,11 +5542,11 @@
         </is>
       </c>
       <c r="P58" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R58" s="2" t="n">
@@ -5556,7 +5556,7 @@
         <v>28</v>
       </c>
       <c r="T58" t="n">
-        <v>-0.5</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U58" t="n">
         <v>27</v>
@@ -5611,10 +5611,10 @@
         <v>28</v>
       </c>
       <c r="K59" t="n">
-        <v>28.2</v>
+        <v>27.4</v>
       </c>
       <c r="L59" t="n">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
@@ -5630,11 +5630,11 @@
         </is>
       </c>
       <c r="P59" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R59" s="2" t="n">
@@ -5644,7 +5644,7 @@
         <v>28</v>
       </c>
       <c r="T59" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U59" t="n">
         <v>28.2</v>
@@ -5718,11 +5718,11 @@
         </is>
       </c>
       <c r="P60" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R60" s="2" t="n">
@@ -5806,11 +5806,11 @@
         </is>
       </c>
       <c r="P61" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R61" s="2" t="n">
@@ -5894,11 +5894,11 @@
         </is>
       </c>
       <c r="P62" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R62" s="2" t="n">
@@ -5982,11 +5982,11 @@
         </is>
       </c>
       <c r="P63" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R63" s="2" t="n">
@@ -6070,11 +6070,11 @@
         </is>
       </c>
       <c r="P64" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R64" s="2" t="n">
@@ -6158,11 +6158,11 @@
         </is>
       </c>
       <c r="P65" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R65" s="2" t="n">
@@ -6246,11 +6246,11 @@
         </is>
       </c>
       <c r="P66" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R66" s="2" t="n">
@@ -6334,11 +6334,11 @@
         </is>
       </c>
       <c r="P67" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R67" s="2" t="n">
@@ -6422,11 +6422,11 @@
         </is>
       </c>
       <c r="P68" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R68" s="2" t="n">
@@ -6506,11 +6506,11 @@
         </is>
       </c>
       <c r="P69" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R69" s="2" t="n">
@@ -6575,10 +6575,10 @@
         <v>21</v>
       </c>
       <c r="K70" t="n">
-        <v>22.8</v>
+        <v>20.1</v>
       </c>
       <c r="L70" t="n">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="P70" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R70" s="2" t="n">
@@ -6608,7 +6608,7 @@
         <v>21</v>
       </c>
       <c r="T70" t="n">
-        <v>1.800000000000001</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U70" t="n">
         <v>21.53333333333333</v>
@@ -6682,11 +6682,11 @@
         </is>
       </c>
       <c r="P71" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R71" s="2" t="n">
@@ -6770,11 +6770,11 @@
         </is>
       </c>
       <c r="P72" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R72" s="2" t="n">
@@ -6858,11 +6858,11 @@
         </is>
       </c>
       <c r="P73" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R73" s="2" t="n">
@@ -6946,11 +6946,11 @@
         </is>
       </c>
       <c r="P74" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R74" s="2" t="n">
@@ -7034,11 +7034,11 @@
         </is>
       </c>
       <c r="P75" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R75" s="2" t="n">
@@ -7120,11 +7120,11 @@
         </is>
       </c>
       <c r="P76" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R76" s="2" t="n">
@@ -7208,11 +7208,11 @@
         </is>
       </c>
       <c r="P77" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R77" s="2" t="n">
@@ -7296,11 +7296,11 @@
         </is>
       </c>
       <c r="P78" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R78" s="2" t="n">
@@ -7384,11 +7384,11 @@
         </is>
       </c>
       <c r="P79" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R79" s="2" t="n">
@@ -7470,11 +7470,11 @@
         </is>
       </c>
       <c r="P80" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R80" s="2" t="n">
@@ -7539,10 +7539,10 @@
         <v>21</v>
       </c>
       <c r="K81" t="n">
-        <v>22</v>
+        <v>19.7</v>
       </c>
       <c r="L81" t="n">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7558,11 +7558,11 @@
         </is>
       </c>
       <c r="P81" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R81" s="2" t="n">
@@ -7572,7 +7572,7 @@
         <v>21</v>
       </c>
       <c r="T81" t="n">
-        <v>1</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U81" t="n">
         <v>21</v>
@@ -7646,11 +7646,11 @@
         </is>
       </c>
       <c r="P82" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R82" s="2" t="n">
@@ -7734,11 +7734,11 @@
         </is>
       </c>
       <c r="P83" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R83" s="2" t="n">
@@ -7822,11 +7822,11 @@
         </is>
       </c>
       <c r="P84" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R84" s="2" t="n">
@@ -7910,11 +7910,11 @@
         </is>
       </c>
       <c r="P85" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R85" s="2" t="n">
@@ -7998,11 +7998,11 @@
         </is>
       </c>
       <c r="P86" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R86" s="2" t="n">
@@ -8086,11 +8086,11 @@
         </is>
       </c>
       <c r="P87" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R87" s="2" t="n">
@@ -8174,11 +8174,11 @@
         </is>
       </c>
       <c r="P88" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R88" s="2" t="n">
@@ -8262,11 +8262,11 @@
         </is>
       </c>
       <c r="P89" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R89" s="2" t="n">
@@ -8348,11 +8348,11 @@
         </is>
       </c>
       <c r="P90" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R90" s="2" t="n">
@@ -8436,11 +8436,11 @@
         </is>
       </c>
       <c r="P91" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R91" s="2" t="n">
@@ -8524,11 +8524,11 @@
         </is>
       </c>
       <c r="P92" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R92" s="2" t="n">
@@ -8612,11 +8612,11 @@
         </is>
       </c>
       <c r="P93" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R93" s="2" t="n">
@@ -8700,11 +8700,11 @@
         </is>
       </c>
       <c r="P94" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R94" s="2" t="n">
@@ -8788,11 +8788,11 @@
         </is>
       </c>
       <c r="P95" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R95" s="2" t="n">
@@ -8876,11 +8876,11 @@
         </is>
       </c>
       <c r="P96" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R96" s="2" t="n">
@@ -8964,11 +8964,11 @@
         </is>
       </c>
       <c r="P97" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R97" s="2" t="n">
@@ -9052,11 +9052,11 @@
         </is>
       </c>
       <c r="P98" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R98" s="2" t="n">
@@ -9121,10 +9121,10 @@
         <v>24.5</v>
       </c>
       <c r="K99" t="n">
-        <v>29.6</v>
+        <v>22.5</v>
       </c>
       <c r="L99" t="n">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="M99" t="inlineStr">
         <is>
@@ -9140,11 +9140,11 @@
         </is>
       </c>
       <c r="P99" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R99" s="2" t="n">
@@ -9154,7 +9154,7 @@
         <v>28</v>
       </c>
       <c r="T99" t="n">
-        <v>5.100000000000001</v>
+        <v>-2</v>
       </c>
       <c r="U99" t="n">
         <v>26.3</v>
@@ -9228,11 +9228,11 @@
         </is>
       </c>
       <c r="P100" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R100" s="2" t="n">
@@ -9316,11 +9316,11 @@
         </is>
       </c>
       <c r="P101" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R101" s="2" t="n">
@@ -9404,11 +9404,11 @@
         </is>
       </c>
       <c r="P102" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R102" s="2" t="n">
@@ -9492,11 +9492,11 @@
         </is>
       </c>
       <c r="P103" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R103" s="2" t="n">
@@ -9580,11 +9580,11 @@
         </is>
       </c>
       <c r="P104" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R104" s="2" t="n">
@@ -9668,11 +9668,11 @@
         </is>
       </c>
       <c r="P105" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R105" s="2" t="n">
@@ -9756,11 +9756,11 @@
         </is>
       </c>
       <c r="P106" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R106" s="2" t="n">
@@ -9844,11 +9844,11 @@
         </is>
       </c>
       <c r="P107" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R107" s="2" t="n">
@@ -9932,11 +9932,11 @@
         </is>
       </c>
       <c r="P108" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R108" s="2" t="n">
@@ -10020,11 +10020,11 @@
         </is>
       </c>
       <c r="P109" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R109" s="2" t="n">
@@ -10108,11 +10108,11 @@
         </is>
       </c>
       <c r="P110" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R110" s="2" t="n">
@@ -10196,11 +10196,11 @@
         </is>
       </c>
       <c r="P111" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R111" s="2" t="n">
@@ -10219,7 +10219,7 @@
         <v>3</v>
       </c>
       <c r="W111" t="n">
-        <v>25.57777777777777</v>
+        <v>25.57777777777778</v>
       </c>
       <c r="X111" t="n">
         <v>21</v>
@@ -10284,11 +10284,11 @@
         </is>
       </c>
       <c r="P112" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R112" s="2" t="n">
@@ -10372,11 +10372,11 @@
         </is>
       </c>
       <c r="P113" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R113" s="2" t="n">
@@ -10460,11 +10460,11 @@
         </is>
       </c>
       <c r="P114" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R114" s="2" t="n">
@@ -10548,11 +10548,11 @@
         </is>
       </c>
       <c r="P115" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R115" s="2" t="n">
@@ -10636,11 +10636,11 @@
         </is>
       </c>
       <c r="P116" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R116" s="2" t="n">
@@ -10724,11 +10724,11 @@
         </is>
       </c>
       <c r="P117" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R117" s="2" t="n">
@@ -10812,11 +10812,11 @@
         </is>
       </c>
       <c r="P118" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R118" s="2" t="n">
@@ -10900,11 +10900,11 @@
         </is>
       </c>
       <c r="P119" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R119" s="2" t="n">
@@ -10988,11 +10988,11 @@
         </is>
       </c>
       <c r="P120" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R120" s="2" t="n">
@@ -11076,11 +11076,11 @@
         </is>
       </c>
       <c r="P121" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R121" s="2" t="n">
@@ -11164,11 +11164,11 @@
         </is>
       </c>
       <c r="P122" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R122" s="2" t="n">
@@ -11252,11 +11252,11 @@
         </is>
       </c>
       <c r="P123" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R123" s="2" t="n">
@@ -11340,11 +11340,11 @@
         </is>
       </c>
       <c r="P124" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R124" s="2" t="n">
@@ -11428,11 +11428,11 @@
         </is>
       </c>
       <c r="P125" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R125" s="2" t="n">
@@ -11516,11 +11516,11 @@
         </is>
       </c>
       <c r="P126" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R126" s="2" t="n">
@@ -11604,11 +11604,11 @@
         </is>
       </c>
       <c r="P127" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R127" s="2" t="n">
@@ -11692,11 +11692,11 @@
         </is>
       </c>
       <c r="P128" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R128" s="2" t="n">
@@ -11780,11 +11780,11 @@
         </is>
       </c>
       <c r="P129" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R129" s="2" t="n">
@@ -11868,11 +11868,11 @@
         </is>
       </c>
       <c r="P130" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R130" s="2" t="n">
@@ -11956,11 +11956,11 @@
         </is>
       </c>
       <c r="P131" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R131" s="2" t="n">
@@ -12044,11 +12044,11 @@
         </is>
       </c>
       <c r="P132" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R132" s="2" t="n">
@@ -12130,11 +12130,11 @@
         </is>
       </c>
       <c r="P133" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R133" s="2" t="n">
@@ -12218,11 +12218,11 @@
         </is>
       </c>
       <c r="P134" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R134" s="2" t="n">
@@ -12306,11 +12306,11 @@
         </is>
       </c>
       <c r="P135" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R135" s="2" t="n">
@@ -12394,11 +12394,11 @@
         </is>
       </c>
       <c r="P136" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R136" s="2" t="n">
@@ -12482,11 +12482,11 @@
         </is>
       </c>
       <c r="P137" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R137" s="2" t="n">
@@ -12570,11 +12570,11 @@
         </is>
       </c>
       <c r="P138" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R138" s="2" t="n">
@@ -12658,11 +12658,11 @@
         </is>
       </c>
       <c r="P139" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R139" s="2" t="n">
@@ -12744,11 +12744,11 @@
         </is>
       </c>
       <c r="P140" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R140" s="2" t="n">
@@ -12832,11 +12832,11 @@
         </is>
       </c>
       <c r="P141" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R141" s="2" t="n">
@@ -12920,11 +12920,11 @@
         </is>
       </c>
       <c r="P142" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R142" s="2" t="n">
@@ -13006,11 +13006,11 @@
         </is>
       </c>
       <c r="P143" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R143" s="2" t="n">
@@ -13094,11 +13094,11 @@
         </is>
       </c>
       <c r="P144" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R144" s="2" t="n">
@@ -13182,11 +13182,11 @@
         </is>
       </c>
       <c r="P145" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R145" s="2" t="n">
@@ -13270,11 +13270,11 @@
         </is>
       </c>
       <c r="P146" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R146" s="2" t="n">
@@ -13358,11 +13358,11 @@
         </is>
       </c>
       <c r="P147" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R147" s="2" t="n">
@@ -13444,11 +13444,11 @@
         </is>
       </c>
       <c r="P148" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R148" s="2" t="n">
@@ -13532,11 +13532,11 @@
         </is>
       </c>
       <c r="P149" s="2" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R149" s="2" t="n">

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-17 06:38:37
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2811,10 +2811,10 @@
         <v>24</v>
       </c>
       <c r="K27" t="n">
-        <v>15.8</v>
+        <v>21.6</v>
       </c>
       <c r="L27" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -2844,7 +2844,7 @@
         <v>28</v>
       </c>
       <c r="T27" t="n">
-        <v>-8.199999999999999</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="U27" t="n">
         <v>19.2</v>
@@ -6563,10 +6563,10 @@
         <v>35</v>
       </c>
       <c r="K70" t="n">
-        <v>31.8</v>
+        <v>38.1</v>
       </c>
       <c r="L70" t="n">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
         <v>41</v>
       </c>
       <c r="T70" t="n">
-        <v>-3.199999999999999</v>
+        <v>3.100000000000001</v>
       </c>
       <c r="U70" t="n">
         <v>35.3</v>
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L77" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L81" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L88" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L93" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -11475,10 +11475,10 @@
         <v>21</v>
       </c>
       <c r="K126" t="n">
-        <v>19.4</v>
+        <v>21.6</v>
       </c>
       <c r="L126" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="M126" t="inlineStr">
         <is>
@@ -11508,7 +11508,7 @@
         <v>21</v>
       </c>
       <c r="T126" t="n">
-        <v>-1.600000000000001</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U126" t="n">
         <v>19.93333333333333</v>
@@ -11651,10 +11651,10 @@
         <v>21</v>
       </c>
       <c r="K128" t="n">
-        <v>20.3</v>
+        <v>23.2</v>
       </c>
       <c r="L128" t="n">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="M128" t="inlineStr">
         <is>
@@ -11684,7 +11684,7 @@
         <v>21</v>
       </c>
       <c r="T128" t="n">
-        <v>-0.6999999999999993</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U128" t="n">
         <v>22.36666666666666</v>
@@ -11869,7 +11869,7 @@
         <v>3</v>
       </c>
       <c r="W130" t="n">
-        <v>34.15555555555556</v>
+        <v>34.15555555555555</v>
       </c>
       <c r="X130" t="n">
         <v>31.5</v>
@@ -21433,7 +21433,7 @@
         <v>3</v>
       </c>
       <c r="W239" t="n">
-        <v>22.92222222222223</v>
+        <v>22.92222222222222</v>
       </c>
       <c r="X239" t="n">
         <v>20.5</v>
@@ -23401,10 +23401,10 @@
         <v>28</v>
       </c>
       <c r="K262" t="n">
-        <v>28.4</v>
+        <v>27.2</v>
       </c>
       <c r="L262" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M262" t="inlineStr">
         <is>
@@ -23434,7 +23434,7 @@
         <v>28</v>
       </c>
       <c r="T262" t="n">
-        <v>0.3999999999999986</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U262" t="n">
         <v>28.06666666666666</v>
@@ -24979,10 +24979,10 @@
         <v>28</v>
       </c>
       <c r="K280" t="n">
-        <v>29</v>
+        <v>28.2</v>
       </c>
       <c r="L280" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="M280" t="inlineStr">
         <is>
@@ -25012,7 +25012,7 @@
         <v>28</v>
       </c>
       <c r="T280" t="n">
-        <v>1</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U280" t="n">
         <v>28.2</v>
@@ -26645,10 +26645,10 @@
         <v>21</v>
       </c>
       <c r="K299" t="n">
-        <v>18</v>
+        <v>21.1</v>
       </c>
       <c r="L299" t="n">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="M299" t="inlineStr">
         <is>
@@ -26678,7 +26678,7 @@
         <v>21</v>
       </c>
       <c r="T299" t="n">
-        <v>-3</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U299" t="n">
         <v>19.53333333333333</v>
@@ -27697,10 +27697,10 @@
         <v>24.5</v>
       </c>
       <c r="K311" t="n">
-        <v>22.6</v>
+        <v>25</v>
       </c>
       <c r="L311" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="M311" t="inlineStr">
         <is>
@@ -27730,7 +27730,7 @@
         <v>28</v>
       </c>
       <c r="T311" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="U311" t="n">
         <v>24.8</v>
@@ -28049,10 +28049,10 @@
         <v>24.5</v>
       </c>
       <c r="K315" t="n">
-        <v>24.7</v>
+        <v>22.8</v>
       </c>
       <c r="L315" t="n">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="M315" t="inlineStr">
         <is>
@@ -28082,7 +28082,7 @@
         <v>28</v>
       </c>
       <c r="T315" t="n">
-        <v>0.1999999999999993</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U315" t="n">
         <v>24.1</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L323" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L331" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -30161,10 +30161,10 @@
         <v>24.5</v>
       </c>
       <c r="K339" t="n">
-        <v>24.7</v>
+        <v>24</v>
       </c>
       <c r="L339" t="n">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="M339" t="inlineStr">
         <is>
@@ -30194,7 +30194,7 @@
         <v>28</v>
       </c>
       <c r="T339" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.5</v>
       </c>
       <c r="U339" t="n">
         <v>24.1</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L353" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-17 15:03:00
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -6475,10 +6475,10 @@
         <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>34.3</v>
+        <v>32.3</v>
       </c>
       <c r="L69" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>41</v>
       </c>
       <c r="T69" t="n">
-        <v>-0.7000000000000028</v>
+        <v>-2.700000000000003</v>
       </c>
       <c r="U69" t="n">
         <v>32.96666666666666</v>
@@ -6563,10 +6563,10 @@
         <v>35</v>
       </c>
       <c r="K70" t="n">
-        <v>38.1</v>
+        <v>31.8</v>
       </c>
       <c r="L70" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
         <v>41</v>
       </c>
       <c r="T70" t="n">
-        <v>3.100000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U70" t="n">
         <v>35.3</v>
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L77" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L81" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L88" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L93" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -10331,10 +10331,10 @@
         <v>35</v>
       </c>
       <c r="K113" t="n">
-        <v>27.3</v>
+        <v>54.5</v>
       </c>
       <c r="L113" t="n">
-        <v>78</v>
+        <v>156</v>
       </c>
       <c r="M113" t="inlineStr">
         <is>
@@ -10364,7 +10364,7 @@
         <v>41</v>
       </c>
       <c r="T113" t="n">
-        <v>-7.699999999999999</v>
+        <v>19.5</v>
       </c>
       <c r="U113" t="n">
         <v>44.9</v>
@@ -11211,10 +11211,10 @@
         <v>28</v>
       </c>
       <c r="K123" t="n">
-        <v>33.5</v>
+        <v>31.6</v>
       </c>
       <c r="L123" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="M123" t="inlineStr">
         <is>
@@ -11244,7 +11244,7 @@
         <v>28</v>
       </c>
       <c r="T123" t="n">
-        <v>5.5</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U123" t="n">
         <v>30.83333333333333</v>
@@ -11299,10 +11299,10 @@
         <v>21</v>
       </c>
       <c r="K124" t="n">
-        <v>23.7</v>
+        <v>20.4</v>
       </c>
       <c r="L124" t="n">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11332,7 +11332,7 @@
         <v>21</v>
       </c>
       <c r="T124" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U124" t="n">
         <v>21.43333333333333</v>
@@ -11387,10 +11387,10 @@
         <v>21</v>
       </c>
       <c r="K125" t="n">
-        <v>22.6</v>
+        <v>18.4</v>
       </c>
       <c r="L125" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="M125" t="inlineStr">
         <is>
@@ -11420,7 +11420,7 @@
         <v>21</v>
       </c>
       <c r="T125" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U125" t="n">
         <v>22.93333333333334</v>
@@ -11563,10 +11563,10 @@
         <v>35</v>
       </c>
       <c r="K127" t="n">
-        <v>30.5</v>
+        <v>35.4</v>
       </c>
       <c r="L127" t="n">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="M127" t="inlineStr">
         <is>
@@ -11596,7 +11596,7 @@
         <v>41</v>
       </c>
       <c r="T127" t="n">
-        <v>-4.5</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U127" t="n">
         <v>34.13333333333333</v>
@@ -11605,7 +11605,7 @@
         <v>3</v>
       </c>
       <c r="W127" t="n">
-        <v>36.32592592592593</v>
+        <v>36.32592592592592</v>
       </c>
       <c r="X127" t="n">
         <v>31.5</v>
@@ -11651,10 +11651,10 @@
         <v>21</v>
       </c>
       <c r="K128" t="n">
-        <v>23.2</v>
+        <v>20.3</v>
       </c>
       <c r="L128" t="n">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="M128" t="inlineStr">
         <is>
@@ -11684,10 +11684,10 @@
         <v>21</v>
       </c>
       <c r="T128" t="n">
-        <v>2.199999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="U128" t="n">
-        <v>22.36666666666666</v>
+        <v>22.36666666666667</v>
       </c>
       <c r="V128" t="n">
         <v>3</v>
@@ -11739,10 +11739,10 @@
         <v>28</v>
       </c>
       <c r="K129" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="L129" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="M129" t="inlineStr">
         <is>
@@ -11772,10 +11772,10 @@
         <v>28</v>
       </c>
       <c r="T129" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U129" t="n">
-        <v>25.36666666666666</v>
+        <v>25.36666666666667</v>
       </c>
       <c r="V129" t="n">
         <v>3</v>
@@ -11827,10 +11827,10 @@
         <v>35</v>
       </c>
       <c r="K130" t="n">
-        <v>33.9</v>
+        <v>30.7</v>
       </c>
       <c r="L130" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -11860,7 +11860,7 @@
         <v>41</v>
       </c>
       <c r="T130" t="n">
-        <v>-1.100000000000001</v>
+        <v>-4.300000000000001</v>
       </c>
       <c r="U130" t="n">
         <v>31.83333333333333</v>
@@ -11915,7 +11915,7 @@
         <v>28</v>
       </c>
       <c r="K131" t="n">
-        <v>27.4</v>
+        <v>27.3</v>
       </c>
       <c r="L131" t="n">
         <v>98</v>
@@ -11948,7 +11948,7 @@
         <v>28</v>
       </c>
       <c r="T131" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="U131" t="n">
         <v>28.23333333333333</v>
@@ -12003,10 +12003,10 @@
         <v>21</v>
       </c>
       <c r="K132" t="n">
-        <v>24</v>
+        <v>20.4</v>
       </c>
       <c r="L132" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="M132" t="inlineStr">
         <is>
@@ -12036,7 +12036,7 @@
         <v>21</v>
       </c>
       <c r="T132" t="n">
-        <v>3</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U132" t="n">
         <v>22.16666666666667</v>
@@ -12091,10 +12091,10 @@
         <v>35</v>
       </c>
       <c r="K133" t="n">
-        <v>36.6</v>
+        <v>36.5</v>
       </c>
       <c r="L133" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M133" t="inlineStr">
         <is>
@@ -12124,7 +12124,7 @@
         <v>41</v>
       </c>
       <c r="T133" t="n">
-        <v>1.600000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="U133" t="n">
         <v>35.63333333333333</v>
@@ -12133,7 +12133,7 @@
         <v>3</v>
       </c>
       <c r="W133" t="n">
-        <v>41.38148148148148</v>
+        <v>41.38148148148147</v>
       </c>
       <c r="X133" t="n">
         <v>31.5</v>
@@ -15951,7 +15951,7 @@
         <v>28</v>
       </c>
       <c r="K177" t="n">
-        <v>26.4</v>
+        <v>26.3</v>
       </c>
       <c r="L177" t="n">
         <v>94</v>
@@ -15984,7 +15984,7 @@
         <v>28</v>
       </c>
       <c r="T177" t="n">
-        <v>-1.600000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U177" t="n">
         <v>26.6</v>
@@ -16039,10 +16039,10 @@
         <v>21</v>
       </c>
       <c r="K178" t="n">
-        <v>13</v>
+        <v>19.3</v>
       </c>
       <c r="L178" t="n">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="M178" t="inlineStr">
         <is>
@@ -16072,7 +16072,7 @@
         <v>21</v>
       </c>
       <c r="T178" t="n">
-        <v>-8</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U178" t="n">
         <v>18.23333333333333</v>
@@ -16213,10 +16213,10 @@
         <v>28</v>
       </c>
       <c r="K180" t="n">
-        <v>23.6</v>
+        <v>29</v>
       </c>
       <c r="L180" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="M180" t="inlineStr">
         <is>
@@ -16246,7 +16246,7 @@
         <v>28</v>
       </c>
       <c r="T180" t="n">
-        <v>-4.399999999999999</v>
+        <v>1</v>
       </c>
       <c r="U180" t="n">
         <v>25.33333333333333</v>
@@ -16301,10 +16301,10 @@
         <v>35</v>
       </c>
       <c r="K181" t="n">
-        <v>38.3</v>
+        <v>34.3</v>
       </c>
       <c r="L181" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="M181" t="inlineStr">
         <is>
@@ -16334,7 +16334,7 @@
         <v>41</v>
       </c>
       <c r="T181" t="n">
-        <v>3.299999999999997</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="U181" t="n">
         <v>35.66666666666666</v>
@@ -16389,7 +16389,7 @@
         <v>21</v>
       </c>
       <c r="K182" t="n">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="L182" t="n">
         <v>108</v>
@@ -16422,10 +16422,10 @@
         <v>21</v>
       </c>
       <c r="T182" t="n">
-        <v>1.699999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U182" t="n">
-        <v>21.86666666666666</v>
+        <v>21.86666666666667</v>
       </c>
       <c r="V182" t="n">
         <v>3</v>
@@ -16477,10 +16477,10 @@
         <v>28</v>
       </c>
       <c r="K183" t="n">
-        <v>36.4</v>
+        <v>40.2</v>
       </c>
       <c r="L183" t="n">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="M183" t="inlineStr">
         <is>
@@ -16510,7 +16510,7 @@
         <v>28</v>
       </c>
       <c r="T183" t="n">
-        <v>8.399999999999999</v>
+        <v>12.2</v>
       </c>
       <c r="U183" t="n">
         <v>33.36666666666667</v>
@@ -16653,10 +16653,10 @@
         <v>28</v>
       </c>
       <c r="K185" t="n">
-        <v>27.6</v>
+        <v>28.5</v>
       </c>
       <c r="L185" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M185" t="inlineStr">
         <is>
@@ -16686,7 +16686,7 @@
         <v>28</v>
       </c>
       <c r="T185" t="n">
-        <v>-0.3999999999999986</v>
+        <v>0.5</v>
       </c>
       <c r="U185" t="n">
         <v>27.5</v>
@@ -16741,10 +16741,10 @@
         <v>28</v>
       </c>
       <c r="K186" t="n">
-        <v>30.3</v>
+        <v>24</v>
       </c>
       <c r="L186" t="n">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="M186" t="inlineStr">
         <is>
@@ -16774,7 +16774,7 @@
         <v>28</v>
       </c>
       <c r="T186" t="n">
-        <v>2.300000000000001</v>
+        <v>-4</v>
       </c>
       <c r="U186" t="n">
         <v>27.23333333333333</v>
@@ -16829,10 +16829,10 @@
         <v>28</v>
       </c>
       <c r="K187" t="n">
-        <v>30.4</v>
+        <v>28.6</v>
       </c>
       <c r="L187" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="M187" t="inlineStr">
         <is>
@@ -16862,7 +16862,7 @@
         <v>28</v>
       </c>
       <c r="T187" t="n">
-        <v>2.399999999999999</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U187" t="n">
         <v>28.83333333333333</v>
@@ -16917,10 +16917,10 @@
         <v>35</v>
       </c>
       <c r="K188" t="n">
-        <v>32.7</v>
+        <v>32.4</v>
       </c>
       <c r="L188" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M188" t="inlineStr">
         <is>
@@ -16950,7 +16950,7 @@
         <v>41</v>
       </c>
       <c r="T188" t="n">
-        <v>-2.299999999999997</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U188" t="n">
         <v>32.26666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-17 17:09:09
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -6475,10 +6475,10 @@
         <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>32.3</v>
+        <v>34.3</v>
       </c>
       <c r="L69" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>41</v>
       </c>
       <c r="T69" t="n">
-        <v>-2.700000000000003</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="U69" t="n">
         <v>32.96666666666666</v>
@@ -6563,10 +6563,10 @@
         <v>35</v>
       </c>
       <c r="K70" t="n">
-        <v>31.8</v>
+        <v>38.1</v>
       </c>
       <c r="L70" t="n">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
         <v>41</v>
       </c>
       <c r="T70" t="n">
-        <v>-3.199999999999999</v>
+        <v>3.100000000000001</v>
       </c>
       <c r="U70" t="n">
         <v>35.3</v>
@@ -10067,10 +10067,10 @@
         <v>35</v>
       </c>
       <c r="K110" t="n">
-        <v>38.4</v>
+        <v>38.1</v>
       </c>
       <c r="L110" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M110" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
         <v>41</v>
       </c>
       <c r="T110" t="n">
-        <v>3.399999999999999</v>
+        <v>3.100000000000001</v>
       </c>
       <c r="U110" t="n">
         <v>36.1</v>
@@ -10331,10 +10331,10 @@
         <v>35</v>
       </c>
       <c r="K113" t="n">
-        <v>54.5</v>
+        <v>27.3</v>
       </c>
       <c r="L113" t="n">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="M113" t="inlineStr">
         <is>
@@ -10364,7 +10364,7 @@
         <v>41</v>
       </c>
       <c r="T113" t="n">
-        <v>19.5</v>
+        <v>-7.699999999999999</v>
       </c>
       <c r="U113" t="n">
         <v>44.9</v>
@@ -10507,10 +10507,10 @@
         <v>35</v>
       </c>
       <c r="K115" t="n">
-        <v>22.5</v>
+        <v>26.3</v>
       </c>
       <c r="L115" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         <v>41</v>
       </c>
       <c r="T115" t="n">
-        <v>-12.5</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="U115" t="n">
         <v>25.5</v>
@@ -11211,10 +11211,10 @@
         <v>28</v>
       </c>
       <c r="K123" t="n">
-        <v>31.6</v>
+        <v>33.5</v>
       </c>
       <c r="L123" t="n">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="M123" t="inlineStr">
         <is>
@@ -11244,7 +11244,7 @@
         <v>28</v>
       </c>
       <c r="T123" t="n">
-        <v>3.600000000000001</v>
+        <v>5.5</v>
       </c>
       <c r="U123" t="n">
         <v>30.83333333333333</v>
@@ -11299,10 +11299,10 @@
         <v>21</v>
       </c>
       <c r="K124" t="n">
-        <v>20.4</v>
+        <v>23.7</v>
       </c>
       <c r="L124" t="n">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11332,7 +11332,7 @@
         <v>21</v>
       </c>
       <c r="T124" t="n">
-        <v>-0.6000000000000014</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U124" t="n">
         <v>21.43333333333333</v>
@@ -11387,10 +11387,10 @@
         <v>21</v>
       </c>
       <c r="K125" t="n">
-        <v>18.4</v>
+        <v>22.6</v>
       </c>
       <c r="L125" t="n">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="M125" t="inlineStr">
         <is>
@@ -11420,7 +11420,7 @@
         <v>21</v>
       </c>
       <c r="T125" t="n">
-        <v>-2.600000000000001</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U125" t="n">
         <v>22.93333333333334</v>
@@ -11563,10 +11563,10 @@
         <v>35</v>
       </c>
       <c r="K127" t="n">
-        <v>35.4</v>
+        <v>30.5</v>
       </c>
       <c r="L127" t="n">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="M127" t="inlineStr">
         <is>
@@ -11596,7 +11596,7 @@
         <v>41</v>
       </c>
       <c r="T127" t="n">
-        <v>0.3999999999999986</v>
+        <v>-4.5</v>
       </c>
       <c r="U127" t="n">
         <v>34.13333333333333</v>
@@ -11605,7 +11605,7 @@
         <v>3</v>
       </c>
       <c r="W127" t="n">
-        <v>36.32592592592592</v>
+        <v>36.32592592592593</v>
       </c>
       <c r="X127" t="n">
         <v>31.5</v>
@@ -11651,10 +11651,10 @@
         <v>21</v>
       </c>
       <c r="K128" t="n">
-        <v>20.3</v>
+        <v>23.2</v>
       </c>
       <c r="L128" t="n">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="M128" t="inlineStr">
         <is>
@@ -11684,10 +11684,10 @@
         <v>21</v>
       </c>
       <c r="T128" t="n">
-        <v>-0.6999999999999993</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U128" t="n">
-        <v>22.36666666666667</v>
+        <v>22.36666666666666</v>
       </c>
       <c r="V128" t="n">
         <v>3</v>
@@ -11739,10 +11739,10 @@
         <v>28</v>
       </c>
       <c r="K129" t="n">
-        <v>24.6</v>
+        <v>27.7</v>
       </c>
       <c r="L129" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="M129" t="inlineStr">
         <is>
@@ -11772,10 +11772,10 @@
         <v>28</v>
       </c>
       <c r="T129" t="n">
-        <v>-3.399999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U129" t="n">
-        <v>25.36666666666667</v>
+        <v>25.36666666666666</v>
       </c>
       <c r="V129" t="n">
         <v>3</v>
@@ -11827,10 +11827,10 @@
         <v>35</v>
       </c>
       <c r="K130" t="n">
-        <v>30.7</v>
+        <v>33.9</v>
       </c>
       <c r="L130" t="n">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -11860,7 +11860,7 @@
         <v>41</v>
       </c>
       <c r="T130" t="n">
-        <v>-4.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U130" t="n">
         <v>31.83333333333333</v>
@@ -11869,7 +11869,7 @@
         <v>3</v>
       </c>
       <c r="W130" t="n">
-        <v>34.15555555555555</v>
+        <v>34.15555555555556</v>
       </c>
       <c r="X130" t="n">
         <v>31.5</v>
@@ -11915,7 +11915,7 @@
         <v>28</v>
       </c>
       <c r="K131" t="n">
-        <v>27.3</v>
+        <v>27.4</v>
       </c>
       <c r="L131" t="n">
         <v>98</v>
@@ -11948,7 +11948,7 @@
         <v>28</v>
       </c>
       <c r="T131" t="n">
-        <v>-0.6999999999999993</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U131" t="n">
         <v>28.23333333333333</v>
@@ -12003,10 +12003,10 @@
         <v>21</v>
       </c>
       <c r="K132" t="n">
-        <v>20.4</v>
+        <v>24</v>
       </c>
       <c r="L132" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="M132" t="inlineStr">
         <is>
@@ -12036,7 +12036,7 @@
         <v>21</v>
       </c>
       <c r="T132" t="n">
-        <v>-0.6000000000000014</v>
+        <v>3</v>
       </c>
       <c r="U132" t="n">
         <v>22.16666666666667</v>
@@ -12091,10 +12091,10 @@
         <v>35</v>
       </c>
       <c r="K133" t="n">
-        <v>36.5</v>
+        <v>36.6</v>
       </c>
       <c r="L133" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="M133" t="inlineStr">
         <is>
@@ -12124,7 +12124,7 @@
         <v>41</v>
       </c>
       <c r="T133" t="n">
-        <v>1.5</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U133" t="n">
         <v>35.63333333333333</v>
@@ -12133,7 +12133,7 @@
         <v>3</v>
       </c>
       <c r="W133" t="n">
-        <v>41.38148148148147</v>
+        <v>41.38148148148148</v>
       </c>
       <c r="X133" t="n">
         <v>31.5</v>
@@ -12443,10 +12443,10 @@
         <v>31</v>
       </c>
       <c r="K137" t="n">
-        <v>31.9</v>
+        <v>30.5</v>
       </c>
       <c r="L137" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="M137" t="inlineStr">
         <is>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="S137" t="inlineStr"/>
       <c r="T137" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.5</v>
       </c>
       <c r="U137" t="n">
         <v>31.23333333333333</v>
@@ -15951,7 +15951,7 @@
         <v>28</v>
       </c>
       <c r="K177" t="n">
-        <v>26.3</v>
+        <v>26.4</v>
       </c>
       <c r="L177" t="n">
         <v>94</v>
@@ -15984,7 +15984,7 @@
         <v>28</v>
       </c>
       <c r="T177" t="n">
-        <v>-1.699999999999999</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U177" t="n">
         <v>26.6</v>
@@ -16039,10 +16039,10 @@
         <v>21</v>
       </c>
       <c r="K178" t="n">
-        <v>19.3</v>
+        <v>13</v>
       </c>
       <c r="L178" t="n">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="M178" t="inlineStr">
         <is>
@@ -16072,7 +16072,7 @@
         <v>21</v>
       </c>
       <c r="T178" t="n">
-        <v>-1.699999999999999</v>
+        <v>-8</v>
       </c>
       <c r="U178" t="n">
         <v>18.23333333333333</v>
@@ -16213,10 +16213,10 @@
         <v>28</v>
       </c>
       <c r="K180" t="n">
-        <v>29</v>
+        <v>23.6</v>
       </c>
       <c r="L180" t="n">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="M180" t="inlineStr">
         <is>
@@ -16246,7 +16246,7 @@
         <v>28</v>
       </c>
       <c r="T180" t="n">
-        <v>1</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="U180" t="n">
         <v>25.33333333333333</v>
@@ -16301,10 +16301,10 @@
         <v>35</v>
       </c>
       <c r="K181" t="n">
-        <v>34.3</v>
+        <v>38.3</v>
       </c>
       <c r="L181" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="M181" t="inlineStr">
         <is>
@@ -16334,7 +16334,7 @@
         <v>41</v>
       </c>
       <c r="T181" t="n">
-        <v>-0.7000000000000028</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U181" t="n">
         <v>35.66666666666666</v>
@@ -16389,7 +16389,7 @@
         <v>21</v>
       </c>
       <c r="K182" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="L182" t="n">
         <v>108</v>
@@ -16422,10 +16422,10 @@
         <v>21</v>
       </c>
       <c r="T182" t="n">
-        <v>1.600000000000001</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="U182" t="n">
-        <v>21.86666666666667</v>
+        <v>21.86666666666666</v>
       </c>
       <c r="V182" t="n">
         <v>3</v>
@@ -16477,10 +16477,10 @@
         <v>28</v>
       </c>
       <c r="K183" t="n">
-        <v>40.2</v>
+        <v>36.4</v>
       </c>
       <c r="L183" t="n">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="M183" t="inlineStr">
         <is>
@@ -16510,7 +16510,7 @@
         <v>28</v>
       </c>
       <c r="T183" t="n">
-        <v>12.2</v>
+        <v>8.399999999999999</v>
       </c>
       <c r="U183" t="n">
         <v>33.36666666666667</v>
@@ -16653,10 +16653,10 @@
         <v>28</v>
       </c>
       <c r="K185" t="n">
-        <v>28.5</v>
+        <v>27.6</v>
       </c>
       <c r="L185" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M185" t="inlineStr">
         <is>
@@ -16686,7 +16686,7 @@
         <v>28</v>
       </c>
       <c r="T185" t="n">
-        <v>0.5</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U185" t="n">
         <v>27.5</v>
@@ -16741,10 +16741,10 @@
         <v>28</v>
       </c>
       <c r="K186" t="n">
-        <v>24</v>
+        <v>30.3</v>
       </c>
       <c r="L186" t="n">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="M186" t="inlineStr">
         <is>
@@ -16774,7 +16774,7 @@
         <v>28</v>
       </c>
       <c r="T186" t="n">
-        <v>-4</v>
+        <v>2.300000000000001</v>
       </c>
       <c r="U186" t="n">
         <v>27.23333333333333</v>
@@ -16829,10 +16829,10 @@
         <v>28</v>
       </c>
       <c r="K187" t="n">
-        <v>28.6</v>
+        <v>30.4</v>
       </c>
       <c r="L187" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="M187" t="inlineStr">
         <is>
@@ -16862,7 +16862,7 @@
         <v>28</v>
       </c>
       <c r="T187" t="n">
-        <v>0.6000000000000014</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U187" t="n">
         <v>28.83333333333333</v>
@@ -16917,10 +16917,10 @@
         <v>35</v>
       </c>
       <c r="K188" t="n">
-        <v>32.4</v>
+        <v>32.7</v>
       </c>
       <c r="L188" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="M188" t="inlineStr">
         <is>
@@ -16950,7 +16950,7 @@
         <v>41</v>
       </c>
       <c r="T188" t="n">
-        <v>-2.600000000000001</v>
+        <v>-2.299999999999997</v>
       </c>
       <c r="U188" t="n">
         <v>32.26666666666667</v>
@@ -21217,10 +21217,10 @@
         <v>31</v>
       </c>
       <c r="K237" t="n">
-        <v>28.1</v>
+        <v>31.5</v>
       </c>
       <c r="L237" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="M237" t="inlineStr">
         <is>
@@ -21248,7 +21248,7 @@
       </c>
       <c r="S237" t="inlineStr"/>
       <c r="T237" t="n">
-        <v>-2.899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="U237" t="n">
         <v>30.6</v>
@@ -23927,10 +23927,10 @@
         <v>28</v>
       </c>
       <c r="K268" t="n">
-        <v>28.1</v>
+        <v>25.8</v>
       </c>
       <c r="L268" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="M268" t="inlineStr">
         <is>
@@ -23960,7 +23960,7 @@
         <v>28</v>
       </c>
       <c r="T268" t="n">
-        <v>0.1000000000000014</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="U268" t="n">
         <v>26.96666666666667</v>
@@ -26119,10 +26119,10 @@
         <v>21</v>
       </c>
       <c r="K293" t="n">
-        <v>22</v>
+        <v>20.8</v>
       </c>
       <c r="L293" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M293" t="inlineStr">
         <is>
@@ -26152,7 +26152,7 @@
         <v>21</v>
       </c>
       <c r="T293" t="n">
-        <v>1</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U293" t="n">
         <v>21.23333333333333</v>
@@ -27435,10 +27435,10 @@
         <v>21</v>
       </c>
       <c r="K308" t="n">
-        <v>22</v>
+        <v>19.4</v>
       </c>
       <c r="L308" t="n">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="M308" t="inlineStr">
         <is>
@@ -27468,7 +27468,7 @@
         <v>21</v>
       </c>
       <c r="T308" t="n">
-        <v>1</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U308" t="n">
         <v>20.8</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L323" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L331" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -29633,10 +29633,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>31.1</v>
+        <v>24</v>
       </c>
       <c r="L333" t="n">
-        <v>127</v>
+        <v>98</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29666,7 +29666,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>6.600000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="U333" t="n">
         <v>29.13333333333334</v>
@@ -29985,10 +29985,10 @@
         <v>24.5</v>
       </c>
       <c r="K337" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="L337" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="M337" t="inlineStr">
         <is>
@@ -30018,7 +30018,7 @@
         <v>28</v>
       </c>
       <c r="T337" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U337" t="n">
         <v>35.8</v>
@@ -31217,10 +31217,10 @@
         <v>24.5</v>
       </c>
       <c r="K351" t="n">
-        <v>26.7</v>
+        <v>24.1</v>
       </c>
       <c r="L351" t="n">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="M351" t="inlineStr">
         <is>
@@ -31250,7 +31250,7 @@
         <v>28</v>
       </c>
       <c r="T351" t="n">
-        <v>2.199999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U351" t="n">
         <v>24.9</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L353" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-17 18:15:49
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2811,10 +2811,10 @@
         <v>24</v>
       </c>
       <c r="K27" t="n">
-        <v>21.6</v>
+        <v>15.8</v>
       </c>
       <c r="L27" t="n">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -2844,7 +2844,7 @@
         <v>28</v>
       </c>
       <c r="T27" t="n">
-        <v>-2.399999999999999</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="U27" t="n">
         <v>19.2</v>
@@ -5247,10 +5247,10 @@
         <v>24</v>
       </c>
       <c r="K55" t="n">
-        <v>22.8</v>
+        <v>25.7</v>
       </c>
       <c r="L55" t="n">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
         <v>28</v>
       </c>
       <c r="T55" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="U55" t="n">
         <v>24.6</v>
@@ -5771,10 +5771,10 @@
         <v>24</v>
       </c>
       <c r="K61" t="n">
-        <v>22.1</v>
+        <v>24.7</v>
       </c>
       <c r="L61" t="n">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="M61" t="inlineStr">
         <is>
@@ -5804,7 +5804,7 @@
         <v>28</v>
       </c>
       <c r="T61" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U61" t="n">
         <v>23.8</v>
@@ -5947,10 +5947,10 @@
         <v>24</v>
       </c>
       <c r="K63" t="n">
-        <v>16.6</v>
+        <v>27.2</v>
       </c>
       <c r="L63" t="n">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="M63" t="inlineStr">
         <is>
@@ -5980,7 +5980,7 @@
         <v>28</v>
       </c>
       <c r="T63" t="n">
-        <v>-7.399999999999999</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="U63" t="n">
         <v>23.4</v>
@@ -7791,10 +7791,10 @@
         <v>21</v>
       </c>
       <c r="K84" t="n">
-        <v>21.2</v>
+        <v>20.2</v>
       </c>
       <c r="L84" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="M84" t="inlineStr">
         <is>
@@ -7824,7 +7824,7 @@
         <v>21</v>
       </c>
       <c r="T84" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U84" t="n">
         <v>22.16666666666667</v>
@@ -8405,10 +8405,10 @@
         <v>35</v>
       </c>
       <c r="K91" t="n">
-        <v>36.7</v>
+        <v>39.1</v>
       </c>
       <c r="L91" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="M91" t="inlineStr">
         <is>
@@ -8438,16 +8438,16 @@
         <v>41</v>
       </c>
       <c r="T91" t="n">
-        <v>1.700000000000003</v>
+        <v>4.100000000000001</v>
       </c>
       <c r="U91" t="n">
-        <v>35.73333333333333</v>
+        <v>35.73333333333334</v>
       </c>
       <c r="V91" t="n">
         <v>3</v>
       </c>
       <c r="W91" t="n">
-        <v>35.86296296296296</v>
+        <v>35.86296296296297</v>
       </c>
       <c r="X91" t="n">
         <v>31.5</v>
@@ -9457,10 +9457,10 @@
         <v>21</v>
       </c>
       <c r="K103" t="n">
-        <v>18.4</v>
+        <v>29</v>
       </c>
       <c r="L103" t="n">
-        <v>88</v>
+        <v>138</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9490,7 +9490,7 @@
         <v>21</v>
       </c>
       <c r="T103" t="n">
-        <v>-2.600000000000001</v>
+        <v>8</v>
       </c>
       <c r="U103" t="n">
         <v>24.53333333333333</v>
@@ -9979,10 +9979,10 @@
         <v>35</v>
       </c>
       <c r="K109" t="n">
-        <v>39.8</v>
+        <v>34.1</v>
       </c>
       <c r="L109" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="M109" t="inlineStr">
         <is>
@@ -10012,7 +10012,7 @@
         <v>41</v>
       </c>
       <c r="T109" t="n">
-        <v>4.799999999999997</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U109" t="n">
         <v>36.83333333333334</v>
@@ -10067,10 +10067,10 @@
         <v>35</v>
       </c>
       <c r="K110" t="n">
-        <v>38.1</v>
+        <v>31.8</v>
       </c>
       <c r="L110" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="M110" t="inlineStr">
         <is>
@@ -10100,7 +10100,7 @@
         <v>41</v>
       </c>
       <c r="T110" t="n">
-        <v>3.100000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U110" t="n">
         <v>36.1</v>
@@ -10507,10 +10507,10 @@
         <v>35</v>
       </c>
       <c r="K115" t="n">
-        <v>26.3</v>
+        <v>22.5</v>
       </c>
       <c r="L115" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         <v>41</v>
       </c>
       <c r="T115" t="n">
-        <v>-8.699999999999999</v>
+        <v>-12.5</v>
       </c>
       <c r="U115" t="n">
         <v>25.5</v>
@@ -10683,10 +10683,10 @@
         <v>35</v>
       </c>
       <c r="K117" t="n">
-        <v>22.7</v>
+        <v>24.2</v>
       </c>
       <c r="L117" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M117" t="inlineStr">
         <is>
@@ -10716,7 +10716,7 @@
         <v>41</v>
       </c>
       <c r="T117" t="n">
-        <v>-12.3</v>
+        <v>-10.8</v>
       </c>
       <c r="U117" t="n">
         <v>23.13333333333334</v>
@@ -12443,10 +12443,10 @@
         <v>31</v>
       </c>
       <c r="K137" t="n">
-        <v>30.5</v>
+        <v>31.9</v>
       </c>
       <c r="L137" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="M137" t="inlineStr">
         <is>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="S137" t="inlineStr"/>
       <c r="T137" t="n">
-        <v>-0.5</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U137" t="n">
         <v>31.23333333333333</v>
@@ -13583,10 +13583,10 @@
         <v>28</v>
       </c>
       <c r="K150" t="n">
-        <v>35.4</v>
+        <v>27.9</v>
       </c>
       <c r="L150" t="n">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="M150" t="inlineStr">
         <is>
@@ -13616,7 +13616,7 @@
         <v>28</v>
       </c>
       <c r="T150" t="n">
-        <v>7.399999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U150" t="n">
         <v>31.73333333333333</v>
@@ -21217,10 +21217,10 @@
         <v>31</v>
       </c>
       <c r="K237" t="n">
-        <v>31.5</v>
+        <v>28.1</v>
       </c>
       <c r="L237" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M237" t="inlineStr">
         <is>
@@ -21248,7 +21248,7 @@
       </c>
       <c r="S237" t="inlineStr"/>
       <c r="T237" t="n">
-        <v>0.5</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="U237" t="n">
         <v>30.6</v>
@@ -21433,7 +21433,7 @@
         <v>3</v>
       </c>
       <c r="W239" t="n">
-        <v>22.92222222222222</v>
+        <v>22.92222222222223</v>
       </c>
       <c r="X239" t="n">
         <v>20.5</v>
@@ -22265,10 +22265,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="L249" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22298,7 +22298,7 @@
         <v>21</v>
       </c>
       <c r="T249" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U249" t="n">
         <v>21.2</v>
@@ -23927,10 +23927,10 @@
         <v>28</v>
       </c>
       <c r="K268" t="n">
-        <v>25.8</v>
+        <v>28.1</v>
       </c>
       <c r="L268" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="M268" t="inlineStr">
         <is>
@@ -23960,7 +23960,7 @@
         <v>28</v>
       </c>
       <c r="T268" t="n">
-        <v>-2.199999999999999</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U268" t="n">
         <v>26.96666666666667</v>
@@ -24979,10 +24979,10 @@
         <v>28</v>
       </c>
       <c r="K280" t="n">
-        <v>28.2</v>
+        <v>29</v>
       </c>
       <c r="L280" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="M280" t="inlineStr">
         <is>
@@ -25012,7 +25012,7 @@
         <v>28</v>
       </c>
       <c r="T280" t="n">
-        <v>0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="U280" t="n">
         <v>28.2</v>
@@ -26119,10 +26119,10 @@
         <v>21</v>
       </c>
       <c r="K293" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="L293" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M293" t="inlineStr">
         <is>
@@ -26152,7 +26152,7 @@
         <v>21</v>
       </c>
       <c r="T293" t="n">
-        <v>-0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="U293" t="n">
         <v>21.23333333333333</v>
@@ -27435,10 +27435,10 @@
         <v>21</v>
       </c>
       <c r="K308" t="n">
-        <v>19.4</v>
+        <v>22</v>
       </c>
       <c r="L308" t="n">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="M308" t="inlineStr">
         <is>
@@ -27468,7 +27468,7 @@
         <v>21</v>
       </c>
       <c r="T308" t="n">
-        <v>-1.600000000000001</v>
+        <v>1</v>
       </c>
       <c r="U308" t="n">
         <v>20.8</v>
@@ -27611,10 +27611,10 @@
         <v>21</v>
       </c>
       <c r="K310" t="n">
-        <v>20.6</v>
+        <v>26.5</v>
       </c>
       <c r="L310" t="n">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="M310" t="inlineStr">
         <is>
@@ -27644,7 +27644,7 @@
         <v>21</v>
       </c>
       <c r="T310" t="n">
-        <v>-0.3999999999999986</v>
+        <v>5.5</v>
       </c>
       <c r="U310" t="n">
         <v>23.9</v>
@@ -29633,10 +29633,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>24</v>
+        <v>31.1</v>
       </c>
       <c r="L333" t="n">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29666,7 +29666,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-0.5</v>
+        <v>6.600000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>29.13333333333334</v>
@@ -29985,10 +29985,10 @@
         <v>24.5</v>
       </c>
       <c r="K337" t="n">
-        <v>25.6</v>
+        <v>24</v>
       </c>
       <c r="L337" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="M337" t="inlineStr">
         <is>
@@ -30018,7 +30018,7 @@
         <v>28</v>
       </c>
       <c r="T337" t="n">
-        <v>1.100000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="U337" t="n">
         <v>35.8</v>
@@ -31217,10 +31217,10 @@
         <v>24.5</v>
       </c>
       <c r="K351" t="n">
-        <v>24.1</v>
+        <v>26.7</v>
       </c>
       <c r="L351" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="M351" t="inlineStr">
         <is>
@@ -31250,7 +31250,7 @@
         <v>28</v>
       </c>
       <c r="T351" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U351" t="n">
         <v>24.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-18 18:35:12
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -7179,10 +7179,10 @@
         <v>31</v>
       </c>
       <c r="K77" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L77" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M77" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
       </c>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U77" t="n">
         <v>32.03333333333333</v>
@@ -7529,10 +7529,10 @@
         <v>31</v>
       </c>
       <c r="K81" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L81" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U81" t="n">
         <v>36</v>
@@ -8143,10 +8143,10 @@
         <v>31</v>
       </c>
       <c r="K88" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L88" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U88" t="n">
         <v>33.63333333333333</v>
@@ -8581,10 +8581,10 @@
         <v>31</v>
       </c>
       <c r="K93" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L93" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U93" t="n">
         <v>32.76666666666667</v>
@@ -11123,10 +11123,10 @@
         <v>21</v>
       </c>
       <c r="K122" t="n">
-        <v>19.3</v>
+        <v>26</v>
       </c>
       <c r="L122" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="M122" t="inlineStr">
         <is>
@@ -11156,7 +11156,7 @@
         <v>21</v>
       </c>
       <c r="T122" t="n">
-        <v>-1.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="U122" t="n">
         <v>23.7</v>
@@ -21043,10 +21043,10 @@
         <v>31</v>
       </c>
       <c r="K235" t="n">
-        <v>32.3</v>
+        <v>31.2</v>
       </c>
       <c r="L235" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="M235" t="inlineStr">
         <is>
@@ -21074,7 +21074,7 @@
       </c>
       <c r="S235" t="inlineStr"/>
       <c r="T235" t="n">
-        <v>1.299999999999997</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U235" t="n">
         <v>29.3</v>
@@ -25507,10 +25507,10 @@
         <v>21</v>
       </c>
       <c r="K286" t="n">
-        <v>22</v>
+        <v>20.8</v>
       </c>
       <c r="L286" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M286" t="inlineStr">
         <is>
@@ -25540,7 +25540,7 @@
         <v>21</v>
       </c>
       <c r="T286" t="n">
-        <v>1</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U286" t="n">
         <v>21.03333333333333</v>
@@ -28753,10 +28753,10 @@
         <v>24.5</v>
       </c>
       <c r="K323" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L323" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M323" t="inlineStr">
         <is>
@@ -28786,7 +28786,7 @@
         <v>28</v>
       </c>
       <c r="T323" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U323" t="n">
         <v>24.66666666666667</v>
@@ -29457,10 +29457,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L331" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29490,7 +29490,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U331" t="n">
         <v>27.1</v>
@@ -29985,10 +29985,10 @@
         <v>24.5</v>
       </c>
       <c r="K337" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="L337" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="M337" t="inlineStr">
         <is>
@@ -30018,7 +30018,7 @@
         <v>28</v>
       </c>
       <c r="T337" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U337" t="n">
         <v>35.8</v>
@@ -31393,10 +31393,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L353" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31426,10 +31426,10 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U353" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V353" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-18 20:03:04
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2811,10 +2811,10 @@
         <v>24</v>
       </c>
       <c r="K27" t="n">
-        <v>21.6</v>
+        <v>15.8</v>
       </c>
       <c r="L27" t="n">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -2844,7 +2844,7 @@
         <v>28</v>
       </c>
       <c r="T27" t="n">
-        <v>-2.399999999999999</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="U27" t="n">
         <v>19.2</v>
@@ -6475,10 +6475,10 @@
         <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>34.3</v>
+        <v>32.3</v>
       </c>
       <c r="L69" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>41</v>
       </c>
       <c r="T69" t="n">
-        <v>-0.7000000000000028</v>
+        <v>-2.700000000000003</v>
       </c>
       <c r="U69" t="n">
         <v>32.96666666666666</v>
@@ -11123,10 +11123,10 @@
         <v>21</v>
       </c>
       <c r="K122" t="n">
-        <v>26</v>
+        <v>19.3</v>
       </c>
       <c r="L122" t="n">
-        <v>124</v>
+        <v>92</v>
       </c>
       <c r="M122" t="inlineStr">
         <is>
@@ -11156,7 +11156,7 @@
         <v>21</v>
       </c>
       <c r="T122" t="n">
-        <v>5</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U122" t="n">
         <v>23.7</v>
@@ -21043,10 +21043,10 @@
         <v>31</v>
       </c>
       <c r="K235" t="n">
-        <v>31.2</v>
+        <v>32.3</v>
       </c>
       <c r="L235" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="M235" t="inlineStr">
         <is>
@@ -21074,7 +21074,7 @@
       </c>
       <c r="S235" t="inlineStr"/>
       <c r="T235" t="n">
-        <v>0.1999999999999993</v>
+        <v>1.299999999999997</v>
       </c>
       <c r="U235" t="n">
         <v>29.3</v>
@@ -21433,7 +21433,7 @@
         <v>3</v>
       </c>
       <c r="W239" t="n">
-        <v>22.92222222222222</v>
+        <v>22.92222222222223</v>
       </c>
       <c r="X239" t="n">
         <v>20.5</v>
@@ -22611,10 +22611,10 @@
         <v>21</v>
       </c>
       <c r="K253" t="n">
-        <v>21.3</v>
+        <v>23.8</v>
       </c>
       <c r="L253" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="M253" t="inlineStr">
         <is>
@@ -22642,7 +22642,7 @@
       </c>
       <c r="S253" t="inlineStr"/>
       <c r="T253" t="n">
-        <v>0.3000000000000007</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U253" t="n">
         <v>21.8</v>
@@ -25507,10 +25507,10 @@
         <v>21</v>
       </c>
       <c r="K286" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="L286" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M286" t="inlineStr">
         <is>
@@ -25540,7 +25540,7 @@
         <v>21</v>
       </c>
       <c r="T286" t="n">
-        <v>-0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="U286" t="n">
         <v>21.03333333333333</v>
@@ -29985,10 +29985,10 @@
         <v>24.5</v>
       </c>
       <c r="K337" t="n">
-        <v>25.6</v>
+        <v>24</v>
       </c>
       <c r="L337" t="n">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="M337" t="inlineStr">
         <is>
@@ -30018,7 +30018,7 @@
         <v>28</v>
       </c>
       <c r="T337" t="n">
-        <v>1.100000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="U337" t="n">
         <v>35.8</v>
@@ -31129,10 +31129,10 @@
         <v>24.5</v>
       </c>
       <c r="K350" t="n">
-        <v>23.6</v>
+        <v>21.1</v>
       </c>
       <c r="L350" t="n">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="M350" t="inlineStr">
         <is>
@@ -31162,7 +31162,7 @@
         <v>28</v>
       </c>
       <c r="T350" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U350" t="n">
         <v>22.63333333333334</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-18 22:18:04
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2811,10 +2811,10 @@
         <v>24</v>
       </c>
       <c r="K27" t="n">
-        <v>15.8</v>
+        <v>21.6</v>
       </c>
       <c r="L27" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -2844,7 +2844,7 @@
         <v>28</v>
       </c>
       <c r="T27" t="n">
-        <v>-8.199999999999999</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="U27" t="n">
         <v>19.2</v>
@@ -3677,10 +3677,10 @@
         <v>28</v>
       </c>
       <c r="K37" t="n">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="L37" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3710,7 +3710,7 @@
         <v>28</v>
       </c>
       <c r="T37" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="U37" t="n">
         <v>30.53333333333333</v>
@@ -3765,10 +3765,10 @@
         <v>28</v>
       </c>
       <c r="K38" t="n">
-        <v>24.9</v>
+        <v>32.4</v>
       </c>
       <c r="L38" t="n">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
         <v>28</v>
       </c>
       <c r="T38" t="n">
-        <v>-3.100000000000001</v>
+        <v>4.399999999999999</v>
       </c>
       <c r="U38" t="n">
         <v>31.5</v>
@@ -4723,10 +4723,10 @@
         <v>24</v>
       </c>
       <c r="K49" t="n">
-        <v>23.8</v>
+        <v>24.9</v>
       </c>
       <c r="L49" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="M49" t="inlineStr">
         <is>
@@ -4756,7 +4756,7 @@
         <v>28</v>
       </c>
       <c r="T49" t="n">
-        <v>-0.1999999999999993</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U49" t="n">
         <v>21.43333333333333</v>
@@ -6475,10 +6475,10 @@
         <v>35</v>
       </c>
       <c r="K69" t="n">
-        <v>32.3</v>
+        <v>34.3</v>
       </c>
       <c r="L69" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="M69" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>41</v>
       </c>
       <c r="T69" t="n">
-        <v>-2.700000000000003</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="U69" t="n">
         <v>32.96666666666666</v>
@@ -9323,7 +9323,7 @@
         <v>3</v>
       </c>
       <c r="W101" t="n">
-        <v>26.17777777777778</v>
+        <v>26.17777777777777</v>
       </c>
       <c r="X101" t="n">
         <v>17.5</v>
@@ -10507,10 +10507,10 @@
         <v>35</v>
       </c>
       <c r="K115" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="L115" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -10540,7 +10540,7 @@
         <v>41</v>
       </c>
       <c r="T115" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="U115" t="n">
         <v>25.5</v>
@@ -11739,10 +11739,10 @@
         <v>28</v>
       </c>
       <c r="K129" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="L129" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="M129" t="inlineStr">
         <is>
@@ -11772,7 +11772,7 @@
         <v>28</v>
       </c>
       <c r="T129" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U129" t="n">
         <v>25.36666666666666</v>
@@ -21433,7 +21433,7 @@
         <v>3</v>
       </c>
       <c r="W239" t="n">
-        <v>22.92222222222223</v>
+        <v>22.92222222222222</v>
       </c>
       <c r="X239" t="n">
         <v>20.5</v>
@@ -22611,10 +22611,10 @@
         <v>21</v>
       </c>
       <c r="K253" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="L253" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="M253" t="inlineStr">
         <is>
@@ -22642,7 +22642,7 @@
       </c>
       <c r="S253" t="inlineStr"/>
       <c r="T253" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U253" t="n">
         <v>21.8</v>
@@ -23577,10 +23577,10 @@
         <v>28</v>
       </c>
       <c r="K264" t="n">
-        <v>24.7</v>
+        <v>32.5</v>
       </c>
       <c r="L264" t="n">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="M264" t="inlineStr">
         <is>
@@ -23610,7 +23610,7 @@
         <v>28</v>
       </c>
       <c r="T264" t="n">
-        <v>-3.300000000000001</v>
+        <v>4.5</v>
       </c>
       <c r="U264" t="n">
         <v>29.5</v>
@@ -28665,10 +28665,10 @@
         <v>24.5</v>
       </c>
       <c r="K322" t="n">
-        <v>21.5</v>
+        <v>33.3</v>
       </c>
       <c r="L322" t="n">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="M322" t="inlineStr">
         <is>
@@ -28698,7 +28698,7 @@
         <v>28</v>
       </c>
       <c r="T322" t="n">
-        <v>-3</v>
+        <v>8.799999999999997</v>
       </c>
       <c r="U322" t="n">
         <v>29.5</v>
@@ -31129,10 +31129,10 @@
         <v>24.5</v>
       </c>
       <c r="K350" t="n">
-        <v>21.1</v>
+        <v>23.6</v>
       </c>
       <c r="L350" t="n">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="M350" t="inlineStr">
         <is>
@@ -31162,7 +31162,7 @@
         <v>28</v>
       </c>
       <c r="T350" t="n">
-        <v>-3.399999999999999</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U350" t="n">
         <v>22.63333333333334</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-19 20:59:50
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4201,10 +4201,10 @@
         <v>31</v>
       </c>
       <c r="K43" t="n">
-        <v>32.8</v>
+        <v>30.1</v>
       </c>
       <c r="L43" t="n">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="M43" t="inlineStr">
         <is>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="n">
-        <v>1.799999999999997</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U43" t="n">
         <v>32.13333333333333</v>
@@ -5073,7 +5073,7 @@
         <v>24</v>
       </c>
       <c r="K53" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="L53" t="n">
         <v>103</v>
@@ -5106,7 +5106,7 @@
         <v>28</v>
       </c>
       <c r="T53" t="n">
-        <v>0.8000000000000007</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U53" t="n">
         <v>23.53333333333333</v>
@@ -7615,10 +7615,10 @@
         <v>28</v>
       </c>
       <c r="K82" t="n">
-        <v>30.7</v>
+        <v>27.7</v>
       </c>
       <c r="L82" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
         <v>28</v>
       </c>
       <c r="T82" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U82" t="n">
         <v>29.2</v>
@@ -11737,10 +11737,10 @@
         <v>35</v>
       </c>
       <c r="K129" t="n">
-        <v>35.4</v>
+        <v>30.5</v>
       </c>
       <c r="L129" t="n">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="M129" t="inlineStr">
         <is>
@@ -11770,7 +11770,7 @@
         <v>41</v>
       </c>
       <c r="T129" t="n">
-        <v>0.3999999999999986</v>
+        <v>-4.5</v>
       </c>
       <c r="U129" t="n">
         <v>34.13333333333333</v>
@@ -12879,10 +12879,10 @@
         <v>28</v>
       </c>
       <c r="K142" t="n">
-        <v>27.9</v>
+        <v>27.4</v>
       </c>
       <c r="L142" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="M142" t="inlineStr">
         <is>
@@ -12912,7 +12912,7 @@
         <v>28</v>
       </c>
       <c r="T142" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U142" t="n">
         <v>28.4</v>
@@ -12967,10 +12967,10 @@
         <v>35</v>
       </c>
       <c r="K143" t="n">
-        <v>33.6</v>
+        <v>42.6</v>
       </c>
       <c r="L143" t="n">
-        <v>96</v>
+        <v>122</v>
       </c>
       <c r="M143" t="inlineStr">
         <is>
@@ -13000,7 +13000,7 @@
         <v>41</v>
       </c>
       <c r="T143" t="n">
-        <v>-1.399999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U143" t="n">
         <v>39.1</v>
@@ -13055,10 +13055,10 @@
         <v>35</v>
       </c>
       <c r="K144" t="n">
-        <v>34.7</v>
+        <v>39.7</v>
       </c>
       <c r="L144" t="n">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="M144" t="inlineStr">
         <is>
@@ -13088,7 +13088,7 @@
         <v>41</v>
       </c>
       <c r="T144" t="n">
-        <v>-0.2999999999999972</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="U144" t="n">
         <v>37.66666666666667</v>
@@ -13143,10 +13143,10 @@
         <v>35</v>
       </c>
       <c r="K145" t="n">
-        <v>29.7</v>
+        <v>39.9</v>
       </c>
       <c r="L145" t="n">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="M145" t="inlineStr">
         <is>
@@ -13176,7 +13176,7 @@
         <v>41</v>
       </c>
       <c r="T145" t="n">
-        <v>-5.300000000000001</v>
+        <v>4.899999999999999</v>
       </c>
       <c r="U145" t="n">
         <v>37</v>
@@ -13231,10 +13231,10 @@
         <v>35</v>
       </c>
       <c r="K146" t="n">
-        <v>41.3</v>
+        <v>37.4</v>
       </c>
       <c r="L146" t="n">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="M146" t="inlineStr">
         <is>
@@ -13264,10 +13264,10 @@
         <v>41</v>
       </c>
       <c r="T146" t="n">
-        <v>6.299999999999997</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U146" t="n">
-        <v>37.06666666666666</v>
+        <v>37.06666666666667</v>
       </c>
       <c r="V146" t="n">
         <v>3</v>
@@ -13319,10 +13319,10 @@
         <v>35</v>
       </c>
       <c r="K147" t="n">
-        <v>46</v>
+        <v>37.5</v>
       </c>
       <c r="L147" t="n">
-        <v>131</v>
+        <v>107</v>
       </c>
       <c r="M147" t="inlineStr">
         <is>
@@ -13352,7 +13352,7 @@
         <v>41</v>
       </c>
       <c r="T147" t="n">
-        <v>11</v>
+        <v>2.5</v>
       </c>
       <c r="U147" t="n">
         <v>38.3</v>
@@ -13407,10 +13407,10 @@
         <v>35</v>
       </c>
       <c r="K148" t="n">
-        <v>26.2</v>
+        <v>27.7</v>
       </c>
       <c r="L148" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="M148" t="inlineStr">
         <is>
@@ -13440,7 +13440,7 @@
         <v>41</v>
       </c>
       <c r="T148" t="n">
-        <v>-8.800000000000001</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="U148" t="n">
         <v>26.5</v>
@@ -13581,10 +13581,10 @@
         <v>35</v>
       </c>
       <c r="K150" t="n">
-        <v>38.2</v>
+        <v>38.6</v>
       </c>
       <c r="L150" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="M150" t="inlineStr">
         <is>
@@ -13614,10 +13614,10 @@
         <v>41</v>
       </c>
       <c r="T150" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U150" t="n">
-        <v>36.56666666666666</v>
+        <v>36.56666666666667</v>
       </c>
       <c r="V150" t="n">
         <v>3</v>
@@ -13669,10 +13669,10 @@
         <v>35</v>
       </c>
       <c r="K151" t="n">
-        <v>34.4</v>
+        <v>36.9</v>
       </c>
       <c r="L151" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="M151" t="inlineStr">
         <is>
@@ -13702,7 +13702,7 @@
         <v>41</v>
       </c>
       <c r="T151" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U151" t="n">
         <v>35.53333333333333</v>
@@ -13711,7 +13711,7 @@
         <v>3</v>
       </c>
       <c r="W151" t="n">
-        <v>36.47037037037036</v>
+        <v>36.47037037037038</v>
       </c>
       <c r="X151" t="n">
         <v>31.5</v>
@@ -13757,10 +13757,10 @@
         <v>28</v>
       </c>
       <c r="K152" t="n">
-        <v>31.9</v>
+        <v>35.4</v>
       </c>
       <c r="L152" t="n">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="M152" t="inlineStr">
         <is>
@@ -13790,7 +13790,7 @@
         <v>28</v>
       </c>
       <c r="T152" t="n">
-        <v>3.899999999999999</v>
+        <v>7.399999999999999</v>
       </c>
       <c r="U152" t="n">
         <v>31.73333333333333</v>
@@ -13845,10 +13845,10 @@
         <v>28</v>
       </c>
       <c r="K153" t="n">
-        <v>30.7</v>
+        <v>30.2</v>
       </c>
       <c r="L153" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="M153" t="inlineStr">
         <is>
@@ -13878,7 +13878,7 @@
         <v>28</v>
       </c>
       <c r="T153" t="n">
-        <v>2.699999999999999</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U153" t="n">
         <v>29.23333333333333</v>
@@ -25945,10 +25945,10 @@
         <v>21</v>
       </c>
       <c r="K291" t="n">
-        <v>20.9</v>
+        <v>20.5</v>
       </c>
       <c r="L291" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="M291" t="inlineStr">
         <is>
@@ -25976,7 +25976,7 @@
       </c>
       <c r="S291" t="inlineStr"/>
       <c r="T291" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.5</v>
       </c>
       <c r="U291" t="n">
         <v>20.2</v>
@@ -26819,10 +26819,10 @@
         <v>21</v>
       </c>
       <c r="K301" t="n">
-        <v>18</v>
+        <v>21.1</v>
       </c>
       <c r="L301" t="n">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="M301" t="inlineStr">
         <is>
@@ -26852,7 +26852,7 @@
         <v>21</v>
       </c>
       <c r="T301" t="n">
-        <v>-3</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U301" t="n">
         <v>19.53333333333333</v>
@@ -28399,10 +28399,10 @@
         <v>24.5</v>
       </c>
       <c r="K319" t="n">
-        <v>23.9</v>
+        <v>23.4</v>
       </c>
       <c r="L319" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="M319" t="inlineStr">
         <is>
@@ -28432,7 +28432,7 @@
         <v>28</v>
       </c>
       <c r="T319" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U319" t="n">
         <v>23.56666666666666</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-19 22:02:08
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3071,10 +3071,10 @@
         <v>28</v>
       </c>
       <c r="K30" t="n">
-        <v>27.1</v>
+        <v>26.9</v>
       </c>
       <c r="L30" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -3104,7 +3104,7 @@
         <v>28</v>
       </c>
       <c r="T30" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U30" t="n">
         <v>27.23333333333333</v>
@@ -3245,10 +3245,10 @@
         <v>31</v>
       </c>
       <c r="K32" t="n">
-        <v>36</v>
+        <v>30.9</v>
       </c>
       <c r="L32" t="n">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="n">
-        <v>5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U32" t="n">
         <v>33.03333333333333</v>
@@ -3331,10 +3331,10 @@
         <v>31</v>
       </c>
       <c r="K33" t="n">
-        <v>31.6</v>
+        <v>29.8</v>
       </c>
       <c r="L33" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
-        <v>0.6000000000000014</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U33" t="n">
         <v>30.4</v>
@@ -3417,10 +3417,10 @@
         <v>31</v>
       </c>
       <c r="K34" t="n">
-        <v>27.8</v>
+        <v>38.5</v>
       </c>
       <c r="L34" t="n">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="n">
-        <v>-3.199999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="U34" t="n">
         <v>35.83333333333334</v>
@@ -3503,10 +3503,10 @@
         <v>28</v>
       </c>
       <c r="K35" t="n">
-        <v>33.2</v>
+        <v>22.1</v>
       </c>
       <c r="L35" t="n">
-        <v>118</v>
+        <v>79</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
         <v>28</v>
       </c>
       <c r="T35" t="n">
-        <v>5.200000000000003</v>
+        <v>-5.899999999999999</v>
       </c>
       <c r="U35" t="n">
         <v>30.1</v>
@@ -3631,7 +3631,7 @@
         <v>3</v>
       </c>
       <c r="W36" t="n">
-        <v>41.12222222222222</v>
+        <v>41.12222222222223</v>
       </c>
       <c r="X36" t="n">
         <v>27.5</v>
@@ -4067,7 +4067,7 @@
         <v>3</v>
       </c>
       <c r="W41" t="n">
-        <v>41.82222222222222</v>
+        <v>38.09999999999999</v>
       </c>
       <c r="X41" t="n">
         <v>27.5</v>
@@ -5335,10 +5335,10 @@
         <v>31</v>
       </c>
       <c r="K56" t="n">
-        <v>38.5</v>
+        <v>30.5</v>
       </c>
       <c r="L56" t="n">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="M56" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="n">
-        <v>7.5</v>
+        <v>-0.5</v>
       </c>
       <c r="U56" t="n">
         <v>35.86666666666667</v>
@@ -5509,10 +5509,10 @@
         <v>24</v>
       </c>
       <c r="K58" t="n">
-        <v>21.2</v>
+        <v>25</v>
       </c>
       <c r="L58" t="n">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -5542,7 +5542,7 @@
         <v>28</v>
       </c>
       <c r="T58" t="n">
-        <v>-2.800000000000001</v>
+        <v>1</v>
       </c>
       <c r="U58" t="n">
         <v>22.7</v>
@@ -5725,7 +5725,7 @@
         <v>3</v>
       </c>
       <c r="W60" t="n">
-        <v>23.14444444444445</v>
+        <v>23.14444444444444</v>
       </c>
       <c r="X60" t="n">
         <v>20.5</v>
@@ -6033,10 +6033,10 @@
         <v>24</v>
       </c>
       <c r="K64" t="n">
-        <v>23.1</v>
+        <v>25.9</v>
       </c>
       <c r="L64" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
@@ -6066,7 +6066,7 @@
         <v>28</v>
       </c>
       <c r="T64" t="n">
-        <v>-0.8999999999999986</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U64" t="n">
         <v>24.1</v>
@@ -7615,10 +7615,10 @@
         <v>28</v>
       </c>
       <c r="K82" t="n">
-        <v>27.7</v>
+        <v>30.7</v>
       </c>
       <c r="L82" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
         <v>28</v>
       </c>
       <c r="T82" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U82" t="n">
         <v>29.2</v>
@@ -12265,10 +12265,10 @@
         <v>35</v>
       </c>
       <c r="K135" t="n">
-        <v>36.6</v>
+        <v>36.5</v>
       </c>
       <c r="L135" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M135" t="inlineStr">
         <is>
@@ -12298,7 +12298,7 @@
         <v>41</v>
       </c>
       <c r="T135" t="n">
-        <v>1.600000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="U135" t="n">
         <v>35.63333333333333</v>
@@ -17179,10 +17179,10 @@
         <v>28</v>
       </c>
       <c r="K191" t="n">
-        <v>25.7</v>
+        <v>26.7</v>
       </c>
       <c r="L191" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="M191" t="inlineStr">
         <is>
@@ -17212,7 +17212,7 @@
         <v>28</v>
       </c>
       <c r="T191" t="n">
-        <v>-2.300000000000001</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U191" t="n">
         <v>26.76666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-20 07:11:46
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2811,10 +2811,10 @@
         <v>24</v>
       </c>
       <c r="K27" t="n">
-        <v>15.8</v>
+        <v>21.6</v>
       </c>
       <c r="L27" t="n">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -2844,7 +2844,7 @@
         <v>28</v>
       </c>
       <c r="T27" t="n">
-        <v>-8.199999999999999</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="U27" t="n">
         <v>19.2</v>
@@ -4897,10 +4897,10 @@
         <v>24</v>
       </c>
       <c r="K51" t="n">
-        <v>24.9</v>
+        <v>23.8</v>
       </c>
       <c r="L51" t="n">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
@@ -4930,7 +4930,7 @@
         <v>28</v>
       </c>
       <c r="T51" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U51" t="n">
         <v>21.43333333333333</v>
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L79" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L83" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -7965,10 +7965,10 @@
         <v>21</v>
       </c>
       <c r="K86" t="n">
-        <v>25.1</v>
+        <v>21.2</v>
       </c>
       <c r="L86" t="n">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="M86" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
         <v>21</v>
       </c>
       <c r="T86" t="n">
-        <v>4.100000000000001</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U86" t="n">
         <v>22.16666666666667</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L90" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L95" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -9455,10 +9455,10 @@
         <v>21</v>
       </c>
       <c r="K103" t="n">
-        <v>20.2</v>
+        <v>24.2</v>
       </c>
       <c r="L103" t="n">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9488,7 +9488,7 @@
         <v>21</v>
       </c>
       <c r="T103" t="n">
-        <v>-0.8000000000000007</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="U103" t="n">
         <v>23.23333333333333</v>
@@ -9631,10 +9631,10 @@
         <v>21</v>
       </c>
       <c r="K105" t="n">
-        <v>29</v>
+        <v>18.4</v>
       </c>
       <c r="L105" t="n">
-        <v>138</v>
+        <v>88</v>
       </c>
       <c r="M105" t="inlineStr">
         <is>
@@ -9664,7 +9664,7 @@
         <v>21</v>
       </c>
       <c r="T105" t="n">
-        <v>8</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U105" t="n">
         <v>24.53333333333333</v>
@@ -10769,10 +10769,10 @@
         <v>28</v>
       </c>
       <c r="K118" t="n">
-        <v>29.7</v>
+        <v>32.7</v>
       </c>
       <c r="L118" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -10802,7 +10802,7 @@
         <v>28</v>
       </c>
       <c r="T118" t="n">
-        <v>1.699999999999999</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="U118" t="n">
         <v>29.6</v>
@@ -11473,10 +11473,10 @@
         <v>21</v>
       </c>
       <c r="K126" t="n">
-        <v>20.2</v>
+        <v>23.7</v>
       </c>
       <c r="L126" t="n">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="M126" t="inlineStr">
         <is>
@@ -11506,7 +11506,7 @@
         <v>21</v>
       </c>
       <c r="T126" t="n">
-        <v>-0.8000000000000007</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U126" t="n">
         <v>21.43333333333333</v>
@@ -21391,10 +21391,10 @@
         <v>31</v>
       </c>
       <c r="K239" t="n">
-        <v>31.5</v>
+        <v>28.1</v>
       </c>
       <c r="L239" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M239" t="inlineStr">
         <is>
@@ -21422,7 +21422,7 @@
       </c>
       <c r="S239" t="inlineStr"/>
       <c r="T239" t="n">
-        <v>0.5</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="U239" t="n">
         <v>30.6</v>
@@ -21607,7 +21607,7 @@
         <v>3</v>
       </c>
       <c r="W241" t="n">
-        <v>22.92222222222223</v>
+        <v>22.92222222222222</v>
       </c>
       <c r="X241" t="n">
         <v>20.5</v>
@@ -22265,10 +22265,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>22.6</v>
+        <v>18.9</v>
       </c>
       <c r="L249" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22296,7 +22296,7 @@
       </c>
       <c r="S249" t="inlineStr"/>
       <c r="T249" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U249" t="n">
         <v>20.5</v>
@@ -28135,10 +28135,10 @@
         <v>24.5</v>
       </c>
       <c r="K316" t="n">
-        <v>23.3</v>
+        <v>25.8</v>
       </c>
       <c r="L316" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="M316" t="inlineStr">
         <is>
@@ -28168,7 +28168,7 @@
         <v>28</v>
       </c>
       <c r="T316" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="U316" t="n">
         <v>24.26666666666667</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29103,10 +29103,10 @@
         <v>24.5</v>
       </c>
       <c r="K327" t="n">
-        <v>29.7</v>
+        <v>31.9</v>
       </c>
       <c r="L327" t="n">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="M327" t="inlineStr">
         <is>
@@ -29136,7 +29136,7 @@
         <v>28</v>
       </c>
       <c r="T327" t="n">
-        <v>5.199999999999999</v>
+        <v>7.399999999999999</v>
       </c>
       <c r="U327" t="n">
         <v>27.5</v>
@@ -29279,10 +29279,10 @@
         <v>24.5</v>
       </c>
       <c r="K329" t="n">
-        <v>23.6</v>
+        <v>27</v>
       </c>
       <c r="L329" t="n">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="M329" t="inlineStr">
         <is>
@@ -29312,7 +29312,7 @@
         <v>28</v>
       </c>
       <c r="T329" t="n">
-        <v>-0.8999999999999986</v>
+        <v>2.5</v>
       </c>
       <c r="U329" t="n">
         <v>24.93333333333333</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -30599,10 +30599,10 @@
         <v>24.5</v>
       </c>
       <c r="K344" t="n">
-        <v>23.5</v>
+        <v>21.6</v>
       </c>
       <c r="L344" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="M344" t="inlineStr">
         <is>
@@ -30632,7 +30632,7 @@
         <v>28</v>
       </c>
       <c r="T344" t="n">
-        <v>-1</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="U344" t="n">
         <v>23.1</v>
@@ -30687,10 +30687,10 @@
         <v>24.5</v>
       </c>
       <c r="K345" t="n">
-        <v>26.3</v>
+        <v>28.4</v>
       </c>
       <c r="L345" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="M345" t="inlineStr">
         <is>
@@ -30720,7 +30720,7 @@
         <v>28</v>
       </c>
       <c r="T345" t="n">
-        <v>1.800000000000001</v>
+        <v>3.899999999999999</v>
       </c>
       <c r="U345" t="n">
         <v>26.36666666666666</v>
@@ -30729,7 +30729,7 @@
         <v>3</v>
       </c>
       <c r="W345" t="n">
-        <v>23.35555555555555</v>
+        <v>23.35555555555556</v>
       </c>
       <c r="X345" t="n">
         <v>21</v>
@@ -30775,10 +30775,10 @@
         <v>24.5</v>
       </c>
       <c r="K346" t="n">
-        <v>23.3</v>
+        <v>25.4</v>
       </c>
       <c r="L346" t="n">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="M346" t="inlineStr">
         <is>
@@ -30808,10 +30808,10 @@
         <v>28</v>
       </c>
       <c r="T346" t="n">
-        <v>-1.199999999999999</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U346" t="n">
-        <v>24.56666666666666</v>
+        <v>24.56666666666667</v>
       </c>
       <c r="V346" t="n">
         <v>3</v>
@@ -30863,10 +30863,10 @@
         <v>24.5</v>
       </c>
       <c r="K347" t="n">
-        <v>22.4</v>
+        <v>24.9</v>
       </c>
       <c r="L347" t="n">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="M347" t="inlineStr">
         <is>
@@ -30896,7 +30896,7 @@
         <v>28</v>
       </c>
       <c r="T347" t="n">
-        <v>-2.100000000000001</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U347" t="n">
         <v>24.03333333333333</v>
@@ -30951,10 +30951,10 @@
         <v>24.5</v>
       </c>
       <c r="K348" t="n">
-        <v>22.3</v>
+        <v>23.3</v>
       </c>
       <c r="L348" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="M348" t="inlineStr">
         <is>
@@ -30984,7 +30984,7 @@
         <v>28</v>
       </c>
       <c r="T348" t="n">
-        <v>-2.199999999999999</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U348" t="n">
         <v>23.03333333333333</v>
@@ -31039,10 +31039,10 @@
         <v>24.5</v>
       </c>
       <c r="K349" t="n">
-        <v>23.5</v>
+        <v>25.4</v>
       </c>
       <c r="L349" t="n">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="M349" t="inlineStr">
         <is>
@@ -31072,7 +31072,7 @@
         <v>28</v>
       </c>
       <c r="T349" t="n">
-        <v>-1</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U349" t="n">
         <v>24.63333333333334</v>
@@ -31127,10 +31127,10 @@
         <v>24.5</v>
       </c>
       <c r="K350" t="n">
-        <v>23.4</v>
+        <v>36.1</v>
       </c>
       <c r="L350" t="n">
-        <v>95</v>
+        <v>147</v>
       </c>
       <c r="M350" t="inlineStr">
         <is>
@@ -31160,7 +31160,7 @@
         <v>28</v>
       </c>
       <c r="T350" t="n">
-        <v>-1.100000000000001</v>
+        <v>11.6</v>
       </c>
       <c r="U350" t="n">
         <v>29.46666666666667</v>
@@ -31215,10 +31215,10 @@
         <v>24.5</v>
       </c>
       <c r="K351" t="n">
-        <v>23.4</v>
+        <v>26.2</v>
       </c>
       <c r="L351" t="n">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="M351" t="inlineStr">
         <is>
@@ -31248,7 +31248,7 @@
         <v>28</v>
       </c>
       <c r="T351" t="n">
-        <v>-1.100000000000001</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="U351" t="n">
         <v>24.5</v>
@@ -31303,10 +31303,10 @@
         <v>24.5</v>
       </c>
       <c r="K352" t="n">
-        <v>23.6</v>
+        <v>23.2</v>
       </c>
       <c r="L352" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M352" t="inlineStr">
         <is>
@@ -31336,7 +31336,7 @@
         <v>28</v>
       </c>
       <c r="T352" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U352" t="n">
         <v>22.63333333333334</v>
@@ -31391,10 +31391,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>26.7</v>
+        <v>24.1</v>
       </c>
       <c r="L353" t="n">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31424,7 +31424,7 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>2.199999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U353" t="n">
         <v>24.9</v>
@@ -31479,10 +31479,10 @@
         <v>24.5</v>
       </c>
       <c r="K354" t="n">
-        <v>27.8</v>
+        <v>22.9</v>
       </c>
       <c r="L354" t="n">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="M354" t="inlineStr">
         <is>
@@ -31512,7 +31512,7 @@
         <v>28</v>
       </c>
       <c r="T354" t="n">
-        <v>3.300000000000001</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U354" t="n">
         <v>25</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-20 18:35:58
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2897,10 +2897,10 @@
         <v>21</v>
       </c>
       <c r="K28" t="n">
-        <v>20.9</v>
+        <v>21.5</v>
       </c>
       <c r="L28" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -2930,7 +2930,7 @@
         <v>21</v>
       </c>
       <c r="T28" t="n">
-        <v>-0.1000000000000014</v>
+        <v>0.5</v>
       </c>
       <c r="U28" t="n">
         <v>21.2</v>
@@ -3593,10 +3593,10 @@
         <v>28</v>
       </c>
       <c r="K36" t="n">
-        <v>26.4</v>
+        <v>22.7</v>
       </c>
       <c r="L36" t="n">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3626,7 +3626,7 @@
         <v>28</v>
       </c>
       <c r="T36" t="n">
-        <v>-1.600000000000001</v>
+        <v>-5.300000000000001</v>
       </c>
       <c r="U36" t="n">
         <v>24.9</v>
@@ -3681,10 +3681,10 @@
         <v>28</v>
       </c>
       <c r="K37" t="n">
-        <v>26</v>
+        <v>29.1</v>
       </c>
       <c r="L37" t="n">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3714,7 +3714,7 @@
         <v>28</v>
       </c>
       <c r="T37" t="n">
-        <v>-2</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U37" t="n">
         <v>27.33333333333333</v>
@@ -3769,10 +3769,10 @@
         <v>28</v>
       </c>
       <c r="K38" t="n">
-        <v>25.1</v>
+        <v>27.1</v>
       </c>
       <c r="L38" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3802,7 +3802,7 @@
         <v>28</v>
       </c>
       <c r="T38" t="n">
-        <v>-2.899999999999999</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U38" t="n">
         <v>26.3</v>
@@ -5523,10 +5523,10 @@
         <v>28</v>
       </c>
       <c r="K58" t="n">
-        <v>27.8</v>
+        <v>27.5</v>
       </c>
       <c r="L58" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M58" t="inlineStr">
         <is>
@@ -5556,7 +5556,7 @@
         <v>28</v>
       </c>
       <c r="T58" t="n">
-        <v>-0.1999999999999993</v>
+        <v>-0.5</v>
       </c>
       <c r="U58" t="n">
         <v>27</v>
@@ -5611,10 +5611,10 @@
         <v>28</v>
       </c>
       <c r="K59" t="n">
-        <v>27.4</v>
+        <v>28.2</v>
       </c>
       <c r="L59" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
@@ -5644,7 +5644,7 @@
         <v>28</v>
       </c>
       <c r="T59" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U59" t="n">
         <v>28.2</v>
@@ -5699,10 +5699,10 @@
         <v>28</v>
       </c>
       <c r="K60" t="n">
-        <v>26.7</v>
+        <v>28.3</v>
       </c>
       <c r="L60" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v>28</v>
       </c>
       <c r="T60" t="n">
-        <v>-1.300000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U60" t="n">
         <v>27.4</v>
@@ -6575,10 +6575,10 @@
         <v>21</v>
       </c>
       <c r="K70" t="n">
-        <v>20.1</v>
+        <v>22.8</v>
       </c>
       <c r="L70" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="M70" t="inlineStr">
         <is>
@@ -6608,7 +6608,7 @@
         <v>21</v>
       </c>
       <c r="T70" t="n">
-        <v>-0.8999999999999986</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="U70" t="n">
         <v>21.53333333333333</v>
@@ -7539,10 +7539,10 @@
         <v>21</v>
       </c>
       <c r="K81" t="n">
-        <v>19.7</v>
+        <v>22</v>
       </c>
       <c r="L81" t="n">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7572,7 +7572,7 @@
         <v>21</v>
       </c>
       <c r="T81" t="n">
-        <v>-1.300000000000001</v>
+        <v>1</v>
       </c>
       <c r="U81" t="n">
         <v>21</v>
@@ -7627,10 +7627,10 @@
         <v>21</v>
       </c>
       <c r="K82" t="n">
-        <v>18.4</v>
+        <v>22.1</v>
       </c>
       <c r="L82" t="n">
-        <v>87</v>
+        <v>105</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7660,7 +7660,7 @@
         <v>21</v>
       </c>
       <c r="T82" t="n">
-        <v>-2.600000000000001</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U82" t="n">
         <v>20.63333333333333</v>
@@ -9385,10 +9385,10 @@
         <v>24.5</v>
       </c>
       <c r="K102" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L102" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M102" t="inlineStr">
         <is>
@@ -9418,7 +9418,7 @@
         <v>28</v>
       </c>
       <c r="T102" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U102" t="n">
         <v>24.66666666666667</v>
@@ -10089,10 +10089,10 @@
         <v>24.5</v>
       </c>
       <c r="K110" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L110" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M110" t="inlineStr">
         <is>
@@ -10122,7 +10122,7 @@
         <v>28</v>
       </c>
       <c r="T110" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U110" t="n">
         <v>27.1</v>
@@ -12025,10 +12025,10 @@
         <v>24.5</v>
       </c>
       <c r="K132" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L132" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M132" t="inlineStr">
         <is>
@@ -12058,10 +12058,10 @@
         <v>28</v>
       </c>
       <c r="T132" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U132" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V132" t="n">
         <v>3</v>
@@ -12199,10 +12199,10 @@
         <v>24.5</v>
       </c>
       <c r="K134" t="n">
-        <v>31.7</v>
+        <v>28.5</v>
       </c>
       <c r="L134" t="n">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="M134" t="inlineStr">
         <is>
@@ -12232,7 +12232,7 @@
         <v>28</v>
       </c>
       <c r="T134" t="n">
-        <v>7.199999999999999</v>
+        <v>4</v>
       </c>
       <c r="U134" t="n">
         <v>28.1</v>
@@ -12639,10 +12639,10 @@
         <v>24.5</v>
       </c>
       <c r="K139" t="n">
-        <v>29.1</v>
+        <v>22.7</v>
       </c>
       <c r="L139" t="n">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M139" t="inlineStr">
         <is>
@@ -12672,7 +12672,7 @@
         <v>28</v>
       </c>
       <c r="T139" t="n">
-        <v>4.600000000000001</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="U139" t="n">
         <v>25.3</v>
@@ -12901,10 +12901,10 @@
         <v>21</v>
       </c>
       <c r="K142" t="n">
-        <v>18.2</v>
+        <v>17.6</v>
       </c>
       <c r="L142" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M142" t="inlineStr">
         <is>
@@ -12932,16 +12932,16 @@
       </c>
       <c r="S142" t="inlineStr"/>
       <c r="T142" t="n">
-        <v>-2.800000000000001</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U142" t="n">
-        <v>18.13333333333333</v>
+        <v>18.13333333333334</v>
       </c>
       <c r="V142" t="n">
         <v>3</v>
       </c>
       <c r="W142" t="n">
-        <v>27.25555555555555</v>
+        <v>27.25555555555556</v>
       </c>
       <c r="X142" t="n">
         <v>17.5</v>
@@ -13247,10 +13247,10 @@
         <v>21</v>
       </c>
       <c r="K146" t="n">
-        <v>21.2</v>
+        <v>19.9</v>
       </c>
       <c r="L146" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="M146" t="inlineStr">
         <is>
@@ -13280,7 +13280,7 @@
         <v>21</v>
       </c>
       <c r="T146" t="n">
-        <v>0.1999999999999993</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U146" t="n">
         <v>20.26666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-21 07:04:34
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -10417,10 +10417,10 @@
         <v>35</v>
       </c>
       <c r="K114" t="n">
-        <v>49.1</v>
+        <v>31.4</v>
       </c>
       <c r="L114" t="n">
-        <v>140</v>
+        <v>90</v>
       </c>
       <c r="M114" t="inlineStr">
         <is>
@@ -10450,7 +10450,7 @@
         <v>41</v>
       </c>
       <c r="T114" t="n">
-        <v>14.1</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="U114" t="n">
         <v>43.96666666666667</v>
@@ -10505,10 +10505,10 @@
         <v>35</v>
       </c>
       <c r="K115" t="n">
-        <v>27.3</v>
+        <v>54.5</v>
       </c>
       <c r="L115" t="n">
-        <v>78</v>
+        <v>156</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -10538,16 +10538,16 @@
         <v>41</v>
       </c>
       <c r="T115" t="n">
-        <v>-7.699999999999999</v>
+        <v>19.5</v>
       </c>
       <c r="U115" t="n">
-        <v>44.9</v>
+        <v>44.90000000000001</v>
       </c>
       <c r="V115" t="n">
         <v>3</v>
       </c>
       <c r="W115" t="n">
-        <v>41.74444444444444</v>
+        <v>41.74444444444445</v>
       </c>
       <c r="X115" t="n">
         <v>31.5</v>
@@ -10593,10 +10593,10 @@
         <v>21</v>
       </c>
       <c r="K116" t="n">
-        <v>24.3</v>
+        <v>19.9</v>
       </c>
       <c r="L116" t="n">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="M116" t="inlineStr">
         <is>
@@ -10626,16 +10626,16 @@
         <v>21</v>
       </c>
       <c r="T116" t="n">
-        <v>3.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U116" t="n">
-        <v>22.56666666666666</v>
+        <v>22.56666666666667</v>
       </c>
       <c r="V116" t="n">
         <v>3</v>
       </c>
       <c r="W116" t="n">
-        <v>36.05555555555555</v>
+        <v>36.05555555555556</v>
       </c>
       <c r="X116" t="n">
         <v>17.5</v>
@@ -12529,10 +12529,10 @@
         <v>35</v>
       </c>
       <c r="K138" t="n">
-        <v>36.5</v>
+        <v>31.4</v>
       </c>
       <c r="L138" t="n">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="M138" t="inlineStr">
         <is>
@@ -12562,7 +12562,7 @@
         <v>41</v>
       </c>
       <c r="T138" t="n">
-        <v>1.5</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="U138" t="n">
         <v>33.46666666666667</v>
@@ -12703,10 +12703,10 @@
         <v>28</v>
       </c>
       <c r="K140" t="n">
-        <v>37.6</v>
+        <v>25.9</v>
       </c>
       <c r="L140" t="n">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="M140" t="inlineStr">
         <is>
@@ -12736,7 +12736,7 @@
         <v>28</v>
       </c>
       <c r="T140" t="n">
-        <v>9.600000000000001</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U140" t="n">
         <v>33.96666666666667</v>
@@ -12879,10 +12879,10 @@
         <v>28</v>
       </c>
       <c r="K142" t="n">
-        <v>27.4</v>
+        <v>27.9</v>
       </c>
       <c r="L142" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="M142" t="inlineStr">
         <is>
@@ -12912,7 +12912,7 @@
         <v>28</v>
       </c>
       <c r="T142" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U142" t="n">
         <v>28.4</v>
@@ -13581,10 +13581,10 @@
         <v>35</v>
       </c>
       <c r="K150" t="n">
-        <v>38.6</v>
+        <v>38.2</v>
       </c>
       <c r="L150" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M150" t="inlineStr">
         <is>
@@ -13614,10 +13614,10 @@
         <v>41</v>
       </c>
       <c r="T150" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U150" t="n">
-        <v>36.56666666666667</v>
+        <v>36.56666666666666</v>
       </c>
       <c r="V150" t="n">
         <v>3</v>
@@ -13669,10 +13669,10 @@
         <v>35</v>
       </c>
       <c r="K151" t="n">
-        <v>36.9</v>
+        <v>34.4</v>
       </c>
       <c r="L151" t="n">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="M151" t="inlineStr">
         <is>
@@ -13702,7 +13702,7 @@
         <v>41</v>
       </c>
       <c r="T151" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U151" t="n">
         <v>35.53333333333333</v>
@@ -13711,7 +13711,7 @@
         <v>3</v>
       </c>
       <c r="W151" t="n">
-        <v>36.47037037037038</v>
+        <v>36.47037037037036</v>
       </c>
       <c r="X151" t="n">
         <v>31.5</v>
@@ -13757,10 +13757,10 @@
         <v>28</v>
       </c>
       <c r="K152" t="n">
-        <v>35.4</v>
+        <v>31.9</v>
       </c>
       <c r="L152" t="n">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="M152" t="inlineStr">
         <is>
@@ -13790,7 +13790,7 @@
         <v>28</v>
       </c>
       <c r="T152" t="n">
-        <v>7.399999999999999</v>
+        <v>3.899999999999999</v>
       </c>
       <c r="U152" t="n">
         <v>31.73333333333333</v>
@@ -13845,10 +13845,10 @@
         <v>28</v>
       </c>
       <c r="K153" t="n">
-        <v>30.2</v>
+        <v>30.7</v>
       </c>
       <c r="L153" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="M153" t="inlineStr">
         <is>
@@ -13878,7 +13878,7 @@
         <v>28</v>
       </c>
       <c r="T153" t="n">
-        <v>2.199999999999999</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U153" t="n">
         <v>29.23333333333333</v>
@@ -14105,10 +14105,10 @@
         <v>35</v>
       </c>
       <c r="K156" t="n">
-        <v>32.4</v>
+        <v>37.3</v>
       </c>
       <c r="L156" t="n">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="M156" t="inlineStr">
         <is>
@@ -14138,7 +14138,7 @@
         <v>41</v>
       </c>
       <c r="T156" t="n">
-        <v>-2.600000000000001</v>
+        <v>2.299999999999997</v>
       </c>
       <c r="U156" t="n">
         <v>36.6</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-21 16:42:12
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X373"/>
+  <dimension ref="A1:X375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3417,10 +3417,10 @@
         <v>31</v>
       </c>
       <c r="K34" t="n">
-        <v>27.8</v>
+        <v>38.5</v>
       </c>
       <c r="L34" t="n">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="n">
-        <v>-3.199999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="U34" t="n">
         <v>35.83333333333334</v>
@@ -3503,10 +3503,10 @@
         <v>28</v>
       </c>
       <c r="K35" t="n">
-        <v>33.2</v>
+        <v>22.1</v>
       </c>
       <c r="L35" t="n">
-        <v>118</v>
+        <v>79</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
         <v>28</v>
       </c>
       <c r="T35" t="n">
-        <v>5.200000000000003</v>
+        <v>-5.899999999999999</v>
       </c>
       <c r="U35" t="n">
         <v>30.1</v>
@@ -3591,10 +3591,10 @@
         <v>31</v>
       </c>
       <c r="K36" t="n">
-        <v>30.9</v>
+        <v>32.6</v>
       </c>
       <c r="L36" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U36" t="n">
         <v>30.8</v>
@@ -3631,7 +3631,7 @@
         <v>3</v>
       </c>
       <c r="W36" t="n">
-        <v>41.12222222222222</v>
+        <v>41.12222222222223</v>
       </c>
       <c r="X36" t="n">
         <v>27.5</v>
@@ -3677,10 +3677,10 @@
         <v>28</v>
       </c>
       <c r="K37" t="n">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="L37" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3710,7 +3710,7 @@
         <v>28</v>
       </c>
       <c r="T37" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="U37" t="n">
         <v>30.53333333333333</v>
@@ -3765,10 +3765,10 @@
         <v>28</v>
       </c>
       <c r="K38" t="n">
-        <v>24.9</v>
+        <v>32.4</v>
       </c>
       <c r="L38" t="n">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
         <v>28</v>
       </c>
       <c r="T38" t="n">
-        <v>-3.100000000000001</v>
+        <v>4.399999999999999</v>
       </c>
       <c r="U38" t="n">
         <v>31.5</v>
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L79" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L83" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L90" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L95" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -10417,10 +10417,10 @@
         <v>35</v>
       </c>
       <c r="K114" t="n">
-        <v>31.4</v>
+        <v>49.1</v>
       </c>
       <c r="L114" t="n">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="M114" t="inlineStr">
         <is>
@@ -10450,7 +10450,7 @@
         <v>41</v>
       </c>
       <c r="T114" t="n">
-        <v>-3.600000000000001</v>
+        <v>14.1</v>
       </c>
       <c r="U114" t="n">
         <v>43.96666666666667</v>
@@ -10505,10 +10505,10 @@
         <v>35</v>
       </c>
       <c r="K115" t="n">
-        <v>54.5</v>
+        <v>27.3</v>
       </c>
       <c r="L115" t="n">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -10538,16 +10538,16 @@
         <v>41</v>
       </c>
       <c r="T115" t="n">
-        <v>19.5</v>
+        <v>-7.699999999999999</v>
       </c>
       <c r="U115" t="n">
-        <v>44.90000000000001</v>
+        <v>44.9</v>
       </c>
       <c r="V115" t="n">
         <v>3</v>
       </c>
       <c r="W115" t="n">
-        <v>41.74444444444445</v>
+        <v>41.74444444444444</v>
       </c>
       <c r="X115" t="n">
         <v>31.5</v>
@@ -10593,10 +10593,10 @@
         <v>21</v>
       </c>
       <c r="K116" t="n">
-        <v>19.9</v>
+        <v>24.3</v>
       </c>
       <c r="L116" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="M116" t="inlineStr">
         <is>
@@ -10626,16 +10626,16 @@
         <v>21</v>
       </c>
       <c r="T116" t="n">
-        <v>-1.100000000000001</v>
+        <v>3.300000000000001</v>
       </c>
       <c r="U116" t="n">
-        <v>22.56666666666667</v>
+        <v>22.56666666666666</v>
       </c>
       <c r="V116" t="n">
         <v>3</v>
       </c>
       <c r="W116" t="n">
-        <v>36.05555555555556</v>
+        <v>36.05555555555555</v>
       </c>
       <c r="X116" t="n">
         <v>17.5</v>
@@ -12529,10 +12529,10 @@
         <v>35</v>
       </c>
       <c r="K138" t="n">
-        <v>31.4</v>
+        <v>36.5</v>
       </c>
       <c r="L138" t="n">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="M138" t="inlineStr">
         <is>
@@ -12562,7 +12562,7 @@
         <v>41</v>
       </c>
       <c r="T138" t="n">
-        <v>-3.600000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="U138" t="n">
         <v>33.46666666666667</v>
@@ -12703,10 +12703,10 @@
         <v>28</v>
       </c>
       <c r="K140" t="n">
-        <v>25.9</v>
+        <v>37.6</v>
       </c>
       <c r="L140" t="n">
-        <v>92</v>
+        <v>134</v>
       </c>
       <c r="M140" t="inlineStr">
         <is>
@@ -12736,7 +12736,7 @@
         <v>28</v>
       </c>
       <c r="T140" t="n">
-        <v>-2.100000000000001</v>
+        <v>9.600000000000001</v>
       </c>
       <c r="U140" t="n">
         <v>33.96666666666667</v>
@@ -12879,10 +12879,10 @@
         <v>28</v>
       </c>
       <c r="K142" t="n">
-        <v>27.9</v>
+        <v>27.4</v>
       </c>
       <c r="L142" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="M142" t="inlineStr">
         <is>
@@ -12912,7 +12912,7 @@
         <v>28</v>
       </c>
       <c r="T142" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U142" t="n">
         <v>28.4</v>
@@ -13581,10 +13581,10 @@
         <v>35</v>
       </c>
       <c r="K150" t="n">
-        <v>38.2</v>
+        <v>38.6</v>
       </c>
       <c r="L150" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="M150" t="inlineStr">
         <is>
@@ -13614,10 +13614,10 @@
         <v>41</v>
       </c>
       <c r="T150" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U150" t="n">
-        <v>36.56666666666666</v>
+        <v>36.56666666666667</v>
       </c>
       <c r="V150" t="n">
         <v>3</v>
@@ -13669,10 +13669,10 @@
         <v>35</v>
       </c>
       <c r="K151" t="n">
-        <v>34.4</v>
+        <v>36.9</v>
       </c>
       <c r="L151" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="M151" t="inlineStr">
         <is>
@@ -13702,7 +13702,7 @@
         <v>41</v>
       </c>
       <c r="T151" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U151" t="n">
         <v>35.53333333333333</v>
@@ -13711,7 +13711,7 @@
         <v>3</v>
       </c>
       <c r="W151" t="n">
-        <v>36.47037037037036</v>
+        <v>36.47037037037038</v>
       </c>
       <c r="X151" t="n">
         <v>31.5</v>
@@ -13757,10 +13757,10 @@
         <v>28</v>
       </c>
       <c r="K152" t="n">
-        <v>31.9</v>
+        <v>35.4</v>
       </c>
       <c r="L152" t="n">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="M152" t="inlineStr">
         <is>
@@ -13790,7 +13790,7 @@
         <v>28</v>
       </c>
       <c r="T152" t="n">
-        <v>3.899999999999999</v>
+        <v>7.399999999999999</v>
       </c>
       <c r="U152" t="n">
         <v>31.73333333333333</v>
@@ -13845,10 +13845,10 @@
         <v>28</v>
       </c>
       <c r="K153" t="n">
-        <v>30.7</v>
+        <v>30.2</v>
       </c>
       <c r="L153" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="M153" t="inlineStr">
         <is>
@@ -13878,7 +13878,7 @@
         <v>28</v>
       </c>
       <c r="T153" t="n">
-        <v>2.699999999999999</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U153" t="n">
         <v>29.23333333333333</v>
@@ -14105,10 +14105,10 @@
         <v>35</v>
       </c>
       <c r="K156" t="n">
-        <v>37.3</v>
+        <v>32.4</v>
       </c>
       <c r="L156" t="n">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="M156" t="inlineStr">
         <is>
@@ -14138,7 +14138,7 @@
         <v>41</v>
       </c>
       <c r="T156" t="n">
-        <v>2.299999999999997</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U156" t="n">
         <v>36.6</v>
@@ -21391,10 +21391,10 @@
         <v>31</v>
       </c>
       <c r="K239" t="n">
-        <v>28.1</v>
+        <v>31.5</v>
       </c>
       <c r="L239" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="M239" t="inlineStr">
         <is>
@@ -21422,7 +21422,7 @@
       </c>
       <c r="S239" t="inlineStr"/>
       <c r="T239" t="n">
-        <v>-2.899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="U239" t="n">
         <v>30.6</v>
@@ -25417,10 +25417,10 @@
         <v>21</v>
       </c>
       <c r="K285" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
       <c r="L285" t="n">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="M285" t="inlineStr">
         <is>
@@ -25450,7 +25450,7 @@
         <v>21</v>
       </c>
       <c r="T285" t="n">
-        <v>-3.399999999999999</v>
+        <v>-3.699999999999999</v>
       </c>
       <c r="U285" t="n">
         <v>17.43333333333333</v>
@@ -25505,10 +25505,10 @@
         <v>21</v>
       </c>
       <c r="K286" t="n">
-        <v>19.8</v>
+        <v>24</v>
       </c>
       <c r="L286" t="n">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="M286" t="inlineStr">
         <is>
@@ -25538,7 +25538,7 @@
         <v>21</v>
       </c>
       <c r="T286" t="n">
-        <v>-1.199999999999999</v>
+        <v>3</v>
       </c>
       <c r="U286" t="n">
         <v>22.96666666666667</v>
@@ -26205,10 +26205,10 @@
         <v>21</v>
       </c>
       <c r="K294" t="n">
-        <v>22.2</v>
+        <v>20.9</v>
       </c>
       <c r="L294" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="M294" t="inlineStr">
         <is>
@@ -26238,7 +26238,7 @@
         <v>21</v>
       </c>
       <c r="T294" t="n">
-        <v>1.199999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U294" t="n">
         <v>22.03333333333333</v>
@@ -27257,10 +27257,10 @@
         <v>21</v>
       </c>
       <c r="K306" t="n">
-        <v>20.4</v>
+        <v>21.2</v>
       </c>
       <c r="L306" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="M306" t="inlineStr">
         <is>
@@ -27290,16 +27290,16 @@
         <v>21</v>
       </c>
       <c r="T306" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U306" t="n">
-        <v>21.16666666666667</v>
+        <v>21.16666666666666</v>
       </c>
       <c r="V306" t="n">
         <v>3</v>
       </c>
       <c r="W306" t="n">
-        <v>22.05555555555556</v>
+        <v>22.05555555555555</v>
       </c>
       <c r="X306" t="n">
         <v>17.5</v>
@@ -28047,10 +28047,10 @@
         <v>24.5</v>
       </c>
       <c r="K315" t="n">
-        <v>22.5</v>
+        <v>21.4</v>
       </c>
       <c r="L315" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="M315" t="inlineStr">
         <is>
@@ -28080,7 +28080,7 @@
         <v>28</v>
       </c>
       <c r="T315" t="n">
-        <v>-2</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="U315" t="n">
         <v>21.53333333333333</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L325" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29279,10 +29279,10 @@
         <v>24.5</v>
       </c>
       <c r="K329" t="n">
-        <v>23.6</v>
+        <v>24.2</v>
       </c>
       <c r="L329" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="M329" t="inlineStr">
         <is>
@@ -29312,10 +29312,10 @@
         <v>28</v>
       </c>
       <c r="T329" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U329" t="n">
-        <v>24.93333333333333</v>
+        <v>24.93333333333334</v>
       </c>
       <c r="V329" t="n">
         <v>3</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L333" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -30599,10 +30599,10 @@
         <v>24.5</v>
       </c>
       <c r="K344" t="n">
-        <v>23.5</v>
+        <v>21.6</v>
       </c>
       <c r="L344" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="M344" t="inlineStr">
         <is>
@@ -30632,7 +30632,7 @@
         <v>28</v>
       </c>
       <c r="T344" t="n">
-        <v>-1</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="U344" t="n">
         <v>23.1</v>
@@ -30687,10 +30687,10 @@
         <v>24.5</v>
       </c>
       <c r="K345" t="n">
-        <v>26.3</v>
+        <v>28.4</v>
       </c>
       <c r="L345" t="n">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="M345" t="inlineStr">
         <is>
@@ -30720,7 +30720,7 @@
         <v>28</v>
       </c>
       <c r="T345" t="n">
-        <v>1.800000000000001</v>
+        <v>3.899999999999999</v>
       </c>
       <c r="U345" t="n">
         <v>26.36666666666666</v>
@@ -30729,7 +30729,7 @@
         <v>3</v>
       </c>
       <c r="W345" t="n">
-        <v>23.35555555555555</v>
+        <v>23.35555555555556</v>
       </c>
       <c r="X345" t="n">
         <v>21</v>
@@ -30775,10 +30775,10 @@
         <v>24.5</v>
       </c>
       <c r="K346" t="n">
-        <v>23.3</v>
+        <v>25.4</v>
       </c>
       <c r="L346" t="n">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="M346" t="inlineStr">
         <is>
@@ -30808,10 +30808,10 @@
         <v>28</v>
       </c>
       <c r="T346" t="n">
-        <v>-1.199999999999999</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U346" t="n">
-        <v>24.56666666666666</v>
+        <v>24.56666666666667</v>
       </c>
       <c r="V346" t="n">
         <v>3</v>
@@ -30951,10 +30951,10 @@
         <v>24.5</v>
       </c>
       <c r="K348" t="n">
-        <v>22.3</v>
+        <v>23.3</v>
       </c>
       <c r="L348" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="M348" t="inlineStr">
         <is>
@@ -30984,7 +30984,7 @@
         <v>28</v>
       </c>
       <c r="T348" t="n">
-        <v>-2.199999999999999</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U348" t="n">
         <v>23.03333333333333</v>
@@ -31039,10 +31039,10 @@
         <v>24.5</v>
       </c>
       <c r="K349" t="n">
-        <v>23.5</v>
+        <v>25.4</v>
       </c>
       <c r="L349" t="n">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="M349" t="inlineStr">
         <is>
@@ -31072,7 +31072,7 @@
         <v>28</v>
       </c>
       <c r="T349" t="n">
-        <v>-1</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U349" t="n">
         <v>24.63333333333334</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L355" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>
@@ -32933,7 +32933,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>PL24</t>
+          <t>PL-48</t>
         </is>
       </c>
       <c r="C371" t="inlineStr"/>
@@ -32944,17 +32944,17 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>CIMEANTACION PLATAFORMA ZARPA Y ZAPATA EJE C-12 ZAPATA EJE E-6</t>
+          <t>Plataforma P1 vigas eje 6-5 entre A-D</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
         <is>
-          <t>9/25/2026 12:00:00 AM</t>
+          <t>10/16/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H371" t="inlineStr"/>
@@ -32965,10 +32965,10 @@
         <v>21</v>
       </c>
       <c r="K371" t="n">
-        <v>18.9</v>
+        <v>20</v>
       </c>
       <c r="L371" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="M371" t="inlineStr">
         <is>
@@ -32996,16 +32996,16 @@
       </c>
       <c r="S371" t="inlineStr"/>
       <c r="T371" t="n">
-        <v>-2.100000000000001</v>
+        <v>-1</v>
       </c>
       <c r="U371" t="n">
-        <v>19.9</v>
+        <v>22.3</v>
       </c>
       <c r="V371" t="n">
         <v>3</v>
       </c>
       <c r="W371" t="n">
-        <v>23.37777777777778</v>
+        <v>20.43333333333333</v>
       </c>
       <c r="X371" t="n">
         <v>17.5</v>
@@ -33019,7 +33019,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>PL30</t>
+          <t>PL-49</t>
         </is>
       </c>
       <c r="C372" t="inlineStr"/>
@@ -33030,17 +33030,17 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>VIGAS PLACA PLATAFORMA PISO 1 EJE A-B, 11,10,09</t>
+          <t>Plataforma P1 placa eje 6-5 entre A-D</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>10/1/2026 12:00:00 AM</t>
+          <t>10/16/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H372" t="inlineStr"/>
@@ -33051,10 +33051,10 @@
         <v>21</v>
       </c>
       <c r="K372" t="n">
-        <v>23.5</v>
+        <v>20.4</v>
       </c>
       <c r="L372" t="n">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="M372" t="inlineStr">
         <is>
@@ -33084,16 +33084,16 @@
         <v>21</v>
       </c>
       <c r="T372" t="n">
-        <v>2.5</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U372" t="n">
-        <v>22.16666666666667</v>
+        <v>19.6</v>
       </c>
       <c r="V372" t="n">
         <v>3</v>
       </c>
       <c r="W372" t="n">
-        <v>25.15555555555556</v>
+        <v>21.95555555555556</v>
       </c>
       <c r="X372" t="n">
         <v>17.5</v>
@@ -33107,7 +33107,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>SC 05</t>
+          <t>PL24</t>
         </is>
       </c>
       <c r="C373" t="inlineStr"/>
@@ -33118,17 +33118,17 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>VIGAS CIMENTACION PLACA SUPERIOR EJE 1-3 ENTRE A Y F-SC</t>
+          <t>CIMEANTACION PLATAFORMA ZARPA Y ZAPATA EJE C-12 ZAPATA EJE E-6</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>9/24/2026 12:00:00 AM</t>
+          <t>9/25/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H373" t="inlineStr"/>
@@ -33139,51 +33139,225 @@
         <v>21</v>
       </c>
       <c r="K373" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="L373" t="n">
+        <v>90</v>
+      </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>AUTOCOMPAC</t>
+        </is>
+      </c>
+      <c r="N373" t="n">
+        <v>21</v>
+      </c>
+      <c r="O373" t="inlineStr">
+        <is>
+          <t>AUTOCOMPAC-21-28</t>
+        </is>
+      </c>
+      <c r="P373" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="Q373" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="R373" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="S373" t="inlineStr"/>
+      <c r="T373" t="n">
+        <v>-2.100000000000001</v>
+      </c>
+      <c r="U373" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="V373" t="n">
+        <v>3</v>
+      </c>
+      <c r="W373" t="n">
+        <v>23.37777777777778</v>
+      </c>
+      <c r="X373" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>VIALE 26</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>PL30</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr"/>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>VIGAS PLACA PLATAFORMA PISO 1 EJE A-B, 11,10,09</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>10/1/2026 12:00:00 AM</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr"/>
+      <c r="I374" t="n">
+        <v>28</v>
+      </c>
+      <c r="J374" t="n">
+        <v>21</v>
+      </c>
+      <c r="K374" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="L374" t="n">
+        <v>112</v>
+      </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>PLACA</t>
+        </is>
+      </c>
+      <c r="N374" t="n">
+        <v>21</v>
+      </c>
+      <c r="O374" t="inlineStr">
+        <is>
+          <t>PLACA-21-28</t>
+        </is>
+      </c>
+      <c r="P374" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="Q374" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="R374" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="S374" t="n">
+        <v>21</v>
+      </c>
+      <c r="T374" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="U374" t="n">
+        <v>22.16666666666667</v>
+      </c>
+      <c r="V374" t="n">
+        <v>3</v>
+      </c>
+      <c r="W374" t="n">
+        <v>25.15555555555556</v>
+      </c>
+      <c r="X374" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>VIALE 26</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>SC 05</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr"/>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>VIGAS CIMENTACION PLACA SUPERIOR EJE 1-3 ENTRE A Y F-SC</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>9/24/2026 12:00:00 AM</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr"/>
+      <c r="I375" t="n">
+        <v>28</v>
+      </c>
+      <c r="J375" t="n">
+        <v>21</v>
+      </c>
+      <c r="K375" t="n">
         <v>19.8</v>
       </c>
-      <c r="L373" t="n">
+      <c r="L375" t="n">
         <v>94</v>
       </c>
-      <c r="M373" t="inlineStr">
+      <c r="M375" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="N373" t="n">
-        <v>21</v>
-      </c>
-      <c r="O373" t="inlineStr">
+      <c r="N375" t="n">
+        <v>21</v>
+      </c>
+      <c r="O375" t="inlineStr">
         <is>
           <t>PLACA-21-28</t>
         </is>
       </c>
-      <c r="P373" s="2" t="n">
-        <v>46316</v>
-      </c>
-      <c r="Q373" t="inlineStr">
-        <is>
-          <t>NUEVO</t>
-        </is>
-      </c>
-      <c r="R373" s="2" t="n">
-        <v>46316</v>
-      </c>
-      <c r="S373" t="n">
-        <v>21</v>
-      </c>
-      <c r="T373" t="n">
+      <c r="P375" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="Q375" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="R375" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="S375" t="n">
+        <v>21</v>
+      </c>
+      <c r="T375" t="n">
         <v>-1.199999999999999</v>
       </c>
-      <c r="U373" t="n">
+      <c r="U375" t="n">
         <v>18.9</v>
       </c>
-      <c r="V373" t="n">
-        <v>3</v>
-      </c>
-      <c r="W373" t="n">
+      <c r="V375" t="n">
+        <v>3</v>
+      </c>
+      <c r="W375" t="n">
         <v>22.93333333333334</v>
       </c>
-      <c r="X373" t="n">
+      <c r="X375" t="n">
         <v>17.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-21 18:42:31
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3765,10 +3765,10 @@
         <v>28</v>
       </c>
       <c r="K38" t="n">
-        <v>32.4</v>
+        <v>24.9</v>
       </c>
       <c r="L38" t="n">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
         <v>28</v>
       </c>
       <c r="T38" t="n">
-        <v>4.399999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="U38" t="n">
         <v>31.5</v>
@@ -3981,7 +3981,7 @@
         <v>3</v>
       </c>
       <c r="W40" t="n">
-        <v>35.58888888888889</v>
+        <v>39.51111111111111</v>
       </c>
       <c r="X40" t="n">
         <v>24.5</v>
@@ -4067,7 +4067,7 @@
         <v>3</v>
       </c>
       <c r="W41" t="n">
-        <v>38.09999999999999</v>
+        <v>39.12222222222223</v>
       </c>
       <c r="X41" t="n">
         <v>27.5</v>
@@ -7615,10 +7615,10 @@
         <v>28</v>
       </c>
       <c r="K82" t="n">
-        <v>30.7</v>
+        <v>27.7</v>
       </c>
       <c r="L82" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
         <v>28</v>
       </c>
       <c r="T82" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U82" t="n">
         <v>29.2</v>
@@ -12617,10 +12617,10 @@
         <v>31</v>
       </c>
       <c r="K139" t="n">
-        <v>31.9</v>
+        <v>30.5</v>
       </c>
       <c r="L139" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="M139" t="inlineStr">
         <is>
@@ -12648,7 +12648,7 @@
       </c>
       <c r="S139" t="inlineStr"/>
       <c r="T139" t="n">
-        <v>0.8999999999999986</v>
+        <v>-0.5</v>
       </c>
       <c r="U139" t="n">
         <v>31.23333333333333</v>
@@ -19723,10 +19723,10 @@
         <v>28</v>
       </c>
       <c r="K220" t="n">
-        <v>28.5</v>
+        <v>27.7</v>
       </c>
       <c r="L220" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M220" t="inlineStr">
         <is>
@@ -19756,7 +19756,7 @@
         <v>28</v>
       </c>
       <c r="T220" t="n">
-        <v>0.5</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U220" t="n">
         <v>28.33333333333333</v>
@@ -20691,10 +20691,10 @@
         <v>28</v>
       </c>
       <c r="K231" t="n">
-        <v>29.3</v>
+        <v>30.1</v>
       </c>
       <c r="L231" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="M231" t="inlineStr">
         <is>
@@ -20724,7 +20724,7 @@
         <v>28</v>
       </c>
       <c r="T231" t="n">
-        <v>1.300000000000001</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="U231" t="n">
         <v>28.96666666666667</v>
@@ -20779,10 +20779,10 @@
         <v>21</v>
       </c>
       <c r="K232" t="n">
-        <v>22.9</v>
+        <v>21.7</v>
       </c>
       <c r="L232" t="n">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="M232" t="inlineStr">
         <is>
@@ -20812,7 +20812,7 @@
         <v>21</v>
       </c>
       <c r="T232" t="n">
-        <v>1.899999999999999</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U232" t="n">
         <v>21.83333333333333</v>
@@ -20953,10 +20953,10 @@
         <v>21</v>
       </c>
       <c r="K234" t="n">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="L234" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="M234" t="inlineStr">
         <is>
@@ -20986,7 +20986,7 @@
         <v>21</v>
       </c>
       <c r="T234" t="n">
-        <v>1.800000000000001</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="U234" t="n">
         <v>21.56666666666667</v>
@@ -21303,10 +21303,10 @@
         <v>42</v>
       </c>
       <c r="K238" t="n">
-        <v>31.1</v>
+        <v>49</v>
       </c>
       <c r="L238" t="n">
-        <v>74</v>
+        <v>116</v>
       </c>
       <c r="M238" t="inlineStr">
         <is>
@@ -21336,7 +21336,7 @@
         <v>48</v>
       </c>
       <c r="T238" t="n">
-        <v>-10.9</v>
+        <v>7</v>
       </c>
       <c r="U238" t="n">
         <v>43.9</v>
@@ -21391,10 +21391,10 @@
         <v>31</v>
       </c>
       <c r="K239" t="n">
-        <v>31.5</v>
+        <v>28.1</v>
       </c>
       <c r="L239" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M239" t="inlineStr">
         <is>
@@ -21422,7 +21422,7 @@
       </c>
       <c r="S239" t="inlineStr"/>
       <c r="T239" t="n">
-        <v>0.5</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="U239" t="n">
         <v>30.6</v>
@@ -22179,10 +22179,10 @@
         <v>21</v>
       </c>
       <c r="K248" t="n">
-        <v>17.3</v>
+        <v>21.6</v>
       </c>
       <c r="L248" t="n">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="M248" t="inlineStr">
         <is>
@@ -22210,7 +22210,7 @@
       </c>
       <c r="S248" t="inlineStr"/>
       <c r="T248" t="n">
-        <v>-3.699999999999999</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U248" t="n">
         <v>19.3</v>
@@ -25417,10 +25417,10 @@
         <v>21</v>
       </c>
       <c r="K285" t="n">
-        <v>17.3</v>
+        <v>17.6</v>
       </c>
       <c r="L285" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="M285" t="inlineStr">
         <is>
@@ -25450,7 +25450,7 @@
         <v>21</v>
       </c>
       <c r="T285" t="n">
-        <v>-3.699999999999999</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U285" t="n">
         <v>17.43333333333333</v>
@@ -25505,10 +25505,10 @@
         <v>21</v>
       </c>
       <c r="K286" t="n">
-        <v>24</v>
+        <v>19.8</v>
       </c>
       <c r="L286" t="n">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="M286" t="inlineStr">
         <is>
@@ -25538,7 +25538,7 @@
         <v>21</v>
       </c>
       <c r="T286" t="n">
-        <v>3</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U286" t="n">
         <v>22.96666666666667</v>
@@ -26205,10 +26205,10 @@
         <v>21</v>
       </c>
       <c r="K294" t="n">
-        <v>20.9</v>
+        <v>22.2</v>
       </c>
       <c r="L294" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="M294" t="inlineStr">
         <is>
@@ -26238,7 +26238,7 @@
         <v>21</v>
       </c>
       <c r="T294" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="U294" t="n">
         <v>22.03333333333333</v>
@@ -27257,10 +27257,10 @@
         <v>21</v>
       </c>
       <c r="K306" t="n">
-        <v>21.2</v>
+        <v>20.4</v>
       </c>
       <c r="L306" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M306" t="inlineStr">
         <is>
@@ -27290,16 +27290,16 @@
         <v>21</v>
       </c>
       <c r="T306" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U306" t="n">
-        <v>21.16666666666666</v>
+        <v>21.16666666666667</v>
       </c>
       <c r="V306" t="n">
         <v>3</v>
       </c>
       <c r="W306" t="n">
-        <v>22.05555555555555</v>
+        <v>22.05555555555556</v>
       </c>
       <c r="X306" t="n">
         <v>17.5</v>
@@ -28047,10 +28047,10 @@
         <v>24.5</v>
       </c>
       <c r="K315" t="n">
-        <v>21.4</v>
+        <v>22.5</v>
       </c>
       <c r="L315" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="M315" t="inlineStr">
         <is>
@@ -28080,7 +28080,7 @@
         <v>28</v>
       </c>
       <c r="T315" t="n">
-        <v>-3.100000000000001</v>
+        <v>-2</v>
       </c>
       <c r="U315" t="n">
         <v>21.53333333333333</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29279,10 +29279,10 @@
         <v>24.5</v>
       </c>
       <c r="K329" t="n">
-        <v>24.2</v>
+        <v>23.6</v>
       </c>
       <c r="L329" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="M329" t="inlineStr">
         <is>
@@ -29312,10 +29312,10 @@
         <v>28</v>
       </c>
       <c r="T329" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U329" t="n">
-        <v>24.93333333333334</v>
+        <v>24.93333333333333</v>
       </c>
       <c r="V329" t="n">
         <v>3</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -30553,7 +30553,7 @@
         <v>3</v>
       </c>
       <c r="W343" t="n">
-        <v>29.64444444444445</v>
+        <v>29.32222222222222</v>
       </c>
       <c r="X343" t="n">
         <v>21</v>
@@ -30599,10 +30599,10 @@
         <v>24.5</v>
       </c>
       <c r="K344" t="n">
-        <v>21.6</v>
+        <v>23.5</v>
       </c>
       <c r="L344" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="M344" t="inlineStr">
         <is>
@@ -30632,7 +30632,7 @@
         <v>28</v>
       </c>
       <c r="T344" t="n">
-        <v>-2.899999999999999</v>
+        <v>-1</v>
       </c>
       <c r="U344" t="n">
         <v>23.1</v>
@@ -30687,10 +30687,10 @@
         <v>24.5</v>
       </c>
       <c r="K345" t="n">
-        <v>28.4</v>
+        <v>26.3</v>
       </c>
       <c r="L345" t="n">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="M345" t="inlineStr">
         <is>
@@ -30720,7 +30720,7 @@
         <v>28</v>
       </c>
       <c r="T345" t="n">
-        <v>3.899999999999999</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="U345" t="n">
         <v>26.36666666666666</v>
@@ -30729,7 +30729,7 @@
         <v>3</v>
       </c>
       <c r="W345" t="n">
-        <v>23.35555555555556</v>
+        <v>23.35555555555555</v>
       </c>
       <c r="X345" t="n">
         <v>21</v>
@@ -30775,10 +30775,10 @@
         <v>24.5</v>
       </c>
       <c r="K346" t="n">
-        <v>25.4</v>
+        <v>23.3</v>
       </c>
       <c r="L346" t="n">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="M346" t="inlineStr">
         <is>
@@ -30808,10 +30808,10 @@
         <v>28</v>
       </c>
       <c r="T346" t="n">
-        <v>0.8999999999999986</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U346" t="n">
-        <v>24.56666666666667</v>
+        <v>24.56666666666666</v>
       </c>
       <c r="V346" t="n">
         <v>3</v>
@@ -30951,10 +30951,10 @@
         <v>24.5</v>
       </c>
       <c r="K348" t="n">
-        <v>23.3</v>
+        <v>22.3</v>
       </c>
       <c r="L348" t="n">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="M348" t="inlineStr">
         <is>
@@ -30984,7 +30984,7 @@
         <v>28</v>
       </c>
       <c r="T348" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="U348" t="n">
         <v>23.03333333333333</v>
@@ -31039,10 +31039,10 @@
         <v>24.5</v>
       </c>
       <c r="K349" t="n">
-        <v>25.4</v>
+        <v>23.5</v>
       </c>
       <c r="L349" t="n">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="M349" t="inlineStr">
         <is>
@@ -31072,7 +31072,7 @@
         <v>28</v>
       </c>
       <c r="T349" t="n">
-        <v>0.8999999999999986</v>
+        <v>-1</v>
       </c>
       <c r="U349" t="n">
         <v>24.63333333333334</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-21 20:02:13
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3417,10 +3417,10 @@
         <v>31</v>
       </c>
       <c r="K34" t="n">
-        <v>38.5</v>
+        <v>27.8</v>
       </c>
       <c r="L34" t="n">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="n">
-        <v>7.5</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U34" t="n">
         <v>35.83333333333334</v>
@@ -3503,10 +3503,10 @@
         <v>28</v>
       </c>
       <c r="K35" t="n">
-        <v>22.1</v>
+        <v>33.2</v>
       </c>
       <c r="L35" t="n">
-        <v>79</v>
+        <v>118</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
         <v>28</v>
       </c>
       <c r="T35" t="n">
-        <v>-5.899999999999999</v>
+        <v>5.200000000000003</v>
       </c>
       <c r="U35" t="n">
         <v>30.1</v>
@@ -3591,10 +3591,10 @@
         <v>31</v>
       </c>
       <c r="K36" t="n">
-        <v>32.6</v>
+        <v>30.9</v>
       </c>
       <c r="L36" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="n">
-        <v>1.600000000000001</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U36" t="n">
         <v>30.8</v>
@@ -3631,7 +3631,7 @@
         <v>3</v>
       </c>
       <c r="W36" t="n">
-        <v>41.12222222222223</v>
+        <v>41.12222222222222</v>
       </c>
       <c r="X36" t="n">
         <v>27.5</v>
@@ -3677,10 +3677,10 @@
         <v>28</v>
       </c>
       <c r="K37" t="n">
-        <v>32.5</v>
+        <v>32</v>
       </c>
       <c r="L37" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3710,7 +3710,7 @@
         <v>28</v>
       </c>
       <c r="T37" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="U37" t="n">
         <v>30.53333333333333</v>
@@ -5073,7 +5073,7 @@
         <v>24</v>
       </c>
       <c r="K53" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="L53" t="n">
         <v>103</v>
@@ -5106,7 +5106,7 @@
         <v>28</v>
       </c>
       <c r="T53" t="n">
-        <v>0.6999999999999993</v>
+        <v>0.8000000000000007</v>
       </c>
       <c r="U53" t="n">
         <v>23.53333333333333</v>
@@ -6385,10 +6385,10 @@
         <v>28</v>
       </c>
       <c r="K68" t="n">
-        <v>30.5</v>
+        <v>27.9</v>
       </c>
       <c r="L68" t="n">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="M68" t="inlineStr">
         <is>
@@ -6418,7 +6418,7 @@
         <v>28</v>
       </c>
       <c r="T68" t="n">
-        <v>2.5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U68" t="n">
         <v>29.13333333333334</v>
@@ -7615,10 +7615,10 @@
         <v>28</v>
       </c>
       <c r="K82" t="n">
-        <v>27.7</v>
+        <v>30.7</v>
       </c>
       <c r="L82" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
         <v>28</v>
       </c>
       <c r="T82" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U82" t="n">
         <v>29.2</v>
@@ -10329,10 +10329,10 @@
         <v>35</v>
       </c>
       <c r="K113" t="n">
-        <v>27.1</v>
+        <v>29.6</v>
       </c>
       <c r="L113" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="M113" t="inlineStr">
         <is>
@@ -10362,7 +10362,7 @@
         <v>41</v>
       </c>
       <c r="T113" t="n">
-        <v>-7.899999999999999</v>
+        <v>-5.399999999999999</v>
       </c>
       <c r="U113" t="n">
         <v>27.33333333333333</v>
@@ -10681,10 +10681,10 @@
         <v>35</v>
       </c>
       <c r="K117" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="L117" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="M117" t="inlineStr">
         <is>
@@ -10714,7 +10714,7 @@
         <v>41</v>
       </c>
       <c r="T117" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="U117" t="n">
         <v>25.5</v>
@@ -11297,10 +11297,10 @@
         <v>21</v>
       </c>
       <c r="K124" t="n">
-        <v>19.3</v>
+        <v>26</v>
       </c>
       <c r="L124" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11330,7 +11330,7 @@
         <v>21</v>
       </c>
       <c r="T124" t="n">
-        <v>-1.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="U124" t="n">
         <v>23.7</v>
@@ -12617,10 +12617,10 @@
         <v>31</v>
       </c>
       <c r="K139" t="n">
-        <v>30.5</v>
+        <v>31.9</v>
       </c>
       <c r="L139" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="M139" t="inlineStr">
         <is>
@@ -12648,7 +12648,7 @@
       </c>
       <c r="S139" t="inlineStr"/>
       <c r="T139" t="n">
-        <v>-0.5</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U139" t="n">
         <v>31.23333333333333</v>
@@ -12703,10 +12703,10 @@
         <v>28</v>
       </c>
       <c r="K140" t="n">
-        <v>37.6</v>
+        <v>25.9</v>
       </c>
       <c r="L140" t="n">
-        <v>134</v>
+        <v>92</v>
       </c>
       <c r="M140" t="inlineStr">
         <is>
@@ -12736,7 +12736,7 @@
         <v>28</v>
       </c>
       <c r="T140" t="n">
-        <v>9.600000000000001</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U140" t="n">
         <v>33.96666666666667</v>
@@ -14721,10 +14721,10 @@
         <v>21</v>
       </c>
       <c r="K163" t="n">
-        <v>20.8</v>
+        <v>26.4</v>
       </c>
       <c r="L163" t="n">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="M163" t="inlineStr">
         <is>
@@ -14754,7 +14754,7 @@
         <v>21</v>
       </c>
       <c r="T163" t="n">
-        <v>-0.1999999999999993</v>
+        <v>5.399999999999999</v>
       </c>
       <c r="U163" t="n">
         <v>24.5</v>
@@ -19109,10 +19109,10 @@
         <v>28</v>
       </c>
       <c r="K213" t="n">
-        <v>26.2</v>
+        <v>32.6</v>
       </c>
       <c r="L213" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="M213" t="inlineStr">
         <is>
@@ -19142,7 +19142,7 @@
         <v>28</v>
       </c>
       <c r="T213" t="n">
-        <v>-1.800000000000001</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="U213" t="n">
         <v>30.03333333333333</v>
@@ -19723,10 +19723,10 @@
         <v>28</v>
       </c>
       <c r="K220" t="n">
-        <v>27.7</v>
+        <v>28.5</v>
       </c>
       <c r="L220" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M220" t="inlineStr">
         <is>
@@ -19756,7 +19756,7 @@
         <v>28</v>
       </c>
       <c r="T220" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.5</v>
       </c>
       <c r="U220" t="n">
         <v>28.33333333333333</v>
@@ -20691,10 +20691,10 @@
         <v>28</v>
       </c>
       <c r="K231" t="n">
-        <v>30.1</v>
+        <v>29.3</v>
       </c>
       <c r="L231" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="M231" t="inlineStr">
         <is>
@@ -20724,7 +20724,7 @@
         <v>28</v>
       </c>
       <c r="T231" t="n">
-        <v>2.100000000000001</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="U231" t="n">
         <v>28.96666666666667</v>
@@ -20779,10 +20779,10 @@
         <v>21</v>
       </c>
       <c r="K232" t="n">
-        <v>21.7</v>
+        <v>22.9</v>
       </c>
       <c r="L232" t="n">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="M232" t="inlineStr">
         <is>
@@ -20812,7 +20812,7 @@
         <v>21</v>
       </c>
       <c r="T232" t="n">
-        <v>0.6999999999999993</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U232" t="n">
         <v>21.83333333333333</v>
@@ -21303,10 +21303,10 @@
         <v>42</v>
       </c>
       <c r="K238" t="n">
-        <v>49</v>
+        <v>31.1</v>
       </c>
       <c r="L238" t="n">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="M238" t="inlineStr">
         <is>
@@ -21336,7 +21336,7 @@
         <v>48</v>
       </c>
       <c r="T238" t="n">
-        <v>7</v>
+        <v>-10.9</v>
       </c>
       <c r="U238" t="n">
         <v>43.9</v>
@@ -22179,10 +22179,10 @@
         <v>21</v>
       </c>
       <c r="K248" t="n">
-        <v>21.6</v>
+        <v>17.3</v>
       </c>
       <c r="L248" t="n">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="M248" t="inlineStr">
         <is>
@@ -22210,7 +22210,7 @@
       </c>
       <c r="S248" t="inlineStr"/>
       <c r="T248" t="n">
-        <v>0.6000000000000014</v>
+        <v>-3.699999999999999</v>
       </c>
       <c r="U248" t="n">
         <v>19.3</v>
@@ -33005,7 +33005,7 @@
         <v>3</v>
       </c>
       <c r="W371" t="n">
-        <v>20.43333333333333</v>
+        <v>26.88888888888889</v>
       </c>
       <c r="X371" t="n">
         <v>17.5</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-22 07:10:18
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2899,10 +2899,10 @@
         <v>31</v>
       </c>
       <c r="K28" t="n">
-        <v>31.1</v>
+        <v>29.3</v>
       </c>
       <c r="L28" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="n">
-        <v>0.1000000000000014</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U28" t="n">
         <v>31.2</v>
@@ -5859,10 +5859,10 @@
         <v>31</v>
       </c>
       <c r="K62" t="n">
-        <v>31.4</v>
+        <v>35.8</v>
       </c>
       <c r="L62" t="n">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
@@ -5890,10 +5890,10 @@
       </c>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="n">
-        <v>0.3999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="U62" t="n">
-        <v>30.66666666666666</v>
+        <v>30.66666666666667</v>
       </c>
       <c r="V62" t="n">
         <v>3</v>
@@ -6121,10 +6121,10 @@
         <v>24</v>
       </c>
       <c r="K65" t="n">
-        <v>16.6</v>
+        <v>27.2</v>
       </c>
       <c r="L65" t="n">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -6154,7 +6154,7 @@
         <v>28</v>
       </c>
       <c r="T65" t="n">
-        <v>-7.399999999999999</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="U65" t="n">
         <v>23.4</v>
@@ -6297,10 +6297,10 @@
         <v>28</v>
       </c>
       <c r="K67" t="n">
-        <v>30.4</v>
+        <v>31.6</v>
       </c>
       <c r="L67" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -6330,7 +6330,7 @@
         <v>28</v>
       </c>
       <c r="T67" t="n">
-        <v>2.399999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U67" t="n">
         <v>29.86666666666666</v>
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L79" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7527,10 +7527,10 @@
         <v>28</v>
       </c>
       <c r="K81" t="n">
-        <v>24.8</v>
+        <v>25.9</v>
       </c>
       <c r="L81" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,10 +7560,10 @@
         <v>28</v>
       </c>
       <c r="T81" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U81" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="V81" t="n">
         <v>3</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L83" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L90" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L95" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -11913,10 +11913,10 @@
         <v>28</v>
       </c>
       <c r="K131" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="L131" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="M131" t="inlineStr">
         <is>
@@ -11946,7 +11946,7 @@
         <v>28</v>
       </c>
       <c r="T131" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U131" t="n">
         <v>25.36666666666666</v>
@@ -24187,10 +24187,10 @@
         <v>28</v>
       </c>
       <c r="K271" t="n">
-        <v>21.8</v>
+        <v>31.4</v>
       </c>
       <c r="L271" t="n">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="M271" t="inlineStr">
         <is>
@@ -24220,7 +24220,7 @@
         <v>28</v>
       </c>
       <c r="T271" t="n">
-        <v>-6.199999999999999</v>
+        <v>3.399999999999999</v>
       </c>
       <c r="U271" t="n">
         <v>28.2</v>
@@ -25241,10 +25241,10 @@
         <v>28</v>
       </c>
       <c r="K283" t="n">
-        <v>27.2</v>
+        <v>28.3</v>
       </c>
       <c r="L283" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="M283" t="inlineStr">
         <is>
@@ -25274,7 +25274,7 @@
         <v>28</v>
       </c>
       <c r="T283" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U283" t="n">
         <v>27.4</v>
@@ -25899,7 +25899,7 @@
         <v>3</v>
       </c>
       <c r="W290" t="n">
-        <v>21.74444444444444</v>
+        <v>21.74444444444445</v>
       </c>
       <c r="X290" t="n">
         <v>17.5</v>
@@ -28617,7 +28617,7 @@
         <v>3</v>
       </c>
       <c r="W321" t="n">
-        <v>27.24444444444444</v>
+        <v>27.24444444444445</v>
       </c>
       <c r="X321" t="n">
         <v>21</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>
@@ -32617,10 +32617,10 @@
         <v>21</v>
       </c>
       <c r="K367" t="n">
-        <v>22.4</v>
+        <v>23.2</v>
       </c>
       <c r="L367" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="M367" t="inlineStr">
         <is>
@@ -32648,7 +32648,7 @@
       </c>
       <c r="S367" t="inlineStr"/>
       <c r="T367" t="n">
-        <v>1.399999999999999</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U367" t="n">
         <v>21.23333333333333</v>
@@ -32789,7 +32789,7 @@
         <v>21</v>
       </c>
       <c r="K369" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="L369" t="n">
         <v>94</v>
@@ -32822,7 +32822,7 @@
         <v>21</v>
       </c>
       <c r="T369" t="n">
-        <v>-1.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U369" t="n">
         <v>20.26666666666667</v>
@@ -32877,10 +32877,10 @@
         <v>21</v>
       </c>
       <c r="K370" t="n">
-        <v>20.7</v>
+        <v>23.6</v>
       </c>
       <c r="L370" t="n">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="M370" t="inlineStr">
         <is>
@@ -32910,7 +32910,7 @@
         <v>21</v>
       </c>
       <c r="T370" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2.600000000000001</v>
       </c>
       <c r="U370" t="n">
         <v>22.76666666666667</v>
@@ -32965,10 +32965,10 @@
         <v>21</v>
       </c>
       <c r="K371" t="n">
-        <v>23.2</v>
+        <v>20</v>
       </c>
       <c r="L371" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="M371" t="inlineStr">
         <is>
@@ -32996,7 +32996,7 @@
       </c>
       <c r="S371" t="inlineStr"/>
       <c r="T371" t="n">
-        <v>2.199999999999999</v>
+        <v>-1</v>
       </c>
       <c r="U371" t="n">
         <v>22.3</v>
@@ -33051,10 +33051,10 @@
         <v>21</v>
       </c>
       <c r="K372" t="n">
-        <v>16.3</v>
+        <v>20.4</v>
       </c>
       <c r="L372" t="n">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="M372" t="inlineStr">
         <is>
@@ -33084,7 +33084,7 @@
         <v>21</v>
       </c>
       <c r="T372" t="n">
-        <v>-4.699999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U372" t="n">
         <v>19.6</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-22 16:53:49
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2899,10 +2899,10 @@
         <v>31</v>
       </c>
       <c r="K28" t="n">
-        <v>29.3</v>
+        <v>31.1</v>
       </c>
       <c r="L28" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="n">
-        <v>-1.699999999999999</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U28" t="n">
         <v>31.2</v>
@@ -5859,10 +5859,10 @@
         <v>31</v>
       </c>
       <c r="K62" t="n">
-        <v>35.8</v>
+        <v>31.4</v>
       </c>
       <c r="L62" t="n">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
@@ -5890,10 +5890,10 @@
       </c>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="n">
-        <v>4.799999999999997</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U62" t="n">
-        <v>30.66666666666667</v>
+        <v>30.66666666666666</v>
       </c>
       <c r="V62" t="n">
         <v>3</v>
@@ -6121,10 +6121,10 @@
         <v>24</v>
       </c>
       <c r="K65" t="n">
-        <v>27.2</v>
+        <v>16.6</v>
       </c>
       <c r="L65" t="n">
-        <v>113</v>
+        <v>69</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -6154,7 +6154,7 @@
         <v>28</v>
       </c>
       <c r="T65" t="n">
-        <v>3.199999999999999</v>
+        <v>-7.399999999999999</v>
       </c>
       <c r="U65" t="n">
         <v>23.4</v>
@@ -6297,10 +6297,10 @@
         <v>28</v>
       </c>
       <c r="K67" t="n">
-        <v>31.6</v>
+        <v>30.4</v>
       </c>
       <c r="L67" t="n">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -6330,7 +6330,7 @@
         <v>28</v>
       </c>
       <c r="T67" t="n">
-        <v>3.600000000000001</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U67" t="n">
         <v>29.86666666666666</v>
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L79" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7527,10 +7527,10 @@
         <v>28</v>
       </c>
       <c r="K81" t="n">
-        <v>25.9</v>
+        <v>24.8</v>
       </c>
       <c r="L81" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,10 +7560,10 @@
         <v>28</v>
       </c>
       <c r="T81" t="n">
-        <v>-2.100000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U81" t="n">
-        <v>25.13333333333333</v>
+        <v>25.13333333333334</v>
       </c>
       <c r="V81" t="n">
         <v>3</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L83" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L90" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L95" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -11913,10 +11913,10 @@
         <v>28</v>
       </c>
       <c r="K131" t="n">
-        <v>24.6</v>
+        <v>27.7</v>
       </c>
       <c r="L131" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="M131" t="inlineStr">
         <is>
@@ -11946,7 +11946,7 @@
         <v>28</v>
       </c>
       <c r="T131" t="n">
-        <v>-3.399999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U131" t="n">
         <v>25.36666666666666</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-23 20:58:23
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X375"/>
+  <dimension ref="A1:X376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22871,10 +22871,10 @@
         <v>21</v>
       </c>
       <c r="K256" t="n">
-        <v>20</v>
+        <v>22.3</v>
       </c>
       <c r="L256" t="n">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="M256" t="inlineStr">
         <is>
@@ -22904,7 +22904,7 @@
         <v>21</v>
       </c>
       <c r="T256" t="n">
-        <v>-1</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="U256" t="n">
         <v>21.8</v>
@@ -23135,10 +23135,10 @@
         <v>28</v>
       </c>
       <c r="K259" t="n">
-        <v>25.6</v>
+        <v>22.7</v>
       </c>
       <c r="L259" t="n">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="M259" t="inlineStr">
         <is>
@@ -23168,7 +23168,7 @@
         <v>28</v>
       </c>
       <c r="T259" t="n">
-        <v>-2.399999999999999</v>
+        <v>-5.300000000000001</v>
       </c>
       <c r="U259" t="n">
         <v>24.9</v>
@@ -23487,10 +23487,10 @@
         <v>28</v>
       </c>
       <c r="K263" t="n">
-        <v>28.1</v>
+        <v>28.9</v>
       </c>
       <c r="L263" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="M263" t="inlineStr">
         <is>
@@ -23520,7 +23520,7 @@
         <v>28</v>
       </c>
       <c r="T263" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U263" t="n">
         <v>28.03333333333333</v>
@@ -25945,10 +25945,10 @@
         <v>21</v>
       </c>
       <c r="K291" t="n">
-        <v>20.9</v>
+        <v>20.5</v>
       </c>
       <c r="L291" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="M291" t="inlineStr">
         <is>
@@ -25976,7 +25976,7 @@
       </c>
       <c r="S291" t="inlineStr"/>
       <c r="T291" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.5</v>
       </c>
       <c r="U291" t="n">
         <v>20.2</v>
@@ -26117,10 +26117,10 @@
         <v>21</v>
       </c>
       <c r="K293" t="n">
-        <v>21.7</v>
+        <v>22.8</v>
       </c>
       <c r="L293" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="M293" t="inlineStr">
         <is>
@@ -26150,7 +26150,7 @@
         <v>21</v>
       </c>
       <c r="T293" t="n">
-        <v>0.6999999999999993</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="U293" t="n">
         <v>21.53333333333333</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -31391,10 +31391,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>24.1</v>
+        <v>26.7</v>
       </c>
       <c r="L353" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31424,7 +31424,7 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U353" t="n">
         <v>24.9</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>
@@ -33281,7 +33281,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>SC 05</t>
+          <t>PL55</t>
         </is>
       </c>
       <c r="C375" t="inlineStr"/>
@@ -33292,17 +33292,17 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>VIGAS CIMENTACION PLACA SUPERIOR EJE 1-3 ENTRE A Y F-SC</t>
+          <t>Muro plataforma B ejes 8 al 9 F Zarpa 11 al 12 F</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>9/24/2026 12:00:00 AM</t>
+          <t>10/22/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H375" t="inlineStr"/>
@@ -33313,51 +33313,139 @@
         <v>21</v>
       </c>
       <c r="K375" t="n">
+        <v>15</v>
+      </c>
+      <c r="L375" t="n">
+        <v>72</v>
+      </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>MURO</t>
+        </is>
+      </c>
+      <c r="N375" t="n">
+        <v>21</v>
+      </c>
+      <c r="O375" t="inlineStr">
+        <is>
+          <t>MURO-21-28</t>
+        </is>
+      </c>
+      <c r="P375" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="Q375" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="R375" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="S375" t="n">
+        <v>21</v>
+      </c>
+      <c r="T375" t="n">
+        <v>-6</v>
+      </c>
+      <c r="U375" t="n">
+        <v>15.66666666666667</v>
+      </c>
+      <c r="V375" t="n">
+        <v>3</v>
+      </c>
+      <c r="W375" t="n">
+        <v>14.77777777777778</v>
+      </c>
+      <c r="X375" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>VIALE 26</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>SC 05</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr"/>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>VIGAS CIMENTACION PLACA SUPERIOR EJE 1-3 ENTRE A Y F-SC</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>9/24/2026 12:00:00 AM</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr"/>
+      <c r="I376" t="n">
+        <v>28</v>
+      </c>
+      <c r="J376" t="n">
+        <v>21</v>
+      </c>
+      <c r="K376" t="n">
         <v>19.8</v>
       </c>
-      <c r="L375" t="n">
+      <c r="L376" t="n">
         <v>94</v>
       </c>
-      <c r="M375" t="inlineStr">
+      <c r="M376" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="N375" t="n">
-        <v>21</v>
-      </c>
-      <c r="O375" t="inlineStr">
+      <c r="N376" t="n">
+        <v>21</v>
+      </c>
+      <c r="O376" t="inlineStr">
         <is>
           <t>PLACA-21-28</t>
         </is>
       </c>
-      <c r="P375" s="2" t="n">
-        <v>46318</v>
-      </c>
-      <c r="Q375" t="inlineStr">
-        <is>
-          <t>NUEVO</t>
-        </is>
-      </c>
-      <c r="R375" s="2" t="n">
-        <v>46318</v>
-      </c>
-      <c r="S375" t="n">
-        <v>21</v>
-      </c>
-      <c r="T375" t="n">
+      <c r="P376" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="Q376" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="R376" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="S376" t="n">
+        <v>21</v>
+      </c>
+      <c r="T376" t="n">
         <v>-1.199999999999999</v>
       </c>
-      <c r="U375" t="n">
+      <c r="U376" t="n">
         <v>18.9</v>
       </c>
-      <c r="V375" t="n">
-        <v>3</v>
-      </c>
-      <c r="W375" t="n">
+      <c r="V376" t="n">
+        <v>3</v>
+      </c>
+      <c r="W376" t="n">
         <v>22.93333333333334</v>
       </c>
-      <c r="X375" t="n">
+      <c r="X376" t="n">
         <v>17.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-24 00:27:01
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -606,11 +606,11 @@
         </is>
       </c>
       <c r="P2" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R2" s="2" t="n">
@@ -694,11 +694,11 @@
         </is>
       </c>
       <c r="P3" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R3" s="2" t="n">
@@ -784,11 +784,11 @@
         </is>
       </c>
       <c r="P4" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R4" s="2" t="n">
@@ -872,11 +872,11 @@
         </is>
       </c>
       <c r="P5" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R5" s="2" t="n">
@@ -962,11 +962,11 @@
         </is>
       </c>
       <c r="P6" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R6" s="2" t="n">
@@ -1052,11 +1052,11 @@
         </is>
       </c>
       <c r="P7" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R7" s="2" t="n">
@@ -1142,11 +1142,11 @@
         </is>
       </c>
       <c r="P8" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R8" s="2" t="n">
@@ -1232,11 +1232,11 @@
         </is>
       </c>
       <c r="P9" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R9" s="2" t="n">
@@ -1320,11 +1320,11 @@
         </is>
       </c>
       <c r="P10" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R10" s="2" t="n">
@@ -1408,11 +1408,11 @@
         </is>
       </c>
       <c r="P11" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R11" s="2" t="n">
@@ -1498,11 +1498,11 @@
         </is>
       </c>
       <c r="P12" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R12" s="2" t="n">
@@ -1586,11 +1586,11 @@
         </is>
       </c>
       <c r="P13" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R13" s="2" t="n">
@@ -1674,11 +1674,11 @@
         </is>
       </c>
       <c r="P14" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R14" s="2" t="n">
@@ -1762,11 +1762,11 @@
         </is>
       </c>
       <c r="P15" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R15" s="2" t="n">
@@ -1852,11 +1852,11 @@
         </is>
       </c>
       <c r="P16" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R16" s="2" t="n">
@@ -1940,11 +1940,11 @@
         </is>
       </c>
       <c r="P17" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R17" s="2" t="n">
@@ -2028,11 +2028,11 @@
         </is>
       </c>
       <c r="P18" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R18" s="2" t="n">
@@ -2118,11 +2118,11 @@
         </is>
       </c>
       <c r="P19" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R19" s="2" t="n">
@@ -2208,11 +2208,11 @@
         </is>
       </c>
       <c r="P20" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R20" s="2" t="n">
@@ -2298,11 +2298,11 @@
         </is>
       </c>
       <c r="P21" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R21" s="2" t="n">
@@ -2388,11 +2388,11 @@
         </is>
       </c>
       <c r="P22" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R22" s="2" t="n">
@@ -2478,11 +2478,11 @@
         </is>
       </c>
       <c r="P23" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R23" s="2" t="n">
@@ -2566,11 +2566,11 @@
         </is>
       </c>
       <c r="P24" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R24" s="2" t="n">
@@ -2654,11 +2654,11 @@
         </is>
       </c>
       <c r="P25" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R25" s="2" t="n">
@@ -2742,11 +2742,11 @@
         </is>
       </c>
       <c r="P26" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R26" s="2" t="n">
@@ -2828,11 +2828,11 @@
         </is>
       </c>
       <c r="P27" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R27" s="2" t="n">
@@ -2897,10 +2897,10 @@
         <v>21</v>
       </c>
       <c r="K28" t="n">
-        <v>21.5</v>
+        <v>21.2</v>
       </c>
       <c r="L28" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -2916,11 +2916,11 @@
         </is>
       </c>
       <c r="P28" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R28" s="2" t="n">
@@ -2930,7 +2930,7 @@
         <v>21</v>
       </c>
       <c r="T28" t="n">
-        <v>0.5</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U28" t="n">
         <v>21.2</v>
@@ -3004,11 +3004,11 @@
         </is>
       </c>
       <c r="P29" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R29" s="2" t="n">
@@ -3090,11 +3090,11 @@
         </is>
       </c>
       <c r="P30" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R30" s="2" t="n">
@@ -3176,11 +3176,11 @@
         </is>
       </c>
       <c r="P31" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R31" s="2" t="n">
@@ -3262,11 +3262,11 @@
         </is>
       </c>
       <c r="P32" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R32" s="2" t="n">
@@ -3348,11 +3348,11 @@
         </is>
       </c>
       <c r="P33" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R33" s="2" t="n">
@@ -3436,11 +3436,11 @@
         </is>
       </c>
       <c r="P34" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R34" s="2" t="n">
@@ -3524,11 +3524,11 @@
         </is>
       </c>
       <c r="P35" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R35" s="2" t="n">
@@ -3612,11 +3612,11 @@
         </is>
       </c>
       <c r="P36" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R36" s="2" t="n">
@@ -3700,11 +3700,11 @@
         </is>
       </c>
       <c r="P37" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R37" s="2" t="n">
@@ -3788,11 +3788,11 @@
         </is>
       </c>
       <c r="P38" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R38" s="2" t="n">
@@ -3876,11 +3876,11 @@
         </is>
       </c>
       <c r="P39" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R39" s="2" t="n">
@@ -3964,11 +3964,11 @@
         </is>
       </c>
       <c r="P40" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R40" s="2" t="n">
@@ -4052,11 +4052,11 @@
         </is>
       </c>
       <c r="P41" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R41" s="2" t="n">
@@ -4140,11 +4140,11 @@
         </is>
       </c>
       <c r="P42" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R42" s="2" t="n">
@@ -4228,11 +4228,11 @@
         </is>
       </c>
       <c r="P43" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R43" s="2" t="n">
@@ -4316,11 +4316,11 @@
         </is>
       </c>
       <c r="P44" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R44" s="2" t="n">
@@ -4385,10 +4385,10 @@
         <v>28</v>
       </c>
       <c r="K45" t="n">
-        <v>29.9</v>
+        <v>32.3</v>
       </c>
       <c r="L45" t="n">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="M45" t="inlineStr">
         <is>
@@ -4404,11 +4404,11 @@
         </is>
       </c>
       <c r="P45" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R45" s="2" t="n">
@@ -4418,7 +4418,7 @@
         <v>28</v>
       </c>
       <c r="T45" t="n">
-        <v>1.899999999999999</v>
+        <v>4.299999999999997</v>
       </c>
       <c r="U45" t="n">
         <v>28.53333333333333</v>
@@ -4490,11 +4490,11 @@
         </is>
       </c>
       <c r="P46" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R46" s="2" t="n">
@@ -4578,11 +4578,11 @@
         </is>
       </c>
       <c r="P47" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R47" s="2" t="n">
@@ -4664,11 +4664,11 @@
         </is>
       </c>
       <c r="P48" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R48" s="2" t="n">
@@ -4752,11 +4752,11 @@
         </is>
       </c>
       <c r="P49" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R49" s="2" t="n">
@@ -4840,11 +4840,11 @@
         </is>
       </c>
       <c r="P50" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R50" s="2" t="n">
@@ -4928,11 +4928,11 @@
         </is>
       </c>
       <c r="P51" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R51" s="2" t="n">
@@ -5016,11 +5016,11 @@
         </is>
       </c>
       <c r="P52" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R52" s="2" t="n">
@@ -5102,11 +5102,11 @@
         </is>
       </c>
       <c r="P53" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R53" s="2" t="n">
@@ -5190,11 +5190,11 @@
         </is>
       </c>
       <c r="P54" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R54" s="2" t="n">
@@ -5278,11 +5278,11 @@
         </is>
       </c>
       <c r="P55" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R55" s="2" t="n">
@@ -5366,11 +5366,11 @@
         </is>
       </c>
       <c r="P56" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R56" s="2" t="n">
@@ -5454,11 +5454,11 @@
         </is>
       </c>
       <c r="P57" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R57" s="2" t="n">
@@ -5542,11 +5542,11 @@
         </is>
       </c>
       <c r="P58" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R58" s="2" t="n">
@@ -5630,11 +5630,11 @@
         </is>
       </c>
       <c r="P59" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R59" s="2" t="n">
@@ -5718,11 +5718,11 @@
         </is>
       </c>
       <c r="P60" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R60" s="2" t="n">
@@ -5806,11 +5806,11 @@
         </is>
       </c>
       <c r="P61" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R61" s="2" t="n">
@@ -5894,11 +5894,11 @@
         </is>
       </c>
       <c r="P62" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R62" s="2" t="n">
@@ -5982,11 +5982,11 @@
         </is>
       </c>
       <c r="P63" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R63" s="2" t="n">
@@ -6070,11 +6070,11 @@
         </is>
       </c>
       <c r="P64" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R64" s="2" t="n">
@@ -6158,11 +6158,11 @@
         </is>
       </c>
       <c r="P65" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R65" s="2" t="n">
@@ -6246,11 +6246,11 @@
         </is>
       </c>
       <c r="P66" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R66" s="2" t="n">
@@ -6334,11 +6334,11 @@
         </is>
       </c>
       <c r="P67" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R67" s="2" t="n">
@@ -6422,11 +6422,11 @@
         </is>
       </c>
       <c r="P68" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R68" s="2" t="n">
@@ -6506,11 +6506,11 @@
         </is>
       </c>
       <c r="P69" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R69" s="2" t="n">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="P70" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R70" s="2" t="n">
@@ -6682,11 +6682,11 @@
         </is>
       </c>
       <c r="P71" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R71" s="2" t="n">
@@ -6770,11 +6770,11 @@
         </is>
       </c>
       <c r="P72" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R72" s="2" t="n">
@@ -6858,11 +6858,11 @@
         </is>
       </c>
       <c r="P73" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R73" s="2" t="n">
@@ -6946,11 +6946,11 @@
         </is>
       </c>
       <c r="P74" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R74" s="2" t="n">
@@ -7034,11 +7034,11 @@
         </is>
       </c>
       <c r="P75" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R75" s="2" t="n">
@@ -7120,11 +7120,11 @@
         </is>
       </c>
       <c r="P76" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R76" s="2" t="n">
@@ -7208,11 +7208,11 @@
         </is>
       </c>
       <c r="P77" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R77" s="2" t="n">
@@ -7296,11 +7296,11 @@
         </is>
       </c>
       <c r="P78" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R78" s="2" t="n">
@@ -7384,11 +7384,11 @@
         </is>
       </c>
       <c r="P79" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R79" s="2" t="n">
@@ -7470,11 +7470,11 @@
         </is>
       </c>
       <c r="P80" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R80" s="2" t="n">
@@ -7558,11 +7558,11 @@
         </is>
       </c>
       <c r="P81" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R81" s="2" t="n">
@@ -7646,11 +7646,11 @@
         </is>
       </c>
       <c r="P82" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R82" s="2" t="n">
@@ -7734,11 +7734,11 @@
         </is>
       </c>
       <c r="P83" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R83" s="2" t="n">
@@ -7822,11 +7822,11 @@
         </is>
       </c>
       <c r="P84" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R84" s="2" t="n">
@@ -7910,11 +7910,11 @@
         </is>
       </c>
       <c r="P85" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R85" s="2" t="n">
@@ -7998,11 +7998,11 @@
         </is>
       </c>
       <c r="P86" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R86" s="2" t="n">
@@ -8086,11 +8086,11 @@
         </is>
       </c>
       <c r="P87" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R87" s="2" t="n">
@@ -8174,11 +8174,11 @@
         </is>
       </c>
       <c r="P88" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R88" s="2" t="n">
@@ -8262,11 +8262,11 @@
         </is>
       </c>
       <c r="P89" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R89" s="2" t="n">
@@ -8348,11 +8348,11 @@
         </is>
       </c>
       <c r="P90" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R90" s="2" t="n">
@@ -8436,11 +8436,11 @@
         </is>
       </c>
       <c r="P91" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R91" s="2" t="n">
@@ -8524,11 +8524,11 @@
         </is>
       </c>
       <c r="P92" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R92" s="2" t="n">
@@ -8612,11 +8612,11 @@
         </is>
       </c>
       <c r="P93" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R93" s="2" t="n">
@@ -8700,11 +8700,11 @@
         </is>
       </c>
       <c r="P94" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R94" s="2" t="n">
@@ -8788,11 +8788,11 @@
         </is>
       </c>
       <c r="P95" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R95" s="2" t="n">
@@ -8876,11 +8876,11 @@
         </is>
       </c>
       <c r="P96" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R96" s="2" t="n">
@@ -8964,11 +8964,11 @@
         </is>
       </c>
       <c r="P97" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R97" s="2" t="n">
@@ -9033,10 +9033,10 @@
         <v>24.5</v>
       </c>
       <c r="K98" t="n">
-        <v>24.6</v>
+        <v>26.4</v>
       </c>
       <c r="L98" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="M98" t="inlineStr">
         <is>
@@ -9052,11 +9052,11 @@
         </is>
       </c>
       <c r="P98" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R98" s="2" t="n">
@@ -9066,7 +9066,7 @@
         <v>28</v>
       </c>
       <c r="T98" t="n">
-        <v>0.1000000000000014</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U98" t="n">
         <v>23.96666666666667</v>
@@ -9140,11 +9140,11 @@
         </is>
       </c>
       <c r="P99" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R99" s="2" t="n">
@@ -9228,11 +9228,11 @@
         </is>
       </c>
       <c r="P100" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R100" s="2" t="n">
@@ -9316,11 +9316,11 @@
         </is>
       </c>
       <c r="P101" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R101" s="2" t="n">
@@ -9404,11 +9404,11 @@
         </is>
       </c>
       <c r="P102" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R102" s="2" t="n">
@@ -9492,11 +9492,11 @@
         </is>
       </c>
       <c r="P103" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R103" s="2" t="n">
@@ -9580,11 +9580,11 @@
         </is>
       </c>
       <c r="P104" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R104" s="2" t="n">
@@ -9668,11 +9668,11 @@
         </is>
       </c>
       <c r="P105" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R105" s="2" t="n">
@@ -9756,11 +9756,11 @@
         </is>
       </c>
       <c r="P106" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R106" s="2" t="n">
@@ -9844,11 +9844,11 @@
         </is>
       </c>
       <c r="P107" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R107" s="2" t="n">
@@ -9932,11 +9932,11 @@
         </is>
       </c>
       <c r="P108" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R108" s="2" t="n">
@@ -10020,11 +10020,11 @@
         </is>
       </c>
       <c r="P109" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R109" s="2" t="n">
@@ -10108,11 +10108,11 @@
         </is>
       </c>
       <c r="P110" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R110" s="2" t="n">
@@ -10196,11 +10196,11 @@
         </is>
       </c>
       <c r="P111" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R111" s="2" t="n">
@@ -10284,11 +10284,11 @@
         </is>
       </c>
       <c r="P112" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R112" s="2" t="n">
@@ -10372,11 +10372,11 @@
         </is>
       </c>
       <c r="P113" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R113" s="2" t="n">
@@ -10460,11 +10460,11 @@
         </is>
       </c>
       <c r="P114" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R114" s="2" t="n">
@@ -10548,11 +10548,11 @@
         </is>
       </c>
       <c r="P115" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R115" s="2" t="n">
@@ -10636,11 +10636,11 @@
         </is>
       </c>
       <c r="P116" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R116" s="2" t="n">
@@ -10724,11 +10724,11 @@
         </is>
       </c>
       <c r="P117" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R117" s="2" t="n">
@@ -10812,11 +10812,11 @@
         </is>
       </c>
       <c r="P118" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R118" s="2" t="n">
@@ -10900,11 +10900,11 @@
         </is>
       </c>
       <c r="P119" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R119" s="2" t="n">
@@ -10988,11 +10988,11 @@
         </is>
       </c>
       <c r="P120" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R120" s="2" t="n">
@@ -11076,11 +11076,11 @@
         </is>
       </c>
       <c r="P121" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R121" s="2" t="n">
@@ -11164,11 +11164,11 @@
         </is>
       </c>
       <c r="P122" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R122" s="2" t="n">
@@ -11252,11 +11252,11 @@
         </is>
       </c>
       <c r="P123" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R123" s="2" t="n">
@@ -11340,11 +11340,11 @@
         </is>
       </c>
       <c r="P124" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R124" s="2" t="n">
@@ -11428,11 +11428,11 @@
         </is>
       </c>
       <c r="P125" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R125" s="2" t="n">
@@ -11516,11 +11516,11 @@
         </is>
       </c>
       <c r="P126" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R126" s="2" t="n">
@@ -11604,11 +11604,11 @@
         </is>
       </c>
       <c r="P127" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R127" s="2" t="n">
@@ -11692,11 +11692,11 @@
         </is>
       </c>
       <c r="P128" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R128" s="2" t="n">
@@ -11780,11 +11780,11 @@
         </is>
       </c>
       <c r="P129" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R129" s="2" t="n">
@@ -11868,11 +11868,11 @@
         </is>
       </c>
       <c r="P130" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R130" s="2" t="n">
@@ -11956,11 +11956,11 @@
         </is>
       </c>
       <c r="P131" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R131" s="2" t="n">
@@ -12044,11 +12044,11 @@
         </is>
       </c>
       <c r="P132" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R132" s="2" t="n">
@@ -12130,11 +12130,11 @@
         </is>
       </c>
       <c r="P133" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R133" s="2" t="n">
@@ -12218,11 +12218,11 @@
         </is>
       </c>
       <c r="P134" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R134" s="2" t="n">
@@ -12306,11 +12306,11 @@
         </is>
       </c>
       <c r="P135" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R135" s="2" t="n">
@@ -12394,11 +12394,11 @@
         </is>
       </c>
       <c r="P136" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R136" s="2" t="n">
@@ -12482,11 +12482,11 @@
         </is>
       </c>
       <c r="P137" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R137" s="2" t="n">
@@ -12570,11 +12570,11 @@
         </is>
       </c>
       <c r="P138" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R138" s="2" t="n">
@@ -12639,10 +12639,10 @@
         <v>24.5</v>
       </c>
       <c r="K139" t="n">
-        <v>29.1</v>
+        <v>22.7</v>
       </c>
       <c r="L139" t="n">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="M139" t="inlineStr">
         <is>
@@ -12658,11 +12658,11 @@
         </is>
       </c>
       <c r="P139" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R139" s="2" t="n">
@@ -12672,7 +12672,7 @@
         <v>28</v>
       </c>
       <c r="T139" t="n">
-        <v>4.600000000000001</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="U139" t="n">
         <v>25.3</v>
@@ -12744,11 +12744,11 @@
         </is>
       </c>
       <c r="P140" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R140" s="2" t="n">
@@ -12832,11 +12832,11 @@
         </is>
       </c>
       <c r="P141" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R141" s="2" t="n">
@@ -12920,11 +12920,11 @@
         </is>
       </c>
       <c r="P142" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R142" s="2" t="n">
@@ -12987,10 +12987,10 @@
         <v>21</v>
       </c>
       <c r="K143" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="L143" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M143" t="inlineStr">
         <is>
@@ -13006,11 +13006,11 @@
         </is>
       </c>
       <c r="P143" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R143" s="2" t="n">
@@ -13020,7 +13020,7 @@
         <v>21</v>
       </c>
       <c r="T143" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U143" t="n">
         <v>20.9</v>
@@ -13094,11 +13094,11 @@
         </is>
       </c>
       <c r="P144" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R144" s="2" t="n">
@@ -13178,11 +13178,11 @@
         </is>
       </c>
       <c r="P145" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R145" s="2" t="n">
@@ -13266,11 +13266,11 @@
         </is>
       </c>
       <c r="P146" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R146" s="2" t="n">
@@ -13354,11 +13354,11 @@
         </is>
       </c>
       <c r="P147" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R147" s="2" t="n">
@@ -13442,11 +13442,11 @@
         </is>
       </c>
       <c r="P148" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R148" s="2" t="n">
@@ -13528,11 +13528,11 @@
         </is>
       </c>
       <c r="P149" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R149" s="2" t="n">
@@ -13616,11 +13616,11 @@
         </is>
       </c>
       <c r="P150" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R150" s="2" t="n">
@@ -13702,11 +13702,11 @@
         </is>
       </c>
       <c r="P151" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R151" s="2" t="n">
@@ -13790,11 +13790,11 @@
         </is>
       </c>
       <c r="P152" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R152" s="2" t="n">
@@ -13878,11 +13878,11 @@
         </is>
       </c>
       <c r="P153" s="2" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>NUEVO</t>
+          <t>EXISTENTE</t>
         </is>
       </c>
       <c r="R153" s="2" t="n">

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-24 06:58:24
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L79" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L83" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L90" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L95" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -10769,10 +10769,10 @@
         <v>28</v>
       </c>
       <c r="K118" t="n">
-        <v>29.7</v>
+        <v>32.7</v>
       </c>
       <c r="L118" t="n">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -10802,7 +10802,7 @@
         <v>28</v>
       </c>
       <c r="T118" t="n">
-        <v>1.699999999999999</v>
+        <v>4.700000000000003</v>
       </c>
       <c r="U118" t="n">
         <v>29.6</v>
@@ -13319,10 +13319,10 @@
         <v>35</v>
       </c>
       <c r="K147" t="n">
-        <v>46</v>
+        <v>37.5</v>
       </c>
       <c r="L147" t="n">
-        <v>131</v>
+        <v>107</v>
       </c>
       <c r="M147" t="inlineStr">
         <is>
@@ -13352,7 +13352,7 @@
         <v>41</v>
       </c>
       <c r="T147" t="n">
-        <v>11</v>
+        <v>2.5</v>
       </c>
       <c r="U147" t="n">
         <v>38.3</v>
@@ -21391,10 +21391,10 @@
         <v>31</v>
       </c>
       <c r="K239" t="n">
-        <v>31.5</v>
+        <v>28.1</v>
       </c>
       <c r="L239" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M239" t="inlineStr">
         <is>
@@ -21422,7 +21422,7 @@
       </c>
       <c r="S239" t="inlineStr"/>
       <c r="T239" t="n">
-        <v>0.5</v>
+        <v>-2.899999999999999</v>
       </c>
       <c r="U239" t="n">
         <v>30.6</v>
@@ -24405,7 +24405,7 @@
         <v>3</v>
       </c>
       <c r="W273" t="n">
-        <v>28.15555555555555</v>
+        <v>28.15555555555556</v>
       </c>
       <c r="X273" t="n">
         <v>24.5</v>
@@ -25153,10 +25153,10 @@
         <v>28</v>
       </c>
       <c r="K282" t="n">
-        <v>29</v>
+        <v>28.2</v>
       </c>
       <c r="L282" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="M282" t="inlineStr">
         <is>
@@ -25186,7 +25186,7 @@
         <v>28</v>
       </c>
       <c r="T282" t="n">
-        <v>1</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U282" t="n">
         <v>28.2</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -29761,7 +29761,7 @@
         <v>3</v>
       </c>
       <c r="W334" t="n">
-        <v>25.57777777777778</v>
+        <v>25.57777777777777</v>
       </c>
       <c r="X334" t="n">
         <v>21</v>
@@ -29895,10 +29895,10 @@
         <v>24.5</v>
       </c>
       <c r="K336" t="n">
-        <v>21</v>
+        <v>26.9</v>
       </c>
       <c r="L336" t="n">
-        <v>86</v>
+        <v>110</v>
       </c>
       <c r="M336" t="inlineStr">
         <is>
@@ -29928,7 +29928,7 @@
         <v>28</v>
       </c>
       <c r="T336" t="n">
-        <v>-3.5</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U336" t="n">
         <v>24.26666666666667</v>
@@ -31127,10 +31127,10 @@
         <v>24.5</v>
       </c>
       <c r="K350" t="n">
-        <v>36.1</v>
+        <v>23.4</v>
       </c>
       <c r="L350" t="n">
-        <v>147</v>
+        <v>95</v>
       </c>
       <c r="M350" t="inlineStr">
         <is>
@@ -31160,7 +31160,7 @@
         <v>28</v>
       </c>
       <c r="T350" t="n">
-        <v>11.6</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U350" t="n">
         <v>29.46666666666667</v>
@@ -31215,10 +31215,10 @@
         <v>24.5</v>
       </c>
       <c r="K351" t="n">
-        <v>26.2</v>
+        <v>23.4</v>
       </c>
       <c r="L351" t="n">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="M351" t="inlineStr">
         <is>
@@ -31248,7 +31248,7 @@
         <v>28</v>
       </c>
       <c r="T351" t="n">
-        <v>1.699999999999999</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U351" t="n">
         <v>24.5</v>
@@ -31303,10 +31303,10 @@
         <v>24.5</v>
       </c>
       <c r="K352" t="n">
-        <v>23.2</v>
+        <v>23.6</v>
       </c>
       <c r="L352" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M352" t="inlineStr">
         <is>
@@ -31336,7 +31336,7 @@
         <v>28</v>
       </c>
       <c r="T352" t="n">
-        <v>-1.300000000000001</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U352" t="n">
         <v>22.63333333333334</v>
@@ -31391,10 +31391,10 @@
         <v>24.5</v>
       </c>
       <c r="K353" t="n">
-        <v>24.1</v>
+        <v>26.7</v>
       </c>
       <c r="L353" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="M353" t="inlineStr">
         <is>
@@ -31424,7 +31424,7 @@
         <v>28</v>
       </c>
       <c r="T353" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U353" t="n">
         <v>24.9</v>
@@ -31479,10 +31479,10 @@
         <v>24.5</v>
       </c>
       <c r="K354" t="n">
-        <v>22.9</v>
+        <v>27.8</v>
       </c>
       <c r="L354" t="n">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="M354" t="inlineStr">
         <is>
@@ -31512,7 +31512,7 @@
         <v>28</v>
       </c>
       <c r="T354" t="n">
-        <v>-1.600000000000001</v>
+        <v>3.300000000000001</v>
       </c>
       <c r="U354" t="n">
         <v>25</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>
@@ -31653,10 +31653,10 @@
         <v>24.5</v>
       </c>
       <c r="K356" t="n">
-        <v>23.7</v>
+        <v>28.8</v>
       </c>
       <c r="L356" t="n">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="M356" t="inlineStr">
         <is>
@@ -31686,7 +31686,7 @@
         <v>28</v>
       </c>
       <c r="T356" t="n">
-        <v>-0.8000000000000007</v>
+        <v>4.300000000000001</v>
       </c>
       <c r="U356" t="n">
         <v>25.6</v>
@@ -31741,10 +31741,10 @@
         <v>24.5</v>
       </c>
       <c r="K357" t="n">
-        <v>24.1</v>
+        <v>28.5</v>
       </c>
       <c r="L357" t="n">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="M357" t="inlineStr">
         <is>
@@ -31774,7 +31774,7 @@
         <v>28</v>
       </c>
       <c r="T357" t="n">
-        <v>-0.3999999999999986</v>
+        <v>4</v>
       </c>
       <c r="U357" t="n">
         <v>28.1</v>
@@ -31829,10 +31829,10 @@
         <v>24.5</v>
       </c>
       <c r="K358" t="n">
-        <v>26.3</v>
+        <v>22.7</v>
       </c>
       <c r="L358" t="n">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="M358" t="inlineStr">
         <is>
@@ -31862,7 +31862,7 @@
         <v>28</v>
       </c>
       <c r="T358" t="n">
-        <v>1.800000000000001</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="U358" t="n">
         <v>24.76666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-24 15:30:09
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5249,10 +5249,10 @@
         <v>31</v>
       </c>
       <c r="K55" t="n">
-        <v>34.5</v>
+        <v>31.6</v>
       </c>
       <c r="L55" t="n">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="n">
-        <v>3.5</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U55" t="n">
         <v>31.46666666666667</v>
@@ -6075,7 +6075,7 @@
         <v>3</v>
       </c>
       <c r="W64" t="n">
-        <v>24.52222222222222</v>
+        <v>24.52222222222223</v>
       </c>
       <c r="X64" t="n">
         <v>20.5</v>
@@ -6121,10 +6121,10 @@
         <v>24</v>
       </c>
       <c r="K65" t="n">
-        <v>16.6</v>
+        <v>26.4</v>
       </c>
       <c r="L65" t="n">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -6154,7 +6154,7 @@
         <v>28</v>
       </c>
       <c r="T65" t="n">
-        <v>-7.399999999999999</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U65" t="n">
         <v>23.4</v>
@@ -6163,7 +6163,7 @@
         <v>3</v>
       </c>
       <c r="W65" t="n">
-        <v>24.64444444444444</v>
+        <v>24.64444444444445</v>
       </c>
       <c r="X65" t="n">
         <v>20.5</v>
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L79" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7527,10 +7527,10 @@
         <v>28</v>
       </c>
       <c r="K81" t="n">
-        <v>24.8</v>
+        <v>25.9</v>
       </c>
       <c r="L81" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,10 +7560,10 @@
         <v>28</v>
       </c>
       <c r="T81" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U81" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="V81" t="n">
         <v>3</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L83" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L90" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L95" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -23751,10 +23751,10 @@
         <v>28</v>
       </c>
       <c r="K266" t="n">
-        <v>24.7</v>
+        <v>32.5</v>
       </c>
       <c r="L266" t="n">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="M266" t="inlineStr">
         <is>
@@ -23784,7 +23784,7 @@
         <v>28</v>
       </c>
       <c r="T266" t="n">
-        <v>-3.300000000000001</v>
+        <v>4.5</v>
       </c>
       <c r="U266" t="n">
         <v>29.5</v>
@@ -26381,10 +26381,10 @@
         <v>21</v>
       </c>
       <c r="K296" t="n">
-        <v>20.4</v>
+        <v>20.8</v>
       </c>
       <c r="L296" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M296" t="inlineStr">
         <is>
@@ -26414,7 +26414,7 @@
         <v>21</v>
       </c>
       <c r="T296" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U296" t="n">
         <v>20.76666666666667</v>
@@ -27959,10 +27959,10 @@
         <v>24.5</v>
       </c>
       <c r="K314" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="L314" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="M314" t="inlineStr">
         <is>
@@ -27992,7 +27992,7 @@
         <v>28</v>
       </c>
       <c r="T314" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U314" t="n">
         <v>25.13333333333334</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L325" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L333" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L355" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>
@@ -31741,10 +31741,10 @@
         <v>24.5</v>
       </c>
       <c r="K357" t="n">
-        <v>28.5</v>
+        <v>31.7</v>
       </c>
       <c r="L357" t="n">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="M357" t="inlineStr">
         <is>
@@ -31774,7 +31774,7 @@
         <v>28</v>
       </c>
       <c r="T357" t="n">
-        <v>4</v>
+        <v>7.199999999999999</v>
       </c>
       <c r="U357" t="n">
         <v>28.1</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-24 17:30:45
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -5249,10 +5249,10 @@
         <v>31</v>
       </c>
       <c r="K55" t="n">
-        <v>31.6</v>
+        <v>34.5</v>
       </c>
       <c r="L55" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="n">
-        <v>0.6000000000000014</v>
+        <v>3.5</v>
       </c>
       <c r="U55" t="n">
         <v>31.46666666666667</v>
@@ -6075,7 +6075,7 @@
         <v>3</v>
       </c>
       <c r="W64" t="n">
-        <v>24.52222222222223</v>
+        <v>24.52222222222222</v>
       </c>
       <c r="X64" t="n">
         <v>20.5</v>
@@ -6121,10 +6121,10 @@
         <v>24</v>
       </c>
       <c r="K65" t="n">
-        <v>26.4</v>
+        <v>16.6</v>
       </c>
       <c r="L65" t="n">
-        <v>110</v>
+        <v>69</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -6154,7 +6154,7 @@
         <v>28</v>
       </c>
       <c r="T65" t="n">
-        <v>2.399999999999999</v>
+        <v>-7.399999999999999</v>
       </c>
       <c r="U65" t="n">
         <v>23.4</v>
@@ -6163,7 +6163,7 @@
         <v>3</v>
       </c>
       <c r="W65" t="n">
-        <v>24.64444444444445</v>
+        <v>24.64444444444444</v>
       </c>
       <c r="X65" t="n">
         <v>20.5</v>
@@ -7527,10 +7527,10 @@
         <v>28</v>
       </c>
       <c r="K81" t="n">
-        <v>25.9</v>
+        <v>24.8</v>
       </c>
       <c r="L81" t="n">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,10 +7560,10 @@
         <v>28</v>
       </c>
       <c r="T81" t="n">
-        <v>-2.100000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U81" t="n">
-        <v>25.13333333333333</v>
+        <v>25.13333333333334</v>
       </c>
       <c r="V81" t="n">
         <v>3</v>
@@ -15245,10 +15245,10 @@
         <v>21</v>
       </c>
       <c r="K169" t="n">
-        <v>25.1</v>
+        <v>20.4</v>
       </c>
       <c r="L169" t="n">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="M169" t="inlineStr">
         <is>
@@ -15278,7 +15278,7 @@
         <v>21</v>
       </c>
       <c r="T169" t="n">
-        <v>4.100000000000001</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U169" t="n">
         <v>24.33333333333333</v>
@@ -15333,10 +15333,10 @@
         <v>35</v>
       </c>
       <c r="K170" t="n">
-        <v>34.7</v>
+        <v>37.2</v>
       </c>
       <c r="L170" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="M170" t="inlineStr">
         <is>
@@ -15366,7 +15366,7 @@
         <v>41</v>
       </c>
       <c r="T170" t="n">
-        <v>-0.2999999999999972</v>
+        <v>2.200000000000003</v>
       </c>
       <c r="U170" t="n">
         <v>37.26666666666667</v>
@@ -15421,10 +15421,10 @@
         <v>21</v>
       </c>
       <c r="K171" t="n">
-        <v>20.8</v>
+        <v>23.4</v>
       </c>
       <c r="L171" t="n">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="M171" t="inlineStr">
         <is>
@@ -15454,7 +15454,7 @@
         <v>21</v>
       </c>
       <c r="T171" t="n">
-        <v>-0.1999999999999993</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U171" t="n">
         <v>23.4</v>
@@ -15685,10 +15685,10 @@
         <v>28</v>
       </c>
       <c r="K174" t="n">
-        <v>27</v>
+        <v>24.8</v>
       </c>
       <c r="L174" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="M174" t="inlineStr">
         <is>
@@ -15718,7 +15718,7 @@
         <v>28</v>
       </c>
       <c r="T174" t="n">
-        <v>-1</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U174" t="n">
         <v>26.4</v>
@@ -16651,10 +16651,10 @@
         <v>28</v>
       </c>
       <c r="K185" t="n">
-        <v>36.4</v>
+        <v>40.2</v>
       </c>
       <c r="L185" t="n">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="M185" t="inlineStr">
         <is>
@@ -16684,7 +16684,7 @@
         <v>28</v>
       </c>
       <c r="T185" t="n">
-        <v>8.399999999999999</v>
+        <v>12.2</v>
       </c>
       <c r="U185" t="n">
         <v>33.36666666666667</v>
@@ -16739,10 +16739,10 @@
         <v>21</v>
       </c>
       <c r="K186" t="n">
-        <v>20.7</v>
+        <v>20.9</v>
       </c>
       <c r="L186" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M186" t="inlineStr">
         <is>
@@ -16772,7 +16772,7 @@
         <v>21</v>
       </c>
       <c r="T186" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U186" t="n">
         <v>21.3</v>
@@ -16827,10 +16827,10 @@
         <v>28</v>
       </c>
       <c r="K187" t="n">
-        <v>27.6</v>
+        <v>28.5</v>
       </c>
       <c r="L187" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M187" t="inlineStr">
         <is>
@@ -16860,7 +16860,7 @@
         <v>28</v>
       </c>
       <c r="T187" t="n">
-        <v>-0.3999999999999986</v>
+        <v>0.5</v>
       </c>
       <c r="U187" t="n">
         <v>27.5</v>
@@ -16915,10 +16915,10 @@
         <v>28</v>
       </c>
       <c r="K188" t="n">
-        <v>30.3</v>
+        <v>24</v>
       </c>
       <c r="L188" t="n">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="M188" t="inlineStr">
         <is>
@@ -16948,7 +16948,7 @@
         <v>28</v>
       </c>
       <c r="T188" t="n">
-        <v>2.300000000000001</v>
+        <v>-4</v>
       </c>
       <c r="U188" t="n">
         <v>27.23333333333333</v>
@@ -17003,10 +17003,10 @@
         <v>28</v>
       </c>
       <c r="K189" t="n">
-        <v>30.4</v>
+        <v>28.6</v>
       </c>
       <c r="L189" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="M189" t="inlineStr">
         <is>
@@ -17036,7 +17036,7 @@
         <v>28</v>
       </c>
       <c r="T189" t="n">
-        <v>2.399999999999999</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U189" t="n">
         <v>28.83333333333333</v>
@@ -17091,10 +17091,10 @@
         <v>35</v>
       </c>
       <c r="K190" t="n">
-        <v>32.7</v>
+        <v>32.4</v>
       </c>
       <c r="L190" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M190" t="inlineStr">
         <is>
@@ -17124,7 +17124,7 @@
         <v>41</v>
       </c>
       <c r="T190" t="n">
-        <v>-2.299999999999997</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U190" t="n">
         <v>32.26666666666667</v>
@@ -23751,10 +23751,10 @@
         <v>28</v>
       </c>
       <c r="K266" t="n">
-        <v>32.5</v>
+        <v>24.7</v>
       </c>
       <c r="L266" t="n">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="M266" t="inlineStr">
         <is>
@@ -23784,7 +23784,7 @@
         <v>28</v>
       </c>
       <c r="T266" t="n">
-        <v>4.5</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="U266" t="n">
         <v>29.5</v>
@@ -26381,10 +26381,10 @@
         <v>21</v>
       </c>
       <c r="K296" t="n">
-        <v>20.8</v>
+        <v>20.4</v>
       </c>
       <c r="L296" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="M296" t="inlineStr">
         <is>
@@ -26414,7 +26414,7 @@
         <v>21</v>
       </c>
       <c r="T296" t="n">
-        <v>-0.1999999999999993</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U296" t="n">
         <v>20.76666666666667</v>
@@ -27959,10 +27959,10 @@
         <v>24.5</v>
       </c>
       <c r="K314" t="n">
-        <v>23.9</v>
+        <v>25.1</v>
       </c>
       <c r="L314" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="M314" t="inlineStr">
         <is>
@@ -27992,7 +27992,7 @@
         <v>28</v>
       </c>
       <c r="T314" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U314" t="n">
         <v>25.13333333333334</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>
@@ -31741,10 +31741,10 @@
         <v>24.5</v>
       </c>
       <c r="K357" t="n">
-        <v>31.7</v>
+        <v>28.5</v>
       </c>
       <c r="L357" t="n">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="M357" t="inlineStr">
         <is>
@@ -31774,7 +31774,7 @@
         <v>28</v>
       </c>
       <c r="T357" t="n">
-        <v>7.199999999999999</v>
+        <v>4</v>
       </c>
       <c r="U357" t="n">
         <v>28.1</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-24 22:20:24
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2985,10 +2985,10 @@
         <v>31</v>
       </c>
       <c r="K29" t="n">
-        <v>16.6</v>
+        <v>32.1</v>
       </c>
       <c r="L29" t="n">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="n">
-        <v>-14.4</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U29" t="n">
         <v>25.6</v>
@@ -5249,10 +5249,10 @@
         <v>31</v>
       </c>
       <c r="K55" t="n">
-        <v>34.5</v>
+        <v>28.3</v>
       </c>
       <c r="L55" t="n">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="n">
-        <v>3.5</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="U55" t="n">
         <v>31.46666666666667</v>
@@ -8229,10 +8229,10 @@
         <v>21</v>
       </c>
       <c r="K89" t="n">
-        <v>19.3</v>
+        <v>26</v>
       </c>
       <c r="L89" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="M89" t="inlineStr">
         <is>
@@ -8262,7 +8262,7 @@
         <v>21</v>
       </c>
       <c r="T89" t="n">
-        <v>-1.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="U89" t="n">
         <v>22</v>
@@ -13669,10 +13669,10 @@
         <v>35</v>
       </c>
       <c r="K151" t="n">
-        <v>34.4</v>
+        <v>36.9</v>
       </c>
       <c r="L151" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="M151" t="inlineStr">
         <is>
@@ -13702,7 +13702,7 @@
         <v>41</v>
       </c>
       <c r="T151" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U151" t="n">
         <v>35.53333333333333</v>
@@ -14809,10 +14809,10 @@
         <v>28</v>
       </c>
       <c r="K164" t="n">
-        <v>29.4</v>
+        <v>31.6</v>
       </c>
       <c r="L164" t="n">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="M164" t="inlineStr">
         <is>
@@ -14842,7 +14842,7 @@
         <v>28</v>
       </c>
       <c r="T164" t="n">
-        <v>1.399999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U164" t="n">
         <v>28.43333333333334</v>
@@ -22179,10 +22179,10 @@
         <v>21</v>
       </c>
       <c r="K248" t="n">
-        <v>19</v>
+        <v>17.3</v>
       </c>
       <c r="L248" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="M248" t="inlineStr">
         <is>
@@ -22210,7 +22210,7 @@
       </c>
       <c r="S248" t="inlineStr"/>
       <c r="T248" t="n">
-        <v>-2</v>
+        <v>-3.699999999999999</v>
       </c>
       <c r="U248" t="n">
         <v>19.3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-25 07:22:37
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3503,10 +3503,10 @@
         <v>28</v>
       </c>
       <c r="K35" t="n">
-        <v>33.2</v>
+        <v>22.1</v>
       </c>
       <c r="L35" t="n">
-        <v>118</v>
+        <v>79</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
         <v>28</v>
       </c>
       <c r="T35" t="n">
-        <v>5.200000000000003</v>
+        <v>-5.899999999999999</v>
       </c>
       <c r="U35" t="n">
         <v>30.1</v>
@@ -3591,10 +3591,10 @@
         <v>31</v>
       </c>
       <c r="K36" t="n">
-        <v>30.9</v>
+        <v>32.6</v>
       </c>
       <c r="L36" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U36" t="n">
         <v>30.8</v>
@@ -3631,7 +3631,7 @@
         <v>3</v>
       </c>
       <c r="W36" t="n">
-        <v>41.12222222222222</v>
+        <v>41.12222222222223</v>
       </c>
       <c r="X36" t="n">
         <v>27.5</v>
@@ -3677,10 +3677,10 @@
         <v>28</v>
       </c>
       <c r="K37" t="n">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="L37" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -3710,7 +3710,7 @@
         <v>28</v>
       </c>
       <c r="T37" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="U37" t="n">
         <v>30.53333333333333</v>
@@ -3765,10 +3765,10 @@
         <v>28</v>
       </c>
       <c r="K38" t="n">
-        <v>24.9</v>
+        <v>32.4</v>
       </c>
       <c r="L38" t="n">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
@@ -3798,7 +3798,7 @@
         <v>28</v>
       </c>
       <c r="T38" t="n">
-        <v>-3.100000000000001</v>
+        <v>4.399999999999999</v>
       </c>
       <c r="U38" t="n">
         <v>31.5</v>
@@ -3939,10 +3939,10 @@
         <v>28</v>
       </c>
       <c r="K40" t="n">
-        <v>36.9</v>
+        <v>31.9</v>
       </c>
       <c r="L40" t="n">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
@@ -3972,7 +3972,7 @@
         <v>28</v>
       </c>
       <c r="T40" t="n">
-        <v>8.899999999999999</v>
+        <v>3.899999999999999</v>
       </c>
       <c r="U40" t="n">
         <v>32.16666666666666</v>
@@ -4027,10 +4027,10 @@
         <v>31</v>
       </c>
       <c r="K41" t="n">
-        <v>25.8</v>
+        <v>38.1</v>
       </c>
       <c r="L41" t="n">
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="n">
-        <v>-5.199999999999999</v>
+        <v>7.100000000000001</v>
       </c>
       <c r="U41" t="n">
         <v>34.63333333333333</v>
@@ -6297,10 +6297,10 @@
         <v>28</v>
       </c>
       <c r="K67" t="n">
-        <v>30.4</v>
+        <v>31.6</v>
       </c>
       <c r="L67" t="n">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="M67" t="inlineStr">
         <is>
@@ -6330,7 +6330,7 @@
         <v>28</v>
       </c>
       <c r="T67" t="n">
-        <v>2.399999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U67" t="n">
         <v>29.86666666666666</v>
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L79" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7527,10 +7527,10 @@
         <v>28</v>
       </c>
       <c r="K81" t="n">
-        <v>24.8</v>
+        <v>25.9</v>
       </c>
       <c r="L81" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="M81" t="inlineStr">
         <is>
@@ -7560,10 +7560,10 @@
         <v>28</v>
       </c>
       <c r="T81" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U81" t="n">
-        <v>25.13333333333334</v>
+        <v>25.13333333333333</v>
       </c>
       <c r="V81" t="n">
         <v>3</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L83" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L90" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L95" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -9497,7 +9497,7 @@
         <v>3</v>
       </c>
       <c r="W103" t="n">
-        <v>26.17777777777778</v>
+        <v>26.17777777777777</v>
       </c>
       <c r="X103" t="n">
         <v>17.5</v>
@@ -10681,10 +10681,10 @@
         <v>35</v>
       </c>
       <c r="K117" t="n">
-        <v>22.5</v>
+        <v>27.7</v>
       </c>
       <c r="L117" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="M117" t="inlineStr">
         <is>
@@ -10714,7 +10714,7 @@
         <v>41</v>
       </c>
       <c r="T117" t="n">
-        <v>-12.5</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="U117" t="n">
         <v>25.5</v>
@@ -12353,10 +12353,10 @@
         <v>28</v>
       </c>
       <c r="K136" t="n">
-        <v>33.1</v>
+        <v>21.2</v>
       </c>
       <c r="L136" t="n">
-        <v>118</v>
+        <v>76</v>
       </c>
       <c r="M136" t="inlineStr">
         <is>
@@ -12386,7 +12386,7 @@
         <v>28</v>
       </c>
       <c r="T136" t="n">
-        <v>5.100000000000001</v>
+        <v>-6.800000000000001</v>
       </c>
       <c r="U136" t="n">
         <v>28.06666666666666</v>
@@ -13887,7 +13887,7 @@
         <v>3</v>
       </c>
       <c r="W153" t="n">
-        <v>33.02222222222222</v>
+        <v>33.02222222222223</v>
       </c>
       <c r="X153" t="n">
         <v>24.5</v>
@@ -17091,10 +17091,10 @@
         <v>35</v>
       </c>
       <c r="K190" t="n">
-        <v>32.7</v>
+        <v>31.7</v>
       </c>
       <c r="L190" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M190" t="inlineStr">
         <is>
@@ -17124,7 +17124,7 @@
         <v>41</v>
       </c>
       <c r="T190" t="n">
-        <v>-2.299999999999997</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="U190" t="n">
         <v>32.26666666666667</v>
@@ -17965,10 +17965,10 @@
         <v>28</v>
       </c>
       <c r="K200" t="n">
-        <v>26.8</v>
+        <v>32.8</v>
       </c>
       <c r="L200" t="n">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="M200" t="inlineStr">
         <is>
@@ -17998,7 +17998,7 @@
         <v>28</v>
       </c>
       <c r="T200" t="n">
-        <v>-1.199999999999999</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="U200" t="n">
         <v>30.93333333333333</v>
@@ -19549,10 +19549,10 @@
         <v>31</v>
       </c>
       <c r="K218" t="n">
-        <v>33.7</v>
+        <v>36.5</v>
       </c>
       <c r="L218" t="n">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="M218" t="inlineStr">
         <is>
@@ -19580,7 +19580,7 @@
       </c>
       <c r="S218" t="inlineStr"/>
       <c r="T218" t="n">
-        <v>2.700000000000003</v>
+        <v>5.5</v>
       </c>
       <c r="U218" t="n">
         <v>33.66666666666666</v>
@@ -20603,10 +20603,10 @@
         <v>28</v>
       </c>
       <c r="K230" t="n">
-        <v>25</v>
+        <v>22.8</v>
       </c>
       <c r="L230" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="M230" t="inlineStr">
         <is>
@@ -20636,7 +20636,7 @@
         <v>28</v>
       </c>
       <c r="T230" t="n">
-        <v>-3</v>
+        <v>-5.199999999999999</v>
       </c>
       <c r="U230" t="n">
         <v>24.76666666666667</v>
@@ -22785,10 +22785,10 @@
         <v>21</v>
       </c>
       <c r="K255" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="L255" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="M255" t="inlineStr">
         <is>
@@ -22816,7 +22816,7 @@
       </c>
       <c r="S255" t="inlineStr"/>
       <c r="T255" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U255" t="n">
         <v>21.8</v>
@@ -22959,10 +22959,10 @@
         <v>21</v>
       </c>
       <c r="K257" t="n">
-        <v>16.6</v>
+        <v>42.6</v>
       </c>
       <c r="L257" t="n">
-        <v>79</v>
+        <v>203</v>
       </c>
       <c r="M257" t="inlineStr">
         <is>
@@ -22992,7 +22992,7 @@
         <v>21</v>
       </c>
       <c r="T257" t="n">
-        <v>-4.399999999999999</v>
+        <v>21.6</v>
       </c>
       <c r="U257" t="n">
         <v>36.33333333333334</v>
@@ -24625,10 +24625,10 @@
         <v>21</v>
       </c>
       <c r="K276" t="n">
-        <v>18.3</v>
+        <v>17.8</v>
       </c>
       <c r="L276" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="M276" t="inlineStr">
         <is>
@@ -24658,7 +24658,7 @@
         <v>21</v>
       </c>
       <c r="T276" t="n">
-        <v>-2.699999999999999</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U276" t="n">
         <v>18.73333333333333</v>
@@ -24801,10 +24801,10 @@
         <v>28</v>
       </c>
       <c r="K278" t="n">
-        <v>32.5</v>
+        <v>27.6</v>
       </c>
       <c r="L278" t="n">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="M278" t="inlineStr">
         <is>
@@ -24834,7 +24834,7 @@
         <v>28</v>
       </c>
       <c r="T278" t="n">
-        <v>4.5</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U278" t="n">
         <v>30.16666666666667</v>
@@ -28575,10 +28575,10 @@
         <v>24.5</v>
       </c>
       <c r="K321" t="n">
-        <v>20.9</v>
+        <v>24.6</v>
       </c>
       <c r="L321" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="M321" t="inlineStr">
         <is>
@@ -28608,7 +28608,7 @@
         <v>28</v>
       </c>
       <c r="T321" t="n">
-        <v>-3.600000000000001</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U321" t="n">
         <v>23.96666666666667</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -29761,7 +29761,7 @@
         <v>3</v>
       </c>
       <c r="W334" t="n">
-        <v>25.57777777777778</v>
+        <v>25.57777777777777</v>
       </c>
       <c r="X334" t="n">
         <v>21</v>
@@ -29807,10 +29807,10 @@
         <v>24.5</v>
       </c>
       <c r="K335" t="n">
-        <v>24</v>
+        <v>31.1</v>
       </c>
       <c r="L335" t="n">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="M335" t="inlineStr">
         <is>
@@ -29840,7 +29840,7 @@
         <v>28</v>
       </c>
       <c r="T335" t="n">
-        <v>-0.5</v>
+        <v>6.600000000000001</v>
       </c>
       <c r="U335" t="n">
         <v>29.13333333333334</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-25 18:50:10
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3591,10 +3591,10 @@
         <v>31</v>
       </c>
       <c r="K36" t="n">
-        <v>28.9</v>
+        <v>30.9</v>
       </c>
       <c r="L36" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="n">
-        <v>-2.100000000000001</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U36" t="n">
         <v>30.8</v>
@@ -4287,10 +4287,10 @@
         <v>24</v>
       </c>
       <c r="K44" t="n">
-        <v>15.7</v>
+        <v>16.2</v>
       </c>
       <c r="L44" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
@@ -4320,7 +4320,7 @@
         <v>28</v>
       </c>
       <c r="T44" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.800000000000001</v>
       </c>
       <c r="U44" t="n">
         <v>16.5</v>
@@ -5859,10 +5859,10 @@
         <v>31</v>
       </c>
       <c r="K62" t="n">
-        <v>35.8</v>
+        <v>31.4</v>
       </c>
       <c r="L62" t="n">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
@@ -5890,10 +5890,10 @@
       </c>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="n">
-        <v>4.799999999999997</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U62" t="n">
-        <v>30.66666666666667</v>
+        <v>30.66666666666666</v>
       </c>
       <c r="V62" t="n">
         <v>3</v>
@@ -6121,10 +6121,10 @@
         <v>24</v>
       </c>
       <c r="K65" t="n">
-        <v>27.2</v>
+        <v>16.6</v>
       </c>
       <c r="L65" t="n">
-        <v>113</v>
+        <v>69</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -6154,7 +6154,7 @@
         <v>28</v>
       </c>
       <c r="T65" t="n">
-        <v>3.199999999999999</v>
+        <v>-7.399999999999999</v>
       </c>
       <c r="U65" t="n">
         <v>23.4</v>
@@ -7527,7 +7527,7 @@
         <v>28</v>
       </c>
       <c r="K81" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="L81" t="n">
         <v>88</v>
@@ -7560,7 +7560,7 @@
         <v>28</v>
       </c>
       <c r="T81" t="n">
-        <v>-3.199999999999999</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="U81" t="n">
         <v>25.13333333333334</v>
@@ -8141,10 +8141,10 @@
         <v>21</v>
       </c>
       <c r="K88" t="n">
-        <v>23.8</v>
+        <v>24.7</v>
       </c>
       <c r="L88" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
         <v>21</v>
       </c>
       <c r="T88" t="n">
-        <v>2.800000000000001</v>
+        <v>3.699999999999999</v>
       </c>
       <c r="U88" t="n">
         <v>22.53333333333333</v>
@@ -8667,10 +8667,10 @@
         <v>35</v>
       </c>
       <c r="K94" t="n">
-        <v>40.3</v>
+        <v>39.8</v>
       </c>
       <c r="L94" t="n">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M94" t="inlineStr">
         <is>
@@ -8700,7 +8700,7 @@
         <v>41</v>
       </c>
       <c r="T94" t="n">
-        <v>5.299999999999997</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="U94" t="n">
         <v>36.16666666666666</v>
@@ -10153,10 +10153,10 @@
         <v>35</v>
       </c>
       <c r="K111" t="n">
-        <v>34.1</v>
+        <v>39.8</v>
       </c>
       <c r="L111" t="n">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -10186,7 +10186,7 @@
         <v>41</v>
       </c>
       <c r="T111" t="n">
-        <v>-0.8999999999999986</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="U111" t="n">
         <v>36.83333333333334</v>
@@ -12791,10 +12791,10 @@
         <v>35</v>
       </c>
       <c r="K141" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="L141" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="M141" t="inlineStr">
         <is>
@@ -12824,7 +12824,7 @@
         <v>41</v>
       </c>
       <c r="T141" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="U141" t="n">
         <v>41</v>
@@ -13407,10 +13407,10 @@
         <v>35</v>
       </c>
       <c r="K148" t="n">
-        <v>25.6</v>
+        <v>27.7</v>
       </c>
       <c r="L148" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="M148" t="inlineStr">
         <is>
@@ -13440,7 +13440,7 @@
         <v>41</v>
       </c>
       <c r="T148" t="n">
-        <v>-9.399999999999999</v>
+        <v>-7.300000000000001</v>
       </c>
       <c r="U148" t="n">
         <v>26.5</v>
@@ -17877,10 +17877,10 @@
         <v>21</v>
       </c>
       <c r="K199" t="n">
-        <v>20.7</v>
+        <v>23.9</v>
       </c>
       <c r="L199" t="n">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="M199" t="inlineStr">
         <is>
@@ -17910,7 +17910,7 @@
         <v>21</v>
       </c>
       <c r="T199" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="U199" t="n">
         <v>22.5</v>
@@ -20603,10 +20603,10 @@
         <v>28</v>
       </c>
       <c r="K230" t="n">
-        <v>22.8</v>
+        <v>25</v>
       </c>
       <c r="L230" t="n">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="M230" t="inlineStr">
         <is>
@@ -20636,7 +20636,7 @@
         <v>28</v>
       </c>
       <c r="T230" t="n">
-        <v>-5.199999999999999</v>
+        <v>-3</v>
       </c>
       <c r="U230" t="n">
         <v>24.76666666666667</v>
@@ -21129,10 +21129,10 @@
         <v>28</v>
       </c>
       <c r="K236" t="n">
-        <v>30.9</v>
+        <v>24.9</v>
       </c>
       <c r="L236" t="n">
-        <v>110</v>
+        <v>89</v>
       </c>
       <c r="M236" t="inlineStr">
         <is>
@@ -21162,7 +21162,7 @@
         <v>28</v>
       </c>
       <c r="T236" t="n">
-        <v>2.899999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="U236" t="n">
         <v>27.93333333333333</v>
@@ -22785,10 +22785,10 @@
         <v>21</v>
       </c>
       <c r="K255" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="L255" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="M255" t="inlineStr">
         <is>
@@ -22816,7 +22816,7 @@
       </c>
       <c r="S255" t="inlineStr"/>
       <c r="T255" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U255" t="n">
         <v>21.8</v>
@@ -25857,10 +25857,10 @@
         <v>21</v>
       </c>
       <c r="K290" t="n">
-        <v>18.4</v>
+        <v>20.2</v>
       </c>
       <c r="L290" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="M290" t="inlineStr">
         <is>
@@ -25890,16 +25890,16 @@
         <v>21</v>
       </c>
       <c r="T290" t="n">
-        <v>-2.600000000000001</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U290" t="n">
-        <v>19.86666666666666</v>
+        <v>19.86666666666667</v>
       </c>
       <c r="V290" t="n">
         <v>3</v>
       </c>
       <c r="W290" t="n">
-        <v>21.74444444444444</v>
+        <v>21.74444444444445</v>
       </c>
       <c r="X290" t="n">
         <v>17.5</v>
@@ -28311,10 +28311,10 @@
         <v>24.5</v>
       </c>
       <c r="K318" t="n">
-        <v>21.3</v>
+        <v>30.7</v>
       </c>
       <c r="L318" t="n">
-        <v>87</v>
+        <v>125</v>
       </c>
       <c r="M318" t="inlineStr">
         <is>
@@ -28344,7 +28344,7 @@
         <v>28</v>
       </c>
       <c r="T318" t="n">
-        <v>-3.199999999999999</v>
+        <v>6.199999999999999</v>
       </c>
       <c r="U318" t="n">
         <v>24.76666666666667</v>
@@ -28399,10 +28399,10 @@
         <v>24.5</v>
       </c>
       <c r="K319" t="n">
-        <v>23.9</v>
+        <v>23.4</v>
       </c>
       <c r="L319" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="M319" t="inlineStr">
         <is>
@@ -28432,7 +28432,7 @@
         <v>28</v>
       </c>
       <c r="T319" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U319" t="n">
         <v>23.56666666666666</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L325" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L333" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L355" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-25 20:19:40
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L79" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7527,7 +7527,7 @@
         <v>28</v>
       </c>
       <c r="K81" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="L81" t="n">
         <v>88</v>
@@ -7560,7 +7560,7 @@
         <v>28</v>
       </c>
       <c r="T81" t="n">
-        <v>-3.300000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U81" t="n">
         <v>25.13333333333334</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L83" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8141,10 +8141,10 @@
         <v>21</v>
       </c>
       <c r="K88" t="n">
-        <v>24.7</v>
+        <v>23.8</v>
       </c>
       <c r="L88" t="n">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -8174,7 +8174,7 @@
         <v>21</v>
       </c>
       <c r="T88" t="n">
-        <v>3.699999999999999</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U88" t="n">
         <v>22.53333333333333</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L90" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L95" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -21129,10 +21129,10 @@
         <v>28</v>
       </c>
       <c r="K236" t="n">
-        <v>24.9</v>
+        <v>30.9</v>
       </c>
       <c r="L236" t="n">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="M236" t="inlineStr">
         <is>
@@ -21162,7 +21162,7 @@
         <v>28</v>
       </c>
       <c r="T236" t="n">
-        <v>-3.100000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="U236" t="n">
         <v>27.93333333333333</v>
@@ -23047,10 +23047,10 @@
         <v>28</v>
       </c>
       <c r="K258" t="n">
-        <v>27.7</v>
+        <v>26.8</v>
       </c>
       <c r="L258" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="M258" t="inlineStr">
         <is>
@@ -23080,7 +23080,7 @@
         <v>28</v>
       </c>
       <c r="T258" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U258" t="n">
         <v>27.16666666666667</v>
@@ -23399,10 +23399,10 @@
         <v>28</v>
       </c>
       <c r="K262" t="n">
-        <v>27.6</v>
+        <v>27.1</v>
       </c>
       <c r="L262" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="M262" t="inlineStr">
         <is>
@@ -23432,7 +23432,7 @@
         <v>28</v>
       </c>
       <c r="T262" t="n">
-        <v>-0.3999999999999986</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U262" t="n">
         <v>27.4</v>
@@ -23487,10 +23487,10 @@
         <v>28</v>
       </c>
       <c r="K263" t="n">
-        <v>28.9</v>
+        <v>28.1</v>
       </c>
       <c r="L263" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="M263" t="inlineStr">
         <is>
@@ -23520,7 +23520,7 @@
         <v>28</v>
       </c>
       <c r="T263" t="n">
-        <v>0.8999999999999986</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U263" t="n">
         <v>28.03333333333333</v>
@@ -23575,10 +23575,10 @@
         <v>28</v>
       </c>
       <c r="K264" t="n">
-        <v>27.2</v>
+        <v>28.4</v>
       </c>
       <c r="L264" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="M264" t="inlineStr">
         <is>
@@ -23608,10 +23608,10 @@
         <v>28</v>
       </c>
       <c r="T264" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U264" t="n">
-        <v>28.06666666666666</v>
+        <v>28.06666666666667</v>
       </c>
       <c r="V264" t="n">
         <v>3</v>
@@ -24889,10 +24889,10 @@
         <v>28</v>
       </c>
       <c r="K279" t="n">
-        <v>27.8</v>
+        <v>26.3</v>
       </c>
       <c r="L279" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="M279" t="inlineStr">
         <is>
@@ -24922,7 +24922,7 @@
         <v>28</v>
       </c>
       <c r="T279" t="n">
-        <v>-0.1999999999999993</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U279" t="n">
         <v>27.36666666666666</v>
@@ -24977,10 +24977,10 @@
         <v>28</v>
       </c>
       <c r="K280" t="n">
-        <v>26.5</v>
+        <v>28.4</v>
       </c>
       <c r="L280" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="M280" t="inlineStr">
         <is>
@@ -25010,7 +25010,7 @@
         <v>28</v>
       </c>
       <c r="T280" t="n">
-        <v>-1.5</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U280" t="n">
         <v>27.53333333333333</v>
@@ -25329,10 +25329,10 @@
         <v>21</v>
       </c>
       <c r="K284" t="n">
-        <v>21.4</v>
+        <v>19.9</v>
       </c>
       <c r="L284" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="M284" t="inlineStr">
         <is>
@@ -25362,7 +25362,7 @@
         <v>21</v>
       </c>
       <c r="T284" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U284" t="n">
         <v>21</v>
@@ -26205,10 +26205,10 @@
         <v>21</v>
       </c>
       <c r="K294" t="n">
-        <v>22.2</v>
+        <v>20.9</v>
       </c>
       <c r="L294" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="M294" t="inlineStr">
         <is>
@@ -26238,7 +26238,7 @@
         <v>21</v>
       </c>
       <c r="T294" t="n">
-        <v>1.199999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U294" t="n">
         <v>22.03333333333333</v>
@@ -27959,10 +27959,10 @@
         <v>24.5</v>
       </c>
       <c r="K314" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="L314" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="M314" t="inlineStr">
         <is>
@@ -27992,7 +27992,7 @@
         <v>28</v>
       </c>
       <c r="T314" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U314" t="n">
         <v>25.13333333333334</v>
@@ -28927,10 +28927,10 @@
         <v>24.5</v>
       </c>
       <c r="K325" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L325" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M325" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         <v>28</v>
       </c>
       <c r="T325" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U325" t="n">
         <v>24.66666666666667</v>
@@ -29631,10 +29631,10 @@
         <v>24.5</v>
       </c>
       <c r="K333" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L333" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M333" t="inlineStr">
         <is>
@@ -29664,7 +29664,7 @@
         <v>28</v>
       </c>
       <c r="T333" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U333" t="n">
         <v>27.1</v>
@@ -29807,10 +29807,10 @@
         <v>24.5</v>
       </c>
       <c r="K335" t="n">
-        <v>31.1</v>
+        <v>24</v>
       </c>
       <c r="L335" t="n">
-        <v>127</v>
+        <v>98</v>
       </c>
       <c r="M335" t="inlineStr">
         <is>
@@ -29840,7 +29840,7 @@
         <v>28</v>
       </c>
       <c r="T335" t="n">
-        <v>6.600000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="U335" t="n">
         <v>29.13333333333334</v>
@@ -31567,10 +31567,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L355" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31600,10 +31600,10 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U355" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V355" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-25 22:23:19
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -23047,10 +23047,10 @@
         <v>28</v>
       </c>
       <c r="K258" t="n">
-        <v>26.8</v>
+        <v>27.7</v>
       </c>
       <c r="L258" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="M258" t="inlineStr">
         <is>
@@ -23080,7 +23080,7 @@
         <v>28</v>
       </c>
       <c r="T258" t="n">
-        <v>-1.199999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U258" t="n">
         <v>27.16666666666667</v>
@@ -23399,10 +23399,10 @@
         <v>28</v>
       </c>
       <c r="K262" t="n">
-        <v>27.1</v>
+        <v>27.6</v>
       </c>
       <c r="L262" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M262" t="inlineStr">
         <is>
@@ -23432,7 +23432,7 @@
         <v>28</v>
       </c>
       <c r="T262" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U262" t="n">
         <v>27.4</v>
@@ -23487,10 +23487,10 @@
         <v>28</v>
       </c>
       <c r="K263" t="n">
-        <v>28.1</v>
+        <v>28.9</v>
       </c>
       <c r="L263" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="M263" t="inlineStr">
         <is>
@@ -23520,7 +23520,7 @@
         <v>28</v>
       </c>
       <c r="T263" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U263" t="n">
         <v>28.03333333333333</v>
@@ -23575,10 +23575,10 @@
         <v>28</v>
       </c>
       <c r="K264" t="n">
-        <v>28.4</v>
+        <v>27.2</v>
       </c>
       <c r="L264" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M264" t="inlineStr">
         <is>
@@ -23608,10 +23608,10 @@
         <v>28</v>
       </c>
       <c r="T264" t="n">
-        <v>0.3999999999999986</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U264" t="n">
-        <v>28.06666666666667</v>
+        <v>28.06666666666666</v>
       </c>
       <c r="V264" t="n">
         <v>3</v>
@@ -24363,10 +24363,10 @@
         <v>28</v>
       </c>
       <c r="K273" t="n">
-        <v>27.2</v>
+        <v>29.8</v>
       </c>
       <c r="L273" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="M273" t="inlineStr">
         <is>
@@ -24396,7 +24396,7 @@
         <v>28</v>
       </c>
       <c r="T273" t="n">
-        <v>-0.8000000000000007</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="U273" t="n">
         <v>28.43333333333333</v>
@@ -24405,7 +24405,7 @@
         <v>3</v>
       </c>
       <c r="W273" t="n">
-        <v>28.15555555555556</v>
+        <v>28.15555555555555</v>
       </c>
       <c r="X273" t="n">
         <v>24.5</v>
@@ -24539,10 +24539,10 @@
         <v>21</v>
       </c>
       <c r="K275" t="n">
-        <v>16.3</v>
+        <v>26.4</v>
       </c>
       <c r="L275" t="n">
-        <v>78</v>
+        <v>126</v>
       </c>
       <c r="M275" t="inlineStr">
         <is>
@@ -24572,7 +24572,7 @@
         <v>21</v>
       </c>
       <c r="T275" t="n">
-        <v>-4.699999999999999</v>
+        <v>5.399999999999999</v>
       </c>
       <c r="U275" t="n">
         <v>22.9</v>
@@ -24889,10 +24889,10 @@
         <v>28</v>
       </c>
       <c r="K279" t="n">
-        <v>26.3</v>
+        <v>27.8</v>
       </c>
       <c r="L279" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="M279" t="inlineStr">
         <is>
@@ -24922,7 +24922,7 @@
         <v>28</v>
       </c>
       <c r="T279" t="n">
-        <v>-1.699999999999999</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U279" t="n">
         <v>27.36666666666666</v>
@@ -24977,10 +24977,10 @@
         <v>28</v>
       </c>
       <c r="K280" t="n">
-        <v>28.4</v>
+        <v>26.5</v>
       </c>
       <c r="L280" t="n">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="M280" t="inlineStr">
         <is>
@@ -25010,7 +25010,7 @@
         <v>28</v>
       </c>
       <c r="T280" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1.5</v>
       </c>
       <c r="U280" t="n">
         <v>27.53333333333333</v>
@@ -25329,10 +25329,10 @@
         <v>21</v>
       </c>
       <c r="K284" t="n">
-        <v>19.9</v>
+        <v>21.4</v>
       </c>
       <c r="L284" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="M284" t="inlineStr">
         <is>
@@ -25362,7 +25362,7 @@
         <v>21</v>
       </c>
       <c r="T284" t="n">
-        <v>-1.100000000000001</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U284" t="n">
         <v>21</v>
@@ -26205,10 +26205,10 @@
         <v>21</v>
       </c>
       <c r="K294" t="n">
-        <v>20.9</v>
+        <v>22.2</v>
       </c>
       <c r="L294" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="M294" t="inlineStr">
         <is>
@@ -26238,7 +26238,7 @@
         <v>21</v>
       </c>
       <c r="T294" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1.199999999999999</v>
       </c>
       <c r="U294" t="n">
         <v>22.03333333333333</v>
@@ -26557,10 +26557,10 @@
         <v>21</v>
       </c>
       <c r="K298" t="n">
-        <v>18.9</v>
+        <v>19.8</v>
       </c>
       <c r="L298" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="M298" t="inlineStr">
         <is>
@@ -26590,7 +26590,7 @@
         <v>21</v>
       </c>
       <c r="T298" t="n">
-        <v>-2.100000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U298" t="n">
         <v>19</v>
@@ -26907,10 +26907,10 @@
         <v>21</v>
       </c>
       <c r="K302" t="n">
-        <v>20.4</v>
+        <v>22.6</v>
       </c>
       <c r="L302" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="M302" t="inlineStr">
         <is>
@@ -26938,7 +26938,7 @@
       </c>
       <c r="S302" t="inlineStr"/>
       <c r="T302" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U302" t="n">
         <v>21.8</v>
@@ -27959,10 +27959,10 @@
         <v>24.5</v>
       </c>
       <c r="K314" t="n">
-        <v>23.9</v>
+        <v>25.1</v>
       </c>
       <c r="L314" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="M314" t="inlineStr">
         <is>
@@ -27992,7 +27992,7 @@
         <v>28</v>
       </c>
       <c r="T314" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U314" t="n">
         <v>25.13333333333334</v>
@@ -28399,10 +28399,10 @@
         <v>24.5</v>
       </c>
       <c r="K319" t="n">
-        <v>23.4</v>
+        <v>23.9</v>
       </c>
       <c r="L319" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="M319" t="inlineStr">
         <is>
@@ -28432,7 +28432,7 @@
         <v>28</v>
       </c>
       <c r="T319" t="n">
-        <v>-1.100000000000001</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U319" t="n">
         <v>23.56666666666666</v>
@@ -29807,10 +29807,10 @@
         <v>24.5</v>
       </c>
       <c r="K335" t="n">
-        <v>24</v>
+        <v>31.1</v>
       </c>
       <c r="L335" t="n">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="M335" t="inlineStr">
         <is>
@@ -29840,7 +29840,7 @@
         <v>28</v>
       </c>
       <c r="T335" t="n">
-        <v>-0.5</v>
+        <v>6.600000000000001</v>
       </c>
       <c r="U335" t="n">
         <v>29.13333333333334</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-26 00:00:39
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -23839,10 +23839,10 @@
         <v>28</v>
       </c>
       <c r="K267" t="n">
-        <v>28.7</v>
+        <v>23.6</v>
       </c>
       <c r="L267" t="n">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="M267" t="inlineStr">
         <is>
@@ -23872,7 +23872,7 @@
         <v>28</v>
       </c>
       <c r="T267" t="n">
-        <v>0.6999999999999993</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="U267" t="n">
         <v>27</v>
@@ -24363,10 +24363,10 @@
         <v>28</v>
       </c>
       <c r="K273" t="n">
-        <v>29.8</v>
+        <v>27.2</v>
       </c>
       <c r="L273" t="n">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="M273" t="inlineStr">
         <is>
@@ -24396,7 +24396,7 @@
         <v>28</v>
       </c>
       <c r="T273" t="n">
-        <v>1.800000000000001</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U273" t="n">
         <v>28.43333333333333</v>
@@ -24405,7 +24405,7 @@
         <v>3</v>
       </c>
       <c r="W273" t="n">
-        <v>28.15555555555555</v>
+        <v>28.15555555555556</v>
       </c>
       <c r="X273" t="n">
         <v>24.5</v>
@@ -24539,10 +24539,10 @@
         <v>21</v>
       </c>
       <c r="K275" t="n">
-        <v>26.4</v>
+        <v>16.3</v>
       </c>
       <c r="L275" t="n">
-        <v>126</v>
+        <v>78</v>
       </c>
       <c r="M275" t="inlineStr">
         <is>
@@ -24572,7 +24572,7 @@
         <v>21</v>
       </c>
       <c r="T275" t="n">
-        <v>5.399999999999999</v>
+        <v>-4.699999999999999</v>
       </c>
       <c r="U275" t="n">
         <v>22.9</v>
@@ -25153,10 +25153,10 @@
         <v>28</v>
       </c>
       <c r="K282" t="n">
-        <v>28.2</v>
+        <v>29</v>
       </c>
       <c r="L282" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="M282" t="inlineStr">
         <is>
@@ -25186,7 +25186,7 @@
         <v>28</v>
       </c>
       <c r="T282" t="n">
-        <v>0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="U282" t="n">
         <v>28.2</v>
@@ -25769,10 +25769,10 @@
         <v>21</v>
       </c>
       <c r="K289" t="n">
-        <v>18.2</v>
+        <v>18.6</v>
       </c>
       <c r="L289" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="M289" t="inlineStr">
         <is>
@@ -25802,7 +25802,7 @@
         <v>21</v>
       </c>
       <c r="T289" t="n">
-        <v>-2.800000000000001</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="U289" t="n">
         <v>18.23333333333333</v>
@@ -26557,10 +26557,10 @@
         <v>21</v>
       </c>
       <c r="K298" t="n">
-        <v>19.8</v>
+        <v>18.9</v>
       </c>
       <c r="L298" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="M298" t="inlineStr">
         <is>
@@ -26590,7 +26590,7 @@
         <v>21</v>
       </c>
       <c r="T298" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U298" t="n">
         <v>19</v>
@@ -26907,10 +26907,10 @@
         <v>21</v>
       </c>
       <c r="K302" t="n">
-        <v>22.6</v>
+        <v>20.4</v>
       </c>
       <c r="L302" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="M302" t="inlineStr">
         <is>
@@ -26938,7 +26938,7 @@
       </c>
       <c r="S302" t="inlineStr"/>
       <c r="T302" t="n">
-        <v>1.600000000000001</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U302" t="n">
         <v>21.8</v>
@@ -28399,10 +28399,10 @@
         <v>24.5</v>
       </c>
       <c r="K319" t="n">
-        <v>23.9</v>
+        <v>23.4</v>
       </c>
       <c r="L319" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="M319" t="inlineStr">
         <is>
@@ -28432,7 +28432,7 @@
         <v>28</v>
       </c>
       <c r="T319" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U319" t="n">
         <v>23.56666666666666</v>
@@ -29455,10 +29455,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>18.6</v>
+        <v>24.3</v>
       </c>
       <c r="L331" t="n">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29488,10 +29488,10 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>-5.899999999999999</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U331" t="n">
-        <v>21.93333333333333</v>
+        <v>21.93333333333334</v>
       </c>
       <c r="V331" t="n">
         <v>3</v>
@@ -32529,10 +32529,10 @@
         <v>21</v>
       </c>
       <c r="K366" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="L366" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M366" t="inlineStr">
         <is>
@@ -32562,7 +32562,7 @@
         <v>21</v>
       </c>
       <c r="T366" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U366" t="n">
         <v>20.9</v>
@@ -32617,10 +32617,10 @@
         <v>21</v>
       </c>
       <c r="K367" t="n">
-        <v>23.2</v>
+        <v>22.4</v>
       </c>
       <c r="L367" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M367" t="inlineStr">
         <is>
@@ -32648,7 +32648,7 @@
       </c>
       <c r="S367" t="inlineStr"/>
       <c r="T367" t="n">
-        <v>2.199999999999999</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="U367" t="n">
         <v>21.23333333333333</v>
@@ -32701,10 +32701,10 @@
         <v>21</v>
       </c>
       <c r="K368" t="n">
-        <v>23.4</v>
+        <v>22</v>
       </c>
       <c r="L368" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="M368" t="inlineStr">
         <is>
@@ -32734,7 +32734,7 @@
         <v>21</v>
       </c>
       <c r="T368" t="n">
-        <v>2.399999999999999</v>
+        <v>1</v>
       </c>
       <c r="U368" t="n">
         <v>22.1</v>
@@ -32789,7 +32789,7 @@
         <v>21</v>
       </c>
       <c r="K369" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="L369" t="n">
         <v>94</v>
@@ -32822,7 +32822,7 @@
         <v>21</v>
       </c>
       <c r="T369" t="n">
-        <v>-1.100000000000001</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U369" t="n">
         <v>20.26666666666667</v>
@@ -32877,10 +32877,10 @@
         <v>21</v>
       </c>
       <c r="K370" t="n">
-        <v>23.6</v>
+        <v>20.7</v>
       </c>
       <c r="L370" t="n">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="M370" t="inlineStr">
         <is>
@@ -32910,7 +32910,7 @@
         <v>21</v>
       </c>
       <c r="T370" t="n">
-        <v>2.600000000000001</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U370" t="n">
         <v>22.76666666666667</v>
@@ -32965,10 +32965,10 @@
         <v>21</v>
       </c>
       <c r="K371" t="n">
-        <v>20</v>
+        <v>23.2</v>
       </c>
       <c r="L371" t="n">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="M371" t="inlineStr">
         <is>
@@ -32996,7 +32996,7 @@
       </c>
       <c r="S371" t="inlineStr"/>
       <c r="T371" t="n">
-        <v>-1</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U371" t="n">
         <v>22.3</v>
@@ -33051,10 +33051,10 @@
         <v>21</v>
       </c>
       <c r="K372" t="n">
-        <v>20.4</v>
+        <v>16.3</v>
       </c>
       <c r="L372" t="n">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="M372" t="inlineStr">
         <is>
@@ -33084,7 +33084,7 @@
         <v>21</v>
       </c>
       <c r="T372" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-4.699999999999999</v>
       </c>
       <c r="U372" t="n">
         <v>19.6</v>
@@ -33225,10 +33225,10 @@
         <v>21</v>
       </c>
       <c r="K374" t="n">
-        <v>23.5</v>
+        <v>22.7</v>
       </c>
       <c r="L374" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="M374" t="inlineStr">
         <is>
@@ -33258,7 +33258,7 @@
         <v>21</v>
       </c>
       <c r="T374" t="n">
-        <v>2.5</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="U374" t="n">
         <v>22.16666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-26 18:19:41
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4809,10 +4809,10 @@
         <v>24</v>
       </c>
       <c r="K50" t="n">
-        <v>30.2</v>
+        <v>17.2</v>
       </c>
       <c r="L50" t="n">
-        <v>126</v>
+        <v>71</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
@@ -4842,7 +4842,7 @@
         <v>28</v>
       </c>
       <c r="T50" t="n">
-        <v>6.199999999999999</v>
+        <v>-6.800000000000001</v>
       </c>
       <c r="U50" t="n">
         <v>24.16666666666667</v>
@@ -4897,10 +4897,10 @@
         <v>24</v>
       </c>
       <c r="K51" t="n">
-        <v>23.8</v>
+        <v>24.9</v>
       </c>
       <c r="L51" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
@@ -4930,7 +4930,7 @@
         <v>28</v>
       </c>
       <c r="T51" t="n">
-        <v>-0.1999999999999993</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U51" t="n">
         <v>21.43333333333333</v>
@@ -5683,10 +5683,10 @@
         <v>24</v>
       </c>
       <c r="K60" t="n">
-        <v>20.8</v>
+        <v>22.4</v>
       </c>
       <c r="L60" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
@@ -5716,7 +5716,7 @@
         <v>28</v>
       </c>
       <c r="T60" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U60" t="n">
         <v>21.53333333333333</v>
@@ -5725,7 +5725,7 @@
         <v>3</v>
       </c>
       <c r="W60" t="n">
-        <v>23.14444444444444</v>
+        <v>23.14444444444445</v>
       </c>
       <c r="X60" t="n">
         <v>20.5</v>
@@ -6033,10 +6033,10 @@
         <v>24</v>
       </c>
       <c r="K64" t="n">
-        <v>25.9</v>
+        <v>23.1</v>
       </c>
       <c r="L64" t="n">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
@@ -6066,7 +6066,7 @@
         <v>28</v>
       </c>
       <c r="T64" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U64" t="n">
         <v>24.1</v>
@@ -6209,10 +6209,10 @@
         <v>24</v>
       </c>
       <c r="K66" t="n">
-        <v>25.7</v>
+        <v>23.4</v>
       </c>
       <c r="L66" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="M66" t="inlineStr">
         <is>
@@ -6242,7 +6242,7 @@
         <v>28</v>
       </c>
       <c r="T66" t="n">
-        <v>1.699999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U66" t="n">
         <v>24.46666666666667</v>
@@ -9015,10 +9015,10 @@
         <v>21</v>
       </c>
       <c r="K98" t="n">
-        <v>22.5</v>
+        <v>23.7</v>
       </c>
       <c r="L98" t="n">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="M98" t="inlineStr">
         <is>
@@ -9048,7 +9048,7 @@
         <v>21</v>
       </c>
       <c r="T98" t="n">
-        <v>1.5</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U98" t="n">
         <v>21.9</v>
@@ -9279,10 +9279,10 @@
         <v>28</v>
       </c>
       <c r="K101" t="n">
-        <v>26.5</v>
+        <v>27.7</v>
       </c>
       <c r="L101" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="M101" t="inlineStr">
         <is>
@@ -9312,7 +9312,7 @@
         <v>28</v>
       </c>
       <c r="T101" t="n">
-        <v>-1.5</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U101" t="n">
         <v>27.96666666666667</v>
@@ -10329,10 +10329,10 @@
         <v>35</v>
       </c>
       <c r="K113" t="n">
-        <v>29.6</v>
+        <v>27.1</v>
       </c>
       <c r="L113" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="M113" t="inlineStr">
         <is>
@@ -10362,7 +10362,7 @@
         <v>41</v>
       </c>
       <c r="T113" t="n">
-        <v>-5.399999999999999</v>
+        <v>-7.899999999999999</v>
       </c>
       <c r="U113" t="n">
         <v>27.33333333333333</v>
@@ -10681,10 +10681,10 @@
         <v>35</v>
       </c>
       <c r="K117" t="n">
-        <v>27.7</v>
+        <v>22.5</v>
       </c>
       <c r="L117" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="M117" t="inlineStr">
         <is>
@@ -10714,7 +10714,7 @@
         <v>41</v>
       </c>
       <c r="T117" t="n">
-        <v>-7.300000000000001</v>
+        <v>-12.5</v>
       </c>
       <c r="U117" t="n">
         <v>25.5</v>
@@ -11121,10 +11121,10 @@
         <v>35</v>
       </c>
       <c r="K122" t="n">
-        <v>34.9</v>
+        <v>37.4</v>
       </c>
       <c r="L122" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="M122" t="inlineStr">
         <is>
@@ -11154,7 +11154,7 @@
         <v>41</v>
       </c>
       <c r="T122" t="n">
-        <v>-0.1000000000000014</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U122" t="n">
         <v>35.63333333333333</v>
@@ -11297,10 +11297,10 @@
         <v>21</v>
       </c>
       <c r="K124" t="n">
-        <v>19.3</v>
+        <v>26</v>
       </c>
       <c r="L124" t="n">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -11330,7 +11330,7 @@
         <v>21</v>
       </c>
       <c r="T124" t="n">
-        <v>-1.699999999999999</v>
+        <v>5</v>
       </c>
       <c r="U124" t="n">
         <v>23.7</v>
@@ -17267,10 +17267,10 @@
         <v>35</v>
       </c>
       <c r="K192" t="n">
-        <v>30.3</v>
+        <v>26.1</v>
       </c>
       <c r="L192" t="n">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="M192" t="inlineStr">
         <is>
@@ -17300,7 +17300,7 @@
         <v>41</v>
       </c>
       <c r="T192" t="n">
-        <v>-4.699999999999999</v>
+        <v>-8.899999999999999</v>
       </c>
       <c r="U192" t="n">
         <v>33.26666666666667</v>
@@ -18933,10 +18933,10 @@
         <v>28</v>
       </c>
       <c r="K211" t="n">
-        <v>25.7</v>
+        <v>29.1</v>
       </c>
       <c r="L211" t="n">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="M211" t="inlineStr">
         <is>
@@ -18966,7 +18966,7 @@
         <v>28</v>
       </c>
       <c r="T211" t="n">
-        <v>-2.300000000000001</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U211" t="n">
         <v>27.53333333333333</v>
@@ -19899,10 +19899,10 @@
         <v>21</v>
       </c>
       <c r="K222" t="n">
-        <v>20.5</v>
+        <v>15.3</v>
       </c>
       <c r="L222" t="n">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="M222" t="inlineStr">
         <is>
@@ -19932,7 +19932,7 @@
         <v>21</v>
       </c>
       <c r="T222" t="n">
-        <v>-0.5</v>
+        <v>-5.699999999999999</v>
       </c>
       <c r="U222" t="n">
         <v>18.26666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-26 21:00:58
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3071,10 +3071,10 @@
         <v>28</v>
       </c>
       <c r="K30" t="n">
-        <v>26.9</v>
+        <v>27.1</v>
       </c>
       <c r="L30" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
@@ -3104,7 +3104,7 @@
         <v>28</v>
       </c>
       <c r="T30" t="n">
-        <v>-1.100000000000001</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U30" t="n">
         <v>27.23333333333333</v>
@@ -3503,10 +3503,10 @@
         <v>28</v>
       </c>
       <c r="K35" t="n">
-        <v>22.1</v>
+        <v>33.2</v>
       </c>
       <c r="L35" t="n">
-        <v>79</v>
+        <v>118</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
         <v>28</v>
       </c>
       <c r="T35" t="n">
-        <v>-5.899999999999999</v>
+        <v>5.200000000000003</v>
       </c>
       <c r="U35" t="n">
         <v>30.1</v>
@@ -9631,10 +9631,10 @@
         <v>21</v>
       </c>
       <c r="K105" t="n">
-        <v>18.4</v>
+        <v>29</v>
       </c>
       <c r="L105" t="n">
-        <v>88</v>
+        <v>138</v>
       </c>
       <c r="M105" t="inlineStr">
         <is>
@@ -9664,7 +9664,7 @@
         <v>21</v>
       </c>
       <c r="T105" t="n">
-        <v>-2.600000000000001</v>
+        <v>8</v>
       </c>
       <c r="U105" t="n">
         <v>24.53333333333333</v>
@@ -15071,10 +15071,10 @@
         <v>21</v>
       </c>
       <c r="K167" t="n">
-        <v>20.9</v>
+        <v>22.9</v>
       </c>
       <c r="L167" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="M167" t="inlineStr">
         <is>
@@ -15104,7 +15104,7 @@
         <v>21</v>
       </c>
       <c r="T167" t="n">
-        <v>-0.1000000000000014</v>
+        <v>1.899999999999999</v>
       </c>
       <c r="U167" t="n">
         <v>22.96666666666667</v>
@@ -18317,10 +18317,10 @@
         <v>28</v>
       </c>
       <c r="K204" t="n">
-        <v>27.6</v>
+        <v>28.7</v>
       </c>
       <c r="L204" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M204" t="inlineStr">
         <is>
@@ -18350,7 +18350,7 @@
         <v>28</v>
       </c>
       <c r="T204" t="n">
-        <v>-0.3999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U204" t="n">
         <v>28</v>
@@ -21303,10 +21303,10 @@
         <v>42</v>
       </c>
       <c r="K238" t="n">
-        <v>49</v>
+        <v>31.1</v>
       </c>
       <c r="L238" t="n">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="M238" t="inlineStr">
         <is>
@@ -21336,7 +21336,7 @@
         <v>48</v>
       </c>
       <c r="T238" t="n">
-        <v>7</v>
+        <v>-10.9</v>
       </c>
       <c r="U238" t="n">
         <v>43.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-26 22:15:42
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3853,10 +3853,10 @@
         <v>31</v>
       </c>
       <c r="K39" t="n">
-        <v>36.5</v>
+        <v>27.8</v>
       </c>
       <c r="L39" t="n">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="M39" t="inlineStr">
         <is>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="n">
-        <v>5.5</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U39" t="n">
         <v>33.03333333333333</v>
@@ -5335,10 +5335,10 @@
         <v>31</v>
       </c>
       <c r="K56" t="n">
-        <v>38.5</v>
+        <v>30.5</v>
       </c>
       <c r="L56" t="n">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="M56" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="n">
-        <v>7.5</v>
+        <v>-0.5</v>
       </c>
       <c r="U56" t="n">
         <v>35.86666666666667</v>
@@ -9455,10 +9455,10 @@
         <v>21</v>
       </c>
       <c r="K103" t="n">
-        <v>24.2</v>
+        <v>20.2</v>
       </c>
       <c r="L103" t="n">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9488,7 +9488,7 @@
         <v>21</v>
       </c>
       <c r="T103" t="n">
-        <v>3.199999999999999</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U103" t="n">
         <v>23.23333333333333</v>
@@ -9497,7 +9497,7 @@
         <v>3</v>
       </c>
       <c r="W103" t="n">
-        <v>26.17777777777778</v>
+        <v>26.17777777777777</v>
       </c>
       <c r="X103" t="n">
         <v>17.5</v>
@@ -9631,10 +9631,10 @@
         <v>21</v>
       </c>
       <c r="K105" t="n">
-        <v>29</v>
+        <v>18.4</v>
       </c>
       <c r="L105" t="n">
-        <v>138</v>
+        <v>88</v>
       </c>
       <c r="M105" t="inlineStr">
         <is>
@@ -9664,7 +9664,7 @@
         <v>21</v>
       </c>
       <c r="T105" t="n">
-        <v>8</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U105" t="n">
         <v>24.53333333333333</v>
@@ -11473,10 +11473,10 @@
         <v>21</v>
       </c>
       <c r="K126" t="n">
-        <v>23.7</v>
+        <v>20.2</v>
       </c>
       <c r="L126" t="n">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="M126" t="inlineStr">
         <is>
@@ -11506,7 +11506,7 @@
         <v>21</v>
       </c>
       <c r="T126" t="n">
-        <v>2.699999999999999</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U126" t="n">
         <v>21.43333333333333</v>
@@ -11825,10 +11825,10 @@
         <v>21</v>
       </c>
       <c r="K130" t="n">
-        <v>23.2</v>
+        <v>20.3</v>
       </c>
       <c r="L130" t="n">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -11858,7 +11858,7 @@
         <v>21</v>
       </c>
       <c r="T130" t="n">
-        <v>2.199999999999999</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="U130" t="n">
         <v>22.36666666666666</v>
@@ -11913,10 +11913,10 @@
         <v>28</v>
       </c>
       <c r="K131" t="n">
-        <v>27.7</v>
+        <v>24.6</v>
       </c>
       <c r="L131" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="M131" t="inlineStr">
         <is>
@@ -11946,7 +11946,7 @@
         <v>28</v>
       </c>
       <c r="T131" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U131" t="n">
         <v>25.36666666666666</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-26 23:40:46
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X377"/>
+  <dimension ref="A1:X378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3853,10 +3853,10 @@
         <v>31</v>
       </c>
       <c r="K39" t="n">
-        <v>27.8</v>
+        <v>36.5</v>
       </c>
       <c r="L39" t="n">
-        <v>90</v>
+        <v>118</v>
       </c>
       <c r="M39" t="inlineStr">
         <is>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="n">
-        <v>-3.199999999999999</v>
+        <v>5.5</v>
       </c>
       <c r="U39" t="n">
         <v>33.03333333333333</v>
@@ -5335,10 +5335,10 @@
         <v>31</v>
       </c>
       <c r="K56" t="n">
-        <v>30.5</v>
+        <v>38.5</v>
       </c>
       <c r="L56" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="M56" t="inlineStr">
         <is>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="n">
-        <v>-0.5</v>
+        <v>7.5</v>
       </c>
       <c r="U56" t="n">
         <v>35.86666666666667</v>
@@ -6209,10 +6209,10 @@
         <v>24</v>
       </c>
       <c r="K66" t="n">
-        <v>25.7</v>
+        <v>23.4</v>
       </c>
       <c r="L66" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="M66" t="inlineStr">
         <is>
@@ -6242,7 +6242,7 @@
         <v>28</v>
       </c>
       <c r="T66" t="n">
-        <v>1.699999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U66" t="n">
         <v>24.46666666666667</v>
@@ -6649,10 +6649,10 @@
         <v>35</v>
       </c>
       <c r="K71" t="n">
-        <v>34.3</v>
+        <v>32.3</v>
       </c>
       <c r="L71" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="M71" t="inlineStr">
         <is>
@@ -6682,7 +6682,7 @@
         <v>41</v>
       </c>
       <c r="T71" t="n">
-        <v>-0.7000000000000028</v>
+        <v>-2.700000000000003</v>
       </c>
       <c r="U71" t="n">
         <v>32.96666666666666</v>
@@ -9455,10 +9455,10 @@
         <v>21</v>
       </c>
       <c r="K103" t="n">
-        <v>20.2</v>
+        <v>24.2</v>
       </c>
       <c r="L103" t="n">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9488,7 +9488,7 @@
         <v>21</v>
       </c>
       <c r="T103" t="n">
-        <v>-0.8000000000000007</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="U103" t="n">
         <v>23.23333333333333</v>
@@ -9497,7 +9497,7 @@
         <v>3</v>
       </c>
       <c r="W103" t="n">
-        <v>26.17777777777777</v>
+        <v>26.17777777777778</v>
       </c>
       <c r="X103" t="n">
         <v>17.5</v>
@@ -11473,10 +11473,10 @@
         <v>21</v>
       </c>
       <c r="K126" t="n">
-        <v>20.2</v>
+        <v>23.7</v>
       </c>
       <c r="L126" t="n">
-        <v>96</v>
+        <v>113</v>
       </c>
       <c r="M126" t="inlineStr">
         <is>
@@ -11506,7 +11506,7 @@
         <v>21</v>
       </c>
       <c r="T126" t="n">
-        <v>-0.8000000000000007</v>
+        <v>2.699999999999999</v>
       </c>
       <c r="U126" t="n">
         <v>21.43333333333333</v>
@@ -11825,10 +11825,10 @@
         <v>21</v>
       </c>
       <c r="K130" t="n">
-        <v>20.3</v>
+        <v>23.2</v>
       </c>
       <c r="L130" t="n">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -11858,7 +11858,7 @@
         <v>21</v>
       </c>
       <c r="T130" t="n">
-        <v>-0.6999999999999993</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U130" t="n">
         <v>22.36666666666666</v>
@@ -11913,10 +11913,10 @@
         <v>28</v>
       </c>
       <c r="K131" t="n">
-        <v>24.6</v>
+        <v>27.7</v>
       </c>
       <c r="L131" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="M131" t="inlineStr">
         <is>
@@ -11946,7 +11946,7 @@
         <v>28</v>
       </c>
       <c r="T131" t="n">
-        <v>-3.399999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U131" t="n">
         <v>25.36666666666666</v>
@@ -33193,7 +33193,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>PL24</t>
+          <t>PL-54</t>
         </is>
       </c>
       <c r="C374" t="inlineStr"/>
@@ -33204,17 +33204,17 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>CIMEANTACION PLATAFORMA ZARPA Y ZAPATA EJE C-12 ZAPATA EJE E-6</t>
+          <t>Muro y zarpa plataforma eje 9-10 entre F, zarpa 9-8 eje F</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>9/25/2026 12:00:00 AM</t>
+          <t>10/21/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H374" t="inlineStr"/>
@@ -33225,14 +33225,14 @@
         <v>21</v>
       </c>
       <c r="K374" t="n">
-        <v>18.9</v>
+        <v>21.1</v>
       </c>
       <c r="L374" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M374" t="inlineStr">
         <is>
-          <t>AUTOCOMPAC</t>
+          <t>MURO</t>
         </is>
       </c>
       <c r="N374" t="n">
@@ -33240,7 +33240,7 @@
       </c>
       <c r="O374" t="inlineStr">
         <is>
-          <t>AUTOCOMPAC-21-28</t>
+          <t>MURO-21-28</t>
         </is>
       </c>
       <c r="P374" s="2" t="n">
@@ -33254,18 +33254,20 @@
       <c r="R374" s="2" t="n">
         <v>46321</v>
       </c>
-      <c r="S374" t="inlineStr"/>
+      <c r="S374" t="n">
+        <v>21</v>
+      </c>
       <c r="T374" t="n">
-        <v>-2.100000000000001</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U374" t="n">
-        <v>19.9</v>
+        <v>21.2</v>
       </c>
       <c r="V374" t="n">
         <v>3</v>
       </c>
       <c r="W374" t="n">
-        <v>23.37777777777778</v>
+        <v>24.18888888888889</v>
       </c>
       <c r="X374" t="n">
         <v>17.5</v>
@@ -33279,7 +33281,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>PL30</t>
+          <t>PL24</t>
         </is>
       </c>
       <c r="C375" t="inlineStr"/>
@@ -33290,17 +33292,17 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>VIGAS PLACA PLATAFORMA PISO 1 EJE A-B, 11,10,09</t>
+          <t>CIMEANTACION PLATAFORMA ZARPA Y ZAPATA EJE C-12 ZAPATA EJE E-6</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
         <is>
-          <t>10/1/2026 12:00:00 AM</t>
+          <t>9/25/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H375" t="inlineStr"/>
@@ -33311,14 +33313,14 @@
         <v>21</v>
       </c>
       <c r="K375" t="n">
-        <v>23.5</v>
+        <v>18.9</v>
       </c>
       <c r="L375" t="n">
-        <v>112</v>
+        <v>90</v>
       </c>
       <c r="M375" t="inlineStr">
         <is>
-          <t>PLACA</t>
+          <t>AUTOCOMPAC</t>
         </is>
       </c>
       <c r="N375" t="n">
@@ -33326,7 +33328,7 @@
       </c>
       <c r="O375" t="inlineStr">
         <is>
-          <t>PLACA-21-28</t>
+          <t>AUTOCOMPAC-21-28</t>
         </is>
       </c>
       <c r="P375" s="2" t="n">
@@ -33340,20 +33342,18 @@
       <c r="R375" s="2" t="n">
         <v>46321</v>
       </c>
-      <c r="S375" t="n">
-        <v>21</v>
-      </c>
+      <c r="S375" t="inlineStr"/>
       <c r="T375" t="n">
-        <v>2.5</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U375" t="n">
-        <v>22.16666666666667</v>
+        <v>19.9</v>
       </c>
       <c r="V375" t="n">
         <v>3</v>
       </c>
       <c r="W375" t="n">
-        <v>25.15555555555556</v>
+        <v>23.37777777777778</v>
       </c>
       <c r="X375" t="n">
         <v>17.5</v>
@@ -33367,7 +33367,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>PL55</t>
+          <t>PL30</t>
         </is>
       </c>
       <c r="C376" t="inlineStr"/>
@@ -33378,17 +33378,17 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Muro plataforma B ejes 8 al 9 F Zarpa 11 al 12 F</t>
+          <t>VIGAS PLACA PLATAFORMA PISO 1 EJE A-B, 11,10,09</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>10/22/2026 12:00:00 AM</t>
+          <t>10/1/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H376" t="inlineStr"/>
@@ -33399,14 +33399,14 @@
         <v>21</v>
       </c>
       <c r="K376" t="n">
-        <v>15</v>
+        <v>23.5</v>
       </c>
       <c r="L376" t="n">
-        <v>72</v>
+        <v>112</v>
       </c>
       <c r="M376" t="inlineStr">
         <is>
-          <t>MURO</t>
+          <t>PLACA</t>
         </is>
       </c>
       <c r="N376" t="n">
@@ -33414,7 +33414,7 @@
       </c>
       <c r="O376" t="inlineStr">
         <is>
-          <t>MURO-21-28</t>
+          <t>PLACA-21-28</t>
         </is>
       </c>
       <c r="P376" s="2" t="n">
@@ -33432,16 +33432,16 @@
         <v>21</v>
       </c>
       <c r="T376" t="n">
-        <v>-6</v>
+        <v>2.5</v>
       </c>
       <c r="U376" t="n">
-        <v>15.66666666666667</v>
+        <v>22.16666666666667</v>
       </c>
       <c r="V376" t="n">
         <v>3</v>
       </c>
       <c r="W376" t="n">
-        <v>21.17777777777778</v>
+        <v>25.15555555555556</v>
       </c>
       <c r="X376" t="n">
         <v>17.5</v>
@@ -33455,7 +33455,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>SC 05</t>
+          <t>PL55</t>
         </is>
       </c>
       <c r="C377" t="inlineStr"/>
@@ -33466,17 +33466,17 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>VIGAS CIMENTACION PLACA SUPERIOR EJE 1-3 ENTRE A Y F-SC</t>
+          <t>Muro plataforma B ejes 8 al 9 F Zarpa 11 al 12 F</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t>9/24/2026 12:00:00 AM</t>
+          <t>10/22/2026 12:00:00 AM</t>
         </is>
       </c>
       <c r="H377" t="inlineStr"/>
@@ -33487,51 +33487,139 @@
         <v>21</v>
       </c>
       <c r="K377" t="n">
+        <v>15</v>
+      </c>
+      <c r="L377" t="n">
+        <v>72</v>
+      </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>MURO</t>
+        </is>
+      </c>
+      <c r="N377" t="n">
+        <v>21</v>
+      </c>
+      <c r="O377" t="inlineStr">
+        <is>
+          <t>MURO-21-28</t>
+        </is>
+      </c>
+      <c r="P377" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="Q377" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="R377" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="S377" t="n">
+        <v>21</v>
+      </c>
+      <c r="T377" t="n">
+        <v>-6</v>
+      </c>
+      <c r="U377" t="n">
+        <v>15.66666666666667</v>
+      </c>
+      <c r="V377" t="n">
+        <v>3</v>
+      </c>
+      <c r="W377" t="n">
+        <v>21.17777777777778</v>
+      </c>
+      <c r="X377" t="n">
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>VIALE 26</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>SC 05</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr"/>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Concreto</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>VIGAS CIMENTACION PLACA SUPERIOR EJE 1-3 ENTRE A Y F-SC</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>9/24/2026 12:00:00 AM</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr"/>
+      <c r="I378" t="n">
+        <v>28</v>
+      </c>
+      <c r="J378" t="n">
+        <v>21</v>
+      </c>
+      <c r="K378" t="n">
         <v>19.8</v>
       </c>
-      <c r="L377" t="n">
+      <c r="L378" t="n">
         <v>94</v>
       </c>
-      <c r="M377" t="inlineStr">
+      <c r="M378" t="inlineStr">
         <is>
           <t>PLACA</t>
         </is>
       </c>
-      <c r="N377" t="n">
-        <v>21</v>
-      </c>
-      <c r="O377" t="inlineStr">
+      <c r="N378" t="n">
+        <v>21</v>
+      </c>
+      <c r="O378" t="inlineStr">
         <is>
           <t>PLACA-21-28</t>
         </is>
       </c>
-      <c r="P377" s="2" t="n">
-        <v>46321</v>
-      </c>
-      <c r="Q377" t="inlineStr">
-        <is>
-          <t>NUEVO</t>
-        </is>
-      </c>
-      <c r="R377" s="2" t="n">
-        <v>46321</v>
-      </c>
-      <c r="S377" t="n">
-        <v>21</v>
-      </c>
-      <c r="T377" t="n">
+      <c r="P378" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="Q378" t="inlineStr">
+        <is>
+          <t>NUEVO</t>
+        </is>
+      </c>
+      <c r="R378" s="2" t="n">
+        <v>46321</v>
+      </c>
+      <c r="S378" t="n">
+        <v>21</v>
+      </c>
+      <c r="T378" t="n">
         <v>-1.199999999999999</v>
       </c>
-      <c r="U377" t="n">
+      <c r="U378" t="n">
         <v>18.9</v>
       </c>
-      <c r="V377" t="n">
-        <v>3</v>
-      </c>
-      <c r="W377" t="n">
+      <c r="V378" t="n">
+        <v>3</v>
+      </c>
+      <c r="W378" t="n">
         <v>22.93333333333334</v>
       </c>
-      <c r="X377" t="n">
+      <c r="X378" t="n">
         <v>17.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-27 17:34:33
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4297,10 +4297,10 @@
         <v>28</v>
       </c>
       <c r="K44" t="n">
-        <v>23.6</v>
+        <v>28.7</v>
       </c>
       <c r="L44" t="n">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
@@ -4330,7 +4330,7 @@
         <v>28</v>
       </c>
       <c r="T44" t="n">
-        <v>-4.399999999999999</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U44" t="n">
         <v>27</v>
@@ -4821,10 +4821,10 @@
         <v>28</v>
       </c>
       <c r="K50" t="n">
-        <v>28.3</v>
+        <v>27.2</v>
       </c>
       <c r="L50" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M50" t="inlineStr">
         <is>
@@ -4854,7 +4854,7 @@
         <v>28</v>
       </c>
       <c r="T50" t="n">
-        <v>0.3000000000000007</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U50" t="n">
         <v>28.43333333333333</v>
@@ -5611,10 +5611,10 @@
         <v>28</v>
       </c>
       <c r="K59" t="n">
-        <v>29</v>
+        <v>28.2</v>
       </c>
       <c r="L59" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="M59" t="inlineStr">
         <is>
@@ -5644,7 +5644,7 @@
         <v>28</v>
       </c>
       <c r="T59" t="n">
-        <v>1</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U59" t="n">
         <v>28.2</v>
@@ -9207,10 +9207,10 @@
         <v>24.5</v>
       </c>
       <c r="K100" t="n">
-        <v>29.6</v>
+        <v>22.5</v>
       </c>
       <c r="L100" t="n">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="M100" t="inlineStr">
         <is>
@@ -9240,7 +9240,7 @@
         <v>28</v>
       </c>
       <c r="T100" t="n">
-        <v>5.100000000000001</v>
+        <v>-2</v>
       </c>
       <c r="U100" t="n">
         <v>26.3</v>
@@ -9471,10 +9471,10 @@
         <v>24.5</v>
       </c>
       <c r="K103" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L103" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9504,7 +9504,7 @@
         <v>28</v>
       </c>
       <c r="T103" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U103" t="n">
         <v>24.66666666666667</v>
@@ -10175,10 +10175,10 @@
         <v>24.5</v>
       </c>
       <c r="K111" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L111" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -10208,7 +10208,7 @@
         <v>28</v>
       </c>
       <c r="T111" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U111" t="n">
         <v>27.1</v>
@@ -12111,10 +12111,10 @@
         <v>24.5</v>
       </c>
       <c r="K133" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L133" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M133" t="inlineStr">
         <is>
@@ -12144,10 +12144,10 @@
         <v>28</v>
       </c>
       <c r="T133" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U133" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V133" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-27 21:48:13
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -11847,10 +11847,10 @@
         <v>24.5</v>
       </c>
       <c r="K130" t="n">
-        <v>23.6</v>
+        <v>23.2</v>
       </c>
       <c r="L130" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -11880,7 +11880,7 @@
         <v>28</v>
       </c>
       <c r="T130" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U130" t="n">
         <v>22.63333333333334</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-27 23:37:29
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -9471,10 +9471,10 @@
         <v>24.5</v>
       </c>
       <c r="K103" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L103" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9504,7 +9504,7 @@
         <v>28</v>
       </c>
       <c r="T103" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U103" t="n">
         <v>24.66666666666667</v>
@@ -10175,10 +10175,10 @@
         <v>24.5</v>
       </c>
       <c r="K111" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L111" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -10208,7 +10208,7 @@
         <v>28</v>
       </c>
       <c r="T111" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U111" t="n">
         <v>27.1</v>
@@ -11847,10 +11847,10 @@
         <v>24.5</v>
       </c>
       <c r="K130" t="n">
-        <v>23.2</v>
+        <v>23.6</v>
       </c>
       <c r="L130" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="M130" t="inlineStr">
         <is>
@@ -11880,7 +11880,7 @@
         <v>28</v>
       </c>
       <c r="T130" t="n">
-        <v>-1.300000000000001</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U130" t="n">
         <v>22.63333333333334</v>
@@ -12111,10 +12111,10 @@
         <v>24.5</v>
       </c>
       <c r="K133" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L133" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M133" t="inlineStr">
         <is>
@@ -12144,10 +12144,10 @@
         <v>28</v>
       </c>
       <c r="T133" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U133" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V133" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-28 08:01:11
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3417,10 +3417,10 @@
         <v>31</v>
       </c>
       <c r="K34" t="n">
-        <v>38.5</v>
+        <v>27.8</v>
       </c>
       <c r="L34" t="n">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="M34" t="inlineStr">
         <is>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="n">
-        <v>7.5</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U34" t="n">
         <v>35.83333333333334</v>
@@ -3503,10 +3503,10 @@
         <v>28</v>
       </c>
       <c r="K35" t="n">
-        <v>22.1</v>
+        <v>33.2</v>
       </c>
       <c r="L35" t="n">
-        <v>79</v>
+        <v>118</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -3536,7 +3536,7 @@
         <v>28</v>
       </c>
       <c r="T35" t="n">
-        <v>-5.899999999999999</v>
+        <v>5.200000000000003</v>
       </c>
       <c r="U35" t="n">
         <v>30.1</v>
@@ -3591,10 +3591,10 @@
         <v>31</v>
       </c>
       <c r="K36" t="n">
-        <v>32.6</v>
+        <v>30.9</v>
       </c>
       <c r="L36" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
       </c>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="n">
-        <v>1.600000000000001</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U36" t="n">
         <v>30.8</v>
@@ -3631,7 +3631,7 @@
         <v>3</v>
       </c>
       <c r="W36" t="n">
-        <v>41.12222222222223</v>
+        <v>41.12222222222222</v>
       </c>
       <c r="X36" t="n">
         <v>27.5</v>
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>32.7</v>
+        <v>30.6</v>
       </c>
       <c r="L79" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>1.700000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>26.8</v>
+        <v>38.6</v>
       </c>
       <c r="L83" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>-4.199999999999999</v>
+        <v>7.600000000000001</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>37</v>
+        <v>34.3</v>
       </c>
       <c r="L90" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>6</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.6</v>
+        <v>34.2</v>
       </c>
       <c r="L95" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.600000000000001</v>
+        <v>3.200000000000003</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -10681,10 +10681,10 @@
         <v>35</v>
       </c>
       <c r="K117" t="n">
-        <v>27.7</v>
+        <v>22.5</v>
       </c>
       <c r="L117" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="M117" t="inlineStr">
         <is>
@@ -10714,7 +10714,7 @@
         <v>41</v>
       </c>
       <c r="T117" t="n">
-        <v>-7.300000000000001</v>
+        <v>-12.5</v>
       </c>
       <c r="U117" t="n">
         <v>25.5</v>
@@ -15861,10 +15861,10 @@
         <v>24</v>
       </c>
       <c r="K176" t="n">
-        <v>29.3</v>
+        <v>26.2</v>
       </c>
       <c r="L176" t="n">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="M176" t="inlineStr">
         <is>
@@ -15894,7 +15894,7 @@
         <v>28</v>
       </c>
       <c r="T176" t="n">
-        <v>5.300000000000001</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U176" t="n">
         <v>24.66666666666667</v>
@@ -22439,10 +22439,10 @@
         <v>21</v>
       </c>
       <c r="K251" t="n">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="L251" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M251" t="inlineStr">
         <is>
@@ -22472,7 +22472,7 @@
         <v>21</v>
       </c>
       <c r="T251" t="n">
-        <v>0.5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U251" t="n">
         <v>21.2</v>
@@ -22871,10 +22871,10 @@
         <v>21</v>
       </c>
       <c r="K256" t="n">
-        <v>22.3</v>
+        <v>23.1</v>
       </c>
       <c r="L256" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="M256" t="inlineStr">
         <is>
@@ -22904,7 +22904,7 @@
         <v>21</v>
       </c>
       <c r="T256" t="n">
-        <v>1.300000000000001</v>
+        <v>2.100000000000001</v>
       </c>
       <c r="U256" t="n">
         <v>21.8</v>
@@ -23399,10 +23399,10 @@
         <v>28</v>
       </c>
       <c r="K262" t="n">
-        <v>27.6</v>
+        <v>27.1</v>
       </c>
       <c r="L262" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="M262" t="inlineStr">
         <is>
@@ -23432,7 +23432,7 @@
         <v>28</v>
       </c>
       <c r="T262" t="n">
-        <v>-0.3999999999999986</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U262" t="n">
         <v>27.4</v>
@@ -23487,10 +23487,10 @@
         <v>28</v>
       </c>
       <c r="K263" t="n">
-        <v>28.9</v>
+        <v>28.1</v>
       </c>
       <c r="L263" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="M263" t="inlineStr">
         <is>
@@ -23520,7 +23520,7 @@
         <v>28</v>
       </c>
       <c r="T263" t="n">
-        <v>0.8999999999999986</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U263" t="n">
         <v>28.03333333333333</v>
@@ -23575,10 +23575,10 @@
         <v>28</v>
       </c>
       <c r="K264" t="n">
-        <v>27.2</v>
+        <v>28.4</v>
       </c>
       <c r="L264" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="M264" t="inlineStr">
         <is>
@@ -23608,10 +23608,10 @@
         <v>28</v>
       </c>
       <c r="T264" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U264" t="n">
-        <v>28.06666666666666</v>
+        <v>28.06666666666667</v>
       </c>
       <c r="V264" t="n">
         <v>3</v>
@@ -25329,10 +25329,10 @@
         <v>21</v>
       </c>
       <c r="K284" t="n">
-        <v>21.4</v>
+        <v>19.9</v>
       </c>
       <c r="L284" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="M284" t="inlineStr">
         <is>
@@ -25362,7 +25362,7 @@
         <v>21</v>
       </c>
       <c r="T284" t="n">
-        <v>0.3999999999999986</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U284" t="n">
         <v>21</v>
@@ -25945,10 +25945,10 @@
         <v>21</v>
       </c>
       <c r="K291" t="n">
-        <v>20.5</v>
+        <v>20.9</v>
       </c>
       <c r="L291" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="M291" t="inlineStr">
         <is>
@@ -25976,7 +25976,7 @@
       </c>
       <c r="S291" t="inlineStr"/>
       <c r="T291" t="n">
-        <v>-0.5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U291" t="n">
         <v>20.2</v>
@@ -26557,10 +26557,10 @@
         <v>21</v>
       </c>
       <c r="K298" t="n">
-        <v>18.9</v>
+        <v>19.8</v>
       </c>
       <c r="L298" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="M298" t="inlineStr">
         <is>
@@ -26590,7 +26590,7 @@
         <v>21</v>
       </c>
       <c r="T298" t="n">
-        <v>-2.100000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U298" t="n">
         <v>19</v>
@@ -31565,10 +31565,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>27.8</v>
+        <v>22.9</v>
       </c>
       <c r="L355" t="n">
-        <v>114</v>
+        <v>93</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31598,7 +31598,7 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>3.300000000000001</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U355" t="n">
         <v>25</v>
@@ -31739,10 +31739,10 @@
         <v>24.5</v>
       </c>
       <c r="K357" t="n">
-        <v>28.8</v>
+        <v>23.7</v>
       </c>
       <c r="L357" t="n">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="M357" t="inlineStr">
         <is>
@@ -31772,7 +31772,7 @@
         <v>28</v>
       </c>
       <c r="T357" t="n">
-        <v>4.300000000000001</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U357" t="n">
         <v>25.6</v>
@@ -31827,10 +31827,10 @@
         <v>24.5</v>
       </c>
       <c r="K358" t="n">
-        <v>28.5</v>
+        <v>24.1</v>
       </c>
       <c r="L358" t="n">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="M358" t="inlineStr">
         <is>
@@ -31860,7 +31860,7 @@
         <v>28</v>
       </c>
       <c r="T358" t="n">
-        <v>4</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U358" t="n">
         <v>28.1</v>
@@ -31915,10 +31915,10 @@
         <v>24.5</v>
       </c>
       <c r="K359" t="n">
-        <v>22.7</v>
+        <v>26.3</v>
       </c>
       <c r="L359" t="n">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="M359" t="inlineStr">
         <is>
@@ -31948,7 +31948,7 @@
         <v>28</v>
       </c>
       <c r="T359" t="n">
-        <v>-1.800000000000001</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="U359" t="n">
         <v>24.76666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-28 18:02:05
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -6075,7 +6075,7 @@
         <v>3</v>
       </c>
       <c r="W64" t="n">
-        <v>24.52222222222222</v>
+        <v>24.52222222222223</v>
       </c>
       <c r="X64" t="n">
         <v>20.5</v>
@@ -6121,10 +6121,10 @@
         <v>24</v>
       </c>
       <c r="K65" t="n">
-        <v>16.6</v>
+        <v>26.4</v>
       </c>
       <c r="L65" t="n">
-        <v>69</v>
+        <v>110</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -6154,7 +6154,7 @@
         <v>28</v>
       </c>
       <c r="T65" t="n">
-        <v>-7.399999999999999</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U65" t="n">
         <v>23.4</v>
@@ -6163,7 +6163,7 @@
         <v>3</v>
       </c>
       <c r="W65" t="n">
-        <v>24.64444444444444</v>
+        <v>24.64444444444445</v>
       </c>
       <c r="X65" t="n">
         <v>20.5</v>
@@ -7089,10 +7089,10 @@
         <v>21</v>
       </c>
       <c r="K76" t="n">
-        <v>24.6</v>
+        <v>23.9</v>
       </c>
       <c r="L76" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="M76" t="inlineStr">
         <is>
@@ -7122,7 +7122,7 @@
         <v>21</v>
       </c>
       <c r="T76" t="n">
-        <v>3.600000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="U76" t="n">
         <v>22.76666666666667</v>
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L79" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L83" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L90" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L95" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -10505,10 +10505,10 @@
         <v>35</v>
       </c>
       <c r="K115" t="n">
-        <v>27.3</v>
+        <v>54.5</v>
       </c>
       <c r="L115" t="n">
-        <v>78</v>
+        <v>156</v>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -10538,7 +10538,7 @@
         <v>41</v>
       </c>
       <c r="T115" t="n">
-        <v>-7.699999999999999</v>
+        <v>19.5</v>
       </c>
       <c r="U115" t="n">
         <v>44.9</v>
@@ -13495,10 +13495,10 @@
         <v>35</v>
       </c>
       <c r="K149" t="n">
-        <v>48.5</v>
+        <v>20.3</v>
       </c>
       <c r="L149" t="n">
-        <v>138</v>
+        <v>58</v>
       </c>
       <c r="M149" t="inlineStr">
         <is>
@@ -13528,7 +13528,7 @@
         <v>41</v>
       </c>
       <c r="T149" t="n">
-        <v>13.5</v>
+        <v>-14.7</v>
       </c>
       <c r="U149" t="n">
         <v>30.76666666666667</v>
@@ -15071,10 +15071,10 @@
         <v>21</v>
       </c>
       <c r="K167" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="L167" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="M167" t="inlineStr">
         <is>
@@ -15104,7 +15104,7 @@
         <v>21</v>
       </c>
       <c r="T167" t="n">
-        <v>1.899999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U167" t="n">
         <v>22.96666666666667</v>
@@ -15245,10 +15245,10 @@
         <v>21</v>
       </c>
       <c r="K169" t="n">
-        <v>25.1</v>
+        <v>20.4</v>
       </c>
       <c r="L169" t="n">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="M169" t="inlineStr">
         <is>
@@ -15278,7 +15278,7 @@
         <v>21</v>
       </c>
       <c r="T169" t="n">
-        <v>4.100000000000001</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U169" t="n">
         <v>24.33333333333333</v>
@@ -15333,10 +15333,10 @@
         <v>35</v>
       </c>
       <c r="K170" t="n">
-        <v>34.7</v>
+        <v>37.2</v>
       </c>
       <c r="L170" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="M170" t="inlineStr">
         <is>
@@ -15366,7 +15366,7 @@
         <v>41</v>
       </c>
       <c r="T170" t="n">
-        <v>-0.2999999999999972</v>
+        <v>2.200000000000003</v>
       </c>
       <c r="U170" t="n">
         <v>37.26666666666667</v>
@@ -15421,10 +15421,10 @@
         <v>21</v>
       </c>
       <c r="K171" t="n">
-        <v>20.8</v>
+        <v>23.4</v>
       </c>
       <c r="L171" t="n">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="M171" t="inlineStr">
         <is>
@@ -15454,7 +15454,7 @@
         <v>21</v>
       </c>
       <c r="T171" t="n">
-        <v>-0.1999999999999993</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U171" t="n">
         <v>23.4</v>
@@ -17267,10 +17267,10 @@
         <v>35</v>
       </c>
       <c r="K192" t="n">
-        <v>26.1</v>
+        <v>43.4</v>
       </c>
       <c r="L192" t="n">
-        <v>74</v>
+        <v>124</v>
       </c>
       <c r="M192" t="inlineStr">
         <is>
@@ -17300,7 +17300,7 @@
         <v>41</v>
       </c>
       <c r="T192" t="n">
-        <v>-8.899999999999999</v>
+        <v>8.399999999999999</v>
       </c>
       <c r="U192" t="n">
         <v>33.26666666666667</v>
@@ -17877,10 +17877,10 @@
         <v>21</v>
       </c>
       <c r="K199" t="n">
-        <v>23.9</v>
+        <v>20.7</v>
       </c>
       <c r="L199" t="n">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="M199" t="inlineStr">
         <is>
@@ -17910,7 +17910,7 @@
         <v>21</v>
       </c>
       <c r="T199" t="n">
-        <v>2.899999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U199" t="n">
         <v>22.5</v>
@@ -17965,10 +17965,10 @@
         <v>28</v>
       </c>
       <c r="K200" t="n">
-        <v>26.8</v>
+        <v>32.8</v>
       </c>
       <c r="L200" t="n">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="M200" t="inlineStr">
         <is>
@@ -17998,7 +17998,7 @@
         <v>28</v>
       </c>
       <c r="T200" t="n">
-        <v>-1.199999999999999</v>
+        <v>4.799999999999997</v>
       </c>
       <c r="U200" t="n">
         <v>30.93333333333333</v>
@@ -18053,10 +18053,10 @@
         <v>21</v>
       </c>
       <c r="K201" t="n">
-        <v>22.4</v>
+        <v>23.3</v>
       </c>
       <c r="L201" t="n">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="M201" t="inlineStr">
         <is>
@@ -18086,7 +18086,7 @@
         <v>21</v>
       </c>
       <c r="T201" t="n">
-        <v>1.399999999999999</v>
+        <v>2.300000000000001</v>
       </c>
       <c r="U201" t="n">
         <v>21.26666666666667</v>
@@ -18141,10 +18141,10 @@
         <v>28</v>
       </c>
       <c r="K202" t="n">
-        <v>29.3</v>
+        <v>26.7</v>
       </c>
       <c r="L202" t="n">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="M202" t="inlineStr">
         <is>
@@ -18174,7 +18174,7 @@
         <v>28</v>
       </c>
       <c r="T202" t="n">
-        <v>1.300000000000001</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U202" t="n">
         <v>29.3</v>
@@ -18229,10 +18229,10 @@
         <v>21</v>
       </c>
       <c r="K203" t="n">
-        <v>23.2</v>
+        <v>20.5</v>
       </c>
       <c r="L203" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="M203" t="inlineStr">
         <is>
@@ -18262,7 +18262,7 @@
         <v>21</v>
       </c>
       <c r="T203" t="n">
-        <v>2.199999999999999</v>
+        <v>-0.5</v>
       </c>
       <c r="U203" t="n">
         <v>21.33333333333333</v>
@@ -18317,10 +18317,10 @@
         <v>28</v>
       </c>
       <c r="K204" t="n">
-        <v>28.7</v>
+        <v>27.6</v>
       </c>
       <c r="L204" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M204" t="inlineStr">
         <is>
@@ -18350,7 +18350,7 @@
         <v>28</v>
       </c>
       <c r="T204" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U204" t="n">
         <v>28</v>
@@ -18405,10 +18405,10 @@
         <v>21</v>
       </c>
       <c r="K205" t="n">
-        <v>20.8</v>
+        <v>21.4</v>
       </c>
       <c r="L205" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M205" t="inlineStr">
         <is>
@@ -18438,7 +18438,7 @@
         <v>21</v>
       </c>
       <c r="T205" t="n">
-        <v>-0.1999999999999993</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U205" t="n">
         <v>21.16666666666667</v>
@@ -18493,10 +18493,10 @@
         <v>21</v>
       </c>
       <c r="K206" t="n">
-        <v>23.1</v>
+        <v>20.7</v>
       </c>
       <c r="L206" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="M206" t="inlineStr">
         <is>
@@ -18526,7 +18526,7 @@
         <v>21</v>
       </c>
       <c r="T206" t="n">
-        <v>2.100000000000001</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U206" t="n">
         <v>22.13333333333334</v>
@@ -18535,7 +18535,7 @@
         <v>3</v>
       </c>
       <c r="W206" t="n">
-        <v>24.33333333333333</v>
+        <v>24.33333333333334</v>
       </c>
       <c r="X206" t="n">
         <v>17.5</v>
@@ -18669,10 +18669,10 @@
         <v>28</v>
       </c>
       <c r="K208" t="n">
-        <v>26.8</v>
+        <v>27.9</v>
       </c>
       <c r="L208" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="M208" t="inlineStr">
         <is>
@@ -18702,7 +18702,7 @@
         <v>28</v>
       </c>
       <c r="T208" t="n">
-        <v>-1.199999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U208" t="n">
         <v>27.86666666666666</v>
@@ -18757,10 +18757,10 @@
         <v>28</v>
       </c>
       <c r="K209" t="n">
-        <v>26.1</v>
+        <v>27.7</v>
       </c>
       <c r="L209" t="n">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="M209" t="inlineStr">
         <is>
@@ -18790,7 +18790,7 @@
         <v>28</v>
       </c>
       <c r="T209" t="n">
-        <v>-1.899999999999999</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U209" t="n">
         <v>27.5</v>
@@ -18845,10 +18845,10 @@
         <v>28</v>
       </c>
       <c r="K210" t="n">
-        <v>27.7</v>
+        <v>28.9</v>
       </c>
       <c r="L210" t="n">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="M210" t="inlineStr">
         <is>
@@ -18878,7 +18878,7 @@
         <v>28</v>
       </c>
       <c r="T210" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U210" t="n">
         <v>28.4</v>
@@ -22439,10 +22439,10 @@
         <v>21</v>
       </c>
       <c r="K251" t="n">
-        <v>20.9</v>
+        <v>21.5</v>
       </c>
       <c r="L251" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M251" t="inlineStr">
         <is>
@@ -22472,7 +22472,7 @@
         <v>21</v>
       </c>
       <c r="T251" t="n">
-        <v>-0.1000000000000014</v>
+        <v>0.5</v>
       </c>
       <c r="U251" t="n">
         <v>21.2</v>
@@ -22871,10 +22871,10 @@
         <v>21</v>
       </c>
       <c r="K256" t="n">
-        <v>23.1</v>
+        <v>22.3</v>
       </c>
       <c r="L256" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M256" t="inlineStr">
         <is>
@@ -22904,7 +22904,7 @@
         <v>21</v>
       </c>
       <c r="T256" t="n">
-        <v>2.100000000000001</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="U256" t="n">
         <v>21.8</v>
@@ -23399,10 +23399,10 @@
         <v>28</v>
       </c>
       <c r="K262" t="n">
-        <v>27.1</v>
+        <v>27.6</v>
       </c>
       <c r="L262" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M262" t="inlineStr">
         <is>
@@ -23432,7 +23432,7 @@
         <v>28</v>
       </c>
       <c r="T262" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U262" t="n">
         <v>27.4</v>
@@ -23487,10 +23487,10 @@
         <v>28</v>
       </c>
       <c r="K263" t="n">
-        <v>28.1</v>
+        <v>28.9</v>
       </c>
       <c r="L263" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="M263" t="inlineStr">
         <is>
@@ -23520,7 +23520,7 @@
         <v>28</v>
       </c>
       <c r="T263" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U263" t="n">
         <v>28.03333333333333</v>
@@ -23575,10 +23575,10 @@
         <v>28</v>
       </c>
       <c r="K264" t="n">
-        <v>28.4</v>
+        <v>27.2</v>
       </c>
       <c r="L264" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M264" t="inlineStr">
         <is>
@@ -23608,10 +23608,10 @@
         <v>28</v>
       </c>
       <c r="T264" t="n">
-        <v>0.3999999999999986</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U264" t="n">
-        <v>28.06666666666667</v>
+        <v>28.06666666666666</v>
       </c>
       <c r="V264" t="n">
         <v>3</v>
@@ -24101,10 +24101,10 @@
         <v>28</v>
       </c>
       <c r="K270" t="n">
-        <v>28.1</v>
+        <v>25.8</v>
       </c>
       <c r="L270" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="M270" t="inlineStr">
         <is>
@@ -24134,7 +24134,7 @@
         <v>28</v>
       </c>
       <c r="T270" t="n">
-        <v>0.1000000000000014</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="U270" t="n">
         <v>26.96666666666667</v>
@@ -24977,10 +24977,10 @@
         <v>28</v>
       </c>
       <c r="K280" t="n">
-        <v>26.5</v>
+        <v>28.4</v>
       </c>
       <c r="L280" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="M280" t="inlineStr">
         <is>
@@ -25010,7 +25010,7 @@
         <v>28</v>
       </c>
       <c r="T280" t="n">
-        <v>-1.5</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U280" t="n">
         <v>27.53333333333333</v>
@@ -25241,10 +25241,10 @@
         <v>28</v>
       </c>
       <c r="K283" t="n">
-        <v>28.3</v>
+        <v>27.2</v>
       </c>
       <c r="L283" t="n">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M283" t="inlineStr">
         <is>
@@ -25274,7 +25274,7 @@
         <v>28</v>
       </c>
       <c r="T283" t="n">
-        <v>0.3000000000000007</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U283" t="n">
         <v>27.4</v>
@@ -25329,10 +25329,10 @@
         <v>21</v>
       </c>
       <c r="K284" t="n">
-        <v>19.9</v>
+        <v>21.4</v>
       </c>
       <c r="L284" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="M284" t="inlineStr">
         <is>
@@ -25362,7 +25362,7 @@
         <v>21</v>
       </c>
       <c r="T284" t="n">
-        <v>-1.100000000000001</v>
+        <v>0.3999999999999986</v>
       </c>
       <c r="U284" t="n">
         <v>21</v>
@@ -25945,10 +25945,10 @@
         <v>21</v>
       </c>
       <c r="K291" t="n">
-        <v>20.9</v>
+        <v>20.5</v>
       </c>
       <c r="L291" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="M291" t="inlineStr">
         <is>
@@ -25976,7 +25976,7 @@
       </c>
       <c r="S291" t="inlineStr"/>
       <c r="T291" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.5</v>
       </c>
       <c r="U291" t="n">
         <v>20.2</v>
@@ -26293,10 +26293,10 @@
         <v>21</v>
       </c>
       <c r="K295" t="n">
-        <v>22</v>
+        <v>20.9</v>
       </c>
       <c r="L295" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M295" t="inlineStr">
         <is>
@@ -26326,7 +26326,7 @@
         <v>21</v>
       </c>
       <c r="T295" t="n">
-        <v>1</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U295" t="n">
         <v>21.23333333333333</v>
@@ -26557,10 +26557,10 @@
         <v>21</v>
       </c>
       <c r="K298" t="n">
-        <v>19.8</v>
+        <v>18.3</v>
       </c>
       <c r="L298" t="n">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="M298" t="inlineStr">
         <is>
@@ -26590,7 +26590,7 @@
         <v>21</v>
       </c>
       <c r="T298" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="U298" t="n">
         <v>19</v>
@@ -27431,10 +27431,10 @@
         <v>21</v>
       </c>
       <c r="K308" t="n">
-        <v>21.2</v>
+        <v>20.9</v>
       </c>
       <c r="L308" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M308" t="inlineStr">
         <is>
@@ -27464,10 +27464,10 @@
         <v>21</v>
       </c>
       <c r="T308" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U308" t="n">
-        <v>21.16666666666666</v>
+        <v>21.16666666666667</v>
       </c>
       <c r="V308" t="n">
         <v>3</v>
@@ -27957,10 +27957,10 @@
         <v>24.5</v>
       </c>
       <c r="K314" t="n">
-        <v>25</v>
+        <v>22.6</v>
       </c>
       <c r="L314" t="n">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="M314" t="inlineStr">
         <is>
@@ -27990,7 +27990,7 @@
         <v>28</v>
       </c>
       <c r="T314" t="n">
-        <v>0.5</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="U314" t="n">
         <v>24.8</v>
@@ -29013,10 +29013,10 @@
         <v>24.5</v>
       </c>
       <c r="K326" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L326" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M326" t="inlineStr">
         <is>
@@ -29046,7 +29046,7 @@
         <v>28</v>
       </c>
       <c r="T326" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U326" t="n">
         <v>24.66666666666667</v>
@@ -29717,10 +29717,10 @@
         <v>24.5</v>
       </c>
       <c r="K334" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L334" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M334" t="inlineStr">
         <is>
@@ -29750,7 +29750,7 @@
         <v>28</v>
       </c>
       <c r="T334" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U334" t="n">
         <v>27.1</v>
@@ -30069,10 +30069,10 @@
         <v>24.5</v>
       </c>
       <c r="K338" t="n">
-        <v>25.3</v>
+        <v>24.5</v>
       </c>
       <c r="L338" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="M338" t="inlineStr">
         <is>
@@ -30102,7 +30102,7 @@
         <v>28</v>
       </c>
       <c r="T338" t="n">
-        <v>0.8000000000000007</v>
+        <v>0</v>
       </c>
       <c r="U338" t="n">
         <v>24.6</v>
@@ -31301,10 +31301,10 @@
         <v>24.5</v>
       </c>
       <c r="K352" t="n">
-        <v>23.4</v>
+        <v>23.9</v>
       </c>
       <c r="L352" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="M352" t="inlineStr">
         <is>
@@ -31334,7 +31334,7 @@
         <v>28</v>
       </c>
       <c r="T352" t="n">
-        <v>-1.100000000000001</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U352" t="n">
         <v>24.5</v>
@@ -31565,10 +31565,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>22.9</v>
+        <v>27.8</v>
       </c>
       <c r="L355" t="n">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31598,7 +31598,7 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-1.600000000000001</v>
+        <v>3.300000000000001</v>
       </c>
       <c r="U355" t="n">
         <v>25</v>
@@ -31653,10 +31653,10 @@
         <v>24.5</v>
       </c>
       <c r="K356" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L356" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M356" t="inlineStr">
         <is>
@@ -31686,10 +31686,10 @@
         <v>28</v>
       </c>
       <c r="T356" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U356" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V356" t="n">
         <v>3</v>
@@ -31739,10 +31739,10 @@
         <v>24.5</v>
       </c>
       <c r="K357" t="n">
-        <v>23.7</v>
+        <v>28.8</v>
       </c>
       <c r="L357" t="n">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="M357" t="inlineStr">
         <is>
@@ -31772,7 +31772,7 @@
         <v>28</v>
       </c>
       <c r="T357" t="n">
-        <v>-0.8000000000000007</v>
+        <v>4.300000000000001</v>
       </c>
       <c r="U357" t="n">
         <v>25.6</v>
@@ -31827,10 +31827,10 @@
         <v>24.5</v>
       </c>
       <c r="K358" t="n">
-        <v>24.1</v>
+        <v>28.5</v>
       </c>
       <c r="L358" t="n">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="M358" t="inlineStr">
         <is>
@@ -31860,7 +31860,7 @@
         <v>28</v>
       </c>
       <c r="T358" t="n">
-        <v>-0.3999999999999986</v>
+        <v>4</v>
       </c>
       <c r="U358" t="n">
         <v>28.1</v>
@@ -31915,10 +31915,10 @@
         <v>24.5</v>
       </c>
       <c r="K359" t="n">
-        <v>26.3</v>
+        <v>22.7</v>
       </c>
       <c r="L359" t="n">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="M359" t="inlineStr">
         <is>
@@ -31948,7 +31948,7 @@
         <v>28</v>
       </c>
       <c r="T359" t="n">
-        <v>1.800000000000001</v>
+        <v>-1.800000000000001</v>
       </c>
       <c r="U359" t="n">
         <v>24.76666666666667</v>
@@ -32529,10 +32529,10 @@
         <v>21</v>
       </c>
       <c r="K366" t="n">
-        <v>17.6</v>
+        <v>18.2</v>
       </c>
       <c r="L366" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="M366" t="inlineStr">
         <is>
@@ -32560,16 +32560,16 @@
       </c>
       <c r="S366" t="inlineStr"/>
       <c r="T366" t="n">
-        <v>-3.399999999999999</v>
+        <v>-2.800000000000001</v>
       </c>
       <c r="U366" t="n">
-        <v>18.13333333333334</v>
+        <v>18.13333333333333</v>
       </c>
       <c r="V366" t="n">
         <v>3</v>
       </c>
       <c r="W366" t="n">
-        <v>27.25555555555556</v>
+        <v>27.25555555555555</v>
       </c>
       <c r="X366" t="n">
         <v>17.5</v>
@@ -33313,7 +33313,7 @@
         <v>21</v>
       </c>
       <c r="K375" t="n">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="L375" t="n">
         <v>90</v>
@@ -33344,7 +33344,7 @@
       </c>
       <c r="S375" t="inlineStr"/>
       <c r="T375" t="n">
-        <v>-2.100000000000001</v>
+        <v>-2.199999999999999</v>
       </c>
       <c r="U375" t="n">
         <v>19.9</v>
@@ -33575,10 +33575,10 @@
         <v>21</v>
       </c>
       <c r="K378" t="n">
-        <v>19.8</v>
+        <v>18.7</v>
       </c>
       <c r="L378" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="M378" t="inlineStr">
         <is>
@@ -33608,7 +33608,7 @@
         <v>21</v>
       </c>
       <c r="T378" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.300000000000001</v>
       </c>
       <c r="U378" t="n">
         <v>18.9</v>
@@ -33617,7 +33617,7 @@
         <v>3</v>
       </c>
       <c r="W378" t="n">
-        <v>22.93333333333334</v>
+        <v>22.93333333333333</v>
       </c>
       <c r="X378" t="n">
         <v>17.5</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-28 22:11:55
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -29013,10 +29013,10 @@
         <v>24.5</v>
       </c>
       <c r="K326" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L326" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M326" t="inlineStr">
         <is>
@@ -29046,7 +29046,7 @@
         <v>28</v>
       </c>
       <c r="T326" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U326" t="n">
         <v>24.66666666666667</v>
@@ -29717,10 +29717,10 @@
         <v>24.5</v>
       </c>
       <c r="K334" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L334" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M334" t="inlineStr">
         <is>
@@ -29750,7 +29750,7 @@
         <v>28</v>
       </c>
       <c r="T334" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U334" t="n">
         <v>27.1</v>
@@ -31653,10 +31653,10 @@
         <v>24.5</v>
       </c>
       <c r="K356" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L356" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M356" t="inlineStr">
         <is>
@@ -31686,10 +31686,10 @@
         <v>28</v>
       </c>
       <c r="T356" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U356" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V356" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-28 23:56:36
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3331,10 +3331,10 @@
         <v>31</v>
       </c>
       <c r="K33" t="n">
-        <v>31.6</v>
+        <v>29.8</v>
       </c>
       <c r="L33" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="M33" t="inlineStr">
         <is>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
-        <v>0.6000000000000014</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U33" t="n">
         <v>30.4</v>
@@ -4897,10 +4897,10 @@
         <v>24</v>
       </c>
       <c r="K51" t="n">
-        <v>23.8</v>
+        <v>24.9</v>
       </c>
       <c r="L51" t="n">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
@@ -4930,7 +4930,7 @@
         <v>28</v>
       </c>
       <c r="T51" t="n">
-        <v>-0.1999999999999993</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U51" t="n">
         <v>21.43333333333333</v>
@@ -6209,10 +6209,10 @@
         <v>24</v>
       </c>
       <c r="K66" t="n">
-        <v>25.7</v>
+        <v>23.4</v>
       </c>
       <c r="L66" t="n">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="M66" t="inlineStr">
         <is>
@@ -6242,7 +6242,7 @@
         <v>28</v>
       </c>
       <c r="T66" t="n">
-        <v>1.699999999999999</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U66" t="n">
         <v>24.46666666666667</v>
@@ -7353,10 +7353,10 @@
         <v>31</v>
       </c>
       <c r="K79" t="n">
-        <v>30.6</v>
+        <v>32.7</v>
       </c>
       <c r="L79" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M79" t="inlineStr">
         <is>
@@ -7384,7 +7384,7 @@
       </c>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>-0.3999999999999986</v>
+        <v>1.700000000000003</v>
       </c>
       <c r="U79" t="n">
         <v>32.03333333333333</v>
@@ -7703,10 +7703,10 @@
         <v>31</v>
       </c>
       <c r="K83" t="n">
-        <v>38.6</v>
+        <v>26.8</v>
       </c>
       <c r="L83" t="n">
-        <v>124</v>
+        <v>86</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -7734,7 +7734,7 @@
       </c>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>7.600000000000001</v>
+        <v>-4.199999999999999</v>
       </c>
       <c r="U83" t="n">
         <v>36</v>
@@ -8317,10 +8317,10 @@
         <v>31</v>
       </c>
       <c r="K90" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
       <c r="L90" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="n">
-        <v>3.299999999999997</v>
+        <v>6</v>
       </c>
       <c r="U90" t="n">
         <v>33.63333333333333</v>
@@ -8755,10 +8755,10 @@
         <v>31</v>
       </c>
       <c r="K95" t="n">
-        <v>34.2</v>
+        <v>34.6</v>
       </c>
       <c r="L95" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -8786,7 +8786,7 @@
       </c>
       <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
-        <v>3.200000000000003</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U95" t="n">
         <v>32.76666666666667</v>
@@ -9455,10 +9455,10 @@
         <v>21</v>
       </c>
       <c r="K103" t="n">
-        <v>24.2</v>
+        <v>20.2</v>
       </c>
       <c r="L103" t="n">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -9488,7 +9488,7 @@
         <v>21</v>
       </c>
       <c r="T103" t="n">
-        <v>3.199999999999999</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U103" t="n">
         <v>23.23333333333333</v>
@@ -14193,10 +14193,10 @@
         <v>35</v>
       </c>
       <c r="K157" t="n">
-        <v>38.2</v>
+        <v>34.6</v>
       </c>
       <c r="L157" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="M157" t="inlineStr">
         <is>
@@ -14226,7 +14226,7 @@
         <v>41</v>
       </c>
       <c r="T157" t="n">
-        <v>3.200000000000003</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U157" t="n">
         <v>36.93333333333334</v>
@@ -14281,10 +14281,10 @@
         <v>35</v>
       </c>
       <c r="K158" t="n">
-        <v>36.7</v>
+        <v>31.5</v>
       </c>
       <c r="L158" t="n">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="M158" t="inlineStr">
         <is>
@@ -14314,7 +14314,7 @@
         <v>41</v>
       </c>
       <c r="T158" t="n">
-        <v>1.700000000000003</v>
+        <v>-3.5</v>
       </c>
       <c r="U158" t="n">
         <v>35.23333333333333</v>
@@ -14457,10 +14457,10 @@
         <v>21</v>
       </c>
       <c r="K160" t="n">
-        <v>22.2</v>
+        <v>24.2</v>
       </c>
       <c r="L160" t="n">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="M160" t="inlineStr">
         <is>
@@ -14490,7 +14490,7 @@
         <v>21</v>
       </c>
       <c r="T160" t="n">
-        <v>1.199999999999999</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="U160" t="n">
         <v>21.83333333333333</v>
@@ -18317,10 +18317,10 @@
         <v>28</v>
       </c>
       <c r="K204" t="n">
-        <v>28.7</v>
+        <v>27.6</v>
       </c>
       <c r="L204" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M204" t="inlineStr">
         <is>
@@ -18350,7 +18350,7 @@
         <v>28</v>
       </c>
       <c r="T204" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U204" t="n">
         <v>28</v>
@@ -20515,10 +20515,10 @@
         <v>21</v>
       </c>
       <c r="K229" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="L229" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M229" t="inlineStr">
         <is>
@@ -20548,7 +20548,7 @@
         <v>21</v>
       </c>
       <c r="T229" t="n">
-        <v>1.600000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="U229" t="n">
         <v>21.96666666666667</v>
@@ -21303,10 +21303,10 @@
         <v>42</v>
       </c>
       <c r="K238" t="n">
-        <v>31.1</v>
+        <v>49</v>
       </c>
       <c r="L238" t="n">
-        <v>74</v>
+        <v>116</v>
       </c>
       <c r="M238" t="inlineStr">
         <is>
@@ -21336,7 +21336,7 @@
         <v>48</v>
       </c>
       <c r="T238" t="n">
-        <v>-10.9</v>
+        <v>7</v>
       </c>
       <c r="U238" t="n">
         <v>43.9</v>
@@ -26907,10 +26907,10 @@
         <v>21</v>
       </c>
       <c r="K302" t="n">
-        <v>17.8</v>
+        <v>18.3</v>
       </c>
       <c r="L302" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="M302" t="inlineStr">
         <is>
@@ -26938,7 +26938,7 @@
       </c>
       <c r="S302" t="inlineStr"/>
       <c r="T302" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="U302" t="n">
         <v>17.9</v>
@@ -29013,10 +29013,10 @@
         <v>24.5</v>
       </c>
       <c r="K326" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L326" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M326" t="inlineStr">
         <is>
@@ -29046,7 +29046,7 @@
         <v>28</v>
       </c>
       <c r="T326" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U326" t="n">
         <v>24.66666666666667</v>
@@ -29717,10 +29717,10 @@
         <v>24.5</v>
       </c>
       <c r="K334" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L334" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M334" t="inlineStr">
         <is>
@@ -29750,7 +29750,7 @@
         <v>28</v>
       </c>
       <c r="T334" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U334" t="n">
         <v>27.1</v>
@@ -31653,10 +31653,10 @@
         <v>24.5</v>
       </c>
       <c r="K356" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L356" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M356" t="inlineStr">
         <is>
@@ -31686,10 +31686,10 @@
         <v>28</v>
       </c>
       <c r="T356" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U356" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V356" t="n">
         <v>3</v>
@@ -32615,10 +32615,10 @@
         <v>21</v>
       </c>
       <c r="K367" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="L367" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M367" t="inlineStr">
         <is>
@@ -32648,7 +32648,7 @@
         <v>21</v>
       </c>
       <c r="T367" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U367" t="n">
         <v>20.9</v>
@@ -32703,10 +32703,10 @@
         <v>21</v>
       </c>
       <c r="K368" t="n">
-        <v>23.2</v>
+        <v>22.4</v>
       </c>
       <c r="L368" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M368" t="inlineStr">
         <is>
@@ -32734,7 +32734,7 @@
       </c>
       <c r="S368" t="inlineStr"/>
       <c r="T368" t="n">
-        <v>2.199999999999999</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="U368" t="n">
         <v>21.23333333333333</v>
@@ -32787,10 +32787,10 @@
         <v>21</v>
       </c>
       <c r="K369" t="n">
-        <v>23.4</v>
+        <v>22</v>
       </c>
       <c r="L369" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="M369" t="inlineStr">
         <is>
@@ -32820,7 +32820,7 @@
         <v>21</v>
       </c>
       <c r="T369" t="n">
-        <v>2.399999999999999</v>
+        <v>1</v>
       </c>
       <c r="U369" t="n">
         <v>22.1</v>
@@ -32875,7 +32875,7 @@
         <v>21</v>
       </c>
       <c r="K370" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="L370" t="n">
         <v>94</v>
@@ -32908,7 +32908,7 @@
         <v>21</v>
       </c>
       <c r="T370" t="n">
-        <v>-1.100000000000001</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U370" t="n">
         <v>20.26666666666667</v>
@@ -32963,10 +32963,10 @@
         <v>21</v>
       </c>
       <c r="K371" t="n">
-        <v>23.6</v>
+        <v>20.7</v>
       </c>
       <c r="L371" t="n">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="M371" t="inlineStr">
         <is>
@@ -32996,7 +32996,7 @@
         <v>21</v>
       </c>
       <c r="T371" t="n">
-        <v>2.600000000000001</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U371" t="n">
         <v>22.76666666666667</v>
@@ -33051,10 +33051,10 @@
         <v>21</v>
       </c>
       <c r="K372" t="n">
-        <v>20</v>
+        <v>23.2</v>
       </c>
       <c r="L372" t="n">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="M372" t="inlineStr">
         <is>
@@ -33082,7 +33082,7 @@
       </c>
       <c r="S372" t="inlineStr"/>
       <c r="T372" t="n">
-        <v>-1</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U372" t="n">
         <v>22.3</v>
@@ -33137,10 +33137,10 @@
         <v>21</v>
       </c>
       <c r="K373" t="n">
-        <v>20.4</v>
+        <v>16.3</v>
       </c>
       <c r="L373" t="n">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="M373" t="inlineStr">
         <is>
@@ -33170,7 +33170,7 @@
         <v>21</v>
       </c>
       <c r="T373" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-4.699999999999999</v>
       </c>
       <c r="U373" t="n">
         <v>19.6</v>
@@ -33399,10 +33399,10 @@
         <v>21</v>
       </c>
       <c r="K376" t="n">
-        <v>23.5</v>
+        <v>22.7</v>
       </c>
       <c r="L376" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="M376" t="inlineStr">
         <is>
@@ -33432,7 +33432,7 @@
         <v>21</v>
       </c>
       <c r="T376" t="n">
-        <v>2.5</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="U376" t="n">
         <v>22.16666666666667</v>
@@ -33487,10 +33487,10 @@
         <v>21</v>
       </c>
       <c r="K377" t="n">
-        <v>15</v>
+        <v>15.9</v>
       </c>
       <c r="L377" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="M377" t="inlineStr">
         <is>
@@ -33520,7 +33520,7 @@
         <v>21</v>
       </c>
       <c r="T377" t="n">
-        <v>-6</v>
+        <v>-5.1</v>
       </c>
       <c r="U377" t="n">
         <v>15.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-29 19:40:22
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2451,10 +2451,10 @@
         <v>31</v>
       </c>
       <c r="K23" t="n">
-        <v>16.6</v>
+        <v>32.1</v>
       </c>
       <c r="L23" t="n">
-        <v>54</v>
+        <v>104</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -2482,7 +2482,7 @@
       </c>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="n">
-        <v>-14.4</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U23" t="n">
         <v>25.6</v>
@@ -3143,10 +3143,10 @@
         <v>28</v>
       </c>
       <c r="K31" t="n">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="L31" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -3176,7 +3176,7 @@
         <v>28</v>
       </c>
       <c r="T31" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="U31" t="n">
         <v>30.53333333333333</v>
@@ -3231,10 +3231,10 @@
         <v>28</v>
       </c>
       <c r="K32" t="n">
-        <v>24.9</v>
+        <v>32.4</v>
       </c>
       <c r="L32" t="n">
-        <v>89</v>
+        <v>116</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3264,7 +3264,7 @@
         <v>28</v>
       </c>
       <c r="T32" t="n">
-        <v>-3.100000000000001</v>
+        <v>4.399999999999999</v>
       </c>
       <c r="U32" t="n">
         <v>31.5</v>
@@ -4451,10 +4451,10 @@
         <v>24</v>
       </c>
       <c r="K46" t="n">
-        <v>25.9</v>
+        <v>22.1</v>
       </c>
       <c r="L46" t="n">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="M46" t="inlineStr">
         <is>
@@ -4484,7 +4484,7 @@
         <v>28</v>
       </c>
       <c r="T46" t="n">
-        <v>1.899999999999999</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="U46" t="n">
         <v>24.23333333333333</v>
@@ -9707,10 +9707,10 @@
         <v>35</v>
       </c>
       <c r="K106" t="n">
-        <v>31.8</v>
+        <v>38.4</v>
       </c>
       <c r="L106" t="n">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="M106" t="inlineStr">
         <is>
@@ -9740,7 +9740,7 @@
         <v>41</v>
       </c>
       <c r="T106" t="n">
-        <v>-3.199999999999999</v>
+        <v>3.399999999999999</v>
       </c>
       <c r="U106" t="n">
         <v>36.1</v>
@@ -11907,10 +11907,10 @@
         <v>35</v>
       </c>
       <c r="K131" t="n">
-        <v>29.2</v>
+        <v>36.1</v>
       </c>
       <c r="L131" t="n">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="M131" t="inlineStr">
         <is>
@@ -11940,7 +11940,7 @@
         <v>41</v>
       </c>
       <c r="T131" t="n">
-        <v>-5.800000000000001</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U131" t="n">
         <v>33.9</v>
@@ -13399,10 +13399,10 @@
         <v>35</v>
       </c>
       <c r="K148" t="n">
-        <v>40.2</v>
+        <v>40.9</v>
       </c>
       <c r="L148" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="M148" t="inlineStr">
         <is>
@@ -13432,7 +13432,7 @@
         <v>41</v>
       </c>
       <c r="T148" t="n">
-        <v>5.200000000000003</v>
+        <v>5.899999999999999</v>
       </c>
       <c r="U148" t="n">
         <v>36</v>
@@ -13485,10 +13485,10 @@
         <v>21</v>
       </c>
       <c r="K149" t="n">
-        <v>24.1</v>
+        <v>25.8</v>
       </c>
       <c r="L149" t="n">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="M149" t="inlineStr">
         <is>
@@ -13518,10 +13518,10 @@
         <v>21</v>
       </c>
       <c r="T149" t="n">
-        <v>3.100000000000001</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U149" t="n">
-        <v>23.43333333333333</v>
+        <v>23.43333333333334</v>
       </c>
       <c r="V149" t="n">
         <v>3</v>
@@ -14099,10 +14099,10 @@
         <v>21</v>
       </c>
       <c r="K156" t="n">
-        <v>24.2</v>
+        <v>24.8</v>
       </c>
       <c r="L156" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="M156" t="inlineStr">
         <is>
@@ -14132,7 +14132,7 @@
         <v>21</v>
       </c>
       <c r="T156" t="n">
-        <v>3.199999999999999</v>
+        <v>3.800000000000001</v>
       </c>
       <c r="U156" t="n">
         <v>22.73333333333333</v>
@@ -14187,10 +14187,10 @@
         <v>21</v>
       </c>
       <c r="K157" t="n">
-        <v>20.8</v>
+        <v>26.3</v>
       </c>
       <c r="L157" t="n">
-        <v>99</v>
+        <v>125</v>
       </c>
       <c r="M157" t="inlineStr">
         <is>
@@ -14220,7 +14220,7 @@
         <v>21</v>
       </c>
       <c r="T157" t="n">
-        <v>-0.1999999999999993</v>
+        <v>5.300000000000001</v>
       </c>
       <c r="U157" t="n">
         <v>24.5</v>
@@ -14275,10 +14275,10 @@
         <v>28</v>
       </c>
       <c r="K158" t="n">
-        <v>31.6</v>
+        <v>29.4</v>
       </c>
       <c r="L158" t="n">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="M158" t="inlineStr">
         <is>
@@ -14308,7 +14308,7 @@
         <v>28</v>
       </c>
       <c r="T158" t="n">
-        <v>3.600000000000001</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="U158" t="n">
         <v>28.43333333333334</v>
@@ -14363,10 +14363,10 @@
         <v>31</v>
       </c>
       <c r="K159" t="n">
-        <v>28.7</v>
+        <v>26.6</v>
       </c>
       <c r="L159" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="M159" t="inlineStr">
         <is>
@@ -14394,7 +14394,7 @@
       </c>
       <c r="S159" t="inlineStr"/>
       <c r="T159" t="n">
-        <v>-2.300000000000001</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="U159" t="n">
         <v>28.66666666666667</v>
@@ -15151,10 +15151,10 @@
         <v>28</v>
       </c>
       <c r="K168" t="n">
-        <v>24.8</v>
+        <v>27</v>
       </c>
       <c r="L168" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="M168" t="inlineStr">
         <is>
@@ -15184,7 +15184,7 @@
         <v>28</v>
       </c>
       <c r="T168" t="n">
-        <v>-3.199999999999999</v>
+        <v>-1</v>
       </c>
       <c r="U168" t="n">
         <v>26.4</v>
@@ -15415,10 +15415,10 @@
         <v>21</v>
       </c>
       <c r="K171" t="n">
-        <v>20.5</v>
+        <v>23.8</v>
       </c>
       <c r="L171" t="n">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="M171" t="inlineStr">
         <is>
@@ -15448,7 +15448,7 @@
         <v>21</v>
       </c>
       <c r="T171" t="n">
-        <v>-0.5</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U171" t="n">
         <v>21.66666666666667</v>
@@ -15503,10 +15503,10 @@
         <v>28</v>
       </c>
       <c r="K172" t="n">
-        <v>27.7</v>
+        <v>31.6</v>
       </c>
       <c r="L172" t="n">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="M172" t="inlineStr">
         <is>
@@ -15536,7 +15536,7 @@
         <v>28</v>
       </c>
       <c r="T172" t="n">
-        <v>-0.3000000000000007</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U172" t="n">
         <v>30.13333333333334</v>
@@ -15591,7 +15591,7 @@
         <v>28</v>
       </c>
       <c r="K173" t="n">
-        <v>26.4</v>
+        <v>26.3</v>
       </c>
       <c r="L173" t="n">
         <v>94</v>
@@ -15624,7 +15624,7 @@
         <v>28</v>
       </c>
       <c r="T173" t="n">
-        <v>-1.600000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U173" t="n">
         <v>26.6</v>
@@ -15679,10 +15679,10 @@
         <v>21</v>
       </c>
       <c r="K174" t="n">
-        <v>13</v>
+        <v>19.3</v>
       </c>
       <c r="L174" t="n">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="M174" t="inlineStr">
         <is>
@@ -15712,7 +15712,7 @@
         <v>21</v>
       </c>
       <c r="T174" t="n">
-        <v>-8</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U174" t="n">
         <v>18.23333333333333</v>
@@ -15853,10 +15853,10 @@
         <v>28</v>
       </c>
       <c r="K176" t="n">
-        <v>23.6</v>
+        <v>29</v>
       </c>
       <c r="L176" t="n">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="M176" t="inlineStr">
         <is>
@@ -15886,7 +15886,7 @@
         <v>28</v>
       </c>
       <c r="T176" t="n">
-        <v>-4.399999999999999</v>
+        <v>1</v>
       </c>
       <c r="U176" t="n">
         <v>25.33333333333333</v>
@@ -15941,10 +15941,10 @@
         <v>35</v>
       </c>
       <c r="K177" t="n">
-        <v>38.3</v>
+        <v>34.3</v>
       </c>
       <c r="L177" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="M177" t="inlineStr">
         <is>
@@ -15974,7 +15974,7 @@
         <v>41</v>
       </c>
       <c r="T177" t="n">
-        <v>3.299999999999997</v>
+        <v>-0.7000000000000028</v>
       </c>
       <c r="U177" t="n">
         <v>35.66666666666666</v>
@@ -16029,7 +16029,7 @@
         <v>21</v>
       </c>
       <c r="K178" t="n">
-        <v>22.7</v>
+        <v>22.6</v>
       </c>
       <c r="L178" t="n">
         <v>108</v>
@@ -16062,10 +16062,10 @@
         <v>21</v>
       </c>
       <c r="T178" t="n">
-        <v>1.699999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U178" t="n">
-        <v>21.86666666666666</v>
+        <v>21.86666666666667</v>
       </c>
       <c r="V178" t="n">
         <v>3</v>
@@ -16117,10 +16117,10 @@
         <v>28</v>
       </c>
       <c r="K179" t="n">
-        <v>36.4</v>
+        <v>40.2</v>
       </c>
       <c r="L179" t="n">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="M179" t="inlineStr">
         <is>
@@ -16150,7 +16150,7 @@
         <v>28</v>
       </c>
       <c r="T179" t="n">
-        <v>8.399999999999999</v>
+        <v>12.2</v>
       </c>
       <c r="U179" t="n">
         <v>33.36666666666667</v>
@@ -16205,10 +16205,10 @@
         <v>21</v>
       </c>
       <c r="K180" t="n">
-        <v>20.7</v>
+        <v>20.9</v>
       </c>
       <c r="L180" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M180" t="inlineStr">
         <is>
@@ -16238,7 +16238,7 @@
         <v>21</v>
       </c>
       <c r="T180" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U180" t="n">
         <v>21.3</v>
@@ -16293,10 +16293,10 @@
         <v>28</v>
       </c>
       <c r="K181" t="n">
-        <v>27.6</v>
+        <v>28.5</v>
       </c>
       <c r="L181" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="M181" t="inlineStr">
         <is>
@@ -16326,7 +16326,7 @@
         <v>28</v>
       </c>
       <c r="T181" t="n">
-        <v>-0.3999999999999986</v>
+        <v>0.5</v>
       </c>
       <c r="U181" t="n">
         <v>27.5</v>
@@ -16381,10 +16381,10 @@
         <v>28</v>
       </c>
       <c r="K182" t="n">
-        <v>30.3</v>
+        <v>24</v>
       </c>
       <c r="L182" t="n">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="M182" t="inlineStr">
         <is>
@@ -16414,7 +16414,7 @@
         <v>28</v>
       </c>
       <c r="T182" t="n">
-        <v>2.300000000000001</v>
+        <v>-4</v>
       </c>
       <c r="U182" t="n">
         <v>27.23333333333333</v>
@@ -16469,10 +16469,10 @@
         <v>28</v>
       </c>
       <c r="K183" t="n">
-        <v>30.4</v>
+        <v>28.6</v>
       </c>
       <c r="L183" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="M183" t="inlineStr">
         <is>
@@ -16502,7 +16502,7 @@
         <v>28</v>
       </c>
       <c r="T183" t="n">
-        <v>2.399999999999999</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U183" t="n">
         <v>28.83333333333333</v>
@@ -16557,10 +16557,10 @@
         <v>35</v>
       </c>
       <c r="K184" t="n">
-        <v>32.7</v>
+        <v>32.4</v>
       </c>
       <c r="L184" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M184" t="inlineStr">
         <is>
@@ -16590,7 +16590,7 @@
         <v>41</v>
       </c>
       <c r="T184" t="n">
-        <v>-2.299999999999997</v>
+        <v>-2.600000000000001</v>
       </c>
       <c r="U184" t="n">
         <v>32.26666666666667</v>
@@ -20419,10 +20419,10 @@
         <v>21</v>
       </c>
       <c r="K228" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="L228" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="M228" t="inlineStr">
         <is>
@@ -20452,7 +20452,7 @@
         <v>21</v>
       </c>
       <c r="T228" t="n">
-        <v>1.699999999999999</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="U228" t="n">
         <v>21.56666666666667</v>
@@ -21993,10 +21993,10 @@
         <v>21</v>
       </c>
       <c r="K246" t="n">
-        <v>21.9</v>
+        <v>22.5</v>
       </c>
       <c r="L246" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="M246" t="inlineStr">
         <is>
@@ -22024,7 +22024,7 @@
       </c>
       <c r="S246" t="inlineStr"/>
       <c r="T246" t="n">
-        <v>0.8999999999999986</v>
+        <v>1.5</v>
       </c>
       <c r="U246" t="n">
         <v>21.73333333333333</v>
@@ -22079,10 +22079,10 @@
         <v>21</v>
       </c>
       <c r="K247" t="n">
-        <v>20.7</v>
+        <v>21.5</v>
       </c>
       <c r="L247" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="M247" t="inlineStr">
         <is>
@@ -22110,7 +22110,7 @@
       </c>
       <c r="S247" t="inlineStr"/>
       <c r="T247" t="n">
-        <v>-0.3000000000000007</v>
+        <v>0.5</v>
       </c>
       <c r="U247" t="n">
         <v>20.63333333333334</v>
@@ -22251,10 +22251,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="L249" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22282,7 +22282,7 @@
       </c>
       <c r="S249" t="inlineStr"/>
       <c r="T249" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U249" t="n">
         <v>21.8</v>
@@ -22689,10 +22689,10 @@
         <v>28</v>
       </c>
       <c r="K254" t="n">
-        <v>26.9</v>
+        <v>29.1</v>
       </c>
       <c r="L254" t="n">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="M254" t="inlineStr">
         <is>
@@ -22722,7 +22722,7 @@
         <v>28</v>
       </c>
       <c r="T254" t="n">
-        <v>-1.100000000000001</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U254" t="n">
         <v>27.33333333333333</v>
@@ -25147,10 +25147,10 @@
         <v>21</v>
       </c>
       <c r="K282" t="n">
-        <v>20.8</v>
+        <v>22</v>
       </c>
       <c r="L282" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="M282" t="inlineStr">
         <is>
@@ -25180,7 +25180,7 @@
         <v>21</v>
       </c>
       <c r="T282" t="n">
-        <v>-0.1999999999999993</v>
+        <v>1</v>
       </c>
       <c r="U282" t="n">
         <v>21.03333333333333</v>
@@ -25583,10 +25583,10 @@
         <v>21</v>
       </c>
       <c r="K287" t="n">
-        <v>21.7</v>
+        <v>22.8</v>
       </c>
       <c r="L287" t="n">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="M287" t="inlineStr">
         <is>
@@ -25616,7 +25616,7 @@
         <v>21</v>
       </c>
       <c r="T287" t="n">
-        <v>0.6999999999999993</v>
+        <v>1.800000000000001</v>
       </c>
       <c r="U287" t="n">
         <v>21.53333333333333</v>
@@ -29359,10 +29359,10 @@
         <v>24.5</v>
       </c>
       <c r="K330" t="n">
-        <v>24</v>
+        <v>31.1</v>
       </c>
       <c r="L330" t="n">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="M330" t="inlineStr">
         <is>
@@ -29392,7 +29392,7 @@
         <v>28</v>
       </c>
       <c r="T330" t="n">
-        <v>-0.5</v>
+        <v>6.600000000000001</v>
       </c>
       <c r="U330" t="n">
         <v>29.13333333333334</v>
@@ -31293,10 +31293,10 @@
         <v>24.5</v>
       </c>
       <c r="K352" t="n">
-        <v>28.5</v>
+        <v>24.1</v>
       </c>
       <c r="L352" t="n">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="M352" t="inlineStr">
         <is>
@@ -31326,7 +31326,7 @@
         <v>28</v>
       </c>
       <c r="T352" t="n">
-        <v>4</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U352" t="n">
         <v>28.1</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-29 20:56:39
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -3143,10 +3143,10 @@
         <v>28</v>
       </c>
       <c r="K31" t="n">
-        <v>32.5</v>
+        <v>32</v>
       </c>
       <c r="L31" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
@@ -3176,7 +3176,7 @@
         <v>28</v>
       </c>
       <c r="T31" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="U31" t="n">
         <v>30.53333333333333</v>
@@ -3231,10 +3231,10 @@
         <v>28</v>
       </c>
       <c r="K32" t="n">
-        <v>32.4</v>
+        <v>24.9</v>
       </c>
       <c r="L32" t="n">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -3264,7 +3264,7 @@
         <v>28</v>
       </c>
       <c r="T32" t="n">
-        <v>4.399999999999999</v>
+        <v>-3.100000000000001</v>
       </c>
       <c r="U32" t="n">
         <v>31.5</v>
@@ -4013,10 +4013,10 @@
         <v>24</v>
       </c>
       <c r="K41" t="n">
-        <v>27.7</v>
+        <v>28.6</v>
       </c>
       <c r="L41" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
         <v>28</v>
       </c>
       <c r="T41" t="n">
-        <v>3.699999999999999</v>
+        <v>4.600000000000001</v>
       </c>
       <c r="U41" t="n">
         <v>26.56666666666666</v>
@@ -13399,10 +13399,10 @@
         <v>35</v>
       </c>
       <c r="K148" t="n">
-        <v>40.9</v>
+        <v>40.2</v>
       </c>
       <c r="L148" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="M148" t="inlineStr">
         <is>
@@ -13432,7 +13432,7 @@
         <v>41</v>
       </c>
       <c r="T148" t="n">
-        <v>5.899999999999999</v>
+        <v>5.200000000000003</v>
       </c>
       <c r="U148" t="n">
         <v>36</v>
@@ -13485,10 +13485,10 @@
         <v>21</v>
       </c>
       <c r="K149" t="n">
-        <v>25.8</v>
+        <v>24.1</v>
       </c>
       <c r="L149" t="n">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="M149" t="inlineStr">
         <is>
@@ -13518,10 +13518,10 @@
         <v>21</v>
       </c>
       <c r="T149" t="n">
-        <v>4.800000000000001</v>
+        <v>3.100000000000001</v>
       </c>
       <c r="U149" t="n">
-        <v>23.43333333333334</v>
+        <v>23.43333333333333</v>
       </c>
       <c r="V149" t="n">
         <v>3</v>
@@ -14099,10 +14099,10 @@
         <v>21</v>
       </c>
       <c r="K156" t="n">
-        <v>24.8</v>
+        <v>24.2</v>
       </c>
       <c r="L156" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="M156" t="inlineStr">
         <is>
@@ -14132,7 +14132,7 @@
         <v>21</v>
       </c>
       <c r="T156" t="n">
-        <v>3.800000000000001</v>
+        <v>3.199999999999999</v>
       </c>
       <c r="U156" t="n">
         <v>22.73333333333333</v>
@@ -14187,10 +14187,10 @@
         <v>21</v>
       </c>
       <c r="K157" t="n">
-        <v>26.3</v>
+        <v>20.8</v>
       </c>
       <c r="L157" t="n">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="M157" t="inlineStr">
         <is>
@@ -14220,7 +14220,7 @@
         <v>21</v>
       </c>
       <c r="T157" t="n">
-        <v>5.300000000000001</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U157" t="n">
         <v>24.5</v>
@@ -14275,10 +14275,10 @@
         <v>28</v>
       </c>
       <c r="K158" t="n">
-        <v>29.4</v>
+        <v>31.6</v>
       </c>
       <c r="L158" t="n">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="M158" t="inlineStr">
         <is>
@@ -14308,7 +14308,7 @@
         <v>28</v>
       </c>
       <c r="T158" t="n">
-        <v>1.399999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U158" t="n">
         <v>28.43333333333334</v>
@@ -15415,10 +15415,10 @@
         <v>21</v>
       </c>
       <c r="K171" t="n">
-        <v>23.8</v>
+        <v>20.5</v>
       </c>
       <c r="L171" t="n">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="M171" t="inlineStr">
         <is>
@@ -15448,7 +15448,7 @@
         <v>21</v>
       </c>
       <c r="T171" t="n">
-        <v>2.800000000000001</v>
+        <v>-0.5</v>
       </c>
       <c r="U171" t="n">
         <v>21.66666666666667</v>
@@ -15503,10 +15503,10 @@
         <v>28</v>
       </c>
       <c r="K172" t="n">
-        <v>31.6</v>
+        <v>27.7</v>
       </c>
       <c r="L172" t="n">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="M172" t="inlineStr">
         <is>
@@ -15536,7 +15536,7 @@
         <v>28</v>
       </c>
       <c r="T172" t="n">
-        <v>3.600000000000001</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U172" t="n">
         <v>30.13333333333334</v>
@@ -15591,7 +15591,7 @@
         <v>28</v>
       </c>
       <c r="K173" t="n">
-        <v>26.3</v>
+        <v>26.4</v>
       </c>
       <c r="L173" t="n">
         <v>94</v>
@@ -15624,7 +15624,7 @@
         <v>28</v>
       </c>
       <c r="T173" t="n">
-        <v>-1.699999999999999</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U173" t="n">
         <v>26.6</v>
@@ -15679,10 +15679,10 @@
         <v>21</v>
       </c>
       <c r="K174" t="n">
-        <v>19.3</v>
+        <v>13</v>
       </c>
       <c r="L174" t="n">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="M174" t="inlineStr">
         <is>
@@ -15712,7 +15712,7 @@
         <v>21</v>
       </c>
       <c r="T174" t="n">
-        <v>-1.699999999999999</v>
+        <v>-8</v>
       </c>
       <c r="U174" t="n">
         <v>18.23333333333333</v>
@@ -15853,10 +15853,10 @@
         <v>28</v>
       </c>
       <c r="K176" t="n">
-        <v>29</v>
+        <v>23.6</v>
       </c>
       <c r="L176" t="n">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="M176" t="inlineStr">
         <is>
@@ -15886,7 +15886,7 @@
         <v>28</v>
       </c>
       <c r="T176" t="n">
-        <v>1</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="U176" t="n">
         <v>25.33333333333333</v>
@@ -15941,10 +15941,10 @@
         <v>35</v>
       </c>
       <c r="K177" t="n">
-        <v>34.3</v>
+        <v>38.3</v>
       </c>
       <c r="L177" t="n">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="M177" t="inlineStr">
         <is>
@@ -15974,7 +15974,7 @@
         <v>41</v>
       </c>
       <c r="T177" t="n">
-        <v>-0.7000000000000028</v>
+        <v>3.299999999999997</v>
       </c>
       <c r="U177" t="n">
         <v>35.66666666666666</v>
@@ -16029,7 +16029,7 @@
         <v>21</v>
       </c>
       <c r="K178" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="L178" t="n">
         <v>108</v>
@@ -16062,10 +16062,10 @@
         <v>21</v>
       </c>
       <c r="T178" t="n">
-        <v>1.600000000000001</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="U178" t="n">
-        <v>21.86666666666667</v>
+        <v>21.86666666666666</v>
       </c>
       <c r="V178" t="n">
         <v>3</v>
@@ -16117,10 +16117,10 @@
         <v>28</v>
       </c>
       <c r="K179" t="n">
-        <v>40.2</v>
+        <v>36.4</v>
       </c>
       <c r="L179" t="n">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="M179" t="inlineStr">
         <is>
@@ -16150,7 +16150,7 @@
         <v>28</v>
       </c>
       <c r="T179" t="n">
-        <v>12.2</v>
+        <v>8.399999999999999</v>
       </c>
       <c r="U179" t="n">
         <v>33.36666666666667</v>
@@ -16205,10 +16205,10 @@
         <v>21</v>
       </c>
       <c r="K180" t="n">
-        <v>20.9</v>
+        <v>20.7</v>
       </c>
       <c r="L180" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M180" t="inlineStr">
         <is>
@@ -16238,7 +16238,7 @@
         <v>21</v>
       </c>
       <c r="T180" t="n">
-        <v>-0.1000000000000014</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U180" t="n">
         <v>21.3</v>
@@ -16293,10 +16293,10 @@
         <v>28</v>
       </c>
       <c r="K181" t="n">
-        <v>28.5</v>
+        <v>27.6</v>
       </c>
       <c r="L181" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="M181" t="inlineStr">
         <is>
@@ -16326,7 +16326,7 @@
         <v>28</v>
       </c>
       <c r="T181" t="n">
-        <v>0.5</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U181" t="n">
         <v>27.5</v>
@@ -16381,10 +16381,10 @@
         <v>28</v>
       </c>
       <c r="K182" t="n">
-        <v>24</v>
+        <v>30.3</v>
       </c>
       <c r="L182" t="n">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="M182" t="inlineStr">
         <is>
@@ -16414,7 +16414,7 @@
         <v>28</v>
       </c>
       <c r="T182" t="n">
-        <v>-4</v>
+        <v>2.300000000000001</v>
       </c>
       <c r="U182" t="n">
         <v>27.23333333333333</v>
@@ -16469,10 +16469,10 @@
         <v>28</v>
       </c>
       <c r="K183" t="n">
-        <v>28.6</v>
+        <v>30.4</v>
       </c>
       <c r="L183" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="M183" t="inlineStr">
         <is>
@@ -16502,7 +16502,7 @@
         <v>28</v>
       </c>
       <c r="T183" t="n">
-        <v>0.6000000000000014</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U183" t="n">
         <v>28.83333333333333</v>
@@ -16557,10 +16557,10 @@
         <v>35</v>
       </c>
       <c r="K184" t="n">
-        <v>32.4</v>
+        <v>32.7</v>
       </c>
       <c r="L184" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="M184" t="inlineStr">
         <is>
@@ -16590,7 +16590,7 @@
         <v>41</v>
       </c>
       <c r="T184" t="n">
-        <v>-2.600000000000001</v>
+        <v>-2.299999999999997</v>
       </c>
       <c r="U184" t="n">
         <v>32.26666666666667</v>
@@ -23217,10 +23217,10 @@
         <v>28</v>
       </c>
       <c r="K260" t="n">
-        <v>24.7</v>
+        <v>32.5</v>
       </c>
       <c r="L260" t="n">
-        <v>88</v>
+        <v>116</v>
       </c>
       <c r="M260" t="inlineStr">
         <is>
@@ -23250,7 +23250,7 @@
         <v>28</v>
       </c>
       <c r="T260" t="n">
-        <v>-3.300000000000001</v>
+        <v>4.5</v>
       </c>
       <c r="U260" t="n">
         <v>29.5</v>
@@ -26023,10 +26023,10 @@
         <v>21</v>
       </c>
       <c r="K292" t="n">
-        <v>18.9</v>
+        <v>19.8</v>
       </c>
       <c r="L292" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="M292" t="inlineStr">
         <is>
@@ -26056,7 +26056,7 @@
         <v>21</v>
       </c>
       <c r="T292" t="n">
-        <v>-2.100000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U292" t="n">
         <v>19</v>
@@ -26373,10 +26373,10 @@
         <v>21</v>
       </c>
       <c r="K296" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="L296" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M296" t="inlineStr">
         <is>
@@ -26404,7 +26404,7 @@
       </c>
       <c r="S296" t="inlineStr"/>
       <c r="T296" t="n">
-        <v>-3.199999999999999</v>
+        <v>-3.399999999999999</v>
       </c>
       <c r="U296" t="n">
         <v>17.9</v>
@@ -31293,10 +31293,10 @@
         <v>24.5</v>
       </c>
       <c r="K352" t="n">
-        <v>24.1</v>
+        <v>28.5</v>
       </c>
       <c r="L352" t="n">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="M352" t="inlineStr">
         <is>
@@ -31326,7 +31326,7 @@
         <v>28</v>
       </c>
       <c r="T352" t="n">
-        <v>-0.3999999999999986</v>
+        <v>4</v>
       </c>
       <c r="U352" t="n">
         <v>28.1</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-29 22:24:07
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -2277,10 +2277,10 @@
         <v>24</v>
       </c>
       <c r="K21" t="n">
-        <v>21.6</v>
+        <v>15.8</v>
       </c>
       <c r="L21" t="n">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         <v>28</v>
       </c>
       <c r="T21" t="n">
-        <v>-2.399999999999999</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="U21" t="n">
         <v>19.2</v>
@@ -2537,10 +2537,10 @@
         <v>28</v>
       </c>
       <c r="K24" t="n">
-        <v>27.1</v>
+        <v>26.9</v>
       </c>
       <c r="L24" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
@@ -2570,7 +2570,7 @@
         <v>28</v>
       </c>
       <c r="T24" t="n">
-        <v>-0.8999999999999986</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U24" t="n">
         <v>27.23333333333333</v>
@@ -2711,10 +2711,10 @@
         <v>31</v>
       </c>
       <c r="K26" t="n">
-        <v>36</v>
+        <v>30.9</v>
       </c>
       <c r="L26" t="n">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
@@ -2742,10 +2742,10 @@
       </c>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="n">
-        <v>5</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U26" t="n">
-        <v>33.03333333333333</v>
+        <v>33.03333333333334</v>
       </c>
       <c r="V26" t="n">
         <v>3</v>
@@ -4013,10 +4013,10 @@
         <v>24</v>
       </c>
       <c r="K41" t="n">
-        <v>28.6</v>
+        <v>27.7</v>
       </c>
       <c r="L41" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
         <v>28</v>
       </c>
       <c r="T41" t="n">
-        <v>4.600000000000001</v>
+        <v>3.699999999999999</v>
       </c>
       <c r="U41" t="n">
         <v>26.56666666666666</v>
@@ -4627,10 +4627,10 @@
         <v>24</v>
       </c>
       <c r="K48" t="n">
-        <v>26.2</v>
+        <v>23.6</v>
       </c>
       <c r="L48" t="n">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="M48" t="inlineStr">
         <is>
@@ -4660,7 +4660,7 @@
         <v>28</v>
       </c>
       <c r="T48" t="n">
-        <v>2.199999999999999</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U48" t="n">
         <v>26.56666666666666</v>
@@ -8921,10 +8921,10 @@
         <v>21</v>
       </c>
       <c r="K97" t="n">
-        <v>24.2</v>
+        <v>20.2</v>
       </c>
       <c r="L97" t="n">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="M97" t="inlineStr">
         <is>
@@ -8954,7 +8954,7 @@
         <v>21</v>
       </c>
       <c r="T97" t="n">
-        <v>3.199999999999999</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U97" t="n">
         <v>23.23333333333333</v>
@@ -10147,10 +10147,10 @@
         <v>35</v>
       </c>
       <c r="K111" t="n">
-        <v>22.5</v>
+        <v>26.3</v>
       </c>
       <c r="L111" t="n">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -10180,7 +10180,7 @@
         <v>41</v>
       </c>
       <c r="T111" t="n">
-        <v>-12.5</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="U111" t="n">
         <v>25.5</v>
@@ -12345,10 +12345,10 @@
         <v>28</v>
       </c>
       <c r="K136" t="n">
-        <v>27.4</v>
+        <v>27.9</v>
       </c>
       <c r="L136" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="M136" t="inlineStr">
         <is>
@@ -12378,7 +12378,7 @@
         <v>28</v>
       </c>
       <c r="T136" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U136" t="n">
         <v>28.4</v>
@@ -12961,10 +12961,10 @@
         <v>35</v>
       </c>
       <c r="K143" t="n">
-        <v>48.5</v>
+        <v>20.3</v>
       </c>
       <c r="L143" t="n">
-        <v>138</v>
+        <v>58</v>
       </c>
       <c r="M143" t="inlineStr">
         <is>
@@ -12994,7 +12994,7 @@
         <v>41</v>
       </c>
       <c r="T143" t="n">
-        <v>13.5</v>
+        <v>-14.7</v>
       </c>
       <c r="U143" t="n">
         <v>30.76666666666667</v>
@@ -14187,10 +14187,10 @@
         <v>21</v>
       </c>
       <c r="K157" t="n">
-        <v>20.8</v>
+        <v>26.3</v>
       </c>
       <c r="L157" t="n">
-        <v>99</v>
+        <v>125</v>
       </c>
       <c r="M157" t="inlineStr">
         <is>
@@ -14220,7 +14220,7 @@
         <v>21</v>
       </c>
       <c r="T157" t="n">
-        <v>-0.1999999999999993</v>
+        <v>5.300000000000001</v>
       </c>
       <c r="U157" t="n">
         <v>24.5</v>
@@ -15151,10 +15151,10 @@
         <v>28</v>
       </c>
       <c r="K168" t="n">
-        <v>27</v>
+        <v>27.4</v>
       </c>
       <c r="L168" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="M168" t="inlineStr">
         <is>
@@ -15184,7 +15184,7 @@
         <v>28</v>
       </c>
       <c r="T168" t="n">
-        <v>-1</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U168" t="n">
         <v>26.4</v>
@@ -16117,10 +16117,10 @@
         <v>28</v>
       </c>
       <c r="K179" t="n">
-        <v>36.4</v>
+        <v>40.2</v>
       </c>
       <c r="L179" t="n">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="M179" t="inlineStr">
         <is>
@@ -16150,7 +16150,7 @@
         <v>28</v>
       </c>
       <c r="T179" t="n">
-        <v>8.399999999999999</v>
+        <v>12.2</v>
       </c>
       <c r="U179" t="n">
         <v>33.36666666666667</v>
@@ -18135,10 +18135,10 @@
         <v>28</v>
       </c>
       <c r="K202" t="n">
-        <v>26.8</v>
+        <v>27.9</v>
       </c>
       <c r="L202" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="M202" t="inlineStr">
         <is>
@@ -18168,7 +18168,7 @@
         <v>28</v>
       </c>
       <c r="T202" t="n">
-        <v>-1.199999999999999</v>
+        <v>-0.1000000000000014</v>
       </c>
       <c r="U202" t="n">
         <v>27.86666666666666</v>
@@ -21073,7 +21073,7 @@
         <v>3</v>
       </c>
       <c r="W235" t="n">
-        <v>22.92222222222222</v>
+        <v>22.92222222222223</v>
       </c>
       <c r="X235" t="n">
         <v>20.5</v>
@@ -23217,10 +23217,10 @@
         <v>28</v>
       </c>
       <c r="K260" t="n">
-        <v>32.5</v>
+        <v>24.7</v>
       </c>
       <c r="L260" t="n">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="M260" t="inlineStr">
         <is>
@@ -23250,7 +23250,7 @@
         <v>28</v>
       </c>
       <c r="T260" t="n">
-        <v>4.5</v>
+        <v>-3.300000000000001</v>
       </c>
       <c r="U260" t="n">
         <v>29.5</v>
@@ -24179,10 +24179,10 @@
         <v>28</v>
       </c>
       <c r="K271" t="n">
-        <v>27.5</v>
+        <v>29.6</v>
       </c>
       <c r="L271" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="M271" t="inlineStr">
         <is>
@@ -24212,7 +24212,7 @@
         <v>28</v>
       </c>
       <c r="T271" t="n">
-        <v>-0.5</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U271" t="n">
         <v>28.6</v>
@@ -24221,7 +24221,7 @@
         <v>3</v>
       </c>
       <c r="W271" t="n">
-        <v>32.9888888888889</v>
+        <v>32.98888888888889</v>
       </c>
       <c r="X271" t="n">
         <v>24.5</v>
@@ -25495,10 +25495,10 @@
         <v>21</v>
       </c>
       <c r="K286" t="n">
-        <v>25.9</v>
+        <v>22.6</v>
       </c>
       <c r="L286" t="n">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="M286" t="inlineStr">
         <is>
@@ -25528,7 +25528,7 @@
         <v>21</v>
       </c>
       <c r="T286" t="n">
-        <v>4.899999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U286" t="n">
         <v>22.7</v>
@@ -26023,10 +26023,10 @@
         <v>21</v>
       </c>
       <c r="K292" t="n">
-        <v>19.8</v>
+        <v>18.9</v>
       </c>
       <c r="L292" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="M292" t="inlineStr">
         <is>
@@ -26056,7 +26056,7 @@
         <v>21</v>
       </c>
       <c r="T292" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U292" t="n">
         <v>19</v>
@@ -26373,10 +26373,10 @@
         <v>21</v>
       </c>
       <c r="K296" t="n">
-        <v>17.6</v>
+        <v>17.8</v>
       </c>
       <c r="L296" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M296" t="inlineStr">
         <is>
@@ -26404,7 +26404,7 @@
       </c>
       <c r="S296" t="inlineStr"/>
       <c r="T296" t="n">
-        <v>-3.399999999999999</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U296" t="n">
         <v>17.9</v>
@@ -29447,10 +29447,10 @@
         <v>24.5</v>
       </c>
       <c r="K331" t="n">
-        <v>26.9</v>
+        <v>21</v>
       </c>
       <c r="L331" t="n">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="M331" t="inlineStr">
         <is>
@@ -29480,7 +29480,7 @@
         <v>28</v>
       </c>
       <c r="T331" t="n">
-        <v>2.399999999999999</v>
+        <v>-3.5</v>
       </c>
       <c r="U331" t="n">
         <v>24.26666666666667</v>
@@ -32081,10 +32081,10 @@
         <v>21</v>
       </c>
       <c r="K361" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="L361" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M361" t="inlineStr">
         <is>
@@ -32114,7 +32114,7 @@
         <v>21</v>
       </c>
       <c r="T361" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U361" t="n">
         <v>20.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-30 08:09:05
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -4189,10 +4189,10 @@
         <v>31</v>
       </c>
       <c r="K43" t="n">
-        <v>38.1</v>
+        <v>37.2</v>
       </c>
       <c r="L43" t="n">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="M43" t="inlineStr">
         <is>
@@ -4220,7 +4220,7 @@
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="n">
-        <v>7.100000000000001</v>
+        <v>6.200000000000003</v>
       </c>
       <c r="U43" t="n">
         <v>31.56666666666667</v>
@@ -4275,10 +4275,10 @@
         <v>24</v>
       </c>
       <c r="K44" t="n">
-        <v>17.2</v>
+        <v>30.2</v>
       </c>
       <c r="L44" t="n">
-        <v>71</v>
+        <v>126</v>
       </c>
       <c r="M44" t="inlineStr">
         <is>
@@ -4308,7 +4308,7 @@
         <v>28</v>
       </c>
       <c r="T44" t="n">
-        <v>-6.800000000000001</v>
+        <v>6.199999999999999</v>
       </c>
       <c r="U44" t="n">
         <v>24.16666666666667</v>
@@ -4975,10 +4975,10 @@
         <v>24</v>
       </c>
       <c r="K52" t="n">
-        <v>21.2</v>
+        <v>21.9</v>
       </c>
       <c r="L52" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="M52" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
         <v>28</v>
       </c>
       <c r="T52" t="n">
-        <v>-2.800000000000001</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U52" t="n">
         <v>22.7</v>
@@ -5237,10 +5237,10 @@
         <v>24</v>
       </c>
       <c r="K55" t="n">
-        <v>25.5</v>
+        <v>26.6</v>
       </c>
       <c r="L55" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="M55" t="inlineStr">
         <is>
@@ -5270,7 +5270,7 @@
         <v>28</v>
       </c>
       <c r="T55" t="n">
-        <v>1.5</v>
+        <v>2.600000000000001</v>
       </c>
       <c r="U55" t="n">
         <v>22.46666666666667</v>
@@ -5675,10 +5675,10 @@
         <v>24</v>
       </c>
       <c r="K60" t="n">
-        <v>23.4</v>
+        <v>25.7</v>
       </c>
       <c r="L60" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="M60" t="inlineStr">
         <is>
@@ -5708,7 +5708,7 @@
         <v>28</v>
       </c>
       <c r="T60" t="n">
-        <v>-0.6000000000000014</v>
+        <v>1.699999999999999</v>
       </c>
       <c r="U60" t="n">
         <v>24.46666666666667</v>
@@ -6027,10 +6027,10 @@
         <v>21</v>
       </c>
       <c r="K64" t="n">
-        <v>19.7</v>
+        <v>20.3</v>
       </c>
       <c r="L64" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
@@ -6060,7 +6060,7 @@
         <v>21</v>
       </c>
       <c r="T64" t="n">
-        <v>-1.300000000000001</v>
+        <v>-0.6999999999999993</v>
       </c>
       <c r="U64" t="n">
         <v>20.03333333333333</v>
@@ -6115,10 +6115,10 @@
         <v>35</v>
       </c>
       <c r="K65" t="n">
-        <v>34.3</v>
+        <v>32.3</v>
       </c>
       <c r="L65" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="M65" t="inlineStr">
         <is>
@@ -6148,7 +6148,7 @@
         <v>41</v>
       </c>
       <c r="T65" t="n">
-        <v>-0.7000000000000028</v>
+        <v>-2.700000000000003</v>
       </c>
       <c r="U65" t="n">
         <v>32.96666666666666</v>
@@ -6993,7 +6993,7 @@
         <v>28</v>
       </c>
       <c r="K75" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="L75" t="n">
         <v>88</v>
@@ -7026,7 +7026,7 @@
         <v>28</v>
       </c>
       <c r="T75" t="n">
-        <v>-3.300000000000001</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U75" t="n">
         <v>25.13333333333334</v>
@@ -7255,10 +7255,10 @@
         <v>21</v>
       </c>
       <c r="K78" t="n">
-        <v>17.9</v>
+        <v>26.4</v>
       </c>
       <c r="L78" t="n">
-        <v>85</v>
+        <v>126</v>
       </c>
       <c r="M78" t="inlineStr">
         <is>
@@ -7288,7 +7288,7 @@
         <v>21</v>
       </c>
       <c r="T78" t="n">
-        <v>-3.100000000000001</v>
+        <v>5.399999999999999</v>
       </c>
       <c r="U78" t="n">
         <v>21.3</v>
@@ -7431,10 +7431,10 @@
         <v>21</v>
       </c>
       <c r="K80" t="n">
-        <v>21.2</v>
+        <v>20.2</v>
       </c>
       <c r="L80" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="M80" t="inlineStr">
         <is>
@@ -7464,7 +7464,7 @@
         <v>21</v>
       </c>
       <c r="T80" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U80" t="n">
         <v>22.16666666666667</v>
@@ -7607,10 +7607,10 @@
         <v>21</v>
       </c>
       <c r="K82" t="n">
-        <v>23.8</v>
+        <v>24.7</v>
       </c>
       <c r="L82" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="M82" t="inlineStr">
         <is>
@@ -7640,7 +7640,7 @@
         <v>21</v>
       </c>
       <c r="T82" t="n">
-        <v>2.800000000000001</v>
+        <v>3.699999999999999</v>
       </c>
       <c r="U82" t="n">
         <v>22.53333333333333</v>
@@ -8175,7 +8175,7 @@
         <v>3</v>
       </c>
       <c r="W88" t="n">
-        <v>38.87407407407407</v>
+        <v>38.87407407407408</v>
       </c>
       <c r="X88" t="n">
         <v>31.5</v>
@@ -8307,10 +8307,10 @@
         <v>35</v>
       </c>
       <c r="K90" t="n">
-        <v>36.7</v>
+        <v>33.9</v>
       </c>
       <c r="L90" t="n">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -8340,7 +8340,7 @@
         <v>41</v>
       </c>
       <c r="T90" t="n">
-        <v>1.700000000000003</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U90" t="n">
         <v>36.2</v>
@@ -9097,10 +9097,10 @@
         <v>21</v>
       </c>
       <c r="K99" t="n">
-        <v>18.4</v>
+        <v>29</v>
       </c>
       <c r="L99" t="n">
-        <v>88</v>
+        <v>138</v>
       </c>
       <c r="M99" t="inlineStr">
         <is>
@@ -9130,7 +9130,7 @@
         <v>21</v>
       </c>
       <c r="T99" t="n">
-        <v>-2.600000000000001</v>
+        <v>8</v>
       </c>
       <c r="U99" t="n">
         <v>24.53333333333333</v>
@@ -10851,10 +10851,10 @@
         <v>28</v>
       </c>
       <c r="K119" t="n">
-        <v>33.5</v>
+        <v>31.6</v>
       </c>
       <c r="L119" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="M119" t="inlineStr">
         <is>
@@ -10884,7 +10884,7 @@
         <v>28</v>
       </c>
       <c r="T119" t="n">
-        <v>5.5</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U119" t="n">
         <v>30.83333333333333</v>
@@ -11467,10 +11467,10 @@
         <v>35</v>
       </c>
       <c r="K126" t="n">
-        <v>33.9</v>
+        <v>30.7</v>
       </c>
       <c r="L126" t="n">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="M126" t="inlineStr">
         <is>
@@ -11500,7 +11500,7 @@
         <v>41</v>
       </c>
       <c r="T126" t="n">
-        <v>-1.100000000000001</v>
+        <v>-4.300000000000001</v>
       </c>
       <c r="U126" t="n">
         <v>31.83333333333333</v>
@@ -12257,10 +12257,10 @@
         <v>35</v>
       </c>
       <c r="K135" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="L135" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="M135" t="inlineStr">
         <is>
@@ -12290,7 +12290,7 @@
         <v>41</v>
       </c>
       <c r="T135" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="U135" t="n">
         <v>41</v>
@@ -17431,10 +17431,10 @@
         <v>28</v>
       </c>
       <c r="K194" t="n">
-        <v>32.8</v>
+        <v>26.8</v>
       </c>
       <c r="L194" t="n">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="M194" t="inlineStr">
         <is>
@@ -17464,7 +17464,7 @@
         <v>28</v>
       </c>
       <c r="T194" t="n">
-        <v>4.799999999999997</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U194" t="n">
         <v>30.93333333333333</v>
@@ -18927,10 +18927,10 @@
         <v>28</v>
       </c>
       <c r="K211" t="n">
-        <v>27.4</v>
+        <v>24.5</v>
       </c>
       <c r="L211" t="n">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="M211" t="inlineStr">
         <is>
@@ -18960,7 +18960,7 @@
         <v>28</v>
       </c>
       <c r="T211" t="n">
-        <v>-0.6000000000000014</v>
+        <v>-3.5</v>
       </c>
       <c r="U211" t="n">
         <v>26.16666666666667</v>
@@ -22251,10 +22251,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="L249" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22282,7 +22282,7 @@
       </c>
       <c r="S249" t="inlineStr"/>
       <c r="T249" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U249" t="n">
         <v>21.8</v>
@@ -22513,10 +22513,10 @@
         <v>28</v>
       </c>
       <c r="K252" t="n">
-        <v>27.7</v>
+        <v>26.8</v>
       </c>
       <c r="L252" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="M252" t="inlineStr">
         <is>
@@ -22546,7 +22546,7 @@
         <v>28</v>
       </c>
       <c r="T252" t="n">
-        <v>-0.3000000000000007</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U252" t="n">
         <v>27.16666666666667</v>
@@ -23567,10 +23567,10 @@
         <v>28</v>
       </c>
       <c r="K264" t="n">
-        <v>25.8</v>
+        <v>28.1</v>
       </c>
       <c r="L264" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="M264" t="inlineStr">
         <is>
@@ -23600,7 +23600,7 @@
         <v>28</v>
       </c>
       <c r="T264" t="n">
-        <v>-2.199999999999999</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U264" t="n">
         <v>26.96666666666667</v>
@@ -24179,10 +24179,10 @@
         <v>28</v>
       </c>
       <c r="K271" t="n">
-        <v>27.5</v>
+        <v>29.6</v>
       </c>
       <c r="L271" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="M271" t="inlineStr">
         <is>
@@ -24212,7 +24212,7 @@
         <v>28</v>
       </c>
       <c r="T271" t="n">
-        <v>-0.5</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U271" t="n">
         <v>28.6</v>
@@ -24221,7 +24221,7 @@
         <v>3</v>
       </c>
       <c r="W271" t="n">
-        <v>32.9888888888889</v>
+        <v>32.98888888888889</v>
       </c>
       <c r="X271" t="n">
         <v>24.5</v>
@@ -24267,10 +24267,10 @@
         <v>28</v>
       </c>
       <c r="K272" t="n">
-        <v>27.6</v>
+        <v>30.4</v>
       </c>
       <c r="L272" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="M272" t="inlineStr">
         <is>
@@ -24300,7 +24300,7 @@
         <v>28</v>
       </c>
       <c r="T272" t="n">
-        <v>-0.3999999999999986</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U272" t="n">
         <v>30.16666666666667</v>
@@ -25495,10 +25495,10 @@
         <v>21</v>
       </c>
       <c r="K286" t="n">
-        <v>25.9</v>
+        <v>22.6</v>
       </c>
       <c r="L286" t="n">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="M286" t="inlineStr">
         <is>
@@ -25528,7 +25528,7 @@
         <v>21</v>
       </c>
       <c r="T286" t="n">
-        <v>4.899999999999999</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U286" t="n">
         <v>22.7</v>
@@ -26545,10 +26545,10 @@
         <v>21</v>
       </c>
       <c r="K298" t="n">
-        <v>20</v>
+        <v>19.4</v>
       </c>
       <c r="L298" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="M298" t="inlineStr">
         <is>
@@ -26578,7 +26578,7 @@
         <v>21</v>
       </c>
       <c r="T298" t="n">
-        <v>-1</v>
+        <v>-1.600000000000001</v>
       </c>
       <c r="U298" t="n">
         <v>20.5</v>
@@ -26985,10 +26985,10 @@
         <v>21</v>
       </c>
       <c r="K303" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="L303" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M303" t="inlineStr">
         <is>
@@ -27018,10 +27018,10 @@
         <v>21</v>
       </c>
       <c r="T303" t="n">
-        <v>-1.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U303" t="n">
-        <v>19.63333333333333</v>
+        <v>19.63333333333334</v>
       </c>
       <c r="V303" t="n">
         <v>3</v>
@@ -27337,10 +27337,10 @@
         <v>21</v>
       </c>
       <c r="K307" t="n">
-        <v>26.5</v>
+        <v>20.6</v>
       </c>
       <c r="L307" t="n">
-        <v>126</v>
+        <v>98</v>
       </c>
       <c r="M307" t="inlineStr">
         <is>
@@ -27370,7 +27370,7 @@
         <v>21</v>
       </c>
       <c r="T307" t="n">
-        <v>5.5</v>
+        <v>-0.3999999999999986</v>
       </c>
       <c r="U307" t="n">
         <v>23.9</v>
@@ -27687,10 +27687,10 @@
         <v>24.5</v>
       </c>
       <c r="K311" t="n">
-        <v>25.8</v>
+        <v>23.3</v>
       </c>
       <c r="L311" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="M311" t="inlineStr">
         <is>
@@ -27720,7 +27720,7 @@
         <v>28</v>
       </c>
       <c r="T311" t="n">
-        <v>1.300000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U311" t="n">
         <v>24.26666666666667</v>
@@ -28127,10 +28127,10 @@
         <v>24.5</v>
       </c>
       <c r="K316" t="n">
-        <v>20.9</v>
+        <v>24.6</v>
       </c>
       <c r="L316" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="M316" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         <v>28</v>
       </c>
       <c r="T316" t="n">
-        <v>-3.600000000000001</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U316" t="n">
         <v>23.96666666666667</v>
@@ -28479,10 +28479,10 @@
         <v>24.5</v>
       </c>
       <c r="K320" t="n">
-        <v>23.6</v>
+        <v>25.2</v>
       </c>
       <c r="L320" t="n">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="M320" t="inlineStr">
         <is>
@@ -28512,7 +28512,7 @@
         <v>28</v>
       </c>
       <c r="T320" t="n">
-        <v>-0.8999999999999986</v>
+        <v>0.6999999999999993</v>
       </c>
       <c r="U320" t="n">
         <v>24.66666666666667</v>
@@ -29183,10 +29183,10 @@
         <v>24.5</v>
       </c>
       <c r="K328" t="n">
-        <v>22.8</v>
+        <v>29.3</v>
       </c>
       <c r="L328" t="n">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="M328" t="inlineStr">
         <is>
@@ -29216,7 +29216,7 @@
         <v>28</v>
       </c>
       <c r="T328" t="n">
-        <v>-1.699999999999999</v>
+        <v>4.800000000000001</v>
       </c>
       <c r="U328" t="n">
         <v>27.1</v>
@@ -31119,10 +31119,10 @@
         <v>24.5</v>
       </c>
       <c r="K350" t="n">
-        <v>12.4</v>
+        <v>27.3</v>
       </c>
       <c r="L350" t="n">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="M350" t="inlineStr">
         <is>
@@ -31152,10 +31152,10 @@
         <v>28</v>
       </c>
       <c r="T350" t="n">
-        <v>-12.1</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U350" t="n">
-        <v>22.86666666666666</v>
+        <v>22.86666666666667</v>
       </c>
       <c r="V350" t="n">
         <v>3</v>
@@ -32081,10 +32081,10 @@
         <v>21</v>
       </c>
       <c r="K361" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="L361" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M361" t="inlineStr">
         <is>
@@ -32114,7 +32114,7 @@
         <v>21</v>
       </c>
       <c r="T361" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U361" t="n">
         <v>20.9</v>
@@ -32779,10 +32779,10 @@
         <v>21</v>
       </c>
       <c r="K369" t="n">
-        <v>18.9</v>
+        <v>22</v>
       </c>
       <c r="L369" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="M369" t="inlineStr">
         <is>
@@ -32810,7 +32810,7 @@
       </c>
       <c r="S369" t="inlineStr"/>
       <c r="T369" t="n">
-        <v>-2.100000000000001</v>
+        <v>1</v>
       </c>
       <c r="U369" t="n">
         <v>19.9</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-31 08:04:49
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -12169,10 +12169,10 @@
         <v>28</v>
       </c>
       <c r="K134" t="n">
-        <v>25.9</v>
+        <v>37.6</v>
       </c>
       <c r="L134" t="n">
-        <v>92</v>
+        <v>134</v>
       </c>
       <c r="M134" t="inlineStr">
         <is>
@@ -12202,7 +12202,7 @@
         <v>28</v>
       </c>
       <c r="T134" t="n">
-        <v>-2.100000000000001</v>
+        <v>9.600000000000001</v>
       </c>
       <c r="U134" t="n">
         <v>33.96666666666667</v>
@@ -12257,10 +12257,10 @@
         <v>35</v>
       </c>
       <c r="K135" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="L135" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="M135" t="inlineStr">
         <is>
@@ -12290,7 +12290,7 @@
         <v>41</v>
       </c>
       <c r="T135" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="U135" t="n">
         <v>41</v>
@@ -21731,10 +21731,10 @@
         <v>21</v>
       </c>
       <c r="K243" t="n">
-        <v>18.9</v>
+        <v>22.6</v>
       </c>
       <c r="L243" t="n">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="M243" t="inlineStr">
         <is>
@@ -21762,7 +21762,7 @@
       </c>
       <c r="S243" t="inlineStr"/>
       <c r="T243" t="n">
-        <v>-2.100000000000001</v>
+        <v>1.600000000000001</v>
       </c>
       <c r="U243" t="n">
         <v>20.5</v>
@@ -22165,10 +22165,10 @@
         <v>21</v>
       </c>
       <c r="K248" t="n">
-        <v>24.6</v>
+        <v>13.3</v>
       </c>
       <c r="L248" t="n">
-        <v>117</v>
+        <v>63</v>
       </c>
       <c r="M248" t="inlineStr">
         <is>
@@ -22196,7 +22196,7 @@
       </c>
       <c r="S248" t="inlineStr"/>
       <c r="T248" t="n">
-        <v>3.600000000000001</v>
+        <v>-7.699999999999999</v>
       </c>
       <c r="U248" t="n">
         <v>20.13333333333334</v>
@@ -26023,10 +26023,10 @@
         <v>21</v>
       </c>
       <c r="K292" t="n">
-        <v>18.9</v>
+        <v>19.8</v>
       </c>
       <c r="L292" t="n">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="M292" t="inlineStr">
         <is>
@@ -26056,7 +26056,7 @@
         <v>21</v>
       </c>
       <c r="T292" t="n">
-        <v>-2.100000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U292" t="n">
         <v>19</v>
@@ -26373,10 +26373,10 @@
         <v>21</v>
       </c>
       <c r="K296" t="n">
-        <v>17.8</v>
+        <v>18.3</v>
       </c>
       <c r="L296" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="M296" t="inlineStr">
         <is>
@@ -26404,7 +26404,7 @@
       </c>
       <c r="S296" t="inlineStr"/>
       <c r="T296" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="U296" t="n">
         <v>17.9</v>
@@ -27423,10 +27423,10 @@
         <v>24.5</v>
       </c>
       <c r="K308" t="n">
-        <v>25</v>
+        <v>22.6</v>
       </c>
       <c r="L308" t="n">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="M308" t="inlineStr">
         <is>
@@ -27456,7 +27456,7 @@
         <v>28</v>
       </c>
       <c r="T308" t="n">
-        <v>0.5</v>
+        <v>-1.899999999999999</v>
       </c>
       <c r="U308" t="n">
         <v>24.8</v>
@@ -27511,10 +27511,10 @@
         <v>24.5</v>
       </c>
       <c r="K309" t="n">
-        <v>25.1</v>
+        <v>23.9</v>
       </c>
       <c r="L309" t="n">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="M309" t="inlineStr">
         <is>
@@ -27544,7 +27544,7 @@
         <v>28</v>
       </c>
       <c r="T309" t="n">
-        <v>0.6000000000000014</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U309" t="n">
         <v>25.13333333333334</v>
@@ -27687,10 +27687,10 @@
         <v>24.5</v>
       </c>
       <c r="K311" t="n">
-        <v>23.3</v>
+        <v>25.8</v>
       </c>
       <c r="L311" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="M311" t="inlineStr">
         <is>
@@ -27720,7 +27720,7 @@
         <v>28</v>
       </c>
       <c r="T311" t="n">
-        <v>-1.199999999999999</v>
+        <v>1.300000000000001</v>
       </c>
       <c r="U311" t="n">
         <v>24.26666666666667</v>
@@ -28303,10 +28303,10 @@
         <v>24.5</v>
       </c>
       <c r="K318" t="n">
-        <v>23.7</v>
+        <v>28.3</v>
       </c>
       <c r="L318" t="n">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="M318" t="inlineStr">
         <is>
@@ -28336,7 +28336,7 @@
         <v>28</v>
       </c>
       <c r="T318" t="n">
-        <v>-0.8000000000000007</v>
+        <v>3.800000000000001</v>
       </c>
       <c r="U318" t="n">
         <v>25.7</v>
@@ -28479,10 +28479,10 @@
         <v>24.5</v>
       </c>
       <c r="K320" t="n">
-        <v>25.2</v>
+        <v>23.6</v>
       </c>
       <c r="L320" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="M320" t="inlineStr">
         <is>
@@ -28512,7 +28512,7 @@
         <v>28</v>
       </c>
       <c r="T320" t="n">
-        <v>0.6999999999999993</v>
+        <v>-0.8999999999999986</v>
       </c>
       <c r="U320" t="n">
         <v>24.66666666666667</v>
@@ -29183,10 +29183,10 @@
         <v>24.5</v>
       </c>
       <c r="K328" t="n">
-        <v>29.3</v>
+        <v>22.8</v>
       </c>
       <c r="L328" t="n">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="M328" t="inlineStr">
         <is>
@@ -29216,7 +29216,7 @@
         <v>28</v>
       </c>
       <c r="T328" t="n">
-        <v>4.800000000000001</v>
+        <v>-1.699999999999999</v>
       </c>
       <c r="U328" t="n">
         <v>27.1</v>
@@ -29711,10 +29711,10 @@
         <v>24.5</v>
       </c>
       <c r="K334" t="n">
-        <v>24</v>
+        <v>25.6</v>
       </c>
       <c r="L334" t="n">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="M334" t="inlineStr">
         <is>
@@ -29744,7 +29744,7 @@
         <v>28</v>
       </c>
       <c r="T334" t="n">
-        <v>-0.5</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U334" t="n">
         <v>35.8</v>
@@ -31119,10 +31119,10 @@
         <v>24.5</v>
       </c>
       <c r="K350" t="n">
-        <v>27.3</v>
+        <v>12.4</v>
       </c>
       <c r="L350" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="M350" t="inlineStr">
         <is>
@@ -31152,10 +31152,10 @@
         <v>28</v>
       </c>
       <c r="T350" t="n">
-        <v>2.800000000000001</v>
+        <v>-12.1</v>
       </c>
       <c r="U350" t="n">
-        <v>22.86666666666667</v>
+        <v>22.86666666666666</v>
       </c>
       <c r="V350" t="n">
         <v>3</v>
@@ -31819,10 +31819,10 @@
         <v>24.5</v>
       </c>
       <c r="K358" t="n">
-        <v>27.4</v>
+        <v>23.2</v>
       </c>
       <c r="L358" t="n">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="M358" t="inlineStr">
         <is>
@@ -31852,7 +31852,7 @@
         <v>28</v>
       </c>
       <c r="T358" t="n">
-        <v>2.899999999999999</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U358" t="n">
         <v>24.7</v>
@@ -32169,10 +32169,10 @@
         <v>21</v>
       </c>
       <c r="K362" t="n">
-        <v>23.2</v>
+        <v>22.4</v>
       </c>
       <c r="L362" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M362" t="inlineStr">
         <is>
@@ -32200,7 +32200,7 @@
       </c>
       <c r="S362" t="inlineStr"/>
       <c r="T362" t="n">
-        <v>2.199999999999999</v>
+        <v>1.399999999999999</v>
       </c>
       <c r="U362" t="n">
         <v>21.23333333333333</v>
@@ -32253,10 +32253,10 @@
         <v>21</v>
       </c>
       <c r="K363" t="n">
-        <v>23.4</v>
+        <v>22</v>
       </c>
       <c r="L363" t="n">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="M363" t="inlineStr">
         <is>
@@ -32286,7 +32286,7 @@
         <v>21</v>
       </c>
       <c r="T363" t="n">
-        <v>2.399999999999999</v>
+        <v>1</v>
       </c>
       <c r="U363" t="n">
         <v>22.1</v>
@@ -32341,7 +32341,7 @@
         <v>21</v>
       </c>
       <c r="K364" t="n">
-        <v>19.9</v>
+        <v>19.7</v>
       </c>
       <c r="L364" t="n">
         <v>94</v>
@@ -32374,7 +32374,7 @@
         <v>21</v>
       </c>
       <c r="T364" t="n">
-        <v>-1.100000000000001</v>
+        <v>-1.300000000000001</v>
       </c>
       <c r="U364" t="n">
         <v>20.26666666666667</v>
@@ -32429,10 +32429,10 @@
         <v>21</v>
       </c>
       <c r="K365" t="n">
-        <v>23.6</v>
+        <v>20.7</v>
       </c>
       <c r="L365" t="n">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="M365" t="inlineStr">
         <is>
@@ -32462,7 +32462,7 @@
         <v>21</v>
       </c>
       <c r="T365" t="n">
-        <v>2.600000000000001</v>
+        <v>-0.3000000000000007</v>
       </c>
       <c r="U365" t="n">
         <v>22.76666666666667</v>
@@ -32691,10 +32691,10 @@
         <v>21</v>
       </c>
       <c r="K368" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="L368" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="M368" t="inlineStr">
         <is>
@@ -32724,7 +32724,7 @@
         <v>21</v>
       </c>
       <c r="T368" t="n">
-        <v>0.1000000000000014</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U368" t="n">
         <v>21.2</v>
@@ -32953,10 +32953,10 @@
         <v>21</v>
       </c>
       <c r="K371" t="n">
-        <v>15</v>
+        <v>15.9</v>
       </c>
       <c r="L371" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="M371" t="inlineStr">
         <is>
@@ -32986,7 +32986,7 @@
         <v>21</v>
       </c>
       <c r="T371" t="n">
-        <v>-6</v>
+        <v>-5.1</v>
       </c>
       <c r="U371" t="n">
         <v>15.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-31 16:53:56
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -21731,10 +21731,10 @@
         <v>21</v>
       </c>
       <c r="K243" t="n">
-        <v>22.6</v>
+        <v>18.9</v>
       </c>
       <c r="L243" t="n">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="M243" t="inlineStr">
         <is>
@@ -21762,7 +21762,7 @@
       </c>
       <c r="S243" t="inlineStr"/>
       <c r="T243" t="n">
-        <v>1.600000000000001</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U243" t="n">
         <v>20.5</v>
@@ -22165,10 +22165,10 @@
         <v>21</v>
       </c>
       <c r="K248" t="n">
-        <v>13.3</v>
+        <v>24.6</v>
       </c>
       <c r="L248" t="n">
-        <v>63</v>
+        <v>117</v>
       </c>
       <c r="M248" t="inlineStr">
         <is>
@@ -22196,7 +22196,7 @@
       </c>
       <c r="S248" t="inlineStr"/>
       <c r="T248" t="n">
-        <v>-7.699999999999999</v>
+        <v>3.600000000000001</v>
       </c>
       <c r="U248" t="n">
         <v>20.13333333333334</v>
@@ -22251,10 +22251,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>21.3</v>
+        <v>23.8</v>
       </c>
       <c r="L249" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22282,7 +22282,7 @@
       </c>
       <c r="S249" t="inlineStr"/>
       <c r="T249" t="n">
-        <v>0.3000000000000007</v>
+        <v>2.800000000000001</v>
       </c>
       <c r="U249" t="n">
         <v>21.8</v>
@@ -22425,10 +22425,10 @@
         <v>21</v>
       </c>
       <c r="K251" t="n">
-        <v>42.6</v>
+        <v>16.6</v>
       </c>
       <c r="L251" t="n">
-        <v>203</v>
+        <v>79</v>
       </c>
       <c r="M251" t="inlineStr">
         <is>
@@ -22458,7 +22458,7 @@
         <v>21</v>
       </c>
       <c r="T251" t="n">
-        <v>21.6</v>
+        <v>-4.399999999999999</v>
       </c>
       <c r="U251" t="n">
         <v>36.33333333333334</v>
@@ -22689,10 +22689,10 @@
         <v>28</v>
       </c>
       <c r="K254" t="n">
-        <v>29.1</v>
+        <v>26</v>
       </c>
       <c r="L254" t="n">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="M254" t="inlineStr">
         <is>
@@ -22722,7 +22722,7 @@
         <v>28</v>
       </c>
       <c r="T254" t="n">
-        <v>1.100000000000001</v>
+        <v>-2</v>
       </c>
       <c r="U254" t="n">
         <v>27.33333333333333</v>
@@ -24091,10 +24091,10 @@
         <v>21</v>
       </c>
       <c r="K270" t="n">
-        <v>17.8</v>
+        <v>18.3</v>
       </c>
       <c r="L270" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="M270" t="inlineStr">
         <is>
@@ -24124,7 +24124,7 @@
         <v>21</v>
       </c>
       <c r="T270" t="n">
-        <v>-3.199999999999999</v>
+        <v>-2.699999999999999</v>
       </c>
       <c r="U270" t="n">
         <v>18.73333333333333</v>
@@ -24619,10 +24619,10 @@
         <v>28</v>
       </c>
       <c r="K276" t="n">
-        <v>28.2</v>
+        <v>27.4</v>
       </c>
       <c r="L276" t="n">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="M276" t="inlineStr">
         <is>
@@ -24652,7 +24652,7 @@
         <v>28</v>
       </c>
       <c r="T276" t="n">
-        <v>0.1999999999999993</v>
+        <v>-0.6000000000000014</v>
       </c>
       <c r="U276" t="n">
         <v>28.2</v>
@@ -26023,10 +26023,10 @@
         <v>21</v>
       </c>
       <c r="K292" t="n">
-        <v>19.8</v>
+        <v>18.9</v>
       </c>
       <c r="L292" t="n">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="M292" t="inlineStr">
         <is>
@@ -26056,7 +26056,7 @@
         <v>21</v>
       </c>
       <c r="T292" t="n">
-        <v>-1.199999999999999</v>
+        <v>-2.100000000000001</v>
       </c>
       <c r="U292" t="n">
         <v>19</v>
@@ -26373,10 +26373,10 @@
         <v>21</v>
       </c>
       <c r="K296" t="n">
-        <v>18.3</v>
+        <v>17.8</v>
       </c>
       <c r="L296" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="M296" t="inlineStr">
         <is>
@@ -26404,7 +26404,7 @@
       </c>
       <c r="S296" t="inlineStr"/>
       <c r="T296" t="n">
-        <v>-2.699999999999999</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U296" t="n">
         <v>17.9</v>
@@ -27423,10 +27423,10 @@
         <v>24.5</v>
       </c>
       <c r="K308" t="n">
-        <v>22.6</v>
+        <v>25</v>
       </c>
       <c r="L308" t="n">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="M308" t="inlineStr">
         <is>
@@ -27456,7 +27456,7 @@
         <v>28</v>
       </c>
       <c r="T308" t="n">
-        <v>-1.899999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="U308" t="n">
         <v>24.8</v>
@@ -27511,10 +27511,10 @@
         <v>24.5</v>
       </c>
       <c r="K309" t="n">
-        <v>23.9</v>
+        <v>25.1</v>
       </c>
       <c r="L309" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="M309" t="inlineStr">
         <is>
@@ -27544,7 +27544,7 @@
         <v>28</v>
       </c>
       <c r="T309" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.6000000000000014</v>
       </c>
       <c r="U309" t="n">
         <v>25.13333333333334</v>
@@ -27687,10 +27687,10 @@
         <v>24.5</v>
       </c>
       <c r="K311" t="n">
-        <v>25.8</v>
+        <v>23.3</v>
       </c>
       <c r="L311" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="M311" t="inlineStr">
         <is>
@@ -27720,7 +27720,7 @@
         <v>28</v>
       </c>
       <c r="T311" t="n">
-        <v>1.300000000000001</v>
+        <v>-1.199999999999999</v>
       </c>
       <c r="U311" t="n">
         <v>24.26666666666667</v>
@@ -28215,10 +28215,10 @@
         <v>24.5</v>
       </c>
       <c r="K317" t="n">
-        <v>22.5</v>
+        <v>29.6</v>
       </c>
       <c r="L317" t="n">
-        <v>92</v>
+        <v>121</v>
       </c>
       <c r="M317" t="inlineStr">
         <is>
@@ -28248,7 +28248,7 @@
         <v>28</v>
       </c>
       <c r="T317" t="n">
-        <v>-2</v>
+        <v>5.100000000000001</v>
       </c>
       <c r="U317" t="n">
         <v>26.3</v>
@@ -28303,10 +28303,10 @@
         <v>24.5</v>
       </c>
       <c r="K318" t="n">
-        <v>28.3</v>
+        <v>23.7</v>
       </c>
       <c r="L318" t="n">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="M318" t="inlineStr">
         <is>
@@ -28336,7 +28336,7 @@
         <v>28</v>
       </c>
       <c r="T318" t="n">
-        <v>3.800000000000001</v>
+        <v>-0.8000000000000007</v>
       </c>
       <c r="U318" t="n">
         <v>25.7</v>
@@ -31819,10 +31819,10 @@
         <v>24.5</v>
       </c>
       <c r="K358" t="n">
-        <v>23.2</v>
+        <v>27.4</v>
       </c>
       <c r="L358" t="n">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="M358" t="inlineStr">
         <is>
@@ -31852,7 +31852,7 @@
         <v>28</v>
       </c>
       <c r="T358" t="n">
-        <v>-1.300000000000001</v>
+        <v>2.899999999999999</v>
       </c>
       <c r="U358" t="n">
         <v>24.7</v>
@@ -32169,10 +32169,10 @@
         <v>21</v>
       </c>
       <c r="K362" t="n">
-        <v>22.4</v>
+        <v>23.2</v>
       </c>
       <c r="L362" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="M362" t="inlineStr">
         <is>
@@ -32200,7 +32200,7 @@
       </c>
       <c r="S362" t="inlineStr"/>
       <c r="T362" t="n">
-        <v>1.399999999999999</v>
+        <v>2.199999999999999</v>
       </c>
       <c r="U362" t="n">
         <v>21.23333333333333</v>
@@ -32253,10 +32253,10 @@
         <v>21</v>
       </c>
       <c r="K363" t="n">
-        <v>22</v>
+        <v>23.4</v>
       </c>
       <c r="L363" t="n">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="M363" t="inlineStr">
         <is>
@@ -32286,7 +32286,7 @@
         <v>21</v>
       </c>
       <c r="T363" t="n">
-        <v>1</v>
+        <v>2.399999999999999</v>
       </c>
       <c r="U363" t="n">
         <v>22.1</v>
@@ -32341,7 +32341,7 @@
         <v>21</v>
       </c>
       <c r="K364" t="n">
-        <v>19.7</v>
+        <v>19.9</v>
       </c>
       <c r="L364" t="n">
         <v>94</v>
@@ -32374,7 +32374,7 @@
         <v>21</v>
       </c>
       <c r="T364" t="n">
-        <v>-1.300000000000001</v>
+        <v>-1.100000000000001</v>
       </c>
       <c r="U364" t="n">
         <v>20.26666666666667</v>
@@ -32429,10 +32429,10 @@
         <v>21</v>
       </c>
       <c r="K365" t="n">
-        <v>20.7</v>
+        <v>23.6</v>
       </c>
       <c r="L365" t="n">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="M365" t="inlineStr">
         <is>
@@ -32462,7 +32462,7 @@
         <v>21</v>
       </c>
       <c r="T365" t="n">
-        <v>-0.3000000000000007</v>
+        <v>2.600000000000001</v>
       </c>
       <c r="U365" t="n">
         <v>22.76666666666667</v>
@@ -32691,10 +32691,10 @@
         <v>21</v>
       </c>
       <c r="K368" t="n">
-        <v>20.2</v>
+        <v>21.1</v>
       </c>
       <c r="L368" t="n">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="M368" t="inlineStr">
         <is>
@@ -32724,7 +32724,7 @@
         <v>21</v>
       </c>
       <c r="T368" t="n">
-        <v>-0.8000000000000007</v>
+        <v>0.1000000000000014</v>
       </c>
       <c r="U368" t="n">
         <v>21.2</v>
@@ -32953,10 +32953,10 @@
         <v>21</v>
       </c>
       <c r="K371" t="n">
-        <v>15.9</v>
+        <v>15</v>
       </c>
       <c r="L371" t="n">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="M371" t="inlineStr">
         <is>
@@ -32986,7 +32986,7 @@
         <v>21</v>
       </c>
       <c r="T371" t="n">
-        <v>-5.1</v>
+        <v>-6</v>
       </c>
       <c r="U371" t="n">
         <v>15.66666666666667</v>

</xml_diff>

<commit_message>
[AUTO] Unificación de datos - 2026-10-31 18:36:17
</commit_message>
<xml_diff>
--- a/desplegable/Incumplimientos.xlsx
+++ b/desplegable/Incumplimientos.xlsx
@@ -21993,10 +21993,10 @@
         <v>21</v>
       </c>
       <c r="K246" t="n">
-        <v>22.5</v>
+        <v>21.9</v>
       </c>
       <c r="L246" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="M246" t="inlineStr">
         <is>
@@ -22024,7 +22024,7 @@
       </c>
       <c r="S246" t="inlineStr"/>
       <c r="T246" t="n">
-        <v>1.5</v>
+        <v>0.8999999999999986</v>
       </c>
       <c r="U246" t="n">
         <v>21.73333333333333</v>
@@ -22251,10 +22251,10 @@
         <v>21</v>
       </c>
       <c r="K249" t="n">
-        <v>23.8</v>
+        <v>21.3</v>
       </c>
       <c r="L249" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="M249" t="inlineStr">
         <is>
@@ -22282,7 +22282,7 @@
       </c>
       <c r="S249" t="inlineStr"/>
       <c r="T249" t="n">
-        <v>2.800000000000001</v>
+        <v>0.3000000000000007</v>
       </c>
       <c r="U249" t="n">
         <v>21.8</v>
@@ -22425,10 +22425,10 @@
         <v>21</v>
       </c>
       <c r="K251" t="n">
-        <v>16.6</v>
+        <v>42.6</v>
       </c>
       <c r="L251" t="n">
-        <v>79</v>
+        <v>203</v>
       </c>
       <c r="M251" t="inlineStr">
         <is>
@@ -22458,7 +22458,7 @@
         <v>21</v>
       </c>
       <c r="T251" t="n">
-        <v>-4.399999999999999</v>
+        <v>21.6</v>
       </c>
       <c r="U251" t="n">
         <v>36.33333333333334</v>
@@ -22689,10 +22689,10 @@
         <v>28</v>
       </c>
       <c r="K254" t="n">
-        <v>26</v>
+        <v>29.1</v>
       </c>
       <c r="L254" t="n">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="M254" t="inlineStr">
         <is>
@@ -22722,7 +22722,7 @@
         <v>28</v>
       </c>
       <c r="T254" t="n">
-        <v>-2</v>
+        <v>1.100000000000001</v>
       </c>
       <c r="U254" t="n">
         <v>27.33333333333333</v>
@@ -24091,10 +24091,10 @@
         <v>21</v>
       </c>
       <c r="K270" t="n">
-        <v>18.3</v>
+        <v>17.8</v>
       </c>
       <c r="L270" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="M270" t="inlineStr">
         <is>
@@ -24124,7 +24124,7 @@
         <v>21</v>
       </c>
       <c r="T270" t="n">
-        <v>-2.699999999999999</v>
+        <v>-3.199999999999999</v>
       </c>
       <c r="U270" t="n">
         <v>18.73333333333333</v>
@@ -24619,10 +24619,10 @@
         <v>28</v>
       </c>
       <c r="K276" t="n">
-        <v>27.4</v>
+        <v>28.2</v>
       </c>
       <c r="L276" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="M276" t="inlineStr">
         <is>
@@ -24652,7 +24652,7 @@
         <v>28</v>
       </c>
       <c r="T276" t="n">
-        <v>-0.6000000000000014</v>
+        <v>0.1999999999999993</v>
       </c>
       <c r="U276" t="n">
         <v>28.2</v>
@@ -25235,10 +25235,10 @@
         <v>21</v>
       </c>
       <c r="K283" t="n">
-        <v>18.2</v>
+        <v>18.6</v>
       </c>
       <c r="L283" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="M283" t="inlineStr">
         <is>
@@ -25268,7 +25268,7 @@
         <v>21</v>
       </c>
       <c r="T283" t="n">
-        <v>-2.800000000000001</v>
+        <v>-2.399999999999999</v>
       </c>
       <c r="U283" t="n">
         <v>18.23333333333333</v>
@@ -28127,10 +28127,10 @@
         <v>24.5</v>
       </c>
       <c r="K316" t="n">
-        <v>24.6</v>
+        <v>20.9</v>
       </c>
       <c r="L316" t="n">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="M316" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         <v>28</v>
       </c>
       <c r="T316" t="n">
-        <v>0.1000000000000014</v>
+        <v>-3.600000000000001</v>
       </c>
       <c r="U316" t="n">
         <v>23.96666666666667</v>
@@ -28215,10 +28215,10 @@
         <v>24.5</v>
       </c>
       <c r="K317" t="n">
-        <v>29.6</v>
+        <v>22.5</v>
       </c>
       <c r="L317" t="n">
-        <v>121</v>
+        <v>92</v>
       </c>
       <c r="M317" t="inlineStr">
         <is>
@@ -28248,7 +28248,7 @@
         <v>28</v>
       </c>
       <c r="T317" t="n">
-        <v>5.100000000000001</v>
+        <v>-2</v>
       </c>
       <c r="U317" t="n">
         <v>26.3</v>
@@ -29007,10 +29007,10 @@
         <v>24.5</v>
       </c>
       <c r="K326" t="n">
-        <v>18.6</v>
+        <v>24.3</v>
       </c>
       <c r="L326" t="n">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="M326" t="inlineStr">
         <is>
@@ -29040,10 +29040,10 @@
         <v>28</v>
       </c>
       <c r="T326" t="n">
-        <v>-5.899999999999999</v>
+        <v>-0.1999999999999993</v>
       </c>
       <c r="U326" t="n">
-        <v>21.93333333333333</v>
+        <v>21.93333333333334</v>
       </c>
       <c r="V326" t="n">
         <v>3</v>
@@ -31557,10 +31557,10 @@
         <v>24.5</v>
       </c>
       <c r="K355" t="n">
-        <v>24</v>
+        <v>29.6</v>
       </c>
       <c r="L355" t="n">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="M355" t="inlineStr">
         <is>
@@ -31590,7 +31590,7 @@
         <v>28</v>
       </c>
       <c r="T355" t="n">
-        <v>-0.5</v>
+        <v>5.100000000000001</v>
       </c>
       <c r="U355" t="n">
         <v>26.4</v>
@@ -32779,10 +32779,10 @@
         <v>21</v>
       </c>
       <c r="K369" t="n">
-        <v>18.9</v>
+        <v>22</v>
       </c>
       <c r="L369" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="M369" t="inlineStr">
         <is>
@@ -32810,7 +32810,7 @@
       </c>
       <c r="S369" t="inlineStr"/>
       <c r="T369" t="n">
-        <v>-2.100000000000001</v>
+        <v>1</v>
       </c>
       <c r="U369" t="n">
         <v>19.9</v>

</xml_diff>